<commit_message>
Mon Sep  7 06:12:22 UTC 2026
</commit_message>
<xml_diff>
--- a/bp.com-content-dam-bp-country-sites-en_au-australia-home-products-services-pricing-tgp-excel.xlsx
+++ b/bp.com-content-dam-bp-country-sites-en_au-australia-home-products-services-pricing-tgp-excel.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://bp365.sharepoint.com/sites/WholesalePricing/Shared Documents/B2C/TGP/Daily TGP/Web TGP/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="14_{360754B7-B8EB-4990-8E42-75843C960E79}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="14_{12F0505E-791A-498B-ACA4-D4122E8588D1}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-28920" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{1B412EEF-F96D-4DF4-A4E9-C7F0F183C2FB}"/>
+    <workbookView xWindow="-28920" yWindow="-60" windowWidth="29040" windowHeight="15720" xr2:uid="{1B412EEF-F96D-4DF4-A4E9-C7F0F183C2FB}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
@@ -808,128 +808,128 @@
     </row>
     <row r="8" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A8" s="7">
-        <v>46270</v>
+        <v>46273</v>
       </c>
       <c r="B8" s="8"/>
       <c r="C8" s="9" t="s">
         <v>10</v>
       </c>
       <c r="D8" s="10">
-        <v>239.99</v>
+        <v>242.28</v>
       </c>
       <c r="E8" s="10">
-        <v>203.64</v>
+        <v>205.55</v>
       </c>
       <c r="F8" s="10">
-        <v>213.64</v>
+        <v>215.55</v>
       </c>
       <c r="G8" s="10">
-        <v>203.6</v>
+        <v>205.52</v>
       </c>
     </row>
     <row r="9" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A9" s="11">
-        <v>46270</v>
+        <v>46273</v>
       </c>
       <c r="B9" s="12"/>
       <c r="C9" s="12" t="s">
         <v>11</v>
       </c>
       <c r="D9" s="13">
-        <v>239.99</v>
+        <v>242.28</v>
       </c>
       <c r="E9" s="13">
-        <v>203.64</v>
+        <v>205.55</v>
       </c>
       <c r="F9" s="13">
-        <v>213.64</v>
+        <v>215.55</v>
       </c>
       <c r="G9" s="13">
-        <v>203.6</v>
+        <v>205.52</v>
       </c>
     </row>
     <row r="10" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A10" s="7">
-        <v>46270</v>
+        <v>46273</v>
       </c>
       <c r="B10" s="8"/>
       <c r="C10" s="9" t="s">
         <v>12</v>
       </c>
       <c r="D10" s="10">
-        <v>236.44</v>
+        <v>238.87</v>
       </c>
       <c r="E10" s="10">
-        <v>200.9</v>
+        <v>202.94</v>
       </c>
       <c r="F10" s="10">
-        <v>210.9</v>
+        <v>212.94</v>
       </c>
       <c r="G10" s="10">
-        <v>201.32</v>
+        <v>203.36</v>
       </c>
     </row>
     <row r="11" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A11" s="11">
-        <v>46269</v>
+        <v>46270</v>
       </c>
       <c r="B11" s="12"/>
       <c r="C11" s="12" t="s">
         <v>10</v>
       </c>
       <c r="D11" s="13">
-        <v>236.7</v>
+        <v>239.99</v>
       </c>
       <c r="E11" s="13">
-        <v>201.18</v>
+        <v>203.64</v>
       </c>
       <c r="F11" s="13">
-        <v>211.18</v>
+        <v>213.64</v>
       </c>
       <c r="G11" s="13">
-        <v>201.14</v>
+        <v>203.6</v>
       </c>
     </row>
     <row r="12" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A12" s="7">
-        <v>46269</v>
+        <v>46270</v>
       </c>
       <c r="B12" s="8"/>
       <c r="C12" s="9" t="s">
         <v>11</v>
       </c>
       <c r="D12" s="10">
-        <v>236.7</v>
+        <v>239.99</v>
       </c>
       <c r="E12" s="10">
-        <v>201.18</v>
+        <v>203.64</v>
       </c>
       <c r="F12" s="10">
-        <v>211.18</v>
+        <v>213.64</v>
       </c>
       <c r="G12" s="10">
-        <v>201.14</v>
+        <v>203.6</v>
       </c>
     </row>
     <row r="13" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A13" s="11">
-        <v>46269</v>
+        <v>46270</v>
       </c>
       <c r="B13" s="12"/>
       <c r="C13" s="12" t="s">
         <v>12</v>
       </c>
       <c r="D13" s="13">
-        <v>234.21</v>
+        <v>236.44</v>
       </c>
       <c r="E13" s="13">
-        <v>198.39</v>
+        <v>200.9</v>
       </c>
       <c r="F13" s="13">
-        <v>208.39</v>
+        <v>210.9</v>
       </c>
       <c r="G13" s="13">
-        <v>198.81</v>
+        <v>201.32</v>
       </c>
     </row>
     <row r="14" spans="1:7" x14ac:dyDescent="0.25">
@@ -973,39 +973,39 @@
     </row>
     <row r="17" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A17" s="7">
-        <v>46270</v>
+        <v>46273</v>
       </c>
       <c r="B17" s="8"/>
       <c r="C17" s="20" t="s">
         <v>14</v>
       </c>
       <c r="D17" s="10">
-        <v>242</v>
+        <v>244.37</v>
       </c>
       <c r="E17" s="10">
-        <v>205.66</v>
+        <v>207.64</v>
       </c>
       <c r="F17" s="10">
-        <v>215.66</v>
+        <v>217.64</v>
       </c>
       <c r="G17" s="17"/>
     </row>
     <row r="18" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A18" s="11">
-        <v>46269</v>
+        <v>46270</v>
       </c>
       <c r="B18" s="12"/>
       <c r="C18" s="12" t="s">
         <v>14</v>
       </c>
       <c r="D18" s="13">
-        <v>238.7</v>
+        <v>242</v>
       </c>
       <c r="E18" s="13">
-        <v>203.17</v>
+        <v>205.66</v>
       </c>
       <c r="F18" s="13">
-        <v>213.17</v>
+        <v>215.66</v>
       </c>
       <c r="G18" s="17"/>
     </row>
@@ -1052,41 +1052,41 @@
     </row>
     <row r="22" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A22" s="7">
-        <v>46270</v>
+        <v>46273</v>
       </c>
       <c r="B22" s="8"/>
       <c r="C22" s="20" t="s">
         <v>16</v>
       </c>
       <c r="D22" s="10">
-        <v>241.13</v>
+        <v>243.42</v>
       </c>
       <c r="E22" s="10">
-        <v>204.34</v>
+        <v>206.25</v>
       </c>
       <c r="F22" s="10">
-        <v>213.94</v>
+        <v>215.85</v>
       </c>
       <c r="G22" s="10">
-        <v>203.05</v>
+        <v>204.97</v>
       </c>
     </row>
     <row r="23" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A23" s="11">
-        <v>46270</v>
+        <v>46273</v>
       </c>
       <c r="B23" s="12"/>
       <c r="C23" s="21" t="s">
         <v>17</v>
       </c>
       <c r="D23" s="13">
-        <v>241.13</v>
+        <v>243.58</v>
       </c>
       <c r="E23" s="13">
-        <v>208.32</v>
+        <v>210.39</v>
       </c>
       <c r="F23" s="13">
-        <v>218.32</v>
+        <v>220.39</v>
       </c>
       <c r="G23" s="13" t="s">
         <v>18</v>
@@ -1094,20 +1094,20 @@
     </row>
     <row r="24" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A24" s="7">
-        <v>46270</v>
+        <v>46273</v>
       </c>
       <c r="B24" s="8"/>
       <c r="C24" s="20" t="s">
         <v>19</v>
       </c>
       <c r="D24" s="10">
-        <v>241.74</v>
+        <v>244.17</v>
       </c>
       <c r="E24" s="10">
-        <v>207.65</v>
+        <v>209.71</v>
       </c>
       <c r="F24" s="10">
-        <v>217.65</v>
+        <v>219.71</v>
       </c>
       <c r="G24" s="10" t="s">
         <v>18</v>
@@ -1115,41 +1115,41 @@
     </row>
     <row r="25" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A25" s="11">
-        <v>46270</v>
+        <v>46273</v>
       </c>
       <c r="B25" s="12"/>
       <c r="C25" s="21" t="s">
         <v>20</v>
       </c>
       <c r="D25" s="13">
-        <v>238.51</v>
+        <v>240.94</v>
       </c>
       <c r="E25" s="13">
-        <v>207.6</v>
+        <v>209.68</v>
       </c>
       <c r="F25" s="13">
-        <v>217.6</v>
+        <v>219.68</v>
       </c>
       <c r="G25" s="13">
-        <v>205.5</v>
+        <v>207.57</v>
       </c>
     </row>
     <row r="26" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A26" s="7">
-        <v>46270</v>
+        <v>46273</v>
       </c>
       <c r="B26" s="8"/>
       <c r="C26" s="20" t="s">
         <v>21</v>
       </c>
       <c r="D26" s="10">
-        <v>240.48</v>
+        <v>242.9</v>
       </c>
       <c r="E26" s="10">
-        <v>208.87</v>
+        <v>210.96</v>
       </c>
       <c r="F26" s="10">
-        <v>218.87</v>
+        <v>220.96</v>
       </c>
       <c r="G26" s="10" t="s">
         <v>18</v>
@@ -1157,41 +1157,41 @@
     </row>
     <row r="27" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A27" s="11">
-        <v>46269</v>
+        <v>46270</v>
       </c>
       <c r="B27" s="12"/>
       <c r="C27" s="12" t="s">
         <v>16</v>
       </c>
       <c r="D27" s="13">
-        <v>237.84</v>
+        <v>241.13</v>
       </c>
       <c r="E27" s="13">
-        <v>201.88</v>
+        <v>204.34</v>
       </c>
       <c r="F27" s="13">
-        <v>211.48</v>
+        <v>213.94</v>
       </c>
       <c r="G27" s="13">
-        <v>200.59</v>
+        <v>203.05</v>
       </c>
     </row>
     <row r="28" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A28" s="7">
-        <v>46269</v>
+        <v>46270</v>
       </c>
       <c r="B28" s="8"/>
       <c r="C28" s="20" t="s">
         <v>17</v>
       </c>
       <c r="D28" s="10">
-        <v>237.79</v>
+        <v>241.13</v>
       </c>
       <c r="E28" s="22">
-        <v>205.8</v>
+        <v>208.32</v>
       </c>
       <c r="F28" s="22">
-        <v>215.8</v>
+        <v>218.32</v>
       </c>
       <c r="G28" s="22" t="s">
         <v>18</v>
@@ -1199,20 +1199,20 @@
     </row>
     <row r="29" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A29" s="11">
-        <v>46269</v>
+        <v>46270</v>
       </c>
       <c r="B29" s="12"/>
       <c r="C29" s="12" t="s">
         <v>19</v>
       </c>
       <c r="D29" s="13">
-        <v>238.41</v>
+        <v>241.74</v>
       </c>
       <c r="E29" s="13">
-        <v>205.13</v>
+        <v>207.65</v>
       </c>
       <c r="F29" s="13">
-        <v>215.13</v>
+        <v>217.65</v>
       </c>
       <c r="G29" s="13" t="s">
         <v>18</v>
@@ -1220,41 +1220,41 @@
     </row>
     <row r="30" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A30" s="7">
-        <v>46269</v>
+        <v>46270</v>
       </c>
       <c r="B30" s="8"/>
       <c r="C30" s="20" t="s">
         <v>20</v>
       </c>
       <c r="D30" s="10">
-        <v>237.6</v>
+        <v>238.51</v>
       </c>
       <c r="E30" s="22">
-        <v>205.07</v>
+        <v>207.6</v>
       </c>
       <c r="F30" s="22">
-        <v>215.07</v>
+        <v>217.6</v>
       </c>
       <c r="G30" s="22">
-        <v>202.97</v>
+        <v>205.5</v>
       </c>
     </row>
     <row r="31" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A31" s="11">
-        <v>46269</v>
+        <v>46270</v>
       </c>
       <c r="B31" s="12"/>
       <c r="C31" s="12" t="s">
         <v>21</v>
       </c>
       <c r="D31" s="13">
-        <v>237.15</v>
+        <v>240.48</v>
       </c>
       <c r="E31" s="13">
-        <v>206.32</v>
+        <v>208.87</v>
       </c>
       <c r="F31" s="13">
-        <v>216.32</v>
+        <v>218.87</v>
       </c>
       <c r="G31" s="13" t="s">
         <v>18</v>
@@ -1301,52 +1301,52 @@
     </row>
     <row r="35" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A35" s="7">
-        <v>46270</v>
+        <v>46273</v>
       </c>
       <c r="B35" s="8"/>
       <c r="C35" s="20" t="s">
         <v>23</v>
       </c>
       <c r="D35" s="10">
-        <v>234.96</v>
+        <v>237.39</v>
       </c>
       <c r="E35" s="10">
-        <v>199.85</v>
+        <v>201.89</v>
       </c>
       <c r="F35" s="10">
-        <v>208.85</v>
+        <v>210.89</v>
       </c>
       <c r="G35" s="17"/>
     </row>
     <row r="36" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A36" s="11">
-        <v>46269</v>
+        <v>46270</v>
       </c>
       <c r="B36" s="12"/>
       <c r="C36" s="12" t="s">
         <v>23</v>
       </c>
       <c r="D36" s="13">
-        <v>232.07</v>
+        <v>234.96</v>
       </c>
       <c r="E36" s="13">
-        <v>197.35</v>
+        <v>199.85</v>
       </c>
       <c r="F36" s="13">
-        <v>206.35</v>
+        <v>208.85</v>
       </c>
       <c r="G36" s="17"/>
     </row>
     <row r="37" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A37" s="7">
-        <v>46270</v>
+        <v>46273</v>
       </c>
       <c r="B37" s="8"/>
       <c r="C37" s="20" t="s">
         <v>24</v>
       </c>
       <c r="D37" s="10">
-        <v>250.58</v>
+        <v>253.01</v>
       </c>
       <c r="E37" s="10" t="s">
         <v>18</v>
@@ -1358,14 +1358,14 @@
     </row>
     <row r="38" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A38" s="11">
-        <v>46269</v>
+        <v>46270</v>
       </c>
       <c r="B38" s="12"/>
       <c r="C38" s="12" t="s">
         <v>24</v>
       </c>
       <c r="D38" s="13">
-        <v>247.69</v>
+        <v>250.58</v>
       </c>
       <c r="E38" s="13" t="s">
         <v>18</v>
@@ -1416,77 +1416,77 @@
     </row>
     <row r="42" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A42" s="7">
-        <v>46270</v>
+        <v>46273</v>
       </c>
       <c r="B42" s="8"/>
       <c r="C42" s="20" t="s">
         <v>26</v>
       </c>
       <c r="D42" s="10">
-        <v>243.34</v>
+        <v>245.83</v>
       </c>
       <c r="E42" s="10">
-        <v>206.05</v>
+        <v>208.08</v>
       </c>
       <c r="F42" s="10">
-        <v>216.05</v>
+        <v>218.08</v>
       </c>
       <c r="G42" s="17"/>
     </row>
     <row r="43" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A43" s="11">
-        <v>46270</v>
+        <v>46273</v>
       </c>
       <c r="B43" s="12"/>
       <c r="C43" s="21" t="s">
         <v>27</v>
       </c>
       <c r="D43" s="13">
-        <v>242.97</v>
+        <v>245.46</v>
       </c>
       <c r="E43" s="13">
-        <v>206.46</v>
+        <v>208.49</v>
       </c>
       <c r="F43" s="13">
-        <v>216.46</v>
+        <v>218.49</v>
       </c>
       <c r="G43" s="17"/>
     </row>
     <row r="44" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A44" s="7">
-        <v>46269</v>
+        <v>46270</v>
       </c>
       <c r="B44" s="8"/>
       <c r="C44" s="20" t="s">
         <v>26</v>
       </c>
       <c r="D44" s="10">
-        <v>239.98</v>
+        <v>243.34</v>
       </c>
       <c r="E44" s="10">
-        <v>203.58</v>
+        <v>206.05</v>
       </c>
       <c r="F44" s="10">
-        <v>213.58</v>
+        <v>216.05</v>
       </c>
       <c r="G44" s="17"/>
     </row>
     <row r="45" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A45" s="11">
-        <v>46269</v>
+        <v>46270</v>
       </c>
       <c r="B45" s="12"/>
       <c r="C45" s="21" t="s">
         <v>27</v>
       </c>
       <c r="D45" s="13">
-        <v>239.62</v>
+        <v>242.97</v>
       </c>
       <c r="E45" s="13">
-        <v>204</v>
+        <v>206.46</v>
       </c>
       <c r="F45" s="13">
-        <v>214</v>
+        <v>216.46</v>
       </c>
       <c r="G45" s="17"/>
     </row>
@@ -1531,77 +1531,77 @@
     </row>
     <row r="49" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A49" s="7">
-        <v>46270</v>
+        <v>46273</v>
       </c>
       <c r="B49" s="8"/>
       <c r="C49" s="20" t="s">
         <v>29</v>
       </c>
       <c r="D49" s="10">
-        <v>234.74</v>
+        <v>237.37</v>
       </c>
       <c r="E49" s="10">
-        <v>198.64</v>
+        <v>200.75</v>
       </c>
       <c r="F49" s="10">
-        <v>208.64</v>
+        <v>210.75</v>
       </c>
       <c r="G49" s="28"/>
     </row>
     <row r="50" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A50" s="11">
-        <v>46270</v>
+        <v>46273</v>
       </c>
       <c r="B50" s="12"/>
       <c r="C50" s="21" t="s">
         <v>30</v>
       </c>
       <c r="D50" s="13">
-        <v>232.99</v>
+        <v>235.61</v>
       </c>
       <c r="E50" s="13">
-        <v>198.58</v>
+        <v>200.68</v>
       </c>
       <c r="F50" s="13">
-        <v>208.58</v>
+        <v>210.68</v>
       </c>
       <c r="G50" s="28"/>
     </row>
     <row r="51" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A51" s="7">
-        <v>46269</v>
+        <v>46270</v>
       </c>
       <c r="B51" s="8"/>
       <c r="C51" s="20" t="s">
         <v>29</v>
       </c>
       <c r="D51" s="10">
-        <v>233.14</v>
+        <v>234.74</v>
       </c>
       <c r="E51" s="10">
-        <v>196.94</v>
+        <v>198.64</v>
       </c>
       <c r="F51" s="10">
-        <v>206.94</v>
+        <v>208.64</v>
       </c>
       <c r="G51" s="17"/>
     </row>
     <row r="52" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A52" s="11">
-        <v>46269</v>
+        <v>46270</v>
       </c>
       <c r="B52" s="12"/>
       <c r="C52" s="21" t="s">
         <v>30</v>
       </c>
       <c r="D52" s="13">
-        <v>231.4</v>
+        <v>232.99</v>
       </c>
       <c r="E52" s="13">
-        <v>196.88</v>
+        <v>198.58</v>
       </c>
       <c r="F52" s="13">
-        <v>206.88</v>
+        <v>208.58</v>
       </c>
       <c r="G52" s="17"/>
     </row>
@@ -1646,52 +1646,52 @@
     </row>
     <row r="56" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A56" s="7">
-        <v>46270</v>
+        <v>46273</v>
       </c>
       <c r="B56" s="8"/>
       <c r="C56" s="20" t="s">
         <v>32</v>
       </c>
       <c r="D56" s="10">
-        <v>253.32</v>
+        <v>255.73</v>
       </c>
       <c r="E56" s="10">
-        <v>218.9</v>
+        <v>221.21</v>
       </c>
       <c r="F56" s="10">
-        <v>228.9</v>
+        <v>231.21</v>
       </c>
       <c r="G56" s="17"/>
     </row>
     <row r="57" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A57" s="11">
-        <v>46270</v>
+        <v>46273</v>
       </c>
       <c r="B57" s="12"/>
       <c r="C57" s="21" t="s">
         <v>33</v>
       </c>
       <c r="D57" s="13">
-        <v>241.98</v>
+        <v>244.42</v>
       </c>
       <c r="E57" s="13">
-        <v>211.89</v>
+        <v>213.85</v>
       </c>
       <c r="F57" s="13">
-        <v>221.89</v>
+        <v>223.85</v>
       </c>
       <c r="G57" s="17"/>
     </row>
     <row r="58" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A58" s="7">
-        <v>46270</v>
+        <v>46273</v>
       </c>
       <c r="B58" s="8"/>
       <c r="C58" s="20" t="s">
         <v>34</v>
       </c>
       <c r="D58" s="10">
-        <v>243.12</v>
+        <v>245.57</v>
       </c>
       <c r="E58" s="10" t="s">
         <v>18</v>
@@ -1703,17 +1703,17 @@
     </row>
     <row r="59" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A59" s="11">
-        <v>46270</v>
+        <v>46273</v>
       </c>
       <c r="B59" s="12"/>
       <c r="C59" s="21" t="s">
         <v>35</v>
       </c>
       <c r="D59" s="13">
-        <v>240.39</v>
+        <v>242.73</v>
       </c>
       <c r="E59" s="13">
-        <v>206.28</v>
+        <v>208.24</v>
       </c>
       <c r="F59" s="13" t="s">
         <v>18</v>
@@ -1722,36 +1722,36 @@
     </row>
     <row r="60" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A60" s="7">
-        <v>46270</v>
+        <v>46273</v>
       </c>
       <c r="B60" s="8"/>
       <c r="C60" s="20" t="s">
         <v>36</v>
       </c>
       <c r="D60" s="10">
-        <v>236.2</v>
+        <v>238.55</v>
       </c>
       <c r="E60" s="10">
-        <v>202.21</v>
+        <v>204.17</v>
       </c>
       <c r="F60" s="10">
-        <v>212.21</v>
+        <v>214.17</v>
       </c>
       <c r="G60" s="17"/>
     </row>
     <row r="61" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A61" s="11">
-        <v>46270</v>
+        <v>46273</v>
       </c>
       <c r="B61" s="12"/>
       <c r="C61" s="21" t="s">
         <v>37</v>
       </c>
       <c r="D61" s="13">
-        <v>241.64</v>
+        <v>244</v>
       </c>
       <c r="E61" s="13">
-        <v>215.99</v>
+        <v>218.18</v>
       </c>
       <c r="F61" s="13" t="s">
         <v>18</v>
@@ -1760,52 +1760,52 @@
     </row>
     <row r="62" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A62" s="7">
-        <v>46269</v>
+        <v>46270</v>
       </c>
       <c r="B62" s="8"/>
       <c r="C62" s="20" t="s">
         <v>32</v>
       </c>
       <c r="D62" s="10">
-        <v>249.99</v>
+        <v>253.32</v>
       </c>
       <c r="E62" s="10">
-        <v>216.25</v>
+        <v>218.9</v>
       </c>
       <c r="F62" s="10">
-        <v>226.25</v>
+        <v>228.9</v>
       </c>
       <c r="G62" s="17"/>
     </row>
     <row r="63" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A63" s="11">
-        <v>46269</v>
+        <v>46270</v>
       </c>
       <c r="B63" s="12"/>
       <c r="C63" s="21" t="s">
         <v>33</v>
       </c>
       <c r="D63" s="13">
-        <v>238.65</v>
+        <v>241.98</v>
       </c>
       <c r="E63" s="13">
-        <v>209.43</v>
+        <v>211.89</v>
       </c>
       <c r="F63" s="13">
-        <v>219.43</v>
+        <v>221.89</v>
       </c>
       <c r="G63" s="17"/>
     </row>
     <row r="64" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A64" s="7">
-        <v>46269</v>
+        <v>46270</v>
       </c>
       <c r="B64" s="8"/>
       <c r="C64" s="20" t="s">
         <v>34</v>
       </c>
       <c r="D64" s="10">
-        <v>239.78</v>
+        <v>243.12</v>
       </c>
       <c r="E64" s="10" t="s">
         <v>18</v>
@@ -1817,17 +1817,17 @@
     </row>
     <row r="65" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A65" s="11">
-        <v>46269</v>
+        <v>46270</v>
       </c>
       <c r="B65" s="12"/>
       <c r="C65" s="21" t="s">
         <v>35</v>
       </c>
       <c r="D65" s="13">
-        <v>237.77</v>
+        <v>240.39</v>
       </c>
       <c r="E65" s="13">
-        <v>203.82</v>
+        <v>206.28</v>
       </c>
       <c r="F65" s="13" t="s">
         <v>18</v>
@@ -1835,35 +1835,35 @@
     </row>
     <row r="66" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A66" s="7">
-        <v>46269</v>
+        <v>46270</v>
       </c>
       <c r="B66" s="8"/>
       <c r="C66" s="20" t="s">
         <v>36</v>
       </c>
       <c r="D66" s="10">
-        <v>233.58</v>
+        <v>236.2</v>
       </c>
       <c r="E66" s="10">
-        <v>199.75</v>
+        <v>202.21</v>
       </c>
       <c r="F66" s="10">
-        <v>209.75</v>
+        <v>212.21</v>
       </c>
     </row>
     <row r="67" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A67" s="11">
-        <v>46269</v>
+        <v>46270</v>
       </c>
       <c r="B67" s="12"/>
       <c r="C67" s="21" t="s">
         <v>37</v>
       </c>
       <c r="D67" s="13">
-        <v>238.36</v>
+        <v>241.64</v>
       </c>
       <c r="E67" s="13">
-        <v>213.4</v>
+        <v>215.99</v>
       </c>
       <c r="F67" s="13" t="s">
         <v>18</v>
@@ -1891,6 +1891,15 @@
 </file>
 
 <file path=customXml/item1.xml><?xml version="1.0" encoding="utf-8"?>
+<?mso-contentType ?>
+<FormTemplates xmlns="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms">
+  <Display>DocumentLibraryForm</Display>
+  <Edit>DocumentLibraryForm</Edit>
+  <New>DocumentLibraryForm</New>
+</FormTemplates>
+</file>
+
+<file path=customXml/item2.xml><?xml version="1.0" encoding="utf-8"?>
 <p:properties xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls">
   <documentManagement>
     <lcf76f155ced4ddcb4097134ff3c332f xmlns="87276d81-85f4-4ef2-9e6e-55066304288f">
@@ -1899,15 +1908,6 @@
     <TaxCatchAll xmlns="b23b8984-eafa-4e79-985e-54f52f3da58e" xsi:nil="true"/>
   </documentManagement>
 </p:properties>
-</file>
-
-<file path=customXml/item2.xml><?xml version="1.0" encoding="utf-8"?>
-<?mso-contentType ?>
-<FormTemplates xmlns="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms">
-  <Display>DocumentLibraryForm</Display>
-  <Edit>DocumentLibraryForm</Edit>
-  <New>DocumentLibraryForm</New>
-</FormTemplates>
 </file>
 
 <file path=customXml/item3.xml><?xml version="1.0" encoding="utf-8"?>
@@ -2171,20 +2171,20 @@
 </file>
 
 <file path=customXml/itemProps1.xml><?xml version="1.0" encoding="utf-8"?>
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{F60519E9-FD90-4339-869C-BC2F85719BB8}">
+  <ds:schemaRefs>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms"/>
+  </ds:schemaRefs>
+</ds:datastoreItem>
+</file>
+
+<file path=customXml/itemProps2.xml><?xml version="1.0" encoding="utf-8"?>
 <ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{57A83D98-2BAE-4D83-823A-D31C464B620C}">
   <ds:schemaRefs>
     <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/properties"/>
     <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
     <ds:schemaRef ds:uri="87276d81-85f4-4ef2-9e6e-55066304288f"/>
     <ds:schemaRef ds:uri="b23b8984-eafa-4e79-985e-54f52f3da58e"/>
-  </ds:schemaRefs>
-</ds:datastoreItem>
-</file>
-
-<file path=customXml/itemProps2.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{F60519E9-FD90-4339-869C-BC2F85719BB8}">
-  <ds:schemaRefs>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms"/>
   </ds:schemaRefs>
 </ds:datastoreItem>
 </file>

</xml_diff>

<commit_message>
Tue Sep  8 06:02:13 UTC 2026
</commit_message>
<xml_diff>
--- a/bp.com-content-dam-bp-country-sites-en_au-australia-home-products-services-pricing-tgp-excel.xlsx
+++ b/bp.com-content-dam-bp-country-sites-en_au-australia-home-products-services-pricing-tgp-excel.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://bp365.sharepoint.com/sites/WholesalePricing/Shared Documents/B2C/TGP/Daily TGP/Web TGP/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="14_{12F0505E-791A-498B-ACA4-D4122E8588D1}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="14_{5435E086-D439-475A-A6D0-16EF83782B8F}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-28920" yWindow="-60" windowWidth="29040" windowHeight="15720" xr2:uid="{1B412EEF-F96D-4DF4-A4E9-C7F0F183C2FB}"/>
   </bookViews>
@@ -808,128 +808,128 @@
     </row>
     <row r="8" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A8" s="7">
-        <v>46273</v>
+        <v>46274</v>
       </c>
       <c r="B8" s="8"/>
       <c r="C8" s="9" t="s">
         <v>10</v>
       </c>
       <c r="D8" s="10">
-        <v>242.28</v>
+        <v>244.01</v>
       </c>
       <c r="E8" s="10">
-        <v>205.55</v>
+        <v>207.38</v>
       </c>
       <c r="F8" s="10">
-        <v>215.55</v>
+        <v>217.38</v>
       </c>
       <c r="G8" s="10">
-        <v>205.52</v>
+        <v>207.34</v>
       </c>
     </row>
     <row r="9" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A9" s="11">
-        <v>46273</v>
+        <v>46274</v>
       </c>
       <c r="B9" s="12"/>
       <c r="C9" s="12" t="s">
         <v>11</v>
       </c>
       <c r="D9" s="13">
-        <v>242.28</v>
+        <v>244.01</v>
       </c>
       <c r="E9" s="13">
-        <v>205.55</v>
+        <v>207.38</v>
       </c>
       <c r="F9" s="13">
-        <v>215.55</v>
+        <v>217.38</v>
       </c>
       <c r="G9" s="13">
-        <v>205.52</v>
+        <v>207.34</v>
       </c>
     </row>
     <row r="10" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A10" s="7">
-        <v>46273</v>
+        <v>46274</v>
       </c>
       <c r="B10" s="8"/>
       <c r="C10" s="9" t="s">
         <v>12</v>
       </c>
       <c r="D10" s="10">
-        <v>238.87</v>
+        <v>240.77</v>
       </c>
       <c r="E10" s="10">
-        <v>202.94</v>
+        <v>204.92</v>
       </c>
       <c r="F10" s="10">
-        <v>212.94</v>
+        <v>214.92</v>
       </c>
       <c r="G10" s="10">
-        <v>203.36</v>
+        <v>205.34</v>
       </c>
     </row>
     <row r="11" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A11" s="11">
-        <v>46270</v>
+        <v>46273</v>
       </c>
       <c r="B11" s="12"/>
       <c r="C11" s="12" t="s">
         <v>10</v>
       </c>
       <c r="D11" s="13">
-        <v>239.99</v>
+        <v>242.28</v>
       </c>
       <c r="E11" s="13">
-        <v>203.64</v>
+        <v>205.55</v>
       </c>
       <c r="F11" s="13">
-        <v>213.64</v>
+        <v>215.55</v>
       </c>
       <c r="G11" s="13">
-        <v>203.6</v>
+        <v>205.52</v>
       </c>
     </row>
     <row r="12" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A12" s="7">
-        <v>46270</v>
+        <v>46273</v>
       </c>
       <c r="B12" s="8"/>
       <c r="C12" s="9" t="s">
         <v>11</v>
       </c>
       <c r="D12" s="10">
-        <v>239.99</v>
+        <v>242.28</v>
       </c>
       <c r="E12" s="10">
-        <v>203.64</v>
+        <v>205.55</v>
       </c>
       <c r="F12" s="10">
-        <v>213.64</v>
+        <v>215.55</v>
       </c>
       <c r="G12" s="10">
-        <v>203.6</v>
+        <v>205.52</v>
       </c>
     </row>
     <row r="13" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A13" s="11">
-        <v>46270</v>
+        <v>46273</v>
       </c>
       <c r="B13" s="12"/>
       <c r="C13" s="12" t="s">
         <v>12</v>
       </c>
       <c r="D13" s="13">
-        <v>236.44</v>
+        <v>238.87</v>
       </c>
       <c r="E13" s="13">
-        <v>200.9</v>
+        <v>202.94</v>
       </c>
       <c r="F13" s="13">
-        <v>210.9</v>
+        <v>212.94</v>
       </c>
       <c r="G13" s="13">
-        <v>201.32</v>
+        <v>203.36</v>
       </c>
     </row>
     <row r="14" spans="1:7" x14ac:dyDescent="0.25">
@@ -973,39 +973,39 @@
     </row>
     <row r="17" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A17" s="7">
-        <v>46273</v>
+        <v>46274</v>
       </c>
       <c r="B17" s="8"/>
       <c r="C17" s="20" t="s">
         <v>14</v>
       </c>
       <c r="D17" s="10">
-        <v>244.37</v>
+        <v>246.16</v>
       </c>
       <c r="E17" s="10">
-        <v>207.64</v>
+        <v>209.53</v>
       </c>
       <c r="F17" s="10">
-        <v>217.64</v>
+        <v>219.53</v>
       </c>
       <c r="G17" s="17"/>
     </row>
     <row r="18" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A18" s="11">
-        <v>46270</v>
+        <v>46273</v>
       </c>
       <c r="B18" s="12"/>
       <c r="C18" s="12" t="s">
         <v>14</v>
       </c>
       <c r="D18" s="13">
-        <v>242</v>
+        <v>244.37</v>
       </c>
       <c r="E18" s="13">
-        <v>205.66</v>
+        <v>207.64</v>
       </c>
       <c r="F18" s="13">
-        <v>215.66</v>
+        <v>217.64</v>
       </c>
       <c r="G18" s="17"/>
     </row>
@@ -1052,41 +1052,41 @@
     </row>
     <row r="22" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A22" s="7">
-        <v>46273</v>
+        <v>46274</v>
       </c>
       <c r="B22" s="8"/>
       <c r="C22" s="20" t="s">
         <v>16</v>
       </c>
       <c r="D22" s="10">
-        <v>243.42</v>
+        <v>245.15</v>
       </c>
       <c r="E22" s="10">
-        <v>206.25</v>
+        <v>208.07</v>
       </c>
       <c r="F22" s="10">
-        <v>215.85</v>
+        <v>217.67</v>
       </c>
       <c r="G22" s="10">
-        <v>204.97</v>
+        <v>206.79</v>
       </c>
     </row>
     <row r="23" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A23" s="11">
-        <v>46273</v>
+        <v>46274</v>
       </c>
       <c r="B23" s="12"/>
       <c r="C23" s="21" t="s">
         <v>17</v>
       </c>
       <c r="D23" s="13">
-        <v>243.58</v>
+        <v>245.49</v>
       </c>
       <c r="E23" s="13">
-        <v>210.39</v>
+        <v>212.42</v>
       </c>
       <c r="F23" s="13">
-        <v>220.39</v>
+        <v>222.42</v>
       </c>
       <c r="G23" s="13" t="s">
         <v>18</v>
@@ -1094,20 +1094,20 @@
     </row>
     <row r="24" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A24" s="7">
-        <v>46273</v>
+        <v>46274</v>
       </c>
       <c r="B24" s="8"/>
       <c r="C24" s="20" t="s">
         <v>19</v>
       </c>
       <c r="D24" s="10">
-        <v>244.17</v>
+        <v>246.07</v>
       </c>
       <c r="E24" s="10">
-        <v>209.71</v>
+        <v>211.73</v>
       </c>
       <c r="F24" s="10">
-        <v>219.71</v>
+        <v>221.73</v>
       </c>
       <c r="G24" s="10" t="s">
         <v>18</v>
@@ -1115,41 +1115,41 @@
     </row>
     <row r="25" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A25" s="11">
-        <v>46273</v>
+        <v>46274</v>
       </c>
       <c r="B25" s="12"/>
       <c r="C25" s="21" t="s">
         <v>20</v>
       </c>
       <c r="D25" s="13">
-        <v>240.94</v>
+        <v>242.85</v>
       </c>
       <c r="E25" s="13">
-        <v>209.68</v>
+        <v>211.71</v>
       </c>
       <c r="F25" s="13">
-        <v>219.68</v>
+        <v>221.71</v>
       </c>
       <c r="G25" s="13">
-        <v>207.57</v>
+        <v>209.61</v>
       </c>
     </row>
     <row r="26" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A26" s="7">
-        <v>46273</v>
+        <v>46274</v>
       </c>
       <c r="B26" s="8"/>
       <c r="C26" s="20" t="s">
         <v>21</v>
       </c>
       <c r="D26" s="10">
-        <v>242.9</v>
+        <v>244.77</v>
       </c>
       <c r="E26" s="10">
-        <v>210.96</v>
+        <v>213.01</v>
       </c>
       <c r="F26" s="10">
-        <v>220.96</v>
+        <v>223.01</v>
       </c>
       <c r="G26" s="10" t="s">
         <v>18</v>
@@ -1157,41 +1157,41 @@
     </row>
     <row r="27" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A27" s="11">
-        <v>46270</v>
+        <v>46273</v>
       </c>
       <c r="B27" s="12"/>
       <c r="C27" s="12" t="s">
         <v>16</v>
       </c>
       <c r="D27" s="13">
-        <v>241.13</v>
+        <v>243.42</v>
       </c>
       <c r="E27" s="13">
-        <v>204.34</v>
+        <v>206.25</v>
       </c>
       <c r="F27" s="13">
-        <v>213.94</v>
+        <v>215.85</v>
       </c>
       <c r="G27" s="13">
-        <v>203.05</v>
+        <v>204.97</v>
       </c>
     </row>
     <row r="28" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A28" s="7">
-        <v>46270</v>
+        <v>46273</v>
       </c>
       <c r="B28" s="8"/>
       <c r="C28" s="20" t="s">
         <v>17</v>
       </c>
       <c r="D28" s="10">
-        <v>241.13</v>
+        <v>243.58</v>
       </c>
       <c r="E28" s="22">
-        <v>208.32</v>
+        <v>210.39</v>
       </c>
       <c r="F28" s="22">
-        <v>218.32</v>
+        <v>220.39</v>
       </c>
       <c r="G28" s="22" t="s">
         <v>18</v>
@@ -1199,20 +1199,20 @@
     </row>
     <row r="29" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A29" s="11">
-        <v>46270</v>
+        <v>46273</v>
       </c>
       <c r="B29" s="12"/>
       <c r="C29" s="12" t="s">
         <v>19</v>
       </c>
       <c r="D29" s="13">
-        <v>241.74</v>
+        <v>244.17</v>
       </c>
       <c r="E29" s="13">
-        <v>207.65</v>
+        <v>209.71</v>
       </c>
       <c r="F29" s="13">
-        <v>217.65</v>
+        <v>219.71</v>
       </c>
       <c r="G29" s="13" t="s">
         <v>18</v>
@@ -1220,41 +1220,41 @@
     </row>
     <row r="30" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A30" s="7">
-        <v>46270</v>
+        <v>46273</v>
       </c>
       <c r="B30" s="8"/>
       <c r="C30" s="20" t="s">
         <v>20</v>
       </c>
       <c r="D30" s="10">
-        <v>238.51</v>
+        <v>240.94</v>
       </c>
       <c r="E30" s="22">
-        <v>207.6</v>
+        <v>209.68</v>
       </c>
       <c r="F30" s="22">
-        <v>217.6</v>
+        <v>219.68</v>
       </c>
       <c r="G30" s="22">
-        <v>205.5</v>
+        <v>207.57</v>
       </c>
     </row>
     <row r="31" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A31" s="11">
-        <v>46270</v>
+        <v>46273</v>
       </c>
       <c r="B31" s="12"/>
       <c r="C31" s="12" t="s">
         <v>21</v>
       </c>
       <c r="D31" s="13">
-        <v>240.48</v>
+        <v>242.9</v>
       </c>
       <c r="E31" s="13">
-        <v>208.87</v>
+        <v>210.96</v>
       </c>
       <c r="F31" s="13">
-        <v>218.87</v>
+        <v>220.96</v>
       </c>
       <c r="G31" s="13" t="s">
         <v>18</v>
@@ -1301,52 +1301,52 @@
     </row>
     <row r="35" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A35" s="7">
-        <v>46273</v>
+        <v>46274</v>
       </c>
       <c r="B35" s="8"/>
       <c r="C35" s="20" t="s">
         <v>23</v>
       </c>
       <c r="D35" s="10">
-        <v>237.39</v>
+        <v>239.3</v>
       </c>
       <c r="E35" s="10">
-        <v>201.89</v>
+        <v>203.88</v>
       </c>
       <c r="F35" s="10">
-        <v>210.89</v>
+        <v>212.88</v>
       </c>
       <c r="G35" s="17"/>
     </row>
     <row r="36" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A36" s="11">
-        <v>46270</v>
+        <v>46273</v>
       </c>
       <c r="B36" s="12"/>
       <c r="C36" s="12" t="s">
         <v>23</v>
       </c>
       <c r="D36" s="13">
-        <v>234.96</v>
+        <v>237.39</v>
       </c>
       <c r="E36" s="13">
-        <v>199.85</v>
+        <v>201.89</v>
       </c>
       <c r="F36" s="13">
-        <v>208.85</v>
+        <v>210.89</v>
       </c>
       <c r="G36" s="17"/>
     </row>
     <row r="37" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A37" s="7">
-        <v>46273</v>
+        <v>46274</v>
       </c>
       <c r="B37" s="8"/>
       <c r="C37" s="20" t="s">
         <v>24</v>
       </c>
       <c r="D37" s="10">
-        <v>253.01</v>
+        <v>254.92</v>
       </c>
       <c r="E37" s="10" t="s">
         <v>18</v>
@@ -1358,14 +1358,14 @@
     </row>
     <row r="38" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A38" s="11">
-        <v>46270</v>
+        <v>46273</v>
       </c>
       <c r="B38" s="12"/>
       <c r="C38" s="12" t="s">
         <v>24</v>
       </c>
       <c r="D38" s="13">
-        <v>250.58</v>
+        <v>253.01</v>
       </c>
       <c r="E38" s="13" t="s">
         <v>18</v>
@@ -1416,77 +1416,77 @@
     </row>
     <row r="42" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A42" s="7">
-        <v>46273</v>
+        <v>46274</v>
       </c>
       <c r="B42" s="8"/>
       <c r="C42" s="20" t="s">
         <v>26</v>
       </c>
       <c r="D42" s="10">
-        <v>245.83</v>
+        <v>247.81</v>
       </c>
       <c r="E42" s="10">
-        <v>208.08</v>
+        <v>210.09</v>
       </c>
       <c r="F42" s="10">
-        <v>218.08</v>
+        <v>220.09</v>
       </c>
       <c r="G42" s="17"/>
     </row>
     <row r="43" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A43" s="11">
-        <v>46273</v>
+        <v>46274</v>
       </c>
       <c r="B43" s="12"/>
       <c r="C43" s="21" t="s">
         <v>27</v>
       </c>
       <c r="D43" s="13">
-        <v>245.46</v>
+        <v>247.44</v>
       </c>
       <c r="E43" s="13">
-        <v>208.49</v>
+        <v>210.5</v>
       </c>
       <c r="F43" s="13">
-        <v>218.49</v>
+        <v>220.5</v>
       </c>
       <c r="G43" s="17"/>
     </row>
     <row r="44" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A44" s="7">
-        <v>46270</v>
+        <v>46273</v>
       </c>
       <c r="B44" s="8"/>
       <c r="C44" s="20" t="s">
         <v>26</v>
       </c>
       <c r="D44" s="10">
-        <v>243.34</v>
+        <v>245.83</v>
       </c>
       <c r="E44" s="10">
-        <v>206.05</v>
+        <v>208.08</v>
       </c>
       <c r="F44" s="10">
-        <v>216.05</v>
+        <v>218.08</v>
       </c>
       <c r="G44" s="17"/>
     </row>
     <row r="45" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A45" s="11">
-        <v>46270</v>
+        <v>46273</v>
       </c>
       <c r="B45" s="12"/>
       <c r="C45" s="21" t="s">
         <v>27</v>
       </c>
       <c r="D45" s="13">
-        <v>242.97</v>
+        <v>245.46</v>
       </c>
       <c r="E45" s="13">
-        <v>206.46</v>
+        <v>208.49</v>
       </c>
       <c r="F45" s="13">
-        <v>216.46</v>
+        <v>218.49</v>
       </c>
       <c r="G45" s="17"/>
     </row>
@@ -1531,77 +1531,77 @@
     </row>
     <row r="49" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A49" s="7">
-        <v>46273</v>
+        <v>46274</v>
       </c>
       <c r="B49" s="8"/>
       <c r="C49" s="20" t="s">
         <v>29</v>
       </c>
       <c r="D49" s="10">
-        <v>237.37</v>
+        <v>239.82</v>
       </c>
       <c r="E49" s="10">
-        <v>200.75</v>
+        <v>203.03</v>
       </c>
       <c r="F49" s="10">
-        <v>210.75</v>
+        <v>213.03</v>
       </c>
       <c r="G49" s="28"/>
     </row>
     <row r="50" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A50" s="11">
-        <v>46273</v>
+        <v>46274</v>
       </c>
       <c r="B50" s="12"/>
       <c r="C50" s="21" t="s">
         <v>30</v>
       </c>
       <c r="D50" s="13">
-        <v>235.61</v>
+        <v>238.02</v>
       </c>
       <c r="E50" s="13">
-        <v>200.68</v>
+        <v>202.96</v>
       </c>
       <c r="F50" s="13">
-        <v>210.68</v>
+        <v>212.96</v>
       </c>
       <c r="G50" s="28"/>
     </row>
     <row r="51" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A51" s="7">
-        <v>46270</v>
+        <v>46273</v>
       </c>
       <c r="B51" s="8"/>
       <c r="C51" s="20" t="s">
         <v>29</v>
       </c>
       <c r="D51" s="10">
-        <v>234.74</v>
+        <v>237.37</v>
       </c>
       <c r="E51" s="10">
-        <v>198.64</v>
+        <v>200.75</v>
       </c>
       <c r="F51" s="10">
-        <v>208.64</v>
+        <v>210.75</v>
       </c>
       <c r="G51" s="17"/>
     </row>
     <row r="52" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A52" s="11">
-        <v>46270</v>
+        <v>46273</v>
       </c>
       <c r="B52" s="12"/>
       <c r="C52" s="21" t="s">
         <v>30</v>
       </c>
       <c r="D52" s="13">
-        <v>232.99</v>
+        <v>235.61</v>
       </c>
       <c r="E52" s="13">
-        <v>198.58</v>
+        <v>200.68</v>
       </c>
       <c r="F52" s="13">
-        <v>208.58</v>
+        <v>210.68</v>
       </c>
       <c r="G52" s="17"/>
     </row>
@@ -1646,52 +1646,52 @@
     </row>
     <row r="56" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A56" s="7">
-        <v>46273</v>
+        <v>46274</v>
       </c>
       <c r="B56" s="8"/>
       <c r="C56" s="20" t="s">
         <v>32</v>
       </c>
       <c r="D56" s="10">
-        <v>255.73</v>
+        <v>257.60000000000002</v>
       </c>
       <c r="E56" s="10">
-        <v>221.21</v>
+        <v>223.66</v>
       </c>
       <c r="F56" s="10">
-        <v>231.21</v>
+        <v>233.66</v>
       </c>
       <c r="G56" s="17"/>
     </row>
     <row r="57" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A57" s="11">
-        <v>46273</v>
+        <v>46274</v>
       </c>
       <c r="B57" s="12"/>
       <c r="C57" s="21" t="s">
         <v>33</v>
       </c>
       <c r="D57" s="13">
-        <v>244.42</v>
+        <v>246.33</v>
       </c>
       <c r="E57" s="13">
-        <v>213.85</v>
+        <v>215.16</v>
       </c>
       <c r="F57" s="13">
-        <v>223.85</v>
+        <v>225.16</v>
       </c>
       <c r="G57" s="17"/>
     </row>
     <row r="58" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A58" s="7">
-        <v>46273</v>
+        <v>46274</v>
       </c>
       <c r="B58" s="8"/>
       <c r="C58" s="20" t="s">
         <v>34</v>
       </c>
       <c r="D58" s="10">
-        <v>245.57</v>
+        <v>247.49</v>
       </c>
       <c r="E58" s="10" t="s">
         <v>18</v>
@@ -1703,17 +1703,17 @@
     </row>
     <row r="59" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A59" s="11">
-        <v>46273</v>
+        <v>46274</v>
       </c>
       <c r="B59" s="12"/>
       <c r="C59" s="21" t="s">
         <v>35</v>
       </c>
       <c r="D59" s="13">
-        <v>242.73</v>
+        <v>244.5</v>
       </c>
       <c r="E59" s="13">
-        <v>208.24</v>
+        <v>209.55</v>
       </c>
       <c r="F59" s="13" t="s">
         <v>18</v>
@@ -1722,36 +1722,36 @@
     </row>
     <row r="60" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A60" s="7">
-        <v>46273</v>
+        <v>46274</v>
       </c>
       <c r="B60" s="8"/>
       <c r="C60" s="20" t="s">
         <v>36</v>
       </c>
       <c r="D60" s="10">
-        <v>238.55</v>
+        <v>240.32</v>
       </c>
       <c r="E60" s="10">
-        <v>204.17</v>
+        <v>205.48</v>
       </c>
       <c r="F60" s="10">
-        <v>214.17</v>
+        <v>215.48</v>
       </c>
       <c r="G60" s="17"/>
     </row>
     <row r="61" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A61" s="11">
-        <v>46273</v>
+        <v>46274</v>
       </c>
       <c r="B61" s="12"/>
       <c r="C61" s="21" t="s">
         <v>37</v>
       </c>
       <c r="D61" s="13">
-        <v>244</v>
+        <v>245.77</v>
       </c>
       <c r="E61" s="13">
-        <v>218.18</v>
+        <v>220.43</v>
       </c>
       <c r="F61" s="13" t="s">
         <v>18</v>
@@ -1760,52 +1760,52 @@
     </row>
     <row r="62" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A62" s="7">
-        <v>46270</v>
+        <v>46273</v>
       </c>
       <c r="B62" s="8"/>
       <c r="C62" s="20" t="s">
         <v>32</v>
       </c>
       <c r="D62" s="10">
-        <v>253.32</v>
+        <v>255.73</v>
       </c>
       <c r="E62" s="10">
-        <v>218.9</v>
+        <v>221.21</v>
       </c>
       <c r="F62" s="10">
-        <v>228.9</v>
+        <v>231.21</v>
       </c>
       <c r="G62" s="17"/>
     </row>
     <row r="63" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A63" s="11">
-        <v>46270</v>
+        <v>46273</v>
       </c>
       <c r="B63" s="12"/>
       <c r="C63" s="21" t="s">
         <v>33</v>
       </c>
       <c r="D63" s="13">
-        <v>241.98</v>
+        <v>244.42</v>
       </c>
       <c r="E63" s="13">
-        <v>211.89</v>
+        <v>213.85</v>
       </c>
       <c r="F63" s="13">
-        <v>221.89</v>
+        <v>223.85</v>
       </c>
       <c r="G63" s="17"/>
     </row>
     <row r="64" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A64" s="7">
-        <v>46270</v>
+        <v>46273</v>
       </c>
       <c r="B64" s="8"/>
       <c r="C64" s="20" t="s">
         <v>34</v>
       </c>
       <c r="D64" s="10">
-        <v>243.12</v>
+        <v>245.57</v>
       </c>
       <c r="E64" s="10" t="s">
         <v>18</v>
@@ -1817,17 +1817,17 @@
     </row>
     <row r="65" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A65" s="11">
-        <v>46270</v>
+        <v>46273</v>
       </c>
       <c r="B65" s="12"/>
       <c r="C65" s="21" t="s">
         <v>35</v>
       </c>
       <c r="D65" s="13">
-        <v>240.39</v>
+        <v>242.73</v>
       </c>
       <c r="E65" s="13">
-        <v>206.28</v>
+        <v>208.24</v>
       </c>
       <c r="F65" s="13" t="s">
         <v>18</v>
@@ -1835,35 +1835,35 @@
     </row>
     <row r="66" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A66" s="7">
-        <v>46270</v>
+        <v>46273</v>
       </c>
       <c r="B66" s="8"/>
       <c r="C66" s="20" t="s">
         <v>36</v>
       </c>
       <c r="D66" s="10">
-        <v>236.2</v>
+        <v>238.55</v>
       </c>
       <c r="E66" s="10">
-        <v>202.21</v>
+        <v>204.17</v>
       </c>
       <c r="F66" s="10">
-        <v>212.21</v>
+        <v>214.17</v>
       </c>
     </row>
     <row r="67" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A67" s="11">
-        <v>46270</v>
+        <v>46273</v>
       </c>
       <c r="B67" s="12"/>
       <c r="C67" s="21" t="s">
         <v>37</v>
       </c>
       <c r="D67" s="13">
-        <v>241.64</v>
+        <v>244</v>
       </c>
       <c r="E67" s="13">
-        <v>215.99</v>
+        <v>218.18</v>
       </c>
       <c r="F67" s="13" t="s">
         <v>18</v>
@@ -1891,26 +1891,6 @@
 </file>
 
 <file path=customXml/item1.xml><?xml version="1.0" encoding="utf-8"?>
-<?mso-contentType ?>
-<FormTemplates xmlns="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms">
-  <Display>DocumentLibraryForm</Display>
-  <Edit>DocumentLibraryForm</Edit>
-  <New>DocumentLibraryForm</New>
-</FormTemplates>
-</file>
-
-<file path=customXml/item2.xml><?xml version="1.0" encoding="utf-8"?>
-<p:properties xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls">
-  <documentManagement>
-    <lcf76f155ced4ddcb4097134ff3c332f xmlns="87276d81-85f4-4ef2-9e6e-55066304288f">
-      <Terms xmlns="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
-    </lcf76f155ced4ddcb4097134ff3c332f>
-    <TaxCatchAll xmlns="b23b8984-eafa-4e79-985e-54f52f3da58e" xsi:nil="true"/>
-  </documentManagement>
-</p:properties>
-</file>
-
-<file path=customXml/item3.xml><?xml version="1.0" encoding="utf-8"?>
 <ct:contentTypeSchema xmlns:ct="http://schemas.microsoft.com/office/2006/metadata/contentType" xmlns:ma="http://schemas.microsoft.com/office/2006/metadata/properties/metaAttributes" ct:_="" ma:_="" ma:contentTypeName="Document" ma:contentTypeID="0x010100D3632DF5622958439304627C030B0427" ma:contentTypeVersion="18" ma:contentTypeDescription="Create a new document." ma:contentTypeScope="" ma:versionID="8c2ecbce386d6bac497f8eb2d8f0fb7a">
   <xsd:schema xmlns:xsd="http://www.w3.org/2001/XMLSchema" xmlns:xs="http://www.w3.org/2001/XMLSchema" xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:ns2="87276d81-85f4-4ef2-9e6e-55066304288f" xmlns:ns3="39e1dda6-d1d8-4c88-a3b9-f1abc1284bad" xmlns:ns4="b23b8984-eafa-4e79-985e-54f52f3da58e" targetNamespace="http://schemas.microsoft.com/office/2006/metadata/properties" ma:root="true" ma:fieldsID="4cfd0c2f651c1ce156ad4fcb44ea61dd" ns2:_="" ns3:_="" ns4:_="">
     <xsd:import namespace="87276d81-85f4-4ef2-9e6e-55066304288f"/>
@@ -2170,26 +2150,27 @@
 </ct:contentTypeSchema>
 </file>
 
-<file path=customXml/itemProps1.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{F60519E9-FD90-4339-869C-BC2F85719BB8}">
-  <ds:schemaRefs>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms"/>
-  </ds:schemaRefs>
-</ds:datastoreItem>
+<file path=customXml/item2.xml><?xml version="1.0" encoding="utf-8"?>
+<?mso-contentType ?>
+<FormTemplates xmlns="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms">
+  <Display>DocumentLibraryForm</Display>
+  <Edit>DocumentLibraryForm</Edit>
+  <New>DocumentLibraryForm</New>
+</FormTemplates>
 </file>
 
-<file path=customXml/itemProps2.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{57A83D98-2BAE-4D83-823A-D31C464B620C}">
-  <ds:schemaRefs>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/properties"/>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
-    <ds:schemaRef ds:uri="87276d81-85f4-4ef2-9e6e-55066304288f"/>
-    <ds:schemaRef ds:uri="b23b8984-eafa-4e79-985e-54f52f3da58e"/>
-  </ds:schemaRefs>
-</ds:datastoreItem>
+<file path=customXml/item3.xml><?xml version="1.0" encoding="utf-8"?>
+<p:properties xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls">
+  <documentManagement>
+    <lcf76f155ced4ddcb4097134ff3c332f xmlns="87276d81-85f4-4ef2-9e6e-55066304288f">
+      <Terms xmlns="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
+    </lcf76f155ced4ddcb4097134ff3c332f>
+    <TaxCatchAll xmlns="b23b8984-eafa-4e79-985e-54f52f3da58e" xsi:nil="true"/>
+  </documentManagement>
+</p:properties>
 </file>
 
-<file path=customXml/itemProps3.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=customXml/itemProps1.xml><?xml version="1.0" encoding="utf-8"?>
 <ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{B44E1863-2778-41F9-ACBA-48420F931671}">
   <ds:schemaRefs>
     <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/contentType"/>
@@ -2209,6 +2190,25 @@
 </ds:datastoreItem>
 </file>
 
+<file path=customXml/itemProps2.xml><?xml version="1.0" encoding="utf-8"?>
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{F60519E9-FD90-4339-869C-BC2F85719BB8}">
+  <ds:schemaRefs>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms"/>
+  </ds:schemaRefs>
+</ds:datastoreItem>
+</file>
+
+<file path=customXml/itemProps3.xml><?xml version="1.0" encoding="utf-8"?>
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{57A83D98-2BAE-4D83-823A-D31C464B620C}">
+  <ds:schemaRefs>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/properties"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
+    <ds:schemaRef ds:uri="87276d81-85f4-4ef2-9e6e-55066304288f"/>
+    <ds:schemaRef ds:uri="b23b8984-eafa-4e79-985e-54f52f3da58e"/>
+  </ds:schemaRefs>
+</ds:datastoreItem>
+</file>
+
 <file path=docMetadata/LabelInfo.xml><?xml version="1.0" encoding="utf-8"?>
 <clbl:labelList xmlns:clbl="http://schemas.microsoft.com/office/2020/mipLabelMetadata">
   <clbl:label id="{569bf4a9-87bd-4dbf-a36c-1db5158e5def}" enabled="1" method="Privileged" siteId="{ea80952e-a476-42d4-aaf4-5457852b0f7e}" removed="0"/>

</xml_diff>

<commit_message>
Wed Sep  9 06:06:33 UTC 2026
</commit_message>
<xml_diff>
--- a/bp.com-content-dam-bp-country-sites-en_au-australia-home-products-services-pricing-tgp-excel.xlsx
+++ b/bp.com-content-dam-bp-country-sites-en_au-australia-home-products-services-pricing-tgp-excel.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://bp365.sharepoint.com/sites/WholesalePricing/Shared Documents/B2C/TGP/Daily TGP/Web TGP/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="14_{5435E086-D439-475A-A6D0-16EF83782B8F}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="14_{C226758B-06B3-482F-9671-3AE14209B915}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-28920" yWindow="-60" windowWidth="29040" windowHeight="15720" xr2:uid="{1B412EEF-F96D-4DF4-A4E9-C7F0F183C2FB}"/>
   </bookViews>
@@ -808,128 +808,128 @@
     </row>
     <row r="8" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A8" s="7">
-        <v>46274</v>
+        <v>46275</v>
       </c>
       <c r="B8" s="8"/>
       <c r="C8" s="9" t="s">
         <v>10</v>
       </c>
       <c r="D8" s="10">
-        <v>244.01</v>
+        <v>246.08</v>
       </c>
       <c r="E8" s="10">
-        <v>207.38</v>
+        <v>210.46</v>
       </c>
       <c r="F8" s="10">
-        <v>217.38</v>
+        <v>220.46</v>
       </c>
       <c r="G8" s="10">
-        <v>207.34</v>
+        <v>210.43</v>
       </c>
     </row>
     <row r="9" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A9" s="11">
-        <v>46274</v>
+        <v>46275</v>
       </c>
       <c r="B9" s="12"/>
       <c r="C9" s="12" t="s">
         <v>11</v>
       </c>
       <c r="D9" s="13">
-        <v>244.01</v>
+        <v>246.08</v>
       </c>
       <c r="E9" s="13">
-        <v>207.38</v>
+        <v>210.46</v>
       </c>
       <c r="F9" s="13">
-        <v>217.38</v>
+        <v>220.46</v>
       </c>
       <c r="G9" s="13">
-        <v>207.34</v>
+        <v>210.43</v>
       </c>
     </row>
     <row r="10" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A10" s="7">
-        <v>46274</v>
+        <v>46275</v>
       </c>
       <c r="B10" s="8"/>
       <c r="C10" s="9" t="s">
         <v>12</v>
       </c>
       <c r="D10" s="10">
-        <v>240.77</v>
+        <v>242.55</v>
       </c>
       <c r="E10" s="10">
-        <v>204.92</v>
+        <v>207.74</v>
       </c>
       <c r="F10" s="10">
-        <v>214.92</v>
+        <v>217.75</v>
       </c>
       <c r="G10" s="10">
-        <v>205.34</v>
+        <v>208.16</v>
       </c>
     </row>
     <row r="11" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A11" s="11">
-        <v>46273</v>
+        <v>46274</v>
       </c>
       <c r="B11" s="12"/>
       <c r="C11" s="12" t="s">
         <v>10</v>
       </c>
       <c r="D11" s="13">
-        <v>242.28</v>
+        <v>244.01</v>
       </c>
       <c r="E11" s="13">
-        <v>205.55</v>
+        <v>207.38</v>
       </c>
       <c r="F11" s="13">
-        <v>215.55</v>
+        <v>217.38</v>
       </c>
       <c r="G11" s="13">
-        <v>205.52</v>
+        <v>207.34</v>
       </c>
     </row>
     <row r="12" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A12" s="7">
-        <v>46273</v>
+        <v>46274</v>
       </c>
       <c r="B12" s="8"/>
       <c r="C12" s="9" t="s">
         <v>11</v>
       </c>
       <c r="D12" s="10">
-        <v>242.28</v>
+        <v>244.01</v>
       </c>
       <c r="E12" s="10">
-        <v>205.55</v>
+        <v>207.38</v>
       </c>
       <c r="F12" s="10">
-        <v>215.55</v>
+        <v>217.38</v>
       </c>
       <c r="G12" s="10">
-        <v>205.52</v>
+        <v>207.34</v>
       </c>
     </row>
     <row r="13" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A13" s="11">
-        <v>46273</v>
+        <v>46274</v>
       </c>
       <c r="B13" s="12"/>
       <c r="C13" s="12" t="s">
         <v>12</v>
       </c>
       <c r="D13" s="13">
-        <v>238.87</v>
+        <v>240.77</v>
       </c>
       <c r="E13" s="13">
-        <v>202.94</v>
+        <v>204.92</v>
       </c>
       <c r="F13" s="13">
-        <v>212.94</v>
+        <v>214.92</v>
       </c>
       <c r="G13" s="13">
-        <v>203.36</v>
+        <v>205.34</v>
       </c>
     </row>
     <row r="14" spans="1:7" x14ac:dyDescent="0.25">
@@ -973,39 +973,39 @@
     </row>
     <row r="17" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A17" s="7">
-        <v>46274</v>
+        <v>46275</v>
       </c>
       <c r="B17" s="8"/>
       <c r="C17" s="20" t="s">
         <v>14</v>
       </c>
       <c r="D17" s="10">
-        <v>246.16</v>
+        <v>247.81</v>
       </c>
       <c r="E17" s="10">
-        <v>209.53</v>
+        <v>212.26</v>
       </c>
       <c r="F17" s="10">
-        <v>219.53</v>
+        <v>222.26</v>
       </c>
       <c r="G17" s="17"/>
     </row>
     <row r="18" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A18" s="11">
-        <v>46273</v>
+        <v>46274</v>
       </c>
       <c r="B18" s="12"/>
       <c r="C18" s="12" t="s">
         <v>14</v>
       </c>
       <c r="D18" s="13">
-        <v>244.37</v>
+        <v>246.16</v>
       </c>
       <c r="E18" s="13">
-        <v>207.64</v>
+        <v>209.53</v>
       </c>
       <c r="F18" s="13">
-        <v>217.64</v>
+        <v>219.53</v>
       </c>
       <c r="G18" s="17"/>
     </row>
@@ -1052,41 +1052,41 @@
     </row>
     <row r="22" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A22" s="7">
-        <v>46274</v>
+        <v>46275</v>
       </c>
       <c r="B22" s="8"/>
       <c r="C22" s="20" t="s">
         <v>16</v>
       </c>
       <c r="D22" s="10">
-        <v>245.15</v>
+        <v>247.22</v>
       </c>
       <c r="E22" s="10">
-        <v>208.07</v>
+        <v>211.16</v>
       </c>
       <c r="F22" s="10">
-        <v>217.67</v>
+        <v>220.76</v>
       </c>
       <c r="G22" s="10">
-        <v>206.79</v>
+        <v>209.88</v>
       </c>
     </row>
     <row r="23" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A23" s="11">
-        <v>46274</v>
+        <v>46275</v>
       </c>
       <c r="B23" s="12"/>
       <c r="C23" s="21" t="s">
         <v>17</v>
       </c>
       <c r="D23" s="13">
-        <v>245.49</v>
+        <v>247.28</v>
       </c>
       <c r="E23" s="13">
-        <v>212.42</v>
+        <v>215.29</v>
       </c>
       <c r="F23" s="13">
-        <v>222.42</v>
+        <v>225.29</v>
       </c>
       <c r="G23" s="13" t="s">
         <v>18</v>
@@ -1094,20 +1094,20 @@
     </row>
     <row r="24" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A24" s="7">
-        <v>46274</v>
+        <v>46275</v>
       </c>
       <c r="B24" s="8"/>
       <c r="C24" s="20" t="s">
         <v>19</v>
       </c>
       <c r="D24" s="10">
-        <v>246.07</v>
+        <v>247.85</v>
       </c>
       <c r="E24" s="10">
-        <v>211.73</v>
+        <v>214.6</v>
       </c>
       <c r="F24" s="10">
-        <v>221.73</v>
+        <v>224.6</v>
       </c>
       <c r="G24" s="10" t="s">
         <v>18</v>
@@ -1115,41 +1115,41 @@
     </row>
     <row r="25" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A25" s="11">
-        <v>46274</v>
+        <v>46275</v>
       </c>
       <c r="B25" s="12"/>
       <c r="C25" s="21" t="s">
         <v>20</v>
       </c>
       <c r="D25" s="13">
-        <v>242.85</v>
+        <v>244.62</v>
       </c>
       <c r="E25" s="13">
-        <v>211.71</v>
+        <v>214.6</v>
       </c>
       <c r="F25" s="13">
-        <v>221.71</v>
+        <v>224.6</v>
       </c>
       <c r="G25" s="13">
-        <v>209.61</v>
+        <v>212.49</v>
       </c>
     </row>
     <row r="26" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A26" s="7">
-        <v>46274</v>
+        <v>46275</v>
       </c>
       <c r="B26" s="8"/>
       <c r="C26" s="20" t="s">
         <v>21</v>
       </c>
       <c r="D26" s="10">
-        <v>244.77</v>
+        <v>246.51</v>
       </c>
       <c r="E26" s="10">
-        <v>213.01</v>
+        <v>215.92</v>
       </c>
       <c r="F26" s="10">
-        <v>223.01</v>
+        <v>225.92</v>
       </c>
       <c r="G26" s="10" t="s">
         <v>18</v>
@@ -1157,41 +1157,41 @@
     </row>
     <row r="27" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A27" s="11">
-        <v>46273</v>
+        <v>46274</v>
       </c>
       <c r="B27" s="12"/>
       <c r="C27" s="12" t="s">
         <v>16</v>
       </c>
       <c r="D27" s="13">
-        <v>243.42</v>
+        <v>245.15</v>
       </c>
       <c r="E27" s="13">
-        <v>206.25</v>
+        <v>208.07</v>
       </c>
       <c r="F27" s="13">
-        <v>215.85</v>
+        <v>217.67</v>
       </c>
       <c r="G27" s="13">
-        <v>204.97</v>
+        <v>206.79</v>
       </c>
     </row>
     <row r="28" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A28" s="7">
-        <v>46273</v>
+        <v>46274</v>
       </c>
       <c r="B28" s="8"/>
       <c r="C28" s="20" t="s">
         <v>17</v>
       </c>
       <c r="D28" s="10">
-        <v>243.58</v>
+        <v>245.49</v>
       </c>
       <c r="E28" s="22">
-        <v>210.39</v>
+        <v>212.42</v>
       </c>
       <c r="F28" s="22">
-        <v>220.39</v>
+        <v>222.42</v>
       </c>
       <c r="G28" s="22" t="s">
         <v>18</v>
@@ -1199,20 +1199,20 @@
     </row>
     <row r="29" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A29" s="11">
-        <v>46273</v>
+        <v>46274</v>
       </c>
       <c r="B29" s="12"/>
       <c r="C29" s="12" t="s">
         <v>19</v>
       </c>
       <c r="D29" s="13">
-        <v>244.17</v>
+        <v>246.07</v>
       </c>
       <c r="E29" s="13">
-        <v>209.71</v>
+        <v>211.73</v>
       </c>
       <c r="F29" s="13">
-        <v>219.71</v>
+        <v>221.73</v>
       </c>
       <c r="G29" s="13" t="s">
         <v>18</v>
@@ -1220,41 +1220,41 @@
     </row>
     <row r="30" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A30" s="7">
-        <v>46273</v>
+        <v>46274</v>
       </c>
       <c r="B30" s="8"/>
       <c r="C30" s="20" t="s">
         <v>20</v>
       </c>
       <c r="D30" s="10">
-        <v>240.94</v>
+        <v>242.85</v>
       </c>
       <c r="E30" s="22">
-        <v>209.68</v>
+        <v>211.71</v>
       </c>
       <c r="F30" s="22">
-        <v>219.68</v>
+        <v>221.71</v>
       </c>
       <c r="G30" s="22">
-        <v>207.57</v>
+        <v>209.61</v>
       </c>
     </row>
     <row r="31" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A31" s="11">
-        <v>46273</v>
+        <v>46274</v>
       </c>
       <c r="B31" s="12"/>
       <c r="C31" s="12" t="s">
         <v>21</v>
       </c>
       <c r="D31" s="13">
-        <v>242.9</v>
+        <v>244.77</v>
       </c>
       <c r="E31" s="13">
-        <v>210.96</v>
+        <v>213.01</v>
       </c>
       <c r="F31" s="13">
-        <v>220.96</v>
+        <v>223.01</v>
       </c>
       <c r="G31" s="13" t="s">
         <v>18</v>
@@ -1301,52 +1301,52 @@
     </row>
     <row r="35" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A35" s="7">
-        <v>46274</v>
+        <v>46275</v>
       </c>
       <c r="B35" s="8"/>
       <c r="C35" s="20" t="s">
         <v>23</v>
       </c>
       <c r="D35" s="10">
-        <v>239.3</v>
+        <v>241.07</v>
       </c>
       <c r="E35" s="10">
-        <v>203.88</v>
+        <v>206.7</v>
       </c>
       <c r="F35" s="10">
-        <v>212.88</v>
+        <v>215.7</v>
       </c>
       <c r="G35" s="17"/>
     </row>
     <row r="36" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A36" s="11">
-        <v>46273</v>
+        <v>46274</v>
       </c>
       <c r="B36" s="12"/>
       <c r="C36" s="12" t="s">
         <v>23</v>
       </c>
       <c r="D36" s="13">
-        <v>237.39</v>
+        <v>239.3</v>
       </c>
       <c r="E36" s="13">
-        <v>201.89</v>
+        <v>203.88</v>
       </c>
       <c r="F36" s="13">
-        <v>210.89</v>
+        <v>212.88</v>
       </c>
       <c r="G36" s="17"/>
     </row>
     <row r="37" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A37" s="7">
-        <v>46274</v>
+        <v>46275</v>
       </c>
       <c r="B37" s="8"/>
       <c r="C37" s="20" t="s">
         <v>24</v>
       </c>
       <c r="D37" s="10">
-        <v>254.92</v>
+        <v>256.69</v>
       </c>
       <c r="E37" s="10" t="s">
         <v>18</v>
@@ -1358,14 +1358,14 @@
     </row>
     <row r="38" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A38" s="11">
-        <v>46273</v>
+        <v>46274</v>
       </c>
       <c r="B38" s="12"/>
       <c r="C38" s="12" t="s">
         <v>24</v>
       </c>
       <c r="D38" s="13">
-        <v>253.01</v>
+        <v>254.92</v>
       </c>
       <c r="E38" s="13" t="s">
         <v>18</v>
@@ -1416,77 +1416,77 @@
     </row>
     <row r="42" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A42" s="7">
-        <v>46274</v>
+        <v>46275</v>
       </c>
       <c r="B42" s="8"/>
       <c r="C42" s="20" t="s">
         <v>26</v>
       </c>
       <c r="D42" s="10">
-        <v>247.81</v>
+        <v>249.68</v>
       </c>
       <c r="E42" s="10">
-        <v>210.09</v>
+        <v>212.95</v>
       </c>
       <c r="F42" s="10">
-        <v>220.09</v>
+        <v>222.95</v>
       </c>
       <c r="G42" s="17"/>
     </row>
     <row r="43" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A43" s="11">
-        <v>46274</v>
+        <v>46275</v>
       </c>
       <c r="B43" s="12"/>
       <c r="C43" s="21" t="s">
         <v>27</v>
       </c>
       <c r="D43" s="13">
-        <v>247.44</v>
+        <v>249.31</v>
       </c>
       <c r="E43" s="13">
-        <v>210.5</v>
+        <v>213.37</v>
       </c>
       <c r="F43" s="13">
-        <v>220.5</v>
+        <v>223.37</v>
       </c>
       <c r="G43" s="17"/>
     </row>
     <row r="44" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A44" s="7">
-        <v>46273</v>
+        <v>46274</v>
       </c>
       <c r="B44" s="8"/>
       <c r="C44" s="20" t="s">
         <v>26</v>
       </c>
       <c r="D44" s="10">
-        <v>245.83</v>
+        <v>247.81</v>
       </c>
       <c r="E44" s="10">
-        <v>208.08</v>
+        <v>210.09</v>
       </c>
       <c r="F44" s="10">
-        <v>218.08</v>
+        <v>220.09</v>
       </c>
       <c r="G44" s="17"/>
     </row>
     <row r="45" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A45" s="11">
-        <v>46273</v>
+        <v>46274</v>
       </c>
       <c r="B45" s="12"/>
       <c r="C45" s="21" t="s">
         <v>27</v>
       </c>
       <c r="D45" s="13">
-        <v>245.46</v>
+        <v>247.44</v>
       </c>
       <c r="E45" s="13">
-        <v>208.49</v>
+        <v>210.5</v>
       </c>
       <c r="F45" s="13">
-        <v>218.49</v>
+        <v>220.5</v>
       </c>
       <c r="G45" s="17"/>
     </row>
@@ -1531,77 +1531,77 @@
     </row>
     <row r="49" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A49" s="7">
-        <v>46274</v>
+        <v>46275</v>
       </c>
       <c r="B49" s="8"/>
       <c r="C49" s="20" t="s">
         <v>29</v>
       </c>
       <c r="D49" s="10">
-        <v>239.82</v>
+        <v>241.95</v>
       </c>
       <c r="E49" s="10">
-        <v>203.03</v>
+        <v>205.88</v>
       </c>
       <c r="F49" s="10">
-        <v>213.03</v>
+        <v>215.88</v>
       </c>
       <c r="G49" s="28"/>
     </row>
     <row r="50" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A50" s="11">
-        <v>46274</v>
+        <v>46275</v>
       </c>
       <c r="B50" s="12"/>
       <c r="C50" s="21" t="s">
         <v>30</v>
       </c>
       <c r="D50" s="13">
-        <v>238.02</v>
+        <v>240.14</v>
       </c>
       <c r="E50" s="13">
-        <v>202.96</v>
+        <v>205.79</v>
       </c>
       <c r="F50" s="13">
-        <v>212.96</v>
+        <v>215.79</v>
       </c>
       <c r="G50" s="28"/>
     </row>
     <row r="51" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A51" s="7">
-        <v>46273</v>
+        <v>46274</v>
       </c>
       <c r="B51" s="8"/>
       <c r="C51" s="20" t="s">
         <v>29</v>
       </c>
       <c r="D51" s="10">
-        <v>237.37</v>
+        <v>239.82</v>
       </c>
       <c r="E51" s="10">
-        <v>200.75</v>
+        <v>203.03</v>
       </c>
       <c r="F51" s="10">
-        <v>210.75</v>
+        <v>213.03</v>
       </c>
       <c r="G51" s="17"/>
     </row>
     <row r="52" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A52" s="11">
-        <v>46273</v>
+        <v>46274</v>
       </c>
       <c r="B52" s="12"/>
       <c r="C52" s="21" t="s">
         <v>30</v>
       </c>
       <c r="D52" s="13">
-        <v>235.61</v>
+        <v>238.02</v>
       </c>
       <c r="E52" s="13">
-        <v>200.68</v>
+        <v>202.96</v>
       </c>
       <c r="F52" s="13">
-        <v>210.68</v>
+        <v>212.96</v>
       </c>
       <c r="G52" s="17"/>
     </row>
@@ -1646,52 +1646,52 @@
     </row>
     <row r="56" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A56" s="7">
-        <v>46274</v>
+        <v>46275</v>
       </c>
       <c r="B56" s="8"/>
       <c r="C56" s="20" t="s">
         <v>32</v>
       </c>
       <c r="D56" s="10">
-        <v>257.60000000000002</v>
+        <v>259.33</v>
       </c>
       <c r="E56" s="10">
-        <v>223.66</v>
+        <v>227</v>
       </c>
       <c r="F56" s="10">
-        <v>233.66</v>
+        <v>237</v>
       </c>
       <c r="G56" s="17"/>
     </row>
     <row r="57" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A57" s="11">
-        <v>46274</v>
+        <v>46275</v>
       </c>
       <c r="B57" s="12"/>
       <c r="C57" s="21" t="s">
         <v>33</v>
       </c>
       <c r="D57" s="13">
-        <v>246.33</v>
+        <v>248.11</v>
       </c>
       <c r="E57" s="13">
-        <v>215.16</v>
+        <v>217.85</v>
       </c>
       <c r="F57" s="13">
-        <v>225.16</v>
+        <v>227.85</v>
       </c>
       <c r="G57" s="17"/>
     </row>
     <row r="58" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A58" s="7">
-        <v>46274</v>
+        <v>46275</v>
       </c>
       <c r="B58" s="8"/>
       <c r="C58" s="20" t="s">
         <v>34</v>
       </c>
       <c r="D58" s="10">
-        <v>247.49</v>
+        <v>249.3</v>
       </c>
       <c r="E58" s="10" t="s">
         <v>18</v>
@@ -1703,17 +1703,17 @@
     </row>
     <row r="59" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A59" s="11">
-        <v>46274</v>
+        <v>46275</v>
       </c>
       <c r="B59" s="12"/>
       <c r="C59" s="21" t="s">
         <v>35</v>
       </c>
       <c r="D59" s="13">
-        <v>244.5</v>
+        <v>246.12</v>
       </c>
       <c r="E59" s="13">
-        <v>209.55</v>
+        <v>212.24</v>
       </c>
       <c r="F59" s="13" t="s">
         <v>18</v>
@@ -1722,36 +1722,36 @@
     </row>
     <row r="60" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A60" s="7">
-        <v>46274</v>
+        <v>46275</v>
       </c>
       <c r="B60" s="8"/>
       <c r="C60" s="20" t="s">
         <v>36</v>
       </c>
       <c r="D60" s="10">
-        <v>240.32</v>
+        <v>241.94</v>
       </c>
       <c r="E60" s="10">
-        <v>205.48</v>
+        <v>208.17</v>
       </c>
       <c r="F60" s="10">
-        <v>215.48</v>
+        <v>218.17</v>
       </c>
       <c r="G60" s="17"/>
     </row>
     <row r="61" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A61" s="11">
-        <v>46274</v>
+        <v>46275</v>
       </c>
       <c r="B61" s="12"/>
       <c r="C61" s="21" t="s">
         <v>37</v>
       </c>
       <c r="D61" s="13">
-        <v>245.77</v>
+        <v>247.41</v>
       </c>
       <c r="E61" s="13">
-        <v>220.43</v>
+        <v>223.54</v>
       </c>
       <c r="F61" s="13" t="s">
         <v>18</v>
@@ -1760,52 +1760,52 @@
     </row>
     <row r="62" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A62" s="7">
-        <v>46273</v>
+        <v>46274</v>
       </c>
       <c r="B62" s="8"/>
       <c r="C62" s="20" t="s">
         <v>32</v>
       </c>
       <c r="D62" s="10">
-        <v>255.73</v>
+        <v>257.60000000000002</v>
       </c>
       <c r="E62" s="10">
-        <v>221.21</v>
+        <v>223.66</v>
       </c>
       <c r="F62" s="10">
-        <v>231.21</v>
+        <v>233.66</v>
       </c>
       <c r="G62" s="17"/>
     </row>
     <row r="63" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A63" s="11">
-        <v>46273</v>
+        <v>46274</v>
       </c>
       <c r="B63" s="12"/>
       <c r="C63" s="21" t="s">
         <v>33</v>
       </c>
       <c r="D63" s="13">
-        <v>244.42</v>
+        <v>246.33</v>
       </c>
       <c r="E63" s="13">
-        <v>213.85</v>
+        <v>215.16</v>
       </c>
       <c r="F63" s="13">
-        <v>223.85</v>
+        <v>225.16</v>
       </c>
       <c r="G63" s="17"/>
     </row>
     <row r="64" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A64" s="7">
-        <v>46273</v>
+        <v>46274</v>
       </c>
       <c r="B64" s="8"/>
       <c r="C64" s="20" t="s">
         <v>34</v>
       </c>
       <c r="D64" s="10">
-        <v>245.57</v>
+        <v>247.49</v>
       </c>
       <c r="E64" s="10" t="s">
         <v>18</v>
@@ -1817,17 +1817,17 @@
     </row>
     <row r="65" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A65" s="11">
-        <v>46273</v>
+        <v>46274</v>
       </c>
       <c r="B65" s="12"/>
       <c r="C65" s="21" t="s">
         <v>35</v>
       </c>
       <c r="D65" s="13">
-        <v>242.73</v>
+        <v>244.5</v>
       </c>
       <c r="E65" s="13">
-        <v>208.24</v>
+        <v>209.55</v>
       </c>
       <c r="F65" s="13" t="s">
         <v>18</v>
@@ -1835,35 +1835,35 @@
     </row>
     <row r="66" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A66" s="7">
-        <v>46273</v>
+        <v>46274</v>
       </c>
       <c r="B66" s="8"/>
       <c r="C66" s="20" t="s">
         <v>36</v>
       </c>
       <c r="D66" s="10">
-        <v>238.55</v>
+        <v>240.32</v>
       </c>
       <c r="E66" s="10">
-        <v>204.17</v>
+        <v>205.48</v>
       </c>
       <c r="F66" s="10">
-        <v>214.17</v>
+        <v>215.48</v>
       </c>
     </row>
     <row r="67" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A67" s="11">
-        <v>46273</v>
+        <v>46274</v>
       </c>
       <c r="B67" s="12"/>
       <c r="C67" s="21" t="s">
         <v>37</v>
       </c>
       <c r="D67" s="13">
-        <v>244</v>
+        <v>245.77</v>
       </c>
       <c r="E67" s="13">
-        <v>218.18</v>
+        <v>220.43</v>
       </c>
       <c r="F67" s="13" t="s">
         <v>18</v>
@@ -1891,6 +1891,26 @@
 </file>
 
 <file path=customXml/item1.xml><?xml version="1.0" encoding="utf-8"?>
+<?mso-contentType ?>
+<FormTemplates xmlns="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms">
+  <Display>DocumentLibraryForm</Display>
+  <Edit>DocumentLibraryForm</Edit>
+  <New>DocumentLibraryForm</New>
+</FormTemplates>
+</file>
+
+<file path=customXml/item2.xml><?xml version="1.0" encoding="utf-8"?>
+<p:properties xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls">
+  <documentManagement>
+    <lcf76f155ced4ddcb4097134ff3c332f xmlns="87276d81-85f4-4ef2-9e6e-55066304288f">
+      <Terms xmlns="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
+    </lcf76f155ced4ddcb4097134ff3c332f>
+    <TaxCatchAll xmlns="b23b8984-eafa-4e79-985e-54f52f3da58e" xsi:nil="true"/>
+  </documentManagement>
+</p:properties>
+</file>
+
+<file path=customXml/item3.xml><?xml version="1.0" encoding="utf-8"?>
 <ct:contentTypeSchema xmlns:ct="http://schemas.microsoft.com/office/2006/metadata/contentType" xmlns:ma="http://schemas.microsoft.com/office/2006/metadata/properties/metaAttributes" ct:_="" ma:_="" ma:contentTypeName="Document" ma:contentTypeID="0x010100D3632DF5622958439304627C030B0427" ma:contentTypeVersion="18" ma:contentTypeDescription="Create a new document." ma:contentTypeScope="" ma:versionID="8c2ecbce386d6bac497f8eb2d8f0fb7a">
   <xsd:schema xmlns:xsd="http://www.w3.org/2001/XMLSchema" xmlns:xs="http://www.w3.org/2001/XMLSchema" xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:ns2="87276d81-85f4-4ef2-9e6e-55066304288f" xmlns:ns3="39e1dda6-d1d8-4c88-a3b9-f1abc1284bad" xmlns:ns4="b23b8984-eafa-4e79-985e-54f52f3da58e" targetNamespace="http://schemas.microsoft.com/office/2006/metadata/properties" ma:root="true" ma:fieldsID="4cfd0c2f651c1ce156ad4fcb44ea61dd" ns2:_="" ns3:_="" ns4:_="">
     <xsd:import namespace="87276d81-85f4-4ef2-9e6e-55066304288f"/>
@@ -2150,27 +2170,26 @@
 </ct:contentTypeSchema>
 </file>
 
-<file path=customXml/item2.xml><?xml version="1.0" encoding="utf-8"?>
-<?mso-contentType ?>
-<FormTemplates xmlns="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms">
-  <Display>DocumentLibraryForm</Display>
-  <Edit>DocumentLibraryForm</Edit>
-  <New>DocumentLibraryForm</New>
-</FormTemplates>
+<file path=customXml/itemProps1.xml><?xml version="1.0" encoding="utf-8"?>
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{F60519E9-FD90-4339-869C-BC2F85719BB8}">
+  <ds:schemaRefs>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms"/>
+  </ds:schemaRefs>
+</ds:datastoreItem>
 </file>
 
-<file path=customXml/item3.xml><?xml version="1.0" encoding="utf-8"?>
-<p:properties xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls">
-  <documentManagement>
-    <lcf76f155ced4ddcb4097134ff3c332f xmlns="87276d81-85f4-4ef2-9e6e-55066304288f">
-      <Terms xmlns="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
-    </lcf76f155ced4ddcb4097134ff3c332f>
-    <TaxCatchAll xmlns="b23b8984-eafa-4e79-985e-54f52f3da58e" xsi:nil="true"/>
-  </documentManagement>
-</p:properties>
+<file path=customXml/itemProps2.xml><?xml version="1.0" encoding="utf-8"?>
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{57A83D98-2BAE-4D83-823A-D31C464B620C}">
+  <ds:schemaRefs>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/properties"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
+    <ds:schemaRef ds:uri="87276d81-85f4-4ef2-9e6e-55066304288f"/>
+    <ds:schemaRef ds:uri="b23b8984-eafa-4e79-985e-54f52f3da58e"/>
+  </ds:schemaRefs>
+</ds:datastoreItem>
 </file>
 
-<file path=customXml/itemProps1.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=customXml/itemProps3.xml><?xml version="1.0" encoding="utf-8"?>
 <ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{B44E1863-2778-41F9-ACBA-48420F931671}">
   <ds:schemaRefs>
     <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/contentType"/>
@@ -2190,25 +2209,6 @@
 </ds:datastoreItem>
 </file>
 
-<file path=customXml/itemProps2.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{F60519E9-FD90-4339-869C-BC2F85719BB8}">
-  <ds:schemaRefs>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms"/>
-  </ds:schemaRefs>
-</ds:datastoreItem>
-</file>
-
-<file path=customXml/itemProps3.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{57A83D98-2BAE-4D83-823A-D31C464B620C}">
-  <ds:schemaRefs>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/properties"/>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
-    <ds:schemaRef ds:uri="87276d81-85f4-4ef2-9e6e-55066304288f"/>
-    <ds:schemaRef ds:uri="b23b8984-eafa-4e79-985e-54f52f3da58e"/>
-  </ds:schemaRefs>
-</ds:datastoreItem>
-</file>
-
 <file path=docMetadata/LabelInfo.xml><?xml version="1.0" encoding="utf-8"?>
 <clbl:labelList xmlns:clbl="http://schemas.microsoft.com/office/2020/mipLabelMetadata">
   <clbl:label id="{569bf4a9-87bd-4dbf-a36c-1db5158e5def}" enabled="1" method="Privileged" siteId="{ea80952e-a476-42d4-aaf4-5457852b0f7e}" removed="0"/>

</xml_diff>

<commit_message>
Thu Sep 10 06:05:55 UTC 2026
</commit_message>
<xml_diff>
--- a/bp.com-content-dam-bp-country-sites-en_au-australia-home-products-services-pricing-tgp-excel.xlsx
+++ b/bp.com-content-dam-bp-country-sites-en_au-australia-home-products-services-pricing-tgp-excel.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://bp365.sharepoint.com/sites/WholesalePricing/Shared Documents/B2C/TGP/Daily TGP/Web TGP/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="14_{C226758B-06B3-482F-9671-3AE14209B915}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="14_{02604CF4-5B85-4EA0-B24E-C4B315B59949}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-28920" yWindow="-60" windowWidth="29040" windowHeight="15720" xr2:uid="{1B412EEF-F96D-4DF4-A4E9-C7F0F183C2FB}"/>
+    <workbookView xWindow="-110" yWindow="-110" windowWidth="19420" windowHeight="11500" xr2:uid="{1B412EEF-F96D-4DF4-A4E9-C7F0F183C2FB}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
@@ -715,15 +715,15 @@
     <pageSetUpPr fitToPage="1"/>
   </sheetPr>
   <dimension ref="A1:G67"/>
-  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
   <cols>
-    <col min="1" max="1" width="76.42578125" bestFit="1" customWidth="1"/>
-    <col min="2" max="2" width="6.42578125"/>
-    <col min="3" max="3" width="18.140625" bestFit="1" customWidth="1"/>
-    <col min="4" max="7" width="7.140625" bestFit="1" customWidth="1"/>
+    <col min="1" max="1" width="76.453125" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="6.453125"/>
+    <col min="3" max="3" width="18.1796875" bestFit="1" customWidth="1"/>
+    <col min="4" max="7" width="7.1796875" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:7" ht="23.25" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:7" ht="22.5" x14ac:dyDescent="0.35">
       <c r="A1" s="30" t="s">
         <v>0</v>
       </c>
@@ -734,7 +734,7 @@
       <c r="F1" s="2"/>
       <c r="G1" s="2"/>
     </row>
-    <row r="2" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="2" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A2" s="3"/>
       <c r="B2" s="1"/>
       <c r="C2" s="1"/>
@@ -743,7 +743,7 @@
       <c r="F2" s="2"/>
       <c r="G2" s="2"/>
     </row>
-    <row r="3" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="3" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A3" s="3" t="s">
         <v>1</v>
       </c>
@@ -754,7 +754,7 @@
       <c r="F3" s="2"/>
       <c r="G3" s="2"/>
     </row>
-    <row r="4" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="4" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A4" s="3" t="s">
         <v>2</v>
       </c>
@@ -765,7 +765,7 @@
       <c r="F4" s="2"/>
       <c r="G4" s="2"/>
     </row>
-    <row r="5" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="5" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A5" s="3"/>
       <c r="B5" s="3"/>
       <c r="C5" s="1"/>
@@ -774,7 +774,7 @@
       <c r="F5" s="2"/>
       <c r="G5" s="2"/>
     </row>
-    <row r="6" spans="1:7" ht="20.25" x14ac:dyDescent="0.25">
+    <row r="6" spans="1:7" ht="20" x14ac:dyDescent="0.35">
       <c r="A6" s="29" t="s">
         <v>3</v>
       </c>
@@ -785,7 +785,7 @@
       <c r="F6" s="2"/>
       <c r="G6" s="2"/>
     </row>
-    <row r="7" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="7" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A7" s="4" t="s">
         <v>4</v>
       </c>
@@ -806,133 +806,133 @@
         <v>9</v>
       </c>
     </row>
-    <row r="8" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="8" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A8" s="7">
-        <v>46275</v>
+        <v>46276</v>
       </c>
       <c r="B8" s="8"/>
       <c r="C8" s="9" t="s">
         <v>10</v>
       </c>
       <c r="D8" s="10">
-        <v>246.08</v>
+        <v>246.84</v>
       </c>
       <c r="E8" s="10">
-        <v>210.46</v>
+        <v>212.58</v>
       </c>
       <c r="F8" s="10">
-        <v>220.46</v>
+        <v>222.58</v>
       </c>
       <c r="G8" s="10">
-        <v>210.43</v>
-      </c>
-    </row>
-    <row r="9" spans="1:7" x14ac:dyDescent="0.25">
+        <v>212.54</v>
+      </c>
+    </row>
+    <row r="9" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A9" s="11">
-        <v>46275</v>
+        <v>46276</v>
       </c>
       <c r="B9" s="12"/>
       <c r="C9" s="12" t="s">
         <v>11</v>
       </c>
       <c r="D9" s="13">
-        <v>246.08</v>
+        <v>246.84</v>
       </c>
       <c r="E9" s="13">
-        <v>210.46</v>
+        <v>212.58</v>
       </c>
       <c r="F9" s="13">
-        <v>220.46</v>
+        <v>222.58</v>
       </c>
       <c r="G9" s="13">
-        <v>210.43</v>
-      </c>
-    </row>
-    <row r="10" spans="1:7" x14ac:dyDescent="0.25">
+        <v>212.54</v>
+      </c>
+    </row>
+    <row r="10" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A10" s="7">
-        <v>46275</v>
+        <v>46276</v>
       </c>
       <c r="B10" s="8"/>
       <c r="C10" s="9" t="s">
         <v>12</v>
       </c>
       <c r="D10" s="10">
-        <v>242.55</v>
+        <v>243.05</v>
       </c>
       <c r="E10" s="10">
-        <v>207.74</v>
+        <v>209.64</v>
       </c>
       <c r="F10" s="10">
-        <v>217.75</v>
+        <v>219.64</v>
       </c>
       <c r="G10" s="10">
-        <v>208.16</v>
-      </c>
-    </row>
-    <row r="11" spans="1:7" x14ac:dyDescent="0.25">
+        <v>210.06</v>
+      </c>
+    </row>
+    <row r="11" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A11" s="11">
-        <v>46274</v>
+        <v>46275</v>
       </c>
       <c r="B11" s="12"/>
       <c r="C11" s="12" t="s">
         <v>10</v>
       </c>
       <c r="D11" s="13">
-        <v>244.01</v>
+        <v>246.08</v>
       </c>
       <c r="E11" s="13">
-        <v>207.38</v>
+        <v>210.46</v>
       </c>
       <c r="F11" s="13">
-        <v>217.38</v>
+        <v>220.46</v>
       </c>
       <c r="G11" s="13">
-        <v>207.34</v>
-      </c>
-    </row>
-    <row r="12" spans="1:7" x14ac:dyDescent="0.25">
+        <v>210.43</v>
+      </c>
+    </row>
+    <row r="12" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A12" s="7">
-        <v>46274</v>
+        <v>46275</v>
       </c>
       <c r="B12" s="8"/>
       <c r="C12" s="9" t="s">
         <v>11</v>
       </c>
       <c r="D12" s="10">
-        <v>244.01</v>
+        <v>246.08</v>
       </c>
       <c r="E12" s="10">
-        <v>207.38</v>
+        <v>210.46</v>
       </c>
       <c r="F12" s="10">
-        <v>217.38</v>
+        <v>220.46</v>
       </c>
       <c r="G12" s="10">
-        <v>207.34</v>
-      </c>
-    </row>
-    <row r="13" spans="1:7" x14ac:dyDescent="0.25">
+        <v>210.43</v>
+      </c>
+    </row>
+    <row r="13" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A13" s="11">
-        <v>46274</v>
+        <v>46275</v>
       </c>
       <c r="B13" s="12"/>
       <c r="C13" s="12" t="s">
         <v>12</v>
       </c>
       <c r="D13" s="13">
-        <v>240.77</v>
+        <v>242.55</v>
       </c>
       <c r="E13" s="13">
-        <v>204.92</v>
+        <v>207.74</v>
       </c>
       <c r="F13" s="13">
-        <v>214.92</v>
+        <v>217.75</v>
       </c>
       <c r="G13" s="13">
-        <v>205.34</v>
-      </c>
-    </row>
-    <row r="14" spans="1:7" x14ac:dyDescent="0.25">
+        <v>208.16</v>
+      </c>
+    </row>
+    <row r="14" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A14" s="14"/>
       <c r="B14" s="14"/>
       <c r="C14" s="15"/>
@@ -941,7 +941,7 @@
       <c r="F14" s="16"/>
       <c r="G14" s="16"/>
     </row>
-    <row r="15" spans="1:7" ht="20.25" x14ac:dyDescent="0.25">
+    <row r="15" spans="1:7" ht="20" x14ac:dyDescent="0.35">
       <c r="A15" s="29" t="s">
         <v>13</v>
       </c>
@@ -952,7 +952,7 @@
       <c r="F15" s="17"/>
       <c r="G15" s="17"/>
     </row>
-    <row r="16" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="16" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A16" s="4" t="s">
         <v>4</v>
       </c>
@@ -971,45 +971,45 @@
       </c>
       <c r="G16" s="17"/>
     </row>
-    <row r="17" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="17" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A17" s="7">
-        <v>46275</v>
+        <v>46276</v>
       </c>
       <c r="B17" s="8"/>
       <c r="C17" s="20" t="s">
         <v>14</v>
       </c>
       <c r="D17" s="10">
-        <v>247.81</v>
+        <v>248.19</v>
       </c>
       <c r="E17" s="10">
-        <v>212.26</v>
+        <v>214.05</v>
       </c>
       <c r="F17" s="10">
-        <v>222.26</v>
+        <v>224.05</v>
       </c>
       <c r="G17" s="17"/>
     </row>
-    <row r="18" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="18" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A18" s="11">
-        <v>46274</v>
+        <v>46275</v>
       </c>
       <c r="B18" s="12"/>
       <c r="C18" s="12" t="s">
         <v>14</v>
       </c>
       <c r="D18" s="13">
-        <v>246.16</v>
+        <v>247.81</v>
       </c>
       <c r="E18" s="13">
-        <v>209.53</v>
+        <v>212.26</v>
       </c>
       <c r="F18" s="13">
-        <v>219.53</v>
+        <v>222.26</v>
       </c>
       <c r="G18" s="17"/>
     </row>
-    <row r="19" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="19" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A19" s="14"/>
       <c r="B19" s="14"/>
       <c r="C19" s="15"/>
@@ -1018,7 +1018,7 @@
       <c r="F19" s="16"/>
       <c r="G19" s="17"/>
     </row>
-    <row r="20" spans="1:7" ht="20.25" x14ac:dyDescent="0.25">
+    <row r="20" spans="1:7" ht="20" x14ac:dyDescent="0.35">
       <c r="A20" s="29" t="s">
         <v>15</v>
       </c>
@@ -1029,7 +1029,7 @@
       <c r="F20" s="17"/>
       <c r="G20" s="17"/>
     </row>
-    <row r="21" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="21" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A21" s="4" t="s">
         <v>4</v>
       </c>
@@ -1050,217 +1050,217 @@
         <v>9</v>
       </c>
     </row>
-    <row r="22" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="22" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A22" s="7">
-        <v>46275</v>
+        <v>46276</v>
       </c>
       <c r="B22" s="8"/>
       <c r="C22" s="20" t="s">
         <v>16</v>
       </c>
       <c r="D22" s="10">
-        <v>247.22</v>
+        <v>247.97</v>
       </c>
       <c r="E22" s="10">
-        <v>211.16</v>
+        <v>213.28</v>
       </c>
       <c r="F22" s="10">
-        <v>220.76</v>
+        <v>222.88</v>
       </c>
       <c r="G22" s="10">
-        <v>209.88</v>
-      </c>
-    </row>
-    <row r="23" spans="1:7" x14ac:dyDescent="0.25">
+        <v>211.99</v>
+      </c>
+    </row>
+    <row r="23" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A23" s="11">
-        <v>46275</v>
+        <v>46276</v>
       </c>
       <c r="B23" s="12"/>
       <c r="C23" s="21" t="s">
         <v>17</v>
       </c>
       <c r="D23" s="13">
-        <v>247.28</v>
+        <v>247.79</v>
       </c>
       <c r="E23" s="13">
-        <v>215.29</v>
+        <v>217.23</v>
       </c>
       <c r="F23" s="13">
-        <v>225.29</v>
+        <v>227.23</v>
       </c>
       <c r="G23" s="13" t="s">
         <v>18</v>
       </c>
     </row>
-    <row r="24" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="24" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A24" s="7">
-        <v>46275</v>
+        <v>46276</v>
       </c>
       <c r="B24" s="8"/>
       <c r="C24" s="20" t="s">
         <v>19</v>
       </c>
       <c r="D24" s="10">
-        <v>247.85</v>
+        <v>248.34</v>
       </c>
       <c r="E24" s="10">
-        <v>214.6</v>
+        <v>216.53</v>
       </c>
       <c r="F24" s="10">
-        <v>224.6</v>
+        <v>226.53</v>
       </c>
       <c r="G24" s="10" t="s">
         <v>18</v>
       </c>
     </row>
-    <row r="25" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="25" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A25" s="11">
-        <v>46275</v>
+        <v>46276</v>
       </c>
       <c r="B25" s="12"/>
       <c r="C25" s="21" t="s">
         <v>20</v>
       </c>
       <c r="D25" s="13">
-        <v>244.62</v>
+        <v>245.13</v>
       </c>
       <c r="E25" s="13">
-        <v>214.6</v>
+        <v>216.55</v>
       </c>
       <c r="F25" s="13">
-        <v>224.6</v>
+        <v>226.55</v>
       </c>
       <c r="G25" s="13">
-        <v>212.49</v>
-      </c>
-    </row>
-    <row r="26" spans="1:7" x14ac:dyDescent="0.25">
+        <v>214.45</v>
+      </c>
+    </row>
+    <row r="26" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A26" s="7">
-        <v>46275</v>
+        <v>46276</v>
       </c>
       <c r="B26" s="8"/>
       <c r="C26" s="20" t="s">
         <v>21</v>
       </c>
       <c r="D26" s="10">
-        <v>246.51</v>
+        <v>246.98</v>
       </c>
       <c r="E26" s="10">
-        <v>215.92</v>
+        <v>217.89</v>
       </c>
       <c r="F26" s="10">
-        <v>225.92</v>
+        <v>227.89</v>
       </c>
       <c r="G26" s="10" t="s">
         <v>18</v>
       </c>
     </row>
-    <row r="27" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="27" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A27" s="11">
-        <v>46274</v>
+        <v>46275</v>
       </c>
       <c r="B27" s="12"/>
       <c r="C27" s="12" t="s">
         <v>16</v>
       </c>
       <c r="D27" s="13">
-        <v>245.15</v>
+        <v>247.22</v>
       </c>
       <c r="E27" s="13">
-        <v>208.07</v>
+        <v>211.16</v>
       </c>
       <c r="F27" s="13">
-        <v>217.67</v>
+        <v>220.76</v>
       </c>
       <c r="G27" s="13">
-        <v>206.79</v>
-      </c>
-    </row>
-    <row r="28" spans="1:7" x14ac:dyDescent="0.25">
+        <v>209.88</v>
+      </c>
+    </row>
+    <row r="28" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A28" s="7">
-        <v>46274</v>
+        <v>46275</v>
       </c>
       <c r="B28" s="8"/>
       <c r="C28" s="20" t="s">
         <v>17</v>
       </c>
       <c r="D28" s="10">
-        <v>245.49</v>
+        <v>247.28</v>
       </c>
       <c r="E28" s="22">
-        <v>212.42</v>
+        <v>215.29</v>
       </c>
       <c r="F28" s="22">
-        <v>222.42</v>
+        <v>225.29</v>
       </c>
       <c r="G28" s="22" t="s">
         <v>18</v>
       </c>
     </row>
-    <row r="29" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="29" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A29" s="11">
-        <v>46274</v>
+        <v>46275</v>
       </c>
       <c r="B29" s="12"/>
       <c r="C29" s="12" t="s">
         <v>19</v>
       </c>
       <c r="D29" s="13">
-        <v>246.07</v>
+        <v>247.85</v>
       </c>
       <c r="E29" s="13">
-        <v>211.73</v>
+        <v>214.6</v>
       </c>
       <c r="F29" s="13">
-        <v>221.73</v>
+        <v>224.6</v>
       </c>
       <c r="G29" s="13" t="s">
         <v>18</v>
       </c>
     </row>
-    <row r="30" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="30" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A30" s="7">
-        <v>46274</v>
+        <v>46275</v>
       </c>
       <c r="B30" s="8"/>
       <c r="C30" s="20" t="s">
         <v>20</v>
       </c>
       <c r="D30" s="10">
-        <v>242.85</v>
+        <v>244.62</v>
       </c>
       <c r="E30" s="22">
-        <v>211.71</v>
+        <v>214.6</v>
       </c>
       <c r="F30" s="22">
-        <v>221.71</v>
+        <v>224.6</v>
       </c>
       <c r="G30" s="22">
-        <v>209.61</v>
-      </c>
-    </row>
-    <row r="31" spans="1:7" x14ac:dyDescent="0.25">
+        <v>212.49</v>
+      </c>
+    </row>
+    <row r="31" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A31" s="11">
-        <v>46274</v>
+        <v>46275</v>
       </c>
       <c r="B31" s="12"/>
       <c r="C31" s="12" t="s">
         <v>21</v>
       </c>
       <c r="D31" s="13">
-        <v>244.77</v>
+        <v>246.51</v>
       </c>
       <c r="E31" s="13">
-        <v>213.01</v>
+        <v>215.92</v>
       </c>
       <c r="F31" s="13">
-        <v>223.01</v>
+        <v>225.92</v>
       </c>
       <c r="G31" s="13" t="s">
         <v>18</v>
       </c>
     </row>
-    <row r="32" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="32" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A32" s="14"/>
       <c r="B32" s="14"/>
       <c r="C32" s="15"/>
@@ -1269,7 +1269,7 @@
       <c r="F32" s="17"/>
       <c r="G32" s="17"/>
     </row>
-    <row r="33" spans="1:7" ht="20.25" x14ac:dyDescent="0.25">
+    <row r="33" spans="1:7" ht="20" x14ac:dyDescent="0.35">
       <c r="A33" s="29" t="s">
         <v>22</v>
       </c>
@@ -1280,7 +1280,7 @@
       <c r="F33" s="17"/>
       <c r="G33" s="17"/>
     </row>
-    <row r="34" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="34" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A34" s="23" t="s">
         <v>4</v>
       </c>
@@ -1299,54 +1299,54 @@
       </c>
       <c r="G34" s="17"/>
     </row>
-    <row r="35" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="35" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A35" s="7">
-        <v>46275</v>
+        <v>46276</v>
       </c>
       <c r="B35" s="8"/>
       <c r="C35" s="20" t="s">
         <v>23</v>
       </c>
       <c r="D35" s="10">
-        <v>241.07</v>
+        <v>241.58</v>
       </c>
       <c r="E35" s="10">
-        <v>206.7</v>
+        <v>208.6</v>
       </c>
       <c r="F35" s="10">
-        <v>215.7</v>
+        <v>217.6</v>
       </c>
       <c r="G35" s="17"/>
     </row>
-    <row r="36" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="36" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A36" s="11">
-        <v>46274</v>
+        <v>46275</v>
       </c>
       <c r="B36" s="12"/>
       <c r="C36" s="12" t="s">
         <v>23</v>
       </c>
       <c r="D36" s="13">
-        <v>239.3</v>
+        <v>241.07</v>
       </c>
       <c r="E36" s="13">
-        <v>203.88</v>
+        <v>206.7</v>
       </c>
       <c r="F36" s="13">
-        <v>212.88</v>
+        <v>215.7</v>
       </c>
       <c r="G36" s="17"/>
     </row>
-    <row r="37" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="37" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A37" s="7">
-        <v>46275</v>
+        <v>46276</v>
       </c>
       <c r="B37" s="8"/>
       <c r="C37" s="20" t="s">
         <v>24</v>
       </c>
       <c r="D37" s="10">
-        <v>256.69</v>
+        <v>257.2</v>
       </c>
       <c r="E37" s="10" t="s">
         <v>18</v>
@@ -1356,16 +1356,16 @@
       </c>
       <c r="G37" s="17"/>
     </row>
-    <row r="38" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="38" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A38" s="11">
-        <v>46274</v>
+        <v>46275</v>
       </c>
       <c r="B38" s="12"/>
       <c r="C38" s="12" t="s">
         <v>24</v>
       </c>
       <c r="D38" s="13">
-        <v>254.92</v>
+        <v>256.69</v>
       </c>
       <c r="E38" s="13" t="s">
         <v>18</v>
@@ -1375,7 +1375,7 @@
       </c>
       <c r="G38" s="17"/>
     </row>
-    <row r="39" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="39" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A39" s="24"/>
       <c r="B39" s="24"/>
       <c r="C39" s="15"/>
@@ -1384,7 +1384,7 @@
       <c r="F39" s="17"/>
       <c r="G39" s="17"/>
     </row>
-    <row r="40" spans="1:7" ht="20.25" x14ac:dyDescent="0.25">
+    <row r="40" spans="1:7" ht="20" x14ac:dyDescent="0.35">
       <c r="A40" s="29" t="s">
         <v>25</v>
       </c>
@@ -1395,7 +1395,7 @@
       <c r="F40" s="17"/>
       <c r="G40" s="17"/>
     </row>
-    <row r="41" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="41" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A41" s="23" t="s">
         <v>4</v>
       </c>
@@ -1414,83 +1414,83 @@
       </c>
       <c r="G41" s="17"/>
     </row>
-    <row r="42" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="42" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A42" s="7">
-        <v>46275</v>
+        <v>46276</v>
       </c>
       <c r="B42" s="8"/>
       <c r="C42" s="20" t="s">
         <v>26</v>
       </c>
       <c r="D42" s="10">
-        <v>249.68</v>
+        <v>250.28</v>
       </c>
       <c r="E42" s="10">
-        <v>212.95</v>
+        <v>214.96</v>
       </c>
       <c r="F42" s="10">
-        <v>222.95</v>
+        <v>224.96</v>
       </c>
       <c r="G42" s="17"/>
     </row>
-    <row r="43" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="43" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A43" s="11">
-        <v>46275</v>
+        <v>46276</v>
       </c>
       <c r="B43" s="12"/>
       <c r="C43" s="21" t="s">
         <v>27</v>
       </c>
       <c r="D43" s="13">
-        <v>249.31</v>
+        <v>249.9</v>
       </c>
       <c r="E43" s="13">
-        <v>213.37</v>
+        <v>215.37</v>
       </c>
       <c r="F43" s="13">
-        <v>223.37</v>
+        <v>225.37</v>
       </c>
       <c r="G43" s="17"/>
     </row>
-    <row r="44" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="44" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A44" s="7">
-        <v>46274</v>
+        <v>46275</v>
       </c>
       <c r="B44" s="8"/>
       <c r="C44" s="20" t="s">
         <v>26</v>
       </c>
       <c r="D44" s="10">
-        <v>247.81</v>
+        <v>249.68</v>
       </c>
       <c r="E44" s="10">
-        <v>210.09</v>
+        <v>212.95</v>
       </c>
       <c r="F44" s="10">
-        <v>220.09</v>
+        <v>222.95</v>
       </c>
       <c r="G44" s="17"/>
     </row>
-    <row r="45" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="45" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A45" s="11">
-        <v>46274</v>
+        <v>46275</v>
       </c>
       <c r="B45" s="12"/>
       <c r="C45" s="21" t="s">
         <v>27</v>
       </c>
       <c r="D45" s="13">
-        <v>247.44</v>
+        <v>249.31</v>
       </c>
       <c r="E45" s="13">
-        <v>210.5</v>
+        <v>213.37</v>
       </c>
       <c r="F45" s="13">
-        <v>220.5</v>
+        <v>223.37</v>
       </c>
       <c r="G45" s="17"/>
     </row>
-    <row r="46" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="46" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A46" s="14"/>
       <c r="B46" s="24"/>
       <c r="C46" s="15"/>
@@ -1499,7 +1499,7 @@
       <c r="F46" s="16"/>
       <c r="G46" s="17"/>
     </row>
-    <row r="47" spans="1:7" ht="20.25" x14ac:dyDescent="0.25">
+    <row r="47" spans="1:7" ht="20" x14ac:dyDescent="0.35">
       <c r="A47" s="25" t="s">
         <v>28</v>
       </c>
@@ -1510,7 +1510,7 @@
       <c r="F47" s="17"/>
       <c r="G47" s="17"/>
     </row>
-    <row r="48" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="48" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A48" s="23" t="s">
         <v>4</v>
       </c>
@@ -1529,83 +1529,83 @@
       </c>
       <c r="G48" s="17"/>
     </row>
-    <row r="49" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="49" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A49" s="7">
-        <v>46275</v>
+        <v>46276</v>
       </c>
       <c r="B49" s="8"/>
       <c r="C49" s="20" t="s">
         <v>29</v>
       </c>
       <c r="D49" s="10">
-        <v>241.95</v>
+        <v>243.3</v>
       </c>
       <c r="E49" s="10">
-        <v>205.88</v>
+        <v>207.95</v>
       </c>
       <c r="F49" s="10">
-        <v>215.88</v>
+        <v>217.95</v>
       </c>
       <c r="G49" s="28"/>
     </row>
-    <row r="50" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="50" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A50" s="11">
-        <v>46275</v>
+        <v>46276</v>
       </c>
       <c r="B50" s="12"/>
       <c r="C50" s="21" t="s">
         <v>30</v>
       </c>
       <c r="D50" s="13">
-        <v>240.14</v>
+        <v>241.45</v>
       </c>
       <c r="E50" s="13">
-        <v>205.79</v>
+        <v>207.85</v>
       </c>
       <c r="F50" s="13">
-        <v>215.79</v>
+        <v>217.85</v>
       </c>
       <c r="G50" s="28"/>
     </row>
-    <row r="51" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="51" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A51" s="7">
-        <v>46274</v>
+        <v>46275</v>
       </c>
       <c r="B51" s="8"/>
       <c r="C51" s="20" t="s">
         <v>29</v>
       </c>
       <c r="D51" s="10">
-        <v>239.82</v>
+        <v>241.95</v>
       </c>
       <c r="E51" s="10">
-        <v>203.03</v>
+        <v>205.88</v>
       </c>
       <c r="F51" s="10">
-        <v>213.03</v>
+        <v>215.88</v>
       </c>
       <c r="G51" s="17"/>
     </row>
-    <row r="52" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="52" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A52" s="11">
-        <v>46274</v>
+        <v>46275</v>
       </c>
       <c r="B52" s="12"/>
       <c r="C52" s="21" t="s">
         <v>30</v>
       </c>
       <c r="D52" s="13">
-        <v>238.02</v>
+        <v>240.14</v>
       </c>
       <c r="E52" s="13">
-        <v>202.96</v>
+        <v>205.79</v>
       </c>
       <c r="F52" s="13">
-        <v>212.96</v>
+        <v>215.79</v>
       </c>
       <c r="G52" s="17"/>
     </row>
-    <row r="53" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="53" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A53" s="14"/>
       <c r="B53" s="14"/>
       <c r="C53" s="15"/>
@@ -1614,7 +1614,7 @@
       <c r="F53" s="16"/>
       <c r="G53" s="17"/>
     </row>
-    <row r="54" spans="1:7" ht="20.25" x14ac:dyDescent="0.25">
+    <row r="54" spans="1:7" ht="20" x14ac:dyDescent="0.35">
       <c r="A54" s="27" t="s">
         <v>31</v>
       </c>
@@ -1625,7 +1625,7 @@
       <c r="F54" s="17"/>
       <c r="G54" s="17"/>
     </row>
-    <row r="55" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="55" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A55" s="23" t="s">
         <v>4</v>
       </c>
@@ -1644,54 +1644,54 @@
       </c>
       <c r="G55" s="17"/>
     </row>
-    <row r="56" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="56" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A56" s="7">
-        <v>46275</v>
+        <v>46276</v>
       </c>
       <c r="B56" s="8"/>
       <c r="C56" s="20" t="s">
         <v>32</v>
       </c>
       <c r="D56" s="10">
-        <v>259.33</v>
+        <v>259.77</v>
       </c>
       <c r="E56" s="10">
-        <v>227</v>
+        <v>229.4</v>
       </c>
       <c r="F56" s="10">
-        <v>237</v>
+        <v>239.4</v>
       </c>
       <c r="G56" s="17"/>
     </row>
-    <row r="57" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="57" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A57" s="11">
-        <v>46275</v>
+        <v>46276</v>
       </c>
       <c r="B57" s="12"/>
       <c r="C57" s="21" t="s">
         <v>33</v>
       </c>
       <c r="D57" s="13">
-        <v>248.11</v>
+        <v>248.62</v>
       </c>
       <c r="E57" s="13">
-        <v>217.85</v>
+        <v>219.61</v>
       </c>
       <c r="F57" s="13">
-        <v>227.85</v>
+        <v>229.61</v>
       </c>
       <c r="G57" s="17"/>
     </row>
-    <row r="58" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="58" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A58" s="7">
-        <v>46275</v>
+        <v>46276</v>
       </c>
       <c r="B58" s="8"/>
       <c r="C58" s="20" t="s">
         <v>34</v>
       </c>
       <c r="D58" s="10">
-        <v>249.3</v>
+        <v>249.83</v>
       </c>
       <c r="E58" s="10" t="s">
         <v>18</v>
@@ -1701,111 +1701,111 @@
       </c>
       <c r="G58" s="17"/>
     </row>
-    <row r="59" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="59" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A59" s="11">
-        <v>46275</v>
+        <v>46276</v>
       </c>
       <c r="B59" s="12"/>
       <c r="C59" s="21" t="s">
         <v>35</v>
       </c>
       <c r="D59" s="13">
-        <v>246.12</v>
+        <v>246.47</v>
       </c>
       <c r="E59" s="13">
-        <v>212.24</v>
+        <v>214</v>
       </c>
       <c r="F59" s="13" t="s">
         <v>18</v>
       </c>
       <c r="G59" s="17"/>
     </row>
-    <row r="60" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="60" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A60" s="7">
-        <v>46275</v>
+        <v>46276</v>
       </c>
       <c r="B60" s="8"/>
       <c r="C60" s="20" t="s">
         <v>36</v>
       </c>
       <c r="D60" s="10">
-        <v>241.94</v>
+        <v>242.29</v>
       </c>
       <c r="E60" s="10">
-        <v>208.17</v>
+        <v>209.93</v>
       </c>
       <c r="F60" s="10">
-        <v>218.17</v>
+        <v>219.93</v>
       </c>
       <c r="G60" s="17"/>
     </row>
-    <row r="61" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="61" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A61" s="11">
-        <v>46275</v>
+        <v>46276</v>
       </c>
       <c r="B61" s="12"/>
       <c r="C61" s="21" t="s">
         <v>37</v>
       </c>
       <c r="D61" s="13">
-        <v>247.41</v>
+        <v>247.78</v>
       </c>
       <c r="E61" s="13">
-        <v>223.54</v>
+        <v>225.72</v>
       </c>
       <c r="F61" s="13" t="s">
         <v>18</v>
       </c>
       <c r="G61" s="17"/>
     </row>
-    <row r="62" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="62" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A62" s="7">
-        <v>46274</v>
+        <v>46275</v>
       </c>
       <c r="B62" s="8"/>
       <c r="C62" s="20" t="s">
         <v>32</v>
       </c>
       <c r="D62" s="10">
-        <v>257.60000000000002</v>
+        <v>259.33</v>
       </c>
       <c r="E62" s="10">
-        <v>223.66</v>
+        <v>227</v>
       </c>
       <c r="F62" s="10">
-        <v>233.66</v>
+        <v>237</v>
       </c>
       <c r="G62" s="17"/>
     </row>
-    <row r="63" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="63" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A63" s="11">
-        <v>46274</v>
+        <v>46275</v>
       </c>
       <c r="B63" s="12"/>
       <c r="C63" s="21" t="s">
         <v>33</v>
       </c>
       <c r="D63" s="13">
-        <v>246.33</v>
+        <v>248.11</v>
       </c>
       <c r="E63" s="13">
-        <v>215.16</v>
+        <v>217.85</v>
       </c>
       <c r="F63" s="13">
-        <v>225.16</v>
+        <v>227.85</v>
       </c>
       <c r="G63" s="17"/>
     </row>
-    <row r="64" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="64" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A64" s="7">
-        <v>46274</v>
+        <v>46275</v>
       </c>
       <c r="B64" s="8"/>
       <c r="C64" s="20" t="s">
         <v>34</v>
       </c>
       <c r="D64" s="10">
-        <v>247.49</v>
+        <v>249.3</v>
       </c>
       <c r="E64" s="10" t="s">
         <v>18</v>
@@ -1815,55 +1815,55 @@
       </c>
       <c r="G64" s="17"/>
     </row>
-    <row r="65" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="65" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A65" s="11">
-        <v>46274</v>
+        <v>46275</v>
       </c>
       <c r="B65" s="12"/>
       <c r="C65" s="21" t="s">
         <v>35</v>
       </c>
       <c r="D65" s="13">
-        <v>244.5</v>
+        <v>246.12</v>
       </c>
       <c r="E65" s="13">
-        <v>209.55</v>
+        <v>212.24</v>
       </c>
       <c r="F65" s="13" t="s">
         <v>18</v>
       </c>
     </row>
-    <row r="66" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="66" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A66" s="7">
-        <v>46274</v>
+        <v>46275</v>
       </c>
       <c r="B66" s="8"/>
       <c r="C66" s="20" t="s">
         <v>36</v>
       </c>
       <c r="D66" s="10">
-        <v>240.32</v>
+        <v>241.94</v>
       </c>
       <c r="E66" s="10">
-        <v>205.48</v>
+        <v>208.17</v>
       </c>
       <c r="F66" s="10">
-        <v>215.48</v>
-      </c>
-    </row>
-    <row r="67" spans="1:6" x14ac:dyDescent="0.25">
+        <v>218.17</v>
+      </c>
+    </row>
+    <row r="67" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A67" s="11">
-        <v>46274</v>
+        <v>46275</v>
       </c>
       <c r="B67" s="12"/>
       <c r="C67" s="21" t="s">
         <v>37</v>
       </c>
       <c r="D67" s="13">
-        <v>245.77</v>
+        <v>247.41</v>
       </c>
       <c r="E67" s="13">
-        <v>220.43</v>
+        <v>223.54</v>
       </c>
       <c r="F67" s="13" t="s">
         <v>18</v>
@@ -1891,15 +1891,6 @@
 </file>
 
 <file path=customXml/item1.xml><?xml version="1.0" encoding="utf-8"?>
-<?mso-contentType ?>
-<FormTemplates xmlns="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms">
-  <Display>DocumentLibraryForm</Display>
-  <Edit>DocumentLibraryForm</Edit>
-  <New>DocumentLibraryForm</New>
-</FormTemplates>
-</file>
-
-<file path=customXml/item2.xml><?xml version="1.0" encoding="utf-8"?>
 <p:properties xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls">
   <documentManagement>
     <lcf76f155ced4ddcb4097134ff3c332f xmlns="87276d81-85f4-4ef2-9e6e-55066304288f">
@@ -1910,7 +1901,7 @@
 </p:properties>
 </file>
 
-<file path=customXml/item3.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=customXml/item2.xml><?xml version="1.0" encoding="utf-8"?>
 <ct:contentTypeSchema xmlns:ct="http://schemas.microsoft.com/office/2006/metadata/contentType" xmlns:ma="http://schemas.microsoft.com/office/2006/metadata/properties/metaAttributes" ct:_="" ma:_="" ma:contentTypeName="Document" ma:contentTypeID="0x010100D3632DF5622958439304627C030B0427" ma:contentTypeVersion="18" ma:contentTypeDescription="Create a new document." ma:contentTypeScope="" ma:versionID="8c2ecbce386d6bac497f8eb2d8f0fb7a">
   <xsd:schema xmlns:xsd="http://www.w3.org/2001/XMLSchema" xmlns:xs="http://www.w3.org/2001/XMLSchema" xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:ns2="87276d81-85f4-4ef2-9e6e-55066304288f" xmlns:ns3="39e1dda6-d1d8-4c88-a3b9-f1abc1284bad" xmlns:ns4="b23b8984-eafa-4e79-985e-54f52f3da58e" targetNamespace="http://schemas.microsoft.com/office/2006/metadata/properties" ma:root="true" ma:fieldsID="4cfd0c2f651c1ce156ad4fcb44ea61dd" ns2:_="" ns3:_="" ns4:_="">
     <xsd:import namespace="87276d81-85f4-4ef2-9e6e-55066304288f"/>
@@ -2170,15 +2161,16 @@
 </ct:contentTypeSchema>
 </file>
 
-<file path=customXml/itemProps1.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{F60519E9-FD90-4339-869C-BC2F85719BB8}">
-  <ds:schemaRefs>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms"/>
-  </ds:schemaRefs>
-</ds:datastoreItem>
+<file path=customXml/item3.xml><?xml version="1.0" encoding="utf-8"?>
+<?mso-contentType ?>
+<FormTemplates xmlns="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms">
+  <Display>DocumentLibraryForm</Display>
+  <Edit>DocumentLibraryForm</Edit>
+  <New>DocumentLibraryForm</New>
+</FormTemplates>
 </file>
 
-<file path=customXml/itemProps2.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=customXml/itemProps1.xml><?xml version="1.0" encoding="utf-8"?>
 <ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{57A83D98-2BAE-4D83-823A-D31C464B620C}">
   <ds:schemaRefs>
     <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/properties"/>
@@ -2189,7 +2181,7 @@
 </ds:datastoreItem>
 </file>
 
-<file path=customXml/itemProps3.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=customXml/itemProps2.xml><?xml version="1.0" encoding="utf-8"?>
 <ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{B44E1863-2778-41F9-ACBA-48420F931671}">
   <ds:schemaRefs>
     <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/contentType"/>
@@ -2209,6 +2201,14 @@
 </ds:datastoreItem>
 </file>
 
+<file path=customXml/itemProps3.xml><?xml version="1.0" encoding="utf-8"?>
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{F60519E9-FD90-4339-869C-BC2F85719BB8}">
+  <ds:schemaRefs>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms"/>
+  </ds:schemaRefs>
+</ds:datastoreItem>
+</file>
+
 <file path=docMetadata/LabelInfo.xml><?xml version="1.0" encoding="utf-8"?>
 <clbl:labelList xmlns:clbl="http://schemas.microsoft.com/office/2020/mipLabelMetadata">
   <clbl:label id="{569bf4a9-87bd-4dbf-a36c-1db5158e5def}" enabled="1" method="Privileged" siteId="{ea80952e-a476-42d4-aaf4-5457852b0f7e}" removed="0"/>

</xml_diff>

<commit_message>
Fri Sep 11 06:08:02 UTC 2026
</commit_message>
<xml_diff>
--- a/bp.com-content-dam-bp-country-sites-en_au-australia-home-products-services-pricing-tgp-excel.xlsx
+++ b/bp.com-content-dam-bp-country-sites-en_au-australia-home-products-services-pricing-tgp-excel.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://bp365.sharepoint.com/sites/WholesalePricing/Shared Documents/B2C/TGP/Daily TGP/Web TGP/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="14_{02604CF4-5B85-4EA0-B24E-C4B315B59949}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="14_{6C331202-AF67-47AC-A154-B283B6CD85AE}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-110" yWindow="-110" windowWidth="19420" windowHeight="11500" xr2:uid="{1B412EEF-F96D-4DF4-A4E9-C7F0F183C2FB}"/>
+    <workbookView xWindow="1470" yWindow="1470" windowWidth="13958" windowHeight="9142" xr2:uid="{1B412EEF-F96D-4DF4-A4E9-C7F0F183C2FB}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
@@ -715,15 +715,15 @@
     <pageSetUpPr fitToPage="1"/>
   </sheetPr>
   <dimension ref="A1:G67"/>
-  <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
+  <sheetFormatPr defaultRowHeight="14.25" x14ac:dyDescent="0.45"/>
   <cols>
-    <col min="1" max="1" width="76.453125" bestFit="1" customWidth="1"/>
-    <col min="2" max="2" width="6.453125"/>
-    <col min="3" max="3" width="18.1796875" bestFit="1" customWidth="1"/>
-    <col min="4" max="7" width="7.1796875" bestFit="1" customWidth="1"/>
+    <col min="1" max="1" width="76.46484375" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="6.46484375"/>
+    <col min="3" max="3" width="18.19921875" bestFit="1" customWidth="1"/>
+    <col min="4" max="7" width="7.19921875" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:7" ht="22.5" x14ac:dyDescent="0.35">
+    <row r="1" spans="1:7" ht="22.15" x14ac:dyDescent="0.45">
       <c r="A1" s="30" t="s">
         <v>0</v>
       </c>
@@ -734,7 +734,7 @@
       <c r="F1" s="2"/>
       <c r="G1" s="2"/>
     </row>
-    <row r="2" spans="1:7" x14ac:dyDescent="0.35">
+    <row r="2" spans="1:7" x14ac:dyDescent="0.45">
       <c r="A2" s="3"/>
       <c r="B2" s="1"/>
       <c r="C2" s="1"/>
@@ -743,7 +743,7 @@
       <c r="F2" s="2"/>
       <c r="G2" s="2"/>
     </row>
-    <row r="3" spans="1:7" x14ac:dyDescent="0.35">
+    <row r="3" spans="1:7" x14ac:dyDescent="0.45">
       <c r="A3" s="3" t="s">
         <v>1</v>
       </c>
@@ -754,7 +754,7 @@
       <c r="F3" s="2"/>
       <c r="G3" s="2"/>
     </row>
-    <row r="4" spans="1:7" x14ac:dyDescent="0.35">
+    <row r="4" spans="1:7" x14ac:dyDescent="0.45">
       <c r="A4" s="3" t="s">
         <v>2</v>
       </c>
@@ -765,7 +765,7 @@
       <c r="F4" s="2"/>
       <c r="G4" s="2"/>
     </row>
-    <row r="5" spans="1:7" x14ac:dyDescent="0.35">
+    <row r="5" spans="1:7" x14ac:dyDescent="0.45">
       <c r="A5" s="3"/>
       <c r="B5" s="3"/>
       <c r="C5" s="1"/>
@@ -774,7 +774,7 @@
       <c r="F5" s="2"/>
       <c r="G5" s="2"/>
     </row>
-    <row r="6" spans="1:7" ht="20" x14ac:dyDescent="0.35">
+    <row r="6" spans="1:7" ht="20.25" x14ac:dyDescent="0.45">
       <c r="A6" s="29" t="s">
         <v>3</v>
       </c>
@@ -785,7 +785,7 @@
       <c r="F6" s="2"/>
       <c r="G6" s="2"/>
     </row>
-    <row r="7" spans="1:7" x14ac:dyDescent="0.35">
+    <row r="7" spans="1:7" x14ac:dyDescent="0.45">
       <c r="A7" s="4" t="s">
         <v>4</v>
       </c>
@@ -806,133 +806,133 @@
         <v>9</v>
       </c>
     </row>
-    <row r="8" spans="1:7" x14ac:dyDescent="0.35">
+    <row r="8" spans="1:7" x14ac:dyDescent="0.45">
       <c r="A8" s="7">
-        <v>46276</v>
+        <v>46277</v>
       </c>
       <c r="B8" s="8"/>
       <c r="C8" s="9" t="s">
         <v>10</v>
       </c>
       <c r="D8" s="10">
-        <v>246.84</v>
+        <v>247.73</v>
       </c>
       <c r="E8" s="10">
-        <v>212.58</v>
+        <v>214.55</v>
       </c>
       <c r="F8" s="10">
-        <v>222.58</v>
+        <v>224.55</v>
       </c>
       <c r="G8" s="10">
-        <v>212.54</v>
-      </c>
-    </row>
-    <row r="9" spans="1:7" x14ac:dyDescent="0.35">
+        <v>214.52</v>
+      </c>
+    </row>
+    <row r="9" spans="1:7" x14ac:dyDescent="0.45">
       <c r="A9" s="11">
-        <v>46276</v>
+        <v>46277</v>
       </c>
       <c r="B9" s="12"/>
       <c r="C9" s="12" t="s">
         <v>11</v>
       </c>
       <c r="D9" s="13">
-        <v>246.84</v>
+        <v>247.73</v>
       </c>
       <c r="E9" s="13">
-        <v>212.58</v>
+        <v>214.55</v>
       </c>
       <c r="F9" s="13">
-        <v>222.58</v>
+        <v>224.55</v>
       </c>
       <c r="G9" s="13">
-        <v>212.54</v>
-      </c>
-    </row>
-    <row r="10" spans="1:7" x14ac:dyDescent="0.35">
+        <v>214.52</v>
+      </c>
+    </row>
+    <row r="10" spans="1:7" x14ac:dyDescent="0.45">
       <c r="A10" s="7">
-        <v>46276</v>
+        <v>46277</v>
       </c>
       <c r="B10" s="8"/>
       <c r="C10" s="9" t="s">
         <v>12</v>
       </c>
       <c r="D10" s="10">
-        <v>243.05</v>
+        <v>243.64</v>
       </c>
       <c r="E10" s="10">
-        <v>209.64</v>
+        <v>211.35</v>
       </c>
       <c r="F10" s="10">
-        <v>219.64</v>
+        <v>221.35</v>
       </c>
       <c r="G10" s="10">
-        <v>210.06</v>
-      </c>
-    </row>
-    <row r="11" spans="1:7" x14ac:dyDescent="0.35">
+        <v>211.77</v>
+      </c>
+    </row>
+    <row r="11" spans="1:7" x14ac:dyDescent="0.45">
       <c r="A11" s="11">
-        <v>46275</v>
+        <v>46276</v>
       </c>
       <c r="B11" s="12"/>
       <c r="C11" s="12" t="s">
         <v>10</v>
       </c>
       <c r="D11" s="13">
-        <v>246.08</v>
+        <v>246.84</v>
       </c>
       <c r="E11" s="13">
-        <v>210.46</v>
+        <v>212.58</v>
       </c>
       <c r="F11" s="13">
-        <v>220.46</v>
+        <v>222.58</v>
       </c>
       <c r="G11" s="13">
-        <v>210.43</v>
-      </c>
-    </row>
-    <row r="12" spans="1:7" x14ac:dyDescent="0.35">
+        <v>212.54</v>
+      </c>
+    </row>
+    <row r="12" spans="1:7" x14ac:dyDescent="0.45">
       <c r="A12" s="7">
-        <v>46275</v>
+        <v>46276</v>
       </c>
       <c r="B12" s="8"/>
       <c r="C12" s="9" t="s">
         <v>11</v>
       </c>
       <c r="D12" s="10">
-        <v>246.08</v>
+        <v>246.84</v>
       </c>
       <c r="E12" s="10">
-        <v>210.46</v>
+        <v>212.58</v>
       </c>
       <c r="F12" s="10">
-        <v>220.46</v>
+        <v>222.58</v>
       </c>
       <c r="G12" s="10">
-        <v>210.43</v>
-      </c>
-    </row>
-    <row r="13" spans="1:7" x14ac:dyDescent="0.35">
+        <v>212.54</v>
+      </c>
+    </row>
+    <row r="13" spans="1:7" x14ac:dyDescent="0.45">
       <c r="A13" s="11">
-        <v>46275</v>
+        <v>46276</v>
       </c>
       <c r="B13" s="12"/>
       <c r="C13" s="12" t="s">
         <v>12</v>
       </c>
       <c r="D13" s="13">
-        <v>242.55</v>
+        <v>243.05</v>
       </c>
       <c r="E13" s="13">
-        <v>207.74</v>
+        <v>209.64</v>
       </c>
       <c r="F13" s="13">
-        <v>217.75</v>
+        <v>219.64</v>
       </c>
       <c r="G13" s="13">
-        <v>208.16</v>
-      </c>
-    </row>
-    <row r="14" spans="1:7" x14ac:dyDescent="0.35">
+        <v>210.06</v>
+      </c>
+    </row>
+    <row r="14" spans="1:7" x14ac:dyDescent="0.45">
       <c r="A14" s="14"/>
       <c r="B14" s="14"/>
       <c r="C14" s="15"/>
@@ -941,7 +941,7 @@
       <c r="F14" s="16"/>
       <c r="G14" s="16"/>
     </row>
-    <row r="15" spans="1:7" ht="20" x14ac:dyDescent="0.35">
+    <row r="15" spans="1:7" ht="20.25" x14ac:dyDescent="0.45">
       <c r="A15" s="29" t="s">
         <v>13</v>
       </c>
@@ -952,7 +952,7 @@
       <c r="F15" s="17"/>
       <c r="G15" s="17"/>
     </row>
-    <row r="16" spans="1:7" x14ac:dyDescent="0.35">
+    <row r="16" spans="1:7" x14ac:dyDescent="0.45">
       <c r="A16" s="4" t="s">
         <v>4</v>
       </c>
@@ -971,45 +971,45 @@
       </c>
       <c r="G16" s="17"/>
     </row>
-    <row r="17" spans="1:7" x14ac:dyDescent="0.35">
+    <row r="17" spans="1:7" x14ac:dyDescent="0.45">
       <c r="A17" s="7">
-        <v>46276</v>
+        <v>46277</v>
       </c>
       <c r="B17" s="8"/>
       <c r="C17" s="20" t="s">
         <v>14</v>
       </c>
       <c r="D17" s="10">
-        <v>248.19</v>
+        <v>248.67</v>
       </c>
       <c r="E17" s="10">
-        <v>214.05</v>
+        <v>215.66</v>
       </c>
       <c r="F17" s="10">
-        <v>224.05</v>
+        <v>225.66</v>
       </c>
       <c r="G17" s="17"/>
     </row>
-    <row r="18" spans="1:7" x14ac:dyDescent="0.35">
+    <row r="18" spans="1:7" x14ac:dyDescent="0.45">
       <c r="A18" s="11">
-        <v>46275</v>
+        <v>46276</v>
       </c>
       <c r="B18" s="12"/>
       <c r="C18" s="12" t="s">
         <v>14</v>
       </c>
       <c r="D18" s="13">
-        <v>247.81</v>
+        <v>248.19</v>
       </c>
       <c r="E18" s="13">
-        <v>212.26</v>
+        <v>214.05</v>
       </c>
       <c r="F18" s="13">
-        <v>222.26</v>
+        <v>224.05</v>
       </c>
       <c r="G18" s="17"/>
     </row>
-    <row r="19" spans="1:7" x14ac:dyDescent="0.35">
+    <row r="19" spans="1:7" x14ac:dyDescent="0.45">
       <c r="A19" s="14"/>
       <c r="B19" s="14"/>
       <c r="C19" s="15"/>
@@ -1018,7 +1018,7 @@
       <c r="F19" s="16"/>
       <c r="G19" s="17"/>
     </row>
-    <row r="20" spans="1:7" ht="20" x14ac:dyDescent="0.35">
+    <row r="20" spans="1:7" ht="20.25" x14ac:dyDescent="0.45">
       <c r="A20" s="29" t="s">
         <v>15</v>
       </c>
@@ -1029,7 +1029,7 @@
       <c r="F20" s="17"/>
       <c r="G20" s="17"/>
     </row>
-    <row r="21" spans="1:7" x14ac:dyDescent="0.35">
+    <row r="21" spans="1:7" x14ac:dyDescent="0.45">
       <c r="A21" s="4" t="s">
         <v>4</v>
       </c>
@@ -1050,217 +1050,217 @@
         <v>9</v>
       </c>
     </row>
-    <row r="22" spans="1:7" x14ac:dyDescent="0.35">
+    <row r="22" spans="1:7" x14ac:dyDescent="0.45">
       <c r="A22" s="7">
-        <v>46276</v>
+        <v>46277</v>
       </c>
       <c r="B22" s="8"/>
       <c r="C22" s="20" t="s">
         <v>16</v>
       </c>
       <c r="D22" s="10">
-        <v>247.97</v>
+        <v>248.86</v>
       </c>
       <c r="E22" s="10">
-        <v>213.28</v>
+        <v>215.25</v>
       </c>
       <c r="F22" s="10">
-        <v>222.88</v>
+        <v>224.85</v>
       </c>
       <c r="G22" s="10">
-        <v>211.99</v>
-      </c>
-    </row>
-    <row r="23" spans="1:7" x14ac:dyDescent="0.35">
+        <v>213.97</v>
+      </c>
+    </row>
+    <row r="23" spans="1:7" x14ac:dyDescent="0.45">
       <c r="A23" s="11">
-        <v>46276</v>
+        <v>46277</v>
       </c>
       <c r="B23" s="12"/>
       <c r="C23" s="21" t="s">
         <v>17</v>
       </c>
       <c r="D23" s="13">
-        <v>247.79</v>
+        <v>248.4</v>
       </c>
       <c r="E23" s="13">
-        <v>217.23</v>
+        <v>218.99</v>
       </c>
       <c r="F23" s="13">
-        <v>227.23</v>
+        <v>228.99</v>
       </c>
       <c r="G23" s="13" t="s">
         <v>18</v>
       </c>
     </row>
-    <row r="24" spans="1:7" x14ac:dyDescent="0.35">
+    <row r="24" spans="1:7" x14ac:dyDescent="0.45">
       <c r="A24" s="7">
-        <v>46276</v>
+        <v>46277</v>
       </c>
       <c r="B24" s="8"/>
       <c r="C24" s="20" t="s">
         <v>19</v>
       </c>
       <c r="D24" s="10">
-        <v>248.34</v>
+        <v>248.94</v>
       </c>
       <c r="E24" s="10">
-        <v>216.53</v>
+        <v>218.29</v>
       </c>
       <c r="F24" s="10">
-        <v>226.53</v>
+        <v>228.29</v>
       </c>
       <c r="G24" s="10" t="s">
         <v>18</v>
       </c>
     </row>
-    <row r="25" spans="1:7" x14ac:dyDescent="0.35">
+    <row r="25" spans="1:7" x14ac:dyDescent="0.45">
       <c r="A25" s="11">
-        <v>46276</v>
+        <v>46277</v>
       </c>
       <c r="B25" s="12"/>
       <c r="C25" s="21" t="s">
         <v>20</v>
       </c>
       <c r="D25" s="13">
-        <v>245.13</v>
+        <v>245.73</v>
       </c>
       <c r="E25" s="13">
-        <v>216.55</v>
+        <v>218.32</v>
       </c>
       <c r="F25" s="13">
-        <v>226.55</v>
+        <v>228.32</v>
       </c>
       <c r="G25" s="13">
-        <v>214.45</v>
-      </c>
-    </row>
-    <row r="26" spans="1:7" x14ac:dyDescent="0.35">
+        <v>216.21</v>
+      </c>
+    </row>
+    <row r="26" spans="1:7" x14ac:dyDescent="0.45">
       <c r="A26" s="7">
-        <v>46276</v>
+        <v>46277</v>
       </c>
       <c r="B26" s="8"/>
       <c r="C26" s="20" t="s">
         <v>21</v>
       </c>
       <c r="D26" s="10">
-        <v>246.98</v>
+        <v>247.54</v>
       </c>
       <c r="E26" s="10">
-        <v>217.89</v>
+        <v>219.67</v>
       </c>
       <c r="F26" s="10">
-        <v>227.89</v>
+        <v>229.67</v>
       </c>
       <c r="G26" s="10" t="s">
         <v>18</v>
       </c>
     </row>
-    <row r="27" spans="1:7" x14ac:dyDescent="0.35">
+    <row r="27" spans="1:7" x14ac:dyDescent="0.45">
       <c r="A27" s="11">
-        <v>46275</v>
+        <v>46276</v>
       </c>
       <c r="B27" s="12"/>
       <c r="C27" s="12" t="s">
         <v>16</v>
       </c>
       <c r="D27" s="13">
-        <v>247.22</v>
+        <v>247.97</v>
       </c>
       <c r="E27" s="13">
-        <v>211.16</v>
+        <v>213.28</v>
       </c>
       <c r="F27" s="13">
-        <v>220.76</v>
+        <v>222.88</v>
       </c>
       <c r="G27" s="13">
-        <v>209.88</v>
-      </c>
-    </row>
-    <row r="28" spans="1:7" x14ac:dyDescent="0.35">
+        <v>211.99</v>
+      </c>
+    </row>
+    <row r="28" spans="1:7" x14ac:dyDescent="0.45">
       <c r="A28" s="7">
-        <v>46275</v>
+        <v>46276</v>
       </c>
       <c r="B28" s="8"/>
       <c r="C28" s="20" t="s">
         <v>17</v>
       </c>
       <c r="D28" s="10">
-        <v>247.28</v>
+        <v>247.79</v>
       </c>
       <c r="E28" s="22">
-        <v>215.29</v>
+        <v>217.23</v>
       </c>
       <c r="F28" s="22">
-        <v>225.29</v>
+        <v>227.23</v>
       </c>
       <c r="G28" s="22" t="s">
         <v>18</v>
       </c>
     </row>
-    <row r="29" spans="1:7" x14ac:dyDescent="0.35">
+    <row r="29" spans="1:7" x14ac:dyDescent="0.45">
       <c r="A29" s="11">
-        <v>46275</v>
+        <v>46276</v>
       </c>
       <c r="B29" s="12"/>
       <c r="C29" s="12" t="s">
         <v>19</v>
       </c>
       <c r="D29" s="13">
-        <v>247.85</v>
+        <v>248.34</v>
       </c>
       <c r="E29" s="13">
-        <v>214.6</v>
+        <v>216.53</v>
       </c>
       <c r="F29" s="13">
-        <v>224.6</v>
+        <v>226.53</v>
       </c>
       <c r="G29" s="13" t="s">
         <v>18</v>
       </c>
     </row>
-    <row r="30" spans="1:7" x14ac:dyDescent="0.35">
+    <row r="30" spans="1:7" x14ac:dyDescent="0.45">
       <c r="A30" s="7">
-        <v>46275</v>
+        <v>46276</v>
       </c>
       <c r="B30" s="8"/>
       <c r="C30" s="20" t="s">
         <v>20</v>
       </c>
       <c r="D30" s="10">
-        <v>244.62</v>
+        <v>245.13</v>
       </c>
       <c r="E30" s="22">
-        <v>214.6</v>
+        <v>216.55</v>
       </c>
       <c r="F30" s="22">
-        <v>224.6</v>
+        <v>226.55</v>
       </c>
       <c r="G30" s="22">
-        <v>212.49</v>
-      </c>
-    </row>
-    <row r="31" spans="1:7" x14ac:dyDescent="0.35">
+        <v>214.45</v>
+      </c>
+    </row>
+    <row r="31" spans="1:7" x14ac:dyDescent="0.45">
       <c r="A31" s="11">
-        <v>46275</v>
+        <v>46276</v>
       </c>
       <c r="B31" s="12"/>
       <c r="C31" s="12" t="s">
         <v>21</v>
       </c>
       <c r="D31" s="13">
-        <v>246.51</v>
+        <v>246.98</v>
       </c>
       <c r="E31" s="13">
-        <v>215.92</v>
+        <v>217.89</v>
       </c>
       <c r="F31" s="13">
-        <v>225.92</v>
+        <v>227.89</v>
       </c>
       <c r="G31" s="13" t="s">
         <v>18</v>
       </c>
     </row>
-    <row r="32" spans="1:7" x14ac:dyDescent="0.35">
+    <row r="32" spans="1:7" x14ac:dyDescent="0.45">
       <c r="A32" s="14"/>
       <c r="B32" s="14"/>
       <c r="C32" s="15"/>
@@ -1269,7 +1269,7 @@
       <c r="F32" s="17"/>
       <c r="G32" s="17"/>
     </row>
-    <row r="33" spans="1:7" ht="20" x14ac:dyDescent="0.35">
+    <row r="33" spans="1:7" ht="20.25" x14ac:dyDescent="0.45">
       <c r="A33" s="29" t="s">
         <v>22</v>
       </c>
@@ -1280,7 +1280,7 @@
       <c r="F33" s="17"/>
       <c r="G33" s="17"/>
     </row>
-    <row r="34" spans="1:7" x14ac:dyDescent="0.35">
+    <row r="34" spans="1:7" x14ac:dyDescent="0.45">
       <c r="A34" s="23" t="s">
         <v>4</v>
       </c>
@@ -1299,54 +1299,54 @@
       </c>
       <c r="G34" s="17"/>
     </row>
-    <row r="35" spans="1:7" x14ac:dyDescent="0.35">
+    <row r="35" spans="1:7" x14ac:dyDescent="0.45">
       <c r="A35" s="7">
-        <v>46276</v>
+        <v>46277</v>
       </c>
       <c r="B35" s="8"/>
       <c r="C35" s="20" t="s">
         <v>23</v>
       </c>
       <c r="D35" s="10">
-        <v>241.58</v>
+        <v>242.18</v>
       </c>
       <c r="E35" s="10">
-        <v>208.6</v>
+        <v>210.31</v>
       </c>
       <c r="F35" s="10">
-        <v>217.6</v>
+        <v>219.31</v>
       </c>
       <c r="G35" s="17"/>
     </row>
-    <row r="36" spans="1:7" x14ac:dyDescent="0.35">
+    <row r="36" spans="1:7" x14ac:dyDescent="0.45">
       <c r="A36" s="11">
-        <v>46275</v>
+        <v>46276</v>
       </c>
       <c r="B36" s="12"/>
       <c r="C36" s="12" t="s">
         <v>23</v>
       </c>
       <c r="D36" s="13">
-        <v>241.07</v>
+        <v>241.58</v>
       </c>
       <c r="E36" s="13">
-        <v>206.7</v>
+        <v>208.6</v>
       </c>
       <c r="F36" s="13">
-        <v>215.7</v>
+        <v>217.6</v>
       </c>
       <c r="G36" s="17"/>
     </row>
-    <row r="37" spans="1:7" x14ac:dyDescent="0.35">
+    <row r="37" spans="1:7" x14ac:dyDescent="0.45">
       <c r="A37" s="7">
-        <v>46276</v>
+        <v>46277</v>
       </c>
       <c r="B37" s="8"/>
       <c r="C37" s="20" t="s">
         <v>24</v>
       </c>
       <c r="D37" s="10">
-        <v>257.2</v>
+        <v>257.8</v>
       </c>
       <c r="E37" s="10" t="s">
         <v>18</v>
@@ -1356,16 +1356,16 @@
       </c>
       <c r="G37" s="17"/>
     </row>
-    <row r="38" spans="1:7" x14ac:dyDescent="0.35">
+    <row r="38" spans="1:7" x14ac:dyDescent="0.45">
       <c r="A38" s="11">
-        <v>46275</v>
+        <v>46276</v>
       </c>
       <c r="B38" s="12"/>
       <c r="C38" s="12" t="s">
         <v>24</v>
       </c>
       <c r="D38" s="13">
-        <v>256.69</v>
+        <v>257.2</v>
       </c>
       <c r="E38" s="13" t="s">
         <v>18</v>
@@ -1375,7 +1375,7 @@
       </c>
       <c r="G38" s="17"/>
     </row>
-    <row r="39" spans="1:7" x14ac:dyDescent="0.35">
+    <row r="39" spans="1:7" x14ac:dyDescent="0.45">
       <c r="A39" s="24"/>
       <c r="B39" s="24"/>
       <c r="C39" s="15"/>
@@ -1384,7 +1384,7 @@
       <c r="F39" s="17"/>
       <c r="G39" s="17"/>
     </row>
-    <row r="40" spans="1:7" ht="20" x14ac:dyDescent="0.35">
+    <row r="40" spans="1:7" ht="20.25" x14ac:dyDescent="0.45">
       <c r="A40" s="29" t="s">
         <v>25</v>
       </c>
@@ -1395,7 +1395,7 @@
       <c r="F40" s="17"/>
       <c r="G40" s="17"/>
     </row>
-    <row r="41" spans="1:7" x14ac:dyDescent="0.35">
+    <row r="41" spans="1:7" x14ac:dyDescent="0.45">
       <c r="A41" s="23" t="s">
         <v>4</v>
       </c>
@@ -1414,83 +1414,83 @@
       </c>
       <c r="G41" s="17"/>
     </row>
-    <row r="42" spans="1:7" x14ac:dyDescent="0.35">
+    <row r="42" spans="1:7" x14ac:dyDescent="0.45">
       <c r="A42" s="7">
-        <v>46276</v>
+        <v>46277</v>
       </c>
       <c r="B42" s="8"/>
       <c r="C42" s="20" t="s">
         <v>26</v>
       </c>
       <c r="D42" s="10">
-        <v>250.28</v>
+        <v>250.97</v>
       </c>
       <c r="E42" s="10">
-        <v>214.96</v>
+        <v>216.78</v>
       </c>
       <c r="F42" s="10">
-        <v>224.96</v>
+        <v>226.78</v>
       </c>
       <c r="G42" s="17"/>
     </row>
-    <row r="43" spans="1:7" x14ac:dyDescent="0.35">
+    <row r="43" spans="1:7" x14ac:dyDescent="0.45">
       <c r="A43" s="11">
-        <v>46276</v>
+        <v>46277</v>
       </c>
       <c r="B43" s="12"/>
       <c r="C43" s="21" t="s">
         <v>27</v>
       </c>
       <c r="D43" s="13">
-        <v>249.9</v>
+        <v>250.59</v>
       </c>
       <c r="E43" s="13">
-        <v>215.37</v>
+        <v>217.2</v>
       </c>
       <c r="F43" s="13">
-        <v>225.37</v>
+        <v>227.2</v>
       </c>
       <c r="G43" s="17"/>
     </row>
-    <row r="44" spans="1:7" x14ac:dyDescent="0.35">
+    <row r="44" spans="1:7" x14ac:dyDescent="0.45">
       <c r="A44" s="7">
-        <v>46275</v>
+        <v>46276</v>
       </c>
       <c r="B44" s="8"/>
       <c r="C44" s="20" t="s">
         <v>26</v>
       </c>
       <c r="D44" s="10">
-        <v>249.68</v>
+        <v>250.28</v>
       </c>
       <c r="E44" s="10">
-        <v>212.95</v>
+        <v>214.96</v>
       </c>
       <c r="F44" s="10">
-        <v>222.95</v>
+        <v>224.96</v>
       </c>
       <c r="G44" s="17"/>
     </row>
-    <row r="45" spans="1:7" x14ac:dyDescent="0.35">
+    <row r="45" spans="1:7" x14ac:dyDescent="0.45">
       <c r="A45" s="11">
-        <v>46275</v>
+        <v>46276</v>
       </c>
       <c r="B45" s="12"/>
       <c r="C45" s="21" t="s">
         <v>27</v>
       </c>
       <c r="D45" s="13">
-        <v>249.31</v>
+        <v>249.9</v>
       </c>
       <c r="E45" s="13">
-        <v>213.37</v>
+        <v>215.37</v>
       </c>
       <c r="F45" s="13">
-        <v>223.37</v>
+        <v>225.37</v>
       </c>
       <c r="G45" s="17"/>
     </row>
-    <row r="46" spans="1:7" x14ac:dyDescent="0.35">
+    <row r="46" spans="1:7" x14ac:dyDescent="0.45">
       <c r="A46" s="14"/>
       <c r="B46" s="24"/>
       <c r="C46" s="15"/>
@@ -1499,7 +1499,7 @@
       <c r="F46" s="16"/>
       <c r="G46" s="17"/>
     </row>
-    <row r="47" spans="1:7" ht="20" x14ac:dyDescent="0.35">
+    <row r="47" spans="1:7" ht="20.25" x14ac:dyDescent="0.45">
       <c r="A47" s="25" t="s">
         <v>28</v>
       </c>
@@ -1510,7 +1510,7 @@
       <c r="F47" s="17"/>
       <c r="G47" s="17"/>
     </row>
-    <row r="48" spans="1:7" x14ac:dyDescent="0.35">
+    <row r="48" spans="1:7" x14ac:dyDescent="0.45">
       <c r="A48" s="23" t="s">
         <v>4</v>
       </c>
@@ -1529,83 +1529,83 @@
       </c>
       <c r="G48" s="17"/>
     </row>
-    <row r="49" spans="1:7" x14ac:dyDescent="0.35">
+    <row r="49" spans="1:7" x14ac:dyDescent="0.45">
       <c r="A49" s="7">
-        <v>46276</v>
+        <v>46277</v>
       </c>
       <c r="B49" s="8"/>
       <c r="C49" s="20" t="s">
         <v>29</v>
       </c>
       <c r="D49" s="10">
-        <v>243.3</v>
+        <v>244</v>
       </c>
       <c r="E49" s="10">
-        <v>207.95</v>
+        <v>209.95</v>
       </c>
       <c r="F49" s="10">
-        <v>217.95</v>
+        <v>219.95</v>
       </c>
       <c r="G49" s="28"/>
     </row>
-    <row r="50" spans="1:7" x14ac:dyDescent="0.35">
+    <row r="50" spans="1:7" x14ac:dyDescent="0.45">
       <c r="A50" s="11">
-        <v>46276</v>
+        <v>46277</v>
       </c>
       <c r="B50" s="12"/>
       <c r="C50" s="21" t="s">
         <v>30</v>
       </c>
       <c r="D50" s="13">
-        <v>241.45</v>
+        <v>242.12</v>
       </c>
       <c r="E50" s="13">
-        <v>207.85</v>
+        <v>209.84</v>
       </c>
       <c r="F50" s="13">
-        <v>217.85</v>
+        <v>219.84</v>
       </c>
       <c r="G50" s="28"/>
     </row>
-    <row r="51" spans="1:7" x14ac:dyDescent="0.35">
+    <row r="51" spans="1:7" x14ac:dyDescent="0.45">
       <c r="A51" s="7">
-        <v>46275</v>
+        <v>46276</v>
       </c>
       <c r="B51" s="8"/>
       <c r="C51" s="20" t="s">
         <v>29</v>
       </c>
       <c r="D51" s="10">
-        <v>241.95</v>
+        <v>243.3</v>
       </c>
       <c r="E51" s="10">
-        <v>205.88</v>
+        <v>207.95</v>
       </c>
       <c r="F51" s="10">
-        <v>215.88</v>
+        <v>217.95</v>
       </c>
       <c r="G51" s="17"/>
     </row>
-    <row r="52" spans="1:7" x14ac:dyDescent="0.35">
+    <row r="52" spans="1:7" x14ac:dyDescent="0.45">
       <c r="A52" s="11">
-        <v>46275</v>
+        <v>46276</v>
       </c>
       <c r="B52" s="12"/>
       <c r="C52" s="21" t="s">
         <v>30</v>
       </c>
       <c r="D52" s="13">
-        <v>240.14</v>
+        <v>241.45</v>
       </c>
       <c r="E52" s="13">
-        <v>205.79</v>
+        <v>207.85</v>
       </c>
       <c r="F52" s="13">
-        <v>215.79</v>
+        <v>217.85</v>
       </c>
       <c r="G52" s="17"/>
     </row>
-    <row r="53" spans="1:7" x14ac:dyDescent="0.35">
+    <row r="53" spans="1:7" x14ac:dyDescent="0.45">
       <c r="A53" s="14"/>
       <c r="B53" s="14"/>
       <c r="C53" s="15"/>
@@ -1614,7 +1614,7 @@
       <c r="F53" s="16"/>
       <c r="G53" s="17"/>
     </row>
-    <row r="54" spans="1:7" ht="20" x14ac:dyDescent="0.35">
+    <row r="54" spans="1:7" ht="20.25" x14ac:dyDescent="0.45">
       <c r="A54" s="27" t="s">
         <v>31</v>
       </c>
@@ -1625,7 +1625,7 @@
       <c r="F54" s="17"/>
       <c r="G54" s="17"/>
     </row>
-    <row r="55" spans="1:7" x14ac:dyDescent="0.35">
+    <row r="55" spans="1:7" x14ac:dyDescent="0.45">
       <c r="A55" s="23" t="s">
         <v>4</v>
       </c>
@@ -1644,54 +1644,54 @@
       </c>
       <c r="G55" s="17"/>
     </row>
-    <row r="56" spans="1:7" x14ac:dyDescent="0.35">
+    <row r="56" spans="1:7" x14ac:dyDescent="0.45">
       <c r="A56" s="7">
-        <v>46276</v>
+        <v>46277</v>
       </c>
       <c r="B56" s="8"/>
       <c r="C56" s="20" t="s">
         <v>32</v>
       </c>
       <c r="D56" s="10">
-        <v>259.77</v>
+        <v>260.32</v>
       </c>
       <c r="E56" s="10">
-        <v>229.4</v>
+        <v>231.62</v>
       </c>
       <c r="F56" s="10">
-        <v>239.4</v>
+        <v>241.62</v>
       </c>
       <c r="G56" s="17"/>
     </row>
-    <row r="57" spans="1:7" x14ac:dyDescent="0.35">
+    <row r="57" spans="1:7" x14ac:dyDescent="0.45">
       <c r="A57" s="11">
-        <v>46276</v>
+        <v>46277</v>
       </c>
       <c r="B57" s="12"/>
       <c r="C57" s="21" t="s">
         <v>33</v>
       </c>
       <c r="D57" s="13">
-        <v>248.62</v>
+        <v>249.22</v>
       </c>
       <c r="E57" s="13">
-        <v>219.61</v>
+        <v>221.19</v>
       </c>
       <c r="F57" s="13">
-        <v>229.61</v>
+        <v>231.19</v>
       </c>
       <c r="G57" s="17"/>
     </row>
-    <row r="58" spans="1:7" x14ac:dyDescent="0.35">
+    <row r="58" spans="1:7" x14ac:dyDescent="0.45">
       <c r="A58" s="7">
-        <v>46276</v>
+        <v>46277</v>
       </c>
       <c r="B58" s="8"/>
       <c r="C58" s="20" t="s">
         <v>34</v>
       </c>
       <c r="D58" s="10">
-        <v>249.83</v>
+        <v>250.45</v>
       </c>
       <c r="E58" s="10" t="s">
         <v>18</v>
@@ -1701,111 +1701,111 @@
       </c>
       <c r="G58" s="17"/>
     </row>
-    <row r="59" spans="1:7" x14ac:dyDescent="0.35">
+    <row r="59" spans="1:7" x14ac:dyDescent="0.45">
       <c r="A59" s="11">
-        <v>46276</v>
+        <v>46277</v>
       </c>
       <c r="B59" s="12"/>
       <c r="C59" s="21" t="s">
         <v>35</v>
       </c>
       <c r="D59" s="13">
-        <v>246.47</v>
+        <v>246.92</v>
       </c>
       <c r="E59" s="13">
-        <v>214</v>
+        <v>215.58</v>
       </c>
       <c r="F59" s="13" t="s">
         <v>18</v>
       </c>
       <c r="G59" s="17"/>
     </row>
-    <row r="60" spans="1:7" x14ac:dyDescent="0.35">
+    <row r="60" spans="1:7" x14ac:dyDescent="0.45">
       <c r="A60" s="7">
-        <v>46276</v>
+        <v>46277</v>
       </c>
       <c r="B60" s="8"/>
       <c r="C60" s="20" t="s">
         <v>36</v>
       </c>
       <c r="D60" s="10">
-        <v>242.29</v>
+        <v>242.74</v>
       </c>
       <c r="E60" s="10">
-        <v>209.93</v>
+        <v>211.51</v>
       </c>
       <c r="F60" s="10">
-        <v>219.93</v>
+        <v>221.51</v>
       </c>
       <c r="G60" s="17"/>
     </row>
-    <row r="61" spans="1:7" x14ac:dyDescent="0.35">
+    <row r="61" spans="1:7" x14ac:dyDescent="0.45">
       <c r="A61" s="11">
-        <v>46276</v>
+        <v>46277</v>
       </c>
       <c r="B61" s="12"/>
       <c r="C61" s="21" t="s">
         <v>37</v>
       </c>
       <c r="D61" s="13">
-        <v>247.78</v>
+        <v>248.23</v>
       </c>
       <c r="E61" s="13">
-        <v>225.72</v>
+        <v>227.72</v>
       </c>
       <c r="F61" s="13" t="s">
         <v>18</v>
       </c>
       <c r="G61" s="17"/>
     </row>
-    <row r="62" spans="1:7" x14ac:dyDescent="0.35">
+    <row r="62" spans="1:7" x14ac:dyDescent="0.45">
       <c r="A62" s="7">
-        <v>46275</v>
+        <v>46276</v>
       </c>
       <c r="B62" s="8"/>
       <c r="C62" s="20" t="s">
         <v>32</v>
       </c>
       <c r="D62" s="10">
-        <v>259.33</v>
+        <v>259.77</v>
       </c>
       <c r="E62" s="10">
-        <v>227</v>
+        <v>229.4</v>
       </c>
       <c r="F62" s="10">
-        <v>237</v>
+        <v>239.4</v>
       </c>
       <c r="G62" s="17"/>
     </row>
-    <row r="63" spans="1:7" x14ac:dyDescent="0.35">
+    <row r="63" spans="1:7" x14ac:dyDescent="0.45">
       <c r="A63" s="11">
-        <v>46275</v>
+        <v>46276</v>
       </c>
       <c r="B63" s="12"/>
       <c r="C63" s="21" t="s">
         <v>33</v>
       </c>
       <c r="D63" s="13">
-        <v>248.11</v>
+        <v>248.62</v>
       </c>
       <c r="E63" s="13">
-        <v>217.85</v>
+        <v>219.61</v>
       </c>
       <c r="F63" s="13">
-        <v>227.85</v>
+        <v>229.61</v>
       </c>
       <c r="G63" s="17"/>
     </row>
-    <row r="64" spans="1:7" x14ac:dyDescent="0.35">
+    <row r="64" spans="1:7" x14ac:dyDescent="0.45">
       <c r="A64" s="7">
-        <v>46275</v>
+        <v>46276</v>
       </c>
       <c r="B64" s="8"/>
       <c r="C64" s="20" t="s">
         <v>34</v>
       </c>
       <c r="D64" s="10">
-        <v>249.3</v>
+        <v>249.83</v>
       </c>
       <c r="E64" s="10" t="s">
         <v>18</v>
@@ -1815,55 +1815,55 @@
       </c>
       <c r="G64" s="17"/>
     </row>
-    <row r="65" spans="1:6" x14ac:dyDescent="0.35">
+    <row r="65" spans="1:6" x14ac:dyDescent="0.45">
       <c r="A65" s="11">
-        <v>46275</v>
+        <v>46276</v>
       </c>
       <c r="B65" s="12"/>
       <c r="C65" s="21" t="s">
         <v>35</v>
       </c>
       <c r="D65" s="13">
-        <v>246.12</v>
+        <v>246.47</v>
       </c>
       <c r="E65" s="13">
-        <v>212.24</v>
+        <v>214</v>
       </c>
       <c r="F65" s="13" t="s">
         <v>18</v>
       </c>
     </row>
-    <row r="66" spans="1:6" x14ac:dyDescent="0.35">
+    <row r="66" spans="1:6" x14ac:dyDescent="0.45">
       <c r="A66" s="7">
-        <v>46275</v>
+        <v>46276</v>
       </c>
       <c r="B66" s="8"/>
       <c r="C66" s="20" t="s">
         <v>36</v>
       </c>
       <c r="D66" s="10">
-        <v>241.94</v>
+        <v>242.29</v>
       </c>
       <c r="E66" s="10">
-        <v>208.17</v>
+        <v>209.93</v>
       </c>
       <c r="F66" s="10">
-        <v>218.17</v>
-      </c>
-    </row>
-    <row r="67" spans="1:6" x14ac:dyDescent="0.35">
+        <v>219.93</v>
+      </c>
+    </row>
+    <row r="67" spans="1:6" x14ac:dyDescent="0.45">
       <c r="A67" s="11">
-        <v>46275</v>
+        <v>46276</v>
       </c>
       <c r="B67" s="12"/>
       <c r="C67" s="21" t="s">
         <v>37</v>
       </c>
       <c r="D67" s="13">
-        <v>247.41</v>
+        <v>247.78</v>
       </c>
       <c r="E67" s="13">
-        <v>223.54</v>
+        <v>225.72</v>
       </c>
       <c r="F67" s="13" t="s">
         <v>18</v>
@@ -1891,14 +1891,12 @@
 </file>
 
 <file path=customXml/item1.xml><?xml version="1.0" encoding="utf-8"?>
-<p:properties xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls">
-  <documentManagement>
-    <lcf76f155ced4ddcb4097134ff3c332f xmlns="87276d81-85f4-4ef2-9e6e-55066304288f">
-      <Terms xmlns="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
-    </lcf76f155ced4ddcb4097134ff3c332f>
-    <TaxCatchAll xmlns="b23b8984-eafa-4e79-985e-54f52f3da58e" xsi:nil="true"/>
-  </documentManagement>
-</p:properties>
+<?mso-contentType ?>
+<FormTemplates xmlns="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms">
+  <Display>DocumentLibraryForm</Display>
+  <Edit>DocumentLibraryForm</Edit>
+  <New>DocumentLibraryForm</New>
+</FormTemplates>
 </file>
 
 <file path=customXml/item2.xml><?xml version="1.0" encoding="utf-8"?>
@@ -2162,21 +2160,20 @@
 </file>
 
 <file path=customXml/item3.xml><?xml version="1.0" encoding="utf-8"?>
-<?mso-contentType ?>
-<FormTemplates xmlns="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms">
-  <Display>DocumentLibraryForm</Display>
-  <Edit>DocumentLibraryForm</Edit>
-  <New>DocumentLibraryForm</New>
-</FormTemplates>
+<p:properties xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls">
+  <documentManagement>
+    <lcf76f155ced4ddcb4097134ff3c332f xmlns="87276d81-85f4-4ef2-9e6e-55066304288f">
+      <Terms xmlns="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
+    </lcf76f155ced4ddcb4097134ff3c332f>
+    <TaxCatchAll xmlns="b23b8984-eafa-4e79-985e-54f52f3da58e" xsi:nil="true"/>
+  </documentManagement>
+</p:properties>
 </file>
 
 <file path=customXml/itemProps1.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{57A83D98-2BAE-4D83-823A-D31C464B620C}">
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{F60519E9-FD90-4339-869C-BC2F85719BB8}">
   <ds:schemaRefs>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/properties"/>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
-    <ds:schemaRef ds:uri="87276d81-85f4-4ef2-9e6e-55066304288f"/>
-    <ds:schemaRef ds:uri="b23b8984-eafa-4e79-985e-54f52f3da58e"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms"/>
   </ds:schemaRefs>
 </ds:datastoreItem>
 </file>
@@ -2202,9 +2199,12 @@
 </file>
 
 <file path=customXml/itemProps3.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{F60519E9-FD90-4339-869C-BC2F85719BB8}">
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{57A83D98-2BAE-4D83-823A-D31C464B620C}">
   <ds:schemaRefs>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/properties"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
+    <ds:schemaRef ds:uri="87276d81-85f4-4ef2-9e6e-55066304288f"/>
+    <ds:schemaRef ds:uri="b23b8984-eafa-4e79-985e-54f52f3da58e"/>
   </ds:schemaRefs>
 </ds:datastoreItem>
 </file>

</xml_diff>

<commit_message>
Mon Sep 14 06:28:26 UTC 2026
</commit_message>
<xml_diff>
--- a/bp.com-content-dam-bp-country-sites-en_au-australia-home-products-services-pricing-tgp-excel.xlsx
+++ b/bp.com-content-dam-bp-country-sites-en_au-australia-home-products-services-pricing-tgp-excel.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://bp365.sharepoint.com/sites/WholesalePricing/Shared Documents/B2C/TGP/Daily TGP/Web TGP/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="14_{6C331202-AF67-47AC-A154-B283B6CD85AE}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="14_{D7E57BB3-B1A4-4ACB-B54A-50CF9BEE6A1A}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="1470" yWindow="1470" windowWidth="13958" windowHeight="9142" xr2:uid="{1B412EEF-F96D-4DF4-A4E9-C7F0F183C2FB}"/>
+    <workbookView xWindow="-110" yWindow="-110" windowWidth="19420" windowHeight="11500" xr2:uid="{1B412EEF-F96D-4DF4-A4E9-C7F0F183C2FB}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
@@ -715,15 +715,15 @@
     <pageSetUpPr fitToPage="1"/>
   </sheetPr>
   <dimension ref="A1:G67"/>
-  <sheetFormatPr defaultRowHeight="14.25" x14ac:dyDescent="0.45"/>
+  <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
   <cols>
-    <col min="1" max="1" width="76.46484375" bestFit="1" customWidth="1"/>
-    <col min="2" max="2" width="6.46484375"/>
-    <col min="3" max="3" width="18.19921875" bestFit="1" customWidth="1"/>
-    <col min="4" max="7" width="7.19921875" bestFit="1" customWidth="1"/>
+    <col min="1" max="1" width="76.453125" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="6.453125"/>
+    <col min="3" max="3" width="18.1796875" bestFit="1" customWidth="1"/>
+    <col min="4" max="7" width="7.1796875" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:7" ht="22.15" x14ac:dyDescent="0.45">
+    <row r="1" spans="1:7" ht="22.5" x14ac:dyDescent="0.35">
       <c r="A1" s="30" t="s">
         <v>0</v>
       </c>
@@ -734,7 +734,7 @@
       <c r="F1" s="2"/>
       <c r="G1" s="2"/>
     </row>
-    <row r="2" spans="1:7" x14ac:dyDescent="0.45">
+    <row r="2" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A2" s="3"/>
       <c r="B2" s="1"/>
       <c r="C2" s="1"/>
@@ -743,7 +743,7 @@
       <c r="F2" s="2"/>
       <c r="G2" s="2"/>
     </row>
-    <row r="3" spans="1:7" x14ac:dyDescent="0.45">
+    <row r="3" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A3" s="3" t="s">
         <v>1</v>
       </c>
@@ -754,7 +754,7 @@
       <c r="F3" s="2"/>
       <c r="G3" s="2"/>
     </row>
-    <row r="4" spans="1:7" x14ac:dyDescent="0.45">
+    <row r="4" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A4" s="3" t="s">
         <v>2</v>
       </c>
@@ -765,7 +765,7 @@
       <c r="F4" s="2"/>
       <c r="G4" s="2"/>
     </row>
-    <row r="5" spans="1:7" x14ac:dyDescent="0.45">
+    <row r="5" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A5" s="3"/>
       <c r="B5" s="3"/>
       <c r="C5" s="1"/>
@@ -774,7 +774,7 @@
       <c r="F5" s="2"/>
       <c r="G5" s="2"/>
     </row>
-    <row r="6" spans="1:7" ht="20.25" x14ac:dyDescent="0.45">
+    <row r="6" spans="1:7" ht="20" x14ac:dyDescent="0.35">
       <c r="A6" s="29" t="s">
         <v>3</v>
       </c>
@@ -785,7 +785,7 @@
       <c r="F6" s="2"/>
       <c r="G6" s="2"/>
     </row>
-    <row r="7" spans="1:7" x14ac:dyDescent="0.45">
+    <row r="7" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A7" s="4" t="s">
         <v>4</v>
       </c>
@@ -806,133 +806,133 @@
         <v>9</v>
       </c>
     </row>
-    <row r="8" spans="1:7" x14ac:dyDescent="0.45">
+    <row r="8" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A8" s="7">
-        <v>46277</v>
+        <v>46280</v>
       </c>
       <c r="B8" s="8"/>
       <c r="C8" s="9" t="s">
         <v>10</v>
       </c>
       <c r="D8" s="10">
-        <v>247.73</v>
+        <v>253.59</v>
       </c>
       <c r="E8" s="10">
-        <v>214.55</v>
+        <v>219.24</v>
       </c>
       <c r="F8" s="10">
-        <v>224.55</v>
+        <v>229.24</v>
       </c>
       <c r="G8" s="10">
-        <v>214.52</v>
-      </c>
-    </row>
-    <row r="9" spans="1:7" x14ac:dyDescent="0.45">
+        <v>219.2</v>
+      </c>
+    </row>
+    <row r="9" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A9" s="11">
-        <v>46277</v>
+        <v>46280</v>
       </c>
       <c r="B9" s="12"/>
       <c r="C9" s="12" t="s">
         <v>11</v>
       </c>
       <c r="D9" s="13">
-        <v>247.73</v>
+        <v>253.59</v>
       </c>
       <c r="E9" s="13">
-        <v>214.55</v>
+        <v>219.24</v>
       </c>
       <c r="F9" s="13">
-        <v>224.55</v>
+        <v>229.24</v>
       </c>
       <c r="G9" s="13">
-        <v>214.52</v>
-      </c>
-    </row>
-    <row r="10" spans="1:7" x14ac:dyDescent="0.45">
+        <v>219.2</v>
+      </c>
+    </row>
+    <row r="10" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A10" s="7">
-        <v>46277</v>
+        <v>46280</v>
       </c>
       <c r="B10" s="8"/>
       <c r="C10" s="9" t="s">
         <v>12</v>
       </c>
       <c r="D10" s="10">
-        <v>243.64</v>
+        <v>249.06</v>
       </c>
       <c r="E10" s="10">
-        <v>211.35</v>
+        <v>215.65</v>
       </c>
       <c r="F10" s="10">
-        <v>221.35</v>
+        <v>225.65</v>
       </c>
       <c r="G10" s="10">
-        <v>211.77</v>
-      </c>
-    </row>
-    <row r="11" spans="1:7" x14ac:dyDescent="0.45">
+        <v>216.07</v>
+      </c>
+    </row>
+    <row r="11" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A11" s="11">
-        <v>46276</v>
+        <v>46277</v>
       </c>
       <c r="B11" s="12"/>
       <c r="C11" s="12" t="s">
         <v>10</v>
       </c>
       <c r="D11" s="13">
-        <v>246.84</v>
+        <v>247.73</v>
       </c>
       <c r="E11" s="13">
-        <v>212.58</v>
+        <v>214.55</v>
       </c>
       <c r="F11" s="13">
-        <v>222.58</v>
+        <v>224.55</v>
       </c>
       <c r="G11" s="13">
-        <v>212.54</v>
-      </c>
-    </row>
-    <row r="12" spans="1:7" x14ac:dyDescent="0.45">
+        <v>214.52</v>
+      </c>
+    </row>
+    <row r="12" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A12" s="7">
-        <v>46276</v>
+        <v>46277</v>
       </c>
       <c r="B12" s="8"/>
       <c r="C12" s="9" t="s">
         <v>11</v>
       </c>
       <c r="D12" s="10">
-        <v>246.84</v>
+        <v>247.73</v>
       </c>
       <c r="E12" s="10">
-        <v>212.58</v>
+        <v>214.55</v>
       </c>
       <c r="F12" s="10">
-        <v>222.58</v>
+        <v>224.55</v>
       </c>
       <c r="G12" s="10">
-        <v>212.54</v>
-      </c>
-    </row>
-    <row r="13" spans="1:7" x14ac:dyDescent="0.45">
+        <v>214.52</v>
+      </c>
+    </row>
+    <row r="13" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A13" s="11">
-        <v>46276</v>
+        <v>46277</v>
       </c>
       <c r="B13" s="12"/>
       <c r="C13" s="12" t="s">
         <v>12</v>
       </c>
       <c r="D13" s="13">
-        <v>243.05</v>
+        <v>243.64</v>
       </c>
       <c r="E13" s="13">
-        <v>209.64</v>
+        <v>211.35</v>
       </c>
       <c r="F13" s="13">
-        <v>219.64</v>
+        <v>221.35</v>
       </c>
       <c r="G13" s="13">
-        <v>210.06</v>
-      </c>
-    </row>
-    <row r="14" spans="1:7" x14ac:dyDescent="0.45">
+        <v>211.77</v>
+      </c>
+    </row>
+    <row r="14" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A14" s="14"/>
       <c r="B14" s="14"/>
       <c r="C14" s="15"/>
@@ -941,7 +941,7 @@
       <c r="F14" s="16"/>
       <c r="G14" s="16"/>
     </row>
-    <row r="15" spans="1:7" ht="20.25" x14ac:dyDescent="0.45">
+    <row r="15" spans="1:7" ht="20" x14ac:dyDescent="0.35">
       <c r="A15" s="29" t="s">
         <v>13</v>
       </c>
@@ -952,7 +952,7 @@
       <c r="F15" s="17"/>
       <c r="G15" s="17"/>
     </row>
-    <row r="16" spans="1:7" x14ac:dyDescent="0.45">
+    <row r="16" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A16" s="4" t="s">
         <v>4</v>
       </c>
@@ -971,45 +971,45 @@
       </c>
       <c r="G16" s="17"/>
     </row>
-    <row r="17" spans="1:7" x14ac:dyDescent="0.45">
+    <row r="17" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A17" s="7">
-        <v>46277</v>
+        <v>46280</v>
       </c>
       <c r="B17" s="8"/>
       <c r="C17" s="20" t="s">
         <v>14</v>
       </c>
       <c r="D17" s="10">
-        <v>248.67</v>
+        <v>253.99</v>
       </c>
       <c r="E17" s="10">
-        <v>215.66</v>
+        <v>219.89</v>
       </c>
       <c r="F17" s="10">
-        <v>225.66</v>
+        <v>229.89</v>
       </c>
       <c r="G17" s="17"/>
     </row>
-    <row r="18" spans="1:7" x14ac:dyDescent="0.45">
+    <row r="18" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A18" s="11">
-        <v>46276</v>
+        <v>46277</v>
       </c>
       <c r="B18" s="12"/>
       <c r="C18" s="12" t="s">
         <v>14</v>
       </c>
       <c r="D18" s="13">
-        <v>248.19</v>
+        <v>248.67</v>
       </c>
       <c r="E18" s="13">
-        <v>214.05</v>
+        <v>215.66</v>
       </c>
       <c r="F18" s="13">
-        <v>224.05</v>
+        <v>225.66</v>
       </c>
       <c r="G18" s="17"/>
     </row>
-    <row r="19" spans="1:7" x14ac:dyDescent="0.45">
+    <row r="19" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A19" s="14"/>
       <c r="B19" s="14"/>
       <c r="C19" s="15"/>
@@ -1018,7 +1018,7 @@
       <c r="F19" s="16"/>
       <c r="G19" s="17"/>
     </row>
-    <row r="20" spans="1:7" ht="20.25" x14ac:dyDescent="0.45">
+    <row r="20" spans="1:7" ht="20" x14ac:dyDescent="0.35">
       <c r="A20" s="29" t="s">
         <v>15</v>
       </c>
@@ -1029,7 +1029,7 @@
       <c r="F20" s="17"/>
       <c r="G20" s="17"/>
     </row>
-    <row r="21" spans="1:7" x14ac:dyDescent="0.45">
+    <row r="21" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A21" s="4" t="s">
         <v>4</v>
       </c>
@@ -1050,217 +1050,217 @@
         <v>9</v>
       </c>
     </row>
-    <row r="22" spans="1:7" x14ac:dyDescent="0.45">
+    <row r="22" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A22" s="7">
-        <v>46277</v>
+        <v>46280</v>
       </c>
       <c r="B22" s="8"/>
       <c r="C22" s="20" t="s">
         <v>16</v>
       </c>
       <c r="D22" s="10">
-        <v>248.86</v>
+        <v>254.72</v>
       </c>
       <c r="E22" s="10">
-        <v>215.25</v>
+        <v>219.93</v>
       </c>
       <c r="F22" s="10">
-        <v>224.85</v>
+        <v>229.53</v>
       </c>
       <c r="G22" s="10">
-        <v>213.97</v>
-      </c>
-    </row>
-    <row r="23" spans="1:7" x14ac:dyDescent="0.45">
+        <v>218.65</v>
+      </c>
+    </row>
+    <row r="23" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A23" s="11">
-        <v>46277</v>
+        <v>46280</v>
       </c>
       <c r="B23" s="12"/>
       <c r="C23" s="21" t="s">
         <v>17</v>
       </c>
       <c r="D23" s="13">
-        <v>248.4</v>
+        <v>253.83</v>
       </c>
       <c r="E23" s="13">
-        <v>218.99</v>
+        <v>223.33</v>
       </c>
       <c r="F23" s="13">
-        <v>228.99</v>
+        <v>233.33</v>
       </c>
       <c r="G23" s="13" t="s">
         <v>18</v>
       </c>
     </row>
-    <row r="24" spans="1:7" x14ac:dyDescent="0.45">
+    <row r="24" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A24" s="7">
-        <v>46277</v>
+        <v>46280</v>
       </c>
       <c r="B24" s="8"/>
       <c r="C24" s="20" t="s">
         <v>19</v>
       </c>
       <c r="D24" s="10">
-        <v>248.94</v>
+        <v>254.36</v>
       </c>
       <c r="E24" s="10">
-        <v>218.29</v>
+        <v>222.62</v>
       </c>
       <c r="F24" s="10">
-        <v>228.29</v>
+        <v>232.62</v>
       </c>
       <c r="G24" s="10" t="s">
         <v>18</v>
       </c>
     </row>
-    <row r="25" spans="1:7" x14ac:dyDescent="0.45">
+    <row r="25" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A25" s="11">
-        <v>46277</v>
+        <v>46280</v>
       </c>
       <c r="B25" s="12"/>
       <c r="C25" s="21" t="s">
         <v>20</v>
       </c>
       <c r="D25" s="13">
-        <v>245.73</v>
+        <v>251.14</v>
       </c>
       <c r="E25" s="13">
-        <v>218.32</v>
+        <v>222.67</v>
       </c>
       <c r="F25" s="13">
-        <v>228.32</v>
+        <v>232.67</v>
       </c>
       <c r="G25" s="13">
-        <v>216.21</v>
-      </c>
-    </row>
-    <row r="26" spans="1:7" x14ac:dyDescent="0.45">
+        <v>220.57</v>
+      </c>
+    </row>
+    <row r="26" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A26" s="7">
-        <v>46277</v>
+        <v>46280</v>
       </c>
       <c r="B26" s="8"/>
       <c r="C26" s="20" t="s">
         <v>21</v>
       </c>
       <c r="D26" s="10">
-        <v>247.54</v>
+        <v>252.94</v>
       </c>
       <c r="E26" s="10">
-        <v>219.67</v>
+        <v>224.05</v>
       </c>
       <c r="F26" s="10">
-        <v>229.67</v>
+        <v>234.05</v>
       </c>
       <c r="G26" s="10" t="s">
         <v>18</v>
       </c>
     </row>
-    <row r="27" spans="1:7" x14ac:dyDescent="0.45">
+    <row r="27" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A27" s="11">
-        <v>46276</v>
+        <v>46277</v>
       </c>
       <c r="B27" s="12"/>
       <c r="C27" s="12" t="s">
         <v>16</v>
       </c>
       <c r="D27" s="13">
-        <v>247.97</v>
+        <v>248.86</v>
       </c>
       <c r="E27" s="13">
-        <v>213.28</v>
+        <v>215.25</v>
       </c>
       <c r="F27" s="13">
-        <v>222.88</v>
+        <v>224.85</v>
       </c>
       <c r="G27" s="13">
-        <v>211.99</v>
-      </c>
-    </row>
-    <row r="28" spans="1:7" x14ac:dyDescent="0.45">
+        <v>213.97</v>
+      </c>
+    </row>
+    <row r="28" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A28" s="7">
-        <v>46276</v>
+        <v>46277</v>
       </c>
       <c r="B28" s="8"/>
       <c r="C28" s="20" t="s">
         <v>17</v>
       </c>
       <c r="D28" s="10">
-        <v>247.79</v>
+        <v>248.4</v>
       </c>
       <c r="E28" s="22">
-        <v>217.23</v>
+        <v>218.99</v>
       </c>
       <c r="F28" s="22">
-        <v>227.23</v>
+        <v>228.99</v>
       </c>
       <c r="G28" s="22" t="s">
         <v>18</v>
       </c>
     </row>
-    <row r="29" spans="1:7" x14ac:dyDescent="0.45">
+    <row r="29" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A29" s="11">
-        <v>46276</v>
+        <v>46277</v>
       </c>
       <c r="B29" s="12"/>
       <c r="C29" s="12" t="s">
         <v>19</v>
       </c>
       <c r="D29" s="13">
-        <v>248.34</v>
+        <v>248.94</v>
       </c>
       <c r="E29" s="13">
-        <v>216.53</v>
+        <v>218.29</v>
       </c>
       <c r="F29" s="13">
-        <v>226.53</v>
+        <v>228.29</v>
       </c>
       <c r="G29" s="13" t="s">
         <v>18</v>
       </c>
     </row>
-    <row r="30" spans="1:7" x14ac:dyDescent="0.45">
+    <row r="30" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A30" s="7">
-        <v>46276</v>
+        <v>46277</v>
       </c>
       <c r="B30" s="8"/>
       <c r="C30" s="20" t="s">
         <v>20</v>
       </c>
       <c r="D30" s="10">
-        <v>245.13</v>
+        <v>245.73</v>
       </c>
       <c r="E30" s="22">
-        <v>216.55</v>
+        <v>218.32</v>
       </c>
       <c r="F30" s="22">
-        <v>226.55</v>
+        <v>228.32</v>
       </c>
       <c r="G30" s="22">
-        <v>214.45</v>
-      </c>
-    </row>
-    <row r="31" spans="1:7" x14ac:dyDescent="0.45">
+        <v>216.21</v>
+      </c>
+    </row>
+    <row r="31" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A31" s="11">
-        <v>46276</v>
+        <v>46277</v>
       </c>
       <c r="B31" s="12"/>
       <c r="C31" s="12" t="s">
         <v>21</v>
       </c>
       <c r="D31" s="13">
-        <v>246.98</v>
+        <v>247.54</v>
       </c>
       <c r="E31" s="13">
-        <v>217.89</v>
+        <v>219.67</v>
       </c>
       <c r="F31" s="13">
-        <v>227.89</v>
+        <v>229.67</v>
       </c>
       <c r="G31" s="13" t="s">
         <v>18</v>
       </c>
     </row>
-    <row r="32" spans="1:7" x14ac:dyDescent="0.45">
+    <row r="32" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A32" s="14"/>
       <c r="B32" s="14"/>
       <c r="C32" s="15"/>
@@ -1269,7 +1269,7 @@
       <c r="F32" s="17"/>
       <c r="G32" s="17"/>
     </row>
-    <row r="33" spans="1:7" ht="20.25" x14ac:dyDescent="0.45">
+    <row r="33" spans="1:7" ht="20" x14ac:dyDescent="0.35">
       <c r="A33" s="29" t="s">
         <v>22</v>
       </c>
@@ -1280,7 +1280,7 @@
       <c r="F33" s="17"/>
       <c r="G33" s="17"/>
     </row>
-    <row r="34" spans="1:7" x14ac:dyDescent="0.45">
+    <row r="34" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A34" s="23" t="s">
         <v>4</v>
       </c>
@@ -1299,54 +1299,54 @@
       </c>
       <c r="G34" s="17"/>
     </row>
-    <row r="35" spans="1:7" x14ac:dyDescent="0.45">
+    <row r="35" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A35" s="7">
-        <v>46277</v>
+        <v>46280</v>
       </c>
       <c r="B35" s="8"/>
       <c r="C35" s="20" t="s">
         <v>23</v>
       </c>
       <c r="D35" s="10">
-        <v>242.18</v>
+        <v>247.6</v>
       </c>
       <c r="E35" s="10">
-        <v>210.31</v>
+        <v>214.61</v>
       </c>
       <c r="F35" s="10">
-        <v>219.31</v>
+        <v>223.61</v>
       </c>
       <c r="G35" s="17"/>
     </row>
-    <row r="36" spans="1:7" x14ac:dyDescent="0.45">
+    <row r="36" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A36" s="11">
-        <v>46276</v>
+        <v>46277</v>
       </c>
       <c r="B36" s="12"/>
       <c r="C36" s="12" t="s">
         <v>23</v>
       </c>
       <c r="D36" s="13">
-        <v>241.58</v>
+        <v>242.18</v>
       </c>
       <c r="E36" s="13">
-        <v>208.6</v>
+        <v>210.31</v>
       </c>
       <c r="F36" s="13">
-        <v>217.6</v>
+        <v>219.31</v>
       </c>
       <c r="G36" s="17"/>
     </row>
-    <row r="37" spans="1:7" x14ac:dyDescent="0.45">
+    <row r="37" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A37" s="7">
-        <v>46277</v>
+        <v>46280</v>
       </c>
       <c r="B37" s="8"/>
       <c r="C37" s="20" t="s">
         <v>24</v>
       </c>
       <c r="D37" s="10">
-        <v>257.8</v>
+        <v>263.22000000000003</v>
       </c>
       <c r="E37" s="10" t="s">
         <v>18</v>
@@ -1356,16 +1356,16 @@
       </c>
       <c r="G37" s="17"/>
     </row>
-    <row r="38" spans="1:7" x14ac:dyDescent="0.45">
+    <row r="38" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A38" s="11">
-        <v>46276</v>
+        <v>46277</v>
       </c>
       <c r="B38" s="12"/>
       <c r="C38" s="12" t="s">
         <v>24</v>
       </c>
       <c r="D38" s="13">
-        <v>257.2</v>
+        <v>257.8</v>
       </c>
       <c r="E38" s="13" t="s">
         <v>18</v>
@@ -1375,7 +1375,7 @@
       </c>
       <c r="G38" s="17"/>
     </row>
-    <row r="39" spans="1:7" x14ac:dyDescent="0.45">
+    <row r="39" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A39" s="24"/>
       <c r="B39" s="24"/>
       <c r="C39" s="15"/>
@@ -1384,7 +1384,7 @@
       <c r="F39" s="17"/>
       <c r="G39" s="17"/>
     </row>
-    <row r="40" spans="1:7" ht="20.25" x14ac:dyDescent="0.45">
+    <row r="40" spans="1:7" ht="20" x14ac:dyDescent="0.35">
       <c r="A40" s="29" t="s">
         <v>25</v>
       </c>
@@ -1395,7 +1395,7 @@
       <c r="F40" s="17"/>
       <c r="G40" s="17"/>
     </row>
-    <row r="41" spans="1:7" x14ac:dyDescent="0.45">
+    <row r="41" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A41" s="23" t="s">
         <v>4</v>
       </c>
@@ -1414,83 +1414,83 @@
       </c>
       <c r="G41" s="17"/>
     </row>
-    <row r="42" spans="1:7" x14ac:dyDescent="0.45">
+    <row r="42" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A42" s="7">
-        <v>46277</v>
+        <v>46280</v>
       </c>
       <c r="B42" s="8"/>
       <c r="C42" s="20" t="s">
         <v>26</v>
       </c>
       <c r="D42" s="10">
-        <v>250.97</v>
+        <v>256.45999999999998</v>
       </c>
       <c r="E42" s="10">
-        <v>216.78</v>
+        <v>221.16</v>
       </c>
       <c r="F42" s="10">
-        <v>226.78</v>
+        <v>231.16</v>
       </c>
       <c r="G42" s="17"/>
     </row>
-    <row r="43" spans="1:7" x14ac:dyDescent="0.45">
+    <row r="43" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A43" s="11">
-        <v>46277</v>
+        <v>46280</v>
       </c>
       <c r="B43" s="12"/>
       <c r="C43" s="21" t="s">
         <v>27</v>
       </c>
       <c r="D43" s="13">
-        <v>250.59</v>
+        <v>256.08</v>
       </c>
       <c r="E43" s="13">
-        <v>217.2</v>
+        <v>221.57</v>
       </c>
       <c r="F43" s="13">
-        <v>227.2</v>
+        <v>231.57</v>
       </c>
       <c r="G43" s="17"/>
     </row>
-    <row r="44" spans="1:7" x14ac:dyDescent="0.45">
+    <row r="44" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A44" s="7">
-        <v>46276</v>
+        <v>46277</v>
       </c>
       <c r="B44" s="8"/>
       <c r="C44" s="20" t="s">
         <v>26</v>
       </c>
       <c r="D44" s="10">
-        <v>250.28</v>
+        <v>250.97</v>
       </c>
       <c r="E44" s="10">
-        <v>214.96</v>
+        <v>216.78</v>
       </c>
       <c r="F44" s="10">
-        <v>224.96</v>
+        <v>226.78</v>
       </c>
       <c r="G44" s="17"/>
     </row>
-    <row r="45" spans="1:7" x14ac:dyDescent="0.45">
+    <row r="45" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A45" s="11">
-        <v>46276</v>
+        <v>46277</v>
       </c>
       <c r="B45" s="12"/>
       <c r="C45" s="21" t="s">
         <v>27</v>
       </c>
       <c r="D45" s="13">
-        <v>249.9</v>
+        <v>250.59</v>
       </c>
       <c r="E45" s="13">
-        <v>215.37</v>
+        <v>217.2</v>
       </c>
       <c r="F45" s="13">
-        <v>225.37</v>
+        <v>227.2</v>
       </c>
       <c r="G45" s="17"/>
     </row>
-    <row r="46" spans="1:7" x14ac:dyDescent="0.45">
+    <row r="46" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A46" s="14"/>
       <c r="B46" s="24"/>
       <c r="C46" s="15"/>
@@ -1499,7 +1499,7 @@
       <c r="F46" s="16"/>
       <c r="G46" s="17"/>
     </row>
-    <row r="47" spans="1:7" ht="20.25" x14ac:dyDescent="0.45">
+    <row r="47" spans="1:7" ht="20" x14ac:dyDescent="0.35">
       <c r="A47" s="25" t="s">
         <v>28</v>
       </c>
@@ -1510,7 +1510,7 @@
       <c r="F47" s="17"/>
       <c r="G47" s="17"/>
     </row>
-    <row r="48" spans="1:7" x14ac:dyDescent="0.45">
+    <row r="48" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A48" s="23" t="s">
         <v>4</v>
       </c>
@@ -1529,83 +1529,83 @@
       </c>
       <c r="G48" s="17"/>
     </row>
-    <row r="49" spans="1:7" x14ac:dyDescent="0.45">
+    <row r="49" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A49" s="7">
-        <v>46277</v>
+        <v>46280</v>
       </c>
       <c r="B49" s="8"/>
       <c r="C49" s="20" t="s">
         <v>29</v>
       </c>
       <c r="D49" s="10">
-        <v>244</v>
+        <v>246.9</v>
       </c>
       <c r="E49" s="10">
-        <v>209.95</v>
+        <v>213.05</v>
       </c>
       <c r="F49" s="10">
-        <v>219.95</v>
+        <v>223.05</v>
       </c>
       <c r="G49" s="28"/>
     </row>
-    <row r="50" spans="1:7" x14ac:dyDescent="0.45">
+    <row r="50" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A50" s="11">
-        <v>46277</v>
+        <v>46280</v>
       </c>
       <c r="B50" s="12"/>
       <c r="C50" s="21" t="s">
         <v>30</v>
       </c>
       <c r="D50" s="13">
-        <v>242.12</v>
+        <v>245</v>
       </c>
       <c r="E50" s="13">
-        <v>209.84</v>
+        <v>212.92</v>
       </c>
       <c r="F50" s="13">
-        <v>219.84</v>
+        <v>222.92</v>
       </c>
       <c r="G50" s="28"/>
     </row>
-    <row r="51" spans="1:7" x14ac:dyDescent="0.45">
+    <row r="51" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A51" s="7">
-        <v>46276</v>
+        <v>46277</v>
       </c>
       <c r="B51" s="8"/>
       <c r="C51" s="20" t="s">
         <v>29</v>
       </c>
       <c r="D51" s="10">
-        <v>243.3</v>
+        <v>244</v>
       </c>
       <c r="E51" s="10">
-        <v>207.95</v>
+        <v>209.95</v>
       </c>
       <c r="F51" s="10">
-        <v>217.95</v>
+        <v>219.95</v>
       </c>
       <c r="G51" s="17"/>
     </row>
-    <row r="52" spans="1:7" x14ac:dyDescent="0.45">
+    <row r="52" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A52" s="11">
-        <v>46276</v>
+        <v>46277</v>
       </c>
       <c r="B52" s="12"/>
       <c r="C52" s="21" t="s">
         <v>30</v>
       </c>
       <c r="D52" s="13">
-        <v>241.45</v>
+        <v>242.12</v>
       </c>
       <c r="E52" s="13">
-        <v>207.85</v>
+        <v>209.84</v>
       </c>
       <c r="F52" s="13">
-        <v>217.85</v>
+        <v>219.84</v>
       </c>
       <c r="G52" s="17"/>
     </row>
-    <row r="53" spans="1:7" x14ac:dyDescent="0.45">
+    <row r="53" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A53" s="14"/>
       <c r="B53" s="14"/>
       <c r="C53" s="15"/>
@@ -1614,7 +1614,7 @@
       <c r="F53" s="16"/>
       <c r="G53" s="17"/>
     </row>
-    <row r="54" spans="1:7" ht="20.25" x14ac:dyDescent="0.45">
+    <row r="54" spans="1:7" ht="20" x14ac:dyDescent="0.35">
       <c r="A54" s="27" t="s">
         <v>31</v>
       </c>
@@ -1625,7 +1625,7 @@
       <c r="F54" s="17"/>
       <c r="G54" s="17"/>
     </row>
-    <row r="55" spans="1:7" x14ac:dyDescent="0.45">
+    <row r="55" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A55" s="23" t="s">
         <v>4</v>
       </c>
@@ -1644,54 +1644,54 @@
       </c>
       <c r="G55" s="17"/>
     </row>
-    <row r="56" spans="1:7" x14ac:dyDescent="0.45">
+    <row r="56" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A56" s="7">
-        <v>46277</v>
+        <v>46280</v>
       </c>
       <c r="B56" s="8"/>
       <c r="C56" s="20" t="s">
         <v>32</v>
       </c>
       <c r="D56" s="10">
-        <v>260.32</v>
+        <v>265.72000000000003</v>
       </c>
       <c r="E56" s="10">
-        <v>231.62</v>
+        <v>236.31</v>
       </c>
       <c r="F56" s="10">
-        <v>241.62</v>
+        <v>246.31</v>
       </c>
       <c r="G56" s="17"/>
     </row>
-    <row r="57" spans="1:7" x14ac:dyDescent="0.45">
+    <row r="57" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A57" s="11">
-        <v>46277</v>
+        <v>46280</v>
       </c>
       <c r="B57" s="12"/>
       <c r="C57" s="21" t="s">
         <v>33</v>
       </c>
       <c r="D57" s="13">
-        <v>249.22</v>
+        <v>254.65</v>
       </c>
       <c r="E57" s="13">
-        <v>221.19</v>
+        <v>225.38</v>
       </c>
       <c r="F57" s="13">
-        <v>231.19</v>
+        <v>235.38</v>
       </c>
       <c r="G57" s="17"/>
     </row>
-    <row r="58" spans="1:7" x14ac:dyDescent="0.45">
+    <row r="58" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A58" s="7">
-        <v>46277</v>
+        <v>46280</v>
       </c>
       <c r="B58" s="8"/>
       <c r="C58" s="20" t="s">
         <v>34</v>
       </c>
       <c r="D58" s="10">
-        <v>250.45</v>
+        <v>255.88</v>
       </c>
       <c r="E58" s="10" t="s">
         <v>18</v>
@@ -1701,111 +1701,111 @@
       </c>
       <c r="G58" s="17"/>
     </row>
-    <row r="59" spans="1:7" x14ac:dyDescent="0.45">
+    <row r="59" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A59" s="11">
-        <v>46277</v>
+        <v>46280</v>
       </c>
       <c r="B59" s="12"/>
       <c r="C59" s="21" t="s">
         <v>35</v>
       </c>
       <c r="D59" s="13">
-        <v>246.92</v>
+        <v>252.21</v>
       </c>
       <c r="E59" s="13">
-        <v>215.58</v>
+        <v>219.76</v>
       </c>
       <c r="F59" s="13" t="s">
         <v>18</v>
       </c>
       <c r="G59" s="17"/>
     </row>
-    <row r="60" spans="1:7" x14ac:dyDescent="0.45">
+    <row r="60" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A60" s="7">
-        <v>46277</v>
+        <v>46280</v>
       </c>
       <c r="B60" s="8"/>
       <c r="C60" s="20" t="s">
         <v>36</v>
       </c>
       <c r="D60" s="10">
-        <v>242.74</v>
+        <v>248.03</v>
       </c>
       <c r="E60" s="10">
-        <v>211.51</v>
+        <v>215.7</v>
       </c>
       <c r="F60" s="10">
-        <v>221.51</v>
+        <v>225.7</v>
       </c>
       <c r="G60" s="17"/>
     </row>
-    <row r="61" spans="1:7" x14ac:dyDescent="0.45">
+    <row r="61" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A61" s="11">
-        <v>46277</v>
+        <v>46280</v>
       </c>
       <c r="B61" s="12"/>
       <c r="C61" s="21" t="s">
         <v>37</v>
       </c>
       <c r="D61" s="13">
-        <v>248.23</v>
+        <v>253.53</v>
       </c>
       <c r="E61" s="13">
-        <v>227.72</v>
+        <v>232.24</v>
       </c>
       <c r="F61" s="13" t="s">
         <v>18</v>
       </c>
       <c r="G61" s="17"/>
     </row>
-    <row r="62" spans="1:7" x14ac:dyDescent="0.45">
+    <row r="62" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A62" s="7">
-        <v>46276</v>
+        <v>46277</v>
       </c>
       <c r="B62" s="8"/>
       <c r="C62" s="20" t="s">
         <v>32</v>
       </c>
       <c r="D62" s="10">
-        <v>259.77</v>
+        <v>260.32</v>
       </c>
       <c r="E62" s="10">
-        <v>229.4</v>
+        <v>231.62</v>
       </c>
       <c r="F62" s="10">
-        <v>239.4</v>
+        <v>241.62</v>
       </c>
       <c r="G62" s="17"/>
     </row>
-    <row r="63" spans="1:7" x14ac:dyDescent="0.45">
+    <row r="63" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A63" s="11">
-        <v>46276</v>
+        <v>46277</v>
       </c>
       <c r="B63" s="12"/>
       <c r="C63" s="21" t="s">
         <v>33</v>
       </c>
       <c r="D63" s="13">
-        <v>248.62</v>
+        <v>249.22</v>
       </c>
       <c r="E63" s="13">
-        <v>219.61</v>
+        <v>221.19</v>
       </c>
       <c r="F63" s="13">
-        <v>229.61</v>
+        <v>231.19</v>
       </c>
       <c r="G63" s="17"/>
     </row>
-    <row r="64" spans="1:7" x14ac:dyDescent="0.45">
+    <row r="64" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A64" s="7">
-        <v>46276</v>
+        <v>46277</v>
       </c>
       <c r="B64" s="8"/>
       <c r="C64" s="20" t="s">
         <v>34</v>
       </c>
       <c r="D64" s="10">
-        <v>249.83</v>
+        <v>250.45</v>
       </c>
       <c r="E64" s="10" t="s">
         <v>18</v>
@@ -1815,55 +1815,55 @@
       </c>
       <c r="G64" s="17"/>
     </row>
-    <row r="65" spans="1:6" x14ac:dyDescent="0.45">
+    <row r="65" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A65" s="11">
-        <v>46276</v>
+        <v>46277</v>
       </c>
       <c r="B65" s="12"/>
       <c r="C65" s="21" t="s">
         <v>35</v>
       </c>
       <c r="D65" s="13">
-        <v>246.47</v>
+        <v>246.92</v>
       </c>
       <c r="E65" s="13">
-        <v>214</v>
+        <v>215.58</v>
       </c>
       <c r="F65" s="13" t="s">
         <v>18</v>
       </c>
     </row>
-    <row r="66" spans="1:6" x14ac:dyDescent="0.45">
+    <row r="66" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A66" s="7">
-        <v>46276</v>
+        <v>46277</v>
       </c>
       <c r="B66" s="8"/>
       <c r="C66" s="20" t="s">
         <v>36</v>
       </c>
       <c r="D66" s="10">
-        <v>242.29</v>
+        <v>242.74</v>
       </c>
       <c r="E66" s="10">
-        <v>209.93</v>
+        <v>211.51</v>
       </c>
       <c r="F66" s="10">
-        <v>219.93</v>
-      </c>
-    </row>
-    <row r="67" spans="1:6" x14ac:dyDescent="0.45">
+        <v>221.51</v>
+      </c>
+    </row>
+    <row r="67" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A67" s="11">
-        <v>46276</v>
+        <v>46277</v>
       </c>
       <c r="B67" s="12"/>
       <c r="C67" s="21" t="s">
         <v>37</v>
       </c>
       <c r="D67" s="13">
-        <v>247.78</v>
+        <v>248.23</v>
       </c>
       <c r="E67" s="13">
-        <v>225.72</v>
+        <v>227.72</v>
       </c>
       <c r="F67" s="13" t="s">
         <v>18</v>
@@ -1891,6 +1891,17 @@
 </file>
 
 <file path=customXml/item1.xml><?xml version="1.0" encoding="utf-8"?>
+<p:properties xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls">
+  <documentManagement>
+    <lcf76f155ced4ddcb4097134ff3c332f xmlns="87276d81-85f4-4ef2-9e6e-55066304288f">
+      <Terms xmlns="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
+    </lcf76f155ced4ddcb4097134ff3c332f>
+    <TaxCatchAll xmlns="b23b8984-eafa-4e79-985e-54f52f3da58e" xsi:nil="true"/>
+  </documentManagement>
+</p:properties>
+</file>
+
+<file path=customXml/item2.xml><?xml version="1.0" encoding="utf-8"?>
 <?mso-contentType ?>
 <FormTemplates xmlns="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms">
   <Display>DocumentLibraryForm</Display>
@@ -1899,7 +1910,7 @@
 </FormTemplates>
 </file>
 
-<file path=customXml/item2.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=customXml/item3.xml><?xml version="1.0" encoding="utf-8"?>
 <ct:contentTypeSchema xmlns:ct="http://schemas.microsoft.com/office/2006/metadata/contentType" xmlns:ma="http://schemas.microsoft.com/office/2006/metadata/properties/metaAttributes" ct:_="" ma:_="" ma:contentTypeName="Document" ma:contentTypeID="0x010100D3632DF5622958439304627C030B0427" ma:contentTypeVersion="18" ma:contentTypeDescription="Create a new document." ma:contentTypeScope="" ma:versionID="8c2ecbce386d6bac497f8eb2d8f0fb7a">
   <xsd:schema xmlns:xsd="http://www.w3.org/2001/XMLSchema" xmlns:xs="http://www.w3.org/2001/XMLSchema" xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:ns2="87276d81-85f4-4ef2-9e6e-55066304288f" xmlns:ns3="39e1dda6-d1d8-4c88-a3b9-f1abc1284bad" xmlns:ns4="b23b8984-eafa-4e79-985e-54f52f3da58e" targetNamespace="http://schemas.microsoft.com/office/2006/metadata/properties" ma:root="true" ma:fieldsID="4cfd0c2f651c1ce156ad4fcb44ea61dd" ns2:_="" ns3:_="" ns4:_="">
     <xsd:import namespace="87276d81-85f4-4ef2-9e6e-55066304288f"/>
@@ -2159,18 +2170,18 @@
 </ct:contentTypeSchema>
 </file>
 
-<file path=customXml/item3.xml><?xml version="1.0" encoding="utf-8"?>
-<p:properties xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls">
-  <documentManagement>
-    <lcf76f155ced4ddcb4097134ff3c332f xmlns="87276d81-85f4-4ef2-9e6e-55066304288f">
-      <Terms xmlns="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
-    </lcf76f155ced4ddcb4097134ff3c332f>
-    <TaxCatchAll xmlns="b23b8984-eafa-4e79-985e-54f52f3da58e" xsi:nil="true"/>
-  </documentManagement>
-</p:properties>
+<file path=customXml/itemProps1.xml><?xml version="1.0" encoding="utf-8"?>
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{57A83D98-2BAE-4D83-823A-D31C464B620C}">
+  <ds:schemaRefs>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/properties"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
+    <ds:schemaRef ds:uri="87276d81-85f4-4ef2-9e6e-55066304288f"/>
+    <ds:schemaRef ds:uri="b23b8984-eafa-4e79-985e-54f52f3da58e"/>
+  </ds:schemaRefs>
+</ds:datastoreItem>
 </file>
 
-<file path=customXml/itemProps1.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=customXml/itemProps2.xml><?xml version="1.0" encoding="utf-8"?>
 <ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{F60519E9-FD90-4339-869C-BC2F85719BB8}">
   <ds:schemaRefs>
     <ds:schemaRef ds:uri="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms"/>
@@ -2178,7 +2189,7 @@
 </ds:datastoreItem>
 </file>
 
-<file path=customXml/itemProps2.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=customXml/itemProps3.xml><?xml version="1.0" encoding="utf-8"?>
 <ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{B44E1863-2778-41F9-ACBA-48420F931671}">
   <ds:schemaRefs>
     <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/contentType"/>
@@ -2198,17 +2209,6 @@
 </ds:datastoreItem>
 </file>
 
-<file path=customXml/itemProps3.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{57A83D98-2BAE-4D83-823A-D31C464B620C}">
-  <ds:schemaRefs>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/properties"/>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
-    <ds:schemaRef ds:uri="87276d81-85f4-4ef2-9e6e-55066304288f"/>
-    <ds:schemaRef ds:uri="b23b8984-eafa-4e79-985e-54f52f3da58e"/>
-  </ds:schemaRefs>
-</ds:datastoreItem>
-</file>
-
 <file path=docMetadata/LabelInfo.xml><?xml version="1.0" encoding="utf-8"?>
 <clbl:labelList xmlns:clbl="http://schemas.microsoft.com/office/2020/mipLabelMetadata">
   <clbl:label id="{569bf4a9-87bd-4dbf-a36c-1db5158e5def}" enabled="1" method="Privileged" siteId="{ea80952e-a476-42d4-aaf4-5457852b0f7e}" removed="0"/>

</xml_diff>

<commit_message>
Tue Sep 15 06:13:09 UTC 2026
</commit_message>
<xml_diff>
--- a/bp.com-content-dam-bp-country-sites-en_au-australia-home-products-services-pricing-tgp-excel.xlsx
+++ b/bp.com-content-dam-bp-country-sites-en_au-australia-home-products-services-pricing-tgp-excel.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://bp365.sharepoint.com/sites/WholesalePricing/Shared Documents/B2C/TGP/Daily TGP/Web TGP/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="14_{D7E57BB3-B1A4-4ACB-B54A-50CF9BEE6A1A}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="14_{E3BBC0BC-4790-4307-A3BF-2D294E7096E0}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-110" yWindow="-110" windowWidth="19420" windowHeight="11500" xr2:uid="{1B412EEF-F96D-4DF4-A4E9-C7F0F183C2FB}"/>
+    <workbookView xWindow="-28920" yWindow="-60" windowWidth="29040" windowHeight="15720" xr2:uid="{1B412EEF-F96D-4DF4-A4E9-C7F0F183C2FB}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
@@ -715,15 +715,15 @@
     <pageSetUpPr fitToPage="1"/>
   </sheetPr>
   <dimension ref="A1:G67"/>
-  <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
+  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
-    <col min="1" max="1" width="76.453125" bestFit="1" customWidth="1"/>
-    <col min="2" max="2" width="6.453125"/>
-    <col min="3" max="3" width="18.1796875" bestFit="1" customWidth="1"/>
-    <col min="4" max="7" width="7.1796875" bestFit="1" customWidth="1"/>
+    <col min="1" max="1" width="76.42578125" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="6.42578125"/>
+    <col min="3" max="3" width="18.140625" bestFit="1" customWidth="1"/>
+    <col min="4" max="7" width="7.140625" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:7" ht="22.5" x14ac:dyDescent="0.35">
+    <row r="1" spans="1:7" ht="23.25" x14ac:dyDescent="0.25">
       <c r="A1" s="30" t="s">
         <v>0</v>
       </c>
@@ -734,7 +734,7 @@
       <c r="F1" s="2"/>
       <c r="G1" s="2"/>
     </row>
-    <row r="2" spans="1:7" x14ac:dyDescent="0.35">
+    <row r="2" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A2" s="3"/>
       <c r="B2" s="1"/>
       <c r="C2" s="1"/>
@@ -743,7 +743,7 @@
       <c r="F2" s="2"/>
       <c r="G2" s="2"/>
     </row>
-    <row r="3" spans="1:7" x14ac:dyDescent="0.35">
+    <row r="3" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A3" s="3" t="s">
         <v>1</v>
       </c>
@@ -754,7 +754,7 @@
       <c r="F3" s="2"/>
       <c r="G3" s="2"/>
     </row>
-    <row r="4" spans="1:7" x14ac:dyDescent="0.35">
+    <row r="4" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A4" s="3" t="s">
         <v>2</v>
       </c>
@@ -765,7 +765,7 @@
       <c r="F4" s="2"/>
       <c r="G4" s="2"/>
     </row>
-    <row r="5" spans="1:7" x14ac:dyDescent="0.35">
+    <row r="5" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A5" s="3"/>
       <c r="B5" s="3"/>
       <c r="C5" s="1"/>
@@ -774,7 +774,7 @@
       <c r="F5" s="2"/>
       <c r="G5" s="2"/>
     </row>
-    <row r="6" spans="1:7" ht="20" x14ac:dyDescent="0.35">
+    <row r="6" spans="1:7" ht="20.25" x14ac:dyDescent="0.25">
       <c r="A6" s="29" t="s">
         <v>3</v>
       </c>
@@ -785,7 +785,7 @@
       <c r="F6" s="2"/>
       <c r="G6" s="2"/>
     </row>
-    <row r="7" spans="1:7" x14ac:dyDescent="0.35">
+    <row r="7" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A7" s="4" t="s">
         <v>4</v>
       </c>
@@ -806,133 +806,133 @@
         <v>9</v>
       </c>
     </row>
-    <row r="8" spans="1:7" x14ac:dyDescent="0.35">
+    <row r="8" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A8" s="7">
-        <v>46280</v>
+        <v>46281</v>
       </c>
       <c r="B8" s="8"/>
       <c r="C8" s="9" t="s">
         <v>10</v>
       </c>
       <c r="D8" s="10">
-        <v>253.59</v>
+        <v>259.89</v>
       </c>
       <c r="E8" s="10">
-        <v>219.24</v>
+        <v>223.16</v>
       </c>
       <c r="F8" s="10">
-        <v>229.24</v>
+        <v>233.16</v>
       </c>
       <c r="G8" s="10">
-        <v>219.2</v>
-      </c>
-    </row>
-    <row r="9" spans="1:7" x14ac:dyDescent="0.35">
+        <v>223.13</v>
+      </c>
+    </row>
+    <row r="9" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A9" s="11">
-        <v>46280</v>
+        <v>46281</v>
       </c>
       <c r="B9" s="12"/>
       <c r="C9" s="12" t="s">
         <v>11</v>
       </c>
       <c r="D9" s="13">
-        <v>253.59</v>
+        <v>259.89</v>
       </c>
       <c r="E9" s="13">
-        <v>219.24</v>
+        <v>223.16</v>
       </c>
       <c r="F9" s="13">
-        <v>229.24</v>
+        <v>233.16</v>
       </c>
       <c r="G9" s="13">
-        <v>219.2</v>
-      </c>
-    </row>
-    <row r="10" spans="1:7" x14ac:dyDescent="0.35">
+        <v>223.13</v>
+      </c>
+    </row>
+    <row r="10" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A10" s="7">
-        <v>46280</v>
+        <v>46281</v>
       </c>
       <c r="B10" s="8"/>
       <c r="C10" s="9" t="s">
         <v>12</v>
       </c>
       <c r="D10" s="10">
-        <v>249.06</v>
+        <v>254.82</v>
       </c>
       <c r="E10" s="10">
-        <v>215.65</v>
+        <v>219.09</v>
       </c>
       <c r="F10" s="10">
-        <v>225.65</v>
+        <v>229.09</v>
       </c>
       <c r="G10" s="10">
-        <v>216.07</v>
-      </c>
-    </row>
-    <row r="11" spans="1:7" x14ac:dyDescent="0.35">
+        <v>219.51</v>
+      </c>
+    </row>
+    <row r="11" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A11" s="11">
-        <v>46277</v>
+        <v>46280</v>
       </c>
       <c r="B11" s="12"/>
       <c r="C11" s="12" t="s">
         <v>10</v>
       </c>
       <c r="D11" s="13">
-        <v>247.73</v>
+        <v>253.59</v>
       </c>
       <c r="E11" s="13">
-        <v>214.55</v>
+        <v>219.24</v>
       </c>
       <c r="F11" s="13">
-        <v>224.55</v>
+        <v>229.24</v>
       </c>
       <c r="G11" s="13">
-        <v>214.52</v>
-      </c>
-    </row>
-    <row r="12" spans="1:7" x14ac:dyDescent="0.35">
+        <v>219.2</v>
+      </c>
+    </row>
+    <row r="12" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A12" s="7">
-        <v>46277</v>
+        <v>46280</v>
       </c>
       <c r="B12" s="8"/>
       <c r="C12" s="9" t="s">
         <v>11</v>
       </c>
       <c r="D12" s="10">
-        <v>247.73</v>
+        <v>253.59</v>
       </c>
       <c r="E12" s="10">
-        <v>214.55</v>
+        <v>219.24</v>
       </c>
       <c r="F12" s="10">
-        <v>224.55</v>
+        <v>229.24</v>
       </c>
       <c r="G12" s="10">
-        <v>214.52</v>
-      </c>
-    </row>
-    <row r="13" spans="1:7" x14ac:dyDescent="0.35">
+        <v>219.2</v>
+      </c>
+    </row>
+    <row r="13" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A13" s="11">
-        <v>46277</v>
+        <v>46280</v>
       </c>
       <c r="B13" s="12"/>
       <c r="C13" s="12" t="s">
         <v>12</v>
       </c>
       <c r="D13" s="13">
-        <v>243.64</v>
+        <v>249.06</v>
       </c>
       <c r="E13" s="13">
-        <v>211.35</v>
+        <v>215.65</v>
       </c>
       <c r="F13" s="13">
-        <v>221.35</v>
+        <v>225.65</v>
       </c>
       <c r="G13" s="13">
-        <v>211.77</v>
-      </c>
-    </row>
-    <row r="14" spans="1:7" x14ac:dyDescent="0.35">
+        <v>216.07</v>
+      </c>
+    </row>
+    <row r="14" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A14" s="14"/>
       <c r="B14" s="14"/>
       <c r="C14" s="15"/>
@@ -941,7 +941,7 @@
       <c r="F14" s="16"/>
       <c r="G14" s="16"/>
     </row>
-    <row r="15" spans="1:7" ht="20" x14ac:dyDescent="0.35">
+    <row r="15" spans="1:7" ht="20.25" x14ac:dyDescent="0.25">
       <c r="A15" s="29" t="s">
         <v>13</v>
       </c>
@@ -952,7 +952,7 @@
       <c r="F15" s="17"/>
       <c r="G15" s="17"/>
     </row>
-    <row r="16" spans="1:7" x14ac:dyDescent="0.35">
+    <row r="16" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A16" s="4" t="s">
         <v>4</v>
       </c>
@@ -971,45 +971,45 @@
       </c>
       <c r="G16" s="17"/>
     </row>
-    <row r="17" spans="1:7" x14ac:dyDescent="0.35">
+    <row r="17" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A17" s="7">
-        <v>46280</v>
+        <v>46281</v>
       </c>
       <c r="B17" s="8"/>
       <c r="C17" s="20" t="s">
         <v>14</v>
       </c>
       <c r="D17" s="10">
-        <v>253.99</v>
+        <v>259.69</v>
       </c>
       <c r="E17" s="10">
-        <v>219.89</v>
+        <v>223.29</v>
       </c>
       <c r="F17" s="10">
-        <v>229.89</v>
+        <v>233.29</v>
       </c>
       <c r="G17" s="17"/>
     </row>
-    <row r="18" spans="1:7" x14ac:dyDescent="0.35">
+    <row r="18" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A18" s="11">
-        <v>46277</v>
+        <v>46280</v>
       </c>
       <c r="B18" s="12"/>
       <c r="C18" s="12" t="s">
         <v>14</v>
       </c>
       <c r="D18" s="13">
-        <v>248.67</v>
+        <v>253.99</v>
       </c>
       <c r="E18" s="13">
-        <v>215.66</v>
+        <v>219.89</v>
       </c>
       <c r="F18" s="13">
-        <v>225.66</v>
+        <v>229.89</v>
       </c>
       <c r="G18" s="17"/>
     </row>
-    <row r="19" spans="1:7" x14ac:dyDescent="0.35">
+    <row r="19" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A19" s="14"/>
       <c r="B19" s="14"/>
       <c r="C19" s="15"/>
@@ -1018,7 +1018,7 @@
       <c r="F19" s="16"/>
       <c r="G19" s="17"/>
     </row>
-    <row r="20" spans="1:7" ht="20" x14ac:dyDescent="0.35">
+    <row r="20" spans="1:7" ht="20.25" x14ac:dyDescent="0.25">
       <c r="A20" s="29" t="s">
         <v>15</v>
       </c>
@@ -1029,7 +1029,7 @@
       <c r="F20" s="17"/>
       <c r="G20" s="17"/>
     </row>
-    <row r="21" spans="1:7" x14ac:dyDescent="0.35">
+    <row r="21" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A21" s="4" t="s">
         <v>4</v>
       </c>
@@ -1050,217 +1050,217 @@
         <v>9</v>
       </c>
     </row>
-    <row r="22" spans="1:7" x14ac:dyDescent="0.35">
+    <row r="22" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A22" s="7">
-        <v>46280</v>
+        <v>46281</v>
       </c>
       <c r="B22" s="8"/>
       <c r="C22" s="20" t="s">
         <v>16</v>
       </c>
       <c r="D22" s="10">
-        <v>254.72</v>
+        <v>261.02</v>
       </c>
       <c r="E22" s="10">
-        <v>219.93</v>
+        <v>223.86</v>
       </c>
       <c r="F22" s="10">
-        <v>229.53</v>
+        <v>233.46</v>
       </c>
       <c r="G22" s="10">
-        <v>218.65</v>
-      </c>
-    </row>
-    <row r="23" spans="1:7" x14ac:dyDescent="0.35">
+        <v>222.57</v>
+      </c>
+    </row>
+    <row r="23" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A23" s="11">
-        <v>46280</v>
+        <v>46281</v>
       </c>
       <c r="B23" s="12"/>
       <c r="C23" s="21" t="s">
         <v>17</v>
       </c>
       <c r="D23" s="13">
-        <v>253.83</v>
+        <v>259.60000000000002</v>
       </c>
       <c r="E23" s="13">
-        <v>223.33</v>
+        <v>226.81</v>
       </c>
       <c r="F23" s="13">
-        <v>233.33</v>
+        <v>236.81</v>
       </c>
       <c r="G23" s="13" t="s">
         <v>18</v>
       </c>
     </row>
-    <row r="24" spans="1:7" x14ac:dyDescent="0.35">
+    <row r="24" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A24" s="7">
-        <v>46280</v>
+        <v>46281</v>
       </c>
       <c r="B24" s="8"/>
       <c r="C24" s="20" t="s">
         <v>19</v>
       </c>
       <c r="D24" s="10">
-        <v>254.36</v>
+        <v>260.12</v>
       </c>
       <c r="E24" s="10">
-        <v>222.62</v>
+        <v>226.09</v>
       </c>
       <c r="F24" s="10">
-        <v>232.62</v>
+        <v>236.09</v>
       </c>
       <c r="G24" s="10" t="s">
         <v>18</v>
       </c>
     </row>
-    <row r="25" spans="1:7" x14ac:dyDescent="0.35">
+    <row r="25" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A25" s="11">
-        <v>46280</v>
+        <v>46281</v>
       </c>
       <c r="B25" s="12"/>
       <c r="C25" s="21" t="s">
         <v>20</v>
       </c>
       <c r="D25" s="13">
-        <v>251.14</v>
+        <v>256.89999999999998</v>
       </c>
       <c r="E25" s="13">
-        <v>222.67</v>
+        <v>226.15</v>
       </c>
       <c r="F25" s="13">
-        <v>232.67</v>
+        <v>236.15</v>
       </c>
       <c r="G25" s="13">
-        <v>220.57</v>
-      </c>
-    </row>
-    <row r="26" spans="1:7" x14ac:dyDescent="0.35">
+        <v>224.04</v>
+      </c>
+    </row>
+    <row r="26" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A26" s="7">
-        <v>46280</v>
+        <v>46281</v>
       </c>
       <c r="B26" s="8"/>
       <c r="C26" s="20" t="s">
         <v>21</v>
       </c>
       <c r="D26" s="10">
-        <v>252.94</v>
+        <v>258.69</v>
       </c>
       <c r="E26" s="10">
-        <v>224.05</v>
+        <v>227.56</v>
       </c>
       <c r="F26" s="10">
-        <v>234.05</v>
+        <v>237.56</v>
       </c>
       <c r="G26" s="10" t="s">
         <v>18</v>
       </c>
     </row>
-    <row r="27" spans="1:7" x14ac:dyDescent="0.35">
+    <row r="27" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A27" s="11">
-        <v>46277</v>
+        <v>46280</v>
       </c>
       <c r="B27" s="12"/>
       <c r="C27" s="12" t="s">
         <v>16</v>
       </c>
       <c r="D27" s="13">
-        <v>248.86</v>
+        <v>254.72</v>
       </c>
       <c r="E27" s="13">
-        <v>215.25</v>
+        <v>219.93</v>
       </c>
       <c r="F27" s="13">
-        <v>224.85</v>
+        <v>229.53</v>
       </c>
       <c r="G27" s="13">
-        <v>213.97</v>
-      </c>
-    </row>
-    <row r="28" spans="1:7" x14ac:dyDescent="0.35">
+        <v>218.65</v>
+      </c>
+    </row>
+    <row r="28" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A28" s="7">
-        <v>46277</v>
+        <v>46280</v>
       </c>
       <c r="B28" s="8"/>
       <c r="C28" s="20" t="s">
         <v>17</v>
       </c>
       <c r="D28" s="10">
-        <v>248.4</v>
+        <v>253.83</v>
       </c>
       <c r="E28" s="22">
-        <v>218.99</v>
+        <v>223.33</v>
       </c>
       <c r="F28" s="22">
-        <v>228.99</v>
+        <v>233.33</v>
       </c>
       <c r="G28" s="22" t="s">
         <v>18</v>
       </c>
     </row>
-    <row r="29" spans="1:7" x14ac:dyDescent="0.35">
+    <row r="29" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A29" s="11">
-        <v>46277</v>
+        <v>46280</v>
       </c>
       <c r="B29" s="12"/>
       <c r="C29" s="12" t="s">
         <v>19</v>
       </c>
       <c r="D29" s="13">
-        <v>248.94</v>
+        <v>254.36</v>
       </c>
       <c r="E29" s="13">
-        <v>218.29</v>
+        <v>222.62</v>
       </c>
       <c r="F29" s="13">
-        <v>228.29</v>
+        <v>232.62</v>
       </c>
       <c r="G29" s="13" t="s">
         <v>18</v>
       </c>
     </row>
-    <row r="30" spans="1:7" x14ac:dyDescent="0.35">
+    <row r="30" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A30" s="7">
-        <v>46277</v>
+        <v>46280</v>
       </c>
       <c r="B30" s="8"/>
       <c r="C30" s="20" t="s">
         <v>20</v>
       </c>
       <c r="D30" s="10">
-        <v>245.73</v>
+        <v>251.14</v>
       </c>
       <c r="E30" s="22">
-        <v>218.32</v>
+        <v>222.67</v>
       </c>
       <c r="F30" s="22">
-        <v>228.32</v>
+        <v>232.67</v>
       </c>
       <c r="G30" s="22">
-        <v>216.21</v>
-      </c>
-    </row>
-    <row r="31" spans="1:7" x14ac:dyDescent="0.35">
+        <v>220.57</v>
+      </c>
+    </row>
+    <row r="31" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A31" s="11">
-        <v>46277</v>
+        <v>46280</v>
       </c>
       <c r="B31" s="12"/>
       <c r="C31" s="12" t="s">
         <v>21</v>
       </c>
       <c r="D31" s="13">
-        <v>247.54</v>
+        <v>252.94</v>
       </c>
       <c r="E31" s="13">
-        <v>219.67</v>
+        <v>224.05</v>
       </c>
       <c r="F31" s="13">
-        <v>229.67</v>
+        <v>234.05</v>
       </c>
       <c r="G31" s="13" t="s">
         <v>18</v>
       </c>
     </row>
-    <row r="32" spans="1:7" x14ac:dyDescent="0.35">
+    <row r="32" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A32" s="14"/>
       <c r="B32" s="14"/>
       <c r="C32" s="15"/>
@@ -1269,7 +1269,7 @@
       <c r="F32" s="17"/>
       <c r="G32" s="17"/>
     </row>
-    <row r="33" spans="1:7" ht="20" x14ac:dyDescent="0.35">
+    <row r="33" spans="1:7" ht="20.25" x14ac:dyDescent="0.25">
       <c r="A33" s="29" t="s">
         <v>22</v>
       </c>
@@ -1280,7 +1280,7 @@
       <c r="F33" s="17"/>
       <c r="G33" s="17"/>
     </row>
-    <row r="34" spans="1:7" x14ac:dyDescent="0.35">
+    <row r="34" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A34" s="23" t="s">
         <v>4</v>
       </c>
@@ -1299,54 +1299,54 @@
       </c>
       <c r="G34" s="17"/>
     </row>
-    <row r="35" spans="1:7" x14ac:dyDescent="0.35">
+    <row r="35" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A35" s="7">
-        <v>46280</v>
+        <v>46281</v>
       </c>
       <c r="B35" s="8"/>
       <c r="C35" s="20" t="s">
         <v>23</v>
       </c>
       <c r="D35" s="10">
-        <v>247.6</v>
+        <v>253.35</v>
       </c>
       <c r="E35" s="10">
-        <v>214.61</v>
+        <v>218.04</v>
       </c>
       <c r="F35" s="10">
-        <v>223.61</v>
+        <v>227.04</v>
       </c>
       <c r="G35" s="17"/>
     </row>
-    <row r="36" spans="1:7" x14ac:dyDescent="0.35">
+    <row r="36" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A36" s="11">
-        <v>46277</v>
+        <v>46280</v>
       </c>
       <c r="B36" s="12"/>
       <c r="C36" s="12" t="s">
         <v>23</v>
       </c>
       <c r="D36" s="13">
-        <v>242.18</v>
+        <v>247.6</v>
       </c>
       <c r="E36" s="13">
-        <v>210.31</v>
+        <v>214.61</v>
       </c>
       <c r="F36" s="13">
-        <v>219.31</v>
+        <v>223.61</v>
       </c>
       <c r="G36" s="17"/>
     </row>
-    <row r="37" spans="1:7" x14ac:dyDescent="0.35">
+    <row r="37" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A37" s="7">
-        <v>46280</v>
+        <v>46281</v>
       </c>
       <c r="B37" s="8"/>
       <c r="C37" s="20" t="s">
         <v>24</v>
       </c>
       <c r="D37" s="10">
-        <v>263.22000000000003</v>
+        <v>268.97000000000003</v>
       </c>
       <c r="E37" s="10" t="s">
         <v>18</v>
@@ -1356,16 +1356,16 @@
       </c>
       <c r="G37" s="17"/>
     </row>
-    <row r="38" spans="1:7" x14ac:dyDescent="0.35">
+    <row r="38" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A38" s="11">
-        <v>46277</v>
+        <v>46280</v>
       </c>
       <c r="B38" s="12"/>
       <c r="C38" s="12" t="s">
         <v>24</v>
       </c>
       <c r="D38" s="13">
-        <v>257.8</v>
+        <v>263.22000000000003</v>
       </c>
       <c r="E38" s="13" t="s">
         <v>18</v>
@@ -1375,7 +1375,7 @@
       </c>
       <c r="G38" s="17"/>
     </row>
-    <row r="39" spans="1:7" x14ac:dyDescent="0.35">
+    <row r="39" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A39" s="24"/>
       <c r="B39" s="24"/>
       <c r="C39" s="15"/>
@@ -1384,7 +1384,7 @@
       <c r="F39" s="17"/>
       <c r="G39" s="17"/>
     </row>
-    <row r="40" spans="1:7" ht="20" x14ac:dyDescent="0.35">
+    <row r="40" spans="1:7" ht="20.25" x14ac:dyDescent="0.25">
       <c r="A40" s="29" t="s">
         <v>25</v>
       </c>
@@ -1395,7 +1395,7 @@
       <c r="F40" s="17"/>
       <c r="G40" s="17"/>
     </row>
-    <row r="41" spans="1:7" x14ac:dyDescent="0.35">
+    <row r="41" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A41" s="23" t="s">
         <v>4</v>
       </c>
@@ -1414,83 +1414,83 @@
       </c>
       <c r="G41" s="17"/>
     </row>
-    <row r="42" spans="1:7" x14ac:dyDescent="0.35">
+    <row r="42" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A42" s="7">
-        <v>46280</v>
+        <v>46281</v>
       </c>
       <c r="B42" s="8"/>
       <c r="C42" s="20" t="s">
         <v>26</v>
       </c>
       <c r="D42" s="10">
-        <v>256.45999999999998</v>
+        <v>262.27</v>
       </c>
       <c r="E42" s="10">
-        <v>221.16</v>
+        <v>224.64</v>
       </c>
       <c r="F42" s="10">
-        <v>231.16</v>
+        <v>234.64</v>
       </c>
       <c r="G42" s="17"/>
     </row>
-    <row r="43" spans="1:7" x14ac:dyDescent="0.35">
+    <row r="43" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A43" s="11">
-        <v>46280</v>
+        <v>46281</v>
       </c>
       <c r="B43" s="12"/>
       <c r="C43" s="21" t="s">
         <v>27</v>
       </c>
       <c r="D43" s="13">
-        <v>256.08</v>
+        <v>261.88</v>
       </c>
       <c r="E43" s="13">
-        <v>221.57</v>
+        <v>225.06</v>
       </c>
       <c r="F43" s="13">
-        <v>231.57</v>
+        <v>235.06</v>
       </c>
       <c r="G43" s="17"/>
     </row>
-    <row r="44" spans="1:7" x14ac:dyDescent="0.35">
+    <row r="44" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A44" s="7">
-        <v>46277</v>
+        <v>46280</v>
       </c>
       <c r="B44" s="8"/>
       <c r="C44" s="20" t="s">
         <v>26</v>
       </c>
       <c r="D44" s="10">
-        <v>250.97</v>
+        <v>256.45999999999998</v>
       </c>
       <c r="E44" s="10">
-        <v>216.78</v>
+        <v>221.16</v>
       </c>
       <c r="F44" s="10">
-        <v>226.78</v>
+        <v>231.16</v>
       </c>
       <c r="G44" s="17"/>
     </row>
-    <row r="45" spans="1:7" x14ac:dyDescent="0.35">
+    <row r="45" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A45" s="11">
-        <v>46277</v>
+        <v>46280</v>
       </c>
       <c r="B45" s="12"/>
       <c r="C45" s="21" t="s">
         <v>27</v>
       </c>
       <c r="D45" s="13">
-        <v>250.59</v>
+        <v>256.08</v>
       </c>
       <c r="E45" s="13">
-        <v>217.2</v>
+        <v>221.57</v>
       </c>
       <c r="F45" s="13">
-        <v>227.2</v>
+        <v>231.57</v>
       </c>
       <c r="G45" s="17"/>
     </row>
-    <row r="46" spans="1:7" x14ac:dyDescent="0.35">
+    <row r="46" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A46" s="14"/>
       <c r="B46" s="24"/>
       <c r="C46" s="15"/>
@@ -1499,7 +1499,7 @@
       <c r="F46" s="16"/>
       <c r="G46" s="17"/>
     </row>
-    <row r="47" spans="1:7" ht="20" x14ac:dyDescent="0.35">
+    <row r="47" spans="1:7" ht="20.25" x14ac:dyDescent="0.25">
       <c r="A47" s="25" t="s">
         <v>28</v>
       </c>
@@ -1510,7 +1510,7 @@
       <c r="F47" s="17"/>
       <c r="G47" s="17"/>
     </row>
-    <row r="48" spans="1:7" x14ac:dyDescent="0.35">
+    <row r="48" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A48" s="23" t="s">
         <v>4</v>
       </c>
@@ -1529,83 +1529,83 @@
       </c>
       <c r="G48" s="17"/>
     </row>
-    <row r="49" spans="1:7" x14ac:dyDescent="0.35">
+    <row r="49" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A49" s="7">
-        <v>46280</v>
+        <v>46281</v>
       </c>
       <c r="B49" s="8"/>
       <c r="C49" s="20" t="s">
         <v>29</v>
       </c>
       <c r="D49" s="10">
-        <v>246.9</v>
+        <v>251.06</v>
       </c>
       <c r="E49" s="10">
-        <v>213.05</v>
+        <v>215.99</v>
       </c>
       <c r="F49" s="10">
-        <v>223.05</v>
+        <v>225.99</v>
       </c>
       <c r="G49" s="28"/>
     </row>
-    <row r="50" spans="1:7" x14ac:dyDescent="0.35">
+    <row r="50" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A50" s="11">
-        <v>46280</v>
+        <v>46281</v>
       </c>
       <c r="B50" s="12"/>
       <c r="C50" s="21" t="s">
         <v>30</v>
       </c>
       <c r="D50" s="13">
-        <v>245</v>
+        <v>249.13</v>
       </c>
       <c r="E50" s="13">
-        <v>212.92</v>
+        <v>215.85</v>
       </c>
       <c r="F50" s="13">
-        <v>222.92</v>
+        <v>225.85</v>
       </c>
       <c r="G50" s="28"/>
     </row>
-    <row r="51" spans="1:7" x14ac:dyDescent="0.35">
+    <row r="51" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A51" s="7">
-        <v>46277</v>
+        <v>46280</v>
       </c>
       <c r="B51" s="8"/>
       <c r="C51" s="20" t="s">
         <v>29</v>
       </c>
       <c r="D51" s="10">
-        <v>244</v>
+        <v>246.9</v>
       </c>
       <c r="E51" s="10">
-        <v>209.95</v>
+        <v>213.05</v>
       </c>
       <c r="F51" s="10">
-        <v>219.95</v>
+        <v>223.05</v>
       </c>
       <c r="G51" s="17"/>
     </row>
-    <row r="52" spans="1:7" x14ac:dyDescent="0.35">
+    <row r="52" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A52" s="11">
-        <v>46277</v>
+        <v>46280</v>
       </c>
       <c r="B52" s="12"/>
       <c r="C52" s="21" t="s">
         <v>30</v>
       </c>
       <c r="D52" s="13">
-        <v>242.12</v>
+        <v>245</v>
       </c>
       <c r="E52" s="13">
-        <v>209.84</v>
+        <v>212.92</v>
       </c>
       <c r="F52" s="13">
-        <v>219.84</v>
+        <v>222.92</v>
       </c>
       <c r="G52" s="17"/>
     </row>
-    <row r="53" spans="1:7" x14ac:dyDescent="0.35">
+    <row r="53" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A53" s="14"/>
       <c r="B53" s="14"/>
       <c r="C53" s="15"/>
@@ -1614,7 +1614,7 @@
       <c r="F53" s="16"/>
       <c r="G53" s="17"/>
     </row>
-    <row r="54" spans="1:7" ht="20" x14ac:dyDescent="0.35">
+    <row r="54" spans="1:7" ht="20.25" x14ac:dyDescent="0.25">
       <c r="A54" s="27" t="s">
         <v>31</v>
       </c>
@@ -1625,7 +1625,7 @@
       <c r="F54" s="17"/>
       <c r="G54" s="17"/>
     </row>
-    <row r="55" spans="1:7" x14ac:dyDescent="0.35">
+    <row r="55" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A55" s="23" t="s">
         <v>4</v>
       </c>
@@ -1644,54 +1644,54 @@
       </c>
       <c r="G55" s="17"/>
     </row>
-    <row r="56" spans="1:7" x14ac:dyDescent="0.35">
+    <row r="56" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A56" s="7">
-        <v>46280</v>
+        <v>46281</v>
       </c>
       <c r="B56" s="8"/>
       <c r="C56" s="20" t="s">
         <v>32</v>
       </c>
       <c r="D56" s="10">
-        <v>265.72000000000003</v>
+        <v>271.49</v>
       </c>
       <c r="E56" s="10">
-        <v>236.31</v>
+        <v>239.99</v>
       </c>
       <c r="F56" s="10">
-        <v>246.31</v>
+        <v>249.99</v>
       </c>
       <c r="G56" s="17"/>
     </row>
-    <row r="57" spans="1:7" x14ac:dyDescent="0.35">
+    <row r="57" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A57" s="11">
-        <v>46280</v>
+        <v>46281</v>
       </c>
       <c r="B57" s="12"/>
       <c r="C57" s="21" t="s">
         <v>33</v>
       </c>
       <c r="D57" s="13">
-        <v>254.65</v>
+        <v>260.42</v>
       </c>
       <c r="E57" s="13">
-        <v>225.38</v>
+        <v>228.74</v>
       </c>
       <c r="F57" s="13">
-        <v>235.38</v>
+        <v>238.74</v>
       </c>
       <c r="G57" s="17"/>
     </row>
-    <row r="58" spans="1:7" x14ac:dyDescent="0.35">
+    <row r="58" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A58" s="7">
-        <v>46280</v>
+        <v>46281</v>
       </c>
       <c r="B58" s="8"/>
       <c r="C58" s="20" t="s">
         <v>34</v>
       </c>
       <c r="D58" s="10">
-        <v>255.88</v>
+        <v>261.64999999999998</v>
       </c>
       <c r="E58" s="10" t="s">
         <v>18</v>
@@ -1701,111 +1701,111 @@
       </c>
       <c r="G58" s="17"/>
     </row>
-    <row r="59" spans="1:7" x14ac:dyDescent="0.35">
+    <row r="59" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A59" s="11">
-        <v>46280</v>
+        <v>46281</v>
       </c>
       <c r="B59" s="12"/>
       <c r="C59" s="21" t="s">
         <v>35</v>
       </c>
       <c r="D59" s="13">
-        <v>252.21</v>
+        <v>257.88</v>
       </c>
       <c r="E59" s="13">
-        <v>219.76</v>
+        <v>223.13</v>
       </c>
       <c r="F59" s="13" t="s">
         <v>18</v>
       </c>
       <c r="G59" s="17"/>
     </row>
-    <row r="60" spans="1:7" x14ac:dyDescent="0.35">
+    <row r="60" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A60" s="7">
-        <v>46280</v>
+        <v>46281</v>
       </c>
       <c r="B60" s="8"/>
       <c r="C60" s="20" t="s">
         <v>36</v>
       </c>
       <c r="D60" s="10">
-        <v>248.03</v>
+        <v>253.7</v>
       </c>
       <c r="E60" s="10">
-        <v>215.7</v>
+        <v>219.06</v>
       </c>
       <c r="F60" s="10">
-        <v>225.7</v>
+        <v>229.06</v>
       </c>
       <c r="G60" s="17"/>
     </row>
-    <row r="61" spans="1:7" x14ac:dyDescent="0.35">
+    <row r="61" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A61" s="11">
-        <v>46280</v>
+        <v>46281</v>
       </c>
       <c r="B61" s="12"/>
       <c r="C61" s="21" t="s">
         <v>37</v>
       </c>
       <c r="D61" s="13">
-        <v>253.53</v>
+        <v>259.20999999999998</v>
       </c>
       <c r="E61" s="13">
-        <v>232.24</v>
+        <v>235.82</v>
       </c>
       <c r="F61" s="13" t="s">
         <v>18</v>
       </c>
       <c r="G61" s="17"/>
     </row>
-    <row r="62" spans="1:7" x14ac:dyDescent="0.35">
+    <row r="62" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A62" s="7">
-        <v>46277</v>
+        <v>46280</v>
       </c>
       <c r="B62" s="8"/>
       <c r="C62" s="20" t="s">
         <v>32</v>
       </c>
       <c r="D62" s="10">
-        <v>260.32</v>
+        <v>265.72000000000003</v>
       </c>
       <c r="E62" s="10">
-        <v>231.62</v>
+        <v>236.31</v>
       </c>
       <c r="F62" s="10">
-        <v>241.62</v>
+        <v>246.31</v>
       </c>
       <c r="G62" s="17"/>
     </row>
-    <row r="63" spans="1:7" x14ac:dyDescent="0.35">
+    <row r="63" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A63" s="11">
-        <v>46277</v>
+        <v>46280</v>
       </c>
       <c r="B63" s="12"/>
       <c r="C63" s="21" t="s">
         <v>33</v>
       </c>
       <c r="D63" s="13">
-        <v>249.22</v>
+        <v>254.65</v>
       </c>
       <c r="E63" s="13">
-        <v>221.19</v>
+        <v>225.38</v>
       </c>
       <c r="F63" s="13">
-        <v>231.19</v>
+        <v>235.38</v>
       </c>
       <c r="G63" s="17"/>
     </row>
-    <row r="64" spans="1:7" x14ac:dyDescent="0.35">
+    <row r="64" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A64" s="7">
-        <v>46277</v>
+        <v>46280</v>
       </c>
       <c r="B64" s="8"/>
       <c r="C64" s="20" t="s">
         <v>34</v>
       </c>
       <c r="D64" s="10">
-        <v>250.45</v>
+        <v>255.88</v>
       </c>
       <c r="E64" s="10" t="s">
         <v>18</v>
@@ -1815,55 +1815,55 @@
       </c>
       <c r="G64" s="17"/>
     </row>
-    <row r="65" spans="1:6" x14ac:dyDescent="0.35">
+    <row r="65" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A65" s="11">
-        <v>46277</v>
+        <v>46280</v>
       </c>
       <c r="B65" s="12"/>
       <c r="C65" s="21" t="s">
         <v>35</v>
       </c>
       <c r="D65" s="13">
-        <v>246.92</v>
+        <v>252.21</v>
       </c>
       <c r="E65" s="13">
-        <v>215.58</v>
+        <v>219.76</v>
       </c>
       <c r="F65" s="13" t="s">
         <v>18</v>
       </c>
     </row>
-    <row r="66" spans="1:6" x14ac:dyDescent="0.35">
+    <row r="66" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A66" s="7">
-        <v>46277</v>
+        <v>46280</v>
       </c>
       <c r="B66" s="8"/>
       <c r="C66" s="20" t="s">
         <v>36</v>
       </c>
       <c r="D66" s="10">
-        <v>242.74</v>
+        <v>248.03</v>
       </c>
       <c r="E66" s="10">
-        <v>211.51</v>
+        <v>215.7</v>
       </c>
       <c r="F66" s="10">
-        <v>221.51</v>
-      </c>
-    </row>
-    <row r="67" spans="1:6" x14ac:dyDescent="0.35">
+        <v>225.7</v>
+      </c>
+    </row>
+    <row r="67" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A67" s="11">
-        <v>46277</v>
+        <v>46280</v>
       </c>
       <c r="B67" s="12"/>
       <c r="C67" s="21" t="s">
         <v>37</v>
       </c>
       <c r="D67" s="13">
-        <v>248.23</v>
+        <v>253.53</v>
       </c>
       <c r="E67" s="13">
-        <v>227.72</v>
+        <v>232.24</v>
       </c>
       <c r="F67" s="13" t="s">
         <v>18</v>
@@ -1891,26 +1891,6 @@
 </file>
 
 <file path=customXml/item1.xml><?xml version="1.0" encoding="utf-8"?>
-<p:properties xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls">
-  <documentManagement>
-    <lcf76f155ced4ddcb4097134ff3c332f xmlns="87276d81-85f4-4ef2-9e6e-55066304288f">
-      <Terms xmlns="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
-    </lcf76f155ced4ddcb4097134ff3c332f>
-    <TaxCatchAll xmlns="b23b8984-eafa-4e79-985e-54f52f3da58e" xsi:nil="true"/>
-  </documentManagement>
-</p:properties>
-</file>
-
-<file path=customXml/item2.xml><?xml version="1.0" encoding="utf-8"?>
-<?mso-contentType ?>
-<FormTemplates xmlns="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms">
-  <Display>DocumentLibraryForm</Display>
-  <Edit>DocumentLibraryForm</Edit>
-  <New>DocumentLibraryForm</New>
-</FormTemplates>
-</file>
-
-<file path=customXml/item3.xml><?xml version="1.0" encoding="utf-8"?>
 <ct:contentTypeSchema xmlns:ct="http://schemas.microsoft.com/office/2006/metadata/contentType" xmlns:ma="http://schemas.microsoft.com/office/2006/metadata/properties/metaAttributes" ct:_="" ma:_="" ma:contentTypeName="Document" ma:contentTypeID="0x010100D3632DF5622958439304627C030B0427" ma:contentTypeVersion="18" ma:contentTypeDescription="Create a new document." ma:contentTypeScope="" ma:versionID="8c2ecbce386d6bac497f8eb2d8f0fb7a">
   <xsd:schema xmlns:xsd="http://www.w3.org/2001/XMLSchema" xmlns:xs="http://www.w3.org/2001/XMLSchema" xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:ns2="87276d81-85f4-4ef2-9e6e-55066304288f" xmlns:ns3="39e1dda6-d1d8-4c88-a3b9-f1abc1284bad" xmlns:ns4="b23b8984-eafa-4e79-985e-54f52f3da58e" targetNamespace="http://schemas.microsoft.com/office/2006/metadata/properties" ma:root="true" ma:fieldsID="4cfd0c2f651c1ce156ad4fcb44ea61dd" ns2:_="" ns3:_="" ns4:_="">
     <xsd:import namespace="87276d81-85f4-4ef2-9e6e-55066304288f"/>
@@ -2170,26 +2150,27 @@
 </ct:contentTypeSchema>
 </file>
 
-<file path=customXml/itemProps1.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{57A83D98-2BAE-4D83-823A-D31C464B620C}">
-  <ds:schemaRefs>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/properties"/>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
-    <ds:schemaRef ds:uri="87276d81-85f4-4ef2-9e6e-55066304288f"/>
-    <ds:schemaRef ds:uri="b23b8984-eafa-4e79-985e-54f52f3da58e"/>
-  </ds:schemaRefs>
-</ds:datastoreItem>
+<file path=customXml/item2.xml><?xml version="1.0" encoding="utf-8"?>
+<p:properties xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls">
+  <documentManagement>
+    <lcf76f155ced4ddcb4097134ff3c332f xmlns="87276d81-85f4-4ef2-9e6e-55066304288f">
+      <Terms xmlns="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
+    </lcf76f155ced4ddcb4097134ff3c332f>
+    <TaxCatchAll xmlns="b23b8984-eafa-4e79-985e-54f52f3da58e" xsi:nil="true"/>
+  </documentManagement>
+</p:properties>
 </file>
 
-<file path=customXml/itemProps2.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{F60519E9-FD90-4339-869C-BC2F85719BB8}">
-  <ds:schemaRefs>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms"/>
-  </ds:schemaRefs>
-</ds:datastoreItem>
+<file path=customXml/item3.xml><?xml version="1.0" encoding="utf-8"?>
+<?mso-contentType ?>
+<FormTemplates xmlns="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms">
+  <Display>DocumentLibraryForm</Display>
+  <Edit>DocumentLibraryForm</Edit>
+  <New>DocumentLibraryForm</New>
+</FormTemplates>
 </file>
 
-<file path=customXml/itemProps3.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=customXml/itemProps1.xml><?xml version="1.0" encoding="utf-8"?>
 <ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{B44E1863-2778-41F9-ACBA-48420F931671}">
   <ds:schemaRefs>
     <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/contentType"/>
@@ -2209,6 +2190,25 @@
 </ds:datastoreItem>
 </file>
 
+<file path=customXml/itemProps2.xml><?xml version="1.0" encoding="utf-8"?>
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{57A83D98-2BAE-4D83-823A-D31C464B620C}">
+  <ds:schemaRefs>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/properties"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
+    <ds:schemaRef ds:uri="87276d81-85f4-4ef2-9e6e-55066304288f"/>
+    <ds:schemaRef ds:uri="b23b8984-eafa-4e79-985e-54f52f3da58e"/>
+  </ds:schemaRefs>
+</ds:datastoreItem>
+</file>
+
+<file path=customXml/itemProps3.xml><?xml version="1.0" encoding="utf-8"?>
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{F60519E9-FD90-4339-869C-BC2F85719BB8}">
+  <ds:schemaRefs>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms"/>
+  </ds:schemaRefs>
+</ds:datastoreItem>
+</file>
+
 <file path=docMetadata/LabelInfo.xml><?xml version="1.0" encoding="utf-8"?>
 <clbl:labelList xmlns:clbl="http://schemas.microsoft.com/office/2020/mipLabelMetadata">
   <clbl:label id="{569bf4a9-87bd-4dbf-a36c-1db5158e5def}" enabled="1" method="Privileged" siteId="{ea80952e-a476-42d4-aaf4-5457852b0f7e}" removed="0"/>

</xml_diff>

<commit_message>
Wed Sep 16 06:11:00 UTC 2026
</commit_message>
<xml_diff>
--- a/bp.com-content-dam-bp-country-sites-en_au-australia-home-products-services-pricing-tgp-excel.xlsx
+++ b/bp.com-content-dam-bp-country-sites-en_au-australia-home-products-services-pricing-tgp-excel.xlsx
@@ -8,14 +8,14 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://bp365.sharepoint.com/sites/WholesalePricing/Shared Documents/B2C/TGP/Daily TGP/Web TGP/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="14_{E3BBC0BC-4790-4307-A3BF-2D294E7096E0}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="14_{ABCA24F9-4456-418E-824F-3BAF0E211324}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-28920" yWindow="-60" windowWidth="29040" windowHeight="15720" xr2:uid="{1B412EEF-F96D-4DF4-A4E9-C7F0F183C2FB}"/>
+    <workbookView xWindow="-110" yWindow="-110" windowWidth="19420" windowHeight="11500" xr2:uid="{1B412EEF-F96D-4DF4-A4E9-C7F0F183C2FB}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
   </sheets>
-  <calcPr calcId="191028"/>
+  <calcPr calcId="191028" concurrentManualCount="12"/>
   <extLst>
     <ext xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" uri="{140A7094-0E35-4892-8432-C4D2E57EDEB5}">
       <x15:workbookPr chartTrackingRefBase="1"/>
@@ -715,15 +715,15 @@
     <pageSetUpPr fitToPage="1"/>
   </sheetPr>
   <dimension ref="A1:G67"/>
-  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
   <cols>
-    <col min="1" max="1" width="76.42578125" bestFit="1" customWidth="1"/>
-    <col min="2" max="2" width="6.42578125"/>
-    <col min="3" max="3" width="18.140625" bestFit="1" customWidth="1"/>
-    <col min="4" max="7" width="7.140625" bestFit="1" customWidth="1"/>
+    <col min="1" max="1" width="76.453125" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="6.453125"/>
+    <col min="3" max="3" width="18.1796875" bestFit="1" customWidth="1"/>
+    <col min="4" max="7" width="7.1796875" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:7" ht="23.25" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:7" ht="22.5" x14ac:dyDescent="0.35">
       <c r="A1" s="30" t="s">
         <v>0</v>
       </c>
@@ -734,7 +734,7 @@
       <c r="F1" s="2"/>
       <c r="G1" s="2"/>
     </row>
-    <row r="2" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="2" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A2" s="3"/>
       <c r="B2" s="1"/>
       <c r="C2" s="1"/>
@@ -743,7 +743,7 @@
       <c r="F2" s="2"/>
       <c r="G2" s="2"/>
     </row>
-    <row r="3" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="3" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A3" s="3" t="s">
         <v>1</v>
       </c>
@@ -754,7 +754,7 @@
       <c r="F3" s="2"/>
       <c r="G3" s="2"/>
     </row>
-    <row r="4" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="4" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A4" s="3" t="s">
         <v>2</v>
       </c>
@@ -765,7 +765,7 @@
       <c r="F4" s="2"/>
       <c r="G4" s="2"/>
     </row>
-    <row r="5" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="5" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A5" s="3"/>
       <c r="B5" s="3"/>
       <c r="C5" s="1"/>
@@ -774,7 +774,7 @@
       <c r="F5" s="2"/>
       <c r="G5" s="2"/>
     </row>
-    <row r="6" spans="1:7" ht="20.25" x14ac:dyDescent="0.25">
+    <row r="6" spans="1:7" ht="20" x14ac:dyDescent="0.35">
       <c r="A6" s="29" t="s">
         <v>3</v>
       </c>
@@ -785,7 +785,7 @@
       <c r="F6" s="2"/>
       <c r="G6" s="2"/>
     </row>
-    <row r="7" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="7" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A7" s="4" t="s">
         <v>4</v>
       </c>
@@ -806,133 +806,133 @@
         <v>9</v>
       </c>
     </row>
-    <row r="8" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="8" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A8" s="7">
-        <v>46281</v>
+        <v>46282</v>
       </c>
       <c r="B8" s="8"/>
       <c r="C8" s="9" t="s">
         <v>10</v>
       </c>
       <c r="D8" s="10">
-        <v>259.89</v>
+        <v>264.92</v>
       </c>
       <c r="E8" s="10">
-        <v>223.16</v>
+        <v>225.88</v>
       </c>
       <c r="F8" s="10">
-        <v>233.16</v>
+        <v>235.88</v>
       </c>
       <c r="G8" s="10">
-        <v>223.13</v>
-      </c>
-    </row>
-    <row r="9" spans="1:7" x14ac:dyDescent="0.25">
+        <v>225.84</v>
+      </c>
+    </row>
+    <row r="9" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A9" s="11">
-        <v>46281</v>
+        <v>46282</v>
       </c>
       <c r="B9" s="12"/>
       <c r="C9" s="12" t="s">
         <v>11</v>
       </c>
       <c r="D9" s="13">
-        <v>259.89</v>
+        <v>264.92</v>
       </c>
       <c r="E9" s="13">
-        <v>223.16</v>
+        <v>225.88</v>
       </c>
       <c r="F9" s="13">
-        <v>233.16</v>
+        <v>235.88</v>
       </c>
       <c r="G9" s="13">
-        <v>223.13</v>
-      </c>
-    </row>
-    <row r="10" spans="1:7" x14ac:dyDescent="0.25">
+        <v>225.84</v>
+      </c>
+    </row>
+    <row r="10" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A10" s="7">
-        <v>46281</v>
+        <v>46282</v>
       </c>
       <c r="B10" s="8"/>
       <c r="C10" s="9" t="s">
         <v>12</v>
       </c>
       <c r="D10" s="10">
-        <v>254.82</v>
+        <v>259.73</v>
       </c>
       <c r="E10" s="10">
-        <v>219.09</v>
+        <v>221.7</v>
       </c>
       <c r="F10" s="10">
-        <v>229.09</v>
+        <v>231.7</v>
       </c>
       <c r="G10" s="10">
-        <v>219.51</v>
-      </c>
-    </row>
-    <row r="11" spans="1:7" x14ac:dyDescent="0.25">
+        <v>222.12</v>
+      </c>
+    </row>
+    <row r="11" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A11" s="11">
-        <v>46280</v>
+        <v>46281</v>
       </c>
       <c r="B11" s="12"/>
       <c r="C11" s="12" t="s">
         <v>10</v>
       </c>
       <c r="D11" s="13">
-        <v>253.59</v>
+        <v>259.89</v>
       </c>
       <c r="E11" s="13">
-        <v>219.24</v>
+        <v>223.16</v>
       </c>
       <c r="F11" s="13">
-        <v>229.24</v>
+        <v>233.16</v>
       </c>
       <c r="G11" s="13">
-        <v>219.2</v>
-      </c>
-    </row>
-    <row r="12" spans="1:7" x14ac:dyDescent="0.25">
+        <v>223.13</v>
+      </c>
+    </row>
+    <row r="12" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A12" s="7">
-        <v>46280</v>
+        <v>46281</v>
       </c>
       <c r="B12" s="8"/>
       <c r="C12" s="9" t="s">
         <v>11</v>
       </c>
       <c r="D12" s="10">
-        <v>253.59</v>
+        <v>259.89</v>
       </c>
       <c r="E12" s="10">
-        <v>219.24</v>
+        <v>223.16</v>
       </c>
       <c r="F12" s="10">
-        <v>229.24</v>
+        <v>233.16</v>
       </c>
       <c r="G12" s="10">
-        <v>219.2</v>
-      </c>
-    </row>
-    <row r="13" spans="1:7" x14ac:dyDescent="0.25">
+        <v>223.13</v>
+      </c>
+    </row>
+    <row r="13" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A13" s="11">
-        <v>46280</v>
+        <v>46281</v>
       </c>
       <c r="B13" s="12"/>
       <c r="C13" s="12" t="s">
         <v>12</v>
       </c>
       <c r="D13" s="13">
-        <v>249.06</v>
+        <v>254.82</v>
       </c>
       <c r="E13" s="13">
-        <v>215.65</v>
+        <v>219.09</v>
       </c>
       <c r="F13" s="13">
-        <v>225.65</v>
+        <v>229.09</v>
       </c>
       <c r="G13" s="13">
-        <v>216.07</v>
-      </c>
-    </row>
-    <row r="14" spans="1:7" x14ac:dyDescent="0.25">
+        <v>219.51</v>
+      </c>
+    </row>
+    <row r="14" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A14" s="14"/>
       <c r="B14" s="14"/>
       <c r="C14" s="15"/>
@@ -941,7 +941,7 @@
       <c r="F14" s="16"/>
       <c r="G14" s="16"/>
     </row>
-    <row r="15" spans="1:7" ht="20.25" x14ac:dyDescent="0.25">
+    <row r="15" spans="1:7" ht="20" x14ac:dyDescent="0.35">
       <c r="A15" s="29" t="s">
         <v>13</v>
       </c>
@@ -952,7 +952,7 @@
       <c r="F15" s="17"/>
       <c r="G15" s="17"/>
     </row>
-    <row r="16" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="16" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A16" s="4" t="s">
         <v>4</v>
       </c>
@@ -971,45 +971,45 @@
       </c>
       <c r="G16" s="17"/>
     </row>
-    <row r="17" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="17" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A17" s="7">
-        <v>46281</v>
+        <v>46282</v>
       </c>
       <c r="B17" s="8"/>
       <c r="C17" s="20" t="s">
         <v>14</v>
       </c>
       <c r="D17" s="10">
-        <v>259.69</v>
+        <v>264.54000000000002</v>
       </c>
       <c r="E17" s="10">
-        <v>223.29</v>
+        <v>225.85</v>
       </c>
       <c r="F17" s="10">
-        <v>233.29</v>
+        <v>235.85</v>
       </c>
       <c r="G17" s="17"/>
     </row>
-    <row r="18" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="18" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A18" s="11">
-        <v>46280</v>
+        <v>46281</v>
       </c>
       <c r="B18" s="12"/>
       <c r="C18" s="12" t="s">
         <v>14</v>
       </c>
       <c r="D18" s="13">
-        <v>253.99</v>
+        <v>259.69</v>
       </c>
       <c r="E18" s="13">
-        <v>219.89</v>
+        <v>223.29</v>
       </c>
       <c r="F18" s="13">
-        <v>229.89</v>
+        <v>233.29</v>
       </c>
       <c r="G18" s="17"/>
     </row>
-    <row r="19" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="19" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A19" s="14"/>
       <c r="B19" s="14"/>
       <c r="C19" s="15"/>
@@ -1018,7 +1018,7 @@
       <c r="F19" s="16"/>
       <c r="G19" s="17"/>
     </row>
-    <row r="20" spans="1:7" ht="20.25" x14ac:dyDescent="0.25">
+    <row r="20" spans="1:7" ht="20" x14ac:dyDescent="0.35">
       <c r="A20" s="29" t="s">
         <v>15</v>
       </c>
@@ -1029,7 +1029,7 @@
       <c r="F20" s="17"/>
       <c r="G20" s="17"/>
     </row>
-    <row r="21" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="21" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A21" s="4" t="s">
         <v>4</v>
       </c>
@@ -1050,217 +1050,217 @@
         <v>9</v>
       </c>
     </row>
-    <row r="22" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="22" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A22" s="7">
-        <v>46281</v>
+        <v>46282</v>
       </c>
       <c r="B22" s="8"/>
       <c r="C22" s="20" t="s">
         <v>16</v>
       </c>
       <c r="D22" s="10">
-        <v>261.02</v>
+        <v>264.94</v>
       </c>
       <c r="E22" s="10">
-        <v>223.86</v>
+        <v>224.37</v>
       </c>
       <c r="F22" s="10">
-        <v>233.46</v>
+        <v>233.97</v>
       </c>
       <c r="G22" s="10">
-        <v>222.57</v>
-      </c>
-    </row>
-    <row r="23" spans="1:7" x14ac:dyDescent="0.25">
+        <v>223.09</v>
+      </c>
+    </row>
+    <row r="23" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A23" s="11">
-        <v>46281</v>
+        <v>46282</v>
       </c>
       <c r="B23" s="12"/>
       <c r="C23" s="21" t="s">
         <v>17</v>
       </c>
       <c r="D23" s="13">
-        <v>259.60000000000002</v>
+        <v>264.52</v>
       </c>
       <c r="E23" s="13">
-        <v>226.81</v>
+        <v>229.45</v>
       </c>
       <c r="F23" s="13">
-        <v>236.81</v>
+        <v>239.45</v>
       </c>
       <c r="G23" s="13" t="s">
         <v>18</v>
       </c>
     </row>
-    <row r="24" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="24" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A24" s="7">
-        <v>46281</v>
+        <v>46282</v>
       </c>
       <c r="B24" s="8"/>
       <c r="C24" s="20" t="s">
         <v>19</v>
       </c>
       <c r="D24" s="10">
-        <v>260.12</v>
+        <v>265.02999999999997</v>
       </c>
       <c r="E24" s="10">
-        <v>226.09</v>
+        <v>228.72</v>
       </c>
       <c r="F24" s="10">
-        <v>236.09</v>
+        <v>238.72</v>
       </c>
       <c r="G24" s="10" t="s">
         <v>18</v>
       </c>
     </row>
-    <row r="25" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="25" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A25" s="11">
-        <v>46281</v>
+        <v>46282</v>
       </c>
       <c r="B25" s="12"/>
       <c r="C25" s="21" t="s">
         <v>20</v>
       </c>
       <c r="D25" s="13">
-        <v>256.89999999999998</v>
+        <v>261.8</v>
       </c>
       <c r="E25" s="13">
-        <v>226.15</v>
+        <v>228.8</v>
       </c>
       <c r="F25" s="13">
-        <v>236.15</v>
+        <v>238.8</v>
       </c>
       <c r="G25" s="13">
-        <v>224.04</v>
-      </c>
-    </row>
-    <row r="26" spans="1:7" x14ac:dyDescent="0.25">
+        <v>226.69</v>
+      </c>
+    </row>
+    <row r="26" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A26" s="7">
-        <v>46281</v>
+        <v>46282</v>
       </c>
       <c r="B26" s="8"/>
       <c r="C26" s="20" t="s">
         <v>21</v>
       </c>
       <c r="D26" s="10">
-        <v>258.69</v>
+        <v>263.58999999999997</v>
       </c>
       <c r="E26" s="10">
-        <v>227.56</v>
+        <v>230.22</v>
       </c>
       <c r="F26" s="10">
-        <v>237.56</v>
+        <v>240.22</v>
       </c>
       <c r="G26" s="10" t="s">
         <v>18</v>
       </c>
     </row>
-    <row r="27" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="27" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A27" s="11">
-        <v>46280</v>
+        <v>46281</v>
       </c>
       <c r="B27" s="12"/>
       <c r="C27" s="12" t="s">
         <v>16</v>
       </c>
       <c r="D27" s="13">
-        <v>254.72</v>
+        <v>261.02</v>
       </c>
       <c r="E27" s="13">
-        <v>219.93</v>
+        <v>223.86</v>
       </c>
       <c r="F27" s="13">
-        <v>229.53</v>
+        <v>233.46</v>
       </c>
       <c r="G27" s="13">
-        <v>218.65</v>
-      </c>
-    </row>
-    <row r="28" spans="1:7" x14ac:dyDescent="0.25">
+        <v>222.57</v>
+      </c>
+    </row>
+    <row r="28" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A28" s="7">
-        <v>46280</v>
+        <v>46281</v>
       </c>
       <c r="B28" s="8"/>
       <c r="C28" s="20" t="s">
         <v>17</v>
       </c>
       <c r="D28" s="10">
-        <v>253.83</v>
+        <v>259.60000000000002</v>
       </c>
       <c r="E28" s="22">
-        <v>223.33</v>
+        <v>226.81</v>
       </c>
       <c r="F28" s="22">
-        <v>233.33</v>
+        <v>236.81</v>
       </c>
       <c r="G28" s="22" t="s">
         <v>18</v>
       </c>
     </row>
-    <row r="29" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="29" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A29" s="11">
-        <v>46280</v>
+        <v>46281</v>
       </c>
       <c r="B29" s="12"/>
       <c r="C29" s="12" t="s">
         <v>19</v>
       </c>
       <c r="D29" s="13">
-        <v>254.36</v>
+        <v>260.12</v>
       </c>
       <c r="E29" s="13">
-        <v>222.62</v>
+        <v>226.09</v>
       </c>
       <c r="F29" s="13">
-        <v>232.62</v>
+        <v>236.09</v>
       </c>
       <c r="G29" s="13" t="s">
         <v>18</v>
       </c>
     </row>
-    <row r="30" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="30" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A30" s="7">
-        <v>46280</v>
+        <v>46281</v>
       </c>
       <c r="B30" s="8"/>
       <c r="C30" s="20" t="s">
         <v>20</v>
       </c>
       <c r="D30" s="10">
-        <v>251.14</v>
+        <v>256.89999999999998</v>
       </c>
       <c r="E30" s="22">
-        <v>222.67</v>
+        <v>226.15</v>
       </c>
       <c r="F30" s="22">
-        <v>232.67</v>
+        <v>236.15</v>
       </c>
       <c r="G30" s="22">
-        <v>220.57</v>
-      </c>
-    </row>
-    <row r="31" spans="1:7" x14ac:dyDescent="0.25">
+        <v>224.04</v>
+      </c>
+    </row>
+    <row r="31" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A31" s="11">
-        <v>46280</v>
+        <v>46281</v>
       </c>
       <c r="B31" s="12"/>
       <c r="C31" s="12" t="s">
         <v>21</v>
       </c>
       <c r="D31" s="13">
-        <v>252.94</v>
+        <v>258.69</v>
       </c>
       <c r="E31" s="13">
-        <v>224.05</v>
+        <v>227.56</v>
       </c>
       <c r="F31" s="13">
-        <v>234.05</v>
+        <v>237.56</v>
       </c>
       <c r="G31" s="13" t="s">
         <v>18</v>
       </c>
     </row>
-    <row r="32" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="32" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A32" s="14"/>
       <c r="B32" s="14"/>
       <c r="C32" s="15"/>
@@ -1269,7 +1269,7 @@
       <c r="F32" s="17"/>
       <c r="G32" s="17"/>
     </row>
-    <row r="33" spans="1:7" ht="20.25" x14ac:dyDescent="0.25">
+    <row r="33" spans="1:7" ht="20" x14ac:dyDescent="0.35">
       <c r="A33" s="29" t="s">
         <v>22</v>
       </c>
@@ -1280,7 +1280,7 @@
       <c r="F33" s="17"/>
       <c r="G33" s="17"/>
     </row>
-    <row r="34" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="34" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A34" s="23" t="s">
         <v>4</v>
       </c>
@@ -1299,54 +1299,54 @@
       </c>
       <c r="G34" s="17"/>
     </row>
-    <row r="35" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="35" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A35" s="7">
-        <v>46281</v>
+        <v>46282</v>
       </c>
       <c r="B35" s="8"/>
       <c r="C35" s="20" t="s">
         <v>23</v>
       </c>
       <c r="D35" s="10">
-        <v>253.35</v>
+        <v>258.26</v>
       </c>
       <c r="E35" s="10">
-        <v>218.04</v>
+        <v>220.65</v>
       </c>
       <c r="F35" s="10">
-        <v>227.04</v>
+        <v>229.65</v>
       </c>
       <c r="G35" s="17"/>
     </row>
-    <row r="36" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="36" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A36" s="11">
-        <v>46280</v>
+        <v>46281</v>
       </c>
       <c r="B36" s="12"/>
       <c r="C36" s="12" t="s">
         <v>23</v>
       </c>
       <c r="D36" s="13">
-        <v>247.6</v>
+        <v>253.35</v>
       </c>
       <c r="E36" s="13">
-        <v>214.61</v>
+        <v>218.04</v>
       </c>
       <c r="F36" s="13">
-        <v>223.61</v>
+        <v>227.04</v>
       </c>
       <c r="G36" s="17"/>
     </row>
-    <row r="37" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="37" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A37" s="7">
-        <v>46281</v>
+        <v>46282</v>
       </c>
       <c r="B37" s="8"/>
       <c r="C37" s="20" t="s">
         <v>24</v>
       </c>
       <c r="D37" s="10">
-        <v>268.97000000000003</v>
+        <v>273.88</v>
       </c>
       <c r="E37" s="10" t="s">
         <v>18</v>
@@ -1356,16 +1356,16 @@
       </c>
       <c r="G37" s="17"/>
     </row>
-    <row r="38" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="38" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A38" s="11">
-        <v>46280</v>
+        <v>46281</v>
       </c>
       <c r="B38" s="12"/>
       <c r="C38" s="12" t="s">
         <v>24</v>
       </c>
       <c r="D38" s="13">
-        <v>263.22000000000003</v>
+        <v>268.97000000000003</v>
       </c>
       <c r="E38" s="13" t="s">
         <v>18</v>
@@ -1375,7 +1375,7 @@
       </c>
       <c r="G38" s="17"/>
     </row>
-    <row r="39" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="39" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A39" s="24"/>
       <c r="B39" s="24"/>
       <c r="C39" s="15"/>
@@ -1384,7 +1384,7 @@
       <c r="F39" s="17"/>
       <c r="G39" s="17"/>
     </row>
-    <row r="40" spans="1:7" ht="20.25" x14ac:dyDescent="0.25">
+    <row r="40" spans="1:7" ht="20" x14ac:dyDescent="0.35">
       <c r="A40" s="29" t="s">
         <v>25</v>
       </c>
@@ -1395,7 +1395,7 @@
       <c r="F40" s="17"/>
       <c r="G40" s="17"/>
     </row>
-    <row r="41" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="41" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A41" s="23" t="s">
         <v>4</v>
       </c>
@@ -1414,83 +1414,83 @@
       </c>
       <c r="G41" s="17"/>
     </row>
-    <row r="42" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="42" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A42" s="7">
-        <v>46281</v>
+        <v>46282</v>
       </c>
       <c r="B42" s="8"/>
       <c r="C42" s="20" t="s">
         <v>26</v>
       </c>
       <c r="D42" s="10">
-        <v>262.27</v>
+        <v>267.23</v>
       </c>
       <c r="E42" s="10">
-        <v>224.64</v>
+        <v>226.88</v>
       </c>
       <c r="F42" s="10">
-        <v>234.64</v>
+        <v>236.88</v>
       </c>
       <c r="G42" s="17"/>
     </row>
-    <row r="43" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="43" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A43" s="11">
-        <v>46281</v>
+        <v>46282</v>
       </c>
       <c r="B43" s="12"/>
       <c r="C43" s="21" t="s">
         <v>27</v>
       </c>
       <c r="D43" s="13">
-        <v>261.88</v>
+        <v>266.83999999999997</v>
       </c>
       <c r="E43" s="13">
-        <v>225.06</v>
+        <v>227.29</v>
       </c>
       <c r="F43" s="13">
-        <v>235.06</v>
+        <v>237.29</v>
       </c>
       <c r="G43" s="17"/>
     </row>
-    <row r="44" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="44" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A44" s="7">
-        <v>46280</v>
+        <v>46281</v>
       </c>
       <c r="B44" s="8"/>
       <c r="C44" s="20" t="s">
         <v>26</v>
       </c>
       <c r="D44" s="10">
-        <v>256.45999999999998</v>
+        <v>262.27</v>
       </c>
       <c r="E44" s="10">
-        <v>221.16</v>
+        <v>224.64</v>
       </c>
       <c r="F44" s="10">
-        <v>231.16</v>
+        <v>234.64</v>
       </c>
       <c r="G44" s="17"/>
     </row>
-    <row r="45" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="45" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A45" s="11">
-        <v>46280</v>
+        <v>46281</v>
       </c>
       <c r="B45" s="12"/>
       <c r="C45" s="21" t="s">
         <v>27</v>
       </c>
       <c r="D45" s="13">
-        <v>256.08</v>
+        <v>261.88</v>
       </c>
       <c r="E45" s="13">
-        <v>221.57</v>
+        <v>225.06</v>
       </c>
       <c r="F45" s="13">
-        <v>231.57</v>
+        <v>235.06</v>
       </c>
       <c r="G45" s="17"/>
     </row>
-    <row r="46" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="46" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A46" s="14"/>
       <c r="B46" s="24"/>
       <c r="C46" s="15"/>
@@ -1499,7 +1499,7 @@
       <c r="F46" s="16"/>
       <c r="G46" s="17"/>
     </row>
-    <row r="47" spans="1:7" ht="20.25" x14ac:dyDescent="0.25">
+    <row r="47" spans="1:7" ht="20" x14ac:dyDescent="0.35">
       <c r="A47" s="25" t="s">
         <v>28</v>
       </c>
@@ -1510,7 +1510,7 @@
       <c r="F47" s="17"/>
       <c r="G47" s="17"/>
     </row>
-    <row r="48" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="48" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A48" s="23" t="s">
         <v>4</v>
       </c>
@@ -1529,83 +1529,83 @@
       </c>
       <c r="G48" s="17"/>
     </row>
-    <row r="49" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="49" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A49" s="7">
-        <v>46281</v>
+        <v>46282</v>
       </c>
       <c r="B49" s="8"/>
       <c r="C49" s="20" t="s">
         <v>29</v>
       </c>
       <c r="D49" s="10">
-        <v>251.06</v>
+        <v>255.51</v>
       </c>
       <c r="E49" s="10">
-        <v>215.99</v>
+        <v>219.23</v>
       </c>
       <c r="F49" s="10">
-        <v>225.99</v>
+        <v>229.23</v>
       </c>
       <c r="G49" s="28"/>
     </row>
-    <row r="50" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="50" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A50" s="11">
-        <v>46281</v>
+        <v>46282</v>
       </c>
       <c r="B50" s="12"/>
       <c r="C50" s="21" t="s">
         <v>30</v>
       </c>
       <c r="D50" s="13">
-        <v>249.13</v>
+        <v>253.55</v>
       </c>
       <c r="E50" s="13">
-        <v>215.85</v>
+        <v>219.08</v>
       </c>
       <c r="F50" s="13">
-        <v>225.85</v>
+        <v>229.08</v>
       </c>
       <c r="G50" s="28"/>
     </row>
-    <row r="51" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="51" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A51" s="7">
-        <v>46280</v>
+        <v>46281</v>
       </c>
       <c r="B51" s="8"/>
       <c r="C51" s="20" t="s">
         <v>29</v>
       </c>
       <c r="D51" s="10">
-        <v>246.9</v>
+        <v>251.06</v>
       </c>
       <c r="E51" s="10">
-        <v>213.05</v>
+        <v>215.99</v>
       </c>
       <c r="F51" s="10">
-        <v>223.05</v>
+        <v>225.99</v>
       </c>
       <c r="G51" s="17"/>
     </row>
-    <row r="52" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="52" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A52" s="11">
-        <v>46280</v>
+        <v>46281</v>
       </c>
       <c r="B52" s="12"/>
       <c r="C52" s="21" t="s">
         <v>30</v>
       </c>
       <c r="D52" s="13">
-        <v>245</v>
+        <v>249.13</v>
       </c>
       <c r="E52" s="13">
-        <v>212.92</v>
+        <v>215.85</v>
       </c>
       <c r="F52" s="13">
-        <v>222.92</v>
+        <v>225.85</v>
       </c>
       <c r="G52" s="17"/>
     </row>
-    <row r="53" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="53" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A53" s="14"/>
       <c r="B53" s="14"/>
       <c r="C53" s="15"/>
@@ -1614,7 +1614,7 @@
       <c r="F53" s="16"/>
       <c r="G53" s="17"/>
     </row>
-    <row r="54" spans="1:7" ht="20.25" x14ac:dyDescent="0.25">
+    <row r="54" spans="1:7" ht="20" x14ac:dyDescent="0.35">
       <c r="A54" s="27" t="s">
         <v>31</v>
       </c>
@@ -1625,7 +1625,7 @@
       <c r="F54" s="17"/>
       <c r="G54" s="17"/>
     </row>
-    <row r="55" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="55" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A55" s="23" t="s">
         <v>4</v>
       </c>
@@ -1644,54 +1644,54 @@
       </c>
       <c r="G55" s="17"/>
     </row>
-    <row r="56" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="56" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A56" s="7">
-        <v>46281</v>
+        <v>46282</v>
       </c>
       <c r="B56" s="8"/>
       <c r="C56" s="20" t="s">
         <v>32</v>
       </c>
       <c r="D56" s="10">
-        <v>271.49</v>
+        <v>276.39999999999998</v>
       </c>
       <c r="E56" s="10">
-        <v>239.99</v>
+        <v>242.85</v>
       </c>
       <c r="F56" s="10">
-        <v>249.99</v>
+        <v>252.85</v>
       </c>
       <c r="G56" s="17"/>
     </row>
-    <row r="57" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="57" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A57" s="11">
-        <v>46281</v>
+        <v>46282</v>
       </c>
       <c r="B57" s="12"/>
       <c r="C57" s="21" t="s">
         <v>33</v>
       </c>
       <c r="D57" s="13">
-        <v>260.42</v>
+        <v>265.33999999999997</v>
       </c>
       <c r="E57" s="13">
-        <v>228.74</v>
+        <v>231.28</v>
       </c>
       <c r="F57" s="13">
-        <v>238.74</v>
+        <v>241.28</v>
       </c>
       <c r="G57" s="17"/>
     </row>
-    <row r="58" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="58" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A58" s="7">
-        <v>46281</v>
+        <v>46282</v>
       </c>
       <c r="B58" s="8"/>
       <c r="C58" s="20" t="s">
         <v>34</v>
       </c>
       <c r="D58" s="10">
-        <v>261.64999999999998</v>
+        <v>266.57</v>
       </c>
       <c r="E58" s="10" t="s">
         <v>18</v>
@@ -1701,111 +1701,111 @@
       </c>
       <c r="G58" s="17"/>
     </row>
-    <row r="59" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="59" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A59" s="11">
-        <v>46281</v>
+        <v>46282</v>
       </c>
       <c r="B59" s="12"/>
       <c r="C59" s="21" t="s">
         <v>35</v>
       </c>
       <c r="D59" s="13">
-        <v>257.88</v>
+        <v>262.7</v>
       </c>
       <c r="E59" s="13">
-        <v>223.13</v>
+        <v>225.66</v>
       </c>
       <c r="F59" s="13" t="s">
         <v>18</v>
       </c>
       <c r="G59" s="17"/>
     </row>
-    <row r="60" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="60" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A60" s="7">
-        <v>46281</v>
+        <v>46282</v>
       </c>
       <c r="B60" s="8"/>
       <c r="C60" s="20" t="s">
         <v>36</v>
       </c>
       <c r="D60" s="10">
-        <v>253.7</v>
+        <v>258.52999999999997</v>
       </c>
       <c r="E60" s="10">
-        <v>219.06</v>
+        <v>221.6</v>
       </c>
       <c r="F60" s="10">
-        <v>229.06</v>
+        <v>231.6</v>
       </c>
       <c r="G60" s="17"/>
     </row>
-    <row r="61" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="61" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A61" s="11">
-        <v>46281</v>
+        <v>46282</v>
       </c>
       <c r="B61" s="12"/>
       <c r="C61" s="21" t="s">
         <v>37</v>
       </c>
       <c r="D61" s="13">
-        <v>259.20999999999998</v>
+        <v>264.02999999999997</v>
       </c>
       <c r="E61" s="13">
-        <v>235.82</v>
+        <v>238.59</v>
       </c>
       <c r="F61" s="13" t="s">
         <v>18</v>
       </c>
       <c r="G61" s="17"/>
     </row>
-    <row r="62" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="62" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A62" s="7">
-        <v>46280</v>
+        <v>46281</v>
       </c>
       <c r="B62" s="8"/>
       <c r="C62" s="20" t="s">
         <v>32</v>
       </c>
       <c r="D62" s="10">
-        <v>265.72000000000003</v>
+        <v>271.49</v>
       </c>
       <c r="E62" s="10">
-        <v>236.31</v>
+        <v>239.99</v>
       </c>
       <c r="F62" s="10">
-        <v>246.31</v>
+        <v>249.99</v>
       </c>
       <c r="G62" s="17"/>
     </row>
-    <row r="63" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="63" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A63" s="11">
-        <v>46280</v>
+        <v>46281</v>
       </c>
       <c r="B63" s="12"/>
       <c r="C63" s="21" t="s">
         <v>33</v>
       </c>
       <c r="D63" s="13">
-        <v>254.65</v>
+        <v>260.42</v>
       </c>
       <c r="E63" s="13">
-        <v>225.38</v>
+        <v>228.74</v>
       </c>
       <c r="F63" s="13">
-        <v>235.38</v>
+        <v>238.74</v>
       </c>
       <c r="G63" s="17"/>
     </row>
-    <row r="64" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="64" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A64" s="7">
-        <v>46280</v>
+        <v>46281</v>
       </c>
       <c r="B64" s="8"/>
       <c r="C64" s="20" t="s">
         <v>34</v>
       </c>
       <c r="D64" s="10">
-        <v>255.88</v>
+        <v>261.64999999999998</v>
       </c>
       <c r="E64" s="10" t="s">
         <v>18</v>
@@ -1815,55 +1815,55 @@
       </c>
       <c r="G64" s="17"/>
     </row>
-    <row r="65" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="65" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A65" s="11">
-        <v>46280</v>
+        <v>46281</v>
       </c>
       <c r="B65" s="12"/>
       <c r="C65" s="21" t="s">
         <v>35</v>
       </c>
       <c r="D65" s="13">
-        <v>252.21</v>
+        <v>257.88</v>
       </c>
       <c r="E65" s="13">
-        <v>219.76</v>
+        <v>223.13</v>
       </c>
       <c r="F65" s="13" t="s">
         <v>18</v>
       </c>
     </row>
-    <row r="66" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="66" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A66" s="7">
-        <v>46280</v>
+        <v>46281</v>
       </c>
       <c r="B66" s="8"/>
       <c r="C66" s="20" t="s">
         <v>36</v>
       </c>
       <c r="D66" s="10">
-        <v>248.03</v>
+        <v>253.7</v>
       </c>
       <c r="E66" s="10">
-        <v>215.7</v>
+        <v>219.06</v>
       </c>
       <c r="F66" s="10">
-        <v>225.7</v>
-      </c>
-    </row>
-    <row r="67" spans="1:6" x14ac:dyDescent="0.25">
+        <v>229.06</v>
+      </c>
+    </row>
+    <row r="67" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A67" s="11">
-        <v>46280</v>
+        <v>46281</v>
       </c>
       <c r="B67" s="12"/>
       <c r="C67" s="21" t="s">
         <v>37</v>
       </c>
       <c r="D67" s="13">
-        <v>253.53</v>
+        <v>259.20999999999998</v>
       </c>
       <c r="E67" s="13">
-        <v>232.24</v>
+        <v>235.82</v>
       </c>
       <c r="F67" s="13" t="s">
         <v>18</v>
@@ -2151,6 +2151,15 @@
 </file>
 
 <file path=customXml/item2.xml><?xml version="1.0" encoding="utf-8"?>
+<?mso-contentType ?>
+<FormTemplates xmlns="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms">
+  <Display>DocumentLibraryForm</Display>
+  <Edit>DocumentLibraryForm</Edit>
+  <New>DocumentLibraryForm</New>
+</FormTemplates>
+</file>
+
+<file path=customXml/item3.xml><?xml version="1.0" encoding="utf-8"?>
 <p:properties xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls">
   <documentManagement>
     <lcf76f155ced4ddcb4097134ff3c332f xmlns="87276d81-85f4-4ef2-9e6e-55066304288f">
@@ -2159,15 +2168,6 @@
     <TaxCatchAll xmlns="b23b8984-eafa-4e79-985e-54f52f3da58e" xsi:nil="true"/>
   </documentManagement>
 </p:properties>
-</file>
-
-<file path=customXml/item3.xml><?xml version="1.0" encoding="utf-8"?>
-<?mso-contentType ?>
-<FormTemplates xmlns="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms">
-  <Display>DocumentLibraryForm</Display>
-  <Edit>DocumentLibraryForm</Edit>
-  <New>DocumentLibraryForm</New>
-</FormTemplates>
 </file>
 
 <file path=customXml/itemProps1.xml><?xml version="1.0" encoding="utf-8"?>
@@ -2191,6 +2191,14 @@
 </file>
 
 <file path=customXml/itemProps2.xml><?xml version="1.0" encoding="utf-8"?>
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{F60519E9-FD90-4339-869C-BC2F85719BB8}">
+  <ds:schemaRefs>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms"/>
+  </ds:schemaRefs>
+</ds:datastoreItem>
+</file>
+
+<file path=customXml/itemProps3.xml><?xml version="1.0" encoding="utf-8"?>
 <ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{57A83D98-2BAE-4D83-823A-D31C464B620C}">
   <ds:schemaRefs>
     <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/properties"/>
@@ -2201,14 +2209,6 @@
 </ds:datastoreItem>
 </file>
 
-<file path=customXml/itemProps3.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{F60519E9-FD90-4339-869C-BC2F85719BB8}">
-  <ds:schemaRefs>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms"/>
-  </ds:schemaRefs>
-</ds:datastoreItem>
-</file>
-
 <file path=docMetadata/LabelInfo.xml><?xml version="1.0" encoding="utf-8"?>
 <clbl:labelList xmlns:clbl="http://schemas.microsoft.com/office/2020/mipLabelMetadata">
   <clbl:label id="{569bf4a9-87bd-4dbf-a36c-1db5158e5def}" enabled="1" method="Privileged" siteId="{ea80952e-a476-42d4-aaf4-5457852b0f7e}" removed="0"/>

</xml_diff>

<commit_message>
Thu Sep 17 06:13:02 UTC 2026
</commit_message>
<xml_diff>
--- a/bp.com-content-dam-bp-country-sites-en_au-australia-home-products-services-pricing-tgp-excel.xlsx
+++ b/bp.com-content-dam-bp-country-sites-en_au-australia-home-products-services-pricing-tgp-excel.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://bp365.sharepoint.com/sites/WholesalePricing/Shared Documents/B2C/TGP/Daily TGP/Web TGP/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="14_{ABCA24F9-4456-418E-824F-3BAF0E211324}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="14_{36936537-8806-4AD9-A44F-C68AAB4B9FF3}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-110" yWindow="-110" windowWidth="19420" windowHeight="11500" xr2:uid="{1B412EEF-F96D-4DF4-A4E9-C7F0F183C2FB}"/>
+    <workbookView xWindow="-28920" yWindow="-60" windowWidth="29040" windowHeight="15720" xr2:uid="{1B412EEF-F96D-4DF4-A4E9-C7F0F183C2FB}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
@@ -715,15 +715,15 @@
     <pageSetUpPr fitToPage="1"/>
   </sheetPr>
   <dimension ref="A1:G67"/>
-  <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
+  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
-    <col min="1" max="1" width="76.453125" bestFit="1" customWidth="1"/>
-    <col min="2" max="2" width="6.453125"/>
-    <col min="3" max="3" width="18.1796875" bestFit="1" customWidth="1"/>
-    <col min="4" max="7" width="7.1796875" bestFit="1" customWidth="1"/>
+    <col min="1" max="1" width="76.42578125" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="6.42578125"/>
+    <col min="3" max="3" width="18.140625" bestFit="1" customWidth="1"/>
+    <col min="4" max="7" width="7.140625" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:7" ht="22.5" x14ac:dyDescent="0.35">
+    <row r="1" spans="1:7" ht="23.25" x14ac:dyDescent="0.25">
       <c r="A1" s="30" t="s">
         <v>0</v>
       </c>
@@ -734,7 +734,7 @@
       <c r="F1" s="2"/>
       <c r="G1" s="2"/>
     </row>
-    <row r="2" spans="1:7" x14ac:dyDescent="0.35">
+    <row r="2" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A2" s="3"/>
       <c r="B2" s="1"/>
       <c r="C2" s="1"/>
@@ -743,7 +743,7 @@
       <c r="F2" s="2"/>
       <c r="G2" s="2"/>
     </row>
-    <row r="3" spans="1:7" x14ac:dyDescent="0.35">
+    <row r="3" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A3" s="3" t="s">
         <v>1</v>
       </c>
@@ -754,7 +754,7 @@
       <c r="F3" s="2"/>
       <c r="G3" s="2"/>
     </row>
-    <row r="4" spans="1:7" x14ac:dyDescent="0.35">
+    <row r="4" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A4" s="3" t="s">
         <v>2</v>
       </c>
@@ -765,7 +765,7 @@
       <c r="F4" s="2"/>
       <c r="G4" s="2"/>
     </row>
-    <row r="5" spans="1:7" x14ac:dyDescent="0.35">
+    <row r="5" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A5" s="3"/>
       <c r="B5" s="3"/>
       <c r="C5" s="1"/>
@@ -774,7 +774,7 @@
       <c r="F5" s="2"/>
       <c r="G5" s="2"/>
     </row>
-    <row r="6" spans="1:7" ht="20" x14ac:dyDescent="0.35">
+    <row r="6" spans="1:7" ht="20.25" x14ac:dyDescent="0.25">
       <c r="A6" s="29" t="s">
         <v>3</v>
       </c>
@@ -785,7 +785,7 @@
       <c r="F6" s="2"/>
       <c r="G6" s="2"/>
     </row>
-    <row r="7" spans="1:7" x14ac:dyDescent="0.35">
+    <row r="7" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A7" s="4" t="s">
         <v>4</v>
       </c>
@@ -806,133 +806,133 @@
         <v>9</v>
       </c>
     </row>
-    <row r="8" spans="1:7" x14ac:dyDescent="0.35">
+    <row r="8" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A8" s="7">
-        <v>46282</v>
+        <v>46283</v>
       </c>
       <c r="B8" s="8"/>
       <c r="C8" s="9" t="s">
         <v>10</v>
       </c>
       <c r="D8" s="10">
-        <v>264.92</v>
+        <v>270.54000000000002</v>
       </c>
       <c r="E8" s="10">
-        <v>225.88</v>
+        <v>229.63</v>
       </c>
       <c r="F8" s="10">
-        <v>235.88</v>
+        <v>239.63</v>
       </c>
       <c r="G8" s="10">
-        <v>225.84</v>
-      </c>
-    </row>
-    <row r="9" spans="1:7" x14ac:dyDescent="0.35">
+        <v>229.6</v>
+      </c>
+    </row>
+    <row r="9" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A9" s="11">
-        <v>46282</v>
+        <v>46283</v>
       </c>
       <c r="B9" s="12"/>
       <c r="C9" s="12" t="s">
         <v>11</v>
       </c>
       <c r="D9" s="13">
-        <v>264.92</v>
+        <v>270.54000000000002</v>
       </c>
       <c r="E9" s="13">
-        <v>225.88</v>
+        <v>229.63</v>
       </c>
       <c r="F9" s="13">
-        <v>235.88</v>
+        <v>239.63</v>
       </c>
       <c r="G9" s="13">
-        <v>225.84</v>
-      </c>
-    </row>
-    <row r="10" spans="1:7" x14ac:dyDescent="0.35">
+        <v>229.6</v>
+      </c>
+    </row>
+    <row r="10" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A10" s="7">
-        <v>46282</v>
+        <v>46283</v>
       </c>
       <c r="B10" s="8"/>
       <c r="C10" s="9" t="s">
         <v>12</v>
       </c>
       <c r="D10" s="10">
-        <v>259.73</v>
+        <v>266.11</v>
       </c>
       <c r="E10" s="10">
-        <v>221.7</v>
+        <v>225.18</v>
       </c>
       <c r="F10" s="10">
-        <v>231.7</v>
+        <v>235.18</v>
       </c>
       <c r="G10" s="10">
-        <v>222.12</v>
-      </c>
-    </row>
-    <row r="11" spans="1:7" x14ac:dyDescent="0.35">
+        <v>225.6</v>
+      </c>
+    </row>
+    <row r="11" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A11" s="11">
-        <v>46281</v>
+        <v>46282</v>
       </c>
       <c r="B11" s="12"/>
       <c r="C11" s="12" t="s">
         <v>10</v>
       </c>
       <c r="D11" s="13">
-        <v>259.89</v>
+        <v>264.92</v>
       </c>
       <c r="E11" s="13">
-        <v>223.16</v>
+        <v>225.88</v>
       </c>
       <c r="F11" s="13">
-        <v>233.16</v>
+        <v>235.88</v>
       </c>
       <c r="G11" s="13">
-        <v>223.13</v>
-      </c>
-    </row>
-    <row r="12" spans="1:7" x14ac:dyDescent="0.35">
+        <v>225.84</v>
+      </c>
+    </row>
+    <row r="12" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A12" s="7">
-        <v>46281</v>
+        <v>46282</v>
       </c>
       <c r="B12" s="8"/>
       <c r="C12" s="9" t="s">
         <v>11</v>
       </c>
       <c r="D12" s="10">
-        <v>259.89</v>
+        <v>264.92</v>
       </c>
       <c r="E12" s="10">
-        <v>223.16</v>
+        <v>225.88</v>
       </c>
       <c r="F12" s="10">
-        <v>233.16</v>
+        <v>235.88</v>
       </c>
       <c r="G12" s="10">
-        <v>223.13</v>
-      </c>
-    </row>
-    <row r="13" spans="1:7" x14ac:dyDescent="0.35">
+        <v>225.84</v>
+      </c>
+    </row>
+    <row r="13" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A13" s="11">
-        <v>46281</v>
+        <v>46282</v>
       </c>
       <c r="B13" s="12"/>
       <c r="C13" s="12" t="s">
         <v>12</v>
       </c>
       <c r="D13" s="13">
-        <v>254.82</v>
+        <v>259.73</v>
       </c>
       <c r="E13" s="13">
-        <v>219.09</v>
+        <v>221.7</v>
       </c>
       <c r="F13" s="13">
-        <v>229.09</v>
+        <v>231.7</v>
       </c>
       <c r="G13" s="13">
-        <v>219.51</v>
-      </c>
-    </row>
-    <row r="14" spans="1:7" x14ac:dyDescent="0.35">
+        <v>222.12</v>
+      </c>
+    </row>
+    <row r="14" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A14" s="14"/>
       <c r="B14" s="14"/>
       <c r="C14" s="15"/>
@@ -941,7 +941,7 @@
       <c r="F14" s="16"/>
       <c r="G14" s="16"/>
     </row>
-    <row r="15" spans="1:7" ht="20" x14ac:dyDescent="0.35">
+    <row r="15" spans="1:7" ht="20.25" x14ac:dyDescent="0.25">
       <c r="A15" s="29" t="s">
         <v>13</v>
       </c>
@@ -952,7 +952,7 @@
       <c r="F15" s="17"/>
       <c r="G15" s="17"/>
     </row>
-    <row r="16" spans="1:7" x14ac:dyDescent="0.35">
+    <row r="16" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A16" s="4" t="s">
         <v>4</v>
       </c>
@@ -971,45 +971,45 @@
       </c>
       <c r="G16" s="17"/>
     </row>
-    <row r="17" spans="1:7" x14ac:dyDescent="0.35">
+    <row r="17" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A17" s="7">
-        <v>46282</v>
+        <v>46283</v>
       </c>
       <c r="B17" s="8"/>
       <c r="C17" s="20" t="s">
         <v>14</v>
       </c>
       <c r="D17" s="10">
-        <v>264.54000000000002</v>
+        <v>270.87</v>
       </c>
       <c r="E17" s="10">
-        <v>225.85</v>
+        <v>229.29</v>
       </c>
       <c r="F17" s="10">
-        <v>235.85</v>
+        <v>239.29</v>
       </c>
       <c r="G17" s="17"/>
     </row>
-    <row r="18" spans="1:7" x14ac:dyDescent="0.35">
+    <row r="18" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A18" s="11">
-        <v>46281</v>
+        <v>46282</v>
       </c>
       <c r="B18" s="12"/>
       <c r="C18" s="12" t="s">
         <v>14</v>
       </c>
       <c r="D18" s="13">
-        <v>259.69</v>
+        <v>264.54000000000002</v>
       </c>
       <c r="E18" s="13">
-        <v>223.29</v>
+        <v>225.85</v>
       </c>
       <c r="F18" s="13">
-        <v>233.29</v>
+        <v>235.85</v>
       </c>
       <c r="G18" s="17"/>
     </row>
-    <row r="19" spans="1:7" x14ac:dyDescent="0.35">
+    <row r="19" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A19" s="14"/>
       <c r="B19" s="14"/>
       <c r="C19" s="15"/>
@@ -1018,7 +1018,7 @@
       <c r="F19" s="16"/>
       <c r="G19" s="17"/>
     </row>
-    <row r="20" spans="1:7" ht="20" x14ac:dyDescent="0.35">
+    <row r="20" spans="1:7" ht="20.25" x14ac:dyDescent="0.25">
       <c r="A20" s="29" t="s">
         <v>15</v>
       </c>
@@ -1029,7 +1029,7 @@
       <c r="F20" s="17"/>
       <c r="G20" s="17"/>
     </row>
-    <row r="21" spans="1:7" x14ac:dyDescent="0.35">
+    <row r="21" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A21" s="4" t="s">
         <v>4</v>
       </c>
@@ -1050,217 +1050,217 @@
         <v>9</v>
       </c>
     </row>
-    <row r="22" spans="1:7" x14ac:dyDescent="0.35">
+    <row r="22" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A22" s="7">
-        <v>46282</v>
+        <v>46283</v>
       </c>
       <c r="B22" s="8"/>
       <c r="C22" s="20" t="s">
         <v>16</v>
       </c>
       <c r="D22" s="10">
-        <v>264.94</v>
+        <v>270.55</v>
       </c>
       <c r="E22" s="10">
-        <v>224.37</v>
+        <v>227.14</v>
       </c>
       <c r="F22" s="10">
-        <v>233.97</v>
+        <v>236.74</v>
       </c>
       <c r="G22" s="10">
-        <v>223.09</v>
-      </c>
-    </row>
-    <row r="23" spans="1:7" x14ac:dyDescent="0.35">
+        <v>225.85</v>
+      </c>
+    </row>
+    <row r="23" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A23" s="11">
-        <v>46282</v>
+        <v>46283</v>
       </c>
       <c r="B23" s="12"/>
       <c r="C23" s="21" t="s">
         <v>17</v>
       </c>
       <c r="D23" s="13">
-        <v>264.52</v>
+        <v>270.92</v>
       </c>
       <c r="E23" s="13">
-        <v>229.45</v>
+        <v>232.96</v>
       </c>
       <c r="F23" s="13">
-        <v>239.45</v>
+        <v>242.96</v>
       </c>
       <c r="G23" s="13" t="s">
         <v>18</v>
       </c>
     </row>
-    <row r="24" spans="1:7" x14ac:dyDescent="0.35">
+    <row r="24" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A24" s="7">
-        <v>46282</v>
+        <v>46283</v>
       </c>
       <c r="B24" s="8"/>
       <c r="C24" s="20" t="s">
         <v>19</v>
       </c>
       <c r="D24" s="10">
-        <v>265.02999999999997</v>
+        <v>271.42</v>
       </c>
       <c r="E24" s="10">
-        <v>228.72</v>
+        <v>232.22</v>
       </c>
       <c r="F24" s="10">
-        <v>238.72</v>
+        <v>242.22</v>
       </c>
       <c r="G24" s="10" t="s">
         <v>18</v>
       </c>
     </row>
-    <row r="25" spans="1:7" x14ac:dyDescent="0.35">
+    <row r="25" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A25" s="11">
-        <v>46282</v>
+        <v>46283</v>
       </c>
       <c r="B25" s="12"/>
       <c r="C25" s="21" t="s">
         <v>20</v>
       </c>
       <c r="D25" s="13">
-        <v>261.8</v>
+        <v>268.17</v>
       </c>
       <c r="E25" s="13">
-        <v>228.8</v>
+        <v>232.3</v>
       </c>
       <c r="F25" s="13">
-        <v>238.8</v>
+        <v>242.3</v>
       </c>
       <c r="G25" s="13">
-        <v>226.69</v>
-      </c>
-    </row>
-    <row r="26" spans="1:7" x14ac:dyDescent="0.35">
+        <v>230.2</v>
+      </c>
+    </row>
+    <row r="26" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A26" s="7">
-        <v>46282</v>
+        <v>46283</v>
       </c>
       <c r="B26" s="8"/>
       <c r="C26" s="20" t="s">
         <v>21</v>
       </c>
       <c r="D26" s="10">
-        <v>263.58999999999997</v>
+        <v>269.95999999999998</v>
       </c>
       <c r="E26" s="10">
-        <v>230.22</v>
+        <v>233.76</v>
       </c>
       <c r="F26" s="10">
-        <v>240.22</v>
+        <v>243.76</v>
       </c>
       <c r="G26" s="10" t="s">
         <v>18</v>
       </c>
     </row>
-    <row r="27" spans="1:7" x14ac:dyDescent="0.35">
+    <row r="27" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A27" s="11">
-        <v>46281</v>
+        <v>46282</v>
       </c>
       <c r="B27" s="12"/>
       <c r="C27" s="12" t="s">
         <v>16</v>
       </c>
       <c r="D27" s="13">
-        <v>261.02</v>
+        <v>264.94</v>
       </c>
       <c r="E27" s="13">
-        <v>223.86</v>
+        <v>224.37</v>
       </c>
       <c r="F27" s="13">
-        <v>233.46</v>
+        <v>233.97</v>
       </c>
       <c r="G27" s="13">
-        <v>222.57</v>
-      </c>
-    </row>
-    <row r="28" spans="1:7" x14ac:dyDescent="0.35">
+        <v>223.09</v>
+      </c>
+    </row>
+    <row r="28" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A28" s="7">
-        <v>46281</v>
+        <v>46282</v>
       </c>
       <c r="B28" s="8"/>
       <c r="C28" s="20" t="s">
         <v>17</v>
       </c>
       <c r="D28" s="10">
-        <v>259.60000000000002</v>
+        <v>264.52</v>
       </c>
       <c r="E28" s="22">
-        <v>226.81</v>
+        <v>229.45</v>
       </c>
       <c r="F28" s="22">
-        <v>236.81</v>
+        <v>239.45</v>
       </c>
       <c r="G28" s="22" t="s">
         <v>18</v>
       </c>
     </row>
-    <row r="29" spans="1:7" x14ac:dyDescent="0.35">
+    <row r="29" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A29" s="11">
-        <v>46281</v>
+        <v>46282</v>
       </c>
       <c r="B29" s="12"/>
       <c r="C29" s="12" t="s">
         <v>19</v>
       </c>
       <c r="D29" s="13">
-        <v>260.12</v>
+        <v>265.02999999999997</v>
       </c>
       <c r="E29" s="13">
-        <v>226.09</v>
+        <v>228.72</v>
       </c>
       <c r="F29" s="13">
-        <v>236.09</v>
+        <v>238.72</v>
       </c>
       <c r="G29" s="13" t="s">
         <v>18</v>
       </c>
     </row>
-    <row r="30" spans="1:7" x14ac:dyDescent="0.35">
+    <row r="30" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A30" s="7">
-        <v>46281</v>
+        <v>46282</v>
       </c>
       <c r="B30" s="8"/>
       <c r="C30" s="20" t="s">
         <v>20</v>
       </c>
       <c r="D30" s="10">
-        <v>256.89999999999998</v>
+        <v>261.8</v>
       </c>
       <c r="E30" s="22">
-        <v>226.15</v>
+        <v>228.8</v>
       </c>
       <c r="F30" s="22">
-        <v>236.15</v>
+        <v>238.8</v>
       </c>
       <c r="G30" s="22">
-        <v>224.04</v>
-      </c>
-    </row>
-    <row r="31" spans="1:7" x14ac:dyDescent="0.35">
+        <v>226.69</v>
+      </c>
+    </row>
+    <row r="31" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A31" s="11">
-        <v>46281</v>
+        <v>46282</v>
       </c>
       <c r="B31" s="12"/>
       <c r="C31" s="12" t="s">
         <v>21</v>
       </c>
       <c r="D31" s="13">
-        <v>258.69</v>
+        <v>263.58999999999997</v>
       </c>
       <c r="E31" s="13">
-        <v>227.56</v>
+        <v>230.22</v>
       </c>
       <c r="F31" s="13">
-        <v>237.56</v>
+        <v>240.22</v>
       </c>
       <c r="G31" s="13" t="s">
         <v>18</v>
       </c>
     </row>
-    <row r="32" spans="1:7" x14ac:dyDescent="0.35">
+    <row r="32" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A32" s="14"/>
       <c r="B32" s="14"/>
       <c r="C32" s="15"/>
@@ -1269,7 +1269,7 @@
       <c r="F32" s="17"/>
       <c r="G32" s="17"/>
     </row>
-    <row r="33" spans="1:7" ht="20" x14ac:dyDescent="0.35">
+    <row r="33" spans="1:7" ht="20.25" x14ac:dyDescent="0.25">
       <c r="A33" s="29" t="s">
         <v>22</v>
       </c>
@@ -1280,7 +1280,7 @@
       <c r="F33" s="17"/>
       <c r="G33" s="17"/>
     </row>
-    <row r="34" spans="1:7" x14ac:dyDescent="0.35">
+    <row r="34" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A34" s="23" t="s">
         <v>4</v>
       </c>
@@ -1299,54 +1299,54 @@
       </c>
       <c r="G34" s="17"/>
     </row>
-    <row r="35" spans="1:7" x14ac:dyDescent="0.35">
+    <row r="35" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A35" s="7">
-        <v>46282</v>
+        <v>46283</v>
       </c>
       <c r="B35" s="8"/>
       <c r="C35" s="20" t="s">
         <v>23</v>
       </c>
       <c r="D35" s="10">
-        <v>258.26</v>
+        <v>264.64</v>
       </c>
       <c r="E35" s="10">
-        <v>220.65</v>
+        <v>223.56</v>
       </c>
       <c r="F35" s="10">
-        <v>229.65</v>
+        <v>232.56</v>
       </c>
       <c r="G35" s="17"/>
     </row>
-    <row r="36" spans="1:7" x14ac:dyDescent="0.35">
+    <row r="36" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A36" s="11">
-        <v>46281</v>
+        <v>46282</v>
       </c>
       <c r="B36" s="12"/>
       <c r="C36" s="12" t="s">
         <v>23</v>
       </c>
       <c r="D36" s="13">
-        <v>253.35</v>
+        <v>258.26</v>
       </c>
       <c r="E36" s="13">
-        <v>218.04</v>
+        <v>220.65</v>
       </c>
       <c r="F36" s="13">
-        <v>227.04</v>
+        <v>229.65</v>
       </c>
       <c r="G36" s="17"/>
     </row>
-    <row r="37" spans="1:7" x14ac:dyDescent="0.35">
+    <row r="37" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A37" s="7">
-        <v>46282</v>
+        <v>46283</v>
       </c>
       <c r="B37" s="8"/>
       <c r="C37" s="20" t="s">
         <v>24</v>
       </c>
       <c r="D37" s="10">
-        <v>273.88</v>
+        <v>280.26</v>
       </c>
       <c r="E37" s="10" t="s">
         <v>18</v>
@@ -1356,16 +1356,16 @@
       </c>
       <c r="G37" s="17"/>
     </row>
-    <row r="38" spans="1:7" x14ac:dyDescent="0.35">
+    <row r="38" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A38" s="11">
-        <v>46281</v>
+        <v>46282</v>
       </c>
       <c r="B38" s="12"/>
       <c r="C38" s="12" t="s">
         <v>24</v>
       </c>
       <c r="D38" s="13">
-        <v>268.97000000000003</v>
+        <v>273.88</v>
       </c>
       <c r="E38" s="13" t="s">
         <v>18</v>
@@ -1375,7 +1375,7 @@
       </c>
       <c r="G38" s="17"/>
     </row>
-    <row r="39" spans="1:7" x14ac:dyDescent="0.35">
+    <row r="39" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A39" s="24"/>
       <c r="B39" s="24"/>
       <c r="C39" s="15"/>
@@ -1384,7 +1384,7 @@
       <c r="F39" s="17"/>
       <c r="G39" s="17"/>
     </row>
-    <row r="40" spans="1:7" ht="20" x14ac:dyDescent="0.35">
+    <row r="40" spans="1:7" ht="20.25" x14ac:dyDescent="0.25">
       <c r="A40" s="29" t="s">
         <v>25</v>
       </c>
@@ -1395,7 +1395,7 @@
       <c r="F40" s="17"/>
       <c r="G40" s="17"/>
     </row>
-    <row r="41" spans="1:7" x14ac:dyDescent="0.35">
+    <row r="41" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A41" s="23" t="s">
         <v>4</v>
       </c>
@@ -1414,83 +1414,83 @@
       </c>
       <c r="G41" s="17"/>
     </row>
-    <row r="42" spans="1:7" x14ac:dyDescent="0.35">
+    <row r="42" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A42" s="7">
-        <v>46282</v>
+        <v>46283</v>
       </c>
       <c r="B42" s="8"/>
       <c r="C42" s="20" t="s">
         <v>26</v>
       </c>
       <c r="D42" s="10">
-        <v>267.23</v>
+        <v>273.67</v>
       </c>
       <c r="E42" s="10">
-        <v>226.88</v>
+        <v>229.97</v>
       </c>
       <c r="F42" s="10">
-        <v>236.88</v>
+        <v>239.97</v>
       </c>
       <c r="G42" s="17"/>
     </row>
-    <row r="43" spans="1:7" x14ac:dyDescent="0.35">
+    <row r="43" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A43" s="11">
-        <v>46282</v>
+        <v>46283</v>
       </c>
       <c r="B43" s="12"/>
       <c r="C43" s="21" t="s">
         <v>27</v>
       </c>
       <c r="D43" s="13">
-        <v>266.83999999999997</v>
+        <v>273.27</v>
       </c>
       <c r="E43" s="13">
-        <v>227.29</v>
+        <v>230.38</v>
       </c>
       <c r="F43" s="13">
-        <v>237.29</v>
+        <v>240.38</v>
       </c>
       <c r="G43" s="17"/>
     </row>
-    <row r="44" spans="1:7" x14ac:dyDescent="0.35">
+    <row r="44" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A44" s="7">
-        <v>46281</v>
+        <v>46282</v>
       </c>
       <c r="B44" s="8"/>
       <c r="C44" s="20" t="s">
         <v>26</v>
       </c>
       <c r="D44" s="10">
-        <v>262.27</v>
+        <v>267.23</v>
       </c>
       <c r="E44" s="10">
-        <v>224.64</v>
+        <v>226.88</v>
       </c>
       <c r="F44" s="10">
-        <v>234.64</v>
+        <v>236.88</v>
       </c>
       <c r="G44" s="17"/>
     </row>
-    <row r="45" spans="1:7" x14ac:dyDescent="0.35">
+    <row r="45" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A45" s="11">
-        <v>46281</v>
+        <v>46282</v>
       </c>
       <c r="B45" s="12"/>
       <c r="C45" s="21" t="s">
         <v>27</v>
       </c>
       <c r="D45" s="13">
-        <v>261.88</v>
+        <v>266.83999999999997</v>
       </c>
       <c r="E45" s="13">
-        <v>225.06</v>
+        <v>227.29</v>
       </c>
       <c r="F45" s="13">
-        <v>235.06</v>
+        <v>237.29</v>
       </c>
       <c r="G45" s="17"/>
     </row>
-    <row r="46" spans="1:7" x14ac:dyDescent="0.35">
+    <row r="46" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A46" s="14"/>
       <c r="B46" s="24"/>
       <c r="C46" s="15"/>
@@ -1499,7 +1499,7 @@
       <c r="F46" s="16"/>
       <c r="G46" s="17"/>
     </row>
-    <row r="47" spans="1:7" ht="20" x14ac:dyDescent="0.35">
+    <row r="47" spans="1:7" ht="20.25" x14ac:dyDescent="0.25">
       <c r="A47" s="25" t="s">
         <v>28</v>
       </c>
@@ -1510,7 +1510,7 @@
       <c r="F47" s="17"/>
       <c r="G47" s="17"/>
     </row>
-    <row r="48" spans="1:7" x14ac:dyDescent="0.35">
+    <row r="48" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A48" s="23" t="s">
         <v>4</v>
       </c>
@@ -1529,83 +1529,83 @@
       </c>
       <c r="G48" s="17"/>
     </row>
-    <row r="49" spans="1:7" x14ac:dyDescent="0.35">
+    <row r="49" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A49" s="7">
-        <v>46282</v>
+        <v>46283</v>
       </c>
       <c r="B49" s="8"/>
       <c r="C49" s="20" t="s">
         <v>29</v>
       </c>
       <c r="D49" s="10">
-        <v>255.51</v>
+        <v>260.45999999999998</v>
       </c>
       <c r="E49" s="10">
-        <v>219.23</v>
+        <v>222.36</v>
       </c>
       <c r="F49" s="10">
-        <v>229.23</v>
+        <v>232.36</v>
       </c>
       <c r="G49" s="28"/>
     </row>
-    <row r="50" spans="1:7" x14ac:dyDescent="0.35">
+    <row r="50" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A50" s="11">
-        <v>46282</v>
+        <v>46283</v>
       </c>
       <c r="B50" s="12"/>
       <c r="C50" s="21" t="s">
         <v>30</v>
       </c>
       <c r="D50" s="13">
-        <v>253.55</v>
+        <v>258.49</v>
       </c>
       <c r="E50" s="13">
-        <v>219.08</v>
+        <v>222.2</v>
       </c>
       <c r="F50" s="13">
-        <v>229.08</v>
+        <v>232.2</v>
       </c>
       <c r="G50" s="28"/>
     </row>
-    <row r="51" spans="1:7" x14ac:dyDescent="0.35">
+    <row r="51" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A51" s="7">
-        <v>46281</v>
+        <v>46282</v>
       </c>
       <c r="B51" s="8"/>
       <c r="C51" s="20" t="s">
         <v>29</v>
       </c>
       <c r="D51" s="10">
-        <v>251.06</v>
+        <v>255.51</v>
       </c>
       <c r="E51" s="10">
-        <v>215.99</v>
+        <v>219.23</v>
       </c>
       <c r="F51" s="10">
-        <v>225.99</v>
+        <v>229.23</v>
       </c>
       <c r="G51" s="17"/>
     </row>
-    <row r="52" spans="1:7" x14ac:dyDescent="0.35">
+    <row r="52" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A52" s="11">
-        <v>46281</v>
+        <v>46282</v>
       </c>
       <c r="B52" s="12"/>
       <c r="C52" s="21" t="s">
         <v>30</v>
       </c>
       <c r="D52" s="13">
-        <v>249.13</v>
+        <v>253.55</v>
       </c>
       <c r="E52" s="13">
-        <v>215.85</v>
+        <v>219.08</v>
       </c>
       <c r="F52" s="13">
-        <v>225.85</v>
+        <v>229.08</v>
       </c>
       <c r="G52" s="17"/>
     </row>
-    <row r="53" spans="1:7" x14ac:dyDescent="0.35">
+    <row r="53" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A53" s="14"/>
       <c r="B53" s="14"/>
       <c r="C53" s="15"/>
@@ -1614,7 +1614,7 @@
       <c r="F53" s="16"/>
       <c r="G53" s="17"/>
     </row>
-    <row r="54" spans="1:7" ht="20" x14ac:dyDescent="0.35">
+    <row r="54" spans="1:7" ht="20.25" x14ac:dyDescent="0.25">
       <c r="A54" s="27" t="s">
         <v>31</v>
       </c>
@@ -1625,7 +1625,7 @@
       <c r="F54" s="17"/>
       <c r="G54" s="17"/>
     </row>
-    <row r="55" spans="1:7" x14ac:dyDescent="0.35">
+    <row r="55" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A55" s="23" t="s">
         <v>4</v>
       </c>
@@ -1644,54 +1644,54 @@
       </c>
       <c r="G55" s="17"/>
     </row>
-    <row r="56" spans="1:7" x14ac:dyDescent="0.35">
+    <row r="56" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A56" s="7">
-        <v>46282</v>
+        <v>46283</v>
       </c>
       <c r="B56" s="8"/>
       <c r="C56" s="20" t="s">
         <v>32</v>
       </c>
       <c r="D56" s="10">
-        <v>276.39999999999998</v>
+        <v>282.8</v>
       </c>
       <c r="E56" s="10">
-        <v>242.85</v>
+        <v>246.55</v>
       </c>
       <c r="F56" s="10">
-        <v>252.85</v>
+        <v>256.55</v>
       </c>
       <c r="G56" s="17"/>
     </row>
-    <row r="57" spans="1:7" x14ac:dyDescent="0.35">
+    <row r="57" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A57" s="11">
-        <v>46282</v>
+        <v>46283</v>
       </c>
       <c r="B57" s="12"/>
       <c r="C57" s="21" t="s">
         <v>33</v>
       </c>
       <c r="D57" s="13">
-        <v>265.33999999999997</v>
+        <v>271.74</v>
       </c>
       <c r="E57" s="13">
-        <v>231.28</v>
+        <v>234.69</v>
       </c>
       <c r="F57" s="13">
-        <v>241.28</v>
+        <v>244.69</v>
       </c>
       <c r="G57" s="17"/>
     </row>
-    <row r="58" spans="1:7" x14ac:dyDescent="0.35">
+    <row r="58" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A58" s="7">
-        <v>46282</v>
+        <v>46283</v>
       </c>
       <c r="B58" s="8"/>
       <c r="C58" s="20" t="s">
         <v>34</v>
       </c>
       <c r="D58" s="10">
-        <v>266.57</v>
+        <v>272.97000000000003</v>
       </c>
       <c r="E58" s="10" t="s">
         <v>18</v>
@@ -1701,111 +1701,111 @@
       </c>
       <c r="G58" s="17"/>
     </row>
-    <row r="59" spans="1:7" x14ac:dyDescent="0.35">
+    <row r="59" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A59" s="11">
-        <v>46282</v>
+        <v>46283</v>
       </c>
       <c r="B59" s="12"/>
       <c r="C59" s="21" t="s">
         <v>35</v>
       </c>
       <c r="D59" s="13">
-        <v>262.7</v>
+        <v>269</v>
       </c>
       <c r="E59" s="13">
-        <v>225.66</v>
+        <v>229.07</v>
       </c>
       <c r="F59" s="13" t="s">
         <v>18</v>
       </c>
       <c r="G59" s="17"/>
     </row>
-    <row r="60" spans="1:7" x14ac:dyDescent="0.35">
+    <row r="60" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A60" s="7">
-        <v>46282</v>
+        <v>46283</v>
       </c>
       <c r="B60" s="8"/>
       <c r="C60" s="20" t="s">
         <v>36</v>
       </c>
       <c r="D60" s="10">
-        <v>258.52999999999997</v>
+        <v>264.83999999999997</v>
       </c>
       <c r="E60" s="10">
-        <v>221.6</v>
+        <v>225.01</v>
       </c>
       <c r="F60" s="10">
-        <v>231.6</v>
+        <v>235.01</v>
       </c>
       <c r="G60" s="17"/>
     </row>
-    <row r="61" spans="1:7" x14ac:dyDescent="0.35">
+    <row r="61" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A61" s="11">
-        <v>46282</v>
+        <v>46283</v>
       </c>
       <c r="B61" s="12"/>
       <c r="C61" s="21" t="s">
         <v>37</v>
       </c>
       <c r="D61" s="13">
-        <v>264.02999999999997</v>
+        <v>270.33</v>
       </c>
       <c r="E61" s="13">
-        <v>238.59</v>
+        <v>242.19</v>
       </c>
       <c r="F61" s="13" t="s">
         <v>18</v>
       </c>
       <c r="G61" s="17"/>
     </row>
-    <row r="62" spans="1:7" x14ac:dyDescent="0.35">
+    <row r="62" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A62" s="7">
-        <v>46281</v>
+        <v>46282</v>
       </c>
       <c r="B62" s="8"/>
       <c r="C62" s="20" t="s">
         <v>32</v>
       </c>
       <c r="D62" s="10">
-        <v>271.49</v>
+        <v>276.39999999999998</v>
       </c>
       <c r="E62" s="10">
-        <v>239.99</v>
+        <v>242.85</v>
       </c>
       <c r="F62" s="10">
-        <v>249.99</v>
+        <v>252.85</v>
       </c>
       <c r="G62" s="17"/>
     </row>
-    <row r="63" spans="1:7" x14ac:dyDescent="0.35">
+    <row r="63" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A63" s="11">
-        <v>46281</v>
+        <v>46282</v>
       </c>
       <c r="B63" s="12"/>
       <c r="C63" s="21" t="s">
         <v>33</v>
       </c>
       <c r="D63" s="13">
-        <v>260.42</v>
+        <v>265.33999999999997</v>
       </c>
       <c r="E63" s="13">
-        <v>228.74</v>
+        <v>231.28</v>
       </c>
       <c r="F63" s="13">
-        <v>238.74</v>
+        <v>241.28</v>
       </c>
       <c r="G63" s="17"/>
     </row>
-    <row r="64" spans="1:7" x14ac:dyDescent="0.35">
+    <row r="64" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A64" s="7">
-        <v>46281</v>
+        <v>46282</v>
       </c>
       <c r="B64" s="8"/>
       <c r="C64" s="20" t="s">
         <v>34</v>
       </c>
       <c r="D64" s="10">
-        <v>261.64999999999998</v>
+        <v>266.57</v>
       </c>
       <c r="E64" s="10" t="s">
         <v>18</v>
@@ -1815,55 +1815,55 @@
       </c>
       <c r="G64" s="17"/>
     </row>
-    <row r="65" spans="1:6" x14ac:dyDescent="0.35">
+    <row r="65" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A65" s="11">
-        <v>46281</v>
+        <v>46282</v>
       </c>
       <c r="B65" s="12"/>
       <c r="C65" s="21" t="s">
         <v>35</v>
       </c>
       <c r="D65" s="13">
-        <v>257.88</v>
+        <v>262.7</v>
       </c>
       <c r="E65" s="13">
-        <v>223.13</v>
+        <v>225.66</v>
       </c>
       <c r="F65" s="13" t="s">
         <v>18</v>
       </c>
     </row>
-    <row r="66" spans="1:6" x14ac:dyDescent="0.35">
+    <row r="66" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A66" s="7">
-        <v>46281</v>
+        <v>46282</v>
       </c>
       <c r="B66" s="8"/>
       <c r="C66" s="20" t="s">
         <v>36</v>
       </c>
       <c r="D66" s="10">
-        <v>253.7</v>
+        <v>258.52999999999997</v>
       </c>
       <c r="E66" s="10">
-        <v>219.06</v>
+        <v>221.6</v>
       </c>
       <c r="F66" s="10">
-        <v>229.06</v>
-      </c>
-    </row>
-    <row r="67" spans="1:6" x14ac:dyDescent="0.35">
+        <v>231.6</v>
+      </c>
+    </row>
+    <row r="67" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A67" s="11">
-        <v>46281</v>
+        <v>46282</v>
       </c>
       <c r="B67" s="12"/>
       <c r="C67" s="21" t="s">
         <v>37</v>
       </c>
       <c r="D67" s="13">
-        <v>259.20999999999998</v>
+        <v>264.02999999999997</v>
       </c>
       <c r="E67" s="13">
-        <v>235.82</v>
+        <v>238.59</v>
       </c>
       <c r="F67" s="13" t="s">
         <v>18</v>

</xml_diff>

<commit_message>
Fri Sep 18 06:02:57 UTC 2026
</commit_message>
<xml_diff>
--- a/bp.com-content-dam-bp-country-sites-en_au-australia-home-products-services-pricing-tgp-excel.xlsx
+++ b/bp.com-content-dam-bp-country-sites-en_au-australia-home-products-services-pricing-tgp-excel.xlsx
@@ -8,14 +8,14 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://bp365.sharepoint.com/sites/WholesalePricing/Shared Documents/B2C/TGP/Daily TGP/Web TGP/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="14_{36936537-8806-4AD9-A44F-C68AAB4B9FF3}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="14_{BA4C5F24-5100-4C3E-A877-C0C02CFC31A1}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-28920" yWindow="-60" windowWidth="29040" windowHeight="15720" xr2:uid="{1B412EEF-F96D-4DF4-A4E9-C7F0F183C2FB}"/>
+    <workbookView xWindow="28680" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{1B412EEF-F96D-4DF4-A4E9-C7F0F183C2FB}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
   </sheets>
-  <calcPr calcId="191028" concurrentManualCount="12"/>
+  <calcPr calcId="191028"/>
   <extLst>
     <ext xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" uri="{140A7094-0E35-4892-8432-C4D2E57EDEB5}">
       <x15:workbookPr chartTrackingRefBase="1"/>
@@ -808,128 +808,128 @@
     </row>
     <row r="8" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A8" s="7">
-        <v>46283</v>
+        <v>46284</v>
       </c>
       <c r="B8" s="8"/>
       <c r="C8" s="9" t="s">
         <v>10</v>
       </c>
       <c r="D8" s="10">
-        <v>270.54000000000002</v>
+        <v>275.92</v>
       </c>
       <c r="E8" s="10">
-        <v>229.63</v>
+        <v>233.2</v>
       </c>
       <c r="F8" s="10">
-        <v>239.63</v>
+        <v>243.2</v>
       </c>
       <c r="G8" s="10">
-        <v>229.6</v>
+        <v>233.16</v>
       </c>
     </row>
     <row r="9" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A9" s="11">
-        <v>46283</v>
+        <v>46284</v>
       </c>
       <c r="B9" s="12"/>
       <c r="C9" s="12" t="s">
         <v>11</v>
       </c>
       <c r="D9" s="13">
-        <v>270.54000000000002</v>
+        <v>275.92</v>
       </c>
       <c r="E9" s="13">
-        <v>229.63</v>
+        <v>233.2</v>
       </c>
       <c r="F9" s="13">
-        <v>239.63</v>
+        <v>243.2</v>
       </c>
       <c r="G9" s="13">
-        <v>229.6</v>
+        <v>233.16</v>
       </c>
     </row>
     <row r="10" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A10" s="7">
-        <v>46283</v>
+        <v>46284</v>
       </c>
       <c r="B10" s="8"/>
       <c r="C10" s="9" t="s">
         <v>12</v>
       </c>
       <c r="D10" s="10">
-        <v>266.11</v>
+        <v>271.10000000000002</v>
       </c>
       <c r="E10" s="10">
-        <v>225.18</v>
+        <v>228.4</v>
       </c>
       <c r="F10" s="10">
-        <v>235.18</v>
+        <v>238.4</v>
       </c>
       <c r="G10" s="10">
-        <v>225.6</v>
+        <v>228.82</v>
       </c>
     </row>
     <row r="11" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A11" s="11">
-        <v>46282</v>
+        <v>46283</v>
       </c>
       <c r="B11" s="12"/>
       <c r="C11" s="12" t="s">
         <v>10</v>
       </c>
       <c r="D11" s="13">
-        <v>264.92</v>
+        <v>270.54000000000002</v>
       </c>
       <c r="E11" s="13">
-        <v>225.88</v>
+        <v>229.63</v>
       </c>
       <c r="F11" s="13">
-        <v>235.88</v>
+        <v>239.63</v>
       </c>
       <c r="G11" s="13">
-        <v>225.84</v>
+        <v>229.6</v>
       </c>
     </row>
     <row r="12" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A12" s="7">
-        <v>46282</v>
+        <v>46283</v>
       </c>
       <c r="B12" s="8"/>
       <c r="C12" s="9" t="s">
         <v>11</v>
       </c>
       <c r="D12" s="10">
-        <v>264.92</v>
+        <v>270.54000000000002</v>
       </c>
       <c r="E12" s="10">
-        <v>225.88</v>
+        <v>229.63</v>
       </c>
       <c r="F12" s="10">
-        <v>235.88</v>
+        <v>239.63</v>
       </c>
       <c r="G12" s="10">
-        <v>225.84</v>
+        <v>229.6</v>
       </c>
     </row>
     <row r="13" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A13" s="11">
-        <v>46282</v>
+        <v>46283</v>
       </c>
       <c r="B13" s="12"/>
       <c r="C13" s="12" t="s">
         <v>12</v>
       </c>
       <c r="D13" s="13">
-        <v>259.73</v>
+        <v>266.11</v>
       </c>
       <c r="E13" s="13">
-        <v>221.7</v>
+        <v>225.18</v>
       </c>
       <c r="F13" s="13">
-        <v>231.7</v>
+        <v>235.18</v>
       </c>
       <c r="G13" s="13">
-        <v>222.12</v>
+        <v>225.6</v>
       </c>
     </row>
     <row r="14" spans="1:7" x14ac:dyDescent="0.25">
@@ -973,39 +973,39 @@
     </row>
     <row r="17" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A17" s="7">
-        <v>46283</v>
+        <v>46284</v>
       </c>
       <c r="B17" s="8"/>
       <c r="C17" s="20" t="s">
         <v>14</v>
       </c>
       <c r="D17" s="10">
-        <v>270.87</v>
+        <v>275.79000000000002</v>
       </c>
       <c r="E17" s="10">
-        <v>229.29</v>
+        <v>232.46</v>
       </c>
       <c r="F17" s="10">
-        <v>239.29</v>
+        <v>242.46</v>
       </c>
       <c r="G17" s="17"/>
     </row>
     <row r="18" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A18" s="11">
-        <v>46282</v>
+        <v>46283</v>
       </c>
       <c r="B18" s="12"/>
       <c r="C18" s="12" t="s">
         <v>14</v>
       </c>
       <c r="D18" s="13">
-        <v>264.54000000000002</v>
+        <v>270.87</v>
       </c>
       <c r="E18" s="13">
-        <v>225.85</v>
+        <v>229.29</v>
       </c>
       <c r="F18" s="13">
-        <v>235.85</v>
+        <v>239.29</v>
       </c>
       <c r="G18" s="17"/>
     </row>
@@ -1052,41 +1052,41 @@
     </row>
     <row r="22" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A22" s="7">
-        <v>46283</v>
+        <v>46284</v>
       </c>
       <c r="B22" s="8"/>
       <c r="C22" s="20" t="s">
         <v>16</v>
       </c>
       <c r="D22" s="10">
-        <v>270.55</v>
+        <v>275.93</v>
       </c>
       <c r="E22" s="10">
-        <v>227.14</v>
+        <v>231.14</v>
       </c>
       <c r="F22" s="10">
-        <v>236.74</v>
+        <v>240.74</v>
       </c>
       <c r="G22" s="10">
-        <v>225.85</v>
+        <v>229.86</v>
       </c>
     </row>
     <row r="23" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A23" s="11">
-        <v>46283</v>
+        <v>46284</v>
       </c>
       <c r="B23" s="12"/>
       <c r="C23" s="21" t="s">
         <v>17</v>
       </c>
       <c r="D23" s="13">
-        <v>270.92</v>
+        <v>275.92</v>
       </c>
       <c r="E23" s="13">
-        <v>232.96</v>
+        <v>236.22</v>
       </c>
       <c r="F23" s="13">
-        <v>242.96</v>
+        <v>246.22</v>
       </c>
       <c r="G23" s="13" t="s">
         <v>18</v>
@@ -1094,20 +1094,20 @@
     </row>
     <row r="24" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A24" s="7">
-        <v>46283</v>
+        <v>46284</v>
       </c>
       <c r="B24" s="8"/>
       <c r="C24" s="20" t="s">
         <v>19</v>
       </c>
       <c r="D24" s="10">
-        <v>271.42</v>
+        <v>276.41000000000003</v>
       </c>
       <c r="E24" s="10">
-        <v>232.22</v>
+        <v>235.47</v>
       </c>
       <c r="F24" s="10">
-        <v>242.22</v>
+        <v>245.47</v>
       </c>
       <c r="G24" s="10" t="s">
         <v>18</v>
@@ -1115,41 +1115,41 @@
     </row>
     <row r="25" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A25" s="11">
-        <v>46283</v>
+        <v>46284</v>
       </c>
       <c r="B25" s="12"/>
       <c r="C25" s="21" t="s">
         <v>20</v>
       </c>
       <c r="D25" s="13">
-        <v>268.17</v>
+        <v>273.16000000000003</v>
       </c>
       <c r="E25" s="13">
-        <v>232.3</v>
+        <v>235.57</v>
       </c>
       <c r="F25" s="13">
-        <v>242.3</v>
+        <v>245.57</v>
       </c>
       <c r="G25" s="13">
-        <v>230.2</v>
+        <v>233.47</v>
       </c>
     </row>
     <row r="26" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A26" s="7">
-        <v>46283</v>
+        <v>46284</v>
       </c>
       <c r="B26" s="8"/>
       <c r="C26" s="20" t="s">
         <v>21</v>
       </c>
       <c r="D26" s="10">
-        <v>269.95999999999998</v>
+        <v>274.94</v>
       </c>
       <c r="E26" s="10">
-        <v>233.76</v>
+        <v>237.05</v>
       </c>
       <c r="F26" s="10">
-        <v>243.76</v>
+        <v>247.05</v>
       </c>
       <c r="G26" s="10" t="s">
         <v>18</v>
@@ -1157,41 +1157,41 @@
     </row>
     <row r="27" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A27" s="11">
-        <v>46282</v>
+        <v>46283</v>
       </c>
       <c r="B27" s="12"/>
       <c r="C27" s="12" t="s">
         <v>16</v>
       </c>
       <c r="D27" s="13">
-        <v>264.94</v>
+        <v>270.55</v>
       </c>
       <c r="E27" s="13">
-        <v>224.37</v>
+        <v>227.14</v>
       </c>
       <c r="F27" s="13">
-        <v>233.97</v>
+        <v>236.74</v>
       </c>
       <c r="G27" s="13">
-        <v>223.09</v>
+        <v>225.85</v>
       </c>
     </row>
     <row r="28" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A28" s="7">
-        <v>46282</v>
+        <v>46283</v>
       </c>
       <c r="B28" s="8"/>
       <c r="C28" s="20" t="s">
         <v>17</v>
       </c>
       <c r="D28" s="10">
-        <v>264.52</v>
+        <v>270.92</v>
       </c>
       <c r="E28" s="22">
-        <v>229.45</v>
+        <v>232.96</v>
       </c>
       <c r="F28" s="22">
-        <v>239.45</v>
+        <v>242.96</v>
       </c>
       <c r="G28" s="22" t="s">
         <v>18</v>
@@ -1199,20 +1199,20 @@
     </row>
     <row r="29" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A29" s="11">
-        <v>46282</v>
+        <v>46283</v>
       </c>
       <c r="B29" s="12"/>
       <c r="C29" s="12" t="s">
         <v>19</v>
       </c>
       <c r="D29" s="13">
-        <v>265.02999999999997</v>
+        <v>271.42</v>
       </c>
       <c r="E29" s="13">
-        <v>228.72</v>
+        <v>232.22</v>
       </c>
       <c r="F29" s="13">
-        <v>238.72</v>
+        <v>242.22</v>
       </c>
       <c r="G29" s="13" t="s">
         <v>18</v>
@@ -1220,41 +1220,41 @@
     </row>
     <row r="30" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A30" s="7">
-        <v>46282</v>
+        <v>46283</v>
       </c>
       <c r="B30" s="8"/>
       <c r="C30" s="20" t="s">
         <v>20</v>
       </c>
       <c r="D30" s="10">
-        <v>261.8</v>
+        <v>268.17</v>
       </c>
       <c r="E30" s="22">
-        <v>228.8</v>
+        <v>232.3</v>
       </c>
       <c r="F30" s="22">
-        <v>238.8</v>
+        <v>242.3</v>
       </c>
       <c r="G30" s="22">
-        <v>226.69</v>
+        <v>230.2</v>
       </c>
     </row>
     <row r="31" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A31" s="11">
-        <v>46282</v>
+        <v>46283</v>
       </c>
       <c r="B31" s="12"/>
       <c r="C31" s="12" t="s">
         <v>21</v>
       </c>
       <c r="D31" s="13">
-        <v>263.58999999999997</v>
+        <v>269.95999999999998</v>
       </c>
       <c r="E31" s="13">
-        <v>230.22</v>
+        <v>233.76</v>
       </c>
       <c r="F31" s="13">
-        <v>240.22</v>
+        <v>243.76</v>
       </c>
       <c r="G31" s="13" t="s">
         <v>18</v>
@@ -1301,52 +1301,52 @@
     </row>
     <row r="35" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A35" s="7">
-        <v>46283</v>
+        <v>46284</v>
       </c>
       <c r="B35" s="8"/>
       <c r="C35" s="20" t="s">
         <v>23</v>
       </c>
       <c r="D35" s="10">
-        <v>264.64</v>
+        <v>269.63</v>
       </c>
       <c r="E35" s="10">
-        <v>223.56</v>
+        <v>227.22</v>
       </c>
       <c r="F35" s="10">
-        <v>232.56</v>
+        <v>236.22</v>
       </c>
       <c r="G35" s="17"/>
     </row>
     <row r="36" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A36" s="11">
-        <v>46282</v>
+        <v>46283</v>
       </c>
       <c r="B36" s="12"/>
       <c r="C36" s="12" t="s">
         <v>23</v>
       </c>
       <c r="D36" s="13">
-        <v>258.26</v>
+        <v>264.64</v>
       </c>
       <c r="E36" s="13">
-        <v>220.65</v>
+        <v>223.56</v>
       </c>
       <c r="F36" s="13">
-        <v>229.65</v>
+        <v>232.56</v>
       </c>
       <c r="G36" s="17"/>
     </row>
     <row r="37" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A37" s="7">
-        <v>46283</v>
+        <v>46284</v>
       </c>
       <c r="B37" s="8"/>
       <c r="C37" s="20" t="s">
         <v>24</v>
       </c>
       <c r="D37" s="10">
-        <v>280.26</v>
+        <v>285.25</v>
       </c>
       <c r="E37" s="10" t="s">
         <v>18</v>
@@ -1358,14 +1358,14 @@
     </row>
     <row r="38" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A38" s="11">
-        <v>46282</v>
+        <v>46283</v>
       </c>
       <c r="B38" s="12"/>
       <c r="C38" s="12" t="s">
         <v>24</v>
       </c>
       <c r="D38" s="13">
-        <v>273.88</v>
+        <v>280.26</v>
       </c>
       <c r="E38" s="13" t="s">
         <v>18</v>
@@ -1416,77 +1416,77 @@
     </row>
     <row r="42" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A42" s="7">
-        <v>46283</v>
+        <v>46284</v>
       </c>
       <c r="B42" s="8"/>
       <c r="C42" s="20" t="s">
         <v>26</v>
       </c>
       <c r="D42" s="10">
-        <v>273.67</v>
+        <v>278.72000000000003</v>
       </c>
       <c r="E42" s="10">
-        <v>229.97</v>
+        <v>232.81</v>
       </c>
       <c r="F42" s="10">
-        <v>239.97</v>
+        <v>242.81</v>
       </c>
       <c r="G42" s="17"/>
     </row>
     <row r="43" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A43" s="11">
-        <v>46283</v>
+        <v>46284</v>
       </c>
       <c r="B43" s="12"/>
       <c r="C43" s="21" t="s">
         <v>27</v>
       </c>
       <c r="D43" s="13">
-        <v>273.27</v>
+        <v>278.31</v>
       </c>
       <c r="E43" s="13">
-        <v>230.38</v>
+        <v>233.23</v>
       </c>
       <c r="F43" s="13">
-        <v>240.38</v>
+        <v>243.23</v>
       </c>
       <c r="G43" s="17"/>
     </row>
     <row r="44" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A44" s="7">
-        <v>46282</v>
+        <v>46283</v>
       </c>
       <c r="B44" s="8"/>
       <c r="C44" s="20" t="s">
         <v>26</v>
       </c>
       <c r="D44" s="10">
-        <v>267.23</v>
+        <v>273.67</v>
       </c>
       <c r="E44" s="10">
-        <v>226.88</v>
+        <v>229.97</v>
       </c>
       <c r="F44" s="10">
-        <v>236.88</v>
+        <v>239.97</v>
       </c>
       <c r="G44" s="17"/>
     </row>
     <row r="45" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A45" s="11">
-        <v>46282</v>
+        <v>46283</v>
       </c>
       <c r="B45" s="12"/>
       <c r="C45" s="21" t="s">
         <v>27</v>
       </c>
       <c r="D45" s="13">
-        <v>266.83999999999997</v>
+        <v>273.27</v>
       </c>
       <c r="E45" s="13">
-        <v>227.29</v>
+        <v>230.38</v>
       </c>
       <c r="F45" s="13">
-        <v>237.29</v>
+        <v>240.38</v>
       </c>
       <c r="G45" s="17"/>
     </row>
@@ -1531,77 +1531,77 @@
     </row>
     <row r="49" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A49" s="7">
-        <v>46283</v>
+        <v>46284</v>
       </c>
       <c r="B49" s="8"/>
       <c r="C49" s="20" t="s">
         <v>29</v>
       </c>
       <c r="D49" s="10">
-        <v>260.45999999999998</v>
+        <v>263.76</v>
       </c>
       <c r="E49" s="10">
-        <v>222.36</v>
+        <v>224.63</v>
       </c>
       <c r="F49" s="10">
-        <v>232.36</v>
+        <v>234.63</v>
       </c>
       <c r="G49" s="28"/>
     </row>
     <row r="50" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A50" s="11">
-        <v>46283</v>
+        <v>46284</v>
       </c>
       <c r="B50" s="12"/>
       <c r="C50" s="21" t="s">
         <v>30</v>
       </c>
       <c r="D50" s="13">
-        <v>258.49</v>
+        <v>261.77</v>
       </c>
       <c r="E50" s="13">
-        <v>222.2</v>
+        <v>224.47</v>
       </c>
       <c r="F50" s="13">
-        <v>232.2</v>
+        <v>234.47</v>
       </c>
       <c r="G50" s="28"/>
     </row>
     <row r="51" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A51" s="7">
-        <v>46282</v>
+        <v>46283</v>
       </c>
       <c r="B51" s="8"/>
       <c r="C51" s="20" t="s">
         <v>29</v>
       </c>
       <c r="D51" s="10">
-        <v>255.51</v>
+        <v>260.45999999999998</v>
       </c>
       <c r="E51" s="10">
-        <v>219.23</v>
+        <v>222.36</v>
       </c>
       <c r="F51" s="10">
-        <v>229.23</v>
+        <v>232.36</v>
       </c>
       <c r="G51" s="17"/>
     </row>
     <row r="52" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A52" s="11">
-        <v>46282</v>
+        <v>46283</v>
       </c>
       <c r="B52" s="12"/>
       <c r="C52" s="21" t="s">
         <v>30</v>
       </c>
       <c r="D52" s="13">
-        <v>253.55</v>
+        <v>258.49</v>
       </c>
       <c r="E52" s="13">
-        <v>219.08</v>
+        <v>222.2</v>
       </c>
       <c r="F52" s="13">
-        <v>229.08</v>
+        <v>232.2</v>
       </c>
       <c r="G52" s="17"/>
     </row>
@@ -1646,52 +1646,52 @@
     </row>
     <row r="56" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A56" s="7">
-        <v>46283</v>
+        <v>46284</v>
       </c>
       <c r="B56" s="8"/>
       <c r="C56" s="20" t="s">
         <v>32</v>
       </c>
       <c r="D56" s="10">
-        <v>282.8</v>
+        <v>287.8</v>
       </c>
       <c r="E56" s="10">
-        <v>246.55</v>
+        <v>250.05</v>
       </c>
       <c r="F56" s="10">
-        <v>256.55</v>
+        <v>260.05</v>
       </c>
       <c r="G56" s="17"/>
     </row>
     <row r="57" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A57" s="11">
-        <v>46283</v>
+        <v>46284</v>
       </c>
       <c r="B57" s="12"/>
       <c r="C57" s="21" t="s">
         <v>33</v>
       </c>
       <c r="D57" s="13">
-        <v>271.74</v>
+        <v>276.74</v>
       </c>
       <c r="E57" s="13">
-        <v>234.69</v>
+        <v>237.83</v>
       </c>
       <c r="F57" s="13">
-        <v>244.69</v>
+        <v>247.83</v>
       </c>
       <c r="G57" s="17"/>
     </row>
     <row r="58" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A58" s="7">
-        <v>46283</v>
+        <v>46284</v>
       </c>
       <c r="B58" s="8"/>
       <c r="C58" s="20" t="s">
         <v>34</v>
       </c>
       <c r="D58" s="10">
-        <v>272.97000000000003</v>
+        <v>277.98</v>
       </c>
       <c r="E58" s="10" t="s">
         <v>18</v>
@@ -1703,17 +1703,17 @@
     </row>
     <row r="59" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A59" s="11">
-        <v>46283</v>
+        <v>46284</v>
       </c>
       <c r="B59" s="12"/>
       <c r="C59" s="21" t="s">
         <v>35</v>
       </c>
       <c r="D59" s="13">
-        <v>269</v>
+        <v>273.89999999999998</v>
       </c>
       <c r="E59" s="13">
-        <v>229.07</v>
+        <v>232.21</v>
       </c>
       <c r="F59" s="13" t="s">
         <v>18</v>
@@ -1722,36 +1722,36 @@
     </row>
     <row r="60" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A60" s="7">
-        <v>46283</v>
+        <v>46284</v>
       </c>
       <c r="B60" s="8"/>
       <c r="C60" s="20" t="s">
         <v>36</v>
       </c>
       <c r="D60" s="10">
-        <v>264.83999999999997</v>
+        <v>269.74</v>
       </c>
       <c r="E60" s="10">
-        <v>225.01</v>
+        <v>228.15</v>
       </c>
       <c r="F60" s="10">
-        <v>235.01</v>
+        <v>238.15</v>
       </c>
       <c r="G60" s="17"/>
     </row>
     <row r="61" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A61" s="11">
-        <v>46283</v>
+        <v>46284</v>
       </c>
       <c r="B61" s="12"/>
       <c r="C61" s="21" t="s">
         <v>37</v>
       </c>
       <c r="D61" s="13">
-        <v>270.33</v>
+        <v>275.23</v>
       </c>
       <c r="E61" s="13">
-        <v>242.19</v>
+        <v>245.58</v>
       </c>
       <c r="F61" s="13" t="s">
         <v>18</v>
@@ -1760,52 +1760,52 @@
     </row>
     <row r="62" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A62" s="7">
-        <v>46282</v>
+        <v>46283</v>
       </c>
       <c r="B62" s="8"/>
       <c r="C62" s="20" t="s">
         <v>32</v>
       </c>
       <c r="D62" s="10">
-        <v>276.39999999999998</v>
+        <v>282.8</v>
       </c>
       <c r="E62" s="10">
-        <v>242.85</v>
+        <v>246.55</v>
       </c>
       <c r="F62" s="10">
-        <v>252.85</v>
+        <v>256.55</v>
       </c>
       <c r="G62" s="17"/>
     </row>
     <row r="63" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A63" s="11">
-        <v>46282</v>
+        <v>46283</v>
       </c>
       <c r="B63" s="12"/>
       <c r="C63" s="21" t="s">
         <v>33</v>
       </c>
       <c r="D63" s="13">
-        <v>265.33999999999997</v>
+        <v>271.74</v>
       </c>
       <c r="E63" s="13">
-        <v>231.28</v>
+        <v>234.69</v>
       </c>
       <c r="F63" s="13">
-        <v>241.28</v>
+        <v>244.69</v>
       </c>
       <c r="G63" s="17"/>
     </row>
     <row r="64" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A64" s="7">
-        <v>46282</v>
+        <v>46283</v>
       </c>
       <c r="B64" s="8"/>
       <c r="C64" s="20" t="s">
         <v>34</v>
       </c>
       <c r="D64" s="10">
-        <v>266.57</v>
+        <v>272.97000000000003</v>
       </c>
       <c r="E64" s="10" t="s">
         <v>18</v>
@@ -1817,17 +1817,17 @@
     </row>
     <row r="65" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A65" s="11">
-        <v>46282</v>
+        <v>46283</v>
       </c>
       <c r="B65" s="12"/>
       <c r="C65" s="21" t="s">
         <v>35</v>
       </c>
       <c r="D65" s="13">
-        <v>262.7</v>
+        <v>269</v>
       </c>
       <c r="E65" s="13">
-        <v>225.66</v>
+        <v>229.07</v>
       </c>
       <c r="F65" s="13" t="s">
         <v>18</v>
@@ -1835,35 +1835,35 @@
     </row>
     <row r="66" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A66" s="7">
-        <v>46282</v>
+        <v>46283</v>
       </c>
       <c r="B66" s="8"/>
       <c r="C66" s="20" t="s">
         <v>36</v>
       </c>
       <c r="D66" s="10">
-        <v>258.52999999999997</v>
+        <v>264.83999999999997</v>
       </c>
       <c r="E66" s="10">
-        <v>221.6</v>
+        <v>225.01</v>
       </c>
       <c r="F66" s="10">
-        <v>231.6</v>
+        <v>235.01</v>
       </c>
     </row>
     <row r="67" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A67" s="11">
-        <v>46282</v>
+        <v>46283</v>
       </c>
       <c r="B67" s="12"/>
       <c r="C67" s="21" t="s">
         <v>37</v>
       </c>
       <c r="D67" s="13">
-        <v>264.02999999999997</v>
+        <v>270.33</v>
       </c>
       <c r="E67" s="13">
-        <v>238.59</v>
+        <v>242.19</v>
       </c>
       <c r="F67" s="13" t="s">
         <v>18</v>

</xml_diff>

<commit_message>
Mon Sep 21 06:33:27 UTC 2026
</commit_message>
<xml_diff>
--- a/bp.com-content-dam-bp-country-sites-en_au-australia-home-products-services-pricing-tgp-excel.xlsx
+++ b/bp.com-content-dam-bp-country-sites-en_au-australia-home-products-services-pricing-tgp-excel.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://bp365.sharepoint.com/sites/WholesalePricing/Shared Documents/B2C/TGP/Daily TGP/Web TGP/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="14_{BA4C5F24-5100-4C3E-A877-C0C02CFC31A1}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="14_{9802BC6A-5284-49A3-ACD4-5E85D8144A09}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="28680" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{1B412EEF-F96D-4DF4-A4E9-C7F0F183C2FB}"/>
+    <workbookView xWindow="-110" yWindow="-110" windowWidth="19420" windowHeight="11500" xr2:uid="{1B412EEF-F96D-4DF4-A4E9-C7F0F183C2FB}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
@@ -715,15 +715,15 @@
     <pageSetUpPr fitToPage="1"/>
   </sheetPr>
   <dimension ref="A1:G67"/>
-  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
   <cols>
-    <col min="1" max="1" width="76.42578125" bestFit="1" customWidth="1"/>
-    <col min="2" max="2" width="6.42578125"/>
-    <col min="3" max="3" width="18.140625" bestFit="1" customWidth="1"/>
-    <col min="4" max="7" width="7.140625" bestFit="1" customWidth="1"/>
+    <col min="1" max="1" width="76.453125" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="6.453125"/>
+    <col min="3" max="3" width="18.1796875" bestFit="1" customWidth="1"/>
+    <col min="4" max="7" width="7.1796875" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:7" ht="23.25" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:7" ht="22.5" x14ac:dyDescent="0.35">
       <c r="A1" s="30" t="s">
         <v>0</v>
       </c>
@@ -734,7 +734,7 @@
       <c r="F1" s="2"/>
       <c r="G1" s="2"/>
     </row>
-    <row r="2" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="2" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A2" s="3"/>
       <c r="B2" s="1"/>
       <c r="C2" s="1"/>
@@ -743,7 +743,7 @@
       <c r="F2" s="2"/>
       <c r="G2" s="2"/>
     </row>
-    <row r="3" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="3" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A3" s="3" t="s">
         <v>1</v>
       </c>
@@ -754,7 +754,7 @@
       <c r="F3" s="2"/>
       <c r="G3" s="2"/>
     </row>
-    <row r="4" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="4" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A4" s="3" t="s">
         <v>2</v>
       </c>
@@ -765,7 +765,7 @@
       <c r="F4" s="2"/>
       <c r="G4" s="2"/>
     </row>
-    <row r="5" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="5" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A5" s="3"/>
       <c r="B5" s="3"/>
       <c r="C5" s="1"/>
@@ -774,7 +774,7 @@
       <c r="F5" s="2"/>
       <c r="G5" s="2"/>
     </row>
-    <row r="6" spans="1:7" ht="20.25" x14ac:dyDescent="0.25">
+    <row r="6" spans="1:7" ht="20" x14ac:dyDescent="0.35">
       <c r="A6" s="29" t="s">
         <v>3</v>
       </c>
@@ -785,7 +785,7 @@
       <c r="F6" s="2"/>
       <c r="G6" s="2"/>
     </row>
-    <row r="7" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="7" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A7" s="4" t="s">
         <v>4</v>
       </c>
@@ -806,133 +806,133 @@
         <v>9</v>
       </c>
     </row>
-    <row r="8" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="8" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A8" s="7">
-        <v>46284</v>
+        <v>46287</v>
       </c>
       <c r="B8" s="8"/>
       <c r="C8" s="9" t="s">
         <v>10</v>
       </c>
       <c r="D8" s="10">
-        <v>275.92</v>
+        <v>276.38</v>
       </c>
       <c r="E8" s="10">
-        <v>233.2</v>
+        <v>234.19</v>
       </c>
       <c r="F8" s="10">
-        <v>243.2</v>
+        <v>244.19</v>
       </c>
       <c r="G8" s="10">
-        <v>233.16</v>
-      </c>
-    </row>
-    <row r="9" spans="1:7" x14ac:dyDescent="0.25">
+        <v>234.15</v>
+      </c>
+    </row>
+    <row r="9" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A9" s="11">
-        <v>46284</v>
+        <v>46287</v>
       </c>
       <c r="B9" s="12"/>
       <c r="C9" s="12" t="s">
         <v>11</v>
       </c>
       <c r="D9" s="13">
-        <v>275.92</v>
+        <v>276.38</v>
       </c>
       <c r="E9" s="13">
-        <v>233.2</v>
+        <v>234.19</v>
       </c>
       <c r="F9" s="13">
-        <v>243.2</v>
+        <v>244.19</v>
       </c>
       <c r="G9" s="13">
-        <v>233.16</v>
-      </c>
-    </row>
-    <row r="10" spans="1:7" x14ac:dyDescent="0.25">
+        <v>234.15</v>
+      </c>
+    </row>
+    <row r="10" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A10" s="7">
-        <v>46284</v>
+        <v>46287</v>
       </c>
       <c r="B10" s="8"/>
       <c r="C10" s="9" t="s">
         <v>12</v>
       </c>
       <c r="D10" s="10">
-        <v>271.10000000000002</v>
+        <v>270.04000000000002</v>
       </c>
       <c r="E10" s="10">
-        <v>228.4</v>
+        <v>229.01</v>
       </c>
       <c r="F10" s="10">
-        <v>238.4</v>
+        <v>239.01</v>
       </c>
       <c r="G10" s="10">
-        <v>228.82</v>
-      </c>
-    </row>
-    <row r="11" spans="1:7" x14ac:dyDescent="0.25">
+        <v>229.42</v>
+      </c>
+    </row>
+    <row r="11" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A11" s="11">
-        <v>46283</v>
+        <v>46284</v>
       </c>
       <c r="B11" s="12"/>
       <c r="C11" s="12" t="s">
         <v>10</v>
       </c>
       <c r="D11" s="13">
-        <v>270.54000000000002</v>
+        <v>275.92</v>
       </c>
       <c r="E11" s="13">
-        <v>229.63</v>
+        <v>233.2</v>
       </c>
       <c r="F11" s="13">
-        <v>239.63</v>
+        <v>243.2</v>
       </c>
       <c r="G11" s="13">
-        <v>229.6</v>
-      </c>
-    </row>
-    <row r="12" spans="1:7" x14ac:dyDescent="0.25">
+        <v>233.16</v>
+      </c>
+    </row>
+    <row r="12" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A12" s="7">
-        <v>46283</v>
+        <v>46284</v>
       </c>
       <c r="B12" s="8"/>
       <c r="C12" s="9" t="s">
         <v>11</v>
       </c>
       <c r="D12" s="10">
-        <v>270.54000000000002</v>
+        <v>275.92</v>
       </c>
       <c r="E12" s="10">
-        <v>229.63</v>
+        <v>233.2</v>
       </c>
       <c r="F12" s="10">
-        <v>239.63</v>
+        <v>243.2</v>
       </c>
       <c r="G12" s="10">
-        <v>229.6</v>
-      </c>
-    </row>
-    <row r="13" spans="1:7" x14ac:dyDescent="0.25">
+        <v>233.16</v>
+      </c>
+    </row>
+    <row r="13" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A13" s="11">
-        <v>46283</v>
+        <v>46284</v>
       </c>
       <c r="B13" s="12"/>
       <c r="C13" s="12" t="s">
         <v>12</v>
       </c>
       <c r="D13" s="13">
-        <v>266.11</v>
+        <v>271.10000000000002</v>
       </c>
       <c r="E13" s="13">
-        <v>225.18</v>
+        <v>228.4</v>
       </c>
       <c r="F13" s="13">
-        <v>235.18</v>
+        <v>238.4</v>
       </c>
       <c r="G13" s="13">
-        <v>225.6</v>
-      </c>
-    </row>
-    <row r="14" spans="1:7" x14ac:dyDescent="0.25">
+        <v>228.82</v>
+      </c>
+    </row>
+    <row r="14" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A14" s="14"/>
       <c r="B14" s="14"/>
       <c r="C14" s="15"/>
@@ -941,7 +941,7 @@
       <c r="F14" s="16"/>
       <c r="G14" s="16"/>
     </row>
-    <row r="15" spans="1:7" ht="20.25" x14ac:dyDescent="0.25">
+    <row r="15" spans="1:7" ht="20" x14ac:dyDescent="0.35">
       <c r="A15" s="29" t="s">
         <v>13</v>
       </c>
@@ -952,7 +952,7 @@
       <c r="F15" s="17"/>
       <c r="G15" s="17"/>
     </row>
-    <row r="16" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="16" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A16" s="4" t="s">
         <v>4</v>
       </c>
@@ -971,45 +971,45 @@
       </c>
       <c r="G16" s="17"/>
     </row>
-    <row r="17" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="17" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A17" s="7">
-        <v>46284</v>
+        <v>46287</v>
       </c>
       <c r="B17" s="8"/>
       <c r="C17" s="20" t="s">
         <v>14</v>
       </c>
       <c r="D17" s="10">
-        <v>275.79000000000002</v>
+        <v>274.66000000000003</v>
       </c>
       <c r="E17" s="10">
-        <v>232.46</v>
+        <v>233.01</v>
       </c>
       <c r="F17" s="10">
-        <v>242.46</v>
+        <v>243.01</v>
       </c>
       <c r="G17" s="17"/>
     </row>
-    <row r="18" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="18" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A18" s="11">
-        <v>46283</v>
+        <v>46284</v>
       </c>
       <c r="B18" s="12"/>
       <c r="C18" s="12" t="s">
         <v>14</v>
       </c>
       <c r="D18" s="13">
-        <v>270.87</v>
+        <v>275.79000000000002</v>
       </c>
       <c r="E18" s="13">
-        <v>229.29</v>
+        <v>232.46</v>
       </c>
       <c r="F18" s="13">
-        <v>239.29</v>
+        <v>242.46</v>
       </c>
       <c r="G18" s="17"/>
     </row>
-    <row r="19" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="19" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A19" s="14"/>
       <c r="B19" s="14"/>
       <c r="C19" s="15"/>
@@ -1018,7 +1018,7 @@
       <c r="F19" s="16"/>
       <c r="G19" s="17"/>
     </row>
-    <row r="20" spans="1:7" ht="20.25" x14ac:dyDescent="0.25">
+    <row r="20" spans="1:7" ht="20" x14ac:dyDescent="0.35">
       <c r="A20" s="29" t="s">
         <v>15</v>
       </c>
@@ -1029,7 +1029,7 @@
       <c r="F20" s="17"/>
       <c r="G20" s="17"/>
     </row>
-    <row r="21" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="21" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A21" s="4" t="s">
         <v>4</v>
       </c>
@@ -1050,217 +1050,217 @@
         <v>9</v>
       </c>
     </row>
-    <row r="22" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="22" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A22" s="7">
-        <v>46284</v>
+        <v>46287</v>
       </c>
       <c r="B22" s="8"/>
       <c r="C22" s="20" t="s">
         <v>16</v>
       </c>
       <c r="D22" s="10">
-        <v>275.93</v>
+        <v>276.39999999999998</v>
       </c>
       <c r="E22" s="10">
-        <v>231.14</v>
+        <v>233.23</v>
       </c>
       <c r="F22" s="10">
-        <v>240.74</v>
+        <v>242.83</v>
       </c>
       <c r="G22" s="10">
-        <v>229.86</v>
-      </c>
-    </row>
-    <row r="23" spans="1:7" x14ac:dyDescent="0.25">
+        <v>231.94</v>
+      </c>
+    </row>
+    <row r="23" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A23" s="11">
-        <v>46284</v>
+        <v>46287</v>
       </c>
       <c r="B23" s="12"/>
       <c r="C23" s="21" t="s">
         <v>17</v>
       </c>
       <c r="D23" s="13">
-        <v>275.92</v>
+        <v>274.86</v>
       </c>
       <c r="E23" s="13">
-        <v>236.22</v>
+        <v>236.85</v>
       </c>
       <c r="F23" s="13">
-        <v>246.22</v>
+        <v>246.85</v>
       </c>
       <c r="G23" s="13" t="s">
         <v>18</v>
       </c>
     </row>
-    <row r="24" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="24" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A24" s="7">
-        <v>46284</v>
+        <v>46287</v>
       </c>
       <c r="B24" s="8"/>
       <c r="C24" s="20" t="s">
         <v>19</v>
       </c>
       <c r="D24" s="10">
-        <v>276.41000000000003</v>
+        <v>275.35000000000002</v>
       </c>
       <c r="E24" s="10">
-        <v>235.47</v>
+        <v>236.1</v>
       </c>
       <c r="F24" s="10">
-        <v>245.47</v>
+        <v>246.1</v>
       </c>
       <c r="G24" s="10" t="s">
         <v>18</v>
       </c>
     </row>
-    <row r="25" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="25" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A25" s="11">
-        <v>46284</v>
+        <v>46287</v>
       </c>
       <c r="B25" s="12"/>
       <c r="C25" s="21" t="s">
         <v>20</v>
       </c>
       <c r="D25" s="13">
-        <v>273.16000000000003</v>
+        <v>272.08999999999997</v>
       </c>
       <c r="E25" s="13">
-        <v>235.57</v>
+        <v>236.21</v>
       </c>
       <c r="F25" s="13">
-        <v>245.57</v>
+        <v>246.21</v>
       </c>
       <c r="G25" s="13">
-        <v>233.47</v>
-      </c>
-    </row>
-    <row r="26" spans="1:7" x14ac:dyDescent="0.25">
+        <v>234.1</v>
+      </c>
+    </row>
+    <row r="26" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A26" s="7">
-        <v>46284</v>
+        <v>46287</v>
       </c>
       <c r="B26" s="8"/>
       <c r="C26" s="20" t="s">
         <v>21</v>
       </c>
       <c r="D26" s="10">
-        <v>274.94</v>
+        <v>273.86</v>
       </c>
       <c r="E26" s="10">
-        <v>237.05</v>
+        <v>237.69</v>
       </c>
       <c r="F26" s="10">
-        <v>247.05</v>
+        <v>247.69</v>
       </c>
       <c r="G26" s="10" t="s">
         <v>18</v>
       </c>
     </row>
-    <row r="27" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="27" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A27" s="11">
-        <v>46283</v>
+        <v>46284</v>
       </c>
       <c r="B27" s="12"/>
       <c r="C27" s="12" t="s">
         <v>16</v>
       </c>
       <c r="D27" s="13">
-        <v>270.55</v>
+        <v>275.93</v>
       </c>
       <c r="E27" s="13">
-        <v>227.14</v>
+        <v>231.14</v>
       </c>
       <c r="F27" s="13">
-        <v>236.74</v>
+        <v>240.74</v>
       </c>
       <c r="G27" s="13">
-        <v>225.85</v>
-      </c>
-    </row>
-    <row r="28" spans="1:7" x14ac:dyDescent="0.25">
+        <v>229.86</v>
+      </c>
+    </row>
+    <row r="28" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A28" s="7">
-        <v>46283</v>
+        <v>46284</v>
       </c>
       <c r="B28" s="8"/>
       <c r="C28" s="20" t="s">
         <v>17</v>
       </c>
       <c r="D28" s="10">
-        <v>270.92</v>
+        <v>275.92</v>
       </c>
       <c r="E28" s="22">
-        <v>232.96</v>
+        <v>236.22</v>
       </c>
       <c r="F28" s="22">
-        <v>242.96</v>
+        <v>246.22</v>
       </c>
       <c r="G28" s="22" t="s">
         <v>18</v>
       </c>
     </row>
-    <row r="29" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="29" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A29" s="11">
-        <v>46283</v>
+        <v>46284</v>
       </c>
       <c r="B29" s="12"/>
       <c r="C29" s="12" t="s">
         <v>19</v>
       </c>
       <c r="D29" s="13">
-        <v>271.42</v>
+        <v>276.41000000000003</v>
       </c>
       <c r="E29" s="13">
-        <v>232.22</v>
+        <v>235.47</v>
       </c>
       <c r="F29" s="13">
-        <v>242.22</v>
+        <v>245.47</v>
       </c>
       <c r="G29" s="13" t="s">
         <v>18</v>
       </c>
     </row>
-    <row r="30" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="30" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A30" s="7">
-        <v>46283</v>
+        <v>46284</v>
       </c>
       <c r="B30" s="8"/>
       <c r="C30" s="20" t="s">
         <v>20</v>
       </c>
       <c r="D30" s="10">
-        <v>268.17</v>
+        <v>273.16000000000003</v>
       </c>
       <c r="E30" s="22">
-        <v>232.3</v>
+        <v>235.57</v>
       </c>
       <c r="F30" s="22">
-        <v>242.3</v>
+        <v>245.57</v>
       </c>
       <c r="G30" s="22">
-        <v>230.2</v>
-      </c>
-    </row>
-    <row r="31" spans="1:7" x14ac:dyDescent="0.25">
+        <v>233.47</v>
+      </c>
+    </row>
+    <row r="31" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A31" s="11">
-        <v>46283</v>
+        <v>46284</v>
       </c>
       <c r="B31" s="12"/>
       <c r="C31" s="12" t="s">
         <v>21</v>
       </c>
       <c r="D31" s="13">
-        <v>269.95999999999998</v>
+        <v>274.94</v>
       </c>
       <c r="E31" s="13">
-        <v>233.76</v>
+        <v>237.05</v>
       </c>
       <c r="F31" s="13">
-        <v>243.76</v>
+        <v>247.05</v>
       </c>
       <c r="G31" s="13" t="s">
         <v>18</v>
       </c>
     </row>
-    <row r="32" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="32" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A32" s="14"/>
       <c r="B32" s="14"/>
       <c r="C32" s="15"/>
@@ -1269,7 +1269,7 @@
       <c r="F32" s="17"/>
       <c r="G32" s="17"/>
     </row>
-    <row r="33" spans="1:7" ht="20.25" x14ac:dyDescent="0.25">
+    <row r="33" spans="1:7" ht="20" x14ac:dyDescent="0.35">
       <c r="A33" s="29" t="s">
         <v>22</v>
       </c>
@@ -1280,7 +1280,7 @@
       <c r="F33" s="17"/>
       <c r="G33" s="17"/>
     </row>
-    <row r="34" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="34" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A34" s="23" t="s">
         <v>4</v>
       </c>
@@ -1299,54 +1299,54 @@
       </c>
       <c r="G34" s="17"/>
     </row>
-    <row r="35" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="35" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A35" s="7">
-        <v>46284</v>
+        <v>46287</v>
       </c>
       <c r="B35" s="8"/>
       <c r="C35" s="20" t="s">
         <v>23</v>
       </c>
       <c r="D35" s="10">
-        <v>269.63</v>
+        <v>268.56</v>
       </c>
       <c r="E35" s="10">
-        <v>227.22</v>
+        <v>227.94</v>
       </c>
       <c r="F35" s="10">
-        <v>236.22</v>
+        <v>236.94</v>
       </c>
       <c r="G35" s="17"/>
     </row>
-    <row r="36" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="36" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A36" s="11">
-        <v>46283</v>
+        <v>46284</v>
       </c>
       <c r="B36" s="12"/>
       <c r="C36" s="12" t="s">
         <v>23</v>
       </c>
       <c r="D36" s="13">
-        <v>264.64</v>
+        <v>269.63</v>
       </c>
       <c r="E36" s="13">
-        <v>223.56</v>
+        <v>227.22</v>
       </c>
       <c r="F36" s="13">
-        <v>232.56</v>
+        <v>236.22</v>
       </c>
       <c r="G36" s="17"/>
     </row>
-    <row r="37" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="37" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A37" s="7">
-        <v>46284</v>
+        <v>46287</v>
       </c>
       <c r="B37" s="8"/>
       <c r="C37" s="20" t="s">
         <v>24</v>
       </c>
       <c r="D37" s="10">
-        <v>285.25</v>
+        <v>284.18</v>
       </c>
       <c r="E37" s="10" t="s">
         <v>18</v>
@@ -1356,16 +1356,16 @@
       </c>
       <c r="G37" s="17"/>
     </row>
-    <row r="38" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="38" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A38" s="11">
-        <v>46283</v>
+        <v>46284</v>
       </c>
       <c r="B38" s="12"/>
       <c r="C38" s="12" t="s">
         <v>24</v>
       </c>
       <c r="D38" s="13">
-        <v>280.26</v>
+        <v>285.25</v>
       </c>
       <c r="E38" s="13" t="s">
         <v>18</v>
@@ -1375,7 +1375,7 @@
       </c>
       <c r="G38" s="17"/>
     </row>
-    <row r="39" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="39" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A39" s="24"/>
       <c r="B39" s="24"/>
       <c r="C39" s="15"/>
@@ -1384,7 +1384,7 @@
       <c r="F39" s="17"/>
       <c r="G39" s="17"/>
     </row>
-    <row r="40" spans="1:7" ht="20.25" x14ac:dyDescent="0.25">
+    <row r="40" spans="1:7" ht="20" x14ac:dyDescent="0.35">
       <c r="A40" s="29" t="s">
         <v>25</v>
       </c>
@@ -1395,7 +1395,7 @@
       <c r="F40" s="17"/>
       <c r="G40" s="17"/>
     </row>
-    <row r="41" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="41" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A41" s="23" t="s">
         <v>4</v>
       </c>
@@ -1414,83 +1414,83 @@
       </c>
       <c r="G41" s="17"/>
     </row>
-    <row r="42" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="42" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A42" s="7">
-        <v>46284</v>
+        <v>46287</v>
       </c>
       <c r="B42" s="8"/>
       <c r="C42" s="20" t="s">
         <v>26</v>
       </c>
       <c r="D42" s="10">
-        <v>278.72000000000003</v>
+        <v>277.7</v>
       </c>
       <c r="E42" s="10">
-        <v>232.81</v>
+        <v>233.06</v>
       </c>
       <c r="F42" s="10">
-        <v>242.81</v>
+        <v>243.06</v>
       </c>
       <c r="G42" s="17"/>
     </row>
-    <row r="43" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="43" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A43" s="11">
-        <v>46284</v>
+        <v>46287</v>
       </c>
       <c r="B43" s="12"/>
       <c r="C43" s="21" t="s">
         <v>27</v>
       </c>
       <c r="D43" s="13">
-        <v>278.31</v>
+        <v>277.3</v>
       </c>
       <c r="E43" s="13">
-        <v>233.23</v>
+        <v>233.48</v>
       </c>
       <c r="F43" s="13">
-        <v>243.23</v>
+        <v>243.48</v>
       </c>
       <c r="G43" s="17"/>
     </row>
-    <row r="44" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="44" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A44" s="7">
-        <v>46283</v>
+        <v>46284</v>
       </c>
       <c r="B44" s="8"/>
       <c r="C44" s="20" t="s">
         <v>26</v>
       </c>
       <c r="D44" s="10">
-        <v>273.67</v>
+        <v>278.72000000000003</v>
       </c>
       <c r="E44" s="10">
-        <v>229.97</v>
+        <v>232.81</v>
       </c>
       <c r="F44" s="10">
-        <v>239.97</v>
+        <v>242.81</v>
       </c>
       <c r="G44" s="17"/>
     </row>
-    <row r="45" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="45" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A45" s="11">
-        <v>46283</v>
+        <v>46284</v>
       </c>
       <c r="B45" s="12"/>
       <c r="C45" s="21" t="s">
         <v>27</v>
       </c>
       <c r="D45" s="13">
-        <v>273.27</v>
+        <v>278.31</v>
       </c>
       <c r="E45" s="13">
-        <v>230.38</v>
+        <v>233.23</v>
       </c>
       <c r="F45" s="13">
-        <v>240.38</v>
+        <v>243.23</v>
       </c>
       <c r="G45" s="17"/>
     </row>
-    <row r="46" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="46" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A46" s="14"/>
       <c r="B46" s="24"/>
       <c r="C46" s="15"/>
@@ -1499,7 +1499,7 @@
       <c r="F46" s="16"/>
       <c r="G46" s="17"/>
     </row>
-    <row r="47" spans="1:7" ht="20.25" x14ac:dyDescent="0.25">
+    <row r="47" spans="1:7" ht="20" x14ac:dyDescent="0.35">
       <c r="A47" s="25" t="s">
         <v>28</v>
       </c>
@@ -1510,7 +1510,7 @@
       <c r="F47" s="17"/>
       <c r="G47" s="17"/>
     </row>
-    <row r="48" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="48" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A48" s="23" t="s">
         <v>4</v>
       </c>
@@ -1529,83 +1529,83 @@
       </c>
       <c r="G48" s="17"/>
     </row>
-    <row r="49" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="49" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A49" s="7">
-        <v>46284</v>
+        <v>46287</v>
       </c>
       <c r="B49" s="8"/>
       <c r="C49" s="20" t="s">
         <v>29</v>
       </c>
       <c r="D49" s="10">
-        <v>263.76</v>
+        <v>266.14</v>
       </c>
       <c r="E49" s="10">
-        <v>224.63</v>
+        <v>226.83</v>
       </c>
       <c r="F49" s="10">
-        <v>234.63</v>
+        <v>236.83</v>
       </c>
       <c r="G49" s="28"/>
     </row>
-    <row r="50" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="50" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A50" s="11">
-        <v>46284</v>
+        <v>46287</v>
       </c>
       <c r="B50" s="12"/>
       <c r="C50" s="21" t="s">
         <v>30</v>
       </c>
       <c r="D50" s="13">
-        <v>261.77</v>
+        <v>264.13</v>
       </c>
       <c r="E50" s="13">
-        <v>224.47</v>
+        <v>226.66</v>
       </c>
       <c r="F50" s="13">
-        <v>234.47</v>
+        <v>236.67</v>
       </c>
       <c r="G50" s="28"/>
     </row>
-    <row r="51" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="51" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A51" s="7">
-        <v>46283</v>
+        <v>46284</v>
       </c>
       <c r="B51" s="8"/>
       <c r="C51" s="20" t="s">
         <v>29</v>
       </c>
       <c r="D51" s="10">
-        <v>260.45999999999998</v>
+        <v>263.76</v>
       </c>
       <c r="E51" s="10">
-        <v>222.36</v>
+        <v>224.63</v>
       </c>
       <c r="F51" s="10">
-        <v>232.36</v>
+        <v>234.63</v>
       </c>
       <c r="G51" s="17"/>
     </row>
-    <row r="52" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="52" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A52" s="11">
-        <v>46283</v>
+        <v>46284</v>
       </c>
       <c r="B52" s="12"/>
       <c r="C52" s="21" t="s">
         <v>30</v>
       </c>
       <c r="D52" s="13">
-        <v>258.49</v>
+        <v>261.77</v>
       </c>
       <c r="E52" s="13">
-        <v>222.2</v>
+        <v>224.47</v>
       </c>
       <c r="F52" s="13">
-        <v>232.2</v>
+        <v>234.47</v>
       </c>
       <c r="G52" s="17"/>
     </row>
-    <row r="53" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="53" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A53" s="14"/>
       <c r="B53" s="14"/>
       <c r="C53" s="15"/>
@@ -1614,7 +1614,7 @@
       <c r="F53" s="16"/>
       <c r="G53" s="17"/>
     </row>
-    <row r="54" spans="1:7" ht="20.25" x14ac:dyDescent="0.25">
+    <row r="54" spans="1:7" ht="20" x14ac:dyDescent="0.35">
       <c r="A54" s="27" t="s">
         <v>31</v>
       </c>
@@ -1625,7 +1625,7 @@
       <c r="F54" s="17"/>
       <c r="G54" s="17"/>
     </row>
-    <row r="55" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="55" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A55" s="23" t="s">
         <v>4</v>
       </c>
@@ -1644,54 +1644,54 @@
       </c>
       <c r="G55" s="17"/>
     </row>
-    <row r="56" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="56" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A56" s="7">
-        <v>46284</v>
+        <v>46287</v>
       </c>
       <c r="B56" s="8"/>
       <c r="C56" s="20" t="s">
         <v>32</v>
       </c>
       <c r="D56" s="10">
-        <v>287.8</v>
+        <v>286.70999999999998</v>
       </c>
       <c r="E56" s="10">
-        <v>250.05</v>
+        <v>250.91</v>
       </c>
       <c r="F56" s="10">
-        <v>260.05</v>
+        <v>260.91000000000003</v>
       </c>
       <c r="G56" s="17"/>
     </row>
-    <row r="57" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="57" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A57" s="11">
-        <v>46284</v>
+        <v>46287</v>
       </c>
       <c r="B57" s="12"/>
       <c r="C57" s="21" t="s">
         <v>33</v>
       </c>
       <c r="D57" s="13">
-        <v>276.74</v>
+        <v>275.68</v>
       </c>
       <c r="E57" s="13">
-        <v>237.83</v>
+        <v>238.37</v>
       </c>
       <c r="F57" s="13">
-        <v>247.83</v>
+        <v>248.37</v>
       </c>
       <c r="G57" s="17"/>
     </row>
-    <row r="58" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="58" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A58" s="7">
-        <v>46284</v>
+        <v>46287</v>
       </c>
       <c r="B58" s="8"/>
       <c r="C58" s="20" t="s">
         <v>34</v>
       </c>
       <c r="D58" s="10">
-        <v>277.98</v>
+        <v>276.92</v>
       </c>
       <c r="E58" s="10" t="s">
         <v>18</v>
@@ -1701,111 +1701,111 @@
       </c>
       <c r="G58" s="17"/>
     </row>
-    <row r="59" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="59" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A59" s="11">
-        <v>46284</v>
+        <v>46287</v>
       </c>
       <c r="B59" s="12"/>
       <c r="C59" s="21" t="s">
         <v>35</v>
       </c>
       <c r="D59" s="13">
-        <v>273.89999999999998</v>
+        <v>272.76</v>
       </c>
       <c r="E59" s="13">
-        <v>232.21</v>
+        <v>232.74</v>
       </c>
       <c r="F59" s="13" t="s">
         <v>18</v>
       </c>
       <c r="G59" s="17"/>
     </row>
-    <row r="60" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="60" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A60" s="7">
-        <v>46284</v>
+        <v>46287</v>
       </c>
       <c r="B60" s="8"/>
       <c r="C60" s="20" t="s">
         <v>36</v>
       </c>
       <c r="D60" s="10">
-        <v>269.74</v>
+        <v>268.58999999999997</v>
       </c>
       <c r="E60" s="10">
-        <v>228.15</v>
+        <v>228.69</v>
       </c>
       <c r="F60" s="10">
-        <v>238.15</v>
+        <v>238.69</v>
       </c>
       <c r="G60" s="17"/>
     </row>
-    <row r="61" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="61" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A61" s="11">
-        <v>46284</v>
+        <v>46287</v>
       </c>
       <c r="B61" s="12"/>
       <c r="C61" s="21" t="s">
         <v>37</v>
       </c>
       <c r="D61" s="13">
-        <v>275.23</v>
+        <v>274.08</v>
       </c>
       <c r="E61" s="13">
-        <v>245.58</v>
+        <v>246.33</v>
       </c>
       <c r="F61" s="13" t="s">
         <v>18</v>
       </c>
       <c r="G61" s="17"/>
     </row>
-    <row r="62" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="62" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A62" s="7">
-        <v>46283</v>
+        <v>46284</v>
       </c>
       <c r="B62" s="8"/>
       <c r="C62" s="20" t="s">
         <v>32</v>
       </c>
       <c r="D62" s="10">
-        <v>282.8</v>
+        <v>287.8</v>
       </c>
       <c r="E62" s="10">
-        <v>246.55</v>
+        <v>250.05</v>
       </c>
       <c r="F62" s="10">
-        <v>256.55</v>
+        <v>260.05</v>
       </c>
       <c r="G62" s="17"/>
     </row>
-    <row r="63" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="63" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A63" s="11">
-        <v>46283</v>
+        <v>46284</v>
       </c>
       <c r="B63" s="12"/>
       <c r="C63" s="21" t="s">
         <v>33</v>
       </c>
       <c r="D63" s="13">
-        <v>271.74</v>
+        <v>276.74</v>
       </c>
       <c r="E63" s="13">
-        <v>234.69</v>
+        <v>237.83</v>
       </c>
       <c r="F63" s="13">
-        <v>244.69</v>
+        <v>247.83</v>
       </c>
       <c r="G63" s="17"/>
     </row>
-    <row r="64" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="64" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A64" s="7">
-        <v>46283</v>
+        <v>46284</v>
       </c>
       <c r="B64" s="8"/>
       <c r="C64" s="20" t="s">
         <v>34</v>
       </c>
       <c r="D64" s="10">
-        <v>272.97000000000003</v>
+        <v>277.98</v>
       </c>
       <c r="E64" s="10" t="s">
         <v>18</v>
@@ -1815,55 +1815,55 @@
       </c>
       <c r="G64" s="17"/>
     </row>
-    <row r="65" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="65" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A65" s="11">
-        <v>46283</v>
+        <v>46284</v>
       </c>
       <c r="B65" s="12"/>
       <c r="C65" s="21" t="s">
         <v>35</v>
       </c>
       <c r="D65" s="13">
-        <v>269</v>
+        <v>273.89999999999998</v>
       </c>
       <c r="E65" s="13">
-        <v>229.07</v>
+        <v>232.21</v>
       </c>
       <c r="F65" s="13" t="s">
         <v>18</v>
       </c>
     </row>
-    <row r="66" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="66" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A66" s="7">
-        <v>46283</v>
+        <v>46284</v>
       </c>
       <c r="B66" s="8"/>
       <c r="C66" s="20" t="s">
         <v>36</v>
       </c>
       <c r="D66" s="10">
-        <v>264.83999999999997</v>
+        <v>269.74</v>
       </c>
       <c r="E66" s="10">
-        <v>225.01</v>
+        <v>228.15</v>
       </c>
       <c r="F66" s="10">
-        <v>235.01</v>
-      </c>
-    </row>
-    <row r="67" spans="1:6" x14ac:dyDescent="0.25">
+        <v>238.15</v>
+      </c>
+    </row>
+    <row r="67" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A67" s="11">
-        <v>46283</v>
+        <v>46284</v>
       </c>
       <c r="B67" s="12"/>
       <c r="C67" s="21" t="s">
         <v>37</v>
       </c>
       <c r="D67" s="13">
-        <v>270.33</v>
+        <v>275.23</v>
       </c>
       <c r="E67" s="13">
-        <v>242.19</v>
+        <v>245.58</v>
       </c>
       <c r="F67" s="13" t="s">
         <v>18</v>
@@ -1891,6 +1891,17 @@
 </file>
 
 <file path=customXml/item1.xml><?xml version="1.0" encoding="utf-8"?>
+<p:properties xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls">
+  <documentManagement>
+    <lcf76f155ced4ddcb4097134ff3c332f xmlns="87276d81-85f4-4ef2-9e6e-55066304288f">
+      <Terms xmlns="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
+    </lcf76f155ced4ddcb4097134ff3c332f>
+    <TaxCatchAll xmlns="b23b8984-eafa-4e79-985e-54f52f3da58e" xsi:nil="true"/>
+  </documentManagement>
+</p:properties>
+</file>
+
+<file path=customXml/item2.xml><?xml version="1.0" encoding="utf-8"?>
 <ct:contentTypeSchema xmlns:ct="http://schemas.microsoft.com/office/2006/metadata/contentType" xmlns:ma="http://schemas.microsoft.com/office/2006/metadata/properties/metaAttributes" ct:_="" ma:_="" ma:contentTypeName="Document" ma:contentTypeID="0x010100D3632DF5622958439304627C030B0427" ma:contentTypeVersion="18" ma:contentTypeDescription="Create a new document." ma:contentTypeScope="" ma:versionID="8c2ecbce386d6bac497f8eb2d8f0fb7a">
   <xsd:schema xmlns:xsd="http://www.w3.org/2001/XMLSchema" xmlns:xs="http://www.w3.org/2001/XMLSchema" xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:ns2="87276d81-85f4-4ef2-9e6e-55066304288f" xmlns:ns3="39e1dda6-d1d8-4c88-a3b9-f1abc1284bad" xmlns:ns4="b23b8984-eafa-4e79-985e-54f52f3da58e" targetNamespace="http://schemas.microsoft.com/office/2006/metadata/properties" ma:root="true" ma:fieldsID="4cfd0c2f651c1ce156ad4fcb44ea61dd" ns2:_="" ns3:_="" ns4:_="">
     <xsd:import namespace="87276d81-85f4-4ef2-9e6e-55066304288f"/>
@@ -2150,7 +2161,7 @@
 </ct:contentTypeSchema>
 </file>
 
-<file path=customXml/item2.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=customXml/item3.xml><?xml version="1.0" encoding="utf-8"?>
 <?mso-contentType ?>
 <FormTemplates xmlns="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms">
   <Display>DocumentLibraryForm</Display>
@@ -2159,18 +2170,18 @@
 </FormTemplates>
 </file>
 
-<file path=customXml/item3.xml><?xml version="1.0" encoding="utf-8"?>
-<p:properties xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls">
-  <documentManagement>
-    <lcf76f155ced4ddcb4097134ff3c332f xmlns="87276d81-85f4-4ef2-9e6e-55066304288f">
-      <Terms xmlns="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
-    </lcf76f155ced4ddcb4097134ff3c332f>
-    <TaxCatchAll xmlns="b23b8984-eafa-4e79-985e-54f52f3da58e" xsi:nil="true"/>
-  </documentManagement>
-</p:properties>
+<file path=customXml/itemProps1.xml><?xml version="1.0" encoding="utf-8"?>
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{57A83D98-2BAE-4D83-823A-D31C464B620C}">
+  <ds:schemaRefs>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/properties"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
+    <ds:schemaRef ds:uri="87276d81-85f4-4ef2-9e6e-55066304288f"/>
+    <ds:schemaRef ds:uri="b23b8984-eafa-4e79-985e-54f52f3da58e"/>
+  </ds:schemaRefs>
+</ds:datastoreItem>
 </file>
 
-<file path=customXml/itemProps1.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=customXml/itemProps2.xml><?xml version="1.0" encoding="utf-8"?>
 <ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{B44E1863-2778-41F9-ACBA-48420F931671}">
   <ds:schemaRefs>
     <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/contentType"/>
@@ -2190,21 +2201,10 @@
 </ds:datastoreItem>
 </file>
 
-<file path=customXml/itemProps2.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=customXml/itemProps3.xml><?xml version="1.0" encoding="utf-8"?>
 <ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{F60519E9-FD90-4339-869C-BC2F85719BB8}">
   <ds:schemaRefs>
     <ds:schemaRef ds:uri="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms"/>
-  </ds:schemaRefs>
-</ds:datastoreItem>
-</file>
-
-<file path=customXml/itemProps3.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{57A83D98-2BAE-4D83-823A-D31C464B620C}">
-  <ds:schemaRefs>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/properties"/>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
-    <ds:schemaRef ds:uri="87276d81-85f4-4ef2-9e6e-55066304288f"/>
-    <ds:schemaRef ds:uri="b23b8984-eafa-4e79-985e-54f52f3da58e"/>
   </ds:schemaRefs>
 </ds:datastoreItem>
 </file>

</xml_diff>

<commit_message>
Tue Sep 22 06:22:29 UTC 2026
</commit_message>
<xml_diff>
--- a/bp.com-content-dam-bp-country-sites-en_au-australia-home-products-services-pricing-tgp-excel.xlsx
+++ b/bp.com-content-dam-bp-country-sites-en_au-australia-home-products-services-pricing-tgp-excel.xlsx
@@ -8,14 +8,14 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://bp365.sharepoint.com/sites/WholesalePricing/Shared Documents/B2C/TGP/Daily TGP/Web TGP/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="14_{9802BC6A-5284-49A3-ACD4-5E85D8144A09}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="14_{7DD8403A-A834-46A5-861F-04E937D9559A}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-110" yWindow="-110" windowWidth="19420" windowHeight="11500" xr2:uid="{1B412EEF-F96D-4DF4-A4E9-C7F0F183C2FB}"/>
+    <workbookView xWindow="-28920" yWindow="-60" windowWidth="29040" windowHeight="15720" xr2:uid="{1B412EEF-F96D-4DF4-A4E9-C7F0F183C2FB}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
   </sheets>
-  <calcPr calcId="191028"/>
+  <calcPr calcId="191028" concurrentManualCount="12"/>
   <extLst>
     <ext xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" uri="{140A7094-0E35-4892-8432-C4D2E57EDEB5}">
       <x15:workbookPr chartTrackingRefBase="1"/>
@@ -715,15 +715,15 @@
     <pageSetUpPr fitToPage="1"/>
   </sheetPr>
   <dimension ref="A1:G67"/>
-  <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
+  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
-    <col min="1" max="1" width="76.453125" bestFit="1" customWidth="1"/>
-    <col min="2" max="2" width="6.453125"/>
-    <col min="3" max="3" width="18.1796875" bestFit="1" customWidth="1"/>
-    <col min="4" max="7" width="7.1796875" bestFit="1" customWidth="1"/>
+    <col min="1" max="1" width="76.42578125" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="6.42578125"/>
+    <col min="3" max="3" width="18.140625" bestFit="1" customWidth="1"/>
+    <col min="4" max="7" width="7.140625" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:7" ht="22.5" x14ac:dyDescent="0.35">
+    <row r="1" spans="1:7" ht="23.25" x14ac:dyDescent="0.25">
       <c r="A1" s="30" t="s">
         <v>0</v>
       </c>
@@ -734,7 +734,7 @@
       <c r="F1" s="2"/>
       <c r="G1" s="2"/>
     </row>
-    <row r="2" spans="1:7" x14ac:dyDescent="0.35">
+    <row r="2" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A2" s="3"/>
       <c r="B2" s="1"/>
       <c r="C2" s="1"/>
@@ -743,7 +743,7 @@
       <c r="F2" s="2"/>
       <c r="G2" s="2"/>
     </row>
-    <row r="3" spans="1:7" x14ac:dyDescent="0.35">
+    <row r="3" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A3" s="3" t="s">
         <v>1</v>
       </c>
@@ -754,7 +754,7 @@
       <c r="F3" s="2"/>
       <c r="G3" s="2"/>
     </row>
-    <row r="4" spans="1:7" x14ac:dyDescent="0.35">
+    <row r="4" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A4" s="3" t="s">
         <v>2</v>
       </c>
@@ -765,7 +765,7 @@
       <c r="F4" s="2"/>
       <c r="G4" s="2"/>
     </row>
-    <row r="5" spans="1:7" x14ac:dyDescent="0.35">
+    <row r="5" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A5" s="3"/>
       <c r="B5" s="3"/>
       <c r="C5" s="1"/>
@@ -774,7 +774,7 @@
       <c r="F5" s="2"/>
       <c r="G5" s="2"/>
     </row>
-    <row r="6" spans="1:7" ht="20" x14ac:dyDescent="0.35">
+    <row r="6" spans="1:7" ht="20.25" x14ac:dyDescent="0.25">
       <c r="A6" s="29" t="s">
         <v>3</v>
       </c>
@@ -785,7 +785,7 @@
       <c r="F6" s="2"/>
       <c r="G6" s="2"/>
     </row>
-    <row r="7" spans="1:7" x14ac:dyDescent="0.35">
+    <row r="7" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A7" s="4" t="s">
         <v>4</v>
       </c>
@@ -806,133 +806,133 @@
         <v>9</v>
       </c>
     </row>
-    <row r="8" spans="1:7" x14ac:dyDescent="0.35">
+    <row r="8" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A8" s="7">
-        <v>46287</v>
+        <v>46288</v>
       </c>
       <c r="B8" s="8"/>
       <c r="C8" s="9" t="s">
         <v>10</v>
       </c>
       <c r="D8" s="10">
-        <v>276.38</v>
+        <v>273.36</v>
       </c>
       <c r="E8" s="10">
-        <v>234.19</v>
+        <v>234.56</v>
       </c>
       <c r="F8" s="10">
-        <v>244.19</v>
+        <v>244.56</v>
       </c>
       <c r="G8" s="10">
-        <v>234.15</v>
-      </c>
-    </row>
-    <row r="9" spans="1:7" x14ac:dyDescent="0.35">
+        <v>234.52</v>
+      </c>
+    </row>
+    <row r="9" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A9" s="11">
-        <v>46287</v>
+        <v>46288</v>
       </c>
       <c r="B9" s="12"/>
       <c r="C9" s="12" t="s">
         <v>11</v>
       </c>
       <c r="D9" s="13">
-        <v>276.38</v>
+        <v>273.36</v>
       </c>
       <c r="E9" s="13">
-        <v>234.19</v>
+        <v>234.56</v>
       </c>
       <c r="F9" s="13">
-        <v>244.19</v>
+        <v>244.56</v>
       </c>
       <c r="G9" s="13">
-        <v>234.15</v>
-      </c>
-    </row>
-    <row r="10" spans="1:7" x14ac:dyDescent="0.35">
+        <v>234.52</v>
+      </c>
+    </row>
+    <row r="10" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A10" s="7">
-        <v>46287</v>
+        <v>46288</v>
       </c>
       <c r="B10" s="8"/>
       <c r="C10" s="9" t="s">
         <v>12</v>
       </c>
       <c r="D10" s="10">
-        <v>270.04000000000002</v>
+        <v>266.67</v>
       </c>
       <c r="E10" s="10">
-        <v>229.01</v>
+        <v>229.08</v>
       </c>
       <c r="F10" s="10">
-        <v>239.01</v>
+        <v>239.08</v>
       </c>
       <c r="G10" s="10">
-        <v>229.42</v>
-      </c>
-    </row>
-    <row r="11" spans="1:7" x14ac:dyDescent="0.35">
+        <v>229.5</v>
+      </c>
+    </row>
+    <row r="11" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A11" s="11">
-        <v>46284</v>
+        <v>46287</v>
       </c>
       <c r="B11" s="12"/>
       <c r="C11" s="12" t="s">
         <v>10</v>
       </c>
       <c r="D11" s="13">
-        <v>275.92</v>
+        <v>276.38</v>
       </c>
       <c r="E11" s="13">
-        <v>233.2</v>
+        <v>234.19</v>
       </c>
       <c r="F11" s="13">
-        <v>243.2</v>
+        <v>244.19</v>
       </c>
       <c r="G11" s="13">
-        <v>233.16</v>
-      </c>
-    </row>
-    <row r="12" spans="1:7" x14ac:dyDescent="0.35">
+        <v>234.15</v>
+      </c>
+    </row>
+    <row r="12" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A12" s="7">
-        <v>46284</v>
+        <v>46287</v>
       </c>
       <c r="B12" s="8"/>
       <c r="C12" s="9" t="s">
         <v>11</v>
       </c>
       <c r="D12" s="10">
-        <v>275.92</v>
+        <v>276.38</v>
       </c>
       <c r="E12" s="10">
-        <v>233.2</v>
+        <v>234.19</v>
       </c>
       <c r="F12" s="10">
-        <v>243.2</v>
+        <v>244.19</v>
       </c>
       <c r="G12" s="10">
-        <v>233.16</v>
-      </c>
-    </row>
-    <row r="13" spans="1:7" x14ac:dyDescent="0.35">
+        <v>234.15</v>
+      </c>
+    </row>
+    <row r="13" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A13" s="11">
-        <v>46284</v>
+        <v>46287</v>
       </c>
       <c r="B13" s="12"/>
       <c r="C13" s="12" t="s">
         <v>12</v>
       </c>
       <c r="D13" s="13">
-        <v>271.10000000000002</v>
+        <v>270.04000000000002</v>
       </c>
       <c r="E13" s="13">
-        <v>228.4</v>
+        <v>229.01</v>
       </c>
       <c r="F13" s="13">
-        <v>238.4</v>
+        <v>239.01</v>
       </c>
       <c r="G13" s="13">
-        <v>228.82</v>
-      </c>
-    </row>
-    <row r="14" spans="1:7" x14ac:dyDescent="0.35">
+        <v>229.42</v>
+      </c>
+    </row>
+    <row r="14" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A14" s="14"/>
       <c r="B14" s="14"/>
       <c r="C14" s="15"/>
@@ -941,7 +941,7 @@
       <c r="F14" s="16"/>
       <c r="G14" s="16"/>
     </row>
-    <row r="15" spans="1:7" ht="20" x14ac:dyDescent="0.35">
+    <row r="15" spans="1:7" ht="20.25" x14ac:dyDescent="0.25">
       <c r="A15" s="29" t="s">
         <v>13</v>
       </c>
@@ -952,7 +952,7 @@
       <c r="F15" s="17"/>
       <c r="G15" s="17"/>
     </row>
-    <row r="16" spans="1:7" x14ac:dyDescent="0.35">
+    <row r="16" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A16" s="4" t="s">
         <v>4</v>
       </c>
@@ -971,45 +971,45 @@
       </c>
       <c r="G16" s="17"/>
     </row>
-    <row r="17" spans="1:7" x14ac:dyDescent="0.35">
+    <row r="17" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A17" s="7">
-        <v>46287</v>
+        <v>46288</v>
       </c>
       <c r="B17" s="8"/>
       <c r="C17" s="20" t="s">
         <v>14</v>
       </c>
       <c r="D17" s="10">
-        <v>274.66000000000003</v>
+        <v>271.24</v>
       </c>
       <c r="E17" s="10">
-        <v>233.01</v>
+        <v>233.03</v>
       </c>
       <c r="F17" s="10">
-        <v>243.01</v>
+        <v>243.03</v>
       </c>
       <c r="G17" s="17"/>
     </row>
-    <row r="18" spans="1:7" x14ac:dyDescent="0.35">
+    <row r="18" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A18" s="11">
-        <v>46284</v>
+        <v>46287</v>
       </c>
       <c r="B18" s="12"/>
       <c r="C18" s="12" t="s">
         <v>14</v>
       </c>
       <c r="D18" s="13">
-        <v>275.79000000000002</v>
+        <v>274.66000000000003</v>
       </c>
       <c r="E18" s="13">
-        <v>232.46</v>
+        <v>233.01</v>
       </c>
       <c r="F18" s="13">
-        <v>242.46</v>
+        <v>243.01</v>
       </c>
       <c r="G18" s="17"/>
     </row>
-    <row r="19" spans="1:7" x14ac:dyDescent="0.35">
+    <row r="19" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A19" s="14"/>
       <c r="B19" s="14"/>
       <c r="C19" s="15"/>
@@ -1018,7 +1018,7 @@
       <c r="F19" s="16"/>
       <c r="G19" s="17"/>
     </row>
-    <row r="20" spans="1:7" ht="20" x14ac:dyDescent="0.35">
+    <row r="20" spans="1:7" ht="20.25" x14ac:dyDescent="0.25">
       <c r="A20" s="29" t="s">
         <v>15</v>
       </c>
@@ -1029,7 +1029,7 @@
       <c r="F20" s="17"/>
       <c r="G20" s="17"/>
     </row>
-    <row r="21" spans="1:7" x14ac:dyDescent="0.35">
+    <row r="21" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A21" s="4" t="s">
         <v>4</v>
       </c>
@@ -1050,217 +1050,217 @@
         <v>9</v>
       </c>
     </row>
-    <row r="22" spans="1:7" x14ac:dyDescent="0.35">
+    <row r="22" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A22" s="7">
-        <v>46287</v>
+        <v>46288</v>
       </c>
       <c r="B22" s="8"/>
       <c r="C22" s="20" t="s">
         <v>16</v>
       </c>
       <c r="D22" s="10">
-        <v>276.39999999999998</v>
+        <v>273.37</v>
       </c>
       <c r="E22" s="10">
-        <v>233.23</v>
+        <v>233.6</v>
       </c>
       <c r="F22" s="10">
-        <v>242.83</v>
+        <v>243.2</v>
       </c>
       <c r="G22" s="10">
-        <v>231.94</v>
-      </c>
-    </row>
-    <row r="23" spans="1:7" x14ac:dyDescent="0.35">
+        <v>232.32</v>
+      </c>
+    </row>
+    <row r="23" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A23" s="11">
-        <v>46287</v>
+        <v>46288</v>
       </c>
       <c r="B23" s="12"/>
       <c r="C23" s="21" t="s">
         <v>17</v>
       </c>
       <c r="D23" s="13">
-        <v>274.86</v>
+        <v>271.5</v>
       </c>
       <c r="E23" s="13">
-        <v>236.85</v>
+        <v>236.95</v>
       </c>
       <c r="F23" s="13">
-        <v>246.85</v>
+        <v>246.95</v>
       </c>
       <c r="G23" s="13" t="s">
         <v>18</v>
       </c>
     </row>
-    <row r="24" spans="1:7" x14ac:dyDescent="0.35">
+    <row r="24" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A24" s="7">
-        <v>46287</v>
+        <v>46288</v>
       </c>
       <c r="B24" s="8"/>
       <c r="C24" s="20" t="s">
         <v>19</v>
       </c>
       <c r="D24" s="10">
-        <v>275.35000000000002</v>
+        <v>271.98</v>
       </c>
       <c r="E24" s="10">
-        <v>236.1</v>
+        <v>236.2</v>
       </c>
       <c r="F24" s="10">
-        <v>246.1</v>
+        <v>246.2</v>
       </c>
       <c r="G24" s="10" t="s">
         <v>18</v>
       </c>
     </row>
-    <row r="25" spans="1:7" x14ac:dyDescent="0.35">
+    <row r="25" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A25" s="11">
-        <v>46287</v>
+        <v>46288</v>
       </c>
       <c r="B25" s="12"/>
       <c r="C25" s="21" t="s">
         <v>20</v>
       </c>
       <c r="D25" s="13">
-        <v>272.08999999999997</v>
+        <v>268.72000000000003</v>
       </c>
       <c r="E25" s="13">
-        <v>236.21</v>
+        <v>236.31</v>
       </c>
       <c r="F25" s="13">
-        <v>246.21</v>
+        <v>246.31</v>
       </c>
       <c r="G25" s="13">
-        <v>234.1</v>
-      </c>
-    </row>
-    <row r="26" spans="1:7" x14ac:dyDescent="0.35">
+        <v>234.21</v>
+      </c>
+    </row>
+    <row r="26" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A26" s="7">
-        <v>46287</v>
+        <v>46288</v>
       </c>
       <c r="B26" s="8"/>
       <c r="C26" s="20" t="s">
         <v>21</v>
       </c>
       <c r="D26" s="10">
-        <v>273.86</v>
+        <v>270.48</v>
       </c>
       <c r="E26" s="10">
-        <v>237.69</v>
+        <v>237.79</v>
       </c>
       <c r="F26" s="10">
-        <v>247.69</v>
+        <v>247.79</v>
       </c>
       <c r="G26" s="10" t="s">
         <v>18</v>
       </c>
     </row>
-    <row r="27" spans="1:7" x14ac:dyDescent="0.35">
+    <row r="27" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A27" s="11">
-        <v>46284</v>
+        <v>46287</v>
       </c>
       <c r="B27" s="12"/>
       <c r="C27" s="12" t="s">
         <v>16</v>
       </c>
       <c r="D27" s="13">
-        <v>275.93</v>
+        <v>276.39999999999998</v>
       </c>
       <c r="E27" s="13">
-        <v>231.14</v>
+        <v>233.23</v>
       </c>
       <c r="F27" s="13">
-        <v>240.74</v>
+        <v>242.83</v>
       </c>
       <c r="G27" s="13">
-        <v>229.86</v>
-      </c>
-    </row>
-    <row r="28" spans="1:7" x14ac:dyDescent="0.35">
+        <v>231.94</v>
+      </c>
+    </row>
+    <row r="28" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A28" s="7">
-        <v>46284</v>
+        <v>46287</v>
       </c>
       <c r="B28" s="8"/>
       <c r="C28" s="20" t="s">
         <v>17</v>
       </c>
       <c r="D28" s="10">
-        <v>275.92</v>
+        <v>274.86</v>
       </c>
       <c r="E28" s="22">
-        <v>236.22</v>
+        <v>236.85</v>
       </c>
       <c r="F28" s="22">
-        <v>246.22</v>
+        <v>246.85</v>
       </c>
       <c r="G28" s="22" t="s">
         <v>18</v>
       </c>
     </row>
-    <row r="29" spans="1:7" x14ac:dyDescent="0.35">
+    <row r="29" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A29" s="11">
-        <v>46284</v>
+        <v>46287</v>
       </c>
       <c r="B29" s="12"/>
       <c r="C29" s="12" t="s">
         <v>19</v>
       </c>
       <c r="D29" s="13">
-        <v>276.41000000000003</v>
+        <v>275.35000000000002</v>
       </c>
       <c r="E29" s="13">
-        <v>235.47</v>
+        <v>236.1</v>
       </c>
       <c r="F29" s="13">
-        <v>245.47</v>
+        <v>246.1</v>
       </c>
       <c r="G29" s="13" t="s">
         <v>18</v>
       </c>
     </row>
-    <row r="30" spans="1:7" x14ac:dyDescent="0.35">
+    <row r="30" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A30" s="7">
-        <v>46284</v>
+        <v>46287</v>
       </c>
       <c r="B30" s="8"/>
       <c r="C30" s="20" t="s">
         <v>20</v>
       </c>
       <c r="D30" s="10">
-        <v>273.16000000000003</v>
+        <v>272.08999999999997</v>
       </c>
       <c r="E30" s="22">
-        <v>235.57</v>
+        <v>236.21</v>
       </c>
       <c r="F30" s="22">
-        <v>245.57</v>
+        <v>246.21</v>
       </c>
       <c r="G30" s="22">
-        <v>233.47</v>
-      </c>
-    </row>
-    <row r="31" spans="1:7" x14ac:dyDescent="0.35">
+        <v>234.1</v>
+      </c>
+    </row>
+    <row r="31" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A31" s="11">
-        <v>46284</v>
+        <v>46287</v>
       </c>
       <c r="B31" s="12"/>
       <c r="C31" s="12" t="s">
         <v>21</v>
       </c>
       <c r="D31" s="13">
-        <v>274.94</v>
+        <v>273.86</v>
       </c>
       <c r="E31" s="13">
-        <v>237.05</v>
+        <v>237.69</v>
       </c>
       <c r="F31" s="13">
-        <v>247.05</v>
+        <v>247.69</v>
       </c>
       <c r="G31" s="13" t="s">
         <v>18</v>
       </c>
     </row>
-    <row r="32" spans="1:7" x14ac:dyDescent="0.35">
+    <row r="32" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A32" s="14"/>
       <c r="B32" s="14"/>
       <c r="C32" s="15"/>
@@ -1269,7 +1269,7 @@
       <c r="F32" s="17"/>
       <c r="G32" s="17"/>
     </row>
-    <row r="33" spans="1:7" ht="20" x14ac:dyDescent="0.35">
+    <row r="33" spans="1:7" ht="20.25" x14ac:dyDescent="0.25">
       <c r="A33" s="29" t="s">
         <v>22</v>
       </c>
@@ -1280,7 +1280,7 @@
       <c r="F33" s="17"/>
       <c r="G33" s="17"/>
     </row>
-    <row r="34" spans="1:7" x14ac:dyDescent="0.35">
+    <row r="34" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A34" s="23" t="s">
         <v>4</v>
       </c>
@@ -1299,54 +1299,54 @@
       </c>
       <c r="G34" s="17"/>
     </row>
-    <row r="35" spans="1:7" x14ac:dyDescent="0.35">
+    <row r="35" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A35" s="7">
-        <v>46287</v>
+        <v>46288</v>
       </c>
       <c r="B35" s="8"/>
       <c r="C35" s="20" t="s">
         <v>23</v>
       </c>
       <c r="D35" s="10">
-        <v>268.56</v>
+        <v>265.2</v>
       </c>
       <c r="E35" s="10">
-        <v>227.94</v>
+        <v>228.01</v>
       </c>
       <c r="F35" s="10">
-        <v>236.94</v>
+        <v>237.01</v>
       </c>
       <c r="G35" s="17"/>
     </row>
-    <row r="36" spans="1:7" x14ac:dyDescent="0.35">
+    <row r="36" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A36" s="11">
-        <v>46284</v>
+        <v>46287</v>
       </c>
       <c r="B36" s="12"/>
       <c r="C36" s="12" t="s">
         <v>23</v>
       </c>
       <c r="D36" s="13">
-        <v>269.63</v>
+        <v>268.56</v>
       </c>
       <c r="E36" s="13">
-        <v>227.22</v>
+        <v>227.94</v>
       </c>
       <c r="F36" s="13">
-        <v>236.22</v>
+        <v>236.94</v>
       </c>
       <c r="G36" s="17"/>
     </row>
-    <row r="37" spans="1:7" x14ac:dyDescent="0.35">
+    <row r="37" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A37" s="7">
-        <v>46287</v>
+        <v>46288</v>
       </c>
       <c r="B37" s="8"/>
       <c r="C37" s="20" t="s">
         <v>24</v>
       </c>
       <c r="D37" s="10">
-        <v>284.18</v>
+        <v>280.82</v>
       </c>
       <c r="E37" s="10" t="s">
         <v>18</v>
@@ -1356,16 +1356,16 @@
       </c>
       <c r="G37" s="17"/>
     </row>
-    <row r="38" spans="1:7" x14ac:dyDescent="0.35">
+    <row r="38" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A38" s="11">
-        <v>46284</v>
+        <v>46287</v>
       </c>
       <c r="B38" s="12"/>
       <c r="C38" s="12" t="s">
         <v>24</v>
       </c>
       <c r="D38" s="13">
-        <v>285.25</v>
+        <v>284.18</v>
       </c>
       <c r="E38" s="13" t="s">
         <v>18</v>
@@ -1375,7 +1375,7 @@
       </c>
       <c r="G38" s="17"/>
     </row>
-    <row r="39" spans="1:7" x14ac:dyDescent="0.35">
+    <row r="39" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A39" s="24"/>
       <c r="B39" s="24"/>
       <c r="C39" s="15"/>
@@ -1384,7 +1384,7 @@
       <c r="F39" s="17"/>
       <c r="G39" s="17"/>
     </row>
-    <row r="40" spans="1:7" ht="20" x14ac:dyDescent="0.35">
+    <row r="40" spans="1:7" ht="20.25" x14ac:dyDescent="0.25">
       <c r="A40" s="29" t="s">
         <v>25</v>
       </c>
@@ -1395,7 +1395,7 @@
       <c r="F40" s="17"/>
       <c r="G40" s="17"/>
     </row>
-    <row r="41" spans="1:7" x14ac:dyDescent="0.35">
+    <row r="41" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A41" s="23" t="s">
         <v>4</v>
       </c>
@@ -1414,83 +1414,83 @@
       </c>
       <c r="G41" s="17"/>
     </row>
-    <row r="42" spans="1:7" x14ac:dyDescent="0.35">
+    <row r="42" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A42" s="7">
-        <v>46287</v>
+        <v>46288</v>
       </c>
       <c r="B42" s="8"/>
       <c r="C42" s="20" t="s">
         <v>26</v>
       </c>
       <c r="D42" s="10">
-        <v>277.7</v>
+        <v>274.38</v>
       </c>
       <c r="E42" s="10">
-        <v>233.06</v>
+        <v>232.79</v>
       </c>
       <c r="F42" s="10">
-        <v>243.06</v>
+        <v>242.79</v>
       </c>
       <c r="G42" s="17"/>
     </row>
-    <row r="43" spans="1:7" x14ac:dyDescent="0.35">
+    <row r="43" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A43" s="11">
-        <v>46287</v>
+        <v>46288</v>
       </c>
       <c r="B43" s="12"/>
       <c r="C43" s="21" t="s">
         <v>27</v>
       </c>
       <c r="D43" s="13">
-        <v>277.3</v>
+        <v>273.98</v>
       </c>
       <c r="E43" s="13">
-        <v>233.48</v>
+        <v>233.2</v>
       </c>
       <c r="F43" s="13">
-        <v>243.48</v>
+        <v>243.2</v>
       </c>
       <c r="G43" s="17"/>
     </row>
-    <row r="44" spans="1:7" x14ac:dyDescent="0.35">
+    <row r="44" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A44" s="7">
-        <v>46284</v>
+        <v>46287</v>
       </c>
       <c r="B44" s="8"/>
       <c r="C44" s="20" t="s">
         <v>26</v>
       </c>
       <c r="D44" s="10">
-        <v>278.72000000000003</v>
+        <v>277.7</v>
       </c>
       <c r="E44" s="10">
-        <v>232.81</v>
+        <v>233.06</v>
       </c>
       <c r="F44" s="10">
-        <v>242.81</v>
+        <v>243.06</v>
       </c>
       <c r="G44" s="17"/>
     </row>
-    <row r="45" spans="1:7" x14ac:dyDescent="0.35">
+    <row r="45" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A45" s="11">
-        <v>46284</v>
+        <v>46287</v>
       </c>
       <c r="B45" s="12"/>
       <c r="C45" s="21" t="s">
         <v>27</v>
       </c>
       <c r="D45" s="13">
-        <v>278.31</v>
+        <v>277.3</v>
       </c>
       <c r="E45" s="13">
-        <v>233.23</v>
+        <v>233.48</v>
       </c>
       <c r="F45" s="13">
-        <v>243.23</v>
+        <v>243.48</v>
       </c>
       <c r="G45" s="17"/>
     </row>
-    <row r="46" spans="1:7" x14ac:dyDescent="0.35">
+    <row r="46" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A46" s="14"/>
       <c r="B46" s="24"/>
       <c r="C46" s="15"/>
@@ -1499,7 +1499,7 @@
       <c r="F46" s="16"/>
       <c r="G46" s="17"/>
     </row>
-    <row r="47" spans="1:7" ht="20" x14ac:dyDescent="0.35">
+    <row r="47" spans="1:7" ht="20.25" x14ac:dyDescent="0.25">
       <c r="A47" s="25" t="s">
         <v>28</v>
       </c>
@@ -1510,7 +1510,7 @@
       <c r="F47" s="17"/>
       <c r="G47" s="17"/>
     </row>
-    <row r="48" spans="1:7" x14ac:dyDescent="0.35">
+    <row r="48" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A48" s="23" t="s">
         <v>4</v>
       </c>
@@ -1529,83 +1529,83 @@
       </c>
       <c r="G48" s="17"/>
     </row>
-    <row r="49" spans="1:7" x14ac:dyDescent="0.35">
+    <row r="49" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A49" s="7">
-        <v>46287</v>
+        <v>46288</v>
       </c>
       <c r="B49" s="8"/>
       <c r="C49" s="20" t="s">
         <v>29</v>
       </c>
       <c r="D49" s="10">
-        <v>266.14</v>
+        <v>267.55</v>
       </c>
       <c r="E49" s="10">
-        <v>226.83</v>
+        <v>228.64</v>
       </c>
       <c r="F49" s="10">
-        <v>236.83</v>
+        <v>238.65</v>
       </c>
       <c r="G49" s="28"/>
     </row>
-    <row r="50" spans="1:7" x14ac:dyDescent="0.35">
+    <row r="50" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A50" s="11">
-        <v>46287</v>
+        <v>46288</v>
       </c>
       <c r="B50" s="12"/>
       <c r="C50" s="21" t="s">
         <v>30</v>
       </c>
       <c r="D50" s="13">
-        <v>264.13</v>
+        <v>265.52</v>
       </c>
       <c r="E50" s="13">
-        <v>226.66</v>
+        <v>228.47</v>
       </c>
       <c r="F50" s="13">
-        <v>236.67</v>
+        <v>238.47</v>
       </c>
       <c r="G50" s="28"/>
     </row>
-    <row r="51" spans="1:7" x14ac:dyDescent="0.35">
+    <row r="51" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A51" s="7">
-        <v>46284</v>
+        <v>46287</v>
       </c>
       <c r="B51" s="8"/>
       <c r="C51" s="20" t="s">
         <v>29</v>
       </c>
       <c r="D51" s="10">
-        <v>263.76</v>
+        <v>266.14</v>
       </c>
       <c r="E51" s="10">
-        <v>224.63</v>
+        <v>226.83</v>
       </c>
       <c r="F51" s="10">
-        <v>234.63</v>
+        <v>236.83</v>
       </c>
       <c r="G51" s="17"/>
     </row>
-    <row r="52" spans="1:7" x14ac:dyDescent="0.35">
+    <row r="52" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A52" s="11">
-        <v>46284</v>
+        <v>46287</v>
       </c>
       <c r="B52" s="12"/>
       <c r="C52" s="21" t="s">
         <v>30</v>
       </c>
       <c r="D52" s="13">
-        <v>261.77</v>
+        <v>264.13</v>
       </c>
       <c r="E52" s="13">
-        <v>224.47</v>
+        <v>226.66</v>
       </c>
       <c r="F52" s="13">
-        <v>234.47</v>
+        <v>236.67</v>
       </c>
       <c r="G52" s="17"/>
     </row>
-    <row r="53" spans="1:7" x14ac:dyDescent="0.35">
+    <row r="53" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A53" s="14"/>
       <c r="B53" s="14"/>
       <c r="C53" s="15"/>
@@ -1614,7 +1614,7 @@
       <c r="F53" s="16"/>
       <c r="G53" s="17"/>
     </row>
-    <row r="54" spans="1:7" ht="20" x14ac:dyDescent="0.35">
+    <row r="54" spans="1:7" ht="20.25" x14ac:dyDescent="0.25">
       <c r="A54" s="27" t="s">
         <v>31</v>
       </c>
@@ -1625,7 +1625,7 @@
       <c r="F54" s="17"/>
       <c r="G54" s="17"/>
     </row>
-    <row r="55" spans="1:7" x14ac:dyDescent="0.35">
+    <row r="55" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A55" s="23" t="s">
         <v>4</v>
       </c>
@@ -1644,54 +1644,54 @@
       </c>
       <c r="G55" s="17"/>
     </row>
-    <row r="56" spans="1:7" x14ac:dyDescent="0.35">
+    <row r="56" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A56" s="7">
-        <v>46287</v>
+        <v>46288</v>
       </c>
       <c r="B56" s="8"/>
       <c r="C56" s="20" t="s">
         <v>32</v>
       </c>
       <c r="D56" s="10">
-        <v>286.70999999999998</v>
+        <v>283.32</v>
       </c>
       <c r="E56" s="10">
-        <v>250.91</v>
+        <v>251.24</v>
       </c>
       <c r="F56" s="10">
-        <v>260.91000000000003</v>
+        <v>261.24</v>
       </c>
       <c r="G56" s="17"/>
     </row>
-    <row r="57" spans="1:7" x14ac:dyDescent="0.35">
+    <row r="57" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A57" s="11">
-        <v>46287</v>
+        <v>46288</v>
       </c>
       <c r="B57" s="12"/>
       <c r="C57" s="21" t="s">
         <v>33</v>
       </c>
       <c r="D57" s="13">
-        <v>275.68</v>
+        <v>272.32</v>
       </c>
       <c r="E57" s="13">
-        <v>238.37</v>
+        <v>238.38</v>
       </c>
       <c r="F57" s="13">
-        <v>248.37</v>
+        <v>248.38</v>
       </c>
       <c r="G57" s="17"/>
     </row>
-    <row r="58" spans="1:7" x14ac:dyDescent="0.35">
+    <row r="58" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A58" s="7">
-        <v>46287</v>
+        <v>46288</v>
       </c>
       <c r="B58" s="8"/>
       <c r="C58" s="20" t="s">
         <v>34</v>
       </c>
       <c r="D58" s="10">
-        <v>276.92</v>
+        <v>273.58</v>
       </c>
       <c r="E58" s="10" t="s">
         <v>18</v>
@@ -1701,111 +1701,111 @@
       </c>
       <c r="G58" s="17"/>
     </row>
-    <row r="59" spans="1:7" x14ac:dyDescent="0.35">
+    <row r="59" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A59" s="11">
-        <v>46287</v>
+        <v>46288</v>
       </c>
       <c r="B59" s="12"/>
       <c r="C59" s="21" t="s">
         <v>35</v>
       </c>
       <c r="D59" s="13">
-        <v>272.76</v>
+        <v>269.33</v>
       </c>
       <c r="E59" s="13">
-        <v>232.74</v>
+        <v>232.76</v>
       </c>
       <c r="F59" s="13" t="s">
         <v>18</v>
       </c>
       <c r="G59" s="17"/>
     </row>
-    <row r="60" spans="1:7" x14ac:dyDescent="0.35">
+    <row r="60" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A60" s="7">
-        <v>46287</v>
+        <v>46288</v>
       </c>
       <c r="B60" s="8"/>
       <c r="C60" s="20" t="s">
         <v>36</v>
       </c>
       <c r="D60" s="10">
-        <v>268.58999999999997</v>
+        <v>265.16000000000003</v>
       </c>
       <c r="E60" s="10">
-        <v>228.69</v>
+        <v>228.7</v>
       </c>
       <c r="F60" s="10">
-        <v>238.69</v>
+        <v>238.7</v>
       </c>
       <c r="G60" s="17"/>
     </row>
-    <row r="61" spans="1:7" x14ac:dyDescent="0.35">
+    <row r="61" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A61" s="11">
-        <v>46287</v>
+        <v>46288</v>
       </c>
       <c r="B61" s="12"/>
       <c r="C61" s="21" t="s">
         <v>37</v>
       </c>
       <c r="D61" s="13">
-        <v>274.08</v>
+        <v>270.64</v>
       </c>
       <c r="E61" s="13">
-        <v>246.33</v>
+        <v>246.55</v>
       </c>
       <c r="F61" s="13" t="s">
         <v>18</v>
       </c>
       <c r="G61" s="17"/>
     </row>
-    <row r="62" spans="1:7" x14ac:dyDescent="0.35">
+    <row r="62" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A62" s="7">
-        <v>46284</v>
+        <v>46287</v>
       </c>
       <c r="B62" s="8"/>
       <c r="C62" s="20" t="s">
         <v>32</v>
       </c>
       <c r="D62" s="10">
-        <v>287.8</v>
+        <v>286.70999999999998</v>
       </c>
       <c r="E62" s="10">
-        <v>250.05</v>
+        <v>250.91</v>
       </c>
       <c r="F62" s="10">
-        <v>260.05</v>
+        <v>260.91000000000003</v>
       </c>
       <c r="G62" s="17"/>
     </row>
-    <row r="63" spans="1:7" x14ac:dyDescent="0.35">
+    <row r="63" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A63" s="11">
-        <v>46284</v>
+        <v>46287</v>
       </c>
       <c r="B63" s="12"/>
       <c r="C63" s="21" t="s">
         <v>33</v>
       </c>
       <c r="D63" s="13">
-        <v>276.74</v>
+        <v>275.68</v>
       </c>
       <c r="E63" s="13">
-        <v>237.83</v>
+        <v>238.37</v>
       </c>
       <c r="F63" s="13">
-        <v>247.83</v>
+        <v>248.37</v>
       </c>
       <c r="G63" s="17"/>
     </row>
-    <row r="64" spans="1:7" x14ac:dyDescent="0.35">
+    <row r="64" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A64" s="7">
-        <v>46284</v>
+        <v>46287</v>
       </c>
       <c r="B64" s="8"/>
       <c r="C64" s="20" t="s">
         <v>34</v>
       </c>
       <c r="D64" s="10">
-        <v>277.98</v>
+        <v>276.92</v>
       </c>
       <c r="E64" s="10" t="s">
         <v>18</v>
@@ -1815,55 +1815,55 @@
       </c>
       <c r="G64" s="17"/>
     </row>
-    <row r="65" spans="1:6" x14ac:dyDescent="0.35">
+    <row r="65" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A65" s="11">
-        <v>46284</v>
+        <v>46287</v>
       </c>
       <c r="B65" s="12"/>
       <c r="C65" s="21" t="s">
         <v>35</v>
       </c>
       <c r="D65" s="13">
-        <v>273.89999999999998</v>
+        <v>272.76</v>
       </c>
       <c r="E65" s="13">
-        <v>232.21</v>
+        <v>232.74</v>
       </c>
       <c r="F65" s="13" t="s">
         <v>18</v>
       </c>
     </row>
-    <row r="66" spans="1:6" x14ac:dyDescent="0.35">
+    <row r="66" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A66" s="7">
-        <v>46284</v>
+        <v>46287</v>
       </c>
       <c r="B66" s="8"/>
       <c r="C66" s="20" t="s">
         <v>36</v>
       </c>
       <c r="D66" s="10">
-        <v>269.74</v>
+        <v>268.58999999999997</v>
       </c>
       <c r="E66" s="10">
-        <v>228.15</v>
+        <v>228.69</v>
       </c>
       <c r="F66" s="10">
-        <v>238.15</v>
-      </c>
-    </row>
-    <row r="67" spans="1:6" x14ac:dyDescent="0.35">
+        <v>238.69</v>
+      </c>
+    </row>
+    <row r="67" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A67" s="11">
-        <v>46284</v>
+        <v>46287</v>
       </c>
       <c r="B67" s="12"/>
       <c r="C67" s="21" t="s">
         <v>37</v>
       </c>
       <c r="D67" s="13">
-        <v>275.23</v>
+        <v>274.08</v>
       </c>
       <c r="E67" s="13">
-        <v>245.58</v>
+        <v>246.33</v>
       </c>
       <c r="F67" s="13" t="s">
         <v>18</v>

</xml_diff>

<commit_message>
Wed Sep 23 06:06:40 UTC 2026
</commit_message>
<xml_diff>
--- a/bp.com-content-dam-bp-country-sites-en_au-australia-home-products-services-pricing-tgp-excel.xlsx
+++ b/bp.com-content-dam-bp-country-sites-en_au-australia-home-products-services-pricing-tgp-excel.xlsx
@@ -1,14 +1,14 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="30131"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="30326"/>
   <workbookPr codeName="ThisWorkbook" defaultThemeVersion="166925"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://bp365.sharepoint.com/sites/WholesalePricing/Shared Documents/B2C/TGP/Daily TGP/Web TGP/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="14_{7DD8403A-A834-46A5-861F-04E937D9559A}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="14_{26F80EAB-9BD4-422D-A701-E3FA97EF024F}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-28920" yWindow="-60" windowWidth="29040" windowHeight="15720" xr2:uid="{1B412EEF-F96D-4DF4-A4E9-C7F0F183C2FB}"/>
   </bookViews>
@@ -808,128 +808,128 @@
     </row>
     <row r="8" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A8" s="7">
-        <v>46288</v>
+        <v>46289</v>
       </c>
       <c r="B8" s="8"/>
       <c r="C8" s="9" t="s">
         <v>10</v>
       </c>
       <c r="D8" s="10">
-        <v>273.36</v>
+        <v>269.89</v>
       </c>
       <c r="E8" s="10">
-        <v>234.56</v>
+        <v>234.64</v>
       </c>
       <c r="F8" s="10">
-        <v>244.56</v>
+        <v>244.64</v>
       </c>
       <c r="G8" s="10">
-        <v>234.52</v>
+        <v>234.6</v>
       </c>
     </row>
     <row r="9" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A9" s="11">
-        <v>46288</v>
+        <v>46289</v>
       </c>
       <c r="B9" s="12"/>
       <c r="C9" s="12" t="s">
         <v>11</v>
       </c>
       <c r="D9" s="13">
-        <v>273.36</v>
+        <v>269.89</v>
       </c>
       <c r="E9" s="13">
-        <v>234.56</v>
+        <v>234.64</v>
       </c>
       <c r="F9" s="13">
-        <v>244.56</v>
+        <v>244.64</v>
       </c>
       <c r="G9" s="13">
-        <v>234.52</v>
+        <v>234.6</v>
       </c>
     </row>
     <row r="10" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A10" s="7">
-        <v>46288</v>
+        <v>46289</v>
       </c>
       <c r="B10" s="8"/>
       <c r="C10" s="9" t="s">
         <v>12</v>
       </c>
       <c r="D10" s="10">
-        <v>266.67</v>
+        <v>262.87</v>
       </c>
       <c r="E10" s="10">
-        <v>229.08</v>
+        <v>228.86</v>
       </c>
       <c r="F10" s="10">
-        <v>239.08</v>
+        <v>238.86</v>
       </c>
       <c r="G10" s="10">
-        <v>229.5</v>
+        <v>229.27</v>
       </c>
     </row>
     <row r="11" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A11" s="11">
-        <v>46287</v>
+        <v>46288</v>
       </c>
       <c r="B11" s="12"/>
       <c r="C11" s="12" t="s">
         <v>10</v>
       </c>
       <c r="D11" s="13">
-        <v>276.38</v>
+        <v>273.36</v>
       </c>
       <c r="E11" s="13">
-        <v>234.19</v>
+        <v>234.56</v>
       </c>
       <c r="F11" s="13">
-        <v>244.19</v>
+        <v>244.56</v>
       </c>
       <c r="G11" s="13">
-        <v>234.15</v>
+        <v>234.52</v>
       </c>
     </row>
     <row r="12" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A12" s="7">
-        <v>46287</v>
+        <v>46288</v>
       </c>
       <c r="B12" s="8"/>
       <c r="C12" s="9" t="s">
         <v>11</v>
       </c>
       <c r="D12" s="10">
-        <v>276.38</v>
+        <v>273.36</v>
       </c>
       <c r="E12" s="10">
-        <v>234.19</v>
+        <v>234.56</v>
       </c>
       <c r="F12" s="10">
-        <v>244.19</v>
+        <v>244.56</v>
       </c>
       <c r="G12" s="10">
-        <v>234.15</v>
+        <v>234.52</v>
       </c>
     </row>
     <row r="13" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A13" s="11">
-        <v>46287</v>
+        <v>46288</v>
       </c>
       <c r="B13" s="12"/>
       <c r="C13" s="12" t="s">
         <v>12</v>
       </c>
       <c r="D13" s="13">
-        <v>270.04000000000002</v>
+        <v>266.67</v>
       </c>
       <c r="E13" s="13">
-        <v>229.01</v>
+        <v>229.08</v>
       </c>
       <c r="F13" s="13">
-        <v>239.01</v>
+        <v>239.08</v>
       </c>
       <c r="G13" s="13">
-        <v>229.42</v>
+        <v>229.5</v>
       </c>
     </row>
     <row r="14" spans="1:7" x14ac:dyDescent="0.25">
@@ -973,39 +973,39 @@
     </row>
     <row r="17" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A17" s="7">
-        <v>46288</v>
+        <v>46289</v>
       </c>
       <c r="B17" s="8"/>
       <c r="C17" s="20" t="s">
         <v>14</v>
       </c>
       <c r="D17" s="10">
-        <v>271.24</v>
+        <v>267.39</v>
       </c>
       <c r="E17" s="10">
-        <v>233.03</v>
+        <v>232.76</v>
       </c>
       <c r="F17" s="10">
-        <v>243.03</v>
+        <v>242.76</v>
       </c>
       <c r="G17" s="17"/>
     </row>
     <row r="18" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A18" s="11">
-        <v>46287</v>
+        <v>46288</v>
       </c>
       <c r="B18" s="12"/>
       <c r="C18" s="12" t="s">
         <v>14</v>
       </c>
       <c r="D18" s="13">
-        <v>274.66000000000003</v>
+        <v>271.24</v>
       </c>
       <c r="E18" s="13">
-        <v>233.01</v>
+        <v>233.03</v>
       </c>
       <c r="F18" s="13">
-        <v>243.01</v>
+        <v>243.03</v>
       </c>
       <c r="G18" s="17"/>
     </row>
@@ -1052,41 +1052,41 @@
     </row>
     <row r="22" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A22" s="7">
-        <v>46288</v>
+        <v>46289</v>
       </c>
       <c r="B22" s="8"/>
       <c r="C22" s="20" t="s">
         <v>16</v>
       </c>
       <c r="D22" s="10">
-        <v>273.37</v>
+        <v>269.91000000000003</v>
       </c>
       <c r="E22" s="10">
-        <v>233.6</v>
+        <v>233.68</v>
       </c>
       <c r="F22" s="10">
-        <v>243.2</v>
+        <v>243.28</v>
       </c>
       <c r="G22" s="10">
-        <v>232.32</v>
+        <v>232.39</v>
       </c>
     </row>
     <row r="23" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A23" s="11">
-        <v>46288</v>
+        <v>46289</v>
       </c>
       <c r="B23" s="12"/>
       <c r="C23" s="21" t="s">
         <v>17</v>
       </c>
       <c r="D23" s="13">
-        <v>271.5</v>
+        <v>267.7</v>
       </c>
       <c r="E23" s="13">
-        <v>236.95</v>
+        <v>236.74</v>
       </c>
       <c r="F23" s="13">
-        <v>246.95</v>
+        <v>246.74</v>
       </c>
       <c r="G23" s="13" t="s">
         <v>18</v>
@@ -1094,20 +1094,20 @@
     </row>
     <row r="24" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A24" s="7">
-        <v>46288</v>
+        <v>46289</v>
       </c>
       <c r="B24" s="8"/>
       <c r="C24" s="20" t="s">
         <v>19</v>
       </c>
       <c r="D24" s="10">
-        <v>271.98</v>
+        <v>268.18</v>
       </c>
       <c r="E24" s="10">
-        <v>236.2</v>
+        <v>235.99</v>
       </c>
       <c r="F24" s="10">
-        <v>246.2</v>
+        <v>245.99</v>
       </c>
       <c r="G24" s="10" t="s">
         <v>18</v>
@@ -1115,41 +1115,41 @@
     </row>
     <row r="25" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A25" s="11">
-        <v>46288</v>
+        <v>46289</v>
       </c>
       <c r="B25" s="12"/>
       <c r="C25" s="21" t="s">
         <v>20</v>
       </c>
       <c r="D25" s="13">
-        <v>268.72000000000003</v>
+        <v>264.91000000000003</v>
       </c>
       <c r="E25" s="13">
-        <v>236.31</v>
+        <v>236.11</v>
       </c>
       <c r="F25" s="13">
-        <v>246.31</v>
+        <v>246.11</v>
       </c>
       <c r="G25" s="13">
-        <v>234.21</v>
+        <v>234</v>
       </c>
     </row>
     <row r="26" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A26" s="7">
-        <v>46288</v>
+        <v>46289</v>
       </c>
       <c r="B26" s="8"/>
       <c r="C26" s="20" t="s">
         <v>21</v>
       </c>
       <c r="D26" s="10">
-        <v>270.48</v>
+        <v>266.66000000000003</v>
       </c>
       <c r="E26" s="10">
-        <v>237.79</v>
+        <v>237.59</v>
       </c>
       <c r="F26" s="10">
-        <v>247.79</v>
+        <v>247.59</v>
       </c>
       <c r="G26" s="10" t="s">
         <v>18</v>
@@ -1157,41 +1157,41 @@
     </row>
     <row r="27" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A27" s="11">
-        <v>46287</v>
+        <v>46288</v>
       </c>
       <c r="B27" s="12"/>
       <c r="C27" s="12" t="s">
         <v>16</v>
       </c>
       <c r="D27" s="13">
-        <v>276.39999999999998</v>
+        <v>273.37</v>
       </c>
       <c r="E27" s="13">
-        <v>233.23</v>
+        <v>233.6</v>
       </c>
       <c r="F27" s="13">
-        <v>242.83</v>
+        <v>243.2</v>
       </c>
       <c r="G27" s="13">
-        <v>231.94</v>
+        <v>232.32</v>
       </c>
     </row>
     <row r="28" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A28" s="7">
-        <v>46287</v>
+        <v>46288</v>
       </c>
       <c r="B28" s="8"/>
       <c r="C28" s="20" t="s">
         <v>17</v>
       </c>
       <c r="D28" s="10">
-        <v>274.86</v>
+        <v>271.5</v>
       </c>
       <c r="E28" s="22">
-        <v>236.85</v>
+        <v>236.95</v>
       </c>
       <c r="F28" s="22">
-        <v>246.85</v>
+        <v>246.95</v>
       </c>
       <c r="G28" s="22" t="s">
         <v>18</v>
@@ -1199,20 +1199,20 @@
     </row>
     <row r="29" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A29" s="11">
-        <v>46287</v>
+        <v>46288</v>
       </c>
       <c r="B29" s="12"/>
       <c r="C29" s="12" t="s">
         <v>19</v>
       </c>
       <c r="D29" s="13">
-        <v>275.35000000000002</v>
+        <v>271.98</v>
       </c>
       <c r="E29" s="13">
-        <v>236.1</v>
+        <v>236.2</v>
       </c>
       <c r="F29" s="13">
-        <v>246.1</v>
+        <v>246.2</v>
       </c>
       <c r="G29" s="13" t="s">
         <v>18</v>
@@ -1220,41 +1220,41 @@
     </row>
     <row r="30" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A30" s="7">
-        <v>46287</v>
+        <v>46288</v>
       </c>
       <c r="B30" s="8"/>
       <c r="C30" s="20" t="s">
         <v>20</v>
       </c>
       <c r="D30" s="10">
-        <v>272.08999999999997</v>
+        <v>268.72000000000003</v>
       </c>
       <c r="E30" s="22">
-        <v>236.21</v>
+        <v>236.31</v>
       </c>
       <c r="F30" s="22">
-        <v>246.21</v>
+        <v>246.31</v>
       </c>
       <c r="G30" s="22">
-        <v>234.1</v>
+        <v>234.21</v>
       </c>
     </row>
     <row r="31" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A31" s="11">
-        <v>46287</v>
+        <v>46288</v>
       </c>
       <c r="B31" s="12"/>
       <c r="C31" s="12" t="s">
         <v>21</v>
       </c>
       <c r="D31" s="13">
-        <v>273.86</v>
+        <v>270.48</v>
       </c>
       <c r="E31" s="13">
-        <v>237.69</v>
+        <v>237.79</v>
       </c>
       <c r="F31" s="13">
-        <v>247.69</v>
+        <v>247.79</v>
       </c>
       <c r="G31" s="13" t="s">
         <v>18</v>
@@ -1301,52 +1301,52 @@
     </row>
     <row r="35" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A35" s="7">
-        <v>46288</v>
+        <v>46289</v>
       </c>
       <c r="B35" s="8"/>
       <c r="C35" s="20" t="s">
         <v>23</v>
       </c>
       <c r="D35" s="10">
-        <v>265.2</v>
+        <v>261.39999999999998</v>
       </c>
       <c r="E35" s="10">
-        <v>228.01</v>
+        <v>227.79</v>
       </c>
       <c r="F35" s="10">
-        <v>237.01</v>
+        <v>236.79</v>
       </c>
       <c r="G35" s="17"/>
     </row>
     <row r="36" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A36" s="11">
-        <v>46287</v>
+        <v>46288</v>
       </c>
       <c r="B36" s="12"/>
       <c r="C36" s="12" t="s">
         <v>23</v>
       </c>
       <c r="D36" s="13">
-        <v>268.56</v>
+        <v>265.2</v>
       </c>
       <c r="E36" s="13">
-        <v>227.94</v>
+        <v>228.01</v>
       </c>
       <c r="F36" s="13">
-        <v>236.94</v>
+        <v>237.01</v>
       </c>
       <c r="G36" s="17"/>
     </row>
     <row r="37" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A37" s="7">
-        <v>46288</v>
+        <v>46289</v>
       </c>
       <c r="B37" s="8"/>
       <c r="C37" s="20" t="s">
         <v>24</v>
       </c>
       <c r="D37" s="10">
-        <v>280.82</v>
+        <v>277.02</v>
       </c>
       <c r="E37" s="10" t="s">
         <v>18</v>
@@ -1358,14 +1358,14 @@
     </row>
     <row r="38" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A38" s="11">
-        <v>46287</v>
+        <v>46288</v>
       </c>
       <c r="B38" s="12"/>
       <c r="C38" s="12" t="s">
         <v>24</v>
       </c>
       <c r="D38" s="13">
-        <v>284.18</v>
+        <v>280.82</v>
       </c>
       <c r="E38" s="13" t="s">
         <v>18</v>
@@ -1416,77 +1416,77 @@
     </row>
     <row r="42" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A42" s="7">
-        <v>46288</v>
+        <v>46289</v>
       </c>
       <c r="B42" s="8"/>
       <c r="C42" s="20" t="s">
         <v>26</v>
       </c>
       <c r="D42" s="10">
-        <v>274.38</v>
+        <v>270.61</v>
       </c>
       <c r="E42" s="10">
-        <v>232.79</v>
+        <v>232.62</v>
       </c>
       <c r="F42" s="10">
-        <v>242.79</v>
+        <v>242.62</v>
       </c>
       <c r="G42" s="17"/>
     </row>
     <row r="43" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A43" s="11">
-        <v>46288</v>
+        <v>46289</v>
       </c>
       <c r="B43" s="12"/>
       <c r="C43" s="21" t="s">
         <v>27</v>
       </c>
       <c r="D43" s="13">
-        <v>273.98</v>
+        <v>270.22000000000003</v>
       </c>
       <c r="E43" s="13">
-        <v>233.2</v>
+        <v>233.03</v>
       </c>
       <c r="F43" s="13">
-        <v>243.2</v>
+        <v>243.03</v>
       </c>
       <c r="G43" s="17"/>
     </row>
     <row r="44" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A44" s="7">
-        <v>46287</v>
+        <v>46288</v>
       </c>
       <c r="B44" s="8"/>
       <c r="C44" s="20" t="s">
         <v>26</v>
       </c>
       <c r="D44" s="10">
-        <v>277.7</v>
+        <v>274.38</v>
       </c>
       <c r="E44" s="10">
-        <v>233.06</v>
+        <v>232.79</v>
       </c>
       <c r="F44" s="10">
-        <v>243.06</v>
+        <v>242.79</v>
       </c>
       <c r="G44" s="17"/>
     </row>
     <row r="45" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A45" s="11">
-        <v>46287</v>
+        <v>46288</v>
       </c>
       <c r="B45" s="12"/>
       <c r="C45" s="21" t="s">
         <v>27</v>
       </c>
       <c r="D45" s="13">
-        <v>277.3</v>
+        <v>273.98</v>
       </c>
       <c r="E45" s="13">
-        <v>233.48</v>
+        <v>233.2</v>
       </c>
       <c r="F45" s="13">
-        <v>243.48</v>
+        <v>243.2</v>
       </c>
       <c r="G45" s="17"/>
     </row>
@@ -1531,77 +1531,77 @@
     </row>
     <row r="49" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A49" s="7">
-        <v>46288</v>
+        <v>46289</v>
       </c>
       <c r="B49" s="8"/>
       <c r="C49" s="20" t="s">
         <v>29</v>
       </c>
       <c r="D49" s="10">
-        <v>267.55</v>
+        <v>265.43</v>
       </c>
       <c r="E49" s="10">
-        <v>228.64</v>
+        <v>228.67</v>
       </c>
       <c r="F49" s="10">
-        <v>238.65</v>
+        <v>238.67</v>
       </c>
       <c r="G49" s="28"/>
     </row>
     <row r="50" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A50" s="11">
-        <v>46288</v>
+        <v>46289</v>
       </c>
       <c r="B50" s="12"/>
       <c r="C50" s="21" t="s">
         <v>30</v>
       </c>
       <c r="D50" s="13">
-        <v>265.52</v>
+        <v>263.37</v>
       </c>
       <c r="E50" s="13">
-        <v>228.47</v>
+        <v>228.48</v>
       </c>
       <c r="F50" s="13">
-        <v>238.47</v>
+        <v>238.48</v>
       </c>
       <c r="G50" s="28"/>
     </row>
     <row r="51" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A51" s="7">
-        <v>46287</v>
+        <v>46288</v>
       </c>
       <c r="B51" s="8"/>
       <c r="C51" s="20" t="s">
         <v>29</v>
       </c>
       <c r="D51" s="10">
-        <v>266.14</v>
+        <v>267.55</v>
       </c>
       <c r="E51" s="10">
-        <v>226.83</v>
+        <v>228.64</v>
       </c>
       <c r="F51" s="10">
-        <v>236.83</v>
+        <v>238.65</v>
       </c>
       <c r="G51" s="17"/>
     </row>
     <row r="52" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A52" s="11">
-        <v>46287</v>
+        <v>46288</v>
       </c>
       <c r="B52" s="12"/>
       <c r="C52" s="21" t="s">
         <v>30</v>
       </c>
       <c r="D52" s="13">
-        <v>264.13</v>
+        <v>265.52</v>
       </c>
       <c r="E52" s="13">
-        <v>226.66</v>
+        <v>228.47</v>
       </c>
       <c r="F52" s="13">
-        <v>236.67</v>
+        <v>238.47</v>
       </c>
       <c r="G52" s="17"/>
     </row>
@@ -1646,52 +1646,52 @@
     </row>
     <row r="56" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A56" s="7">
-        <v>46288</v>
+        <v>46289</v>
       </c>
       <c r="B56" s="8"/>
       <c r="C56" s="20" t="s">
         <v>32</v>
       </c>
       <c r="D56" s="10">
-        <v>283.32</v>
+        <v>279.49</v>
       </c>
       <c r="E56" s="10">
-        <v>251.24</v>
+        <v>251.21</v>
       </c>
       <c r="F56" s="10">
-        <v>261.24</v>
+        <v>261.20999999999998</v>
       </c>
       <c r="G56" s="17"/>
     </row>
     <row r="57" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A57" s="11">
-        <v>46288</v>
+        <v>46289</v>
       </c>
       <c r="B57" s="12"/>
       <c r="C57" s="21" t="s">
         <v>33</v>
       </c>
       <c r="D57" s="13">
-        <v>272.32</v>
+        <v>268.51</v>
       </c>
       <c r="E57" s="13">
-        <v>238.38</v>
+        <v>238.11</v>
       </c>
       <c r="F57" s="13">
-        <v>248.38</v>
+        <v>248.11</v>
       </c>
       <c r="G57" s="17"/>
     </row>
     <row r="58" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A58" s="7">
-        <v>46288</v>
+        <v>46289</v>
       </c>
       <c r="B58" s="8"/>
       <c r="C58" s="20" t="s">
         <v>34</v>
       </c>
       <c r="D58" s="10">
-        <v>273.58</v>
+        <v>269.77999999999997</v>
       </c>
       <c r="E58" s="10" t="s">
         <v>18</v>
@@ -1703,17 +1703,17 @@
     </row>
     <row r="59" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A59" s="11">
-        <v>46288</v>
+        <v>46289</v>
       </c>
       <c r="B59" s="12"/>
       <c r="C59" s="21" t="s">
         <v>35</v>
       </c>
       <c r="D59" s="13">
-        <v>269.33</v>
+        <v>265.47000000000003</v>
       </c>
       <c r="E59" s="13">
-        <v>232.76</v>
+        <v>232.48</v>
       </c>
       <c r="F59" s="13" t="s">
         <v>18</v>
@@ -1722,36 +1722,36 @@
     </row>
     <row r="60" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A60" s="7">
-        <v>46288</v>
+        <v>46289</v>
       </c>
       <c r="B60" s="8"/>
       <c r="C60" s="20" t="s">
         <v>36</v>
       </c>
       <c r="D60" s="10">
-        <v>265.16000000000003</v>
+        <v>261.31</v>
       </c>
       <c r="E60" s="10">
-        <v>228.7</v>
+        <v>228.43</v>
       </c>
       <c r="F60" s="10">
-        <v>238.7</v>
+        <v>238.43</v>
       </c>
       <c r="G60" s="17"/>
     </row>
     <row r="61" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A61" s="11">
-        <v>46288</v>
+        <v>46289</v>
       </c>
       <c r="B61" s="12"/>
       <c r="C61" s="21" t="s">
         <v>37</v>
       </c>
       <c r="D61" s="13">
-        <v>270.64</v>
+        <v>266.77999999999997</v>
       </c>
       <c r="E61" s="13">
-        <v>246.55</v>
+        <v>246.43</v>
       </c>
       <c r="F61" s="13" t="s">
         <v>18</v>
@@ -1760,52 +1760,52 @@
     </row>
     <row r="62" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A62" s="7">
-        <v>46287</v>
+        <v>46288</v>
       </c>
       <c r="B62" s="8"/>
       <c r="C62" s="20" t="s">
         <v>32</v>
       </c>
       <c r="D62" s="10">
-        <v>286.70999999999998</v>
+        <v>283.32</v>
       </c>
       <c r="E62" s="10">
-        <v>250.91</v>
+        <v>251.24</v>
       </c>
       <c r="F62" s="10">
-        <v>260.91000000000003</v>
+        <v>261.24</v>
       </c>
       <c r="G62" s="17"/>
     </row>
     <row r="63" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A63" s="11">
-        <v>46287</v>
+        <v>46288</v>
       </c>
       <c r="B63" s="12"/>
       <c r="C63" s="21" t="s">
         <v>33</v>
       </c>
       <c r="D63" s="13">
-        <v>275.68</v>
+        <v>272.32</v>
       </c>
       <c r="E63" s="13">
-        <v>238.37</v>
+        <v>238.38</v>
       </c>
       <c r="F63" s="13">
-        <v>248.37</v>
+        <v>248.38</v>
       </c>
       <c r="G63" s="17"/>
     </row>
     <row r="64" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A64" s="7">
-        <v>46287</v>
+        <v>46288</v>
       </c>
       <c r="B64" s="8"/>
       <c r="C64" s="20" t="s">
         <v>34</v>
       </c>
       <c r="D64" s="10">
-        <v>276.92</v>
+        <v>273.58</v>
       </c>
       <c r="E64" s="10" t="s">
         <v>18</v>
@@ -1817,17 +1817,17 @@
     </row>
     <row r="65" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A65" s="11">
-        <v>46287</v>
+        <v>46288</v>
       </c>
       <c r="B65" s="12"/>
       <c r="C65" s="21" t="s">
         <v>35</v>
       </c>
       <c r="D65" s="13">
-        <v>272.76</v>
+        <v>269.33</v>
       </c>
       <c r="E65" s="13">
-        <v>232.74</v>
+        <v>232.76</v>
       </c>
       <c r="F65" s="13" t="s">
         <v>18</v>
@@ -1835,35 +1835,35 @@
     </row>
     <row r="66" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A66" s="7">
-        <v>46287</v>
+        <v>46288</v>
       </c>
       <c r="B66" s="8"/>
       <c r="C66" s="20" t="s">
         <v>36</v>
       </c>
       <c r="D66" s="10">
-        <v>268.58999999999997</v>
+        <v>265.16000000000003</v>
       </c>
       <c r="E66" s="10">
-        <v>228.69</v>
+        <v>228.7</v>
       </c>
       <c r="F66" s="10">
-        <v>238.69</v>
+        <v>238.7</v>
       </c>
     </row>
     <row r="67" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A67" s="11">
-        <v>46287</v>
+        <v>46288</v>
       </c>
       <c r="B67" s="12"/>
       <c r="C67" s="21" t="s">
         <v>37</v>
       </c>
       <c r="D67" s="13">
-        <v>274.08</v>
+        <v>270.64</v>
       </c>
       <c r="E67" s="13">
-        <v>246.33</v>
+        <v>246.55</v>
       </c>
       <c r="F67" s="13" t="s">
         <v>18</v>

</xml_diff>

<commit_message>
Thu Sep 24 06:15:51 UTC 2026
</commit_message>
<xml_diff>
--- a/bp.com-content-dam-bp-country-sites-en_au-australia-home-products-services-pricing-tgp-excel.xlsx
+++ b/bp.com-content-dam-bp-country-sites-en_au-australia-home-products-services-pricing-tgp-excel.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://bp365.sharepoint.com/sites/WholesalePricing/Shared Documents/B2C/TGP/Daily TGP/Web TGP/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="14_{26F80EAB-9BD4-422D-A701-E3FA97EF024F}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="14_{34A09CBA-7C4D-4EF2-9C47-AA9809C45408}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-28920" yWindow="-60" windowWidth="29040" windowHeight="15720" xr2:uid="{1B412EEF-F96D-4DF4-A4E9-C7F0F183C2FB}"/>
   </bookViews>
@@ -808,128 +808,128 @@
     </row>
     <row r="8" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A8" s="7">
-        <v>46289</v>
+        <v>46290</v>
       </c>
       <c r="B8" s="8"/>
       <c r="C8" s="9" t="s">
         <v>10</v>
       </c>
       <c r="D8" s="10">
-        <v>269.89</v>
+        <v>266.55</v>
       </c>
       <c r="E8" s="10">
-        <v>234.64</v>
+        <v>233.88</v>
       </c>
       <c r="F8" s="10">
-        <v>244.64</v>
+        <v>243.88</v>
       </c>
       <c r="G8" s="10">
-        <v>234.6</v>
+        <v>233.85</v>
       </c>
     </row>
     <row r="9" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A9" s="11">
-        <v>46289</v>
+        <v>46290</v>
       </c>
       <c r="B9" s="12"/>
       <c r="C9" s="12" t="s">
         <v>11</v>
       </c>
       <c r="D9" s="13">
-        <v>269.89</v>
+        <v>266.55</v>
       </c>
       <c r="E9" s="13">
-        <v>234.64</v>
+        <v>233.88</v>
       </c>
       <c r="F9" s="13">
-        <v>244.64</v>
+        <v>243.88</v>
       </c>
       <c r="G9" s="13">
-        <v>234.6</v>
+        <v>233.85</v>
       </c>
     </row>
     <row r="10" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A10" s="7">
-        <v>46289</v>
+        <v>46290</v>
       </c>
       <c r="B10" s="8"/>
       <c r="C10" s="9" t="s">
         <v>12</v>
       </c>
       <c r="D10" s="10">
-        <v>262.87</v>
+        <v>259.18</v>
       </c>
       <c r="E10" s="10">
-        <v>228.86</v>
+        <v>227.79</v>
       </c>
       <c r="F10" s="10">
-        <v>238.86</v>
+        <v>237.79</v>
       </c>
       <c r="G10" s="10">
-        <v>229.27</v>
+        <v>228.21</v>
       </c>
     </row>
     <row r="11" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A11" s="11">
-        <v>46288</v>
+        <v>46289</v>
       </c>
       <c r="B11" s="12"/>
       <c r="C11" s="12" t="s">
         <v>10</v>
       </c>
       <c r="D11" s="13">
-        <v>273.36</v>
+        <v>269.89</v>
       </c>
       <c r="E11" s="13">
-        <v>234.56</v>
+        <v>234.64</v>
       </c>
       <c r="F11" s="13">
-        <v>244.56</v>
+        <v>244.64</v>
       </c>
       <c r="G11" s="13">
-        <v>234.52</v>
+        <v>234.6</v>
       </c>
     </row>
     <row r="12" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A12" s="7">
-        <v>46288</v>
+        <v>46289</v>
       </c>
       <c r="B12" s="8"/>
       <c r="C12" s="9" t="s">
         <v>11</v>
       </c>
       <c r="D12" s="10">
-        <v>273.36</v>
+        <v>269.89</v>
       </c>
       <c r="E12" s="10">
-        <v>234.56</v>
+        <v>234.64</v>
       </c>
       <c r="F12" s="10">
-        <v>244.56</v>
+        <v>244.64</v>
       </c>
       <c r="G12" s="10">
-        <v>234.52</v>
+        <v>234.6</v>
       </c>
     </row>
     <row r="13" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A13" s="11">
-        <v>46288</v>
+        <v>46289</v>
       </c>
       <c r="B13" s="12"/>
       <c r="C13" s="12" t="s">
         <v>12</v>
       </c>
       <c r="D13" s="13">
-        <v>266.67</v>
+        <v>262.87</v>
       </c>
       <c r="E13" s="13">
-        <v>229.08</v>
+        <v>228.86</v>
       </c>
       <c r="F13" s="13">
-        <v>239.08</v>
+        <v>238.86</v>
       </c>
       <c r="G13" s="13">
-        <v>229.5</v>
+        <v>229.27</v>
       </c>
     </row>
     <row r="14" spans="1:7" x14ac:dyDescent="0.25">
@@ -973,39 +973,39 @@
     </row>
     <row r="17" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A17" s="7">
-        <v>46289</v>
+        <v>46290</v>
       </c>
       <c r="B17" s="8"/>
       <c r="C17" s="20" t="s">
         <v>14</v>
       </c>
       <c r="D17" s="10">
-        <v>267.39</v>
+        <v>263.62</v>
       </c>
       <c r="E17" s="10">
-        <v>232.76</v>
+        <v>231.63</v>
       </c>
       <c r="F17" s="10">
-        <v>242.76</v>
+        <v>241.63</v>
       </c>
       <c r="G17" s="17"/>
     </row>
     <row r="18" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A18" s="11">
-        <v>46288</v>
+        <v>46289</v>
       </c>
       <c r="B18" s="12"/>
       <c r="C18" s="12" t="s">
         <v>14</v>
       </c>
       <c r="D18" s="13">
-        <v>271.24</v>
+        <v>267.39</v>
       </c>
       <c r="E18" s="13">
-        <v>233.03</v>
+        <v>232.76</v>
       </c>
       <c r="F18" s="13">
-        <v>243.03</v>
+        <v>242.76</v>
       </c>
       <c r="G18" s="17"/>
     </row>
@@ -1052,41 +1052,41 @@
     </row>
     <row r="22" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A22" s="7">
-        <v>46289</v>
+        <v>46290</v>
       </c>
       <c r="B22" s="8"/>
       <c r="C22" s="20" t="s">
         <v>16</v>
       </c>
       <c r="D22" s="10">
-        <v>269.91000000000003</v>
+        <v>267.12</v>
       </c>
       <c r="E22" s="10">
-        <v>233.68</v>
+        <v>231.83</v>
       </c>
       <c r="F22" s="10">
-        <v>243.28</v>
+        <v>241.43</v>
       </c>
       <c r="G22" s="10">
-        <v>232.39</v>
+        <v>230.54</v>
       </c>
     </row>
     <row r="23" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A23" s="11">
-        <v>46289</v>
+        <v>46290</v>
       </c>
       <c r="B23" s="12"/>
       <c r="C23" s="21" t="s">
         <v>17</v>
       </c>
       <c r="D23" s="13">
-        <v>267.7</v>
+        <v>264.02</v>
       </c>
       <c r="E23" s="13">
-        <v>236.74</v>
+        <v>235.7</v>
       </c>
       <c r="F23" s="13">
-        <v>246.74</v>
+        <v>245.7</v>
       </c>
       <c r="G23" s="13" t="s">
         <v>18</v>
@@ -1094,20 +1094,20 @@
     </row>
     <row r="24" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A24" s="7">
-        <v>46289</v>
+        <v>46290</v>
       </c>
       <c r="B24" s="8"/>
       <c r="C24" s="20" t="s">
         <v>19</v>
       </c>
       <c r="D24" s="10">
-        <v>268.18</v>
+        <v>264.48</v>
       </c>
       <c r="E24" s="10">
-        <v>235.99</v>
+        <v>234.95</v>
       </c>
       <c r="F24" s="10">
-        <v>245.99</v>
+        <v>244.95</v>
       </c>
       <c r="G24" s="10" t="s">
         <v>18</v>
@@ -1115,41 +1115,41 @@
     </row>
     <row r="25" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A25" s="11">
-        <v>46289</v>
+        <v>46290</v>
       </c>
       <c r="B25" s="12"/>
       <c r="C25" s="21" t="s">
         <v>20</v>
       </c>
       <c r="D25" s="13">
-        <v>264.91000000000003</v>
+        <v>261.22000000000003</v>
       </c>
       <c r="E25" s="13">
-        <v>236.11</v>
+        <v>235.07</v>
       </c>
       <c r="F25" s="13">
-        <v>246.11</v>
+        <v>245.07</v>
       </c>
       <c r="G25" s="13">
-        <v>234</v>
+        <v>232.97</v>
       </c>
     </row>
     <row r="26" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A26" s="7">
-        <v>46289</v>
+        <v>46290</v>
       </c>
       <c r="B26" s="8"/>
       <c r="C26" s="20" t="s">
         <v>21</v>
       </c>
       <c r="D26" s="10">
-        <v>266.66000000000003</v>
+        <v>262.94</v>
       </c>
       <c r="E26" s="10">
-        <v>237.59</v>
+        <v>236.55</v>
       </c>
       <c r="F26" s="10">
-        <v>247.59</v>
+        <v>246.55</v>
       </c>
       <c r="G26" s="10" t="s">
         <v>18</v>
@@ -1157,41 +1157,41 @@
     </row>
     <row r="27" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A27" s="11">
-        <v>46288</v>
+        <v>46289</v>
       </c>
       <c r="B27" s="12"/>
       <c r="C27" s="12" t="s">
         <v>16</v>
       </c>
       <c r="D27" s="13">
-        <v>273.37</v>
+        <v>269.91000000000003</v>
       </c>
       <c r="E27" s="13">
-        <v>233.6</v>
+        <v>233.68</v>
       </c>
       <c r="F27" s="13">
-        <v>243.2</v>
+        <v>243.28</v>
       </c>
       <c r="G27" s="13">
-        <v>232.32</v>
+        <v>232.39</v>
       </c>
     </row>
     <row r="28" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A28" s="7">
-        <v>46288</v>
+        <v>46289</v>
       </c>
       <c r="B28" s="8"/>
       <c r="C28" s="20" t="s">
         <v>17</v>
       </c>
       <c r="D28" s="10">
-        <v>271.5</v>
+        <v>267.7</v>
       </c>
       <c r="E28" s="22">
-        <v>236.95</v>
+        <v>236.74</v>
       </c>
       <c r="F28" s="22">
-        <v>246.95</v>
+        <v>246.74</v>
       </c>
       <c r="G28" s="22" t="s">
         <v>18</v>
@@ -1199,20 +1199,20 @@
     </row>
     <row r="29" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A29" s="11">
-        <v>46288</v>
+        <v>46289</v>
       </c>
       <c r="B29" s="12"/>
       <c r="C29" s="12" t="s">
         <v>19</v>
       </c>
       <c r="D29" s="13">
-        <v>271.98</v>
+        <v>268.18</v>
       </c>
       <c r="E29" s="13">
-        <v>236.2</v>
+        <v>235.99</v>
       </c>
       <c r="F29" s="13">
-        <v>246.2</v>
+        <v>245.99</v>
       </c>
       <c r="G29" s="13" t="s">
         <v>18</v>
@@ -1220,41 +1220,41 @@
     </row>
     <row r="30" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A30" s="7">
-        <v>46288</v>
+        <v>46289</v>
       </c>
       <c r="B30" s="8"/>
       <c r="C30" s="20" t="s">
         <v>20</v>
       </c>
       <c r="D30" s="10">
-        <v>268.72000000000003</v>
+        <v>264.91000000000003</v>
       </c>
       <c r="E30" s="22">
-        <v>236.31</v>
+        <v>236.11</v>
       </c>
       <c r="F30" s="22">
-        <v>246.31</v>
+        <v>246.11</v>
       </c>
       <c r="G30" s="22">
-        <v>234.21</v>
+        <v>234</v>
       </c>
     </row>
     <row r="31" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A31" s="11">
-        <v>46288</v>
+        <v>46289</v>
       </c>
       <c r="B31" s="12"/>
       <c r="C31" s="12" t="s">
         <v>21</v>
       </c>
       <c r="D31" s="13">
-        <v>270.48</v>
+        <v>266.66000000000003</v>
       </c>
       <c r="E31" s="13">
-        <v>237.79</v>
+        <v>237.59</v>
       </c>
       <c r="F31" s="13">
-        <v>247.79</v>
+        <v>247.59</v>
       </c>
       <c r="G31" s="13" t="s">
         <v>18</v>
@@ -1301,52 +1301,52 @@
     </row>
     <row r="35" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A35" s="7">
-        <v>46289</v>
+        <v>46290</v>
       </c>
       <c r="B35" s="8"/>
       <c r="C35" s="20" t="s">
         <v>23</v>
       </c>
       <c r="D35" s="10">
-        <v>261.39999999999998</v>
+        <v>257.70999999999998</v>
       </c>
       <c r="E35" s="10">
-        <v>227.79</v>
+        <v>226.73</v>
       </c>
       <c r="F35" s="10">
-        <v>236.79</v>
+        <v>235.73</v>
       </c>
       <c r="G35" s="17"/>
     </row>
     <row r="36" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A36" s="11">
-        <v>46288</v>
+        <v>46289</v>
       </c>
       <c r="B36" s="12"/>
       <c r="C36" s="12" t="s">
         <v>23</v>
       </c>
       <c r="D36" s="13">
-        <v>265.2</v>
+        <v>261.39999999999998</v>
       </c>
       <c r="E36" s="13">
-        <v>228.01</v>
+        <v>227.79</v>
       </c>
       <c r="F36" s="13">
-        <v>237.01</v>
+        <v>236.79</v>
       </c>
       <c r="G36" s="17"/>
     </row>
     <row r="37" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A37" s="7">
-        <v>46289</v>
+        <v>46290</v>
       </c>
       <c r="B37" s="8"/>
       <c r="C37" s="20" t="s">
         <v>24</v>
       </c>
       <c r="D37" s="10">
-        <v>277.02</v>
+        <v>273.33</v>
       </c>
       <c r="E37" s="10" t="s">
         <v>18</v>
@@ -1358,14 +1358,14 @@
     </row>
     <row r="38" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A38" s="11">
-        <v>46288</v>
+        <v>46289</v>
       </c>
       <c r="B38" s="12"/>
       <c r="C38" s="12" t="s">
         <v>24</v>
       </c>
       <c r="D38" s="13">
-        <v>280.82</v>
+        <v>277.02</v>
       </c>
       <c r="E38" s="13" t="s">
         <v>18</v>
@@ -1416,77 +1416,77 @@
     </row>
     <row r="42" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A42" s="7">
-        <v>46289</v>
+        <v>46290</v>
       </c>
       <c r="B42" s="8"/>
       <c r="C42" s="20" t="s">
         <v>26</v>
       </c>
       <c r="D42" s="10">
-        <v>270.61</v>
+        <v>266.97000000000003</v>
       </c>
       <c r="E42" s="10">
-        <v>232.62</v>
+        <v>231.64</v>
       </c>
       <c r="F42" s="10">
-        <v>242.62</v>
+        <v>241.64</v>
       </c>
       <c r="G42" s="17"/>
     </row>
     <row r="43" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A43" s="11">
-        <v>46289</v>
+        <v>46290</v>
       </c>
       <c r="B43" s="12"/>
       <c r="C43" s="21" t="s">
         <v>27</v>
       </c>
       <c r="D43" s="13">
-        <v>270.22000000000003</v>
+        <v>266.58</v>
       </c>
       <c r="E43" s="13">
-        <v>233.03</v>
+        <v>232.05</v>
       </c>
       <c r="F43" s="13">
-        <v>243.03</v>
+        <v>242.05</v>
       </c>
       <c r="G43" s="17"/>
     </row>
     <row r="44" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A44" s="7">
-        <v>46288</v>
+        <v>46289</v>
       </c>
       <c r="B44" s="8"/>
       <c r="C44" s="20" t="s">
         <v>26</v>
       </c>
       <c r="D44" s="10">
-        <v>274.38</v>
+        <v>270.61</v>
       </c>
       <c r="E44" s="10">
-        <v>232.79</v>
+        <v>232.62</v>
       </c>
       <c r="F44" s="10">
-        <v>242.79</v>
+        <v>242.62</v>
       </c>
       <c r="G44" s="17"/>
     </row>
     <row r="45" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A45" s="11">
-        <v>46288</v>
+        <v>46289</v>
       </c>
       <c r="B45" s="12"/>
       <c r="C45" s="21" t="s">
         <v>27</v>
       </c>
       <c r="D45" s="13">
-        <v>273.98</v>
+        <v>270.22000000000003</v>
       </c>
       <c r="E45" s="13">
-        <v>233.2</v>
+        <v>233.03</v>
       </c>
       <c r="F45" s="13">
-        <v>243.2</v>
+        <v>243.03</v>
       </c>
       <c r="G45" s="17"/>
     </row>
@@ -1531,77 +1531,77 @@
     </row>
     <row r="49" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A49" s="7">
-        <v>46289</v>
+        <v>46290</v>
       </c>
       <c r="B49" s="8"/>
       <c r="C49" s="20" t="s">
         <v>29</v>
       </c>
       <c r="D49" s="10">
-        <v>265.43</v>
+        <v>263.64</v>
       </c>
       <c r="E49" s="10">
-        <v>228.67</v>
+        <v>228.59</v>
       </c>
       <c r="F49" s="10">
-        <v>238.67</v>
+        <v>238.59</v>
       </c>
       <c r="G49" s="28"/>
     </row>
     <row r="50" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A50" s="11">
-        <v>46289</v>
+        <v>46290</v>
       </c>
       <c r="B50" s="12"/>
       <c r="C50" s="21" t="s">
         <v>30</v>
       </c>
       <c r="D50" s="13">
-        <v>263.37</v>
+        <v>261.56</v>
       </c>
       <c r="E50" s="13">
-        <v>228.48</v>
+        <v>228.39</v>
       </c>
       <c r="F50" s="13">
-        <v>238.48</v>
+        <v>238.39</v>
       </c>
       <c r="G50" s="28"/>
     </row>
     <row r="51" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A51" s="7">
-        <v>46288</v>
+        <v>46289</v>
       </c>
       <c r="B51" s="8"/>
       <c r="C51" s="20" t="s">
         <v>29</v>
       </c>
       <c r="D51" s="10">
-        <v>267.55</v>
+        <v>265.43</v>
       </c>
       <c r="E51" s="10">
-        <v>228.64</v>
+        <v>228.67</v>
       </c>
       <c r="F51" s="10">
-        <v>238.65</v>
+        <v>238.67</v>
       </c>
       <c r="G51" s="17"/>
     </row>
     <row r="52" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A52" s="11">
-        <v>46288</v>
+        <v>46289</v>
       </c>
       <c r="B52" s="12"/>
       <c r="C52" s="21" t="s">
         <v>30</v>
       </c>
       <c r="D52" s="13">
-        <v>265.52</v>
+        <v>263.37</v>
       </c>
       <c r="E52" s="13">
-        <v>228.47</v>
+        <v>228.48</v>
       </c>
       <c r="F52" s="13">
-        <v>238.47</v>
+        <v>238.48</v>
       </c>
       <c r="G52" s="17"/>
     </row>
@@ -1646,52 +1646,52 @@
     </row>
     <row r="56" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A56" s="7">
-        <v>46289</v>
+        <v>46290</v>
       </c>
       <c r="B56" s="8"/>
       <c r="C56" s="20" t="s">
         <v>32</v>
       </c>
       <c r="D56" s="10">
-        <v>279.49</v>
+        <v>275.76</v>
       </c>
       <c r="E56" s="10">
-        <v>251.21</v>
+        <v>250.46</v>
       </c>
       <c r="F56" s="10">
-        <v>261.20999999999998</v>
+        <v>260.45999999999998</v>
       </c>
       <c r="G56" s="17"/>
     </row>
     <row r="57" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A57" s="11">
-        <v>46289</v>
+        <v>46290</v>
       </c>
       <c r="B57" s="12"/>
       <c r="C57" s="21" t="s">
         <v>33</v>
       </c>
       <c r="D57" s="13">
-        <v>268.51</v>
+        <v>264.82</v>
       </c>
       <c r="E57" s="13">
-        <v>238.11</v>
+        <v>236.97</v>
       </c>
       <c r="F57" s="13">
-        <v>248.11</v>
+        <v>246.97</v>
       </c>
       <c r="G57" s="17"/>
     </row>
     <row r="58" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A58" s="7">
-        <v>46289</v>
+        <v>46290</v>
       </c>
       <c r="B58" s="8"/>
       <c r="C58" s="20" t="s">
         <v>34</v>
       </c>
       <c r="D58" s="10">
-        <v>269.77999999999997</v>
+        <v>266.11</v>
       </c>
       <c r="E58" s="10" t="s">
         <v>18</v>
@@ -1703,17 +1703,17 @@
     </row>
     <row r="59" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A59" s="11">
-        <v>46289</v>
+        <v>46290</v>
       </c>
       <c r="B59" s="12"/>
       <c r="C59" s="21" t="s">
         <v>35</v>
       </c>
       <c r="D59" s="13">
-        <v>265.47000000000003</v>
+        <v>261.7</v>
       </c>
       <c r="E59" s="13">
-        <v>232.48</v>
+        <v>231.34</v>
       </c>
       <c r="F59" s="13" t="s">
         <v>18</v>
@@ -1722,36 +1722,36 @@
     </row>
     <row r="60" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A60" s="7">
-        <v>46289</v>
+        <v>46290</v>
       </c>
       <c r="B60" s="8"/>
       <c r="C60" s="20" t="s">
         <v>36</v>
       </c>
       <c r="D60" s="10">
-        <v>261.31</v>
+        <v>257.52999999999997</v>
       </c>
       <c r="E60" s="10">
-        <v>228.43</v>
+        <v>227.29</v>
       </c>
       <c r="F60" s="10">
-        <v>238.43</v>
+        <v>237.29</v>
       </c>
       <c r="G60" s="17"/>
     </row>
     <row r="61" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A61" s="11">
-        <v>46289</v>
+        <v>46290</v>
       </c>
       <c r="B61" s="12"/>
       <c r="C61" s="21" t="s">
         <v>37</v>
       </c>
       <c r="D61" s="13">
-        <v>266.77999999999997</v>
+        <v>262.99</v>
       </c>
       <c r="E61" s="13">
-        <v>246.43</v>
+        <v>245.54</v>
       </c>
       <c r="F61" s="13" t="s">
         <v>18</v>
@@ -1760,52 +1760,52 @@
     </row>
     <row r="62" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A62" s="7">
-        <v>46288</v>
+        <v>46289</v>
       </c>
       <c r="B62" s="8"/>
       <c r="C62" s="20" t="s">
         <v>32</v>
       </c>
       <c r="D62" s="10">
-        <v>283.32</v>
+        <v>279.49</v>
       </c>
       <c r="E62" s="10">
-        <v>251.24</v>
+        <v>251.21</v>
       </c>
       <c r="F62" s="10">
-        <v>261.24</v>
+        <v>261.20999999999998</v>
       </c>
       <c r="G62" s="17"/>
     </row>
     <row r="63" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A63" s="11">
-        <v>46288</v>
+        <v>46289</v>
       </c>
       <c r="B63" s="12"/>
       <c r="C63" s="21" t="s">
         <v>33</v>
       </c>
       <c r="D63" s="13">
-        <v>272.32</v>
+        <v>268.51</v>
       </c>
       <c r="E63" s="13">
-        <v>238.38</v>
+        <v>238.11</v>
       </c>
       <c r="F63" s="13">
-        <v>248.38</v>
+        <v>248.11</v>
       </c>
       <c r="G63" s="17"/>
     </row>
     <row r="64" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A64" s="7">
-        <v>46288</v>
+        <v>46289</v>
       </c>
       <c r="B64" s="8"/>
       <c r="C64" s="20" t="s">
         <v>34</v>
       </c>
       <c r="D64" s="10">
-        <v>273.58</v>
+        <v>269.77999999999997</v>
       </c>
       <c r="E64" s="10" t="s">
         <v>18</v>
@@ -1817,17 +1817,17 @@
     </row>
     <row r="65" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A65" s="11">
-        <v>46288</v>
+        <v>46289</v>
       </c>
       <c r="B65" s="12"/>
       <c r="C65" s="21" t="s">
         <v>35</v>
       </c>
       <c r="D65" s="13">
-        <v>269.33</v>
+        <v>265.47000000000003</v>
       </c>
       <c r="E65" s="13">
-        <v>232.76</v>
+        <v>232.48</v>
       </c>
       <c r="F65" s="13" t="s">
         <v>18</v>
@@ -1835,35 +1835,35 @@
     </row>
     <row r="66" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A66" s="7">
-        <v>46288</v>
+        <v>46289</v>
       </c>
       <c r="B66" s="8"/>
       <c r="C66" s="20" t="s">
         <v>36</v>
       </c>
       <c r="D66" s="10">
-        <v>265.16000000000003</v>
+        <v>261.31</v>
       </c>
       <c r="E66" s="10">
-        <v>228.7</v>
+        <v>228.43</v>
       </c>
       <c r="F66" s="10">
-        <v>238.7</v>
+        <v>238.43</v>
       </c>
     </row>
     <row r="67" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A67" s="11">
-        <v>46288</v>
+        <v>46289</v>
       </c>
       <c r="B67" s="12"/>
       <c r="C67" s="21" t="s">
         <v>37</v>
       </c>
       <c r="D67" s="13">
-        <v>270.64</v>
+        <v>266.77999999999997</v>
       </c>
       <c r="E67" s="13">
-        <v>246.55</v>
+        <v>246.43</v>
       </c>
       <c r="F67" s="13" t="s">
         <v>18</v>
@@ -1902,6 +1902,15 @@
 </file>
 
 <file path=customXml/item2.xml><?xml version="1.0" encoding="utf-8"?>
+<?mso-contentType ?>
+<FormTemplates xmlns="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms">
+  <Display>DocumentLibraryForm</Display>
+  <Edit>DocumentLibraryForm</Edit>
+  <New>DocumentLibraryForm</New>
+</FormTemplates>
+</file>
+
+<file path=customXml/item3.xml><?xml version="1.0" encoding="utf-8"?>
 <ct:contentTypeSchema xmlns:ct="http://schemas.microsoft.com/office/2006/metadata/contentType" xmlns:ma="http://schemas.microsoft.com/office/2006/metadata/properties/metaAttributes" ct:_="" ma:_="" ma:contentTypeName="Document" ma:contentTypeID="0x010100D3632DF5622958439304627C030B0427" ma:contentTypeVersion="18" ma:contentTypeDescription="Create a new document." ma:contentTypeScope="" ma:versionID="8c2ecbce386d6bac497f8eb2d8f0fb7a">
   <xsd:schema xmlns:xsd="http://www.w3.org/2001/XMLSchema" xmlns:xs="http://www.w3.org/2001/XMLSchema" xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:ns2="87276d81-85f4-4ef2-9e6e-55066304288f" xmlns:ns3="39e1dda6-d1d8-4c88-a3b9-f1abc1284bad" xmlns:ns4="b23b8984-eafa-4e79-985e-54f52f3da58e" targetNamespace="http://schemas.microsoft.com/office/2006/metadata/properties" ma:root="true" ma:fieldsID="4cfd0c2f651c1ce156ad4fcb44ea61dd" ns2:_="" ns3:_="" ns4:_="">
     <xsd:import namespace="87276d81-85f4-4ef2-9e6e-55066304288f"/>
@@ -2161,15 +2170,6 @@
 </ct:contentTypeSchema>
 </file>
 
-<file path=customXml/item3.xml><?xml version="1.0" encoding="utf-8"?>
-<?mso-contentType ?>
-<FormTemplates xmlns="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms">
-  <Display>DocumentLibraryForm</Display>
-  <Edit>DocumentLibraryForm</Edit>
-  <New>DocumentLibraryForm</New>
-</FormTemplates>
-</file>
-
 <file path=customXml/itemProps1.xml><?xml version="1.0" encoding="utf-8"?>
 <ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{57A83D98-2BAE-4D83-823A-D31C464B620C}">
   <ds:schemaRefs>
@@ -2182,6 +2182,14 @@
 </file>
 
 <file path=customXml/itemProps2.xml><?xml version="1.0" encoding="utf-8"?>
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{F60519E9-FD90-4339-869C-BC2F85719BB8}">
+  <ds:schemaRefs>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms"/>
+  </ds:schemaRefs>
+</ds:datastoreItem>
+</file>
+
+<file path=customXml/itemProps3.xml><?xml version="1.0" encoding="utf-8"?>
 <ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{B44E1863-2778-41F9-ACBA-48420F931671}">
   <ds:schemaRefs>
     <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/contentType"/>
@@ -2201,14 +2209,6 @@
 </ds:datastoreItem>
 </file>
 
-<file path=customXml/itemProps3.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{F60519E9-FD90-4339-869C-BC2F85719BB8}">
-  <ds:schemaRefs>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms"/>
-  </ds:schemaRefs>
-</ds:datastoreItem>
-</file>
-
 <file path=docMetadata/LabelInfo.xml><?xml version="1.0" encoding="utf-8"?>
 <clbl:labelList xmlns:clbl="http://schemas.microsoft.com/office/2020/mipLabelMetadata">
   <clbl:label id="{569bf4a9-87bd-4dbf-a36c-1db5158e5def}" enabled="1" method="Privileged" siteId="{ea80952e-a476-42d4-aaf4-5457852b0f7e}" removed="0"/>

</xml_diff>

<commit_message>
Fri Sep 25 06:12:18 UTC 2026
</commit_message>
<xml_diff>
--- a/bp.com-content-dam-bp-country-sites-en_au-australia-home-products-services-pricing-tgp-excel.xlsx
+++ b/bp.com-content-dam-bp-country-sites-en_au-australia-home-products-services-pricing-tgp-excel.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://bp365.sharepoint.com/sites/WholesalePricing/Shared Documents/B2C/TGP/Daily TGP/Web TGP/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="14_{34A09CBA-7C4D-4EF2-9C47-AA9809C45408}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="14_{88A4DA0F-68E9-4B21-9911-0DDFD8E7A97A}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-28920" yWindow="-60" windowWidth="29040" windowHeight="15720" xr2:uid="{1B412EEF-F96D-4DF4-A4E9-C7F0F183C2FB}"/>
+    <workbookView xWindow="-110" yWindow="-110" windowWidth="19420" windowHeight="11500" xr2:uid="{1B412EEF-F96D-4DF4-A4E9-C7F0F183C2FB}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
@@ -808,128 +808,128 @@
     </row>
     <row r="8" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A8" s="7">
-        <v>46290</v>
+        <v>46291</v>
       </c>
       <c r="B8" s="8"/>
       <c r="C8" s="9" t="s">
         <v>10</v>
       </c>
       <c r="D8" s="10">
-        <v>266.55</v>
+        <v>265</v>
       </c>
       <c r="E8" s="10">
-        <v>233.88</v>
+        <v>231.06</v>
       </c>
       <c r="F8" s="10">
-        <v>243.88</v>
+        <v>241.06</v>
       </c>
       <c r="G8" s="10">
-        <v>233.85</v>
+        <v>231.02</v>
       </c>
     </row>
     <row r="9" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A9" s="11">
-        <v>46290</v>
+        <v>46291</v>
       </c>
       <c r="B9" s="12"/>
       <c r="C9" s="12" t="s">
         <v>11</v>
       </c>
       <c r="D9" s="13">
-        <v>266.55</v>
+        <v>265</v>
       </c>
       <c r="E9" s="13">
-        <v>233.88</v>
+        <v>231.06</v>
       </c>
       <c r="F9" s="13">
-        <v>243.88</v>
+        <v>241.06</v>
       </c>
       <c r="G9" s="13">
-        <v>233.85</v>
+        <v>231.02</v>
       </c>
     </row>
     <row r="10" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A10" s="7">
-        <v>46290</v>
+        <v>46291</v>
       </c>
       <c r="B10" s="8"/>
       <c r="C10" s="9" t="s">
         <v>12</v>
       </c>
       <c r="D10" s="10">
-        <v>259.18</v>
+        <v>257.18</v>
       </c>
       <c r="E10" s="10">
-        <v>227.79</v>
+        <v>227.87</v>
       </c>
       <c r="F10" s="10">
-        <v>237.79</v>
+        <v>237.87</v>
       </c>
       <c r="G10" s="10">
-        <v>228.21</v>
+        <v>228.29</v>
       </c>
     </row>
     <row r="11" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A11" s="11">
-        <v>46289</v>
+        <v>46290</v>
       </c>
       <c r="B11" s="12"/>
       <c r="C11" s="12" t="s">
         <v>10</v>
       </c>
       <c r="D11" s="13">
-        <v>269.89</v>
+        <v>266.55</v>
       </c>
       <c r="E11" s="13">
-        <v>234.64</v>
+        <v>233.88</v>
       </c>
       <c r="F11" s="13">
-        <v>244.64</v>
+        <v>243.88</v>
       </c>
       <c r="G11" s="13">
-        <v>234.6</v>
+        <v>233.85</v>
       </c>
     </row>
     <row r="12" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A12" s="7">
-        <v>46289</v>
+        <v>46290</v>
       </c>
       <c r="B12" s="8"/>
       <c r="C12" s="9" t="s">
         <v>11</v>
       </c>
       <c r="D12" s="10">
-        <v>269.89</v>
+        <v>266.55</v>
       </c>
       <c r="E12" s="10">
-        <v>234.64</v>
+        <v>233.88</v>
       </c>
       <c r="F12" s="10">
-        <v>244.64</v>
+        <v>243.88</v>
       </c>
       <c r="G12" s="10">
-        <v>234.6</v>
+        <v>233.85</v>
       </c>
     </row>
     <row r="13" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A13" s="11">
-        <v>46289</v>
+        <v>46290</v>
       </c>
       <c r="B13" s="12"/>
       <c r="C13" s="12" t="s">
         <v>12</v>
       </c>
       <c r="D13" s="13">
-        <v>262.87</v>
+        <v>259.18</v>
       </c>
       <c r="E13" s="13">
-        <v>228.86</v>
+        <v>227.79</v>
       </c>
       <c r="F13" s="13">
-        <v>238.86</v>
+        <v>237.79</v>
       </c>
       <c r="G13" s="13">
-        <v>229.27</v>
+        <v>228.21</v>
       </c>
     </row>
     <row r="14" spans="1:7" x14ac:dyDescent="0.25">
@@ -973,39 +973,39 @@
     </row>
     <row r="17" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A17" s="7">
-        <v>46290</v>
+        <v>46291</v>
       </c>
       <c r="B17" s="8"/>
       <c r="C17" s="20" t="s">
         <v>14</v>
       </c>
       <c r="D17" s="10">
-        <v>263.62</v>
+        <v>261.56</v>
       </c>
       <c r="E17" s="10">
-        <v>231.63</v>
+        <v>231.65</v>
       </c>
       <c r="F17" s="10">
-        <v>241.63</v>
+        <v>241.65</v>
       </c>
       <c r="G17" s="17"/>
     </row>
     <row r="18" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A18" s="11">
-        <v>46289</v>
+        <v>46290</v>
       </c>
       <c r="B18" s="12"/>
       <c r="C18" s="12" t="s">
         <v>14</v>
       </c>
       <c r="D18" s="13">
-        <v>267.39</v>
+        <v>263.62</v>
       </c>
       <c r="E18" s="13">
-        <v>232.76</v>
+        <v>231.63</v>
       </c>
       <c r="F18" s="13">
-        <v>242.76</v>
+        <v>241.63</v>
       </c>
       <c r="G18" s="17"/>
     </row>
@@ -1052,41 +1052,41 @@
     </row>
     <row r="22" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A22" s="7">
-        <v>46290</v>
+        <v>46291</v>
       </c>
       <c r="B22" s="8"/>
       <c r="C22" s="20" t="s">
         <v>16</v>
       </c>
       <c r="D22" s="10">
-        <v>267.12</v>
+        <v>265.57</v>
       </c>
       <c r="E22" s="10">
-        <v>231.83</v>
+        <v>229.77</v>
       </c>
       <c r="F22" s="10">
-        <v>241.43</v>
+        <v>239.37</v>
       </c>
       <c r="G22" s="10">
-        <v>230.54</v>
+        <v>228.49</v>
       </c>
     </row>
     <row r="23" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A23" s="11">
-        <v>46290</v>
+        <v>46291</v>
       </c>
       <c r="B23" s="12"/>
       <c r="C23" s="21" t="s">
         <v>17</v>
       </c>
       <c r="D23" s="13">
-        <v>264.02</v>
+        <v>262.02999999999997</v>
       </c>
       <c r="E23" s="13">
-        <v>235.7</v>
+        <v>235.8</v>
       </c>
       <c r="F23" s="13">
-        <v>245.7</v>
+        <v>245.8</v>
       </c>
       <c r="G23" s="13" t="s">
         <v>18</v>
@@ -1094,20 +1094,20 @@
     </row>
     <row r="24" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A24" s="7">
-        <v>46290</v>
+        <v>46291</v>
       </c>
       <c r="B24" s="8"/>
       <c r="C24" s="20" t="s">
         <v>19</v>
       </c>
       <c r="D24" s="10">
-        <v>264.48</v>
+        <v>262.48</v>
       </c>
       <c r="E24" s="10">
-        <v>234.95</v>
+        <v>235.06</v>
       </c>
       <c r="F24" s="10">
-        <v>244.95</v>
+        <v>245.06</v>
       </c>
       <c r="G24" s="10" t="s">
         <v>18</v>
@@ -1115,41 +1115,41 @@
     </row>
     <row r="25" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A25" s="11">
-        <v>46290</v>
+        <v>46291</v>
       </c>
       <c r="B25" s="12"/>
       <c r="C25" s="21" t="s">
         <v>20</v>
       </c>
       <c r="D25" s="13">
-        <v>261.22000000000003</v>
+        <v>259.20999999999998</v>
       </c>
       <c r="E25" s="13">
-        <v>235.07</v>
+        <v>235.18</v>
       </c>
       <c r="F25" s="13">
-        <v>245.07</v>
+        <v>245.18</v>
       </c>
       <c r="G25" s="13">
-        <v>232.97</v>
+        <v>233.08</v>
       </c>
     </row>
     <row r="26" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A26" s="7">
-        <v>46290</v>
+        <v>46291</v>
       </c>
       <c r="B26" s="8"/>
       <c r="C26" s="20" t="s">
         <v>21</v>
       </c>
       <c r="D26" s="10">
-        <v>262.94</v>
+        <v>260.93</v>
       </c>
       <c r="E26" s="10">
-        <v>236.55</v>
+        <v>236.66</v>
       </c>
       <c r="F26" s="10">
-        <v>246.55</v>
+        <v>246.66</v>
       </c>
       <c r="G26" s="10" t="s">
         <v>18</v>
@@ -1157,41 +1157,41 @@
     </row>
     <row r="27" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A27" s="11">
-        <v>46289</v>
+        <v>46290</v>
       </c>
       <c r="B27" s="12"/>
       <c r="C27" s="12" t="s">
         <v>16</v>
       </c>
       <c r="D27" s="13">
-        <v>269.91000000000003</v>
+        <v>267.12</v>
       </c>
       <c r="E27" s="13">
-        <v>233.68</v>
+        <v>231.83</v>
       </c>
       <c r="F27" s="13">
-        <v>243.28</v>
+        <v>241.43</v>
       </c>
       <c r="G27" s="13">
-        <v>232.39</v>
+        <v>230.54</v>
       </c>
     </row>
     <row r="28" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A28" s="7">
-        <v>46289</v>
+        <v>46290</v>
       </c>
       <c r="B28" s="8"/>
       <c r="C28" s="20" t="s">
         <v>17</v>
       </c>
       <c r="D28" s="10">
-        <v>267.7</v>
+        <v>264.02</v>
       </c>
       <c r="E28" s="22">
-        <v>236.74</v>
+        <v>235.7</v>
       </c>
       <c r="F28" s="22">
-        <v>246.74</v>
+        <v>245.7</v>
       </c>
       <c r="G28" s="22" t="s">
         <v>18</v>
@@ -1199,20 +1199,20 @@
     </row>
     <row r="29" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A29" s="11">
-        <v>46289</v>
+        <v>46290</v>
       </c>
       <c r="B29" s="12"/>
       <c r="C29" s="12" t="s">
         <v>19</v>
       </c>
       <c r="D29" s="13">
-        <v>268.18</v>
+        <v>264.48</v>
       </c>
       <c r="E29" s="13">
-        <v>235.99</v>
+        <v>234.95</v>
       </c>
       <c r="F29" s="13">
-        <v>245.99</v>
+        <v>244.95</v>
       </c>
       <c r="G29" s="13" t="s">
         <v>18</v>
@@ -1220,41 +1220,41 @@
     </row>
     <row r="30" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A30" s="7">
-        <v>46289</v>
+        <v>46290</v>
       </c>
       <c r="B30" s="8"/>
       <c r="C30" s="20" t="s">
         <v>20</v>
       </c>
       <c r="D30" s="10">
-        <v>264.91000000000003</v>
+        <v>261.22000000000003</v>
       </c>
       <c r="E30" s="22">
-        <v>236.11</v>
+        <v>235.07</v>
       </c>
       <c r="F30" s="22">
-        <v>246.11</v>
+        <v>245.07</v>
       </c>
       <c r="G30" s="22">
-        <v>234</v>
+        <v>232.97</v>
       </c>
     </row>
     <row r="31" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A31" s="11">
-        <v>46289</v>
+        <v>46290</v>
       </c>
       <c r="B31" s="12"/>
       <c r="C31" s="12" t="s">
         <v>21</v>
       </c>
       <c r="D31" s="13">
-        <v>266.66000000000003</v>
+        <v>262.94</v>
       </c>
       <c r="E31" s="13">
-        <v>237.59</v>
+        <v>236.55</v>
       </c>
       <c r="F31" s="13">
-        <v>247.59</v>
+        <v>246.55</v>
       </c>
       <c r="G31" s="13" t="s">
         <v>18</v>
@@ -1301,52 +1301,52 @@
     </row>
     <row r="35" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A35" s="7">
-        <v>46290</v>
+        <v>46291</v>
       </c>
       <c r="B35" s="8"/>
       <c r="C35" s="20" t="s">
         <v>23</v>
       </c>
       <c r="D35" s="10">
-        <v>257.70999999999998</v>
+        <v>255.72</v>
       </c>
       <c r="E35" s="10">
-        <v>226.73</v>
+        <v>226.81</v>
       </c>
       <c r="F35" s="10">
-        <v>235.73</v>
+        <v>235.81</v>
       </c>
       <c r="G35" s="17"/>
     </row>
     <row r="36" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A36" s="11">
-        <v>46289</v>
+        <v>46290</v>
       </c>
       <c r="B36" s="12"/>
       <c r="C36" s="12" t="s">
         <v>23</v>
       </c>
       <c r="D36" s="13">
-        <v>261.39999999999998</v>
+        <v>257.70999999999998</v>
       </c>
       <c r="E36" s="13">
-        <v>227.79</v>
+        <v>226.73</v>
       </c>
       <c r="F36" s="13">
-        <v>236.79</v>
+        <v>235.73</v>
       </c>
       <c r="G36" s="17"/>
     </row>
     <row r="37" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A37" s="7">
-        <v>46290</v>
+        <v>46291</v>
       </c>
       <c r="B37" s="8"/>
       <c r="C37" s="20" t="s">
         <v>24</v>
       </c>
       <c r="D37" s="10">
-        <v>273.33</v>
+        <v>271.33999999999997</v>
       </c>
       <c r="E37" s="10" t="s">
         <v>18</v>
@@ -1358,14 +1358,14 @@
     </row>
     <row r="38" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A38" s="11">
-        <v>46289</v>
+        <v>46290</v>
       </c>
       <c r="B38" s="12"/>
       <c r="C38" s="12" t="s">
         <v>24</v>
       </c>
       <c r="D38" s="13">
-        <v>277.02</v>
+        <v>273.33</v>
       </c>
       <c r="E38" s="13" t="s">
         <v>18</v>
@@ -1416,77 +1416,77 @@
     </row>
     <row r="42" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A42" s="7">
-        <v>46290</v>
+        <v>46291</v>
       </c>
       <c r="B42" s="8"/>
       <c r="C42" s="20" t="s">
         <v>26</v>
       </c>
       <c r="D42" s="10">
-        <v>266.97000000000003</v>
+        <v>265.02</v>
       </c>
       <c r="E42" s="10">
-        <v>231.64</v>
+        <v>231.78</v>
       </c>
       <c r="F42" s="10">
-        <v>241.64</v>
+        <v>241.78</v>
       </c>
       <c r="G42" s="17"/>
     </row>
     <row r="43" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A43" s="11">
-        <v>46290</v>
+        <v>46291</v>
       </c>
       <c r="B43" s="12"/>
       <c r="C43" s="21" t="s">
         <v>27</v>
       </c>
       <c r="D43" s="13">
-        <v>266.58</v>
+        <v>264.63</v>
       </c>
       <c r="E43" s="13">
-        <v>232.05</v>
+        <v>232.19</v>
       </c>
       <c r="F43" s="13">
-        <v>242.05</v>
+        <v>242.19</v>
       </c>
       <c r="G43" s="17"/>
     </row>
     <row r="44" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A44" s="7">
-        <v>46289</v>
+        <v>46290</v>
       </c>
       <c r="B44" s="8"/>
       <c r="C44" s="20" t="s">
         <v>26</v>
       </c>
       <c r="D44" s="10">
-        <v>270.61</v>
+        <v>266.97000000000003</v>
       </c>
       <c r="E44" s="10">
-        <v>232.62</v>
+        <v>231.64</v>
       </c>
       <c r="F44" s="10">
-        <v>242.62</v>
+        <v>241.64</v>
       </c>
       <c r="G44" s="17"/>
     </row>
     <row r="45" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A45" s="11">
-        <v>46289</v>
+        <v>46290</v>
       </c>
       <c r="B45" s="12"/>
       <c r="C45" s="21" t="s">
         <v>27</v>
       </c>
       <c r="D45" s="13">
-        <v>270.22000000000003</v>
+        <v>266.58</v>
       </c>
       <c r="E45" s="13">
-        <v>233.03</v>
+        <v>232.05</v>
       </c>
       <c r="F45" s="13">
-        <v>243.03</v>
+        <v>242.05</v>
       </c>
       <c r="G45" s="17"/>
     </row>
@@ -1531,77 +1531,77 @@
     </row>
     <row r="49" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A49" s="7">
-        <v>46290</v>
+        <v>46291</v>
       </c>
       <c r="B49" s="8"/>
       <c r="C49" s="20" t="s">
         <v>29</v>
       </c>
       <c r="D49" s="10">
-        <v>263.64</v>
+        <v>262.01</v>
       </c>
       <c r="E49" s="10">
-        <v>228.59</v>
+        <v>229.06</v>
       </c>
       <c r="F49" s="10">
-        <v>238.59</v>
+        <v>239.06</v>
       </c>
       <c r="G49" s="28"/>
     </row>
     <row r="50" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A50" s="11">
-        <v>46290</v>
+        <v>46291</v>
       </c>
       <c r="B50" s="12"/>
       <c r="C50" s="21" t="s">
         <v>30</v>
       </c>
       <c r="D50" s="13">
-        <v>261.56</v>
+        <v>259.89999999999998</v>
       </c>
       <c r="E50" s="13">
-        <v>228.39</v>
+        <v>228.84</v>
       </c>
       <c r="F50" s="13">
-        <v>238.39</v>
+        <v>238.84</v>
       </c>
       <c r="G50" s="28"/>
     </row>
     <row r="51" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A51" s="7">
-        <v>46289</v>
+        <v>46290</v>
       </c>
       <c r="B51" s="8"/>
       <c r="C51" s="20" t="s">
         <v>29</v>
       </c>
       <c r="D51" s="10">
-        <v>265.43</v>
+        <v>263.64</v>
       </c>
       <c r="E51" s="10">
-        <v>228.67</v>
+        <v>228.59</v>
       </c>
       <c r="F51" s="10">
-        <v>238.67</v>
+        <v>238.59</v>
       </c>
       <c r="G51" s="17"/>
     </row>
     <row r="52" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A52" s="11">
-        <v>46289</v>
+        <v>46290</v>
       </c>
       <c r="B52" s="12"/>
       <c r="C52" s="21" t="s">
         <v>30</v>
       </c>
       <c r="D52" s="13">
-        <v>263.37</v>
+        <v>261.56</v>
       </c>
       <c r="E52" s="13">
-        <v>228.48</v>
+        <v>228.39</v>
       </c>
       <c r="F52" s="13">
-        <v>238.48</v>
+        <v>238.39</v>
       </c>
       <c r="G52" s="17"/>
     </row>
@@ -1646,52 +1646,52 @@
     </row>
     <row r="56" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A56" s="7">
-        <v>46290</v>
+        <v>46291</v>
       </c>
       <c r="B56" s="8"/>
       <c r="C56" s="20" t="s">
         <v>32</v>
       </c>
       <c r="D56" s="10">
-        <v>275.76</v>
+        <v>273.75</v>
       </c>
       <c r="E56" s="10">
-        <v>250.46</v>
+        <v>250.77</v>
       </c>
       <c r="F56" s="10">
-        <v>260.45999999999998</v>
+        <v>260.77</v>
       </c>
       <c r="G56" s="17"/>
     </row>
     <row r="57" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A57" s="11">
-        <v>46290</v>
+        <v>46291</v>
       </c>
       <c r="B57" s="12"/>
       <c r="C57" s="21" t="s">
         <v>33</v>
       </c>
       <c r="D57" s="13">
-        <v>264.82</v>
+        <v>262.83</v>
       </c>
       <c r="E57" s="13">
-        <v>236.97</v>
+        <v>236.99</v>
       </c>
       <c r="F57" s="13">
-        <v>246.97</v>
+        <v>246.99</v>
       </c>
       <c r="G57" s="17"/>
     </row>
     <row r="58" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A58" s="7">
-        <v>46290</v>
+        <v>46291</v>
       </c>
       <c r="B58" s="8"/>
       <c r="C58" s="20" t="s">
         <v>34</v>
       </c>
       <c r="D58" s="10">
-        <v>266.11</v>
+        <v>264.13</v>
       </c>
       <c r="E58" s="10" t="s">
         <v>18</v>
@@ -1703,17 +1703,17 @@
     </row>
     <row r="59" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A59" s="11">
-        <v>46290</v>
+        <v>46291</v>
       </c>
       <c r="B59" s="12"/>
       <c r="C59" s="21" t="s">
         <v>35</v>
       </c>
       <c r="D59" s="13">
-        <v>261.7</v>
+        <v>259.64</v>
       </c>
       <c r="E59" s="13">
-        <v>231.34</v>
+        <v>231.36</v>
       </c>
       <c r="F59" s="13" t="s">
         <v>18</v>
@@ -1722,36 +1722,36 @@
     </row>
     <row r="60" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A60" s="7">
-        <v>46290</v>
+        <v>46291</v>
       </c>
       <c r="B60" s="8"/>
       <c r="C60" s="20" t="s">
         <v>36</v>
       </c>
       <c r="D60" s="10">
-        <v>257.52999999999997</v>
+        <v>255.47</v>
       </c>
       <c r="E60" s="10">
-        <v>227.29</v>
+        <v>227.31</v>
       </c>
       <c r="F60" s="10">
-        <v>237.29</v>
+        <v>237.31</v>
       </c>
       <c r="G60" s="17"/>
     </row>
     <row r="61" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A61" s="11">
-        <v>46290</v>
+        <v>46291</v>
       </c>
       <c r="B61" s="12"/>
       <c r="C61" s="21" t="s">
         <v>37</v>
       </c>
       <c r="D61" s="13">
-        <v>262.99</v>
+        <v>260.92</v>
       </c>
       <c r="E61" s="13">
-        <v>245.54</v>
+        <v>245.76</v>
       </c>
       <c r="F61" s="13" t="s">
         <v>18</v>
@@ -1760,52 +1760,52 @@
     </row>
     <row r="62" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A62" s="7">
-        <v>46289</v>
+        <v>46290</v>
       </c>
       <c r="B62" s="8"/>
       <c r="C62" s="20" t="s">
         <v>32</v>
       </c>
       <c r="D62" s="10">
-        <v>279.49</v>
+        <v>275.76</v>
       </c>
       <c r="E62" s="10">
-        <v>251.21</v>
+        <v>250.46</v>
       </c>
       <c r="F62" s="10">
-        <v>261.20999999999998</v>
+        <v>260.45999999999998</v>
       </c>
       <c r="G62" s="17"/>
     </row>
     <row r="63" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A63" s="11">
-        <v>46289</v>
+        <v>46290</v>
       </c>
       <c r="B63" s="12"/>
       <c r="C63" s="21" t="s">
         <v>33</v>
       </c>
       <c r="D63" s="13">
-        <v>268.51</v>
+        <v>264.82</v>
       </c>
       <c r="E63" s="13">
-        <v>238.11</v>
+        <v>236.97</v>
       </c>
       <c r="F63" s="13">
-        <v>248.11</v>
+        <v>246.97</v>
       </c>
       <c r="G63" s="17"/>
     </row>
     <row r="64" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A64" s="7">
-        <v>46289</v>
+        <v>46290</v>
       </c>
       <c r="B64" s="8"/>
       <c r="C64" s="20" t="s">
         <v>34</v>
       </c>
       <c r="D64" s="10">
-        <v>269.77999999999997</v>
+        <v>266.11</v>
       </c>
       <c r="E64" s="10" t="s">
         <v>18</v>
@@ -1817,17 +1817,17 @@
     </row>
     <row r="65" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A65" s="11">
-        <v>46289</v>
+        <v>46290</v>
       </c>
       <c r="B65" s="12"/>
       <c r="C65" s="21" t="s">
         <v>35</v>
       </c>
       <c r="D65" s="13">
-        <v>265.47000000000003</v>
+        <v>261.7</v>
       </c>
       <c r="E65" s="13">
-        <v>232.48</v>
+        <v>231.34</v>
       </c>
       <c r="F65" s="13" t="s">
         <v>18</v>
@@ -1835,35 +1835,35 @@
     </row>
     <row r="66" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A66" s="7">
-        <v>46289</v>
+        <v>46290</v>
       </c>
       <c r="B66" s="8"/>
       <c r="C66" s="20" t="s">
         <v>36</v>
       </c>
       <c r="D66" s="10">
-        <v>261.31</v>
+        <v>257.52999999999997</v>
       </c>
       <c r="E66" s="10">
-        <v>228.43</v>
+        <v>227.29</v>
       </c>
       <c r="F66" s="10">
-        <v>238.43</v>
+        <v>237.29</v>
       </c>
     </row>
     <row r="67" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A67" s="11">
-        <v>46289</v>
+        <v>46290</v>
       </c>
       <c r="B67" s="12"/>
       <c r="C67" s="21" t="s">
         <v>37</v>
       </c>
       <c r="D67" s="13">
-        <v>266.77999999999997</v>
+        <v>262.99</v>
       </c>
       <c r="E67" s="13">
-        <v>246.43</v>
+        <v>245.54</v>
       </c>
       <c r="F67" s="13" t="s">
         <v>18</v>
@@ -1891,6 +1891,15 @@
 </file>
 
 <file path=customXml/item1.xml><?xml version="1.0" encoding="utf-8"?>
+<?mso-contentType ?>
+<FormTemplates xmlns="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms">
+  <Display>DocumentLibraryForm</Display>
+  <Edit>DocumentLibraryForm</Edit>
+  <New>DocumentLibraryForm</New>
+</FormTemplates>
+</file>
+
+<file path=customXml/item2.xml><?xml version="1.0" encoding="utf-8"?>
 <p:properties xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls">
   <documentManagement>
     <lcf76f155ced4ddcb4097134ff3c332f xmlns="87276d81-85f4-4ef2-9e6e-55066304288f">
@@ -1899,15 +1908,6 @@
     <TaxCatchAll xmlns="b23b8984-eafa-4e79-985e-54f52f3da58e" xsi:nil="true"/>
   </documentManagement>
 </p:properties>
-</file>
-
-<file path=customXml/item2.xml><?xml version="1.0" encoding="utf-8"?>
-<?mso-contentType ?>
-<FormTemplates xmlns="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms">
-  <Display>DocumentLibraryForm</Display>
-  <Edit>DocumentLibraryForm</Edit>
-  <New>DocumentLibraryForm</New>
-</FormTemplates>
 </file>
 
 <file path=customXml/item3.xml><?xml version="1.0" encoding="utf-8"?>
@@ -2171,20 +2171,20 @@
 </file>
 
 <file path=customXml/itemProps1.xml><?xml version="1.0" encoding="utf-8"?>
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{F60519E9-FD90-4339-869C-BC2F85719BB8}">
+  <ds:schemaRefs>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms"/>
+  </ds:schemaRefs>
+</ds:datastoreItem>
+</file>
+
+<file path=customXml/itemProps2.xml><?xml version="1.0" encoding="utf-8"?>
 <ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{57A83D98-2BAE-4D83-823A-D31C464B620C}">
   <ds:schemaRefs>
     <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/properties"/>
     <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
     <ds:schemaRef ds:uri="87276d81-85f4-4ef2-9e6e-55066304288f"/>
     <ds:schemaRef ds:uri="b23b8984-eafa-4e79-985e-54f52f3da58e"/>
-  </ds:schemaRefs>
-</ds:datastoreItem>
-</file>
-
-<file path=customXml/itemProps2.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{F60519E9-FD90-4339-869C-BC2F85719BB8}">
-  <ds:schemaRefs>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms"/>
   </ds:schemaRefs>
 </ds:datastoreItem>
 </file>

</xml_diff>

<commit_message>
Mon Sep 28 07:04:18 UTC 2026
</commit_message>
<xml_diff>
--- a/bp.com-content-dam-bp-country-sites-en_au-australia-home-products-services-pricing-tgp-excel.xlsx
+++ b/bp.com-content-dam-bp-country-sites-en_au-australia-home-products-services-pricing-tgp-excel.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://bp365.sharepoint.com/sites/WholesalePricing/Shared Documents/B2C/TGP/Daily TGP/Web TGP/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="14_{88A4DA0F-68E9-4B21-9911-0DDFD8E7A97A}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="14_{4C1D3E27-72AB-4068-BADA-1BAD2E0663D8}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-110" yWindow="-110" windowWidth="19420" windowHeight="11500" xr2:uid="{1B412EEF-F96D-4DF4-A4E9-C7F0F183C2FB}"/>
   </bookViews>
@@ -715,15 +715,15 @@
     <pageSetUpPr fitToPage="1"/>
   </sheetPr>
   <dimension ref="A1:G67"/>
-  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
   <cols>
-    <col min="1" max="1" width="76.42578125" bestFit="1" customWidth="1"/>
-    <col min="2" max="2" width="6.42578125"/>
-    <col min="3" max="3" width="18.140625" bestFit="1" customWidth="1"/>
-    <col min="4" max="7" width="7.140625" bestFit="1" customWidth="1"/>
+    <col min="1" max="1" width="76.453125" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="6.453125"/>
+    <col min="3" max="3" width="18.1796875" bestFit="1" customWidth="1"/>
+    <col min="4" max="7" width="7.1796875" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:7" ht="23.25" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:7" ht="22.5" x14ac:dyDescent="0.35">
       <c r="A1" s="30" t="s">
         <v>0</v>
       </c>
@@ -734,7 +734,7 @@
       <c r="F1" s="2"/>
       <c r="G1" s="2"/>
     </row>
-    <row r="2" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="2" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A2" s="3"/>
       <c r="B2" s="1"/>
       <c r="C2" s="1"/>
@@ -743,7 +743,7 @@
       <c r="F2" s="2"/>
       <c r="G2" s="2"/>
     </row>
-    <row r="3" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="3" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A3" s="3" t="s">
         <v>1</v>
       </c>
@@ -754,7 +754,7 @@
       <c r="F3" s="2"/>
       <c r="G3" s="2"/>
     </row>
-    <row r="4" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="4" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A4" s="3" t="s">
         <v>2</v>
       </c>
@@ -765,7 +765,7 @@
       <c r="F4" s="2"/>
       <c r="G4" s="2"/>
     </row>
-    <row r="5" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="5" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A5" s="3"/>
       <c r="B5" s="3"/>
       <c r="C5" s="1"/>
@@ -774,7 +774,7 @@
       <c r="F5" s="2"/>
       <c r="G5" s="2"/>
     </row>
-    <row r="6" spans="1:7" ht="20.25" x14ac:dyDescent="0.25">
+    <row r="6" spans="1:7" ht="20" x14ac:dyDescent="0.35">
       <c r="A6" s="29" t="s">
         <v>3</v>
       </c>
@@ -785,7 +785,7 @@
       <c r="F6" s="2"/>
       <c r="G6" s="2"/>
     </row>
-    <row r="7" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="7" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A7" s="4" t="s">
         <v>4</v>
       </c>
@@ -806,133 +806,133 @@
         <v>9</v>
       </c>
     </row>
-    <row r="8" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="8" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A8" s="7">
-        <v>46291</v>
+        <v>46294</v>
       </c>
       <c r="B8" s="8"/>
       <c r="C8" s="9" t="s">
         <v>10</v>
       </c>
       <c r="D8" s="10">
-        <v>265</v>
+        <v>264.13</v>
       </c>
       <c r="E8" s="10">
-        <v>231.06</v>
+        <v>228.23</v>
       </c>
       <c r="F8" s="10">
-        <v>241.06</v>
+        <v>238.23</v>
       </c>
       <c r="G8" s="10">
-        <v>231.02</v>
-      </c>
-    </row>
-    <row r="9" spans="1:7" x14ac:dyDescent="0.25">
+        <v>228.19</v>
+      </c>
+    </row>
+    <row r="9" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A9" s="11">
-        <v>46291</v>
+        <v>46294</v>
       </c>
       <c r="B9" s="12"/>
       <c r="C9" s="12" t="s">
         <v>11</v>
       </c>
       <c r="D9" s="13">
-        <v>265</v>
+        <v>264.13</v>
       </c>
       <c r="E9" s="13">
-        <v>231.06</v>
+        <v>228.23</v>
       </c>
       <c r="F9" s="13">
-        <v>241.06</v>
+        <v>238.23</v>
       </c>
       <c r="G9" s="13">
-        <v>231.02</v>
-      </c>
-    </row>
-    <row r="10" spans="1:7" x14ac:dyDescent="0.25">
+        <v>228.19</v>
+      </c>
+    </row>
+    <row r="10" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A10" s="7">
-        <v>46291</v>
+        <v>46294</v>
       </c>
       <c r="B10" s="8"/>
       <c r="C10" s="9" t="s">
         <v>12</v>
       </c>
       <c r="D10" s="10">
-        <v>257.18</v>
+        <v>256.04000000000002</v>
       </c>
       <c r="E10" s="10">
-        <v>227.87</v>
+        <v>225.91</v>
       </c>
       <c r="F10" s="10">
-        <v>237.87</v>
+        <v>235.91</v>
       </c>
       <c r="G10" s="10">
-        <v>228.29</v>
-      </c>
-    </row>
-    <row r="11" spans="1:7" x14ac:dyDescent="0.25">
+        <v>226.32</v>
+      </c>
+    </row>
+    <row r="11" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A11" s="11">
-        <v>46290</v>
+        <v>46291</v>
       </c>
       <c r="B11" s="12"/>
       <c r="C11" s="12" t="s">
         <v>10</v>
       </c>
       <c r="D11" s="13">
-        <v>266.55</v>
+        <v>265</v>
       </c>
       <c r="E11" s="13">
-        <v>233.88</v>
+        <v>231.06</v>
       </c>
       <c r="F11" s="13">
-        <v>243.88</v>
+        <v>241.06</v>
       </c>
       <c r="G11" s="13">
-        <v>233.85</v>
-      </c>
-    </row>
-    <row r="12" spans="1:7" x14ac:dyDescent="0.25">
+        <v>231.02</v>
+      </c>
+    </row>
+    <row r="12" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A12" s="7">
-        <v>46290</v>
+        <v>46291</v>
       </c>
       <c r="B12" s="8"/>
       <c r="C12" s="9" t="s">
         <v>11</v>
       </c>
       <c r="D12" s="10">
-        <v>266.55</v>
+        <v>265</v>
       </c>
       <c r="E12" s="10">
-        <v>233.88</v>
+        <v>231.06</v>
       </c>
       <c r="F12" s="10">
-        <v>243.88</v>
+        <v>241.06</v>
       </c>
       <c r="G12" s="10">
-        <v>233.85</v>
-      </c>
-    </row>
-    <row r="13" spans="1:7" x14ac:dyDescent="0.25">
+        <v>231.02</v>
+      </c>
+    </row>
+    <row r="13" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A13" s="11">
-        <v>46290</v>
+        <v>46291</v>
       </c>
       <c r="B13" s="12"/>
       <c r="C13" s="12" t="s">
         <v>12</v>
       </c>
       <c r="D13" s="13">
-        <v>259.18</v>
+        <v>257.18</v>
       </c>
       <c r="E13" s="13">
-        <v>227.79</v>
+        <v>227.87</v>
       </c>
       <c r="F13" s="13">
-        <v>237.79</v>
+        <v>237.87</v>
       </c>
       <c r="G13" s="13">
-        <v>228.21</v>
-      </c>
-    </row>
-    <row r="14" spans="1:7" x14ac:dyDescent="0.25">
+        <v>228.29</v>
+      </c>
+    </row>
+    <row r="14" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A14" s="14"/>
       <c r="B14" s="14"/>
       <c r="C14" s="15"/>
@@ -941,7 +941,7 @@
       <c r="F14" s="16"/>
       <c r="G14" s="16"/>
     </row>
-    <row r="15" spans="1:7" ht="20.25" x14ac:dyDescent="0.25">
+    <row r="15" spans="1:7" ht="20" x14ac:dyDescent="0.35">
       <c r="A15" s="29" t="s">
         <v>13</v>
       </c>
@@ -952,7 +952,7 @@
       <c r="F15" s="17"/>
       <c r="G15" s="17"/>
     </row>
-    <row r="16" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="16" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A16" s="4" t="s">
         <v>4</v>
       </c>
@@ -971,45 +971,45 @@
       </c>
       <c r="G16" s="17"/>
     </row>
-    <row r="17" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="17" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A17" s="7">
-        <v>46291</v>
+        <v>46294</v>
       </c>
       <c r="B17" s="8"/>
       <c r="C17" s="20" t="s">
         <v>14</v>
       </c>
       <c r="D17" s="10">
-        <v>261.56</v>
+        <v>260.33</v>
       </c>
       <c r="E17" s="10">
-        <v>231.65</v>
+        <v>231.8</v>
       </c>
       <c r="F17" s="10">
-        <v>241.65</v>
+        <v>241.8</v>
       </c>
       <c r="G17" s="17"/>
     </row>
-    <row r="18" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="18" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A18" s="11">
-        <v>46290</v>
+        <v>46291</v>
       </c>
       <c r="B18" s="12"/>
       <c r="C18" s="12" t="s">
         <v>14</v>
       </c>
       <c r="D18" s="13">
-        <v>263.62</v>
+        <v>261.56</v>
       </c>
       <c r="E18" s="13">
-        <v>231.63</v>
+        <v>231.65</v>
       </c>
       <c r="F18" s="13">
-        <v>241.63</v>
+        <v>241.65</v>
       </c>
       <c r="G18" s="17"/>
     </row>
-    <row r="19" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="19" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A19" s="14"/>
       <c r="B19" s="14"/>
       <c r="C19" s="15"/>
@@ -1018,7 +1018,7 @@
       <c r="F19" s="16"/>
       <c r="G19" s="17"/>
     </row>
-    <row r="20" spans="1:7" ht="20.25" x14ac:dyDescent="0.25">
+    <row r="20" spans="1:7" ht="20" x14ac:dyDescent="0.35">
       <c r="A20" s="29" t="s">
         <v>15</v>
       </c>
@@ -1029,7 +1029,7 @@
       <c r="F20" s="17"/>
       <c r="G20" s="17"/>
     </row>
-    <row r="21" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="21" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A21" s="4" t="s">
         <v>4</v>
       </c>
@@ -1050,217 +1050,217 @@
         <v>9</v>
       </c>
     </row>
-    <row r="22" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="22" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A22" s="7">
-        <v>46291</v>
+        <v>46294</v>
       </c>
       <c r="B22" s="8"/>
       <c r="C22" s="20" t="s">
         <v>16</v>
       </c>
       <c r="D22" s="10">
-        <v>265.57</v>
+        <v>264.7</v>
       </c>
       <c r="E22" s="10">
-        <v>229.77</v>
+        <v>227.82</v>
       </c>
       <c r="F22" s="10">
-        <v>239.37</v>
+        <v>237.42</v>
       </c>
       <c r="G22" s="10">
-        <v>228.49</v>
-      </c>
-    </row>
-    <row r="23" spans="1:7" x14ac:dyDescent="0.25">
+        <v>226.54</v>
+      </c>
+    </row>
+    <row r="23" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A23" s="11">
-        <v>46291</v>
+        <v>46294</v>
       </c>
       <c r="B23" s="12"/>
       <c r="C23" s="21" t="s">
         <v>17</v>
       </c>
       <c r="D23" s="13">
-        <v>262.02999999999997</v>
+        <v>260.89999999999998</v>
       </c>
       <c r="E23" s="13">
-        <v>235.8</v>
+        <v>236.07</v>
       </c>
       <c r="F23" s="13">
-        <v>245.8</v>
+        <v>246.07</v>
       </c>
       <c r="G23" s="13" t="s">
         <v>18</v>
       </c>
     </row>
-    <row r="24" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="24" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A24" s="7">
-        <v>46291</v>
+        <v>46294</v>
       </c>
       <c r="B24" s="8"/>
       <c r="C24" s="20" t="s">
         <v>19</v>
       </c>
       <c r="D24" s="10">
-        <v>262.48</v>
+        <v>261.35000000000002</v>
       </c>
       <c r="E24" s="10">
-        <v>235.06</v>
+        <v>235.33</v>
       </c>
       <c r="F24" s="10">
-        <v>245.06</v>
+        <v>245.33</v>
       </c>
       <c r="G24" s="10" t="s">
         <v>18</v>
       </c>
     </row>
-    <row r="25" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="25" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A25" s="11">
-        <v>46291</v>
+        <v>46294</v>
       </c>
       <c r="B25" s="12"/>
       <c r="C25" s="21" t="s">
         <v>20</v>
       </c>
       <c r="D25" s="13">
-        <v>259.20999999999998</v>
+        <v>258.07</v>
       </c>
       <c r="E25" s="13">
-        <v>235.18</v>
+        <v>235.46</v>
       </c>
       <c r="F25" s="13">
-        <v>245.18</v>
+        <v>245.46</v>
       </c>
       <c r="G25" s="13">
-        <v>233.08</v>
-      </c>
-    </row>
-    <row r="26" spans="1:7" x14ac:dyDescent="0.25">
+        <v>233.36</v>
+      </c>
+    </row>
+    <row r="26" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A26" s="7">
-        <v>46291</v>
+        <v>46294</v>
       </c>
       <c r="B26" s="8"/>
       <c r="C26" s="20" t="s">
         <v>21</v>
       </c>
       <c r="D26" s="10">
-        <v>260.93</v>
+        <v>259.77</v>
       </c>
       <c r="E26" s="10">
-        <v>236.66</v>
+        <v>236.94</v>
       </c>
       <c r="F26" s="10">
-        <v>246.66</v>
+        <v>246.94</v>
       </c>
       <c r="G26" s="10" t="s">
         <v>18</v>
       </c>
     </row>
-    <row r="27" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="27" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A27" s="11">
-        <v>46290</v>
+        <v>46291</v>
       </c>
       <c r="B27" s="12"/>
       <c r="C27" s="12" t="s">
         <v>16</v>
       </c>
       <c r="D27" s="13">
-        <v>267.12</v>
+        <v>265.57</v>
       </c>
       <c r="E27" s="13">
-        <v>231.83</v>
+        <v>229.77</v>
       </c>
       <c r="F27" s="13">
-        <v>241.43</v>
+        <v>239.37</v>
       </c>
       <c r="G27" s="13">
-        <v>230.54</v>
-      </c>
-    </row>
-    <row r="28" spans="1:7" x14ac:dyDescent="0.25">
+        <v>228.49</v>
+      </c>
+    </row>
+    <row r="28" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A28" s="7">
-        <v>46290</v>
+        <v>46291</v>
       </c>
       <c r="B28" s="8"/>
       <c r="C28" s="20" t="s">
         <v>17</v>
       </c>
       <c r="D28" s="10">
-        <v>264.02</v>
+        <v>262.02999999999997</v>
       </c>
       <c r="E28" s="22">
-        <v>235.7</v>
+        <v>235.8</v>
       </c>
       <c r="F28" s="22">
-        <v>245.7</v>
+        <v>245.8</v>
       </c>
       <c r="G28" s="22" t="s">
         <v>18</v>
       </c>
     </row>
-    <row r="29" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="29" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A29" s="11">
-        <v>46290</v>
+        <v>46291</v>
       </c>
       <c r="B29" s="12"/>
       <c r="C29" s="12" t="s">
         <v>19</v>
       </c>
       <c r="D29" s="13">
-        <v>264.48</v>
+        <v>262.48</v>
       </c>
       <c r="E29" s="13">
-        <v>234.95</v>
+        <v>235.06</v>
       </c>
       <c r="F29" s="13">
-        <v>244.95</v>
+        <v>245.06</v>
       </c>
       <c r="G29" s="13" t="s">
         <v>18</v>
       </c>
     </row>
-    <row r="30" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="30" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A30" s="7">
-        <v>46290</v>
+        <v>46291</v>
       </c>
       <c r="B30" s="8"/>
       <c r="C30" s="20" t="s">
         <v>20</v>
       </c>
       <c r="D30" s="10">
-        <v>261.22000000000003</v>
+        <v>259.20999999999998</v>
       </c>
       <c r="E30" s="22">
-        <v>235.07</v>
+        <v>235.18</v>
       </c>
       <c r="F30" s="22">
-        <v>245.07</v>
+        <v>245.18</v>
       </c>
       <c r="G30" s="22">
-        <v>232.97</v>
-      </c>
-    </row>
-    <row r="31" spans="1:7" x14ac:dyDescent="0.25">
+        <v>233.08</v>
+      </c>
+    </row>
+    <row r="31" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A31" s="11">
-        <v>46290</v>
+        <v>46291</v>
       </c>
       <c r="B31" s="12"/>
       <c r="C31" s="12" t="s">
         <v>21</v>
       </c>
       <c r="D31" s="13">
-        <v>262.94</v>
+        <v>260.93</v>
       </c>
       <c r="E31" s="13">
-        <v>236.55</v>
+        <v>236.66</v>
       </c>
       <c r="F31" s="13">
-        <v>246.55</v>
+        <v>246.66</v>
       </c>
       <c r="G31" s="13" t="s">
         <v>18</v>
       </c>
     </row>
-    <row r="32" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="32" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A32" s="14"/>
       <c r="B32" s="14"/>
       <c r="C32" s="15"/>
@@ -1269,7 +1269,7 @@
       <c r="F32" s="17"/>
       <c r="G32" s="17"/>
     </row>
-    <row r="33" spans="1:7" ht="20.25" x14ac:dyDescent="0.25">
+    <row r="33" spans="1:7" ht="20" x14ac:dyDescent="0.35">
       <c r="A33" s="29" t="s">
         <v>22</v>
       </c>
@@ -1280,7 +1280,7 @@
       <c r="F33" s="17"/>
       <c r="G33" s="17"/>
     </row>
-    <row r="34" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="34" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A34" s="23" t="s">
         <v>4</v>
       </c>
@@ -1299,54 +1299,54 @@
       </c>
       <c r="G34" s="17"/>
     </row>
-    <row r="35" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="35" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A35" s="7">
-        <v>46291</v>
+        <v>46294</v>
       </c>
       <c r="B35" s="8"/>
       <c r="C35" s="20" t="s">
         <v>23</v>
       </c>
       <c r="D35" s="10">
-        <v>255.72</v>
+        <v>254.58</v>
       </c>
       <c r="E35" s="10">
-        <v>226.81</v>
+        <v>223.74</v>
       </c>
       <c r="F35" s="10">
-        <v>235.81</v>
+        <v>232.74</v>
       </c>
       <c r="G35" s="17"/>
     </row>
-    <row r="36" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="36" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A36" s="11">
-        <v>46290</v>
+        <v>46291</v>
       </c>
       <c r="B36" s="12"/>
       <c r="C36" s="12" t="s">
         <v>23</v>
       </c>
       <c r="D36" s="13">
-        <v>257.70999999999998</v>
+        <v>255.72</v>
       </c>
       <c r="E36" s="13">
-        <v>226.73</v>
+        <v>226.81</v>
       </c>
       <c r="F36" s="13">
-        <v>235.73</v>
+        <v>235.81</v>
       </c>
       <c r="G36" s="17"/>
     </row>
-    <row r="37" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="37" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A37" s="7">
-        <v>46291</v>
+        <v>46294</v>
       </c>
       <c r="B37" s="8"/>
       <c r="C37" s="20" t="s">
         <v>24</v>
       </c>
       <c r="D37" s="10">
-        <v>271.33999999999997</v>
+        <v>270.2</v>
       </c>
       <c r="E37" s="10" t="s">
         <v>18</v>
@@ -1356,16 +1356,16 @@
       </c>
       <c r="G37" s="17"/>
     </row>
-    <row r="38" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="38" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A38" s="11">
-        <v>46290</v>
+        <v>46291</v>
       </c>
       <c r="B38" s="12"/>
       <c r="C38" s="12" t="s">
         <v>24</v>
       </c>
       <c r="D38" s="13">
-        <v>273.33</v>
+        <v>271.33999999999997</v>
       </c>
       <c r="E38" s="13" t="s">
         <v>18</v>
@@ -1375,7 +1375,7 @@
       </c>
       <c r="G38" s="17"/>
     </row>
-    <row r="39" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="39" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A39" s="24"/>
       <c r="B39" s="24"/>
       <c r="C39" s="15"/>
@@ -1384,7 +1384,7 @@
       <c r="F39" s="17"/>
       <c r="G39" s="17"/>
     </row>
-    <row r="40" spans="1:7" ht="20.25" x14ac:dyDescent="0.25">
+    <row r="40" spans="1:7" ht="20" x14ac:dyDescent="0.35">
       <c r="A40" s="29" t="s">
         <v>25</v>
       </c>
@@ -1395,7 +1395,7 @@
       <c r="F40" s="17"/>
       <c r="G40" s="17"/>
     </row>
-    <row r="41" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="41" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A41" s="23" t="s">
         <v>4</v>
       </c>
@@ -1414,83 +1414,83 @@
       </c>
       <c r="G41" s="17"/>
     </row>
-    <row r="42" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="42" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A42" s="7">
-        <v>46291</v>
+        <v>46294</v>
       </c>
       <c r="B42" s="8"/>
       <c r="C42" s="20" t="s">
         <v>26</v>
       </c>
       <c r="D42" s="10">
-        <v>265.02</v>
+        <v>263.95999999999998</v>
       </c>
       <c r="E42" s="10">
-        <v>231.78</v>
+        <v>232.08</v>
       </c>
       <c r="F42" s="10">
-        <v>241.78</v>
+        <v>242.08</v>
       </c>
       <c r="G42" s="17"/>
     </row>
-    <row r="43" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="43" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A43" s="11">
-        <v>46291</v>
+        <v>46294</v>
       </c>
       <c r="B43" s="12"/>
       <c r="C43" s="21" t="s">
         <v>27</v>
       </c>
       <c r="D43" s="13">
-        <v>264.63</v>
+        <v>263.57</v>
       </c>
       <c r="E43" s="13">
-        <v>232.19</v>
+        <v>232.49</v>
       </c>
       <c r="F43" s="13">
-        <v>242.19</v>
+        <v>242.49</v>
       </c>
       <c r="G43" s="17"/>
     </row>
-    <row r="44" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="44" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A44" s="7">
-        <v>46290</v>
+        <v>46291</v>
       </c>
       <c r="B44" s="8"/>
       <c r="C44" s="20" t="s">
         <v>26</v>
       </c>
       <c r="D44" s="10">
-        <v>266.97000000000003</v>
+        <v>265.02</v>
       </c>
       <c r="E44" s="10">
-        <v>231.64</v>
+        <v>231.78</v>
       </c>
       <c r="F44" s="10">
-        <v>241.64</v>
+        <v>241.78</v>
       </c>
       <c r="G44" s="17"/>
     </row>
-    <row r="45" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="45" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A45" s="11">
-        <v>46290</v>
+        <v>46291</v>
       </c>
       <c r="B45" s="12"/>
       <c r="C45" s="21" t="s">
         <v>27</v>
       </c>
       <c r="D45" s="13">
-        <v>266.58</v>
+        <v>264.63</v>
       </c>
       <c r="E45" s="13">
-        <v>232.05</v>
+        <v>232.19</v>
       </c>
       <c r="F45" s="13">
-        <v>242.05</v>
+        <v>242.19</v>
       </c>
       <c r="G45" s="17"/>
     </row>
-    <row r="46" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="46" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A46" s="14"/>
       <c r="B46" s="24"/>
       <c r="C46" s="15"/>
@@ -1499,7 +1499,7 @@
       <c r="F46" s="16"/>
       <c r="G46" s="17"/>
     </row>
-    <row r="47" spans="1:7" ht="20.25" x14ac:dyDescent="0.25">
+    <row r="47" spans="1:7" ht="20" x14ac:dyDescent="0.35">
       <c r="A47" s="25" t="s">
         <v>28</v>
       </c>
@@ -1510,7 +1510,7 @@
       <c r="F47" s="17"/>
       <c r="G47" s="17"/>
     </row>
-    <row r="48" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="48" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A48" s="23" t="s">
         <v>4</v>
       </c>
@@ -1529,83 +1529,83 @@
       </c>
       <c r="G48" s="17"/>
     </row>
-    <row r="49" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="49" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A49" s="7">
-        <v>46291</v>
+        <v>46294</v>
       </c>
       <c r="B49" s="8"/>
       <c r="C49" s="20" t="s">
         <v>29</v>
       </c>
       <c r="D49" s="10">
-        <v>262.01</v>
+        <v>259.01</v>
       </c>
       <c r="E49" s="10">
-        <v>229.06</v>
+        <v>228.95</v>
       </c>
       <c r="F49" s="10">
-        <v>239.06</v>
+        <v>238.95</v>
       </c>
       <c r="G49" s="28"/>
     </row>
-    <row r="50" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="50" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A50" s="11">
-        <v>46291</v>
+        <v>46294</v>
       </c>
       <c r="B50" s="12"/>
       <c r="C50" s="21" t="s">
         <v>30</v>
       </c>
       <c r="D50" s="13">
-        <v>259.89999999999998</v>
+        <v>256.86</v>
       </c>
       <c r="E50" s="13">
-        <v>228.84</v>
+        <v>228.72</v>
       </c>
       <c r="F50" s="13">
-        <v>238.84</v>
+        <v>238.72</v>
       </c>
       <c r="G50" s="28"/>
     </row>
-    <row r="51" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="51" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A51" s="7">
-        <v>46290</v>
+        <v>46291</v>
       </c>
       <c r="B51" s="8"/>
       <c r="C51" s="20" t="s">
         <v>29</v>
       </c>
       <c r="D51" s="10">
-        <v>263.64</v>
+        <v>262.01</v>
       </c>
       <c r="E51" s="10">
-        <v>228.59</v>
+        <v>229.06</v>
       </c>
       <c r="F51" s="10">
-        <v>238.59</v>
+        <v>239.06</v>
       </c>
       <c r="G51" s="17"/>
     </row>
-    <row r="52" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="52" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A52" s="11">
-        <v>46290</v>
+        <v>46291</v>
       </c>
       <c r="B52" s="12"/>
       <c r="C52" s="21" t="s">
         <v>30</v>
       </c>
       <c r="D52" s="13">
-        <v>261.56</v>
+        <v>259.89999999999998</v>
       </c>
       <c r="E52" s="13">
-        <v>228.39</v>
+        <v>228.84</v>
       </c>
       <c r="F52" s="13">
-        <v>238.39</v>
+        <v>238.84</v>
       </c>
       <c r="G52" s="17"/>
     </row>
-    <row r="53" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="53" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A53" s="14"/>
       <c r="B53" s="14"/>
       <c r="C53" s="15"/>
@@ -1614,7 +1614,7 @@
       <c r="F53" s="16"/>
       <c r="G53" s="17"/>
     </row>
-    <row r="54" spans="1:7" ht="20.25" x14ac:dyDescent="0.25">
+    <row r="54" spans="1:7" ht="20" x14ac:dyDescent="0.35">
       <c r="A54" s="27" t="s">
         <v>31</v>
       </c>
@@ -1625,7 +1625,7 @@
       <c r="F54" s="17"/>
       <c r="G54" s="17"/>
     </row>
-    <row r="55" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="55" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A55" s="23" t="s">
         <v>4</v>
       </c>
@@ -1644,54 +1644,54 @@
       </c>
       <c r="G55" s="17"/>
     </row>
-    <row r="56" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="56" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A56" s="7">
-        <v>46291</v>
+        <v>46294</v>
       </c>
       <c r="B56" s="8"/>
       <c r="C56" s="20" t="s">
         <v>32</v>
       </c>
       <c r="D56" s="10">
-        <v>273.75</v>
+        <v>272.58999999999997</v>
       </c>
       <c r="E56" s="10">
-        <v>250.77</v>
+        <v>251.4</v>
       </c>
       <c r="F56" s="10">
-        <v>260.77</v>
+        <v>261.39999999999998</v>
       </c>
       <c r="G56" s="17"/>
     </row>
-    <row r="57" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="57" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A57" s="11">
-        <v>46291</v>
+        <v>46294</v>
       </c>
       <c r="B57" s="12"/>
       <c r="C57" s="21" t="s">
         <v>33</v>
       </c>
       <c r="D57" s="13">
-        <v>262.83</v>
+        <v>261.7</v>
       </c>
       <c r="E57" s="13">
-        <v>236.99</v>
+        <v>237.12</v>
       </c>
       <c r="F57" s="13">
-        <v>246.99</v>
+        <v>247.12</v>
       </c>
       <c r="G57" s="17"/>
     </row>
-    <row r="58" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="58" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A58" s="7">
-        <v>46291</v>
+        <v>46294</v>
       </c>
       <c r="B58" s="8"/>
       <c r="C58" s="20" t="s">
         <v>34</v>
       </c>
       <c r="D58" s="10">
-        <v>264.13</v>
+        <v>263.01</v>
       </c>
       <c r="E58" s="10" t="s">
         <v>18</v>
@@ -1701,111 +1701,111 @@
       </c>
       <c r="G58" s="17"/>
     </row>
-    <row r="59" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="59" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A59" s="11">
-        <v>46291</v>
+        <v>46294</v>
       </c>
       <c r="B59" s="12"/>
       <c r="C59" s="21" t="s">
         <v>35</v>
       </c>
       <c r="D59" s="13">
-        <v>259.64</v>
+        <v>258.38</v>
       </c>
       <c r="E59" s="13">
-        <v>231.36</v>
+        <v>231.5</v>
       </c>
       <c r="F59" s="13" t="s">
         <v>18</v>
       </c>
       <c r="G59" s="17"/>
     </row>
-    <row r="60" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="60" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A60" s="7">
-        <v>46291</v>
+        <v>46294</v>
       </c>
       <c r="B60" s="8"/>
       <c r="C60" s="20" t="s">
         <v>36</v>
       </c>
       <c r="D60" s="10">
-        <v>255.47</v>
+        <v>254.21</v>
       </c>
       <c r="E60" s="10">
-        <v>227.31</v>
+        <v>227.44</v>
       </c>
       <c r="F60" s="10">
-        <v>237.31</v>
+        <v>237.44</v>
       </c>
       <c r="G60" s="17"/>
     </row>
-    <row r="61" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="61" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A61" s="11">
-        <v>46291</v>
+        <v>46294</v>
       </c>
       <c r="B61" s="12"/>
       <c r="C61" s="21" t="s">
         <v>37</v>
       </c>
       <c r="D61" s="13">
-        <v>260.92</v>
+        <v>259.64999999999998</v>
       </c>
       <c r="E61" s="13">
-        <v>245.76</v>
+        <v>246.21</v>
       </c>
       <c r="F61" s="13" t="s">
         <v>18</v>
       </c>
       <c r="G61" s="17"/>
     </row>
-    <row r="62" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="62" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A62" s="7">
-        <v>46290</v>
+        <v>46291</v>
       </c>
       <c r="B62" s="8"/>
       <c r="C62" s="20" t="s">
         <v>32</v>
       </c>
       <c r="D62" s="10">
-        <v>275.76</v>
+        <v>273.75</v>
       </c>
       <c r="E62" s="10">
-        <v>250.46</v>
+        <v>250.77</v>
       </c>
       <c r="F62" s="10">
-        <v>260.45999999999998</v>
+        <v>260.77</v>
       </c>
       <c r="G62" s="17"/>
     </row>
-    <row r="63" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="63" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A63" s="11">
-        <v>46290</v>
+        <v>46291</v>
       </c>
       <c r="B63" s="12"/>
       <c r="C63" s="21" t="s">
         <v>33</v>
       </c>
       <c r="D63" s="13">
-        <v>264.82</v>
+        <v>262.83</v>
       </c>
       <c r="E63" s="13">
-        <v>236.97</v>
+        <v>236.99</v>
       </c>
       <c r="F63" s="13">
-        <v>246.97</v>
+        <v>246.99</v>
       </c>
       <c r="G63" s="17"/>
     </row>
-    <row r="64" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="64" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A64" s="7">
-        <v>46290</v>
+        <v>46291</v>
       </c>
       <c r="B64" s="8"/>
       <c r="C64" s="20" t="s">
         <v>34</v>
       </c>
       <c r="D64" s="10">
-        <v>266.11</v>
+        <v>264.13</v>
       </c>
       <c r="E64" s="10" t="s">
         <v>18</v>
@@ -1815,55 +1815,55 @@
       </c>
       <c r="G64" s="17"/>
     </row>
-    <row r="65" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="65" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A65" s="11">
-        <v>46290</v>
+        <v>46291</v>
       </c>
       <c r="B65" s="12"/>
       <c r="C65" s="21" t="s">
         <v>35</v>
       </c>
       <c r="D65" s="13">
-        <v>261.7</v>
+        <v>259.64</v>
       </c>
       <c r="E65" s="13">
-        <v>231.34</v>
+        <v>231.36</v>
       </c>
       <c r="F65" s="13" t="s">
         <v>18</v>
       </c>
     </row>
-    <row r="66" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="66" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A66" s="7">
-        <v>46290</v>
+        <v>46291</v>
       </c>
       <c r="B66" s="8"/>
       <c r="C66" s="20" t="s">
         <v>36</v>
       </c>
       <c r="D66" s="10">
-        <v>257.52999999999997</v>
+        <v>255.47</v>
       </c>
       <c r="E66" s="10">
-        <v>227.29</v>
+        <v>227.31</v>
       </c>
       <c r="F66" s="10">
-        <v>237.29</v>
-      </c>
-    </row>
-    <row r="67" spans="1:6" x14ac:dyDescent="0.25">
+        <v>237.31</v>
+      </c>
+    </row>
+    <row r="67" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A67" s="11">
-        <v>46290</v>
+        <v>46291</v>
       </c>
       <c r="B67" s="12"/>
       <c r="C67" s="21" t="s">
         <v>37</v>
       </c>
       <c r="D67" s="13">
-        <v>262.99</v>
+        <v>260.92</v>
       </c>
       <c r="E67" s="13">
-        <v>245.54</v>
+        <v>245.76</v>
       </c>
       <c r="F67" s="13" t="s">
         <v>18</v>
@@ -1900,17 +1900,6 @@
 </file>
 
 <file path=customXml/item2.xml><?xml version="1.0" encoding="utf-8"?>
-<p:properties xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls">
-  <documentManagement>
-    <lcf76f155ced4ddcb4097134ff3c332f xmlns="87276d81-85f4-4ef2-9e6e-55066304288f">
-      <Terms xmlns="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
-    </lcf76f155ced4ddcb4097134ff3c332f>
-    <TaxCatchAll xmlns="b23b8984-eafa-4e79-985e-54f52f3da58e" xsi:nil="true"/>
-  </documentManagement>
-</p:properties>
-</file>
-
-<file path=customXml/item3.xml><?xml version="1.0" encoding="utf-8"?>
 <ct:contentTypeSchema xmlns:ct="http://schemas.microsoft.com/office/2006/metadata/contentType" xmlns:ma="http://schemas.microsoft.com/office/2006/metadata/properties/metaAttributes" ct:_="" ma:_="" ma:contentTypeName="Document" ma:contentTypeID="0x010100D3632DF5622958439304627C030B0427" ma:contentTypeVersion="18" ma:contentTypeDescription="Create a new document." ma:contentTypeScope="" ma:versionID="8c2ecbce386d6bac497f8eb2d8f0fb7a">
   <xsd:schema xmlns:xsd="http://www.w3.org/2001/XMLSchema" xmlns:xs="http://www.w3.org/2001/XMLSchema" xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:ns2="87276d81-85f4-4ef2-9e6e-55066304288f" xmlns:ns3="39e1dda6-d1d8-4c88-a3b9-f1abc1284bad" xmlns:ns4="b23b8984-eafa-4e79-985e-54f52f3da58e" targetNamespace="http://schemas.microsoft.com/office/2006/metadata/properties" ma:root="true" ma:fieldsID="4cfd0c2f651c1ce156ad4fcb44ea61dd" ns2:_="" ns3:_="" ns4:_="">
     <xsd:import namespace="87276d81-85f4-4ef2-9e6e-55066304288f"/>
@@ -2170,6 +2159,17 @@
 </ct:contentTypeSchema>
 </file>
 
+<file path=customXml/item3.xml><?xml version="1.0" encoding="utf-8"?>
+<p:properties xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls">
+  <documentManagement>
+    <lcf76f155ced4ddcb4097134ff3c332f xmlns="87276d81-85f4-4ef2-9e6e-55066304288f">
+      <Terms xmlns="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
+    </lcf76f155ced4ddcb4097134ff3c332f>
+    <TaxCatchAll xmlns="b23b8984-eafa-4e79-985e-54f52f3da58e" xsi:nil="true"/>
+  </documentManagement>
+</p:properties>
+</file>
+
 <file path=customXml/itemProps1.xml><?xml version="1.0" encoding="utf-8"?>
 <ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{F60519E9-FD90-4339-869C-BC2F85719BB8}">
   <ds:schemaRefs>
@@ -2179,17 +2179,6 @@
 </file>
 
 <file path=customXml/itemProps2.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{57A83D98-2BAE-4D83-823A-D31C464B620C}">
-  <ds:schemaRefs>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/properties"/>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
-    <ds:schemaRef ds:uri="87276d81-85f4-4ef2-9e6e-55066304288f"/>
-    <ds:schemaRef ds:uri="b23b8984-eafa-4e79-985e-54f52f3da58e"/>
-  </ds:schemaRefs>
-</ds:datastoreItem>
-</file>
-
-<file path=customXml/itemProps3.xml><?xml version="1.0" encoding="utf-8"?>
 <ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{B44E1863-2778-41F9-ACBA-48420F931671}">
   <ds:schemaRefs>
     <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/contentType"/>
@@ -2209,6 +2198,17 @@
 </ds:datastoreItem>
 </file>
 
+<file path=customXml/itemProps3.xml><?xml version="1.0" encoding="utf-8"?>
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{57A83D98-2BAE-4D83-823A-D31C464B620C}">
+  <ds:schemaRefs>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/properties"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
+    <ds:schemaRef ds:uri="87276d81-85f4-4ef2-9e6e-55066304288f"/>
+    <ds:schemaRef ds:uri="b23b8984-eafa-4e79-985e-54f52f3da58e"/>
+  </ds:schemaRefs>
+</ds:datastoreItem>
+</file>
+
 <file path=docMetadata/LabelInfo.xml><?xml version="1.0" encoding="utf-8"?>
 <clbl:labelList xmlns:clbl="http://schemas.microsoft.com/office/2020/mipLabelMetadata">
   <clbl:label id="{569bf4a9-87bd-4dbf-a36c-1db5158e5def}" enabled="1" method="Privileged" siteId="{ea80952e-a476-42d4-aaf4-5457852b0f7e}" removed="0"/>

</xml_diff>

<commit_message>
Tue Sep 29 07:02:03 UTC 2026
</commit_message>
<xml_diff>
--- a/bp.com-content-dam-bp-country-sites-en_au-australia-home-products-services-pricing-tgp-excel.xlsx
+++ b/bp.com-content-dam-bp-country-sites-en_au-australia-home-products-services-pricing-tgp-excel.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://bp365.sharepoint.com/sites/WholesalePricing/Shared Documents/B2C/TGP/Daily TGP/Web TGP/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="14_{4C1D3E27-72AB-4068-BADA-1BAD2E0663D8}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="14_{28C56BA8-8CE0-4226-80FC-646D55D88B7F}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-110" yWindow="-110" windowWidth="19420" windowHeight="11500" xr2:uid="{1B412EEF-F96D-4DF4-A4E9-C7F0F183C2FB}"/>
+    <workbookView xWindow="-28920" yWindow="-60" windowWidth="29040" windowHeight="15720" xr2:uid="{1B412EEF-F96D-4DF4-A4E9-C7F0F183C2FB}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
@@ -808,128 +808,128 @@
     </row>
     <row r="8" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A8" s="7">
-        <v>46294</v>
+        <v>46295</v>
       </c>
       <c r="B8" s="8"/>
       <c r="C8" s="9" t="s">
         <v>10</v>
       </c>
       <c r="D8" s="10">
-        <v>264.13</v>
+        <v>262.06</v>
       </c>
       <c r="E8" s="10">
-        <v>228.23</v>
+        <v>229.41</v>
       </c>
       <c r="F8" s="10">
-        <v>238.23</v>
+        <v>239.42</v>
       </c>
       <c r="G8" s="10">
-        <v>228.19</v>
+        <v>229.38</v>
       </c>
     </row>
     <row r="9" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A9" s="11">
-        <v>46294</v>
+        <v>46295</v>
       </c>
       <c r="B9" s="12"/>
       <c r="C9" s="12" t="s">
         <v>11</v>
       </c>
       <c r="D9" s="13">
-        <v>264.13</v>
+        <v>262.06</v>
       </c>
       <c r="E9" s="13">
-        <v>228.23</v>
+        <v>229.41</v>
       </c>
       <c r="F9" s="13">
-        <v>238.23</v>
+        <v>239.42</v>
       </c>
       <c r="G9" s="13">
-        <v>228.19</v>
+        <v>229.38</v>
       </c>
     </row>
     <row r="10" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A10" s="7">
-        <v>46294</v>
+        <v>46295</v>
       </c>
       <c r="B10" s="8"/>
       <c r="C10" s="9" t="s">
         <v>12</v>
       </c>
       <c r="D10" s="10">
-        <v>256.04000000000002</v>
+        <v>256.99</v>
       </c>
       <c r="E10" s="10">
-        <v>225.91</v>
+        <v>226.85</v>
       </c>
       <c r="F10" s="10">
-        <v>235.91</v>
+        <v>236.85</v>
       </c>
       <c r="G10" s="10">
-        <v>226.32</v>
+        <v>227.27</v>
       </c>
     </row>
     <row r="11" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A11" s="11">
-        <v>46291</v>
+        <v>46294</v>
       </c>
       <c r="B11" s="12"/>
       <c r="C11" s="12" t="s">
         <v>10</v>
       </c>
       <c r="D11" s="13">
-        <v>265</v>
+        <v>264.13</v>
       </c>
       <c r="E11" s="13">
-        <v>231.06</v>
+        <v>228.23</v>
       </c>
       <c r="F11" s="13">
-        <v>241.06</v>
+        <v>238.23</v>
       </c>
       <c r="G11" s="13">
-        <v>231.02</v>
+        <v>228.19</v>
       </c>
     </row>
     <row r="12" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A12" s="7">
-        <v>46291</v>
+        <v>46294</v>
       </c>
       <c r="B12" s="8"/>
       <c r="C12" s="9" t="s">
         <v>11</v>
       </c>
       <c r="D12" s="10">
-        <v>265</v>
+        <v>264.13</v>
       </c>
       <c r="E12" s="10">
-        <v>231.06</v>
+        <v>228.23</v>
       </c>
       <c r="F12" s="10">
-        <v>241.06</v>
+        <v>238.23</v>
       </c>
       <c r="G12" s="10">
-        <v>231.02</v>
+        <v>228.19</v>
       </c>
     </row>
     <row r="13" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A13" s="11">
-        <v>46291</v>
+        <v>46294</v>
       </c>
       <c r="B13" s="12"/>
       <c r="C13" s="12" t="s">
         <v>12</v>
       </c>
       <c r="D13" s="13">
-        <v>257.18</v>
+        <v>256.04000000000002</v>
       </c>
       <c r="E13" s="13">
-        <v>227.87</v>
+        <v>225.91</v>
       </c>
       <c r="F13" s="13">
-        <v>237.87</v>
+        <v>235.91</v>
       </c>
       <c r="G13" s="13">
-        <v>228.29</v>
+        <v>226.32</v>
       </c>
     </row>
     <row r="14" spans="1:7" x14ac:dyDescent="0.35">
@@ -973,39 +973,39 @@
     </row>
     <row r="17" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A17" s="7">
-        <v>46294</v>
+        <v>46295</v>
       </c>
       <c r="B17" s="8"/>
       <c r="C17" s="20" t="s">
         <v>14</v>
       </c>
       <c r="D17" s="10">
-        <v>260.33</v>
+        <v>261.17</v>
       </c>
       <c r="E17" s="10">
-        <v>231.8</v>
+        <v>232.65</v>
       </c>
       <c r="F17" s="10">
-        <v>241.8</v>
+        <v>242.65</v>
       </c>
       <c r="G17" s="17"/>
     </row>
     <row r="18" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A18" s="11">
-        <v>46291</v>
+        <v>46294</v>
       </c>
       <c r="B18" s="12"/>
       <c r="C18" s="12" t="s">
         <v>14</v>
       </c>
       <c r="D18" s="13">
-        <v>261.56</v>
+        <v>260.33</v>
       </c>
       <c r="E18" s="13">
-        <v>231.65</v>
+        <v>231.8</v>
       </c>
       <c r="F18" s="13">
-        <v>241.65</v>
+        <v>241.8</v>
       </c>
       <c r="G18" s="17"/>
     </row>
@@ -1052,41 +1052,41 @@
     </row>
     <row r="22" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A22" s="7">
-        <v>46294</v>
+        <v>46295</v>
       </c>
       <c r="B22" s="8"/>
       <c r="C22" s="20" t="s">
         <v>16</v>
       </c>
       <c r="D22" s="10">
-        <v>264.7</v>
+        <v>263.18</v>
       </c>
       <c r="E22" s="10">
-        <v>227.82</v>
+        <v>227.91</v>
       </c>
       <c r="F22" s="10">
-        <v>237.42</v>
+        <v>237.51</v>
       </c>
       <c r="G22" s="10">
-        <v>226.54</v>
+        <v>226.62</v>
       </c>
     </row>
     <row r="23" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A23" s="11">
-        <v>46294</v>
+        <v>46295</v>
       </c>
       <c r="B23" s="12"/>
       <c r="C23" s="21" t="s">
         <v>17</v>
       </c>
       <c r="D23" s="13">
-        <v>260.89999999999998</v>
+        <v>261.86</v>
       </c>
       <c r="E23" s="13">
-        <v>236.07</v>
+        <v>237.06</v>
       </c>
       <c r="F23" s="13">
-        <v>246.07</v>
+        <v>247.06</v>
       </c>
       <c r="G23" s="13" t="s">
         <v>18</v>
@@ -1094,20 +1094,20 @@
     </row>
     <row r="24" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A24" s="7">
-        <v>46294</v>
+        <v>46295</v>
       </c>
       <c r="B24" s="8"/>
       <c r="C24" s="20" t="s">
         <v>19</v>
       </c>
       <c r="D24" s="10">
-        <v>261.35000000000002</v>
+        <v>262.3</v>
       </c>
       <c r="E24" s="10">
-        <v>235.33</v>
+        <v>236.31</v>
       </c>
       <c r="F24" s="10">
-        <v>245.33</v>
+        <v>246.31</v>
       </c>
       <c r="G24" s="10" t="s">
         <v>18</v>
@@ -1115,41 +1115,41 @@
     </row>
     <row r="25" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A25" s="11">
-        <v>46294</v>
+        <v>46295</v>
       </c>
       <c r="B25" s="12"/>
       <c r="C25" s="21" t="s">
         <v>20</v>
       </c>
       <c r="D25" s="13">
-        <v>258.07</v>
+        <v>259.01</v>
       </c>
       <c r="E25" s="13">
-        <v>235.46</v>
+        <v>236.46</v>
       </c>
       <c r="F25" s="13">
-        <v>245.46</v>
+        <v>246.46</v>
       </c>
       <c r="G25" s="13">
-        <v>233.36</v>
+        <v>234.36</v>
       </c>
     </row>
     <row r="26" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A26" s="7">
-        <v>46294</v>
+        <v>46295</v>
       </c>
       <c r="B26" s="8"/>
       <c r="C26" s="20" t="s">
         <v>21</v>
       </c>
       <c r="D26" s="10">
-        <v>259.77</v>
+        <v>260.69</v>
       </c>
       <c r="E26" s="10">
-        <v>236.94</v>
+        <v>237.94</v>
       </c>
       <c r="F26" s="10">
-        <v>246.94</v>
+        <v>247.94</v>
       </c>
       <c r="G26" s="10" t="s">
         <v>18</v>
@@ -1157,41 +1157,41 @@
     </row>
     <row r="27" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A27" s="11">
-        <v>46291</v>
+        <v>46294</v>
       </c>
       <c r="B27" s="12"/>
       <c r="C27" s="12" t="s">
         <v>16</v>
       </c>
       <c r="D27" s="13">
-        <v>265.57</v>
+        <v>264.7</v>
       </c>
       <c r="E27" s="13">
-        <v>229.77</v>
+        <v>227.82</v>
       </c>
       <c r="F27" s="13">
-        <v>239.37</v>
+        <v>237.42</v>
       </c>
       <c r="G27" s="13">
-        <v>228.49</v>
+        <v>226.54</v>
       </c>
     </row>
     <row r="28" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A28" s="7">
-        <v>46291</v>
+        <v>46294</v>
       </c>
       <c r="B28" s="8"/>
       <c r="C28" s="20" t="s">
         <v>17</v>
       </c>
       <c r="D28" s="10">
-        <v>262.02999999999997</v>
+        <v>260.89999999999998</v>
       </c>
       <c r="E28" s="22">
-        <v>235.8</v>
+        <v>236.07</v>
       </c>
       <c r="F28" s="22">
-        <v>245.8</v>
+        <v>246.07</v>
       </c>
       <c r="G28" s="22" t="s">
         <v>18</v>
@@ -1199,20 +1199,20 @@
     </row>
     <row r="29" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A29" s="11">
-        <v>46291</v>
+        <v>46294</v>
       </c>
       <c r="B29" s="12"/>
       <c r="C29" s="12" t="s">
         <v>19</v>
       </c>
       <c r="D29" s="13">
-        <v>262.48</v>
+        <v>261.35000000000002</v>
       </c>
       <c r="E29" s="13">
-        <v>235.06</v>
+        <v>235.33</v>
       </c>
       <c r="F29" s="13">
-        <v>245.06</v>
+        <v>245.33</v>
       </c>
       <c r="G29" s="13" t="s">
         <v>18</v>
@@ -1220,41 +1220,41 @@
     </row>
     <row r="30" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A30" s="7">
-        <v>46291</v>
+        <v>46294</v>
       </c>
       <c r="B30" s="8"/>
       <c r="C30" s="20" t="s">
         <v>20</v>
       </c>
       <c r="D30" s="10">
-        <v>259.20999999999998</v>
+        <v>258.07</v>
       </c>
       <c r="E30" s="22">
-        <v>235.18</v>
+        <v>235.46</v>
       </c>
       <c r="F30" s="22">
-        <v>245.18</v>
+        <v>245.46</v>
       </c>
       <c r="G30" s="22">
-        <v>233.08</v>
+        <v>233.36</v>
       </c>
     </row>
     <row r="31" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A31" s="11">
-        <v>46291</v>
+        <v>46294</v>
       </c>
       <c r="B31" s="12"/>
       <c r="C31" s="12" t="s">
         <v>21</v>
       </c>
       <c r="D31" s="13">
-        <v>260.93</v>
+        <v>259.77</v>
       </c>
       <c r="E31" s="13">
-        <v>236.66</v>
+        <v>236.94</v>
       </c>
       <c r="F31" s="13">
-        <v>246.66</v>
+        <v>246.94</v>
       </c>
       <c r="G31" s="13" t="s">
         <v>18</v>
@@ -1301,52 +1301,52 @@
     </row>
     <row r="35" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A35" s="7">
-        <v>46294</v>
+        <v>46295</v>
       </c>
       <c r="B35" s="8"/>
       <c r="C35" s="20" t="s">
         <v>23</v>
       </c>
       <c r="D35" s="10">
-        <v>254.58</v>
+        <v>255.53</v>
       </c>
       <c r="E35" s="10">
-        <v>223.74</v>
+        <v>224.68</v>
       </c>
       <c r="F35" s="10">
-        <v>232.74</v>
+        <v>233.68</v>
       </c>
       <c r="G35" s="17"/>
     </row>
     <row r="36" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A36" s="11">
-        <v>46291</v>
+        <v>46294</v>
       </c>
       <c r="B36" s="12"/>
       <c r="C36" s="12" t="s">
         <v>23</v>
       </c>
       <c r="D36" s="13">
-        <v>255.72</v>
+        <v>254.58</v>
       </c>
       <c r="E36" s="13">
-        <v>226.81</v>
+        <v>223.74</v>
       </c>
       <c r="F36" s="13">
-        <v>235.81</v>
+        <v>232.74</v>
       </c>
       <c r="G36" s="17"/>
     </row>
     <row r="37" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A37" s="7">
-        <v>46294</v>
+        <v>46295</v>
       </c>
       <c r="B37" s="8"/>
       <c r="C37" s="20" t="s">
         <v>24</v>
       </c>
       <c r="D37" s="10">
-        <v>270.2</v>
+        <v>271.14999999999998</v>
       </c>
       <c r="E37" s="10" t="s">
         <v>18</v>
@@ -1358,14 +1358,14 @@
     </row>
     <row r="38" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A38" s="11">
-        <v>46291</v>
+        <v>46294</v>
       </c>
       <c r="B38" s="12"/>
       <c r="C38" s="12" t="s">
         <v>24</v>
       </c>
       <c r="D38" s="13">
-        <v>271.33999999999997</v>
+        <v>270.2</v>
       </c>
       <c r="E38" s="13" t="s">
         <v>18</v>
@@ -1416,77 +1416,77 @@
     </row>
     <row r="42" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A42" s="7">
-        <v>46294</v>
+        <v>46295</v>
       </c>
       <c r="B42" s="8"/>
       <c r="C42" s="20" t="s">
         <v>26</v>
       </c>
       <c r="D42" s="10">
-        <v>263.95999999999998</v>
+        <v>265</v>
       </c>
       <c r="E42" s="10">
-        <v>232.08</v>
+        <v>233.1</v>
       </c>
       <c r="F42" s="10">
-        <v>242.08</v>
+        <v>243.1</v>
       </c>
       <c r="G42" s="17"/>
     </row>
     <row r="43" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A43" s="11">
-        <v>46294</v>
+        <v>46295</v>
       </c>
       <c r="B43" s="12"/>
       <c r="C43" s="21" t="s">
         <v>27</v>
       </c>
       <c r="D43" s="13">
-        <v>263.57</v>
+        <v>264.61</v>
       </c>
       <c r="E43" s="13">
-        <v>232.49</v>
+        <v>233.51</v>
       </c>
       <c r="F43" s="13">
-        <v>242.49</v>
+        <v>243.51</v>
       </c>
       <c r="G43" s="17"/>
     </row>
     <row r="44" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A44" s="7">
-        <v>46291</v>
+        <v>46294</v>
       </c>
       <c r="B44" s="8"/>
       <c r="C44" s="20" t="s">
         <v>26</v>
       </c>
       <c r="D44" s="10">
-        <v>265.02</v>
+        <v>263.95999999999998</v>
       </c>
       <c r="E44" s="10">
-        <v>231.78</v>
+        <v>232.08</v>
       </c>
       <c r="F44" s="10">
-        <v>241.78</v>
+        <v>242.08</v>
       </c>
       <c r="G44" s="17"/>
     </row>
     <row r="45" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A45" s="11">
-        <v>46291</v>
+        <v>46294</v>
       </c>
       <c r="B45" s="12"/>
       <c r="C45" s="21" t="s">
         <v>27</v>
       </c>
       <c r="D45" s="13">
-        <v>264.63</v>
+        <v>263.57</v>
       </c>
       <c r="E45" s="13">
-        <v>232.19</v>
+        <v>232.49</v>
       </c>
       <c r="F45" s="13">
-        <v>242.19</v>
+        <v>242.49</v>
       </c>
       <c r="G45" s="17"/>
     </row>
@@ -1531,77 +1531,77 @@
     </row>
     <row r="49" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A49" s="7">
-        <v>46294</v>
+        <v>46295</v>
       </c>
       <c r="B49" s="8"/>
       <c r="C49" s="20" t="s">
         <v>29</v>
       </c>
       <c r="D49" s="10">
-        <v>259.01</v>
+        <v>257.52</v>
       </c>
       <c r="E49" s="10">
-        <v>228.95</v>
+        <v>229.12</v>
       </c>
       <c r="F49" s="10">
-        <v>238.95</v>
+        <v>239.12</v>
       </c>
       <c r="G49" s="28"/>
     </row>
     <row r="50" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A50" s="11">
-        <v>46294</v>
+        <v>46295</v>
       </c>
       <c r="B50" s="12"/>
       <c r="C50" s="21" t="s">
         <v>30</v>
       </c>
       <c r="D50" s="13">
-        <v>256.86</v>
+        <v>255.34</v>
       </c>
       <c r="E50" s="13">
-        <v>228.72</v>
+        <v>228.88</v>
       </c>
       <c r="F50" s="13">
-        <v>238.72</v>
+        <v>238.88</v>
       </c>
       <c r="G50" s="28"/>
     </row>
     <row r="51" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A51" s="7">
-        <v>46291</v>
+        <v>46294</v>
       </c>
       <c r="B51" s="8"/>
       <c r="C51" s="20" t="s">
         <v>29</v>
       </c>
       <c r="D51" s="10">
-        <v>262.01</v>
+        <v>259.01</v>
       </c>
       <c r="E51" s="10">
-        <v>229.06</v>
+        <v>228.95</v>
       </c>
       <c r="F51" s="10">
-        <v>239.06</v>
+        <v>238.95</v>
       </c>
       <c r="G51" s="17"/>
     </row>
     <row r="52" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A52" s="11">
-        <v>46291</v>
+        <v>46294</v>
       </c>
       <c r="B52" s="12"/>
       <c r="C52" s="21" t="s">
         <v>30</v>
       </c>
       <c r="D52" s="13">
-        <v>259.89999999999998</v>
+        <v>256.86</v>
       </c>
       <c r="E52" s="13">
-        <v>228.84</v>
+        <v>228.72</v>
       </c>
       <c r="F52" s="13">
-        <v>238.84</v>
+        <v>238.72</v>
       </c>
       <c r="G52" s="17"/>
     </row>
@@ -1646,52 +1646,52 @@
     </row>
     <row r="56" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A56" s="7">
-        <v>46294</v>
+        <v>46295</v>
       </c>
       <c r="B56" s="8"/>
       <c r="C56" s="20" t="s">
         <v>32</v>
       </c>
       <c r="D56" s="10">
-        <v>272.58999999999997</v>
+        <v>273.52</v>
       </c>
       <c r="E56" s="10">
-        <v>251.4</v>
+        <v>252.78</v>
       </c>
       <c r="F56" s="10">
-        <v>261.39999999999998</v>
+        <v>262.77999999999997</v>
       </c>
       <c r="G56" s="17"/>
     </row>
     <row r="57" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A57" s="11">
-        <v>46294</v>
+        <v>46295</v>
       </c>
       <c r="B57" s="12"/>
       <c r="C57" s="21" t="s">
         <v>33</v>
       </c>
       <c r="D57" s="13">
-        <v>261.7</v>
+        <v>262.66000000000003</v>
       </c>
       <c r="E57" s="13">
-        <v>237.12</v>
+        <v>237.95</v>
       </c>
       <c r="F57" s="13">
-        <v>247.12</v>
+        <v>247.95</v>
       </c>
       <c r="G57" s="17"/>
     </row>
     <row r="58" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A58" s="7">
-        <v>46294</v>
+        <v>46295</v>
       </c>
       <c r="B58" s="8"/>
       <c r="C58" s="20" t="s">
         <v>34</v>
       </c>
       <c r="D58" s="10">
-        <v>263.01</v>
+        <v>263.99</v>
       </c>
       <c r="E58" s="10" t="s">
         <v>18</v>
@@ -1703,17 +1703,17 @@
     </row>
     <row r="59" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A59" s="11">
-        <v>46294</v>
+        <v>46295</v>
       </c>
       <c r="B59" s="12"/>
       <c r="C59" s="21" t="s">
         <v>35</v>
       </c>
       <c r="D59" s="13">
-        <v>258.38</v>
+        <v>259.2</v>
       </c>
       <c r="E59" s="13">
-        <v>231.5</v>
+        <v>232.32</v>
       </c>
       <c r="F59" s="13" t="s">
         <v>18</v>
@@ -1722,36 +1722,36 @@
     </row>
     <row r="60" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A60" s="7">
-        <v>46294</v>
+        <v>46295</v>
       </c>
       <c r="B60" s="8"/>
       <c r="C60" s="20" t="s">
         <v>36</v>
       </c>
       <c r="D60" s="10">
-        <v>254.21</v>
+        <v>255.03</v>
       </c>
       <c r="E60" s="10">
-        <v>227.44</v>
+        <v>228.27</v>
       </c>
       <c r="F60" s="10">
-        <v>237.44</v>
+        <v>238.27</v>
       </c>
       <c r="G60" s="17"/>
     </row>
     <row r="61" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A61" s="11">
-        <v>46294</v>
+        <v>46295</v>
       </c>
       <c r="B61" s="12"/>
       <c r="C61" s="21" t="s">
         <v>37</v>
       </c>
       <c r="D61" s="13">
-        <v>259.64999999999998</v>
+        <v>260.45999999999998</v>
       </c>
       <c r="E61" s="13">
-        <v>246.21</v>
+        <v>247.41</v>
       </c>
       <c r="F61" s="13" t="s">
         <v>18</v>
@@ -1760,52 +1760,52 @@
     </row>
     <row r="62" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A62" s="7">
-        <v>46291</v>
+        <v>46294</v>
       </c>
       <c r="B62" s="8"/>
       <c r="C62" s="20" t="s">
         <v>32</v>
       </c>
       <c r="D62" s="10">
-        <v>273.75</v>
+        <v>272.58999999999997</v>
       </c>
       <c r="E62" s="10">
-        <v>250.77</v>
+        <v>251.4</v>
       </c>
       <c r="F62" s="10">
-        <v>260.77</v>
+        <v>261.39999999999998</v>
       </c>
       <c r="G62" s="17"/>
     </row>
     <row r="63" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A63" s="11">
-        <v>46291</v>
+        <v>46294</v>
       </c>
       <c r="B63" s="12"/>
       <c r="C63" s="21" t="s">
         <v>33</v>
       </c>
       <c r="D63" s="13">
-        <v>262.83</v>
+        <v>261.7</v>
       </c>
       <c r="E63" s="13">
-        <v>236.99</v>
+        <v>237.12</v>
       </c>
       <c r="F63" s="13">
-        <v>246.99</v>
+        <v>247.12</v>
       </c>
       <c r="G63" s="17"/>
     </row>
     <row r="64" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A64" s="7">
-        <v>46291</v>
+        <v>46294</v>
       </c>
       <c r="B64" s="8"/>
       <c r="C64" s="20" t="s">
         <v>34</v>
       </c>
       <c r="D64" s="10">
-        <v>264.13</v>
+        <v>263.01</v>
       </c>
       <c r="E64" s="10" t="s">
         <v>18</v>
@@ -1817,17 +1817,17 @@
     </row>
     <row r="65" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A65" s="11">
-        <v>46291</v>
+        <v>46294</v>
       </c>
       <c r="B65" s="12"/>
       <c r="C65" s="21" t="s">
         <v>35</v>
       </c>
       <c r="D65" s="13">
-        <v>259.64</v>
+        <v>258.38</v>
       </c>
       <c r="E65" s="13">
-        <v>231.36</v>
+        <v>231.5</v>
       </c>
       <c r="F65" s="13" t="s">
         <v>18</v>
@@ -1835,35 +1835,35 @@
     </row>
     <row r="66" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A66" s="7">
-        <v>46291</v>
+        <v>46294</v>
       </c>
       <c r="B66" s="8"/>
       <c r="C66" s="20" t="s">
         <v>36</v>
       </c>
       <c r="D66" s="10">
-        <v>255.47</v>
+        <v>254.21</v>
       </c>
       <c r="E66" s="10">
-        <v>227.31</v>
+        <v>227.44</v>
       </c>
       <c r="F66" s="10">
-        <v>237.31</v>
+        <v>237.44</v>
       </c>
     </row>
     <row r="67" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A67" s="11">
-        <v>46291</v>
+        <v>46294</v>
       </c>
       <c r="B67" s="12"/>
       <c r="C67" s="21" t="s">
         <v>37</v>
       </c>
       <c r="D67" s="13">
-        <v>260.92</v>
+        <v>259.64999999999998</v>
       </c>
       <c r="E67" s="13">
-        <v>245.76</v>
+        <v>246.21</v>
       </c>
       <c r="F67" s="13" t="s">
         <v>18</v>
@@ -1900,6 +1900,17 @@
 </file>
 
 <file path=customXml/item2.xml><?xml version="1.0" encoding="utf-8"?>
+<p:properties xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls">
+  <documentManagement>
+    <lcf76f155ced4ddcb4097134ff3c332f xmlns="87276d81-85f4-4ef2-9e6e-55066304288f">
+      <Terms xmlns="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
+    </lcf76f155ced4ddcb4097134ff3c332f>
+    <TaxCatchAll xmlns="b23b8984-eafa-4e79-985e-54f52f3da58e" xsi:nil="true"/>
+  </documentManagement>
+</p:properties>
+</file>
+
+<file path=customXml/item3.xml><?xml version="1.0" encoding="utf-8"?>
 <ct:contentTypeSchema xmlns:ct="http://schemas.microsoft.com/office/2006/metadata/contentType" xmlns:ma="http://schemas.microsoft.com/office/2006/metadata/properties/metaAttributes" ct:_="" ma:_="" ma:contentTypeName="Document" ma:contentTypeID="0x010100D3632DF5622958439304627C030B0427" ma:contentTypeVersion="18" ma:contentTypeDescription="Create a new document." ma:contentTypeScope="" ma:versionID="8c2ecbce386d6bac497f8eb2d8f0fb7a">
   <xsd:schema xmlns:xsd="http://www.w3.org/2001/XMLSchema" xmlns:xs="http://www.w3.org/2001/XMLSchema" xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:ns2="87276d81-85f4-4ef2-9e6e-55066304288f" xmlns:ns3="39e1dda6-d1d8-4c88-a3b9-f1abc1284bad" xmlns:ns4="b23b8984-eafa-4e79-985e-54f52f3da58e" targetNamespace="http://schemas.microsoft.com/office/2006/metadata/properties" ma:root="true" ma:fieldsID="4cfd0c2f651c1ce156ad4fcb44ea61dd" ns2:_="" ns3:_="" ns4:_="">
     <xsd:import namespace="87276d81-85f4-4ef2-9e6e-55066304288f"/>
@@ -2159,17 +2170,6 @@
 </ct:contentTypeSchema>
 </file>
 
-<file path=customXml/item3.xml><?xml version="1.0" encoding="utf-8"?>
-<p:properties xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls">
-  <documentManagement>
-    <lcf76f155ced4ddcb4097134ff3c332f xmlns="87276d81-85f4-4ef2-9e6e-55066304288f">
-      <Terms xmlns="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
-    </lcf76f155ced4ddcb4097134ff3c332f>
-    <TaxCatchAll xmlns="b23b8984-eafa-4e79-985e-54f52f3da58e" xsi:nil="true"/>
-  </documentManagement>
-</p:properties>
-</file>
-
 <file path=customXml/itemProps1.xml><?xml version="1.0" encoding="utf-8"?>
 <ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{F60519E9-FD90-4339-869C-BC2F85719BB8}">
   <ds:schemaRefs>
@@ -2179,6 +2179,17 @@
 </file>
 
 <file path=customXml/itemProps2.xml><?xml version="1.0" encoding="utf-8"?>
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{57A83D98-2BAE-4D83-823A-D31C464B620C}">
+  <ds:schemaRefs>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/properties"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
+    <ds:schemaRef ds:uri="87276d81-85f4-4ef2-9e6e-55066304288f"/>
+    <ds:schemaRef ds:uri="b23b8984-eafa-4e79-985e-54f52f3da58e"/>
+  </ds:schemaRefs>
+</ds:datastoreItem>
+</file>
+
+<file path=customXml/itemProps3.xml><?xml version="1.0" encoding="utf-8"?>
 <ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{B44E1863-2778-41F9-ACBA-48420F931671}">
   <ds:schemaRefs>
     <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/contentType"/>
@@ -2198,17 +2209,6 @@
 </ds:datastoreItem>
 </file>
 
-<file path=customXml/itemProps3.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{57A83D98-2BAE-4D83-823A-D31C464B620C}">
-  <ds:schemaRefs>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/properties"/>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
-    <ds:schemaRef ds:uri="87276d81-85f4-4ef2-9e6e-55066304288f"/>
-    <ds:schemaRef ds:uri="b23b8984-eafa-4e79-985e-54f52f3da58e"/>
-  </ds:schemaRefs>
-</ds:datastoreItem>
-</file>
-
 <file path=docMetadata/LabelInfo.xml><?xml version="1.0" encoding="utf-8"?>
 <clbl:labelList xmlns:clbl="http://schemas.microsoft.com/office/2020/mipLabelMetadata">
   <clbl:label id="{569bf4a9-87bd-4dbf-a36c-1db5158e5def}" enabled="1" method="Privileged" siteId="{ea80952e-a476-42d4-aaf4-5457852b0f7e}" removed="0"/>

</xml_diff>

<commit_message>
Wed Sep 30 06:52:03 UTC 2026
</commit_message>
<xml_diff>
--- a/bp.com-content-dam-bp-country-sites-en_au-australia-home-products-services-pricing-tgp-excel.xlsx
+++ b/bp.com-content-dam-bp-country-sites-en_au-australia-home-products-services-pricing-tgp-excel.xlsx
@@ -8,14 +8,14 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://bp365.sharepoint.com/sites/WholesalePricing/Shared Documents/B2C/TGP/Daily TGP/Web TGP/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="14_{28C56BA8-8CE0-4226-80FC-646D55D88B7F}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="14_{A8CA0E1F-F5B4-4C8C-94C1-F03920793B08}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-28920" yWindow="-60" windowWidth="29040" windowHeight="15720" xr2:uid="{1B412EEF-F96D-4DF4-A4E9-C7F0F183C2FB}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
   </sheets>
-  <calcPr calcId="191028" concurrentManualCount="12"/>
+  <calcPr calcId="191028"/>
   <extLst>
     <ext xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" uri="{140A7094-0E35-4892-8432-C4D2E57EDEB5}">
       <x15:workbookPr chartTrackingRefBase="1"/>
@@ -715,15 +715,15 @@
     <pageSetUpPr fitToPage="1"/>
   </sheetPr>
   <dimension ref="A1:G67"/>
-  <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
+  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
-    <col min="1" max="1" width="76.453125" bestFit="1" customWidth="1"/>
-    <col min="2" max="2" width="6.453125"/>
-    <col min="3" max="3" width="18.1796875" bestFit="1" customWidth="1"/>
-    <col min="4" max="7" width="7.1796875" bestFit="1" customWidth="1"/>
+    <col min="1" max="1" width="76.42578125" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="6.42578125"/>
+    <col min="3" max="3" width="18.140625" bestFit="1" customWidth="1"/>
+    <col min="4" max="7" width="7.140625" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:7" ht="22.5" x14ac:dyDescent="0.35">
+    <row r="1" spans="1:7" ht="23.25" x14ac:dyDescent="0.25">
       <c r="A1" s="30" t="s">
         <v>0</v>
       </c>
@@ -734,7 +734,7 @@
       <c r="F1" s="2"/>
       <c r="G1" s="2"/>
     </row>
-    <row r="2" spans="1:7" x14ac:dyDescent="0.35">
+    <row r="2" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A2" s="3"/>
       <c r="B2" s="1"/>
       <c r="C2" s="1"/>
@@ -743,7 +743,7 @@
       <c r="F2" s="2"/>
       <c r="G2" s="2"/>
     </row>
-    <row r="3" spans="1:7" x14ac:dyDescent="0.35">
+    <row r="3" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A3" s="3" t="s">
         <v>1</v>
       </c>
@@ -754,7 +754,7 @@
       <c r="F3" s="2"/>
       <c r="G3" s="2"/>
     </row>
-    <row r="4" spans="1:7" x14ac:dyDescent="0.35">
+    <row r="4" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A4" s="3" t="s">
         <v>2</v>
       </c>
@@ -765,7 +765,7 @@
       <c r="F4" s="2"/>
       <c r="G4" s="2"/>
     </row>
-    <row r="5" spans="1:7" x14ac:dyDescent="0.35">
+    <row r="5" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A5" s="3"/>
       <c r="B5" s="3"/>
       <c r="C5" s="1"/>
@@ -774,7 +774,7 @@
       <c r="F5" s="2"/>
       <c r="G5" s="2"/>
     </row>
-    <row r="6" spans="1:7" ht="20" x14ac:dyDescent="0.35">
+    <row r="6" spans="1:7" ht="20.25" x14ac:dyDescent="0.25">
       <c r="A6" s="29" t="s">
         <v>3</v>
       </c>
@@ -785,7 +785,7 @@
       <c r="F6" s="2"/>
       <c r="G6" s="2"/>
     </row>
-    <row r="7" spans="1:7" x14ac:dyDescent="0.35">
+    <row r="7" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A7" s="4" t="s">
         <v>4</v>
       </c>
@@ -806,133 +806,133 @@
         <v>9</v>
       </c>
     </row>
-    <row r="8" spans="1:7" x14ac:dyDescent="0.35">
+    <row r="8" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A8" s="7">
-        <v>46295</v>
+        <v>46296</v>
       </c>
       <c r="B8" s="8"/>
       <c r="C8" s="9" t="s">
         <v>10</v>
       </c>
       <c r="D8" s="10">
-        <v>262.06</v>
+        <v>261.42</v>
       </c>
       <c r="E8" s="10">
-        <v>229.41</v>
+        <v>230.61</v>
       </c>
       <c r="F8" s="10">
-        <v>239.42</v>
+        <v>240.61</v>
       </c>
       <c r="G8" s="10">
-        <v>229.38</v>
-      </c>
-    </row>
-    <row r="9" spans="1:7" x14ac:dyDescent="0.35">
+        <v>228.22</v>
+      </c>
+    </row>
+    <row r="9" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A9" s="11">
-        <v>46295</v>
+        <v>46296</v>
       </c>
       <c r="B9" s="12"/>
       <c r="C9" s="12" t="s">
         <v>11</v>
       </c>
       <c r="D9" s="13">
-        <v>262.06</v>
+        <v>261.42</v>
       </c>
       <c r="E9" s="13">
-        <v>229.41</v>
+        <v>230.61</v>
       </c>
       <c r="F9" s="13">
-        <v>239.42</v>
+        <v>240.61</v>
       </c>
       <c r="G9" s="13">
-        <v>229.38</v>
-      </c>
-    </row>
-    <row r="10" spans="1:7" x14ac:dyDescent="0.35">
+        <v>228.22</v>
+      </c>
+    </row>
+    <row r="10" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A10" s="7">
-        <v>46295</v>
+        <v>46296</v>
       </c>
       <c r="B10" s="8"/>
       <c r="C10" s="9" t="s">
         <v>12</v>
       </c>
       <c r="D10" s="10">
-        <v>256.99</v>
+        <v>257.22000000000003</v>
       </c>
       <c r="E10" s="10">
-        <v>226.85</v>
+        <v>227.84</v>
       </c>
       <c r="F10" s="10">
-        <v>236.85</v>
+        <v>237.84</v>
       </c>
       <c r="G10" s="10">
-        <v>227.27</v>
-      </c>
-    </row>
-    <row r="11" spans="1:7" x14ac:dyDescent="0.35">
+        <v>226.25</v>
+      </c>
+    </row>
+    <row r="11" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A11" s="11">
-        <v>46294</v>
+        <v>46295</v>
       </c>
       <c r="B11" s="12"/>
       <c r="C11" s="12" t="s">
         <v>10</v>
       </c>
       <c r="D11" s="13">
-        <v>264.13</v>
+        <v>262.06</v>
       </c>
       <c r="E11" s="13">
-        <v>228.23</v>
+        <v>229.41</v>
       </c>
       <c r="F11" s="13">
-        <v>238.23</v>
+        <v>239.42</v>
       </c>
       <c r="G11" s="13">
-        <v>228.19</v>
-      </c>
-    </row>
-    <row r="12" spans="1:7" x14ac:dyDescent="0.35">
+        <v>229.38</v>
+      </c>
+    </row>
+    <row r="12" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A12" s="7">
-        <v>46294</v>
+        <v>46295</v>
       </c>
       <c r="B12" s="8"/>
       <c r="C12" s="9" t="s">
         <v>11</v>
       </c>
       <c r="D12" s="10">
-        <v>264.13</v>
+        <v>262.06</v>
       </c>
       <c r="E12" s="10">
-        <v>228.23</v>
+        <v>229.41</v>
       </c>
       <c r="F12" s="10">
-        <v>238.23</v>
+        <v>239.42</v>
       </c>
       <c r="G12" s="10">
-        <v>228.19</v>
-      </c>
-    </row>
-    <row r="13" spans="1:7" x14ac:dyDescent="0.35">
+        <v>229.38</v>
+      </c>
+    </row>
+    <row r="13" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A13" s="11">
-        <v>46294</v>
+        <v>46295</v>
       </c>
       <c r="B13" s="12"/>
       <c r="C13" s="12" t="s">
         <v>12</v>
       </c>
       <c r="D13" s="13">
-        <v>256.04000000000002</v>
+        <v>256.99</v>
       </c>
       <c r="E13" s="13">
-        <v>225.91</v>
+        <v>226.85</v>
       </c>
       <c r="F13" s="13">
-        <v>235.91</v>
+        <v>236.85</v>
       </c>
       <c r="G13" s="13">
-        <v>226.32</v>
-      </c>
-    </row>
-    <row r="14" spans="1:7" x14ac:dyDescent="0.35">
+        <v>227.27</v>
+      </c>
+    </row>
+    <row r="14" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A14" s="14"/>
       <c r="B14" s="14"/>
       <c r="C14" s="15"/>
@@ -941,7 +941,7 @@
       <c r="F14" s="16"/>
       <c r="G14" s="16"/>
     </row>
-    <row r="15" spans="1:7" ht="20" x14ac:dyDescent="0.35">
+    <row r="15" spans="1:7" ht="20.25" x14ac:dyDescent="0.25">
       <c r="A15" s="29" t="s">
         <v>13</v>
       </c>
@@ -952,7 +952,7 @@
       <c r="F15" s="17"/>
       <c r="G15" s="17"/>
     </row>
-    <row r="16" spans="1:7" x14ac:dyDescent="0.35">
+    <row r="16" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A16" s="4" t="s">
         <v>4</v>
       </c>
@@ -971,45 +971,45 @@
       </c>
       <c r="G16" s="17"/>
     </row>
-    <row r="17" spans="1:7" x14ac:dyDescent="0.35">
+    <row r="17" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A17" s="7">
-        <v>46295</v>
+        <v>46296</v>
       </c>
       <c r="B17" s="8"/>
       <c r="C17" s="20" t="s">
         <v>14</v>
       </c>
       <c r="D17" s="10">
-        <v>261.17</v>
+        <v>261.27</v>
       </c>
       <c r="E17" s="10">
-        <v>232.65</v>
+        <v>233.53</v>
       </c>
       <c r="F17" s="10">
-        <v>242.65</v>
+        <v>243.53</v>
       </c>
       <c r="G17" s="17"/>
     </row>
-    <row r="18" spans="1:7" x14ac:dyDescent="0.35">
+    <row r="18" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A18" s="11">
-        <v>46294</v>
+        <v>46295</v>
       </c>
       <c r="B18" s="12"/>
       <c r="C18" s="12" t="s">
         <v>14</v>
       </c>
       <c r="D18" s="13">
-        <v>260.33</v>
+        <v>261.17</v>
       </c>
       <c r="E18" s="13">
-        <v>231.8</v>
+        <v>232.65</v>
       </c>
       <c r="F18" s="13">
-        <v>241.8</v>
+        <v>242.65</v>
       </c>
       <c r="G18" s="17"/>
     </row>
-    <row r="19" spans="1:7" x14ac:dyDescent="0.35">
+    <row r="19" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A19" s="14"/>
       <c r="B19" s="14"/>
       <c r="C19" s="15"/>
@@ -1018,7 +1018,7 @@
       <c r="F19" s="16"/>
       <c r="G19" s="17"/>
     </row>
-    <row r="20" spans="1:7" ht="20" x14ac:dyDescent="0.35">
+    <row r="20" spans="1:7" ht="20.25" x14ac:dyDescent="0.25">
       <c r="A20" s="29" t="s">
         <v>15</v>
       </c>
@@ -1029,7 +1029,7 @@
       <c r="F20" s="17"/>
       <c r="G20" s="17"/>
     </row>
-    <row r="21" spans="1:7" x14ac:dyDescent="0.35">
+    <row r="21" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A21" s="4" t="s">
         <v>4</v>
       </c>
@@ -1050,217 +1050,217 @@
         <v>9</v>
       </c>
     </row>
-    <row r="22" spans="1:7" x14ac:dyDescent="0.35">
+    <row r="22" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A22" s="7">
-        <v>46295</v>
+        <v>46296</v>
       </c>
       <c r="B22" s="8"/>
       <c r="C22" s="20" t="s">
         <v>16</v>
       </c>
       <c r="D22" s="10">
-        <v>263.18</v>
+        <v>262.54000000000002</v>
       </c>
       <c r="E22" s="10">
-        <v>227.91</v>
+        <v>228.55</v>
       </c>
       <c r="F22" s="10">
-        <v>237.51</v>
+        <v>238.15</v>
       </c>
       <c r="G22" s="10">
-        <v>226.62</v>
-      </c>
-    </row>
-    <row r="23" spans="1:7" x14ac:dyDescent="0.35">
+        <v>224.92</v>
+      </c>
+    </row>
+    <row r="23" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A23" s="11">
-        <v>46295</v>
+        <v>46296</v>
       </c>
       <c r="B23" s="12"/>
       <c r="C23" s="21" t="s">
         <v>17</v>
       </c>
       <c r="D23" s="13">
-        <v>261.86</v>
+        <v>262.11</v>
       </c>
       <c r="E23" s="13">
-        <v>237.06</v>
+        <v>238.1</v>
       </c>
       <c r="F23" s="13">
-        <v>247.06</v>
+        <v>248.1</v>
       </c>
       <c r="G23" s="13" t="s">
         <v>18</v>
       </c>
     </row>
-    <row r="24" spans="1:7" x14ac:dyDescent="0.35">
+    <row r="24" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A24" s="7">
-        <v>46295</v>
+        <v>46296</v>
       </c>
       <c r="B24" s="8"/>
       <c r="C24" s="20" t="s">
         <v>19</v>
       </c>
       <c r="D24" s="10">
-        <v>262.3</v>
+        <v>262.52999999999997</v>
       </c>
       <c r="E24" s="10">
-        <v>236.31</v>
+        <v>237.35</v>
       </c>
       <c r="F24" s="10">
-        <v>246.31</v>
+        <v>247.35</v>
       </c>
       <c r="G24" s="10" t="s">
         <v>18</v>
       </c>
     </row>
-    <row r="25" spans="1:7" x14ac:dyDescent="0.35">
+    <row r="25" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A25" s="11">
-        <v>46295</v>
+        <v>46296</v>
       </c>
       <c r="B25" s="12"/>
       <c r="C25" s="21" t="s">
         <v>20</v>
       </c>
       <c r="D25" s="13">
-        <v>259.01</v>
+        <v>259.22000000000003</v>
       </c>
       <c r="E25" s="13">
-        <v>236.46</v>
+        <v>237.52</v>
       </c>
       <c r="F25" s="13">
-        <v>246.46</v>
+        <v>247.52</v>
       </c>
       <c r="G25" s="13">
-        <v>234.36</v>
-      </c>
-    </row>
-    <row r="26" spans="1:7" x14ac:dyDescent="0.35">
+        <v>233.36</v>
+      </c>
+    </row>
+    <row r="26" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A26" s="7">
-        <v>46295</v>
+        <v>46296</v>
       </c>
       <c r="B26" s="8"/>
       <c r="C26" s="20" t="s">
         <v>21</v>
       </c>
       <c r="D26" s="10">
-        <v>260.69</v>
+        <v>260.88</v>
       </c>
       <c r="E26" s="10">
-        <v>237.94</v>
+        <v>239</v>
       </c>
       <c r="F26" s="10">
-        <v>247.94</v>
+        <v>249</v>
       </c>
       <c r="G26" s="10" t="s">
         <v>18</v>
       </c>
     </row>
-    <row r="27" spans="1:7" x14ac:dyDescent="0.35">
+    <row r="27" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A27" s="11">
-        <v>46294</v>
+        <v>46295</v>
       </c>
       <c r="B27" s="12"/>
       <c r="C27" s="12" t="s">
         <v>16</v>
       </c>
       <c r="D27" s="13">
-        <v>264.7</v>
+        <v>263.18</v>
       </c>
       <c r="E27" s="13">
-        <v>227.82</v>
+        <v>227.91</v>
       </c>
       <c r="F27" s="13">
-        <v>237.42</v>
+        <v>237.51</v>
       </c>
       <c r="G27" s="13">
-        <v>226.54</v>
-      </c>
-    </row>
-    <row r="28" spans="1:7" x14ac:dyDescent="0.35">
+        <v>226.62</v>
+      </c>
+    </row>
+    <row r="28" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A28" s="7">
-        <v>46294</v>
+        <v>46295</v>
       </c>
       <c r="B28" s="8"/>
       <c r="C28" s="20" t="s">
         <v>17</v>
       </c>
       <c r="D28" s="10">
-        <v>260.89999999999998</v>
+        <v>261.86</v>
       </c>
       <c r="E28" s="22">
-        <v>236.07</v>
+        <v>237.06</v>
       </c>
       <c r="F28" s="22">
-        <v>246.07</v>
+        <v>247.06</v>
       </c>
       <c r="G28" s="22" t="s">
         <v>18</v>
       </c>
     </row>
-    <row r="29" spans="1:7" x14ac:dyDescent="0.35">
+    <row r="29" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A29" s="11">
-        <v>46294</v>
+        <v>46295</v>
       </c>
       <c r="B29" s="12"/>
       <c r="C29" s="12" t="s">
         <v>19</v>
       </c>
       <c r="D29" s="13">
-        <v>261.35000000000002</v>
+        <v>262.3</v>
       </c>
       <c r="E29" s="13">
-        <v>235.33</v>
+        <v>236.31</v>
       </c>
       <c r="F29" s="13">
-        <v>245.33</v>
+        <v>246.31</v>
       </c>
       <c r="G29" s="13" t="s">
         <v>18</v>
       </c>
     </row>
-    <row r="30" spans="1:7" x14ac:dyDescent="0.35">
+    <row r="30" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A30" s="7">
-        <v>46294</v>
+        <v>46295</v>
       </c>
       <c r="B30" s="8"/>
       <c r="C30" s="20" t="s">
         <v>20</v>
       </c>
       <c r="D30" s="10">
-        <v>258.07</v>
+        <v>259.01</v>
       </c>
       <c r="E30" s="22">
-        <v>235.46</v>
+        <v>236.46</v>
       </c>
       <c r="F30" s="22">
-        <v>245.46</v>
+        <v>246.46</v>
       </c>
       <c r="G30" s="22">
-        <v>233.36</v>
-      </c>
-    </row>
-    <row r="31" spans="1:7" x14ac:dyDescent="0.35">
+        <v>234.36</v>
+      </c>
+    </row>
+    <row r="31" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A31" s="11">
-        <v>46294</v>
+        <v>46295</v>
       </c>
       <c r="B31" s="12"/>
       <c r="C31" s="12" t="s">
         <v>21</v>
       </c>
       <c r="D31" s="13">
-        <v>259.77</v>
+        <v>260.69</v>
       </c>
       <c r="E31" s="13">
-        <v>236.94</v>
+        <v>237.94</v>
       </c>
       <c r="F31" s="13">
-        <v>246.94</v>
+        <v>247.94</v>
       </c>
       <c r="G31" s="13" t="s">
         <v>18</v>
       </c>
     </row>
-    <row r="32" spans="1:7" x14ac:dyDescent="0.35">
+    <row r="32" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A32" s="14"/>
       <c r="B32" s="14"/>
       <c r="C32" s="15"/>
@@ -1269,7 +1269,7 @@
       <c r="F32" s="17"/>
       <c r="G32" s="17"/>
     </row>
-    <row r="33" spans="1:7" ht="20" x14ac:dyDescent="0.35">
+    <row r="33" spans="1:7" ht="20.25" x14ac:dyDescent="0.25">
       <c r="A33" s="29" t="s">
         <v>22</v>
       </c>
@@ -1280,7 +1280,7 @@
       <c r="F33" s="17"/>
       <c r="G33" s="17"/>
     </row>
-    <row r="34" spans="1:7" x14ac:dyDescent="0.35">
+    <row r="34" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A34" s="23" t="s">
         <v>4</v>
       </c>
@@ -1299,54 +1299,54 @@
       </c>
       <c r="G34" s="17"/>
     </row>
-    <row r="35" spans="1:7" x14ac:dyDescent="0.35">
+    <row r="35" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A35" s="7">
-        <v>46295</v>
+        <v>46296</v>
       </c>
       <c r="B35" s="8"/>
       <c r="C35" s="20" t="s">
         <v>23</v>
       </c>
       <c r="D35" s="10">
-        <v>255.53</v>
+        <v>255.76</v>
       </c>
       <c r="E35" s="10">
-        <v>224.68</v>
+        <v>225.67</v>
       </c>
       <c r="F35" s="10">
-        <v>233.68</v>
+        <v>234.67</v>
       </c>
       <c r="G35" s="17"/>
     </row>
-    <row r="36" spans="1:7" x14ac:dyDescent="0.35">
+    <row r="36" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A36" s="11">
-        <v>46294</v>
+        <v>46295</v>
       </c>
       <c r="B36" s="12"/>
       <c r="C36" s="12" t="s">
         <v>23</v>
       </c>
       <c r="D36" s="13">
-        <v>254.58</v>
+        <v>255.53</v>
       </c>
       <c r="E36" s="13">
-        <v>223.74</v>
+        <v>224.68</v>
       </c>
       <c r="F36" s="13">
-        <v>232.74</v>
+        <v>233.68</v>
       </c>
       <c r="G36" s="17"/>
     </row>
-    <row r="37" spans="1:7" x14ac:dyDescent="0.35">
+    <row r="37" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A37" s="7">
-        <v>46295</v>
+        <v>46296</v>
       </c>
       <c r="B37" s="8"/>
       <c r="C37" s="20" t="s">
         <v>24</v>
       </c>
       <c r="D37" s="10">
-        <v>271.14999999999998</v>
+        <v>271.38</v>
       </c>
       <c r="E37" s="10" t="s">
         <v>18</v>
@@ -1356,16 +1356,16 @@
       </c>
       <c r="G37" s="17"/>
     </row>
-    <row r="38" spans="1:7" x14ac:dyDescent="0.35">
+    <row r="38" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A38" s="11">
-        <v>46294</v>
+        <v>46295</v>
       </c>
       <c r="B38" s="12"/>
       <c r="C38" s="12" t="s">
         <v>24</v>
       </c>
       <c r="D38" s="13">
-        <v>270.2</v>
+        <v>271.14999999999998</v>
       </c>
       <c r="E38" s="13" t="s">
         <v>18</v>
@@ -1375,7 +1375,7 @@
       </c>
       <c r="G38" s="17"/>
     </row>
-    <row r="39" spans="1:7" x14ac:dyDescent="0.35">
+    <row r="39" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A39" s="24"/>
       <c r="B39" s="24"/>
       <c r="C39" s="15"/>
@@ -1384,7 +1384,7 @@
       <c r="F39" s="17"/>
       <c r="G39" s="17"/>
     </row>
-    <row r="40" spans="1:7" ht="20" x14ac:dyDescent="0.35">
+    <row r="40" spans="1:7" ht="20.25" x14ac:dyDescent="0.25">
       <c r="A40" s="29" t="s">
         <v>25</v>
       </c>
@@ -1395,7 +1395,7 @@
       <c r="F40" s="17"/>
       <c r="G40" s="17"/>
     </row>
-    <row r="41" spans="1:7" x14ac:dyDescent="0.35">
+    <row r="41" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A41" s="23" t="s">
         <v>4</v>
       </c>
@@ -1414,83 +1414,83 @@
       </c>
       <c r="G41" s="17"/>
     </row>
-    <row r="42" spans="1:7" x14ac:dyDescent="0.35">
+    <row r="42" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A42" s="7">
-        <v>46295</v>
+        <v>46296</v>
       </c>
       <c r="B42" s="8"/>
       <c r="C42" s="20" t="s">
         <v>26</v>
       </c>
       <c r="D42" s="10">
-        <v>265</v>
+        <v>265.32</v>
       </c>
       <c r="E42" s="10">
-        <v>233.1</v>
+        <v>234.18</v>
       </c>
       <c r="F42" s="10">
-        <v>243.1</v>
+        <v>244.18</v>
       </c>
       <c r="G42" s="17"/>
     </row>
-    <row r="43" spans="1:7" x14ac:dyDescent="0.35">
+    <row r="43" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A43" s="11">
-        <v>46295</v>
+        <v>46296</v>
       </c>
       <c r="B43" s="12"/>
       <c r="C43" s="21" t="s">
         <v>27</v>
       </c>
       <c r="D43" s="13">
-        <v>264.61</v>
+        <v>264.93</v>
       </c>
       <c r="E43" s="13">
-        <v>233.51</v>
+        <v>234.6</v>
       </c>
       <c r="F43" s="13">
-        <v>243.51</v>
+        <v>244.6</v>
       </c>
       <c r="G43" s="17"/>
     </row>
-    <row r="44" spans="1:7" x14ac:dyDescent="0.35">
+    <row r="44" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A44" s="7">
-        <v>46294</v>
+        <v>46295</v>
       </c>
       <c r="B44" s="8"/>
       <c r="C44" s="20" t="s">
         <v>26</v>
       </c>
       <c r="D44" s="10">
-        <v>263.95999999999998</v>
+        <v>265</v>
       </c>
       <c r="E44" s="10">
-        <v>232.08</v>
+        <v>233.1</v>
       </c>
       <c r="F44" s="10">
-        <v>242.08</v>
+        <v>243.1</v>
       </c>
       <c r="G44" s="17"/>
     </row>
-    <row r="45" spans="1:7" x14ac:dyDescent="0.35">
+    <row r="45" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A45" s="11">
-        <v>46294</v>
+        <v>46295</v>
       </c>
       <c r="B45" s="12"/>
       <c r="C45" s="21" t="s">
         <v>27</v>
       </c>
       <c r="D45" s="13">
-        <v>263.57</v>
+        <v>264.61</v>
       </c>
       <c r="E45" s="13">
-        <v>232.49</v>
+        <v>233.51</v>
       </c>
       <c r="F45" s="13">
-        <v>242.49</v>
+        <v>243.51</v>
       </c>
       <c r="G45" s="17"/>
     </row>
-    <row r="46" spans="1:7" x14ac:dyDescent="0.35">
+    <row r="46" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A46" s="14"/>
       <c r="B46" s="24"/>
       <c r="C46" s="15"/>
@@ -1499,7 +1499,7 @@
       <c r="F46" s="16"/>
       <c r="G46" s="17"/>
     </row>
-    <row r="47" spans="1:7" ht="20" x14ac:dyDescent="0.35">
+    <row r="47" spans="1:7" ht="20.25" x14ac:dyDescent="0.25">
       <c r="A47" s="25" t="s">
         <v>28</v>
       </c>
@@ -1510,7 +1510,7 @@
       <c r="F47" s="17"/>
       <c r="G47" s="17"/>
     </row>
-    <row r="48" spans="1:7" x14ac:dyDescent="0.35">
+    <row r="48" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A48" s="23" t="s">
         <v>4</v>
       </c>
@@ -1529,83 +1529,83 @@
       </c>
       <c r="G48" s="17"/>
     </row>
-    <row r="49" spans="1:7" x14ac:dyDescent="0.35">
+    <row r="49" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A49" s="7">
-        <v>46295</v>
+        <v>46296</v>
       </c>
       <c r="B49" s="8"/>
       <c r="C49" s="20" t="s">
         <v>29</v>
       </c>
       <c r="D49" s="10">
-        <v>257.52</v>
+        <v>256.32</v>
       </c>
       <c r="E49" s="10">
-        <v>229.12</v>
+        <v>229.42</v>
       </c>
       <c r="F49" s="10">
-        <v>239.12</v>
+        <v>239.42</v>
       </c>
       <c r="G49" s="28"/>
     </row>
-    <row r="50" spans="1:7" x14ac:dyDescent="0.35">
+    <row r="50" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A50" s="11">
-        <v>46295</v>
+        <v>46296</v>
       </c>
       <c r="B50" s="12"/>
       <c r="C50" s="21" t="s">
         <v>30</v>
       </c>
       <c r="D50" s="13">
-        <v>255.34</v>
+        <v>254.09</v>
       </c>
       <c r="E50" s="13">
-        <v>228.88</v>
+        <v>229.16</v>
       </c>
       <c r="F50" s="13">
-        <v>238.88</v>
+        <v>239.16</v>
       </c>
       <c r="G50" s="28"/>
     </row>
-    <row r="51" spans="1:7" x14ac:dyDescent="0.35">
+    <row r="51" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A51" s="7">
-        <v>46294</v>
+        <v>46295</v>
       </c>
       <c r="B51" s="8"/>
       <c r="C51" s="20" t="s">
         <v>29</v>
       </c>
       <c r="D51" s="10">
-        <v>259.01</v>
+        <v>257.52</v>
       </c>
       <c r="E51" s="10">
-        <v>228.95</v>
+        <v>229.12</v>
       </c>
       <c r="F51" s="10">
-        <v>238.95</v>
+        <v>239.12</v>
       </c>
       <c r="G51" s="17"/>
     </row>
-    <row r="52" spans="1:7" x14ac:dyDescent="0.35">
+    <row r="52" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A52" s="11">
-        <v>46294</v>
+        <v>46295</v>
       </c>
       <c r="B52" s="12"/>
       <c r="C52" s="21" t="s">
         <v>30</v>
       </c>
       <c r="D52" s="13">
-        <v>256.86</v>
+        <v>255.34</v>
       </c>
       <c r="E52" s="13">
-        <v>228.72</v>
+        <v>228.88</v>
       </c>
       <c r="F52" s="13">
-        <v>238.72</v>
+        <v>238.88</v>
       </c>
       <c r="G52" s="17"/>
     </row>
-    <row r="53" spans="1:7" x14ac:dyDescent="0.35">
+    <row r="53" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A53" s="14"/>
       <c r="B53" s="14"/>
       <c r="C53" s="15"/>
@@ -1614,7 +1614,7 @@
       <c r="F53" s="16"/>
       <c r="G53" s="17"/>
     </row>
-    <row r="54" spans="1:7" ht="20" x14ac:dyDescent="0.35">
+    <row r="54" spans="1:7" ht="20.25" x14ac:dyDescent="0.25">
       <c r="A54" s="27" t="s">
         <v>31</v>
       </c>
@@ -1625,7 +1625,7 @@
       <c r="F54" s="17"/>
       <c r="G54" s="17"/>
     </row>
-    <row r="55" spans="1:7" x14ac:dyDescent="0.35">
+    <row r="55" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A55" s="23" t="s">
         <v>4</v>
       </c>
@@ -1644,54 +1644,54 @@
       </c>
       <c r="G55" s="17"/>
     </row>
-    <row r="56" spans="1:7" x14ac:dyDescent="0.35">
+    <row r="56" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A56" s="7">
-        <v>46295</v>
+        <v>46296</v>
       </c>
       <c r="B56" s="8"/>
       <c r="C56" s="20" t="s">
         <v>32</v>
       </c>
       <c r="D56" s="10">
-        <v>273.52</v>
+        <v>273.72000000000003</v>
       </c>
       <c r="E56" s="10">
-        <v>252.78</v>
+        <v>254.29</v>
       </c>
       <c r="F56" s="10">
-        <v>262.77999999999997</v>
+        <v>264.29000000000002</v>
       </c>
       <c r="G56" s="17"/>
     </row>
-    <row r="57" spans="1:7" x14ac:dyDescent="0.35">
+    <row r="57" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A57" s="11">
-        <v>46295</v>
+        <v>46296</v>
       </c>
       <c r="B57" s="12"/>
       <c r="C57" s="21" t="s">
         <v>33</v>
       </c>
       <c r="D57" s="13">
-        <v>262.66000000000003</v>
+        <v>262.89999999999998</v>
       </c>
       <c r="E57" s="13">
-        <v>237.95</v>
+        <v>238.81</v>
       </c>
       <c r="F57" s="13">
-        <v>247.95</v>
+        <v>248.81</v>
       </c>
       <c r="G57" s="17"/>
     </row>
-    <row r="58" spans="1:7" x14ac:dyDescent="0.35">
+    <row r="58" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A58" s="7">
-        <v>46295</v>
+        <v>46296</v>
       </c>
       <c r="B58" s="8"/>
       <c r="C58" s="20" t="s">
         <v>34</v>
       </c>
       <c r="D58" s="10">
-        <v>263.99</v>
+        <v>264.24</v>
       </c>
       <c r="E58" s="10" t="s">
         <v>18</v>
@@ -1701,111 +1701,111 @@
       </c>
       <c r="G58" s="17"/>
     </row>
-    <row r="59" spans="1:7" x14ac:dyDescent="0.35">
+    <row r="59" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A59" s="11">
-        <v>46295</v>
+        <v>46296</v>
       </c>
       <c r="B59" s="12"/>
       <c r="C59" s="21" t="s">
         <v>35</v>
       </c>
       <c r="D59" s="13">
-        <v>259.2</v>
+        <v>259.27</v>
       </c>
       <c r="E59" s="13">
-        <v>232.32</v>
+        <v>233.18</v>
       </c>
       <c r="F59" s="13" t="s">
         <v>18</v>
       </c>
       <c r="G59" s="17"/>
     </row>
-    <row r="60" spans="1:7" x14ac:dyDescent="0.35">
+    <row r="60" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A60" s="7">
-        <v>46295</v>
+        <v>46296</v>
       </c>
       <c r="B60" s="8"/>
       <c r="C60" s="20" t="s">
         <v>36</v>
       </c>
       <c r="D60" s="10">
-        <v>255.03</v>
+        <v>255.1</v>
       </c>
       <c r="E60" s="10">
-        <v>228.27</v>
+        <v>229.13</v>
       </c>
       <c r="F60" s="10">
-        <v>238.27</v>
+        <v>239.13</v>
       </c>
       <c r="G60" s="17"/>
     </row>
-    <row r="61" spans="1:7" x14ac:dyDescent="0.35">
+    <row r="61" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A61" s="11">
-        <v>46295</v>
+        <v>46296</v>
       </c>
       <c r="B61" s="12"/>
       <c r="C61" s="21" t="s">
         <v>37</v>
       </c>
       <c r="D61" s="13">
-        <v>260.45999999999998</v>
+        <v>260.51</v>
       </c>
       <c r="E61" s="13">
-        <v>247.41</v>
+        <v>248.7</v>
       </c>
       <c r="F61" s="13" t="s">
         <v>18</v>
       </c>
       <c r="G61" s="17"/>
     </row>
-    <row r="62" spans="1:7" x14ac:dyDescent="0.35">
+    <row r="62" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A62" s="7">
-        <v>46294</v>
+        <v>46295</v>
       </c>
       <c r="B62" s="8"/>
       <c r="C62" s="20" t="s">
         <v>32</v>
       </c>
       <c r="D62" s="10">
-        <v>272.58999999999997</v>
+        <v>273.52</v>
       </c>
       <c r="E62" s="10">
-        <v>251.4</v>
+        <v>252.78</v>
       </c>
       <c r="F62" s="10">
-        <v>261.39999999999998</v>
+        <v>262.77999999999997</v>
       </c>
       <c r="G62" s="17"/>
     </row>
-    <row r="63" spans="1:7" x14ac:dyDescent="0.35">
+    <row r="63" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A63" s="11">
-        <v>46294</v>
+        <v>46295</v>
       </c>
       <c r="B63" s="12"/>
       <c r="C63" s="21" t="s">
         <v>33</v>
       </c>
       <c r="D63" s="13">
-        <v>261.7</v>
+        <v>262.66000000000003</v>
       </c>
       <c r="E63" s="13">
-        <v>237.12</v>
+        <v>237.95</v>
       </c>
       <c r="F63" s="13">
-        <v>247.12</v>
+        <v>247.95</v>
       </c>
       <c r="G63" s="17"/>
     </row>
-    <row r="64" spans="1:7" x14ac:dyDescent="0.35">
+    <row r="64" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A64" s="7">
-        <v>46294</v>
+        <v>46295</v>
       </c>
       <c r="B64" s="8"/>
       <c r="C64" s="20" t="s">
         <v>34</v>
       </c>
       <c r="D64" s="10">
-        <v>263.01</v>
+        <v>263.99</v>
       </c>
       <c r="E64" s="10" t="s">
         <v>18</v>
@@ -1815,55 +1815,55 @@
       </c>
       <c r="G64" s="17"/>
     </row>
-    <row r="65" spans="1:6" x14ac:dyDescent="0.35">
+    <row r="65" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A65" s="11">
-        <v>46294</v>
+        <v>46295</v>
       </c>
       <c r="B65" s="12"/>
       <c r="C65" s="21" t="s">
         <v>35</v>
       </c>
       <c r="D65" s="13">
-        <v>258.38</v>
+        <v>259.2</v>
       </c>
       <c r="E65" s="13">
-        <v>231.5</v>
+        <v>232.32</v>
       </c>
       <c r="F65" s="13" t="s">
         <v>18</v>
       </c>
     </row>
-    <row r="66" spans="1:6" x14ac:dyDescent="0.35">
+    <row r="66" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A66" s="7">
-        <v>46294</v>
+        <v>46295</v>
       </c>
       <c r="B66" s="8"/>
       <c r="C66" s="20" t="s">
         <v>36</v>
       </c>
       <c r="D66" s="10">
-        <v>254.21</v>
+        <v>255.03</v>
       </c>
       <c r="E66" s="10">
-        <v>227.44</v>
+        <v>228.27</v>
       </c>
       <c r="F66" s="10">
-        <v>237.44</v>
-      </c>
-    </row>
-    <row r="67" spans="1:6" x14ac:dyDescent="0.35">
+        <v>238.27</v>
+      </c>
+    </row>
+    <row r="67" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A67" s="11">
-        <v>46294</v>
+        <v>46295</v>
       </c>
       <c r="B67" s="12"/>
       <c r="C67" s="21" t="s">
         <v>37</v>
       </c>
       <c r="D67" s="13">
-        <v>259.64999999999998</v>
+        <v>260.45999999999998</v>
       </c>
       <c r="E67" s="13">
-        <v>246.21</v>
+        <v>247.41</v>
       </c>
       <c r="F67" s="13" t="s">
         <v>18</v>
@@ -1891,15 +1891,6 @@
 </file>
 
 <file path=customXml/item1.xml><?xml version="1.0" encoding="utf-8"?>
-<?mso-contentType ?>
-<FormTemplates xmlns="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms">
-  <Display>DocumentLibraryForm</Display>
-  <Edit>DocumentLibraryForm</Edit>
-  <New>DocumentLibraryForm</New>
-</FormTemplates>
-</file>
-
-<file path=customXml/item2.xml><?xml version="1.0" encoding="utf-8"?>
 <p:properties xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls">
   <documentManagement>
     <lcf76f155ced4ddcb4097134ff3c332f xmlns="87276d81-85f4-4ef2-9e6e-55066304288f">
@@ -1908,6 +1899,15 @@
     <TaxCatchAll xmlns="b23b8984-eafa-4e79-985e-54f52f3da58e" xsi:nil="true"/>
   </documentManagement>
 </p:properties>
+</file>
+
+<file path=customXml/item2.xml><?xml version="1.0" encoding="utf-8"?>
+<?mso-contentType ?>
+<FormTemplates xmlns="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms">
+  <Display>DocumentLibraryForm</Display>
+  <Edit>DocumentLibraryForm</Edit>
+  <New>DocumentLibraryForm</New>
+</FormTemplates>
 </file>
 
 <file path=customXml/item3.xml><?xml version="1.0" encoding="utf-8"?>
@@ -2171,20 +2171,20 @@
 </file>
 
 <file path=customXml/itemProps1.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{F60519E9-FD90-4339-869C-BC2F85719BB8}">
-  <ds:schemaRefs>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms"/>
-  </ds:schemaRefs>
-</ds:datastoreItem>
-</file>
-
-<file path=customXml/itemProps2.xml><?xml version="1.0" encoding="utf-8"?>
 <ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{57A83D98-2BAE-4D83-823A-D31C464B620C}">
   <ds:schemaRefs>
     <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/properties"/>
     <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
     <ds:schemaRef ds:uri="87276d81-85f4-4ef2-9e6e-55066304288f"/>
     <ds:schemaRef ds:uri="b23b8984-eafa-4e79-985e-54f52f3da58e"/>
+  </ds:schemaRefs>
+</ds:datastoreItem>
+</file>
+
+<file path=customXml/itemProps2.xml><?xml version="1.0" encoding="utf-8"?>
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{F60519E9-FD90-4339-869C-BC2F85719BB8}">
+  <ds:schemaRefs>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms"/>
   </ds:schemaRefs>
 </ds:datastoreItem>
 </file>

</xml_diff>

<commit_message>
Thu Oct  1 07:18:30 UTC 2026
</commit_message>
<xml_diff>
--- a/bp.com-content-dam-bp-country-sites-en_au-australia-home-products-services-pricing-tgp-excel.xlsx
+++ b/bp.com-content-dam-bp-country-sites-en_au-australia-home-products-services-pricing-tgp-excel.xlsx
@@ -8,14 +8,14 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://bp365.sharepoint.com/sites/WholesalePricing/Shared Documents/B2C/TGP/Daily TGP/Web TGP/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="14_{A8CA0E1F-F5B4-4C8C-94C1-F03920793B08}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="14_{2A783A92-666D-4996-9693-5633558FB425}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-28920" yWindow="-60" windowWidth="29040" windowHeight="15720" xr2:uid="{1B412EEF-F96D-4DF4-A4E9-C7F0F183C2FB}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
   </sheets>
-  <calcPr calcId="191028"/>
+  <calcPr calcId="191028" concurrentManualCount="12"/>
   <extLst>
     <ext xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" uri="{140A7094-0E35-4892-8432-C4D2E57EDEB5}">
       <x15:workbookPr chartTrackingRefBase="1"/>
@@ -808,128 +808,128 @@
     </row>
     <row r="8" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A8" s="7">
-        <v>46296</v>
+        <v>46297</v>
       </c>
       <c r="B8" s="8"/>
       <c r="C8" s="9" t="s">
         <v>10</v>
       </c>
       <c r="D8" s="10">
-        <v>261.42</v>
+        <v>261.19</v>
       </c>
       <c r="E8" s="10">
-        <v>230.61</v>
+        <v>232.14</v>
       </c>
       <c r="F8" s="10">
-        <v>240.61</v>
+        <v>242.14</v>
       </c>
       <c r="G8" s="10">
-        <v>228.22</v>
+        <v>229.75</v>
       </c>
     </row>
     <row r="9" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A9" s="11">
-        <v>46296</v>
+        <v>46297</v>
       </c>
       <c r="B9" s="12"/>
       <c r="C9" s="12" t="s">
         <v>11</v>
       </c>
       <c r="D9" s="13">
-        <v>261.42</v>
+        <v>261.19</v>
       </c>
       <c r="E9" s="13">
-        <v>230.61</v>
+        <v>232.14</v>
       </c>
       <c r="F9" s="13">
-        <v>240.61</v>
+        <v>242.14</v>
       </c>
       <c r="G9" s="13">
-        <v>228.22</v>
+        <v>229.75</v>
       </c>
     </row>
     <row r="10" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A10" s="7">
-        <v>46296</v>
+        <v>46297</v>
       </c>
       <c r="B10" s="8"/>
       <c r="C10" s="9" t="s">
         <v>12</v>
       </c>
       <c r="D10" s="10">
-        <v>257.22000000000003</v>
+        <v>256.83</v>
       </c>
       <c r="E10" s="10">
-        <v>227.84</v>
+        <v>229.24</v>
       </c>
       <c r="F10" s="10">
-        <v>237.84</v>
+        <v>239.24</v>
       </c>
       <c r="G10" s="10">
-        <v>226.25</v>
+        <v>227.64</v>
       </c>
     </row>
     <row r="11" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A11" s="11">
-        <v>46295</v>
+        <v>46296</v>
       </c>
       <c r="B11" s="12"/>
       <c r="C11" s="12" t="s">
         <v>10</v>
       </c>
       <c r="D11" s="13">
-        <v>262.06</v>
+        <v>261.42</v>
       </c>
       <c r="E11" s="13">
-        <v>229.41</v>
+        <v>230.61</v>
       </c>
       <c r="F11" s="13">
-        <v>239.42</v>
+        <v>240.61</v>
       </c>
       <c r="G11" s="13">
-        <v>229.38</v>
+        <v>228.22</v>
       </c>
     </row>
     <row r="12" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A12" s="7">
-        <v>46295</v>
+        <v>46296</v>
       </c>
       <c r="B12" s="8"/>
       <c r="C12" s="9" t="s">
         <v>11</v>
       </c>
       <c r="D12" s="10">
-        <v>262.06</v>
+        <v>261.42</v>
       </c>
       <c r="E12" s="10">
-        <v>229.41</v>
+        <v>230.61</v>
       </c>
       <c r="F12" s="10">
-        <v>239.42</v>
+        <v>240.61</v>
       </c>
       <c r="G12" s="10">
-        <v>229.38</v>
+        <v>228.22</v>
       </c>
     </row>
     <row r="13" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A13" s="11">
-        <v>46295</v>
+        <v>46296</v>
       </c>
       <c r="B13" s="12"/>
       <c r="C13" s="12" t="s">
         <v>12</v>
       </c>
       <c r="D13" s="13">
-        <v>256.99</v>
+        <v>257.22000000000003</v>
       </c>
       <c r="E13" s="13">
-        <v>226.85</v>
+        <v>227.84</v>
       </c>
       <c r="F13" s="13">
-        <v>236.85</v>
+        <v>237.84</v>
       </c>
       <c r="G13" s="13">
-        <v>227.27</v>
+        <v>226.25</v>
       </c>
     </row>
     <row r="14" spans="1:7" x14ac:dyDescent="0.25">
@@ -973,39 +973,39 @@
     </row>
     <row r="17" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A17" s="7">
-        <v>46296</v>
+        <v>46297</v>
       </c>
       <c r="B17" s="8"/>
       <c r="C17" s="20" t="s">
         <v>14</v>
       </c>
       <c r="D17" s="10">
-        <v>261.27</v>
+        <v>260.76</v>
       </c>
       <c r="E17" s="10">
-        <v>233.53</v>
+        <v>234.83</v>
       </c>
       <c r="F17" s="10">
-        <v>243.53</v>
+        <v>244.83</v>
       </c>
       <c r="G17" s="17"/>
     </row>
     <row r="18" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A18" s="11">
-        <v>46295</v>
+        <v>46296</v>
       </c>
       <c r="B18" s="12"/>
       <c r="C18" s="12" t="s">
         <v>14</v>
       </c>
       <c r="D18" s="13">
-        <v>261.17</v>
+        <v>261.27</v>
       </c>
       <c r="E18" s="13">
-        <v>232.65</v>
+        <v>233.53</v>
       </c>
       <c r="F18" s="13">
-        <v>242.65</v>
+        <v>243.53</v>
       </c>
       <c r="G18" s="17"/>
     </row>
@@ -1052,41 +1052,41 @@
     </row>
     <row r="22" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A22" s="7">
-        <v>46296</v>
+        <v>46297</v>
       </c>
       <c r="B22" s="8"/>
       <c r="C22" s="20" t="s">
         <v>16</v>
       </c>
       <c r="D22" s="10">
-        <v>262.54000000000002</v>
+        <v>262.31</v>
       </c>
       <c r="E22" s="10">
-        <v>228.55</v>
+        <v>230.08</v>
       </c>
       <c r="F22" s="10">
-        <v>238.15</v>
+        <v>239.68</v>
       </c>
       <c r="G22" s="10">
-        <v>224.92</v>
+        <v>226.45</v>
       </c>
     </row>
     <row r="23" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A23" s="11">
-        <v>46296</v>
+        <v>46297</v>
       </c>
       <c r="B23" s="12"/>
       <c r="C23" s="21" t="s">
         <v>17</v>
       </c>
       <c r="D23" s="13">
-        <v>262.11</v>
+        <v>261.73</v>
       </c>
       <c r="E23" s="13">
-        <v>238.1</v>
+        <v>239.55</v>
       </c>
       <c r="F23" s="13">
-        <v>248.1</v>
+        <v>249.55</v>
       </c>
       <c r="G23" s="13" t="s">
         <v>18</v>
@@ -1094,20 +1094,20 @@
     </row>
     <row r="24" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A24" s="7">
-        <v>46296</v>
+        <v>46297</v>
       </c>
       <c r="B24" s="8"/>
       <c r="C24" s="20" t="s">
         <v>19</v>
       </c>
       <c r="D24" s="10">
-        <v>262.52999999999997</v>
+        <v>262.14</v>
       </c>
       <c r="E24" s="10">
-        <v>237.35</v>
+        <v>238.79</v>
       </c>
       <c r="F24" s="10">
-        <v>247.35</v>
+        <v>248.79</v>
       </c>
       <c r="G24" s="10" t="s">
         <v>18</v>
@@ -1115,41 +1115,41 @@
     </row>
     <row r="25" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A25" s="11">
-        <v>46296</v>
+        <v>46297</v>
       </c>
       <c r="B25" s="12"/>
       <c r="C25" s="21" t="s">
         <v>20</v>
       </c>
       <c r="D25" s="13">
-        <v>259.22000000000003</v>
+        <v>258.82</v>
       </c>
       <c r="E25" s="13">
-        <v>237.52</v>
+        <v>238.97</v>
       </c>
       <c r="F25" s="13">
-        <v>247.52</v>
+        <v>248.97</v>
       </c>
       <c r="G25" s="13">
-        <v>233.36</v>
+        <v>234.81</v>
       </c>
     </row>
     <row r="26" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A26" s="7">
-        <v>46296</v>
+        <v>46297</v>
       </c>
       <c r="B26" s="8"/>
       <c r="C26" s="20" t="s">
         <v>21</v>
       </c>
       <c r="D26" s="10">
-        <v>260.88</v>
+        <v>260.47000000000003</v>
       </c>
       <c r="E26" s="10">
-        <v>239</v>
+        <v>240.47</v>
       </c>
       <c r="F26" s="10">
-        <v>249</v>
+        <v>250.47</v>
       </c>
       <c r="G26" s="10" t="s">
         <v>18</v>
@@ -1157,41 +1157,41 @@
     </row>
     <row r="27" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A27" s="11">
-        <v>46295</v>
+        <v>46296</v>
       </c>
       <c r="B27" s="12"/>
       <c r="C27" s="12" t="s">
         <v>16</v>
       </c>
       <c r="D27" s="13">
-        <v>263.18</v>
+        <v>262.54000000000002</v>
       </c>
       <c r="E27" s="13">
-        <v>227.91</v>
+        <v>228.55</v>
       </c>
       <c r="F27" s="13">
-        <v>237.51</v>
+        <v>238.15</v>
       </c>
       <c r="G27" s="13">
-        <v>226.62</v>
+        <v>224.92</v>
       </c>
     </row>
     <row r="28" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A28" s="7">
-        <v>46295</v>
+        <v>46296</v>
       </c>
       <c r="B28" s="8"/>
       <c r="C28" s="20" t="s">
         <v>17</v>
       </c>
       <c r="D28" s="10">
-        <v>261.86</v>
+        <v>262.11</v>
       </c>
       <c r="E28" s="22">
-        <v>237.06</v>
+        <v>238.1</v>
       </c>
       <c r="F28" s="22">
-        <v>247.06</v>
+        <v>248.1</v>
       </c>
       <c r="G28" s="22" t="s">
         <v>18</v>
@@ -1199,20 +1199,20 @@
     </row>
     <row r="29" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A29" s="11">
-        <v>46295</v>
+        <v>46296</v>
       </c>
       <c r="B29" s="12"/>
       <c r="C29" s="12" t="s">
         <v>19</v>
       </c>
       <c r="D29" s="13">
-        <v>262.3</v>
+        <v>262.52999999999997</v>
       </c>
       <c r="E29" s="13">
-        <v>236.31</v>
+        <v>237.35</v>
       </c>
       <c r="F29" s="13">
-        <v>246.31</v>
+        <v>247.35</v>
       </c>
       <c r="G29" s="13" t="s">
         <v>18</v>
@@ -1220,41 +1220,41 @@
     </row>
     <row r="30" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A30" s="7">
-        <v>46295</v>
+        <v>46296</v>
       </c>
       <c r="B30" s="8"/>
       <c r="C30" s="20" t="s">
         <v>20</v>
       </c>
       <c r="D30" s="10">
-        <v>259.01</v>
+        <v>259.22000000000003</v>
       </c>
       <c r="E30" s="22">
-        <v>236.46</v>
+        <v>237.52</v>
       </c>
       <c r="F30" s="22">
-        <v>246.46</v>
+        <v>247.52</v>
       </c>
       <c r="G30" s="22">
-        <v>234.36</v>
+        <v>233.36</v>
       </c>
     </row>
     <row r="31" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A31" s="11">
-        <v>46295</v>
+        <v>46296</v>
       </c>
       <c r="B31" s="12"/>
       <c r="C31" s="12" t="s">
         <v>21</v>
       </c>
       <c r="D31" s="13">
-        <v>260.69</v>
+        <v>260.88</v>
       </c>
       <c r="E31" s="13">
-        <v>237.94</v>
+        <v>239</v>
       </c>
       <c r="F31" s="13">
-        <v>247.94</v>
+        <v>249</v>
       </c>
       <c r="G31" s="13" t="s">
         <v>18</v>
@@ -1301,52 +1301,52 @@
     </row>
     <row r="35" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A35" s="7">
-        <v>46296</v>
+        <v>46297</v>
       </c>
       <c r="B35" s="8"/>
       <c r="C35" s="20" t="s">
         <v>23</v>
       </c>
       <c r="D35" s="10">
-        <v>255.76</v>
+        <v>255.37</v>
       </c>
       <c r="E35" s="10">
-        <v>225.67</v>
+        <v>227.07</v>
       </c>
       <c r="F35" s="10">
-        <v>234.67</v>
+        <v>236.07</v>
       </c>
       <c r="G35" s="17"/>
     </row>
     <row r="36" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A36" s="11">
-        <v>46295</v>
+        <v>46296</v>
       </c>
       <c r="B36" s="12"/>
       <c r="C36" s="12" t="s">
         <v>23</v>
       </c>
       <c r="D36" s="13">
-        <v>255.53</v>
+        <v>255.76</v>
       </c>
       <c r="E36" s="13">
-        <v>224.68</v>
+        <v>225.67</v>
       </c>
       <c r="F36" s="13">
-        <v>233.68</v>
+        <v>234.67</v>
       </c>
       <c r="G36" s="17"/>
     </row>
     <row r="37" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A37" s="7">
-        <v>46296</v>
+        <v>46297</v>
       </c>
       <c r="B37" s="8"/>
       <c r="C37" s="20" t="s">
         <v>24</v>
       </c>
       <c r="D37" s="10">
-        <v>271.38</v>
+        <v>270.99</v>
       </c>
       <c r="E37" s="10" t="s">
         <v>18</v>
@@ -1358,14 +1358,14 @@
     </row>
     <row r="38" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A38" s="11">
-        <v>46295</v>
+        <v>46296</v>
       </c>
       <c r="B38" s="12"/>
       <c r="C38" s="12" t="s">
         <v>24</v>
       </c>
       <c r="D38" s="13">
-        <v>271.14999999999998</v>
+        <v>271.38</v>
       </c>
       <c r="E38" s="13" t="s">
         <v>18</v>
@@ -1416,77 +1416,77 @@
     </row>
     <row r="42" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A42" s="7">
-        <v>46296</v>
+        <v>46297</v>
       </c>
       <c r="B42" s="8"/>
       <c r="C42" s="20" t="s">
         <v>26</v>
       </c>
       <c r="D42" s="10">
-        <v>265.32</v>
+        <v>265.02999999999997</v>
       </c>
       <c r="E42" s="10">
-        <v>234.18</v>
+        <v>235.66</v>
       </c>
       <c r="F42" s="10">
-        <v>244.18</v>
+        <v>245.66</v>
       </c>
       <c r="G42" s="17"/>
     </row>
     <row r="43" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A43" s="11">
-        <v>46296</v>
+        <v>46297</v>
       </c>
       <c r="B43" s="12"/>
       <c r="C43" s="21" t="s">
         <v>27</v>
       </c>
       <c r="D43" s="13">
-        <v>264.93</v>
+        <v>264.64</v>
       </c>
       <c r="E43" s="13">
-        <v>234.6</v>
+        <v>236.07</v>
       </c>
       <c r="F43" s="13">
-        <v>244.6</v>
+        <v>246.07</v>
       </c>
       <c r="G43" s="17"/>
     </row>
     <row r="44" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A44" s="7">
-        <v>46295</v>
+        <v>46296</v>
       </c>
       <c r="B44" s="8"/>
       <c r="C44" s="20" t="s">
         <v>26</v>
       </c>
       <c r="D44" s="10">
-        <v>265</v>
+        <v>265.32</v>
       </c>
       <c r="E44" s="10">
-        <v>233.1</v>
+        <v>234.18</v>
       </c>
       <c r="F44" s="10">
-        <v>243.1</v>
+        <v>244.18</v>
       </c>
       <c r="G44" s="17"/>
     </row>
     <row r="45" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A45" s="11">
-        <v>46295</v>
+        <v>46296</v>
       </c>
       <c r="B45" s="12"/>
       <c r="C45" s="21" t="s">
         <v>27</v>
       </c>
       <c r="D45" s="13">
-        <v>264.61</v>
+        <v>264.93</v>
       </c>
       <c r="E45" s="13">
-        <v>233.51</v>
+        <v>234.6</v>
       </c>
       <c r="F45" s="13">
-        <v>243.51</v>
+        <v>244.6</v>
       </c>
       <c r="G45" s="17"/>
     </row>
@@ -1531,77 +1531,77 @@
     </row>
     <row r="49" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A49" s="7">
-        <v>46296</v>
+        <v>46297</v>
       </c>
       <c r="B49" s="8"/>
       <c r="C49" s="20" t="s">
         <v>29</v>
       </c>
       <c r="D49" s="10">
-        <v>256.32</v>
+        <v>256.66000000000003</v>
       </c>
       <c r="E49" s="10">
-        <v>229.42</v>
+        <v>230.27</v>
       </c>
       <c r="F49" s="10">
-        <v>239.42</v>
+        <v>240.27</v>
       </c>
       <c r="G49" s="28"/>
     </row>
     <row r="50" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A50" s="11">
-        <v>46296</v>
+        <v>46297</v>
       </c>
       <c r="B50" s="12"/>
       <c r="C50" s="21" t="s">
         <v>30</v>
       </c>
       <c r="D50" s="13">
-        <v>254.09</v>
+        <v>254.39</v>
       </c>
       <c r="E50" s="13">
-        <v>229.16</v>
+        <v>229.99</v>
       </c>
       <c r="F50" s="13">
-        <v>239.16</v>
+        <v>239.99</v>
       </c>
       <c r="G50" s="28"/>
     </row>
     <row r="51" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A51" s="7">
-        <v>46295</v>
+        <v>46296</v>
       </c>
       <c r="B51" s="8"/>
       <c r="C51" s="20" t="s">
         <v>29</v>
       </c>
       <c r="D51" s="10">
-        <v>257.52</v>
+        <v>256.32</v>
       </c>
       <c r="E51" s="10">
-        <v>229.12</v>
+        <v>229.42</v>
       </c>
       <c r="F51" s="10">
-        <v>239.12</v>
+        <v>239.42</v>
       </c>
       <c r="G51" s="17"/>
     </row>
     <row r="52" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A52" s="11">
-        <v>46295</v>
+        <v>46296</v>
       </c>
       <c r="B52" s="12"/>
       <c r="C52" s="21" t="s">
         <v>30</v>
       </c>
       <c r="D52" s="13">
-        <v>255.34</v>
+        <v>254.09</v>
       </c>
       <c r="E52" s="13">
-        <v>228.88</v>
+        <v>229.16</v>
       </c>
       <c r="F52" s="13">
-        <v>238.88</v>
+        <v>239.16</v>
       </c>
       <c r="G52" s="17"/>
     </row>
@@ -1646,52 +1646,52 @@
     </row>
     <row r="56" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A56" s="7">
-        <v>46296</v>
+        <v>46297</v>
       </c>
       <c r="B56" s="8"/>
       <c r="C56" s="20" t="s">
         <v>32</v>
       </c>
       <c r="D56" s="10">
-        <v>273.72000000000003</v>
+        <v>273.31</v>
       </c>
       <c r="E56" s="10">
-        <v>254.29</v>
+        <v>256.16000000000003</v>
       </c>
       <c r="F56" s="10">
-        <v>264.29000000000002</v>
+        <v>266.16000000000003</v>
       </c>
       <c r="G56" s="17"/>
     </row>
     <row r="57" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A57" s="11">
-        <v>46296</v>
+        <v>46297</v>
       </c>
       <c r="B57" s="12"/>
       <c r="C57" s="21" t="s">
         <v>33</v>
       </c>
       <c r="D57" s="13">
-        <v>262.89999999999998</v>
+        <v>262.52</v>
       </c>
       <c r="E57" s="13">
-        <v>238.81</v>
+        <v>240.08</v>
       </c>
       <c r="F57" s="13">
-        <v>248.81</v>
+        <v>250.08</v>
       </c>
       <c r="G57" s="17"/>
     </row>
     <row r="58" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A58" s="7">
-        <v>46296</v>
+        <v>46297</v>
       </c>
       <c r="B58" s="8"/>
       <c r="C58" s="20" t="s">
         <v>34</v>
       </c>
       <c r="D58" s="10">
-        <v>264.24</v>
+        <v>263.88</v>
       </c>
       <c r="E58" s="10" t="s">
         <v>18</v>
@@ -1703,17 +1703,17 @@
     </row>
     <row r="59" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A59" s="11">
-        <v>46296</v>
+        <v>46297</v>
       </c>
       <c r="B59" s="12"/>
       <c r="C59" s="21" t="s">
         <v>35</v>
       </c>
       <c r="D59" s="13">
-        <v>259.27</v>
+        <v>258.74</v>
       </c>
       <c r="E59" s="13">
-        <v>233.18</v>
+        <v>234.45</v>
       </c>
       <c r="F59" s="13" t="s">
         <v>18</v>
@@ -1722,36 +1722,36 @@
     </row>
     <row r="60" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A60" s="7">
-        <v>46296</v>
+        <v>46297</v>
       </c>
       <c r="B60" s="8"/>
       <c r="C60" s="20" t="s">
         <v>36</v>
       </c>
       <c r="D60" s="10">
-        <v>255.1</v>
+        <v>254.57</v>
       </c>
       <c r="E60" s="10">
-        <v>229.13</v>
+        <v>230.4</v>
       </c>
       <c r="F60" s="10">
-        <v>239.13</v>
+        <v>240.4</v>
       </c>
       <c r="G60" s="17"/>
     </row>
     <row r="61" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A61" s="11">
-        <v>46296</v>
+        <v>46297</v>
       </c>
       <c r="B61" s="12"/>
       <c r="C61" s="21" t="s">
         <v>37</v>
       </c>
       <c r="D61" s="13">
-        <v>260.51</v>
+        <v>259.97000000000003</v>
       </c>
       <c r="E61" s="13">
-        <v>248.7</v>
+        <v>250.37</v>
       </c>
       <c r="F61" s="13" t="s">
         <v>18</v>
@@ -1760,52 +1760,52 @@
     </row>
     <row r="62" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A62" s="7">
-        <v>46295</v>
+        <v>46296</v>
       </c>
       <c r="B62" s="8"/>
       <c r="C62" s="20" t="s">
         <v>32</v>
       </c>
       <c r="D62" s="10">
-        <v>273.52</v>
+        <v>273.72000000000003</v>
       </c>
       <c r="E62" s="10">
-        <v>252.78</v>
+        <v>254.29</v>
       </c>
       <c r="F62" s="10">
-        <v>262.77999999999997</v>
+        <v>264.29000000000002</v>
       </c>
       <c r="G62" s="17"/>
     </row>
     <row r="63" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A63" s="11">
-        <v>46295</v>
+        <v>46296</v>
       </c>
       <c r="B63" s="12"/>
       <c r="C63" s="21" t="s">
         <v>33</v>
       </c>
       <c r="D63" s="13">
-        <v>262.66000000000003</v>
+        <v>262.89999999999998</v>
       </c>
       <c r="E63" s="13">
-        <v>237.95</v>
+        <v>238.81</v>
       </c>
       <c r="F63" s="13">
-        <v>247.95</v>
+        <v>248.81</v>
       </c>
       <c r="G63" s="17"/>
     </row>
     <row r="64" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A64" s="7">
-        <v>46295</v>
+        <v>46296</v>
       </c>
       <c r="B64" s="8"/>
       <c r="C64" s="20" t="s">
         <v>34</v>
       </c>
       <c r="D64" s="10">
-        <v>263.99</v>
+        <v>264.24</v>
       </c>
       <c r="E64" s="10" t="s">
         <v>18</v>
@@ -1817,17 +1817,17 @@
     </row>
     <row r="65" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A65" s="11">
-        <v>46295</v>
+        <v>46296</v>
       </c>
       <c r="B65" s="12"/>
       <c r="C65" s="21" t="s">
         <v>35</v>
       </c>
       <c r="D65" s="13">
-        <v>259.2</v>
+        <v>259.27</v>
       </c>
       <c r="E65" s="13">
-        <v>232.32</v>
+        <v>233.18</v>
       </c>
       <c r="F65" s="13" t="s">
         <v>18</v>
@@ -1835,35 +1835,35 @@
     </row>
     <row r="66" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A66" s="7">
-        <v>46295</v>
+        <v>46296</v>
       </c>
       <c r="B66" s="8"/>
       <c r="C66" s="20" t="s">
         <v>36</v>
       </c>
       <c r="D66" s="10">
-        <v>255.03</v>
+        <v>255.1</v>
       </c>
       <c r="E66" s="10">
-        <v>228.27</v>
+        <v>229.13</v>
       </c>
       <c r="F66" s="10">
-        <v>238.27</v>
+        <v>239.13</v>
       </c>
     </row>
     <row r="67" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A67" s="11">
-        <v>46295</v>
+        <v>46296</v>
       </c>
       <c r="B67" s="12"/>
       <c r="C67" s="21" t="s">
         <v>37</v>
       </c>
       <c r="D67" s="13">
-        <v>260.45999999999998</v>
+        <v>260.51</v>
       </c>
       <c r="E67" s="13">
-        <v>247.41</v>
+        <v>248.7</v>
       </c>
       <c r="F67" s="13" t="s">
         <v>18</v>
@@ -1891,6 +1891,15 @@
 </file>
 
 <file path=customXml/item1.xml><?xml version="1.0" encoding="utf-8"?>
+<?mso-contentType ?>
+<FormTemplates xmlns="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms">
+  <Display>DocumentLibraryForm</Display>
+  <Edit>DocumentLibraryForm</Edit>
+  <New>DocumentLibraryForm</New>
+</FormTemplates>
+</file>
+
+<file path=customXml/item2.xml><?xml version="1.0" encoding="utf-8"?>
 <p:properties xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls">
   <documentManagement>
     <lcf76f155ced4ddcb4097134ff3c332f xmlns="87276d81-85f4-4ef2-9e6e-55066304288f">
@@ -1899,15 +1908,6 @@
     <TaxCatchAll xmlns="b23b8984-eafa-4e79-985e-54f52f3da58e" xsi:nil="true"/>
   </documentManagement>
 </p:properties>
-</file>
-
-<file path=customXml/item2.xml><?xml version="1.0" encoding="utf-8"?>
-<?mso-contentType ?>
-<FormTemplates xmlns="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms">
-  <Display>DocumentLibraryForm</Display>
-  <Edit>DocumentLibraryForm</Edit>
-  <New>DocumentLibraryForm</New>
-</FormTemplates>
 </file>
 
 <file path=customXml/item3.xml><?xml version="1.0" encoding="utf-8"?>
@@ -2171,20 +2171,20 @@
 </file>
 
 <file path=customXml/itemProps1.xml><?xml version="1.0" encoding="utf-8"?>
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{F60519E9-FD90-4339-869C-BC2F85719BB8}">
+  <ds:schemaRefs>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms"/>
+  </ds:schemaRefs>
+</ds:datastoreItem>
+</file>
+
+<file path=customXml/itemProps2.xml><?xml version="1.0" encoding="utf-8"?>
 <ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{57A83D98-2BAE-4D83-823A-D31C464B620C}">
   <ds:schemaRefs>
     <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/properties"/>
     <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
     <ds:schemaRef ds:uri="87276d81-85f4-4ef2-9e6e-55066304288f"/>
     <ds:schemaRef ds:uri="b23b8984-eafa-4e79-985e-54f52f3da58e"/>
-  </ds:schemaRefs>
-</ds:datastoreItem>
-</file>
-
-<file path=customXml/itemProps2.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{F60519E9-FD90-4339-869C-BC2F85719BB8}">
-  <ds:schemaRefs>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms"/>
   </ds:schemaRefs>
 </ds:datastoreItem>
 </file>

</xml_diff>

<commit_message>
Fri Oct  2 07:05:23 UTC 2026
</commit_message>
<xml_diff>
--- a/bp.com-content-dam-bp-country-sites-en_au-australia-home-products-services-pricing-tgp-excel.xlsx
+++ b/bp.com-content-dam-bp-country-sites-en_au-australia-home-products-services-pricing-tgp-excel.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://bp365.sharepoint.com/sites/WholesalePricing/Shared Documents/B2C/TGP/Daily TGP/Web TGP/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="14_{2A783A92-666D-4996-9693-5633558FB425}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="14_{E320625B-A69D-404F-8DD6-CCF5CE37F89F}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-28920" yWindow="-60" windowWidth="29040" windowHeight="15720" xr2:uid="{1B412EEF-F96D-4DF4-A4E9-C7F0F183C2FB}"/>
+    <workbookView xWindow="-28920" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{1B412EEF-F96D-4DF4-A4E9-C7F0F183C2FB}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
@@ -808,128 +808,128 @@
     </row>
     <row r="8" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A8" s="7">
-        <v>46297</v>
+        <v>46298</v>
       </c>
       <c r="B8" s="8"/>
       <c r="C8" s="9" t="s">
         <v>10</v>
       </c>
       <c r="D8" s="10">
-        <v>261.19</v>
+        <v>260.33</v>
       </c>
       <c r="E8" s="10">
-        <v>232.14</v>
+        <v>231.27</v>
       </c>
       <c r="F8" s="10">
-        <v>242.14</v>
+        <v>241.27</v>
       </c>
       <c r="G8" s="10">
-        <v>229.75</v>
+        <v>228.88</v>
       </c>
     </row>
     <row r="9" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A9" s="11">
-        <v>46297</v>
+        <v>46298</v>
       </c>
       <c r="B9" s="12"/>
       <c r="C9" s="12" t="s">
         <v>11</v>
       </c>
       <c r="D9" s="13">
-        <v>261.19</v>
+        <v>260.33</v>
       </c>
       <c r="E9" s="13">
-        <v>232.14</v>
+        <v>231.27</v>
       </c>
       <c r="F9" s="13">
-        <v>242.14</v>
+        <v>241.27</v>
       </c>
       <c r="G9" s="13">
-        <v>229.75</v>
+        <v>228.88</v>
       </c>
     </row>
     <row r="10" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A10" s="7">
-        <v>46297</v>
+        <v>46298</v>
       </c>
       <c r="B10" s="8"/>
       <c r="C10" s="9" t="s">
         <v>12</v>
       </c>
       <c r="D10" s="10">
-        <v>256.83</v>
+        <v>257.8</v>
       </c>
       <c r="E10" s="10">
-        <v>229.24</v>
+        <v>231.83</v>
       </c>
       <c r="F10" s="10">
-        <v>239.24</v>
+        <v>241.83</v>
       </c>
       <c r="G10" s="10">
-        <v>227.64</v>
+        <v>230.24</v>
       </c>
     </row>
     <row r="11" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A11" s="11">
-        <v>46296</v>
+        <v>46297</v>
       </c>
       <c r="B11" s="12"/>
       <c r="C11" s="12" t="s">
         <v>10</v>
       </c>
       <c r="D11" s="13">
-        <v>261.42</v>
+        <v>261.19</v>
       </c>
       <c r="E11" s="13">
-        <v>230.61</v>
+        <v>232.14</v>
       </c>
       <c r="F11" s="13">
-        <v>240.61</v>
+        <v>242.14</v>
       </c>
       <c r="G11" s="13">
-        <v>228.22</v>
+        <v>229.75</v>
       </c>
     </row>
     <row r="12" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A12" s="7">
-        <v>46296</v>
+        <v>46297</v>
       </c>
       <c r="B12" s="8"/>
       <c r="C12" s="9" t="s">
         <v>11</v>
       </c>
       <c r="D12" s="10">
-        <v>261.42</v>
+        <v>261.19</v>
       </c>
       <c r="E12" s="10">
-        <v>230.61</v>
+        <v>232.14</v>
       </c>
       <c r="F12" s="10">
-        <v>240.61</v>
+        <v>242.14</v>
       </c>
       <c r="G12" s="10">
-        <v>228.22</v>
+        <v>229.75</v>
       </c>
     </row>
     <row r="13" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A13" s="11">
-        <v>46296</v>
+        <v>46297</v>
       </c>
       <c r="B13" s="12"/>
       <c r="C13" s="12" t="s">
         <v>12</v>
       </c>
       <c r="D13" s="13">
-        <v>257.22000000000003</v>
+        <v>256.83</v>
       </c>
       <c r="E13" s="13">
-        <v>227.84</v>
+        <v>229.24</v>
       </c>
       <c r="F13" s="13">
-        <v>237.84</v>
+        <v>239.24</v>
       </c>
       <c r="G13" s="13">
-        <v>226.25</v>
+        <v>227.64</v>
       </c>
     </row>
     <row r="14" spans="1:7" x14ac:dyDescent="0.25">
@@ -973,39 +973,39 @@
     </row>
     <row r="17" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A17" s="7">
-        <v>46297</v>
+        <v>46298</v>
       </c>
       <c r="B17" s="8"/>
       <c r="C17" s="20" t="s">
         <v>14</v>
       </c>
       <c r="D17" s="10">
-        <v>260.76</v>
+        <v>261.56</v>
       </c>
       <c r="E17" s="10">
-        <v>234.83</v>
+        <v>237.28</v>
       </c>
       <c r="F17" s="10">
-        <v>244.83</v>
+        <v>247.28</v>
       </c>
       <c r="G17" s="17"/>
     </row>
     <row r="18" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A18" s="11">
-        <v>46296</v>
+        <v>46297</v>
       </c>
       <c r="B18" s="12"/>
       <c r="C18" s="12" t="s">
         <v>14</v>
       </c>
       <c r="D18" s="13">
-        <v>261.27</v>
+        <v>260.76</v>
       </c>
       <c r="E18" s="13">
-        <v>233.53</v>
+        <v>234.83</v>
       </c>
       <c r="F18" s="13">
-        <v>243.53</v>
+        <v>244.83</v>
       </c>
       <c r="G18" s="17"/>
     </row>
@@ -1052,41 +1052,41 @@
     </row>
     <row r="22" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A22" s="7">
-        <v>46297</v>
+        <v>46298</v>
       </c>
       <c r="B22" s="8"/>
       <c r="C22" s="20" t="s">
         <v>16</v>
       </c>
       <c r="D22" s="10">
-        <v>262.31</v>
+        <v>261.45</v>
       </c>
       <c r="E22" s="10">
-        <v>230.08</v>
+        <v>231.95</v>
       </c>
       <c r="F22" s="10">
-        <v>239.68</v>
+        <v>241.55</v>
       </c>
       <c r="G22" s="10">
-        <v>226.45</v>
+        <v>228.32</v>
       </c>
     </row>
     <row r="23" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A23" s="11">
-        <v>46297</v>
+        <v>46298</v>
       </c>
       <c r="B23" s="12"/>
       <c r="C23" s="21" t="s">
         <v>17</v>
       </c>
       <c r="D23" s="13">
-        <v>261.73</v>
+        <v>262.73</v>
       </c>
       <c r="E23" s="13">
-        <v>239.55</v>
+        <v>242.21</v>
       </c>
       <c r="F23" s="13">
-        <v>249.55</v>
+        <v>252.21</v>
       </c>
       <c r="G23" s="13" t="s">
         <v>18</v>
@@ -1094,20 +1094,20 @@
     </row>
     <row r="24" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A24" s="7">
-        <v>46297</v>
+        <v>46298</v>
       </c>
       <c r="B24" s="8"/>
       <c r="C24" s="20" t="s">
         <v>19</v>
       </c>
       <c r="D24" s="10">
-        <v>262.14</v>
+        <v>263.11</v>
       </c>
       <c r="E24" s="10">
-        <v>238.79</v>
+        <v>241.45</v>
       </c>
       <c r="F24" s="10">
-        <v>248.79</v>
+        <v>251.45</v>
       </c>
       <c r="G24" s="10" t="s">
         <v>18</v>
@@ -1115,41 +1115,41 @@
     </row>
     <row r="25" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A25" s="11">
-        <v>46297</v>
+        <v>46298</v>
       </c>
       <c r="B25" s="12"/>
       <c r="C25" s="21" t="s">
         <v>20</v>
       </c>
       <c r="D25" s="13">
-        <v>258.82</v>
+        <v>259.77999999999997</v>
       </c>
       <c r="E25" s="13">
-        <v>238.97</v>
+        <v>241.66</v>
       </c>
       <c r="F25" s="13">
-        <v>248.97</v>
+        <v>251.66</v>
       </c>
       <c r="G25" s="13">
-        <v>234.81</v>
+        <v>237.5</v>
       </c>
     </row>
     <row r="26" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A26" s="7">
-        <v>46297</v>
+        <v>46298</v>
       </c>
       <c r="B26" s="8"/>
       <c r="C26" s="20" t="s">
         <v>21</v>
       </c>
       <c r="D26" s="10">
-        <v>260.47000000000003</v>
+        <v>261.39999999999998</v>
       </c>
       <c r="E26" s="10">
-        <v>240.47</v>
+        <v>243.17</v>
       </c>
       <c r="F26" s="10">
-        <v>250.47</v>
+        <v>253.17</v>
       </c>
       <c r="G26" s="10" t="s">
         <v>18</v>
@@ -1157,41 +1157,41 @@
     </row>
     <row r="27" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A27" s="11">
-        <v>46296</v>
+        <v>46297</v>
       </c>
       <c r="B27" s="12"/>
       <c r="C27" s="12" t="s">
         <v>16</v>
       </c>
       <c r="D27" s="13">
-        <v>262.54000000000002</v>
+        <v>262.31</v>
       </c>
       <c r="E27" s="13">
-        <v>228.55</v>
+        <v>230.08</v>
       </c>
       <c r="F27" s="13">
-        <v>238.15</v>
+        <v>239.68</v>
       </c>
       <c r="G27" s="13">
-        <v>224.92</v>
+        <v>226.45</v>
       </c>
     </row>
     <row r="28" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A28" s="7">
-        <v>46296</v>
+        <v>46297</v>
       </c>
       <c r="B28" s="8"/>
       <c r="C28" s="20" t="s">
         <v>17</v>
       </c>
       <c r="D28" s="10">
-        <v>262.11</v>
+        <v>261.73</v>
       </c>
       <c r="E28" s="22">
-        <v>238.1</v>
+        <v>239.55</v>
       </c>
       <c r="F28" s="22">
-        <v>248.1</v>
+        <v>249.55</v>
       </c>
       <c r="G28" s="22" t="s">
         <v>18</v>
@@ -1199,20 +1199,20 @@
     </row>
     <row r="29" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A29" s="11">
-        <v>46296</v>
+        <v>46297</v>
       </c>
       <c r="B29" s="12"/>
       <c r="C29" s="12" t="s">
         <v>19</v>
       </c>
       <c r="D29" s="13">
-        <v>262.52999999999997</v>
+        <v>262.14</v>
       </c>
       <c r="E29" s="13">
-        <v>237.35</v>
+        <v>238.79</v>
       </c>
       <c r="F29" s="13">
-        <v>247.35</v>
+        <v>248.79</v>
       </c>
       <c r="G29" s="13" t="s">
         <v>18</v>
@@ -1220,41 +1220,41 @@
     </row>
     <row r="30" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A30" s="7">
-        <v>46296</v>
+        <v>46297</v>
       </c>
       <c r="B30" s="8"/>
       <c r="C30" s="20" t="s">
         <v>20</v>
       </c>
       <c r="D30" s="10">
-        <v>259.22000000000003</v>
+        <v>258.82</v>
       </c>
       <c r="E30" s="22">
-        <v>237.52</v>
+        <v>238.97</v>
       </c>
       <c r="F30" s="22">
-        <v>247.52</v>
+        <v>248.97</v>
       </c>
       <c r="G30" s="22">
-        <v>233.36</v>
+        <v>234.81</v>
       </c>
     </row>
     <row r="31" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A31" s="11">
-        <v>46296</v>
+        <v>46297</v>
       </c>
       <c r="B31" s="12"/>
       <c r="C31" s="12" t="s">
         <v>21</v>
       </c>
       <c r="D31" s="13">
-        <v>260.88</v>
+        <v>260.47000000000003</v>
       </c>
       <c r="E31" s="13">
-        <v>239</v>
+        <v>240.47</v>
       </c>
       <c r="F31" s="13">
-        <v>249</v>
+        <v>250.47</v>
       </c>
       <c r="G31" s="13" t="s">
         <v>18</v>
@@ -1301,52 +1301,52 @@
     </row>
     <row r="35" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A35" s="7">
-        <v>46297</v>
+        <v>46298</v>
       </c>
       <c r="B35" s="8"/>
       <c r="C35" s="20" t="s">
         <v>23</v>
       </c>
       <c r="D35" s="10">
-        <v>255.37</v>
+        <v>256.35000000000002</v>
       </c>
       <c r="E35" s="10">
-        <v>227.07</v>
+        <v>228.56</v>
       </c>
       <c r="F35" s="10">
-        <v>236.07</v>
+        <v>237.56</v>
       </c>
       <c r="G35" s="17"/>
     </row>
     <row r="36" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A36" s="11">
-        <v>46296</v>
+        <v>46297</v>
       </c>
       <c r="B36" s="12"/>
       <c r="C36" s="12" t="s">
         <v>23</v>
       </c>
       <c r="D36" s="13">
-        <v>255.76</v>
+        <v>255.37</v>
       </c>
       <c r="E36" s="13">
-        <v>225.67</v>
+        <v>227.07</v>
       </c>
       <c r="F36" s="13">
-        <v>234.67</v>
+        <v>236.07</v>
       </c>
       <c r="G36" s="17"/>
     </row>
     <row r="37" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A37" s="7">
-        <v>46297</v>
+        <v>46298</v>
       </c>
       <c r="B37" s="8"/>
       <c r="C37" s="20" t="s">
         <v>24</v>
       </c>
       <c r="D37" s="10">
-        <v>270.99</v>
+        <v>271.97000000000003</v>
       </c>
       <c r="E37" s="10" t="s">
         <v>18</v>
@@ -1358,14 +1358,14 @@
     </row>
     <row r="38" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A38" s="11">
-        <v>46296</v>
+        <v>46297</v>
       </c>
       <c r="B38" s="12"/>
       <c r="C38" s="12" t="s">
         <v>24</v>
       </c>
       <c r="D38" s="13">
-        <v>271.38</v>
+        <v>270.99</v>
       </c>
       <c r="E38" s="13" t="s">
         <v>18</v>
@@ -1416,77 +1416,77 @@
     </row>
     <row r="42" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A42" s="7">
-        <v>46297</v>
+        <v>46298</v>
       </c>
       <c r="B42" s="8"/>
       <c r="C42" s="20" t="s">
         <v>26</v>
       </c>
       <c r="D42" s="10">
-        <v>265.02999999999997</v>
+        <v>266.14</v>
       </c>
       <c r="E42" s="10">
-        <v>235.66</v>
+        <v>238.4</v>
       </c>
       <c r="F42" s="10">
-        <v>245.66</v>
+        <v>248.4</v>
       </c>
       <c r="G42" s="17"/>
     </row>
     <row r="43" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A43" s="11">
-        <v>46297</v>
+        <v>46298</v>
       </c>
       <c r="B43" s="12"/>
       <c r="C43" s="21" t="s">
         <v>27</v>
       </c>
       <c r="D43" s="13">
-        <v>264.64</v>
+        <v>265.75</v>
       </c>
       <c r="E43" s="13">
-        <v>236.07</v>
+        <v>238.81</v>
       </c>
       <c r="F43" s="13">
-        <v>246.07</v>
+        <v>248.81</v>
       </c>
       <c r="G43" s="17"/>
     </row>
     <row r="44" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A44" s="7">
-        <v>46296</v>
+        <v>46297</v>
       </c>
       <c r="B44" s="8"/>
       <c r="C44" s="20" t="s">
         <v>26</v>
       </c>
       <c r="D44" s="10">
-        <v>265.32</v>
+        <v>265.02999999999997</v>
       </c>
       <c r="E44" s="10">
-        <v>234.18</v>
+        <v>235.66</v>
       </c>
       <c r="F44" s="10">
-        <v>244.18</v>
+        <v>245.66</v>
       </c>
       <c r="G44" s="17"/>
     </row>
     <row r="45" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A45" s="11">
-        <v>46296</v>
+        <v>46297</v>
       </c>
       <c r="B45" s="12"/>
       <c r="C45" s="21" t="s">
         <v>27</v>
       </c>
       <c r="D45" s="13">
-        <v>264.93</v>
+        <v>264.64</v>
       </c>
       <c r="E45" s="13">
-        <v>234.6</v>
+        <v>236.07</v>
       </c>
       <c r="F45" s="13">
-        <v>244.6</v>
+        <v>246.07</v>
       </c>
       <c r="G45" s="17"/>
     </row>
@@ -1531,77 +1531,77 @@
     </row>
     <row r="49" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A49" s="7">
-        <v>46297</v>
+        <v>46298</v>
       </c>
       <c r="B49" s="8"/>
       <c r="C49" s="20" t="s">
         <v>29</v>
       </c>
       <c r="D49" s="10">
-        <v>256.66000000000003</v>
+        <v>258.44</v>
       </c>
       <c r="E49" s="10">
-        <v>230.27</v>
+        <v>232.76</v>
       </c>
       <c r="F49" s="10">
-        <v>240.27</v>
+        <v>242.76</v>
       </c>
       <c r="G49" s="28"/>
     </row>
     <row r="50" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A50" s="11">
-        <v>46297</v>
+        <v>46298</v>
       </c>
       <c r="B50" s="12"/>
       <c r="C50" s="21" t="s">
         <v>30</v>
       </c>
       <c r="D50" s="13">
-        <v>254.39</v>
+        <v>256.13</v>
       </c>
       <c r="E50" s="13">
-        <v>229.99</v>
+        <v>232.45</v>
       </c>
       <c r="F50" s="13">
-        <v>239.99</v>
+        <v>242.45</v>
       </c>
       <c r="G50" s="28"/>
     </row>
     <row r="51" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A51" s="7">
-        <v>46296</v>
+        <v>46297</v>
       </c>
       <c r="B51" s="8"/>
       <c r="C51" s="20" t="s">
         <v>29</v>
       </c>
       <c r="D51" s="10">
-        <v>256.32</v>
+        <v>256.66000000000003</v>
       </c>
       <c r="E51" s="10">
-        <v>229.42</v>
+        <v>230.27</v>
       </c>
       <c r="F51" s="10">
-        <v>239.42</v>
+        <v>240.27</v>
       </c>
       <c r="G51" s="17"/>
     </row>
     <row r="52" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A52" s="11">
-        <v>46296</v>
+        <v>46297</v>
       </c>
       <c r="B52" s="12"/>
       <c r="C52" s="21" t="s">
         <v>30</v>
       </c>
       <c r="D52" s="13">
-        <v>254.09</v>
+        <v>254.39</v>
       </c>
       <c r="E52" s="13">
-        <v>229.16</v>
+        <v>229.99</v>
       </c>
       <c r="F52" s="13">
-        <v>239.16</v>
+        <v>239.99</v>
       </c>
       <c r="G52" s="17"/>
     </row>
@@ -1646,52 +1646,52 @@
     </row>
     <row r="56" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A56" s="7">
-        <v>46297</v>
+        <v>46298</v>
       </c>
       <c r="B56" s="8"/>
       <c r="C56" s="20" t="s">
         <v>32</v>
       </c>
       <c r="D56" s="10">
-        <v>273.31</v>
+        <v>274.23</v>
       </c>
       <c r="E56" s="10">
-        <v>256.16000000000003</v>
+        <v>259.47000000000003</v>
       </c>
       <c r="F56" s="10">
-        <v>266.16000000000003</v>
+        <v>269.47000000000003</v>
       </c>
       <c r="G56" s="17"/>
     </row>
     <row r="57" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A57" s="11">
-        <v>46297</v>
+        <v>46298</v>
       </c>
       <c r="B57" s="12"/>
       <c r="C57" s="21" t="s">
         <v>33</v>
       </c>
       <c r="D57" s="13">
-        <v>262.52</v>
+        <v>263.51</v>
       </c>
       <c r="E57" s="13">
-        <v>240.08</v>
+        <v>242.49</v>
       </c>
       <c r="F57" s="13">
-        <v>250.08</v>
+        <v>252.49</v>
       </c>
       <c r="G57" s="17"/>
     </row>
     <row r="58" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A58" s="7">
-        <v>46297</v>
+        <v>46298</v>
       </c>
       <c r="B58" s="8"/>
       <c r="C58" s="20" t="s">
         <v>34</v>
       </c>
       <c r="D58" s="10">
-        <v>263.88</v>
+        <v>264.89999999999998</v>
       </c>
       <c r="E58" s="10" t="s">
         <v>18</v>
@@ -1703,17 +1703,17 @@
     </row>
     <row r="59" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A59" s="11">
-        <v>46297</v>
+        <v>46298</v>
       </c>
       <c r="B59" s="12"/>
       <c r="C59" s="21" t="s">
         <v>35</v>
       </c>
       <c r="D59" s="13">
-        <v>258.74</v>
+        <v>259.5</v>
       </c>
       <c r="E59" s="13">
-        <v>234.45</v>
+        <v>236.86</v>
       </c>
       <c r="F59" s="13" t="s">
         <v>18</v>
@@ -1722,36 +1722,36 @@
     </row>
     <row r="60" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A60" s="7">
-        <v>46297</v>
+        <v>46298</v>
       </c>
       <c r="B60" s="8"/>
       <c r="C60" s="20" t="s">
         <v>36</v>
       </c>
       <c r="D60" s="10">
-        <v>254.57</v>
+        <v>255.33</v>
       </c>
       <c r="E60" s="10">
-        <v>230.4</v>
+        <v>232.81</v>
       </c>
       <c r="F60" s="10">
-        <v>240.4</v>
+        <v>242.81</v>
       </c>
       <c r="G60" s="17"/>
     </row>
     <row r="61" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A61" s="11">
-        <v>46297</v>
+        <v>46298</v>
       </c>
       <c r="B61" s="12"/>
       <c r="C61" s="21" t="s">
         <v>37</v>
       </c>
       <c r="D61" s="13">
-        <v>259.97000000000003</v>
+        <v>260.72000000000003</v>
       </c>
       <c r="E61" s="13">
-        <v>250.37</v>
+        <v>253.37</v>
       </c>
       <c r="F61" s="13" t="s">
         <v>18</v>
@@ -1760,52 +1760,52 @@
     </row>
     <row r="62" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A62" s="7">
-        <v>46296</v>
+        <v>46297</v>
       </c>
       <c r="B62" s="8"/>
       <c r="C62" s="20" t="s">
         <v>32</v>
       </c>
       <c r="D62" s="10">
-        <v>273.72000000000003</v>
+        <v>273.31</v>
       </c>
       <c r="E62" s="10">
-        <v>254.29</v>
+        <v>256.16000000000003</v>
       </c>
       <c r="F62" s="10">
-        <v>264.29000000000002</v>
+        <v>266.16000000000003</v>
       </c>
       <c r="G62" s="17"/>
     </row>
     <row r="63" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A63" s="11">
-        <v>46296</v>
+        <v>46297</v>
       </c>
       <c r="B63" s="12"/>
       <c r="C63" s="21" t="s">
         <v>33</v>
       </c>
       <c r="D63" s="13">
-        <v>262.89999999999998</v>
+        <v>262.52</v>
       </c>
       <c r="E63" s="13">
-        <v>238.81</v>
+        <v>240.08</v>
       </c>
       <c r="F63" s="13">
-        <v>248.81</v>
+        <v>250.08</v>
       </c>
       <c r="G63" s="17"/>
     </row>
     <row r="64" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A64" s="7">
-        <v>46296</v>
+        <v>46297</v>
       </c>
       <c r="B64" s="8"/>
       <c r="C64" s="20" t="s">
         <v>34</v>
       </c>
       <c r="D64" s="10">
-        <v>264.24</v>
+        <v>263.88</v>
       </c>
       <c r="E64" s="10" t="s">
         <v>18</v>
@@ -1817,17 +1817,17 @@
     </row>
     <row r="65" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A65" s="11">
-        <v>46296</v>
+        <v>46297</v>
       </c>
       <c r="B65" s="12"/>
       <c r="C65" s="21" t="s">
         <v>35</v>
       </c>
       <c r="D65" s="13">
-        <v>259.27</v>
+        <v>258.74</v>
       </c>
       <c r="E65" s="13">
-        <v>233.18</v>
+        <v>234.45</v>
       </c>
       <c r="F65" s="13" t="s">
         <v>18</v>
@@ -1835,35 +1835,35 @@
     </row>
     <row r="66" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A66" s="7">
-        <v>46296</v>
+        <v>46297</v>
       </c>
       <c r="B66" s="8"/>
       <c r="C66" s="20" t="s">
         <v>36</v>
       </c>
       <c r="D66" s="10">
-        <v>255.1</v>
+        <v>254.57</v>
       </c>
       <c r="E66" s="10">
-        <v>229.13</v>
+        <v>230.4</v>
       </c>
       <c r="F66" s="10">
-        <v>239.13</v>
+        <v>240.4</v>
       </c>
     </row>
     <row r="67" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A67" s="11">
-        <v>46296</v>
+        <v>46297</v>
       </c>
       <c r="B67" s="12"/>
       <c r="C67" s="21" t="s">
         <v>37</v>
       </c>
       <c r="D67" s="13">
-        <v>260.51</v>
+        <v>259.97000000000003</v>
       </c>
       <c r="E67" s="13">
-        <v>248.7</v>
+        <v>250.37</v>
       </c>
       <c r="F67" s="13" t="s">
         <v>18</v>
@@ -1900,17 +1900,6 @@
 </file>
 
 <file path=customXml/item2.xml><?xml version="1.0" encoding="utf-8"?>
-<p:properties xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls">
-  <documentManagement>
-    <lcf76f155ced4ddcb4097134ff3c332f xmlns="87276d81-85f4-4ef2-9e6e-55066304288f">
-      <Terms xmlns="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
-    </lcf76f155ced4ddcb4097134ff3c332f>
-    <TaxCatchAll xmlns="b23b8984-eafa-4e79-985e-54f52f3da58e" xsi:nil="true"/>
-  </documentManagement>
-</p:properties>
-</file>
-
-<file path=customXml/item3.xml><?xml version="1.0" encoding="utf-8"?>
 <ct:contentTypeSchema xmlns:ct="http://schemas.microsoft.com/office/2006/metadata/contentType" xmlns:ma="http://schemas.microsoft.com/office/2006/metadata/properties/metaAttributes" ct:_="" ma:_="" ma:contentTypeName="Document" ma:contentTypeID="0x010100D3632DF5622958439304627C030B0427" ma:contentTypeVersion="18" ma:contentTypeDescription="Create a new document." ma:contentTypeScope="" ma:versionID="8c2ecbce386d6bac497f8eb2d8f0fb7a">
   <xsd:schema xmlns:xsd="http://www.w3.org/2001/XMLSchema" xmlns:xs="http://www.w3.org/2001/XMLSchema" xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:ns2="87276d81-85f4-4ef2-9e6e-55066304288f" xmlns:ns3="39e1dda6-d1d8-4c88-a3b9-f1abc1284bad" xmlns:ns4="b23b8984-eafa-4e79-985e-54f52f3da58e" targetNamespace="http://schemas.microsoft.com/office/2006/metadata/properties" ma:root="true" ma:fieldsID="4cfd0c2f651c1ce156ad4fcb44ea61dd" ns2:_="" ns3:_="" ns4:_="">
     <xsd:import namespace="87276d81-85f4-4ef2-9e6e-55066304288f"/>
@@ -2170,6 +2159,17 @@
 </ct:contentTypeSchema>
 </file>
 
+<file path=customXml/item3.xml><?xml version="1.0" encoding="utf-8"?>
+<p:properties xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls">
+  <documentManagement>
+    <lcf76f155ced4ddcb4097134ff3c332f xmlns="87276d81-85f4-4ef2-9e6e-55066304288f">
+      <Terms xmlns="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
+    </lcf76f155ced4ddcb4097134ff3c332f>
+    <TaxCatchAll xmlns="b23b8984-eafa-4e79-985e-54f52f3da58e" xsi:nil="true"/>
+  </documentManagement>
+</p:properties>
+</file>
+
 <file path=customXml/itemProps1.xml><?xml version="1.0" encoding="utf-8"?>
 <ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{F60519E9-FD90-4339-869C-BC2F85719BB8}">
   <ds:schemaRefs>
@@ -2179,17 +2179,6 @@
 </file>
 
 <file path=customXml/itemProps2.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{57A83D98-2BAE-4D83-823A-D31C464B620C}">
-  <ds:schemaRefs>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/properties"/>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
-    <ds:schemaRef ds:uri="87276d81-85f4-4ef2-9e6e-55066304288f"/>
-    <ds:schemaRef ds:uri="b23b8984-eafa-4e79-985e-54f52f3da58e"/>
-  </ds:schemaRefs>
-</ds:datastoreItem>
-</file>
-
-<file path=customXml/itemProps3.xml><?xml version="1.0" encoding="utf-8"?>
 <ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{B44E1863-2778-41F9-ACBA-48420F931671}">
   <ds:schemaRefs>
     <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/contentType"/>
@@ -2209,6 +2198,17 @@
 </ds:datastoreItem>
 </file>
 
+<file path=customXml/itemProps3.xml><?xml version="1.0" encoding="utf-8"?>
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{57A83D98-2BAE-4D83-823A-D31C464B620C}">
+  <ds:schemaRefs>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/properties"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
+    <ds:schemaRef ds:uri="87276d81-85f4-4ef2-9e6e-55066304288f"/>
+    <ds:schemaRef ds:uri="b23b8984-eafa-4e79-985e-54f52f3da58e"/>
+  </ds:schemaRefs>
+</ds:datastoreItem>
+</file>
+
 <file path=docMetadata/LabelInfo.xml><?xml version="1.0" encoding="utf-8"?>
 <clbl:labelList xmlns:clbl="http://schemas.microsoft.com/office/2020/mipLabelMetadata">
   <clbl:label id="{569bf4a9-87bd-4dbf-a36c-1db5158e5def}" enabled="1" method="Privileged" siteId="{ea80952e-a476-42d4-aaf4-5457852b0f7e}" removed="0"/>

</xml_diff>

<commit_message>
Mon Oct  5 07:13:18 UTC 2026
</commit_message>
<xml_diff>
--- a/bp.com-content-dam-bp-country-sites-en_au-australia-home-products-services-pricing-tgp-excel.xlsx
+++ b/bp.com-content-dam-bp-country-sites-en_au-australia-home-products-services-pricing-tgp-excel.xlsx
@@ -8,14 +8,14 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://bp365.sharepoint.com/sites/WholesalePricing/Shared Documents/B2C/TGP/Daily TGP/Web TGP/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="14_{E320625B-A69D-404F-8DD6-CCF5CE37F89F}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="14_{675F50F3-9A37-4DB0-A9C5-58F9852F5865}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-28920" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{1B412EEF-F96D-4DF4-A4E9-C7F0F183C2FB}"/>
+    <workbookView xWindow="-8595" yWindow="-16320" windowWidth="29040" windowHeight="15720" xr2:uid="{1B412EEF-F96D-4DF4-A4E9-C7F0F183C2FB}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
   </sheets>
-  <calcPr calcId="191028" concurrentManualCount="12"/>
+  <calcPr calcId="191028"/>
   <extLst>
     <ext xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" uri="{140A7094-0E35-4892-8432-C4D2E57EDEB5}">
       <x15:workbookPr chartTrackingRefBase="1"/>
@@ -715,15 +715,15 @@
     <pageSetUpPr fitToPage="1"/>
   </sheetPr>
   <dimension ref="A1:G67"/>
-  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <sheetFormatPr defaultRowHeight="14.25" x14ac:dyDescent="0.45"/>
   <cols>
-    <col min="1" max="1" width="76.42578125" bestFit="1" customWidth="1"/>
-    <col min="2" max="2" width="6.42578125"/>
-    <col min="3" max="3" width="18.140625" bestFit="1" customWidth="1"/>
-    <col min="4" max="7" width="7.140625" bestFit="1" customWidth="1"/>
+    <col min="1" max="1" width="76.3984375" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="6.3984375"/>
+    <col min="3" max="3" width="18.1328125" bestFit="1" customWidth="1"/>
+    <col min="4" max="7" width="7.1328125" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:7" ht="23.25" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:7" ht="22.15" x14ac:dyDescent="0.45">
       <c r="A1" s="30" t="s">
         <v>0</v>
       </c>
@@ -734,7 +734,7 @@
       <c r="F1" s="2"/>
       <c r="G1" s="2"/>
     </row>
-    <row r="2" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="2" spans="1:7" x14ac:dyDescent="0.45">
       <c r="A2" s="3"/>
       <c r="B2" s="1"/>
       <c r="C2" s="1"/>
@@ -743,7 +743,7 @@
       <c r="F2" s="2"/>
       <c r="G2" s="2"/>
     </row>
-    <row r="3" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="3" spans="1:7" x14ac:dyDescent="0.45">
       <c r="A3" s="3" t="s">
         <v>1</v>
       </c>
@@ -754,7 +754,7 @@
       <c r="F3" s="2"/>
       <c r="G3" s="2"/>
     </row>
-    <row r="4" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="4" spans="1:7" x14ac:dyDescent="0.45">
       <c r="A4" s="3" t="s">
         <v>2</v>
       </c>
@@ -765,7 +765,7 @@
       <c r="F4" s="2"/>
       <c r="G4" s="2"/>
     </row>
-    <row r="5" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="5" spans="1:7" x14ac:dyDescent="0.45">
       <c r="A5" s="3"/>
       <c r="B5" s="3"/>
       <c r="C5" s="1"/>
@@ -774,7 +774,7 @@
       <c r="F5" s="2"/>
       <c r="G5" s="2"/>
     </row>
-    <row r="6" spans="1:7" ht="20.25" x14ac:dyDescent="0.25">
+    <row r="6" spans="1:7" ht="20.25" x14ac:dyDescent="0.45">
       <c r="A6" s="29" t="s">
         <v>3</v>
       </c>
@@ -785,7 +785,7 @@
       <c r="F6" s="2"/>
       <c r="G6" s="2"/>
     </row>
-    <row r="7" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="7" spans="1:7" x14ac:dyDescent="0.45">
       <c r="A7" s="4" t="s">
         <v>4</v>
       </c>
@@ -806,133 +806,133 @@
         <v>9</v>
       </c>
     </row>
-    <row r="8" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="8" spans="1:7" x14ac:dyDescent="0.45">
       <c r="A8" s="7">
-        <v>46298</v>
+        <v>46301</v>
       </c>
       <c r="B8" s="8"/>
       <c r="C8" s="9" t="s">
         <v>10</v>
       </c>
       <c r="D8" s="10">
-        <v>260.33</v>
+        <v>260.49</v>
       </c>
       <c r="E8" s="10">
-        <v>231.27</v>
+        <v>233.42</v>
       </c>
       <c r="F8" s="10">
-        <v>241.27</v>
+        <v>243.42</v>
       </c>
       <c r="G8" s="10">
-        <v>228.88</v>
-      </c>
-    </row>
-    <row r="9" spans="1:7" x14ac:dyDescent="0.25">
+        <v>231.03</v>
+      </c>
+    </row>
+    <row r="9" spans="1:7" x14ac:dyDescent="0.45">
       <c r="A9" s="11">
-        <v>46298</v>
+        <v>46301</v>
       </c>
       <c r="B9" s="12"/>
       <c r="C9" s="12" t="s">
         <v>11</v>
       </c>
       <c r="D9" s="13">
-        <v>260.33</v>
+        <v>260.49</v>
       </c>
       <c r="E9" s="13">
-        <v>231.27</v>
+        <v>233.42</v>
       </c>
       <c r="F9" s="13">
-        <v>241.27</v>
+        <v>243.42</v>
       </c>
       <c r="G9" s="13">
-        <v>228.88</v>
-      </c>
-    </row>
-    <row r="10" spans="1:7" x14ac:dyDescent="0.25">
+        <v>231.03</v>
+      </c>
+    </row>
+    <row r="10" spans="1:7" x14ac:dyDescent="0.45">
       <c r="A10" s="7">
-        <v>46298</v>
+        <v>46301</v>
       </c>
       <c r="B10" s="8"/>
       <c r="C10" s="9" t="s">
         <v>12</v>
       </c>
       <c r="D10" s="10">
-        <v>257.8</v>
+        <v>258.17</v>
       </c>
       <c r="E10" s="10">
-        <v>231.83</v>
+        <v>234.17</v>
       </c>
       <c r="F10" s="10">
-        <v>241.83</v>
+        <v>244.17</v>
       </c>
       <c r="G10" s="10">
-        <v>230.24</v>
-      </c>
-    </row>
-    <row r="11" spans="1:7" x14ac:dyDescent="0.25">
+        <v>232.58</v>
+      </c>
+    </row>
+    <row r="11" spans="1:7" x14ac:dyDescent="0.45">
       <c r="A11" s="11">
-        <v>46297</v>
+        <v>46298</v>
       </c>
       <c r="B11" s="12"/>
       <c r="C11" s="12" t="s">
         <v>10</v>
       </c>
       <c r="D11" s="13">
-        <v>261.19</v>
+        <v>260.33</v>
       </c>
       <c r="E11" s="13">
-        <v>232.14</v>
+        <v>231.27</v>
       </c>
       <c r="F11" s="13">
-        <v>242.14</v>
+        <v>241.27</v>
       </c>
       <c r="G11" s="13">
-        <v>229.75</v>
-      </c>
-    </row>
-    <row r="12" spans="1:7" x14ac:dyDescent="0.25">
+        <v>228.88</v>
+      </c>
+    </row>
+    <row r="12" spans="1:7" x14ac:dyDescent="0.45">
       <c r="A12" s="7">
-        <v>46297</v>
+        <v>46298</v>
       </c>
       <c r="B12" s="8"/>
       <c r="C12" s="9" t="s">
         <v>11</v>
       </c>
       <c r="D12" s="10">
-        <v>261.19</v>
+        <v>260.33</v>
       </c>
       <c r="E12" s="10">
-        <v>232.14</v>
+        <v>231.27</v>
       </c>
       <c r="F12" s="10">
-        <v>242.14</v>
+        <v>241.27</v>
       </c>
       <c r="G12" s="10">
-        <v>229.75</v>
-      </c>
-    </row>
-    <row r="13" spans="1:7" x14ac:dyDescent="0.25">
+        <v>228.88</v>
+      </c>
+    </row>
+    <row r="13" spans="1:7" x14ac:dyDescent="0.45">
       <c r="A13" s="11">
-        <v>46297</v>
+        <v>46298</v>
       </c>
       <c r="B13" s="12"/>
       <c r="C13" s="12" t="s">
         <v>12</v>
       </c>
       <c r="D13" s="13">
-        <v>256.83</v>
+        <v>257.8</v>
       </c>
       <c r="E13" s="13">
-        <v>229.24</v>
+        <v>231.83</v>
       </c>
       <c r="F13" s="13">
-        <v>239.24</v>
+        <v>241.83</v>
       </c>
       <c r="G13" s="13">
-        <v>227.64</v>
-      </c>
-    </row>
-    <row r="14" spans="1:7" x14ac:dyDescent="0.25">
+        <v>230.24</v>
+      </c>
+    </row>
+    <row r="14" spans="1:7" x14ac:dyDescent="0.45">
       <c r="A14" s="14"/>
       <c r="B14" s="14"/>
       <c r="C14" s="15"/>
@@ -941,7 +941,7 @@
       <c r="F14" s="16"/>
       <c r="G14" s="16"/>
     </row>
-    <row r="15" spans="1:7" ht="20.25" x14ac:dyDescent="0.25">
+    <row r="15" spans="1:7" ht="20.25" x14ac:dyDescent="0.45">
       <c r="A15" s="29" t="s">
         <v>13</v>
       </c>
@@ -952,7 +952,7 @@
       <c r="F15" s="17"/>
       <c r="G15" s="17"/>
     </row>
-    <row r="16" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="16" spans="1:7" x14ac:dyDescent="0.45">
       <c r="A16" s="4" t="s">
         <v>4</v>
       </c>
@@ -971,45 +971,45 @@
       </c>
       <c r="G16" s="17"/>
     </row>
-    <row r="17" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="17" spans="1:7" x14ac:dyDescent="0.45">
       <c r="A17" s="7">
-        <v>46298</v>
+        <v>46301</v>
       </c>
       <c r="B17" s="8"/>
       <c r="C17" s="20" t="s">
         <v>14</v>
       </c>
       <c r="D17" s="10">
-        <v>261.56</v>
+        <v>261.77</v>
       </c>
       <c r="E17" s="10">
-        <v>237.28</v>
+        <v>239.48</v>
       </c>
       <c r="F17" s="10">
-        <v>247.28</v>
+        <v>249.48</v>
       </c>
       <c r="G17" s="17"/>
     </row>
-    <row r="18" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="18" spans="1:7" x14ac:dyDescent="0.45">
       <c r="A18" s="11">
-        <v>46297</v>
+        <v>46298</v>
       </c>
       <c r="B18" s="12"/>
       <c r="C18" s="12" t="s">
         <v>14</v>
       </c>
       <c r="D18" s="13">
-        <v>260.76</v>
+        <v>261.56</v>
       </c>
       <c r="E18" s="13">
-        <v>234.83</v>
+        <v>237.28</v>
       </c>
       <c r="F18" s="13">
-        <v>244.83</v>
+        <v>247.28</v>
       </c>
       <c r="G18" s="17"/>
     </row>
-    <row r="19" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="19" spans="1:7" x14ac:dyDescent="0.45">
       <c r="A19" s="14"/>
       <c r="B19" s="14"/>
       <c r="C19" s="15"/>
@@ -1018,7 +1018,7 @@
       <c r="F19" s="16"/>
       <c r="G19" s="17"/>
     </row>
-    <row r="20" spans="1:7" ht="20.25" x14ac:dyDescent="0.25">
+    <row r="20" spans="1:7" ht="20.25" x14ac:dyDescent="0.45">
       <c r="A20" s="29" t="s">
         <v>15</v>
       </c>
@@ -1029,7 +1029,7 @@
       <c r="F20" s="17"/>
       <c r="G20" s="17"/>
     </row>
-    <row r="21" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="21" spans="1:7" x14ac:dyDescent="0.45">
       <c r="A21" s="4" t="s">
         <v>4</v>
       </c>
@@ -1050,217 +1050,217 @@
         <v>9</v>
       </c>
     </row>
-    <row r="22" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="22" spans="1:7" x14ac:dyDescent="0.45">
       <c r="A22" s="7">
-        <v>46298</v>
+        <v>46301</v>
       </c>
       <c r="B22" s="8"/>
       <c r="C22" s="20" t="s">
         <v>16</v>
       </c>
       <c r="D22" s="10">
-        <v>261.45</v>
+        <v>261.62</v>
       </c>
       <c r="E22" s="10">
-        <v>231.95</v>
+        <v>233</v>
       </c>
       <c r="F22" s="10">
-        <v>241.55</v>
+        <v>242.6</v>
       </c>
       <c r="G22" s="10">
-        <v>228.32</v>
-      </c>
-    </row>
-    <row r="23" spans="1:7" x14ac:dyDescent="0.25">
+        <v>229.37</v>
+      </c>
+    </row>
+    <row r="23" spans="1:7" x14ac:dyDescent="0.45">
       <c r="A23" s="11">
-        <v>46298</v>
+        <v>46301</v>
       </c>
       <c r="B23" s="12"/>
       <c r="C23" s="21" t="s">
         <v>17</v>
       </c>
       <c r="D23" s="13">
-        <v>262.73</v>
+        <v>263.11</v>
       </c>
       <c r="E23" s="13">
-        <v>242.21</v>
+        <v>244.62</v>
       </c>
       <c r="F23" s="13">
-        <v>252.21</v>
+        <v>254.62</v>
       </c>
       <c r="G23" s="13" t="s">
         <v>18</v>
       </c>
     </row>
-    <row r="24" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="24" spans="1:7" x14ac:dyDescent="0.45">
       <c r="A24" s="7">
-        <v>46298</v>
+        <v>46301</v>
       </c>
       <c r="B24" s="8"/>
       <c r="C24" s="20" t="s">
         <v>19</v>
       </c>
       <c r="D24" s="10">
-        <v>263.11</v>
+        <v>263.48</v>
       </c>
       <c r="E24" s="10">
-        <v>241.45</v>
+        <v>243.85</v>
       </c>
       <c r="F24" s="10">
-        <v>251.45</v>
+        <v>253.85</v>
       </c>
       <c r="G24" s="10" t="s">
         <v>18</v>
       </c>
     </row>
-    <row r="25" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="25" spans="1:7" x14ac:dyDescent="0.45">
       <c r="A25" s="11">
-        <v>46298</v>
+        <v>46301</v>
       </c>
       <c r="B25" s="12"/>
       <c r="C25" s="21" t="s">
         <v>20</v>
       </c>
       <c r="D25" s="13">
-        <v>259.77999999999997</v>
+        <v>260.14</v>
       </c>
       <c r="E25" s="13">
-        <v>241.66</v>
+        <v>244.08</v>
       </c>
       <c r="F25" s="13">
-        <v>251.66</v>
+        <v>254.08</v>
       </c>
       <c r="G25" s="13">
-        <v>237.5</v>
-      </c>
-    </row>
-    <row r="26" spans="1:7" x14ac:dyDescent="0.25">
+        <v>239.92</v>
+      </c>
+    </row>
+    <row r="26" spans="1:7" x14ac:dyDescent="0.45">
       <c r="A26" s="7">
-        <v>46298</v>
+        <v>46301</v>
       </c>
       <c r="B26" s="8"/>
       <c r="C26" s="20" t="s">
         <v>21</v>
       </c>
       <c r="D26" s="10">
-        <v>261.39999999999998</v>
+        <v>261.72000000000003</v>
       </c>
       <c r="E26" s="10">
-        <v>243.17</v>
+        <v>245.61</v>
       </c>
       <c r="F26" s="10">
-        <v>253.17</v>
+        <v>255.61</v>
       </c>
       <c r="G26" s="10" t="s">
         <v>18</v>
       </c>
     </row>
-    <row r="27" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="27" spans="1:7" x14ac:dyDescent="0.45">
       <c r="A27" s="11">
-        <v>46297</v>
+        <v>46298</v>
       </c>
       <c r="B27" s="12"/>
       <c r="C27" s="12" t="s">
         <v>16</v>
       </c>
       <c r="D27" s="13">
-        <v>262.31</v>
+        <v>261.45</v>
       </c>
       <c r="E27" s="13">
-        <v>230.08</v>
+        <v>231.95</v>
       </c>
       <c r="F27" s="13">
-        <v>239.68</v>
+        <v>241.55</v>
       </c>
       <c r="G27" s="13">
-        <v>226.45</v>
-      </c>
-    </row>
-    <row r="28" spans="1:7" x14ac:dyDescent="0.25">
+        <v>228.32</v>
+      </c>
+    </row>
+    <row r="28" spans="1:7" x14ac:dyDescent="0.45">
       <c r="A28" s="7">
-        <v>46297</v>
+        <v>46298</v>
       </c>
       <c r="B28" s="8"/>
       <c r="C28" s="20" t="s">
         <v>17</v>
       </c>
       <c r="D28" s="10">
-        <v>261.73</v>
+        <v>262.73</v>
       </c>
       <c r="E28" s="22">
-        <v>239.55</v>
+        <v>242.21</v>
       </c>
       <c r="F28" s="22">
-        <v>249.55</v>
+        <v>252.21</v>
       </c>
       <c r="G28" s="22" t="s">
         <v>18</v>
       </c>
     </row>
-    <row r="29" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="29" spans="1:7" x14ac:dyDescent="0.45">
       <c r="A29" s="11">
-        <v>46297</v>
+        <v>46298</v>
       </c>
       <c r="B29" s="12"/>
       <c r="C29" s="12" t="s">
         <v>19</v>
       </c>
       <c r="D29" s="13">
-        <v>262.14</v>
+        <v>263.11</v>
       </c>
       <c r="E29" s="13">
-        <v>238.79</v>
+        <v>241.45</v>
       </c>
       <c r="F29" s="13">
-        <v>248.79</v>
+        <v>251.45</v>
       </c>
       <c r="G29" s="13" t="s">
         <v>18</v>
       </c>
     </row>
-    <row r="30" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="30" spans="1:7" x14ac:dyDescent="0.45">
       <c r="A30" s="7">
-        <v>46297</v>
+        <v>46298</v>
       </c>
       <c r="B30" s="8"/>
       <c r="C30" s="20" t="s">
         <v>20</v>
       </c>
       <c r="D30" s="10">
-        <v>258.82</v>
+        <v>259.77999999999997</v>
       </c>
       <c r="E30" s="22">
-        <v>238.97</v>
+        <v>241.66</v>
       </c>
       <c r="F30" s="22">
-        <v>248.97</v>
+        <v>251.66</v>
       </c>
       <c r="G30" s="22">
-        <v>234.81</v>
-      </c>
-    </row>
-    <row r="31" spans="1:7" x14ac:dyDescent="0.25">
+        <v>237.5</v>
+      </c>
+    </row>
+    <row r="31" spans="1:7" x14ac:dyDescent="0.45">
       <c r="A31" s="11">
-        <v>46297</v>
+        <v>46298</v>
       </c>
       <c r="B31" s="12"/>
       <c r="C31" s="12" t="s">
         <v>21</v>
       </c>
       <c r="D31" s="13">
-        <v>260.47000000000003</v>
+        <v>261.39999999999998</v>
       </c>
       <c r="E31" s="13">
-        <v>240.47</v>
+        <v>243.17</v>
       </c>
       <c r="F31" s="13">
-        <v>250.47</v>
+        <v>253.17</v>
       </c>
       <c r="G31" s="13" t="s">
         <v>18</v>
       </c>
     </row>
-    <row r="32" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="32" spans="1:7" x14ac:dyDescent="0.45">
       <c r="A32" s="14"/>
       <c r="B32" s="14"/>
       <c r="C32" s="15"/>
@@ -1269,7 +1269,7 @@
       <c r="F32" s="17"/>
       <c r="G32" s="17"/>
     </row>
-    <row r="33" spans="1:7" ht="20.25" x14ac:dyDescent="0.25">
+    <row r="33" spans="1:7" ht="20.25" x14ac:dyDescent="0.45">
       <c r="A33" s="29" t="s">
         <v>22</v>
       </c>
@@ -1280,7 +1280,7 @@
       <c r="F33" s="17"/>
       <c r="G33" s="17"/>
     </row>
-    <row r="34" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="34" spans="1:7" x14ac:dyDescent="0.45">
       <c r="A34" s="23" t="s">
         <v>4</v>
       </c>
@@ -1299,54 +1299,54 @@
       </c>
       <c r="G34" s="17"/>
     </row>
-    <row r="35" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="35" spans="1:7" x14ac:dyDescent="0.45">
       <c r="A35" s="7">
-        <v>46298</v>
+        <v>46301</v>
       </c>
       <c r="B35" s="8"/>
       <c r="C35" s="20" t="s">
         <v>23</v>
       </c>
       <c r="D35" s="10">
-        <v>256.35000000000002</v>
+        <v>256.70999999999998</v>
       </c>
       <c r="E35" s="10">
-        <v>228.56</v>
+        <v>229.8</v>
       </c>
       <c r="F35" s="10">
-        <v>237.56</v>
+        <v>238.8</v>
       </c>
       <c r="G35" s="17"/>
     </row>
-    <row r="36" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="36" spans="1:7" x14ac:dyDescent="0.45">
       <c r="A36" s="11">
-        <v>46297</v>
+        <v>46298</v>
       </c>
       <c r="B36" s="12"/>
       <c r="C36" s="12" t="s">
         <v>23</v>
       </c>
       <c r="D36" s="13">
-        <v>255.37</v>
+        <v>256.35000000000002</v>
       </c>
       <c r="E36" s="13">
-        <v>227.07</v>
+        <v>228.56</v>
       </c>
       <c r="F36" s="13">
-        <v>236.07</v>
+        <v>237.56</v>
       </c>
       <c r="G36" s="17"/>
     </row>
-    <row r="37" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="37" spans="1:7" x14ac:dyDescent="0.45">
       <c r="A37" s="7">
-        <v>46298</v>
+        <v>46301</v>
       </c>
       <c r="B37" s="8"/>
       <c r="C37" s="20" t="s">
         <v>24</v>
       </c>
       <c r="D37" s="10">
-        <v>271.97000000000003</v>
+        <v>272.33</v>
       </c>
       <c r="E37" s="10" t="s">
         <v>18</v>
@@ -1356,16 +1356,16 @@
       </c>
       <c r="G37" s="17"/>
     </row>
-    <row r="38" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="38" spans="1:7" x14ac:dyDescent="0.45">
       <c r="A38" s="11">
-        <v>46297</v>
+        <v>46298</v>
       </c>
       <c r="B38" s="12"/>
       <c r="C38" s="12" t="s">
         <v>24</v>
       </c>
       <c r="D38" s="13">
-        <v>270.99</v>
+        <v>271.97000000000003</v>
       </c>
       <c r="E38" s="13" t="s">
         <v>18</v>
@@ -1375,7 +1375,7 @@
       </c>
       <c r="G38" s="17"/>
     </row>
-    <row r="39" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="39" spans="1:7" x14ac:dyDescent="0.45">
       <c r="A39" s="24"/>
       <c r="B39" s="24"/>
       <c r="C39" s="15"/>
@@ -1384,7 +1384,7 @@
       <c r="F39" s="17"/>
       <c r="G39" s="17"/>
     </row>
-    <row r="40" spans="1:7" ht="20.25" x14ac:dyDescent="0.25">
+    <row r="40" spans="1:7" ht="20.25" x14ac:dyDescent="0.45">
       <c r="A40" s="29" t="s">
         <v>25</v>
       </c>
@@ -1395,7 +1395,7 @@
       <c r="F40" s="17"/>
       <c r="G40" s="17"/>
     </row>
-    <row r="41" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="41" spans="1:7" x14ac:dyDescent="0.45">
       <c r="A41" s="23" t="s">
         <v>4</v>
       </c>
@@ -1414,83 +1414,83 @@
       </c>
       <c r="G41" s="17"/>
     </row>
-    <row r="42" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="42" spans="1:7" x14ac:dyDescent="0.45">
       <c r="A42" s="7">
-        <v>46298</v>
+        <v>46301</v>
       </c>
       <c r="B42" s="8"/>
       <c r="C42" s="20" t="s">
         <v>26</v>
       </c>
       <c r="D42" s="10">
-        <v>266.14</v>
+        <v>266.62</v>
       </c>
       <c r="E42" s="10">
-        <v>238.4</v>
+        <v>240.86</v>
       </c>
       <c r="F42" s="10">
-        <v>248.4</v>
+        <v>250.86</v>
       </c>
       <c r="G42" s="17"/>
     </row>
-    <row r="43" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="43" spans="1:7" x14ac:dyDescent="0.45">
       <c r="A43" s="11">
-        <v>46298</v>
+        <v>46301</v>
       </c>
       <c r="B43" s="12"/>
       <c r="C43" s="21" t="s">
         <v>27</v>
       </c>
       <c r="D43" s="13">
-        <v>265.75</v>
+        <v>266.23</v>
       </c>
       <c r="E43" s="13">
-        <v>238.81</v>
+        <v>241.27</v>
       </c>
       <c r="F43" s="13">
-        <v>248.81</v>
+        <v>251.27</v>
       </c>
       <c r="G43" s="17"/>
     </row>
-    <row r="44" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="44" spans="1:7" x14ac:dyDescent="0.45">
       <c r="A44" s="7">
-        <v>46297</v>
+        <v>46298</v>
       </c>
       <c r="B44" s="8"/>
       <c r="C44" s="20" t="s">
         <v>26</v>
       </c>
       <c r="D44" s="10">
-        <v>265.02999999999997</v>
+        <v>266.14</v>
       </c>
       <c r="E44" s="10">
-        <v>235.66</v>
+        <v>238.4</v>
       </c>
       <c r="F44" s="10">
-        <v>245.66</v>
+        <v>248.4</v>
       </c>
       <c r="G44" s="17"/>
     </row>
-    <row r="45" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="45" spans="1:7" x14ac:dyDescent="0.45">
       <c r="A45" s="11">
-        <v>46297</v>
+        <v>46298</v>
       </c>
       <c r="B45" s="12"/>
       <c r="C45" s="21" t="s">
         <v>27</v>
       </c>
       <c r="D45" s="13">
-        <v>264.64</v>
+        <v>265.75</v>
       </c>
       <c r="E45" s="13">
-        <v>236.07</v>
+        <v>238.81</v>
       </c>
       <c r="F45" s="13">
-        <v>246.07</v>
+        <v>248.81</v>
       </c>
       <c r="G45" s="17"/>
     </row>
-    <row r="46" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="46" spans="1:7" x14ac:dyDescent="0.45">
       <c r="A46" s="14"/>
       <c r="B46" s="24"/>
       <c r="C46" s="15"/>
@@ -1499,7 +1499,7 @@
       <c r="F46" s="16"/>
       <c r="G46" s="17"/>
     </row>
-    <row r="47" spans="1:7" ht="20.25" x14ac:dyDescent="0.25">
+    <row r="47" spans="1:7" ht="20.25" x14ac:dyDescent="0.45">
       <c r="A47" s="25" t="s">
         <v>28</v>
       </c>
@@ -1510,7 +1510,7 @@
       <c r="F47" s="17"/>
       <c r="G47" s="17"/>
     </row>
-    <row r="48" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="48" spans="1:7" x14ac:dyDescent="0.45">
       <c r="A48" s="23" t="s">
         <v>4</v>
       </c>
@@ -1529,83 +1529,83 @@
       </c>
       <c r="G48" s="17"/>
     </row>
-    <row r="49" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="49" spans="1:7" x14ac:dyDescent="0.45">
       <c r="A49" s="7">
-        <v>46298</v>
+        <v>46301</v>
       </c>
       <c r="B49" s="8"/>
       <c r="C49" s="20" t="s">
         <v>29</v>
       </c>
       <c r="D49" s="10">
-        <v>258.44</v>
+        <v>258.33999999999997</v>
       </c>
       <c r="E49" s="10">
-        <v>232.76</v>
+        <v>235.09</v>
       </c>
       <c r="F49" s="10">
-        <v>242.76</v>
+        <v>245.09</v>
       </c>
       <c r="G49" s="28"/>
     </row>
-    <row r="50" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="50" spans="1:7" x14ac:dyDescent="0.45">
       <c r="A50" s="11">
-        <v>46298</v>
+        <v>46301</v>
       </c>
       <c r="B50" s="12"/>
       <c r="C50" s="21" t="s">
         <v>30</v>
       </c>
       <c r="D50" s="13">
-        <v>256.13</v>
+        <v>255.96</v>
       </c>
       <c r="E50" s="13">
-        <v>232.45</v>
+        <v>234.76</v>
       </c>
       <c r="F50" s="13">
-        <v>242.45</v>
+        <v>244.76</v>
       </c>
       <c r="G50" s="28"/>
     </row>
-    <row r="51" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="51" spans="1:7" x14ac:dyDescent="0.45">
       <c r="A51" s="7">
-        <v>46297</v>
+        <v>46298</v>
       </c>
       <c r="B51" s="8"/>
       <c r="C51" s="20" t="s">
         <v>29</v>
       </c>
       <c r="D51" s="10">
-        <v>256.66000000000003</v>
+        <v>258.44</v>
       </c>
       <c r="E51" s="10">
-        <v>230.27</v>
+        <v>232.76</v>
       </c>
       <c r="F51" s="10">
-        <v>240.27</v>
+        <v>242.76</v>
       </c>
       <c r="G51" s="17"/>
     </row>
-    <row r="52" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="52" spans="1:7" x14ac:dyDescent="0.45">
       <c r="A52" s="11">
-        <v>46297</v>
+        <v>46298</v>
       </c>
       <c r="B52" s="12"/>
       <c r="C52" s="21" t="s">
         <v>30</v>
       </c>
       <c r="D52" s="13">
-        <v>254.39</v>
+        <v>256.13</v>
       </c>
       <c r="E52" s="13">
-        <v>229.99</v>
+        <v>232.45</v>
       </c>
       <c r="F52" s="13">
-        <v>239.99</v>
+        <v>242.45</v>
       </c>
       <c r="G52" s="17"/>
     </row>
-    <row r="53" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="53" spans="1:7" x14ac:dyDescent="0.45">
       <c r="A53" s="14"/>
       <c r="B53" s="14"/>
       <c r="C53" s="15"/>
@@ -1614,7 +1614,7 @@
       <c r="F53" s="16"/>
       <c r="G53" s="17"/>
     </row>
-    <row r="54" spans="1:7" ht="20.25" x14ac:dyDescent="0.25">
+    <row r="54" spans="1:7" ht="20.25" x14ac:dyDescent="0.45">
       <c r="A54" s="27" t="s">
         <v>31</v>
       </c>
@@ -1625,7 +1625,7 @@
       <c r="F54" s="17"/>
       <c r="G54" s="17"/>
     </row>
-    <row r="55" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="55" spans="1:7" x14ac:dyDescent="0.45">
       <c r="A55" s="23" t="s">
         <v>4</v>
       </c>
@@ -1644,54 +1644,54 @@
       </c>
       <c r="G55" s="17"/>
     </row>
-    <row r="56" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="56" spans="1:7" x14ac:dyDescent="0.45">
       <c r="A56" s="7">
-        <v>46298</v>
+        <v>46301</v>
       </c>
       <c r="B56" s="8"/>
       <c r="C56" s="20" t="s">
         <v>32</v>
       </c>
       <c r="D56" s="10">
-        <v>274.23</v>
+        <v>274.55</v>
       </c>
       <c r="E56" s="10">
-        <v>259.47000000000003</v>
+        <v>262.45999999999998</v>
       </c>
       <c r="F56" s="10">
-        <v>269.47000000000003</v>
+        <v>272.45999999999998</v>
       </c>
       <c r="G56" s="17"/>
     </row>
-    <row r="57" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="57" spans="1:7" x14ac:dyDescent="0.45">
       <c r="A57" s="11">
-        <v>46298</v>
+        <v>46301</v>
       </c>
       <c r="B57" s="12"/>
       <c r="C57" s="21" t="s">
         <v>33</v>
       </c>
       <c r="D57" s="13">
-        <v>263.51</v>
+        <v>263.89</v>
       </c>
       <c r="E57" s="13">
-        <v>242.49</v>
+        <v>244.66</v>
       </c>
       <c r="F57" s="13">
-        <v>252.49</v>
+        <v>254.66</v>
       </c>
       <c r="G57" s="17"/>
     </row>
-    <row r="58" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="58" spans="1:7" x14ac:dyDescent="0.45">
       <c r="A58" s="7">
-        <v>46298</v>
+        <v>46301</v>
       </c>
       <c r="B58" s="8"/>
       <c r="C58" s="20" t="s">
         <v>34</v>
       </c>
       <c r="D58" s="10">
-        <v>264.89999999999998</v>
+        <v>265.3</v>
       </c>
       <c r="E58" s="10" t="s">
         <v>18</v>
@@ -1701,111 +1701,111 @@
       </c>
       <c r="G58" s="17"/>
     </row>
-    <row r="59" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="59" spans="1:7" x14ac:dyDescent="0.45">
       <c r="A59" s="11">
-        <v>46298</v>
+        <v>46301</v>
       </c>
       <c r="B59" s="12"/>
       <c r="C59" s="21" t="s">
         <v>35</v>
       </c>
       <c r="D59" s="13">
-        <v>259.5</v>
+        <v>259.67</v>
       </c>
       <c r="E59" s="13">
-        <v>236.86</v>
+        <v>239.03</v>
       </c>
       <c r="F59" s="13" t="s">
         <v>18</v>
       </c>
       <c r="G59" s="17"/>
     </row>
-    <row r="60" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="60" spans="1:7" x14ac:dyDescent="0.45">
       <c r="A60" s="7">
-        <v>46298</v>
+        <v>46301</v>
       </c>
       <c r="B60" s="8"/>
       <c r="C60" s="20" t="s">
         <v>36</v>
       </c>
       <c r="D60" s="10">
-        <v>255.33</v>
+        <v>255.5</v>
       </c>
       <c r="E60" s="10">
-        <v>232.81</v>
+        <v>234.98</v>
       </c>
       <c r="F60" s="10">
-        <v>242.81</v>
+        <v>244.98</v>
       </c>
       <c r="G60" s="17"/>
     </row>
-    <row r="61" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="61" spans="1:7" x14ac:dyDescent="0.45">
       <c r="A61" s="11">
-        <v>46298</v>
+        <v>46301</v>
       </c>
       <c r="B61" s="12"/>
       <c r="C61" s="21" t="s">
         <v>37</v>
       </c>
       <c r="D61" s="13">
-        <v>260.72000000000003</v>
+        <v>260.88</v>
       </c>
       <c r="E61" s="13">
-        <v>253.37</v>
+        <v>256.08</v>
       </c>
       <c r="F61" s="13" t="s">
         <v>18</v>
       </c>
       <c r="G61" s="17"/>
     </row>
-    <row r="62" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="62" spans="1:7" x14ac:dyDescent="0.45">
       <c r="A62" s="7">
-        <v>46297</v>
+        <v>46298</v>
       </c>
       <c r="B62" s="8"/>
       <c r="C62" s="20" t="s">
         <v>32</v>
       </c>
       <c r="D62" s="10">
-        <v>273.31</v>
+        <v>274.23</v>
       </c>
       <c r="E62" s="10">
-        <v>256.16000000000003</v>
+        <v>259.47000000000003</v>
       </c>
       <c r="F62" s="10">
-        <v>266.16000000000003</v>
+        <v>269.47000000000003</v>
       </c>
       <c r="G62" s="17"/>
     </row>
-    <row r="63" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="63" spans="1:7" x14ac:dyDescent="0.45">
       <c r="A63" s="11">
-        <v>46297</v>
+        <v>46298</v>
       </c>
       <c r="B63" s="12"/>
       <c r="C63" s="21" t="s">
         <v>33</v>
       </c>
       <c r="D63" s="13">
-        <v>262.52</v>
+        <v>263.51</v>
       </c>
       <c r="E63" s="13">
-        <v>240.08</v>
+        <v>242.49</v>
       </c>
       <c r="F63" s="13">
-        <v>250.08</v>
+        <v>252.49</v>
       </c>
       <c r="G63" s="17"/>
     </row>
-    <row r="64" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="64" spans="1:7" x14ac:dyDescent="0.45">
       <c r="A64" s="7">
-        <v>46297</v>
+        <v>46298</v>
       </c>
       <c r="B64" s="8"/>
       <c r="C64" s="20" t="s">
         <v>34</v>
       </c>
       <c r="D64" s="10">
-        <v>263.88</v>
+        <v>264.89999999999998</v>
       </c>
       <c r="E64" s="10" t="s">
         <v>18</v>
@@ -1815,55 +1815,55 @@
       </c>
       <c r="G64" s="17"/>
     </row>
-    <row r="65" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="65" spans="1:6" x14ac:dyDescent="0.45">
       <c r="A65" s="11">
-        <v>46297</v>
+        <v>46298</v>
       </c>
       <c r="B65" s="12"/>
       <c r="C65" s="21" t="s">
         <v>35</v>
       </c>
       <c r="D65" s="13">
-        <v>258.74</v>
+        <v>259.5</v>
       </c>
       <c r="E65" s="13">
-        <v>234.45</v>
+        <v>236.86</v>
       </c>
       <c r="F65" s="13" t="s">
         <v>18</v>
       </c>
     </row>
-    <row r="66" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="66" spans="1:6" x14ac:dyDescent="0.45">
       <c r="A66" s="7">
-        <v>46297</v>
+        <v>46298</v>
       </c>
       <c r="B66" s="8"/>
       <c r="C66" s="20" t="s">
         <v>36</v>
       </c>
       <c r="D66" s="10">
-        <v>254.57</v>
+        <v>255.33</v>
       </c>
       <c r="E66" s="10">
-        <v>230.4</v>
+        <v>232.81</v>
       </c>
       <c r="F66" s="10">
-        <v>240.4</v>
-      </c>
-    </row>
-    <row r="67" spans="1:6" x14ac:dyDescent="0.25">
+        <v>242.81</v>
+      </c>
+    </row>
+    <row r="67" spans="1:6" x14ac:dyDescent="0.45">
       <c r="A67" s="11">
-        <v>46297</v>
+        <v>46298</v>
       </c>
       <c r="B67" s="12"/>
       <c r="C67" s="21" t="s">
         <v>37</v>
       </c>
       <c r="D67" s="13">
-        <v>259.97000000000003</v>
+        <v>260.72000000000003</v>
       </c>
       <c r="E67" s="13">
-        <v>250.37</v>
+        <v>253.37</v>
       </c>
       <c r="F67" s="13" t="s">
         <v>18</v>
@@ -1900,6 +1900,17 @@
 </file>
 
 <file path=customXml/item2.xml><?xml version="1.0" encoding="utf-8"?>
+<p:properties xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls">
+  <documentManagement>
+    <lcf76f155ced4ddcb4097134ff3c332f xmlns="87276d81-85f4-4ef2-9e6e-55066304288f">
+      <Terms xmlns="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
+    </lcf76f155ced4ddcb4097134ff3c332f>
+    <TaxCatchAll xmlns="b23b8984-eafa-4e79-985e-54f52f3da58e" xsi:nil="true"/>
+  </documentManagement>
+</p:properties>
+</file>
+
+<file path=customXml/item3.xml><?xml version="1.0" encoding="utf-8"?>
 <ct:contentTypeSchema xmlns:ct="http://schemas.microsoft.com/office/2006/metadata/contentType" xmlns:ma="http://schemas.microsoft.com/office/2006/metadata/properties/metaAttributes" ct:_="" ma:_="" ma:contentTypeName="Document" ma:contentTypeID="0x010100D3632DF5622958439304627C030B0427" ma:contentTypeVersion="18" ma:contentTypeDescription="Create a new document." ma:contentTypeScope="" ma:versionID="8c2ecbce386d6bac497f8eb2d8f0fb7a">
   <xsd:schema xmlns:xsd="http://www.w3.org/2001/XMLSchema" xmlns:xs="http://www.w3.org/2001/XMLSchema" xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:ns2="87276d81-85f4-4ef2-9e6e-55066304288f" xmlns:ns3="39e1dda6-d1d8-4c88-a3b9-f1abc1284bad" xmlns:ns4="b23b8984-eafa-4e79-985e-54f52f3da58e" targetNamespace="http://schemas.microsoft.com/office/2006/metadata/properties" ma:root="true" ma:fieldsID="4cfd0c2f651c1ce156ad4fcb44ea61dd" ns2:_="" ns3:_="" ns4:_="">
     <xsd:import namespace="87276d81-85f4-4ef2-9e6e-55066304288f"/>
@@ -2159,17 +2170,6 @@
 </ct:contentTypeSchema>
 </file>
 
-<file path=customXml/item3.xml><?xml version="1.0" encoding="utf-8"?>
-<p:properties xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls">
-  <documentManagement>
-    <lcf76f155ced4ddcb4097134ff3c332f xmlns="87276d81-85f4-4ef2-9e6e-55066304288f">
-      <Terms xmlns="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
-    </lcf76f155ced4ddcb4097134ff3c332f>
-    <TaxCatchAll xmlns="b23b8984-eafa-4e79-985e-54f52f3da58e" xsi:nil="true"/>
-  </documentManagement>
-</p:properties>
-</file>
-
 <file path=customXml/itemProps1.xml><?xml version="1.0" encoding="utf-8"?>
 <ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{F60519E9-FD90-4339-869C-BC2F85719BB8}">
   <ds:schemaRefs>
@@ -2179,6 +2179,17 @@
 </file>
 
 <file path=customXml/itemProps2.xml><?xml version="1.0" encoding="utf-8"?>
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{57A83D98-2BAE-4D83-823A-D31C464B620C}">
+  <ds:schemaRefs>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/properties"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
+    <ds:schemaRef ds:uri="87276d81-85f4-4ef2-9e6e-55066304288f"/>
+    <ds:schemaRef ds:uri="b23b8984-eafa-4e79-985e-54f52f3da58e"/>
+  </ds:schemaRefs>
+</ds:datastoreItem>
+</file>
+
+<file path=customXml/itemProps3.xml><?xml version="1.0" encoding="utf-8"?>
 <ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{B44E1863-2778-41F9-ACBA-48420F931671}">
   <ds:schemaRefs>
     <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/contentType"/>
@@ -2198,17 +2209,6 @@
 </ds:datastoreItem>
 </file>
 
-<file path=customXml/itemProps3.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{57A83D98-2BAE-4D83-823A-D31C464B620C}">
-  <ds:schemaRefs>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/properties"/>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
-    <ds:schemaRef ds:uri="87276d81-85f4-4ef2-9e6e-55066304288f"/>
-    <ds:schemaRef ds:uri="b23b8984-eafa-4e79-985e-54f52f3da58e"/>
-  </ds:schemaRefs>
-</ds:datastoreItem>
-</file>
-
 <file path=docMetadata/LabelInfo.xml><?xml version="1.0" encoding="utf-8"?>
 <clbl:labelList xmlns:clbl="http://schemas.microsoft.com/office/2020/mipLabelMetadata">
   <clbl:label id="{569bf4a9-87bd-4dbf-a36c-1db5158e5def}" enabled="1" method="Privileged" siteId="{ea80952e-a476-42d4-aaf4-5457852b0f7e}" removed="0"/>

</xml_diff>

<commit_message>
Tue Oct  6 07:39:03 UTC 2026
</commit_message>
<xml_diff>
--- a/bp.com-content-dam-bp-country-sites-en_au-australia-home-products-services-pricing-tgp-excel.xlsx
+++ b/bp.com-content-dam-bp-country-sites-en_au-australia-home-products-services-pricing-tgp-excel.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://bp365.sharepoint.com/sites/WholesalePricing/Shared Documents/B2C/TGP/Daily TGP/Web TGP/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="14_{675F50F3-9A37-4DB0-A9C5-58F9852F5865}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="14_{53F5A58C-9A1A-4C92-A8D9-CF60591FAF5A}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-8595" yWindow="-16320" windowWidth="29040" windowHeight="15720" xr2:uid="{1B412EEF-F96D-4DF4-A4E9-C7F0F183C2FB}"/>
+    <workbookView xWindow="-28920" yWindow="-60" windowWidth="29040" windowHeight="15720" xr2:uid="{1B412EEF-F96D-4DF4-A4E9-C7F0F183C2FB}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
@@ -715,15 +715,15 @@
     <pageSetUpPr fitToPage="1"/>
   </sheetPr>
   <dimension ref="A1:G67"/>
-  <sheetFormatPr defaultRowHeight="14.25" x14ac:dyDescent="0.45"/>
+  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
-    <col min="1" max="1" width="76.3984375" bestFit="1" customWidth="1"/>
-    <col min="2" max="2" width="6.3984375"/>
-    <col min="3" max="3" width="18.1328125" bestFit="1" customWidth="1"/>
-    <col min="4" max="7" width="7.1328125" bestFit="1" customWidth="1"/>
+    <col min="1" max="1" width="76.42578125" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="6.42578125"/>
+    <col min="3" max="3" width="18.140625" bestFit="1" customWidth="1"/>
+    <col min="4" max="7" width="7.140625" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:7" ht="22.15" x14ac:dyDescent="0.45">
+    <row r="1" spans="1:7" ht="23.25" x14ac:dyDescent="0.25">
       <c r="A1" s="30" t="s">
         <v>0</v>
       </c>
@@ -734,7 +734,7 @@
       <c r="F1" s="2"/>
       <c r="G1" s="2"/>
     </row>
-    <row r="2" spans="1:7" x14ac:dyDescent="0.45">
+    <row r="2" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A2" s="3"/>
       <c r="B2" s="1"/>
       <c r="C2" s="1"/>
@@ -743,7 +743,7 @@
       <c r="F2" s="2"/>
       <c r="G2" s="2"/>
     </row>
-    <row r="3" spans="1:7" x14ac:dyDescent="0.45">
+    <row r="3" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A3" s="3" t="s">
         <v>1</v>
       </c>
@@ -754,7 +754,7 @@
       <c r="F3" s="2"/>
       <c r="G3" s="2"/>
     </row>
-    <row r="4" spans="1:7" x14ac:dyDescent="0.45">
+    <row r="4" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A4" s="3" t="s">
         <v>2</v>
       </c>
@@ -765,7 +765,7 @@
       <c r="F4" s="2"/>
       <c r="G4" s="2"/>
     </row>
-    <row r="5" spans="1:7" x14ac:dyDescent="0.45">
+    <row r="5" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A5" s="3"/>
       <c r="B5" s="3"/>
       <c r="C5" s="1"/>
@@ -774,7 +774,7 @@
       <c r="F5" s="2"/>
       <c r="G5" s="2"/>
     </row>
-    <row r="6" spans="1:7" ht="20.25" x14ac:dyDescent="0.45">
+    <row r="6" spans="1:7" ht="20.25" x14ac:dyDescent="0.25">
       <c r="A6" s="29" t="s">
         <v>3</v>
       </c>
@@ -785,7 +785,7 @@
       <c r="F6" s="2"/>
       <c r="G6" s="2"/>
     </row>
-    <row r="7" spans="1:7" x14ac:dyDescent="0.45">
+    <row r="7" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A7" s="4" t="s">
         <v>4</v>
       </c>
@@ -806,133 +806,133 @@
         <v>9</v>
       </c>
     </row>
-    <row r="8" spans="1:7" x14ac:dyDescent="0.45">
+    <row r="8" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A8" s="7">
-        <v>46301</v>
+        <v>46302</v>
       </c>
       <c r="B8" s="8"/>
       <c r="C8" s="9" t="s">
         <v>10</v>
       </c>
       <c r="D8" s="10">
-        <v>260.49</v>
+        <v>259.45</v>
       </c>
       <c r="E8" s="10">
-        <v>233.42</v>
+        <v>234.76</v>
       </c>
       <c r="F8" s="10">
-        <v>243.42</v>
+        <v>244.76</v>
       </c>
       <c r="G8" s="10">
-        <v>231.03</v>
-      </c>
-    </row>
-    <row r="9" spans="1:7" x14ac:dyDescent="0.45">
+        <v>232.37</v>
+      </c>
+    </row>
+    <row r="9" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A9" s="11">
-        <v>46301</v>
+        <v>46302</v>
       </c>
       <c r="B9" s="12"/>
       <c r="C9" s="12" t="s">
         <v>11</v>
       </c>
       <c r="D9" s="13">
-        <v>260.49</v>
+        <v>259.45</v>
       </c>
       <c r="E9" s="13">
-        <v>233.42</v>
+        <v>234.76</v>
       </c>
       <c r="F9" s="13">
-        <v>243.42</v>
+        <v>244.76</v>
       </c>
       <c r="G9" s="13">
-        <v>231.03</v>
-      </c>
-    </row>
-    <row r="10" spans="1:7" x14ac:dyDescent="0.45">
+        <v>232.37</v>
+      </c>
+    </row>
+    <row r="10" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A10" s="7">
-        <v>46301</v>
+        <v>46302</v>
       </c>
       <c r="B10" s="8"/>
       <c r="C10" s="9" t="s">
         <v>12</v>
       </c>
       <c r="D10" s="10">
-        <v>258.17</v>
+        <v>257.36</v>
       </c>
       <c r="E10" s="10">
-        <v>234.17</v>
+        <v>235.72</v>
       </c>
       <c r="F10" s="10">
-        <v>244.17</v>
+        <v>245.72</v>
       </c>
       <c r="G10" s="10">
-        <v>232.58</v>
-      </c>
-    </row>
-    <row r="11" spans="1:7" x14ac:dyDescent="0.45">
+        <v>234.13</v>
+      </c>
+    </row>
+    <row r="11" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A11" s="11">
-        <v>46298</v>
+        <v>46301</v>
       </c>
       <c r="B11" s="12"/>
       <c r="C11" s="12" t="s">
         <v>10</v>
       </c>
       <c r="D11" s="13">
-        <v>260.33</v>
+        <v>260.49</v>
       </c>
       <c r="E11" s="13">
-        <v>231.27</v>
+        <v>233.42</v>
       </c>
       <c r="F11" s="13">
-        <v>241.27</v>
+        <v>243.42</v>
       </c>
       <c r="G11" s="13">
-        <v>228.88</v>
-      </c>
-    </row>
-    <row r="12" spans="1:7" x14ac:dyDescent="0.45">
+        <v>231.03</v>
+      </c>
+    </row>
+    <row r="12" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A12" s="7">
-        <v>46298</v>
+        <v>46301</v>
       </c>
       <c r="B12" s="8"/>
       <c r="C12" s="9" t="s">
         <v>11</v>
       </c>
       <c r="D12" s="10">
-        <v>260.33</v>
+        <v>260.49</v>
       </c>
       <c r="E12" s="10">
-        <v>231.27</v>
+        <v>233.42</v>
       </c>
       <c r="F12" s="10">
-        <v>241.27</v>
+        <v>243.42</v>
       </c>
       <c r="G12" s="10">
-        <v>228.88</v>
-      </c>
-    </row>
-    <row r="13" spans="1:7" x14ac:dyDescent="0.45">
+        <v>231.03</v>
+      </c>
+    </row>
+    <row r="13" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A13" s="11">
-        <v>46298</v>
+        <v>46301</v>
       </c>
       <c r="B13" s="12"/>
       <c r="C13" s="12" t="s">
         <v>12</v>
       </c>
       <c r="D13" s="13">
-        <v>257.8</v>
+        <v>258.17</v>
       </c>
       <c r="E13" s="13">
-        <v>231.83</v>
+        <v>234.17</v>
       </c>
       <c r="F13" s="13">
-        <v>241.83</v>
+        <v>244.17</v>
       </c>
       <c r="G13" s="13">
-        <v>230.24</v>
-      </c>
-    </row>
-    <row r="14" spans="1:7" x14ac:dyDescent="0.45">
+        <v>232.58</v>
+      </c>
+    </row>
+    <row r="14" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A14" s="14"/>
       <c r="B14" s="14"/>
       <c r="C14" s="15"/>
@@ -941,7 +941,7 @@
       <c r="F14" s="16"/>
       <c r="G14" s="16"/>
     </row>
-    <row r="15" spans="1:7" ht="20.25" x14ac:dyDescent="0.45">
+    <row r="15" spans="1:7" ht="20.25" x14ac:dyDescent="0.25">
       <c r="A15" s="29" t="s">
         <v>13</v>
       </c>
@@ -952,7 +952,7 @@
       <c r="F15" s="17"/>
       <c r="G15" s="17"/>
     </row>
-    <row r="16" spans="1:7" x14ac:dyDescent="0.45">
+    <row r="16" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A16" s="4" t="s">
         <v>4</v>
       </c>
@@ -971,45 +971,45 @@
       </c>
       <c r="G16" s="17"/>
     </row>
-    <row r="17" spans="1:7" x14ac:dyDescent="0.45">
+    <row r="17" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A17" s="7">
-        <v>46301</v>
+        <v>46302</v>
       </c>
       <c r="B17" s="8"/>
       <c r="C17" s="20" t="s">
         <v>14</v>
       </c>
       <c r="D17" s="10">
-        <v>261.77</v>
+        <v>260.83</v>
       </c>
       <c r="E17" s="10">
-        <v>239.48</v>
+        <v>240.93</v>
       </c>
       <c r="F17" s="10">
-        <v>249.48</v>
+        <v>250.93</v>
       </c>
       <c r="G17" s="17"/>
     </row>
-    <row r="18" spans="1:7" x14ac:dyDescent="0.45">
+    <row r="18" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A18" s="11">
-        <v>46298</v>
+        <v>46301</v>
       </c>
       <c r="B18" s="12"/>
       <c r="C18" s="12" t="s">
         <v>14</v>
       </c>
       <c r="D18" s="13">
-        <v>261.56</v>
+        <v>261.77</v>
       </c>
       <c r="E18" s="13">
-        <v>237.28</v>
+        <v>239.48</v>
       </c>
       <c r="F18" s="13">
-        <v>247.28</v>
+        <v>249.48</v>
       </c>
       <c r="G18" s="17"/>
     </row>
-    <row r="19" spans="1:7" x14ac:dyDescent="0.45">
+    <row r="19" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A19" s="14"/>
       <c r="B19" s="14"/>
       <c r="C19" s="15"/>
@@ -1018,7 +1018,7 @@
       <c r="F19" s="16"/>
       <c r="G19" s="17"/>
     </row>
-    <row r="20" spans="1:7" ht="20.25" x14ac:dyDescent="0.45">
+    <row r="20" spans="1:7" ht="20.25" x14ac:dyDescent="0.25">
       <c r="A20" s="29" t="s">
         <v>15</v>
       </c>
@@ -1029,7 +1029,7 @@
       <c r="F20" s="17"/>
       <c r="G20" s="17"/>
     </row>
-    <row r="21" spans="1:7" x14ac:dyDescent="0.45">
+    <row r="21" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A21" s="4" t="s">
         <v>4</v>
       </c>
@@ -1050,217 +1050,217 @@
         <v>9</v>
       </c>
     </row>
-    <row r="22" spans="1:7" x14ac:dyDescent="0.45">
+    <row r="22" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A22" s="7">
-        <v>46301</v>
+        <v>46302</v>
       </c>
       <c r="B22" s="8"/>
       <c r="C22" s="20" t="s">
         <v>16</v>
       </c>
       <c r="D22" s="10">
-        <v>261.62</v>
+        <v>260.58</v>
       </c>
       <c r="E22" s="10">
-        <v>233</v>
+        <v>234.34</v>
       </c>
       <c r="F22" s="10">
-        <v>242.6</v>
+        <v>243.94</v>
       </c>
       <c r="G22" s="10">
-        <v>229.37</v>
-      </c>
-    </row>
-    <row r="23" spans="1:7" x14ac:dyDescent="0.45">
+        <v>230.71</v>
+      </c>
+    </row>
+    <row r="23" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A23" s="11">
-        <v>46301</v>
+        <v>46302</v>
       </c>
       <c r="B23" s="12"/>
       <c r="C23" s="21" t="s">
         <v>17</v>
       </c>
       <c r="D23" s="13">
-        <v>263.11</v>
+        <v>262.31</v>
       </c>
       <c r="E23" s="13">
-        <v>244.62</v>
+        <v>246.22</v>
       </c>
       <c r="F23" s="13">
-        <v>254.62</v>
+        <v>256.22000000000003</v>
       </c>
       <c r="G23" s="13" t="s">
         <v>18</v>
       </c>
     </row>
-    <row r="24" spans="1:7" x14ac:dyDescent="0.45">
+    <row r="24" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A24" s="7">
-        <v>46301</v>
+        <v>46302</v>
       </c>
       <c r="B24" s="8"/>
       <c r="C24" s="20" t="s">
         <v>19</v>
       </c>
       <c r="D24" s="10">
-        <v>263.48</v>
+        <v>262.66000000000003</v>
       </c>
       <c r="E24" s="10">
-        <v>243.85</v>
+        <v>245.45</v>
       </c>
       <c r="F24" s="10">
-        <v>253.85</v>
+        <v>255.45</v>
       </c>
       <c r="G24" s="10" t="s">
         <v>18</v>
       </c>
     </row>
-    <row r="25" spans="1:7" x14ac:dyDescent="0.45">
+    <row r="25" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A25" s="11">
-        <v>46301</v>
+        <v>46302</v>
       </c>
       <c r="B25" s="12"/>
       <c r="C25" s="21" t="s">
         <v>20</v>
       </c>
       <c r="D25" s="13">
-        <v>260.14</v>
+        <v>259.32</v>
       </c>
       <c r="E25" s="13">
-        <v>244.08</v>
+        <v>245.69</v>
       </c>
       <c r="F25" s="13">
-        <v>254.08</v>
+        <v>255.69</v>
       </c>
       <c r="G25" s="13">
-        <v>239.92</v>
-      </c>
-    </row>
-    <row r="26" spans="1:7" x14ac:dyDescent="0.45">
+        <v>241.53</v>
+      </c>
+    </row>
+    <row r="26" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A26" s="7">
-        <v>46301</v>
+        <v>46302</v>
       </c>
       <c r="B26" s="8"/>
       <c r="C26" s="20" t="s">
         <v>21</v>
       </c>
       <c r="D26" s="10">
-        <v>261.72000000000003</v>
+        <v>260.87</v>
       </c>
       <c r="E26" s="10">
-        <v>245.61</v>
+        <v>247.23</v>
       </c>
       <c r="F26" s="10">
-        <v>255.61</v>
+        <v>257.23</v>
       </c>
       <c r="G26" s="10" t="s">
         <v>18</v>
       </c>
     </row>
-    <row r="27" spans="1:7" x14ac:dyDescent="0.45">
+    <row r="27" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A27" s="11">
-        <v>46298</v>
+        <v>46301</v>
       </c>
       <c r="B27" s="12"/>
       <c r="C27" s="12" t="s">
         <v>16</v>
       </c>
       <c r="D27" s="13">
-        <v>261.45</v>
+        <v>261.62</v>
       </c>
       <c r="E27" s="13">
-        <v>231.95</v>
+        <v>233</v>
       </c>
       <c r="F27" s="13">
-        <v>241.55</v>
+        <v>242.6</v>
       </c>
       <c r="G27" s="13">
-        <v>228.32</v>
-      </c>
-    </row>
-    <row r="28" spans="1:7" x14ac:dyDescent="0.45">
+        <v>229.37</v>
+      </c>
+    </row>
+    <row r="28" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A28" s="7">
-        <v>46298</v>
+        <v>46301</v>
       </c>
       <c r="B28" s="8"/>
       <c r="C28" s="20" t="s">
         <v>17</v>
       </c>
       <c r="D28" s="10">
-        <v>262.73</v>
+        <v>263.11</v>
       </c>
       <c r="E28" s="22">
-        <v>242.21</v>
+        <v>244.62</v>
       </c>
       <c r="F28" s="22">
-        <v>252.21</v>
+        <v>254.62</v>
       </c>
       <c r="G28" s="22" t="s">
         <v>18</v>
       </c>
     </row>
-    <row r="29" spans="1:7" x14ac:dyDescent="0.45">
+    <row r="29" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A29" s="11">
-        <v>46298</v>
+        <v>46301</v>
       </c>
       <c r="B29" s="12"/>
       <c r="C29" s="12" t="s">
         <v>19</v>
       </c>
       <c r="D29" s="13">
-        <v>263.11</v>
+        <v>263.48</v>
       </c>
       <c r="E29" s="13">
-        <v>241.45</v>
+        <v>243.85</v>
       </c>
       <c r="F29" s="13">
-        <v>251.45</v>
+        <v>253.85</v>
       </c>
       <c r="G29" s="13" t="s">
         <v>18</v>
       </c>
     </row>
-    <row r="30" spans="1:7" x14ac:dyDescent="0.45">
+    <row r="30" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A30" s="7">
-        <v>46298</v>
+        <v>46301</v>
       </c>
       <c r="B30" s="8"/>
       <c r="C30" s="20" t="s">
         <v>20</v>
       </c>
       <c r="D30" s="10">
-        <v>259.77999999999997</v>
+        <v>260.14</v>
       </c>
       <c r="E30" s="22">
-        <v>241.66</v>
+        <v>244.08</v>
       </c>
       <c r="F30" s="22">
-        <v>251.66</v>
+        <v>254.08</v>
       </c>
       <c r="G30" s="22">
-        <v>237.5</v>
-      </c>
-    </row>
-    <row r="31" spans="1:7" x14ac:dyDescent="0.45">
+        <v>239.92</v>
+      </c>
+    </row>
+    <row r="31" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A31" s="11">
-        <v>46298</v>
+        <v>46301</v>
       </c>
       <c r="B31" s="12"/>
       <c r="C31" s="12" t="s">
         <v>21</v>
       </c>
       <c r="D31" s="13">
-        <v>261.39999999999998</v>
+        <v>261.72000000000003</v>
       </c>
       <c r="E31" s="13">
-        <v>243.17</v>
+        <v>245.61</v>
       </c>
       <c r="F31" s="13">
-        <v>253.17</v>
+        <v>255.61</v>
       </c>
       <c r="G31" s="13" t="s">
         <v>18</v>
       </c>
     </row>
-    <row r="32" spans="1:7" x14ac:dyDescent="0.45">
+    <row r="32" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A32" s="14"/>
       <c r="B32" s="14"/>
       <c r="C32" s="15"/>
@@ -1269,7 +1269,7 @@
       <c r="F32" s="17"/>
       <c r="G32" s="17"/>
     </row>
-    <row r="33" spans="1:7" ht="20.25" x14ac:dyDescent="0.45">
+    <row r="33" spans="1:7" ht="20.25" x14ac:dyDescent="0.25">
       <c r="A33" s="29" t="s">
         <v>22</v>
       </c>
@@ -1280,7 +1280,7 @@
       <c r="F33" s="17"/>
       <c r="G33" s="17"/>
     </row>
-    <row r="34" spans="1:7" x14ac:dyDescent="0.45">
+    <row r="34" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A34" s="23" t="s">
         <v>4</v>
       </c>
@@ -1299,54 +1299,54 @@
       </c>
       <c r="G34" s="17"/>
     </row>
-    <row r="35" spans="1:7" x14ac:dyDescent="0.45">
+    <row r="35" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A35" s="7">
-        <v>46301</v>
+        <v>46302</v>
       </c>
       <c r="B35" s="8"/>
       <c r="C35" s="20" t="s">
         <v>23</v>
       </c>
       <c r="D35" s="10">
-        <v>256.70999999999998</v>
+        <v>255.91</v>
       </c>
       <c r="E35" s="10">
-        <v>229.8</v>
+        <v>231.35</v>
       </c>
       <c r="F35" s="10">
-        <v>238.8</v>
+        <v>240.35</v>
       </c>
       <c r="G35" s="17"/>
     </row>
-    <row r="36" spans="1:7" x14ac:dyDescent="0.45">
+    <row r="36" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A36" s="11">
-        <v>46298</v>
+        <v>46301</v>
       </c>
       <c r="B36" s="12"/>
       <c r="C36" s="12" t="s">
         <v>23</v>
       </c>
       <c r="D36" s="13">
-        <v>256.35000000000002</v>
+        <v>256.70999999999998</v>
       </c>
       <c r="E36" s="13">
-        <v>228.56</v>
+        <v>229.8</v>
       </c>
       <c r="F36" s="13">
-        <v>237.56</v>
+        <v>238.8</v>
       </c>
       <c r="G36" s="17"/>
     </row>
-    <row r="37" spans="1:7" x14ac:dyDescent="0.45">
+    <row r="37" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A37" s="7">
-        <v>46301</v>
+        <v>46302</v>
       </c>
       <c r="B37" s="8"/>
       <c r="C37" s="20" t="s">
         <v>24</v>
       </c>
       <c r="D37" s="10">
-        <v>272.33</v>
+        <v>271.52999999999997</v>
       </c>
       <c r="E37" s="10" t="s">
         <v>18</v>
@@ -1356,16 +1356,16 @@
       </c>
       <c r="G37" s="17"/>
     </row>
-    <row r="38" spans="1:7" x14ac:dyDescent="0.45">
+    <row r="38" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A38" s="11">
-        <v>46298</v>
+        <v>46301</v>
       </c>
       <c r="B38" s="12"/>
       <c r="C38" s="12" t="s">
         <v>24</v>
       </c>
       <c r="D38" s="13">
-        <v>271.97000000000003</v>
+        <v>272.33</v>
       </c>
       <c r="E38" s="13" t="s">
         <v>18</v>
@@ -1375,7 +1375,7 @@
       </c>
       <c r="G38" s="17"/>
     </row>
-    <row r="39" spans="1:7" x14ac:dyDescent="0.45">
+    <row r="39" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A39" s="24"/>
       <c r="B39" s="24"/>
       <c r="C39" s="15"/>
@@ -1384,7 +1384,7 @@
       <c r="F39" s="17"/>
       <c r="G39" s="17"/>
     </row>
-    <row r="40" spans="1:7" ht="20.25" x14ac:dyDescent="0.45">
+    <row r="40" spans="1:7" ht="20.25" x14ac:dyDescent="0.25">
       <c r="A40" s="29" t="s">
         <v>25</v>
       </c>
@@ -1395,7 +1395,7 @@
       <c r="F40" s="17"/>
       <c r="G40" s="17"/>
     </row>
-    <row r="41" spans="1:7" x14ac:dyDescent="0.45">
+    <row r="41" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A41" s="23" t="s">
         <v>4</v>
       </c>
@@ -1414,83 +1414,83 @@
       </c>
       <c r="G41" s="17"/>
     </row>
-    <row r="42" spans="1:7" x14ac:dyDescent="0.45">
+    <row r="42" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A42" s="7">
-        <v>46301</v>
+        <v>46302</v>
       </c>
       <c r="B42" s="8"/>
       <c r="C42" s="20" t="s">
         <v>26</v>
       </c>
       <c r="D42" s="10">
-        <v>266.62</v>
+        <v>265.91000000000003</v>
       </c>
       <c r="E42" s="10">
-        <v>240.86</v>
+        <v>242.51</v>
       </c>
       <c r="F42" s="10">
-        <v>250.86</v>
+        <v>252.51</v>
       </c>
       <c r="G42" s="17"/>
     </row>
-    <row r="43" spans="1:7" x14ac:dyDescent="0.45">
+    <row r="43" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A43" s="11">
-        <v>46301</v>
+        <v>46302</v>
       </c>
       <c r="B43" s="12"/>
       <c r="C43" s="21" t="s">
         <v>27</v>
       </c>
       <c r="D43" s="13">
-        <v>266.23</v>
+        <v>265.52</v>
       </c>
       <c r="E43" s="13">
-        <v>241.27</v>
+        <v>242.92</v>
       </c>
       <c r="F43" s="13">
-        <v>251.27</v>
+        <v>252.92</v>
       </c>
       <c r="G43" s="17"/>
     </row>
-    <row r="44" spans="1:7" x14ac:dyDescent="0.45">
+    <row r="44" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A44" s="7">
-        <v>46298</v>
+        <v>46301</v>
       </c>
       <c r="B44" s="8"/>
       <c r="C44" s="20" t="s">
         <v>26</v>
       </c>
       <c r="D44" s="10">
-        <v>266.14</v>
+        <v>266.62</v>
       </c>
       <c r="E44" s="10">
-        <v>238.4</v>
+        <v>240.86</v>
       </c>
       <c r="F44" s="10">
-        <v>248.4</v>
+        <v>250.86</v>
       </c>
       <c r="G44" s="17"/>
     </row>
-    <row r="45" spans="1:7" x14ac:dyDescent="0.45">
+    <row r="45" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A45" s="11">
-        <v>46298</v>
+        <v>46301</v>
       </c>
       <c r="B45" s="12"/>
       <c r="C45" s="21" t="s">
         <v>27</v>
       </c>
       <c r="D45" s="13">
-        <v>265.75</v>
+        <v>266.23</v>
       </c>
       <c r="E45" s="13">
-        <v>238.81</v>
+        <v>241.27</v>
       </c>
       <c r="F45" s="13">
-        <v>248.81</v>
+        <v>251.27</v>
       </c>
       <c r="G45" s="17"/>
     </row>
-    <row r="46" spans="1:7" x14ac:dyDescent="0.45">
+    <row r="46" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A46" s="14"/>
       <c r="B46" s="24"/>
       <c r="C46" s="15"/>
@@ -1499,7 +1499,7 @@
       <c r="F46" s="16"/>
       <c r="G46" s="17"/>
     </row>
-    <row r="47" spans="1:7" ht="20.25" x14ac:dyDescent="0.45">
+    <row r="47" spans="1:7" ht="20.25" x14ac:dyDescent="0.25">
       <c r="A47" s="25" t="s">
         <v>28</v>
       </c>
@@ -1510,7 +1510,7 @@
       <c r="F47" s="17"/>
       <c r="G47" s="17"/>
     </row>
-    <row r="48" spans="1:7" x14ac:dyDescent="0.45">
+    <row r="48" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A48" s="23" t="s">
         <v>4</v>
       </c>
@@ -1529,83 +1529,83 @@
       </c>
       <c r="G48" s="17"/>
     </row>
-    <row r="49" spans="1:7" x14ac:dyDescent="0.45">
+    <row r="49" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A49" s="7">
-        <v>46301</v>
+        <v>46302</v>
       </c>
       <c r="B49" s="8"/>
       <c r="C49" s="20" t="s">
         <v>29</v>
       </c>
       <c r="D49" s="10">
-        <v>258.33999999999997</v>
+        <v>257.63</v>
       </c>
       <c r="E49" s="10">
-        <v>235.09</v>
+        <v>236.24</v>
       </c>
       <c r="F49" s="10">
-        <v>245.09</v>
+        <v>246.24</v>
       </c>
       <c r="G49" s="28"/>
     </row>
-    <row r="50" spans="1:7" x14ac:dyDescent="0.45">
+    <row r="50" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A50" s="11">
-        <v>46301</v>
+        <v>46302</v>
       </c>
       <c r="B50" s="12"/>
       <c r="C50" s="21" t="s">
         <v>30</v>
       </c>
       <c r="D50" s="13">
-        <v>255.96</v>
+        <v>255.2</v>
       </c>
       <c r="E50" s="13">
-        <v>234.76</v>
+        <v>235.89</v>
       </c>
       <c r="F50" s="13">
-        <v>244.76</v>
+        <v>245.89</v>
       </c>
       <c r="G50" s="28"/>
     </row>
-    <row r="51" spans="1:7" x14ac:dyDescent="0.45">
+    <row r="51" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A51" s="7">
-        <v>46298</v>
+        <v>46301</v>
       </c>
       <c r="B51" s="8"/>
       <c r="C51" s="20" t="s">
         <v>29</v>
       </c>
       <c r="D51" s="10">
-        <v>258.44</v>
+        <v>258.33999999999997</v>
       </c>
       <c r="E51" s="10">
-        <v>232.76</v>
+        <v>235.09</v>
       </c>
       <c r="F51" s="10">
-        <v>242.76</v>
+        <v>245.09</v>
       </c>
       <c r="G51" s="17"/>
     </row>
-    <row r="52" spans="1:7" x14ac:dyDescent="0.45">
+    <row r="52" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A52" s="11">
-        <v>46298</v>
+        <v>46301</v>
       </c>
       <c r="B52" s="12"/>
       <c r="C52" s="21" t="s">
         <v>30</v>
       </c>
       <c r="D52" s="13">
-        <v>256.13</v>
+        <v>255.96</v>
       </c>
       <c r="E52" s="13">
-        <v>232.45</v>
+        <v>234.76</v>
       </c>
       <c r="F52" s="13">
-        <v>242.45</v>
+        <v>244.76</v>
       </c>
       <c r="G52" s="17"/>
     </row>
-    <row r="53" spans="1:7" x14ac:dyDescent="0.45">
+    <row r="53" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A53" s="14"/>
       <c r="B53" s="14"/>
       <c r="C53" s="15"/>
@@ -1614,7 +1614,7 @@
       <c r="F53" s="16"/>
       <c r="G53" s="17"/>
     </row>
-    <row r="54" spans="1:7" ht="20.25" x14ac:dyDescent="0.45">
+    <row r="54" spans="1:7" ht="20.25" x14ac:dyDescent="0.25">
       <c r="A54" s="27" t="s">
         <v>31</v>
       </c>
@@ -1625,7 +1625,7 @@
       <c r="F54" s="17"/>
       <c r="G54" s="17"/>
     </row>
-    <row r="55" spans="1:7" x14ac:dyDescent="0.45">
+    <row r="55" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A55" s="23" t="s">
         <v>4</v>
       </c>
@@ -1644,54 +1644,54 @@
       </c>
       <c r="G55" s="17"/>
     </row>
-    <row r="56" spans="1:7" x14ac:dyDescent="0.45">
+    <row r="56" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A56" s="7">
-        <v>46301</v>
+        <v>46302</v>
       </c>
       <c r="B56" s="8"/>
       <c r="C56" s="20" t="s">
         <v>32</v>
       </c>
       <c r="D56" s="10">
-        <v>274.55</v>
+        <v>273.7</v>
       </c>
       <c r="E56" s="10">
-        <v>262.45999999999998</v>
+        <v>264.52</v>
       </c>
       <c r="F56" s="10">
-        <v>272.45999999999998</v>
+        <v>274.52</v>
       </c>
       <c r="G56" s="17"/>
     </row>
-    <row r="57" spans="1:7" x14ac:dyDescent="0.45">
+    <row r="57" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A57" s="11">
-        <v>46301</v>
+        <v>46302</v>
       </c>
       <c r="B57" s="12"/>
       <c r="C57" s="21" t="s">
         <v>33</v>
       </c>
       <c r="D57" s="13">
-        <v>263.89</v>
+        <v>263.08</v>
       </c>
       <c r="E57" s="13">
-        <v>244.66</v>
+        <v>246.07</v>
       </c>
       <c r="F57" s="13">
-        <v>254.66</v>
+        <v>256.07</v>
       </c>
       <c r="G57" s="17"/>
     </row>
-    <row r="58" spans="1:7" x14ac:dyDescent="0.45">
+    <row r="58" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A58" s="7">
-        <v>46301</v>
+        <v>46302</v>
       </c>
       <c r="B58" s="8"/>
       <c r="C58" s="20" t="s">
         <v>34</v>
       </c>
       <c r="D58" s="10">
-        <v>265.3</v>
+        <v>264.51</v>
       </c>
       <c r="E58" s="10" t="s">
         <v>18</v>
@@ -1701,111 +1701,111 @@
       </c>
       <c r="G58" s="17"/>
     </row>
-    <row r="59" spans="1:7" x14ac:dyDescent="0.45">
+    <row r="59" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A59" s="11">
-        <v>46301</v>
+        <v>46302</v>
       </c>
       <c r="B59" s="12"/>
       <c r="C59" s="21" t="s">
         <v>35</v>
       </c>
       <c r="D59" s="13">
-        <v>259.67</v>
+        <v>258.70999999999998</v>
       </c>
       <c r="E59" s="13">
-        <v>239.03</v>
+        <v>240.44</v>
       </c>
       <c r="F59" s="13" t="s">
         <v>18</v>
       </c>
       <c r="G59" s="17"/>
     </row>
-    <row r="60" spans="1:7" x14ac:dyDescent="0.45">
+    <row r="60" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A60" s="7">
-        <v>46301</v>
+        <v>46302</v>
       </c>
       <c r="B60" s="8"/>
       <c r="C60" s="20" t="s">
         <v>36</v>
       </c>
       <c r="D60" s="10">
-        <v>255.5</v>
+        <v>254.54</v>
       </c>
       <c r="E60" s="10">
-        <v>234.98</v>
+        <v>236.39</v>
       </c>
       <c r="F60" s="10">
-        <v>244.98</v>
+        <v>246.39</v>
       </c>
       <c r="G60" s="17"/>
     </row>
-    <row r="61" spans="1:7" x14ac:dyDescent="0.45">
+    <row r="61" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A61" s="11">
-        <v>46301</v>
+        <v>46302</v>
       </c>
       <c r="B61" s="12"/>
       <c r="C61" s="21" t="s">
         <v>37</v>
       </c>
       <c r="D61" s="13">
-        <v>260.88</v>
+        <v>259.91000000000003</v>
       </c>
       <c r="E61" s="13">
-        <v>256.08</v>
+        <v>257.92</v>
       </c>
       <c r="F61" s="13" t="s">
         <v>18</v>
       </c>
       <c r="G61" s="17"/>
     </row>
-    <row r="62" spans="1:7" x14ac:dyDescent="0.45">
+    <row r="62" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A62" s="7">
-        <v>46298</v>
+        <v>46301</v>
       </c>
       <c r="B62" s="8"/>
       <c r="C62" s="20" t="s">
         <v>32</v>
       </c>
       <c r="D62" s="10">
-        <v>274.23</v>
+        <v>274.55</v>
       </c>
       <c r="E62" s="10">
-        <v>259.47000000000003</v>
+        <v>262.45999999999998</v>
       </c>
       <c r="F62" s="10">
-        <v>269.47000000000003</v>
+        <v>272.45999999999998</v>
       </c>
       <c r="G62" s="17"/>
     </row>
-    <row r="63" spans="1:7" x14ac:dyDescent="0.45">
+    <row r="63" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A63" s="11">
-        <v>46298</v>
+        <v>46301</v>
       </c>
       <c r="B63" s="12"/>
       <c r="C63" s="21" t="s">
         <v>33</v>
       </c>
       <c r="D63" s="13">
-        <v>263.51</v>
+        <v>263.89</v>
       </c>
       <c r="E63" s="13">
-        <v>242.49</v>
+        <v>244.66</v>
       </c>
       <c r="F63" s="13">
-        <v>252.49</v>
+        <v>254.66</v>
       </c>
       <c r="G63" s="17"/>
     </row>
-    <row r="64" spans="1:7" x14ac:dyDescent="0.45">
+    <row r="64" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A64" s="7">
-        <v>46298</v>
+        <v>46301</v>
       </c>
       <c r="B64" s="8"/>
       <c r="C64" s="20" t="s">
         <v>34</v>
       </c>
       <c r="D64" s="10">
-        <v>264.89999999999998</v>
+        <v>265.3</v>
       </c>
       <c r="E64" s="10" t="s">
         <v>18</v>
@@ -1815,55 +1815,55 @@
       </c>
       <c r="G64" s="17"/>
     </row>
-    <row r="65" spans="1:6" x14ac:dyDescent="0.45">
+    <row r="65" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A65" s="11">
-        <v>46298</v>
+        <v>46301</v>
       </c>
       <c r="B65" s="12"/>
       <c r="C65" s="21" t="s">
         <v>35</v>
       </c>
       <c r="D65" s="13">
-        <v>259.5</v>
+        <v>259.67</v>
       </c>
       <c r="E65" s="13">
-        <v>236.86</v>
+        <v>239.03</v>
       </c>
       <c r="F65" s="13" t="s">
         <v>18</v>
       </c>
     </row>
-    <row r="66" spans="1:6" x14ac:dyDescent="0.45">
+    <row r="66" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A66" s="7">
-        <v>46298</v>
+        <v>46301</v>
       </c>
       <c r="B66" s="8"/>
       <c r="C66" s="20" t="s">
         <v>36</v>
       </c>
       <c r="D66" s="10">
-        <v>255.33</v>
+        <v>255.5</v>
       </c>
       <c r="E66" s="10">
-        <v>232.81</v>
+        <v>234.98</v>
       </c>
       <c r="F66" s="10">
-        <v>242.81</v>
-      </c>
-    </row>
-    <row r="67" spans="1:6" x14ac:dyDescent="0.45">
+        <v>244.98</v>
+      </c>
+    </row>
+    <row r="67" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A67" s="11">
-        <v>46298</v>
+        <v>46301</v>
       </c>
       <c r="B67" s="12"/>
       <c r="C67" s="21" t="s">
         <v>37</v>
       </c>
       <c r="D67" s="13">
-        <v>260.72000000000003</v>
+        <v>260.88</v>
       </c>
       <c r="E67" s="13">
-        <v>253.37</v>
+        <v>256.08</v>
       </c>
       <c r="F67" s="13" t="s">
         <v>18</v>
@@ -1891,26 +1891,6 @@
 </file>
 
 <file path=customXml/item1.xml><?xml version="1.0" encoding="utf-8"?>
-<?mso-contentType ?>
-<FormTemplates xmlns="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms">
-  <Display>DocumentLibraryForm</Display>
-  <Edit>DocumentLibraryForm</Edit>
-  <New>DocumentLibraryForm</New>
-</FormTemplates>
-</file>
-
-<file path=customXml/item2.xml><?xml version="1.0" encoding="utf-8"?>
-<p:properties xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls">
-  <documentManagement>
-    <lcf76f155ced4ddcb4097134ff3c332f xmlns="87276d81-85f4-4ef2-9e6e-55066304288f">
-      <Terms xmlns="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
-    </lcf76f155ced4ddcb4097134ff3c332f>
-    <TaxCatchAll xmlns="b23b8984-eafa-4e79-985e-54f52f3da58e" xsi:nil="true"/>
-  </documentManagement>
-</p:properties>
-</file>
-
-<file path=customXml/item3.xml><?xml version="1.0" encoding="utf-8"?>
 <ct:contentTypeSchema xmlns:ct="http://schemas.microsoft.com/office/2006/metadata/contentType" xmlns:ma="http://schemas.microsoft.com/office/2006/metadata/properties/metaAttributes" ct:_="" ma:_="" ma:contentTypeName="Document" ma:contentTypeID="0x010100D3632DF5622958439304627C030B0427" ma:contentTypeVersion="18" ma:contentTypeDescription="Create a new document." ma:contentTypeScope="" ma:versionID="8c2ecbce386d6bac497f8eb2d8f0fb7a">
   <xsd:schema xmlns:xsd="http://www.w3.org/2001/XMLSchema" xmlns:xs="http://www.w3.org/2001/XMLSchema" xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:ns2="87276d81-85f4-4ef2-9e6e-55066304288f" xmlns:ns3="39e1dda6-d1d8-4c88-a3b9-f1abc1284bad" xmlns:ns4="b23b8984-eafa-4e79-985e-54f52f3da58e" targetNamespace="http://schemas.microsoft.com/office/2006/metadata/properties" ma:root="true" ma:fieldsID="4cfd0c2f651c1ce156ad4fcb44ea61dd" ns2:_="" ns3:_="" ns4:_="">
     <xsd:import namespace="87276d81-85f4-4ef2-9e6e-55066304288f"/>
@@ -2170,26 +2150,27 @@
 </ct:contentTypeSchema>
 </file>
 
-<file path=customXml/itemProps1.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{F60519E9-FD90-4339-869C-BC2F85719BB8}">
-  <ds:schemaRefs>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms"/>
-  </ds:schemaRefs>
-</ds:datastoreItem>
+<file path=customXml/item2.xml><?xml version="1.0" encoding="utf-8"?>
+<?mso-contentType ?>
+<FormTemplates xmlns="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms">
+  <Display>DocumentLibraryForm</Display>
+  <Edit>DocumentLibraryForm</Edit>
+  <New>DocumentLibraryForm</New>
+</FormTemplates>
 </file>
 
-<file path=customXml/itemProps2.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{57A83D98-2BAE-4D83-823A-D31C464B620C}">
-  <ds:schemaRefs>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/properties"/>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
-    <ds:schemaRef ds:uri="87276d81-85f4-4ef2-9e6e-55066304288f"/>
-    <ds:schemaRef ds:uri="b23b8984-eafa-4e79-985e-54f52f3da58e"/>
-  </ds:schemaRefs>
-</ds:datastoreItem>
+<file path=customXml/item3.xml><?xml version="1.0" encoding="utf-8"?>
+<p:properties xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls">
+  <documentManagement>
+    <lcf76f155ced4ddcb4097134ff3c332f xmlns="87276d81-85f4-4ef2-9e6e-55066304288f">
+      <Terms xmlns="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
+    </lcf76f155ced4ddcb4097134ff3c332f>
+    <TaxCatchAll xmlns="b23b8984-eafa-4e79-985e-54f52f3da58e" xsi:nil="true"/>
+  </documentManagement>
+</p:properties>
 </file>
 
-<file path=customXml/itemProps3.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=customXml/itemProps1.xml><?xml version="1.0" encoding="utf-8"?>
 <ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{B44E1863-2778-41F9-ACBA-48420F931671}">
   <ds:schemaRefs>
     <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/contentType"/>
@@ -2209,6 +2190,25 @@
 </ds:datastoreItem>
 </file>
 
+<file path=customXml/itemProps2.xml><?xml version="1.0" encoding="utf-8"?>
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{F60519E9-FD90-4339-869C-BC2F85719BB8}">
+  <ds:schemaRefs>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms"/>
+  </ds:schemaRefs>
+</ds:datastoreItem>
+</file>
+
+<file path=customXml/itemProps3.xml><?xml version="1.0" encoding="utf-8"?>
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{57A83D98-2BAE-4D83-823A-D31C464B620C}">
+  <ds:schemaRefs>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/properties"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
+    <ds:schemaRef ds:uri="87276d81-85f4-4ef2-9e6e-55066304288f"/>
+    <ds:schemaRef ds:uri="b23b8984-eafa-4e79-985e-54f52f3da58e"/>
+  </ds:schemaRefs>
+</ds:datastoreItem>
+</file>
+
 <file path=docMetadata/LabelInfo.xml><?xml version="1.0" encoding="utf-8"?>
 <clbl:labelList xmlns:clbl="http://schemas.microsoft.com/office/2020/mipLabelMetadata">
   <clbl:label id="{569bf4a9-87bd-4dbf-a36c-1db5158e5def}" enabled="1" method="Privileged" siteId="{ea80952e-a476-42d4-aaf4-5457852b0f7e}" removed="0"/>

</xml_diff>

<commit_message>
Wed Oct  7 07:19:42 UTC 2026
</commit_message>
<xml_diff>
--- a/bp.com-content-dam-bp-country-sites-en_au-australia-home-products-services-pricing-tgp-excel.xlsx
+++ b/bp.com-content-dam-bp-country-sites-en_au-australia-home-products-services-pricing-tgp-excel.xlsx
@@ -8,14 +8,14 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://bp365.sharepoint.com/sites/WholesalePricing/Shared Documents/B2C/TGP/Daily TGP/Web TGP/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="14_{53F5A58C-9A1A-4C92-A8D9-CF60591FAF5A}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="14_{4E732A02-49B6-4485-8258-62E7190CD32E}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-28920" yWindow="-60" windowWidth="29040" windowHeight="15720" xr2:uid="{1B412EEF-F96D-4DF4-A4E9-C7F0F183C2FB}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
   </sheets>
-  <calcPr calcId="191028"/>
+  <calcPr calcId="191028" calcOnSave="0"/>
   <extLst>
     <ext xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" uri="{140A7094-0E35-4892-8432-C4D2E57EDEB5}">
       <x15:workbookPr chartTrackingRefBase="1"/>
@@ -808,128 +808,128 @@
     </row>
     <row r="8" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A8" s="7">
-        <v>46302</v>
+        <v>46303</v>
       </c>
       <c r="B8" s="8"/>
       <c r="C8" s="9" t="s">
         <v>10</v>
       </c>
       <c r="D8" s="10">
-        <v>259.45</v>
+        <v>260.22000000000003</v>
       </c>
       <c r="E8" s="10">
-        <v>234.76</v>
+        <v>236.63</v>
       </c>
       <c r="F8" s="10">
-        <v>244.76</v>
+        <v>246.63</v>
       </c>
       <c r="G8" s="10">
-        <v>232.37</v>
+        <v>234.24</v>
       </c>
     </row>
     <row r="9" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A9" s="11">
-        <v>46302</v>
+        <v>46303</v>
       </c>
       <c r="B9" s="12"/>
       <c r="C9" s="12" t="s">
         <v>11</v>
       </c>
       <c r="D9" s="13">
-        <v>259.45</v>
+        <v>260.22000000000003</v>
       </c>
       <c r="E9" s="13">
-        <v>234.76</v>
+        <v>236.63</v>
       </c>
       <c r="F9" s="13">
-        <v>244.76</v>
+        <v>246.63</v>
       </c>
       <c r="G9" s="13">
-        <v>232.37</v>
+        <v>234.24</v>
       </c>
     </row>
     <row r="10" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A10" s="7">
-        <v>46302</v>
+        <v>46303</v>
       </c>
       <c r="B10" s="8"/>
       <c r="C10" s="9" t="s">
         <v>12</v>
       </c>
       <c r="D10" s="10">
-        <v>257.36</v>
+        <v>256.7</v>
       </c>
       <c r="E10" s="10">
-        <v>235.72</v>
+        <v>237.25</v>
       </c>
       <c r="F10" s="10">
-        <v>245.72</v>
+        <v>247.25</v>
       </c>
       <c r="G10" s="10">
-        <v>234.13</v>
+        <v>235.65</v>
       </c>
     </row>
     <row r="11" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A11" s="11">
-        <v>46301</v>
+        <v>46302</v>
       </c>
       <c r="B11" s="12"/>
       <c r="C11" s="12" t="s">
         <v>10</v>
       </c>
       <c r="D11" s="13">
-        <v>260.49</v>
+        <v>259.45</v>
       </c>
       <c r="E11" s="13">
-        <v>233.42</v>
+        <v>234.76</v>
       </c>
       <c r="F11" s="13">
-        <v>243.42</v>
+        <v>244.76</v>
       </c>
       <c r="G11" s="13">
-        <v>231.03</v>
+        <v>232.37</v>
       </c>
     </row>
     <row r="12" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A12" s="7">
-        <v>46301</v>
+        <v>46302</v>
       </c>
       <c r="B12" s="8"/>
       <c r="C12" s="9" t="s">
         <v>11</v>
       </c>
       <c r="D12" s="10">
-        <v>260.49</v>
+        <v>259.45</v>
       </c>
       <c r="E12" s="10">
-        <v>233.42</v>
+        <v>234.76</v>
       </c>
       <c r="F12" s="10">
-        <v>243.42</v>
+        <v>244.76</v>
       </c>
       <c r="G12" s="10">
-        <v>231.03</v>
+        <v>232.37</v>
       </c>
     </row>
     <row r="13" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A13" s="11">
-        <v>46301</v>
+        <v>46302</v>
       </c>
       <c r="B13" s="12"/>
       <c r="C13" s="12" t="s">
         <v>12</v>
       </c>
       <c r="D13" s="13">
-        <v>258.17</v>
+        <v>257.36</v>
       </c>
       <c r="E13" s="13">
-        <v>234.17</v>
+        <v>235.72</v>
       </c>
       <c r="F13" s="13">
-        <v>244.17</v>
+        <v>245.72</v>
       </c>
       <c r="G13" s="13">
-        <v>232.58</v>
+        <v>234.13</v>
       </c>
     </row>
     <row r="14" spans="1:7" x14ac:dyDescent="0.25">
@@ -973,39 +973,39 @@
     </row>
     <row r="17" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A17" s="7">
-        <v>46302</v>
+        <v>46303</v>
       </c>
       <c r="B17" s="8"/>
       <c r="C17" s="20" t="s">
         <v>14</v>
       </c>
       <c r="D17" s="10">
-        <v>260.83</v>
+        <v>260.07</v>
       </c>
       <c r="E17" s="10">
-        <v>240.93</v>
+        <v>242.36</v>
       </c>
       <c r="F17" s="10">
-        <v>250.93</v>
+        <v>252.36</v>
       </c>
       <c r="G17" s="17"/>
     </row>
     <row r="18" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A18" s="11">
-        <v>46301</v>
+        <v>46302</v>
       </c>
       <c r="B18" s="12"/>
       <c r="C18" s="12" t="s">
         <v>14</v>
       </c>
       <c r="D18" s="13">
-        <v>261.77</v>
+        <v>260.83</v>
       </c>
       <c r="E18" s="13">
-        <v>239.48</v>
+        <v>240.93</v>
       </c>
       <c r="F18" s="13">
-        <v>249.48</v>
+        <v>250.93</v>
       </c>
       <c r="G18" s="17"/>
     </row>
@@ -1052,41 +1052,41 @@
     </row>
     <row r="22" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A22" s="7">
-        <v>46302</v>
+        <v>46303</v>
       </c>
       <c r="B22" s="8"/>
       <c r="C22" s="20" t="s">
         <v>16</v>
       </c>
       <c r="D22" s="10">
-        <v>260.58</v>
+        <v>261.35000000000002</v>
       </c>
       <c r="E22" s="10">
-        <v>234.34</v>
+        <v>236.21</v>
       </c>
       <c r="F22" s="10">
-        <v>243.94</v>
+        <v>245.81</v>
       </c>
       <c r="G22" s="10">
-        <v>230.71</v>
+        <v>232.58</v>
       </c>
     </row>
     <row r="23" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A23" s="11">
-        <v>46302</v>
+        <v>46303</v>
       </c>
       <c r="B23" s="12"/>
       <c r="C23" s="21" t="s">
         <v>17</v>
       </c>
       <c r="D23" s="13">
-        <v>262.31</v>
+        <v>261.67</v>
       </c>
       <c r="E23" s="13">
-        <v>246.22</v>
+        <v>247.79</v>
       </c>
       <c r="F23" s="13">
-        <v>256.22000000000003</v>
+        <v>257.79000000000002</v>
       </c>
       <c r="G23" s="13" t="s">
         <v>18</v>
@@ -1094,20 +1094,20 @@
     </row>
     <row r="24" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A24" s="7">
-        <v>46302</v>
+        <v>46303</v>
       </c>
       <c r="B24" s="8"/>
       <c r="C24" s="20" t="s">
         <v>19</v>
       </c>
       <c r="D24" s="10">
-        <v>262.66000000000003</v>
+        <v>262.01</v>
       </c>
       <c r="E24" s="10">
-        <v>245.45</v>
+        <v>247.01</v>
       </c>
       <c r="F24" s="10">
-        <v>255.45</v>
+        <v>257.02</v>
       </c>
       <c r="G24" s="10" t="s">
         <v>18</v>
@@ -1115,41 +1115,41 @@
     </row>
     <row r="25" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A25" s="11">
-        <v>46302</v>
+        <v>46303</v>
       </c>
       <c r="B25" s="12"/>
       <c r="C25" s="21" t="s">
         <v>20</v>
       </c>
       <c r="D25" s="13">
-        <v>259.32</v>
+        <v>258.66000000000003</v>
       </c>
       <c r="E25" s="13">
-        <v>245.69</v>
+        <v>247.27</v>
       </c>
       <c r="F25" s="13">
-        <v>255.69</v>
+        <v>257.27</v>
       </c>
       <c r="G25" s="13">
-        <v>241.53</v>
+        <v>243.11</v>
       </c>
     </row>
     <row r="26" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A26" s="7">
-        <v>46302</v>
+        <v>46303</v>
       </c>
       <c r="B26" s="8"/>
       <c r="C26" s="20" t="s">
         <v>21</v>
       </c>
       <c r="D26" s="10">
-        <v>260.87</v>
+        <v>260.19</v>
       </c>
       <c r="E26" s="10">
-        <v>247.23</v>
+        <v>248.82</v>
       </c>
       <c r="F26" s="10">
-        <v>257.23</v>
+        <v>258.82</v>
       </c>
       <c r="G26" s="10" t="s">
         <v>18</v>
@@ -1157,41 +1157,41 @@
     </row>
     <row r="27" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A27" s="11">
-        <v>46301</v>
+        <v>46302</v>
       </c>
       <c r="B27" s="12"/>
       <c r="C27" s="12" t="s">
         <v>16</v>
       </c>
       <c r="D27" s="13">
-        <v>261.62</v>
+        <v>260.58</v>
       </c>
       <c r="E27" s="13">
-        <v>233</v>
+        <v>234.34</v>
       </c>
       <c r="F27" s="13">
-        <v>242.6</v>
+        <v>243.94</v>
       </c>
       <c r="G27" s="13">
-        <v>229.37</v>
+        <v>230.71</v>
       </c>
     </row>
     <row r="28" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A28" s="7">
-        <v>46301</v>
+        <v>46302</v>
       </c>
       <c r="B28" s="8"/>
       <c r="C28" s="20" t="s">
         <v>17</v>
       </c>
       <c r="D28" s="10">
-        <v>263.11</v>
+        <v>262.31</v>
       </c>
       <c r="E28" s="22">
-        <v>244.62</v>
+        <v>246.22</v>
       </c>
       <c r="F28" s="22">
-        <v>254.62</v>
+        <v>256.22000000000003</v>
       </c>
       <c r="G28" s="22" t="s">
         <v>18</v>
@@ -1199,20 +1199,20 @@
     </row>
     <row r="29" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A29" s="11">
-        <v>46301</v>
+        <v>46302</v>
       </c>
       <c r="B29" s="12"/>
       <c r="C29" s="12" t="s">
         <v>19</v>
       </c>
       <c r="D29" s="13">
-        <v>263.48</v>
+        <v>262.66000000000003</v>
       </c>
       <c r="E29" s="13">
-        <v>243.85</v>
+        <v>245.45</v>
       </c>
       <c r="F29" s="13">
-        <v>253.85</v>
+        <v>255.45</v>
       </c>
       <c r="G29" s="13" t="s">
         <v>18</v>
@@ -1220,41 +1220,41 @@
     </row>
     <row r="30" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A30" s="7">
-        <v>46301</v>
+        <v>46302</v>
       </c>
       <c r="B30" s="8"/>
       <c r="C30" s="20" t="s">
         <v>20</v>
       </c>
       <c r="D30" s="10">
-        <v>260.14</v>
+        <v>259.32</v>
       </c>
       <c r="E30" s="22">
-        <v>244.08</v>
+        <v>245.69</v>
       </c>
       <c r="F30" s="22">
-        <v>254.08</v>
+        <v>255.69</v>
       </c>
       <c r="G30" s="22">
-        <v>239.92</v>
+        <v>241.53</v>
       </c>
     </row>
     <row r="31" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A31" s="11">
-        <v>46301</v>
+        <v>46302</v>
       </c>
       <c r="B31" s="12"/>
       <c r="C31" s="12" t="s">
         <v>21</v>
       </c>
       <c r="D31" s="13">
-        <v>261.72000000000003</v>
+        <v>260.87</v>
       </c>
       <c r="E31" s="13">
-        <v>245.61</v>
+        <v>247.23</v>
       </c>
       <c r="F31" s="13">
-        <v>255.61</v>
+        <v>257.23</v>
       </c>
       <c r="G31" s="13" t="s">
         <v>18</v>
@@ -1301,52 +1301,52 @@
     </row>
     <row r="35" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A35" s="7">
-        <v>46302</v>
+        <v>46303</v>
       </c>
       <c r="B35" s="8"/>
       <c r="C35" s="20" t="s">
         <v>23</v>
       </c>
       <c r="D35" s="10">
-        <v>255.91</v>
+        <v>255.26</v>
       </c>
       <c r="E35" s="10">
-        <v>231.35</v>
+        <v>232.87</v>
       </c>
       <c r="F35" s="10">
-        <v>240.35</v>
+        <v>241.87</v>
       </c>
       <c r="G35" s="17"/>
     </row>
     <row r="36" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A36" s="11">
-        <v>46301</v>
+        <v>46302</v>
       </c>
       <c r="B36" s="12"/>
       <c r="C36" s="12" t="s">
         <v>23</v>
       </c>
       <c r="D36" s="13">
-        <v>256.70999999999998</v>
+        <v>255.91</v>
       </c>
       <c r="E36" s="13">
-        <v>229.8</v>
+        <v>231.35</v>
       </c>
       <c r="F36" s="13">
-        <v>238.8</v>
+        <v>240.35</v>
       </c>
       <c r="G36" s="17"/>
     </row>
     <row r="37" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A37" s="7">
-        <v>46302</v>
+        <v>46303</v>
       </c>
       <c r="B37" s="8"/>
       <c r="C37" s="20" t="s">
         <v>24</v>
       </c>
       <c r="D37" s="10">
-        <v>271.52999999999997</v>
+        <v>270.88</v>
       </c>
       <c r="E37" s="10" t="s">
         <v>18</v>
@@ -1358,14 +1358,14 @@
     </row>
     <row r="38" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A38" s="11">
-        <v>46301</v>
+        <v>46302</v>
       </c>
       <c r="B38" s="12"/>
       <c r="C38" s="12" t="s">
         <v>24</v>
       </c>
       <c r="D38" s="13">
-        <v>272.33</v>
+        <v>271.52999999999997</v>
       </c>
       <c r="E38" s="13" t="s">
         <v>18</v>
@@ -1416,77 +1416,77 @@
     </row>
     <row r="42" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A42" s="7">
-        <v>46302</v>
+        <v>46303</v>
       </c>
       <c r="B42" s="8"/>
       <c r="C42" s="20" t="s">
         <v>26</v>
       </c>
       <c r="D42" s="10">
-        <v>265.91000000000003</v>
+        <v>265.33999999999997</v>
       </c>
       <c r="E42" s="10">
-        <v>242.51</v>
+        <v>244.12</v>
       </c>
       <c r="F42" s="10">
-        <v>252.51</v>
+        <v>254.12</v>
       </c>
       <c r="G42" s="17"/>
     </row>
     <row r="43" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A43" s="11">
-        <v>46302</v>
+        <v>46303</v>
       </c>
       <c r="B43" s="12"/>
       <c r="C43" s="21" t="s">
         <v>27</v>
       </c>
       <c r="D43" s="13">
-        <v>265.52</v>
+        <v>264.95</v>
       </c>
       <c r="E43" s="13">
-        <v>242.92</v>
+        <v>244.54</v>
       </c>
       <c r="F43" s="13">
-        <v>252.92</v>
+        <v>254.54</v>
       </c>
       <c r="G43" s="17"/>
     </row>
     <row r="44" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A44" s="7">
-        <v>46301</v>
+        <v>46302</v>
       </c>
       <c r="B44" s="8"/>
       <c r="C44" s="20" t="s">
         <v>26</v>
       </c>
       <c r="D44" s="10">
-        <v>266.62</v>
+        <v>265.91000000000003</v>
       </c>
       <c r="E44" s="10">
-        <v>240.86</v>
+        <v>242.51</v>
       </c>
       <c r="F44" s="10">
-        <v>250.86</v>
+        <v>252.51</v>
       </c>
       <c r="G44" s="17"/>
     </row>
     <row r="45" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A45" s="11">
-        <v>46301</v>
+        <v>46302</v>
       </c>
       <c r="B45" s="12"/>
       <c r="C45" s="21" t="s">
         <v>27</v>
       </c>
       <c r="D45" s="13">
-        <v>266.23</v>
+        <v>265.52</v>
       </c>
       <c r="E45" s="13">
-        <v>241.27</v>
+        <v>242.92</v>
       </c>
       <c r="F45" s="13">
-        <v>251.27</v>
+        <v>252.92</v>
       </c>
       <c r="G45" s="17"/>
     </row>
@@ -1531,77 +1531,77 @@
     </row>
     <row r="49" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A49" s="7">
-        <v>46302</v>
+        <v>46303</v>
       </c>
       <c r="B49" s="8"/>
       <c r="C49" s="20" t="s">
         <v>29</v>
       </c>
       <c r="D49" s="10">
-        <v>257.63</v>
+        <v>257.33</v>
       </c>
       <c r="E49" s="10">
-        <v>236.24</v>
+        <v>237.47</v>
       </c>
       <c r="F49" s="10">
-        <v>246.24</v>
+        <v>247.47</v>
       </c>
       <c r="G49" s="28"/>
     </row>
     <row r="50" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A50" s="11">
-        <v>46302</v>
+        <v>46303</v>
       </c>
       <c r="B50" s="12"/>
       <c r="C50" s="21" t="s">
         <v>30</v>
       </c>
       <c r="D50" s="13">
-        <v>255.2</v>
+        <v>254.86</v>
       </c>
       <c r="E50" s="13">
-        <v>235.89</v>
+        <v>237.1</v>
       </c>
       <c r="F50" s="13">
-        <v>245.89</v>
+        <v>247.1</v>
       </c>
       <c r="G50" s="28"/>
     </row>
     <row r="51" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A51" s="7">
-        <v>46301</v>
+        <v>46302</v>
       </c>
       <c r="B51" s="8"/>
       <c r="C51" s="20" t="s">
         <v>29</v>
       </c>
       <c r="D51" s="10">
-        <v>258.33999999999997</v>
+        <v>257.63</v>
       </c>
       <c r="E51" s="10">
-        <v>235.09</v>
+        <v>236.24</v>
       </c>
       <c r="F51" s="10">
-        <v>245.09</v>
+        <v>246.24</v>
       </c>
       <c r="G51" s="17"/>
     </row>
     <row r="52" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A52" s="11">
-        <v>46301</v>
+        <v>46302</v>
       </c>
       <c r="B52" s="12"/>
       <c r="C52" s="21" t="s">
         <v>30</v>
       </c>
       <c r="D52" s="13">
-        <v>255.96</v>
+        <v>255.2</v>
       </c>
       <c r="E52" s="13">
-        <v>234.76</v>
+        <v>235.89</v>
       </c>
       <c r="F52" s="13">
-        <v>244.76</v>
+        <v>245.89</v>
       </c>
       <c r="G52" s="17"/>
     </row>
@@ -1646,52 +1646,52 @@
     </row>
     <row r="56" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A56" s="7">
-        <v>46302</v>
+        <v>46303</v>
       </c>
       <c r="B56" s="8"/>
       <c r="C56" s="20" t="s">
         <v>32</v>
       </c>
       <c r="D56" s="10">
-        <v>273.7</v>
+        <v>273.01</v>
       </c>
       <c r="E56" s="10">
-        <v>264.52</v>
+        <v>266.49</v>
       </c>
       <c r="F56" s="10">
-        <v>274.52</v>
+        <v>276.49</v>
       </c>
       <c r="G56" s="17"/>
     </row>
     <row r="57" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A57" s="11">
-        <v>46302</v>
+        <v>46303</v>
       </c>
       <c r="B57" s="12"/>
       <c r="C57" s="21" t="s">
         <v>33</v>
       </c>
       <c r="D57" s="13">
-        <v>263.08</v>
+        <v>262.44</v>
       </c>
       <c r="E57" s="13">
-        <v>246.07</v>
+        <v>247.48</v>
       </c>
       <c r="F57" s="13">
-        <v>256.07</v>
+        <v>257.48</v>
       </c>
       <c r="G57" s="17"/>
     </row>
     <row r="58" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A58" s="7">
-        <v>46302</v>
+        <v>46303</v>
       </c>
       <c r="B58" s="8"/>
       <c r="C58" s="20" t="s">
         <v>34</v>
       </c>
       <c r="D58" s="10">
-        <v>264.51</v>
+        <v>263.88</v>
       </c>
       <c r="E58" s="10" t="s">
         <v>18</v>
@@ -1703,17 +1703,17 @@
     </row>
     <row r="59" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A59" s="11">
-        <v>46302</v>
+        <v>46303</v>
       </c>
       <c r="B59" s="12"/>
       <c r="C59" s="21" t="s">
         <v>35</v>
       </c>
       <c r="D59" s="13">
-        <v>258.70999999999998</v>
+        <v>258.48</v>
       </c>
       <c r="E59" s="13">
-        <v>240.44</v>
+        <v>241.85</v>
       </c>
       <c r="F59" s="13" t="s">
         <v>18</v>
@@ -1722,36 +1722,36 @@
     </row>
     <row r="60" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A60" s="7">
-        <v>46302</v>
+        <v>46303</v>
       </c>
       <c r="B60" s="8"/>
       <c r="C60" s="20" t="s">
         <v>36</v>
       </c>
       <c r="D60" s="10">
-        <v>254.54</v>
+        <v>254.31</v>
       </c>
       <c r="E60" s="10">
-        <v>236.39</v>
+        <v>237.8</v>
       </c>
       <c r="F60" s="10">
-        <v>246.39</v>
+        <v>247.8</v>
       </c>
       <c r="G60" s="17"/>
     </row>
     <row r="61" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A61" s="11">
-        <v>46302</v>
+        <v>46303</v>
       </c>
       <c r="B61" s="12"/>
       <c r="C61" s="21" t="s">
         <v>37</v>
       </c>
       <c r="D61" s="13">
-        <v>259.91000000000003</v>
+        <v>259.13</v>
       </c>
       <c r="E61" s="13">
-        <v>257.92</v>
+        <v>259.7</v>
       </c>
       <c r="F61" s="13" t="s">
         <v>18</v>
@@ -1760,52 +1760,52 @@
     </row>
     <row r="62" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A62" s="7">
-        <v>46301</v>
+        <v>46302</v>
       </c>
       <c r="B62" s="8"/>
       <c r="C62" s="20" t="s">
         <v>32</v>
       </c>
       <c r="D62" s="10">
-        <v>274.55</v>
+        <v>273.7</v>
       </c>
       <c r="E62" s="10">
-        <v>262.45999999999998</v>
+        <v>264.52</v>
       </c>
       <c r="F62" s="10">
-        <v>272.45999999999998</v>
+        <v>274.52</v>
       </c>
       <c r="G62" s="17"/>
     </row>
     <row r="63" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A63" s="11">
-        <v>46301</v>
+        <v>46302</v>
       </c>
       <c r="B63" s="12"/>
       <c r="C63" s="21" t="s">
         <v>33</v>
       </c>
       <c r="D63" s="13">
-        <v>263.89</v>
+        <v>263.08</v>
       </c>
       <c r="E63" s="13">
-        <v>244.66</v>
+        <v>246.07</v>
       </c>
       <c r="F63" s="13">
-        <v>254.66</v>
+        <v>256.07</v>
       </c>
       <c r="G63" s="17"/>
     </row>
     <row r="64" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A64" s="7">
-        <v>46301</v>
+        <v>46302</v>
       </c>
       <c r="B64" s="8"/>
       <c r="C64" s="20" t="s">
         <v>34</v>
       </c>
       <c r="D64" s="10">
-        <v>265.3</v>
+        <v>264.51</v>
       </c>
       <c r="E64" s="10" t="s">
         <v>18</v>
@@ -1817,17 +1817,17 @@
     </row>
     <row r="65" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A65" s="11">
-        <v>46301</v>
+        <v>46302</v>
       </c>
       <c r="B65" s="12"/>
       <c r="C65" s="21" t="s">
         <v>35</v>
       </c>
       <c r="D65" s="13">
-        <v>259.67</v>
+        <v>258.70999999999998</v>
       </c>
       <c r="E65" s="13">
-        <v>239.03</v>
+        <v>240.44</v>
       </c>
       <c r="F65" s="13" t="s">
         <v>18</v>
@@ -1835,35 +1835,35 @@
     </row>
     <row r="66" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A66" s="7">
-        <v>46301</v>
+        <v>46302</v>
       </c>
       <c r="B66" s="8"/>
       <c r="C66" s="20" t="s">
         <v>36</v>
       </c>
       <c r="D66" s="10">
-        <v>255.5</v>
+        <v>254.54</v>
       </c>
       <c r="E66" s="10">
-        <v>234.98</v>
+        <v>236.39</v>
       </c>
       <c r="F66" s="10">
-        <v>244.98</v>
+        <v>246.39</v>
       </c>
     </row>
     <row r="67" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A67" s="11">
-        <v>46301</v>
+        <v>46302</v>
       </c>
       <c r="B67" s="12"/>
       <c r="C67" s="21" t="s">
         <v>37</v>
       </c>
       <c r="D67" s="13">
-        <v>260.88</v>
+        <v>259.91000000000003</v>
       </c>
       <c r="E67" s="13">
-        <v>256.08</v>
+        <v>257.92</v>
       </c>
       <c r="F67" s="13" t="s">
         <v>18</v>
@@ -1891,6 +1891,26 @@
 </file>
 
 <file path=customXml/item1.xml><?xml version="1.0" encoding="utf-8"?>
+<?mso-contentType ?>
+<FormTemplates xmlns="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms">
+  <Display>DocumentLibraryForm</Display>
+  <Edit>DocumentLibraryForm</Edit>
+  <New>DocumentLibraryForm</New>
+</FormTemplates>
+</file>
+
+<file path=customXml/item2.xml><?xml version="1.0" encoding="utf-8"?>
+<p:properties xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls">
+  <documentManagement>
+    <lcf76f155ced4ddcb4097134ff3c332f xmlns="87276d81-85f4-4ef2-9e6e-55066304288f">
+      <Terms xmlns="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
+    </lcf76f155ced4ddcb4097134ff3c332f>
+    <TaxCatchAll xmlns="b23b8984-eafa-4e79-985e-54f52f3da58e" xsi:nil="true"/>
+  </documentManagement>
+</p:properties>
+</file>
+
+<file path=customXml/item3.xml><?xml version="1.0" encoding="utf-8"?>
 <ct:contentTypeSchema xmlns:ct="http://schemas.microsoft.com/office/2006/metadata/contentType" xmlns:ma="http://schemas.microsoft.com/office/2006/metadata/properties/metaAttributes" ct:_="" ma:_="" ma:contentTypeName="Document" ma:contentTypeID="0x010100D3632DF5622958439304627C030B0427" ma:contentTypeVersion="18" ma:contentTypeDescription="Create a new document." ma:contentTypeScope="" ma:versionID="8c2ecbce386d6bac497f8eb2d8f0fb7a">
   <xsd:schema xmlns:xsd="http://www.w3.org/2001/XMLSchema" xmlns:xs="http://www.w3.org/2001/XMLSchema" xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:ns2="87276d81-85f4-4ef2-9e6e-55066304288f" xmlns:ns3="39e1dda6-d1d8-4c88-a3b9-f1abc1284bad" xmlns:ns4="b23b8984-eafa-4e79-985e-54f52f3da58e" targetNamespace="http://schemas.microsoft.com/office/2006/metadata/properties" ma:root="true" ma:fieldsID="4cfd0c2f651c1ce156ad4fcb44ea61dd" ns2:_="" ns3:_="" ns4:_="">
     <xsd:import namespace="87276d81-85f4-4ef2-9e6e-55066304288f"/>
@@ -2150,27 +2170,26 @@
 </ct:contentTypeSchema>
 </file>
 
-<file path=customXml/item2.xml><?xml version="1.0" encoding="utf-8"?>
-<?mso-contentType ?>
-<FormTemplates xmlns="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms">
-  <Display>DocumentLibraryForm</Display>
-  <Edit>DocumentLibraryForm</Edit>
-  <New>DocumentLibraryForm</New>
-</FormTemplates>
+<file path=customXml/itemProps1.xml><?xml version="1.0" encoding="utf-8"?>
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{F60519E9-FD90-4339-869C-BC2F85719BB8}">
+  <ds:schemaRefs>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms"/>
+  </ds:schemaRefs>
+</ds:datastoreItem>
 </file>
 
-<file path=customXml/item3.xml><?xml version="1.0" encoding="utf-8"?>
-<p:properties xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls">
-  <documentManagement>
-    <lcf76f155ced4ddcb4097134ff3c332f xmlns="87276d81-85f4-4ef2-9e6e-55066304288f">
-      <Terms xmlns="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
-    </lcf76f155ced4ddcb4097134ff3c332f>
-    <TaxCatchAll xmlns="b23b8984-eafa-4e79-985e-54f52f3da58e" xsi:nil="true"/>
-  </documentManagement>
-</p:properties>
+<file path=customXml/itemProps2.xml><?xml version="1.0" encoding="utf-8"?>
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{57A83D98-2BAE-4D83-823A-D31C464B620C}">
+  <ds:schemaRefs>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/properties"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
+    <ds:schemaRef ds:uri="87276d81-85f4-4ef2-9e6e-55066304288f"/>
+    <ds:schemaRef ds:uri="b23b8984-eafa-4e79-985e-54f52f3da58e"/>
+  </ds:schemaRefs>
+</ds:datastoreItem>
 </file>
 
-<file path=customXml/itemProps1.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=customXml/itemProps3.xml><?xml version="1.0" encoding="utf-8"?>
 <ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{B44E1863-2778-41F9-ACBA-48420F931671}">
   <ds:schemaRefs>
     <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/contentType"/>
@@ -2190,25 +2209,6 @@
 </ds:datastoreItem>
 </file>
 
-<file path=customXml/itemProps2.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{F60519E9-FD90-4339-869C-BC2F85719BB8}">
-  <ds:schemaRefs>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms"/>
-  </ds:schemaRefs>
-</ds:datastoreItem>
-</file>
-
-<file path=customXml/itemProps3.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{57A83D98-2BAE-4D83-823A-D31C464B620C}">
-  <ds:schemaRefs>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/properties"/>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
-    <ds:schemaRef ds:uri="87276d81-85f4-4ef2-9e6e-55066304288f"/>
-    <ds:schemaRef ds:uri="b23b8984-eafa-4e79-985e-54f52f3da58e"/>
-  </ds:schemaRefs>
-</ds:datastoreItem>
-</file>
-
 <file path=docMetadata/LabelInfo.xml><?xml version="1.0" encoding="utf-8"?>
 <clbl:labelList xmlns:clbl="http://schemas.microsoft.com/office/2020/mipLabelMetadata">
   <clbl:label id="{569bf4a9-87bd-4dbf-a36c-1db5158e5def}" enabled="1" method="Privileged" siteId="{ea80952e-a476-42d4-aaf4-5457852b0f7e}" removed="0"/>

</xml_diff>

<commit_message>
Thu Oct  8 07:33:18 UTC 2026
</commit_message>
<xml_diff>
--- a/bp.com-content-dam-bp-country-sites-en_au-australia-home-products-services-pricing-tgp-excel.xlsx
+++ b/bp.com-content-dam-bp-country-sites-en_au-australia-home-products-services-pricing-tgp-excel.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://bp365.sharepoint.com/sites/WholesalePricing/Shared Documents/B2C/TGP/Daily TGP/Web TGP/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="14_{4E732A02-49B6-4485-8258-62E7190CD32E}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="14_{7AA9A883-8E9D-426C-BA68-AA56CC5C61BF}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-28920" yWindow="-60" windowWidth="29040" windowHeight="15720" xr2:uid="{1B412EEF-F96D-4DF4-A4E9-C7F0F183C2FB}"/>
+    <workbookView xWindow="-8595" yWindow="-16320" windowWidth="29040" windowHeight="15720" xr2:uid="{1B412EEF-F96D-4DF4-A4E9-C7F0F183C2FB}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
@@ -715,15 +715,15 @@
     <pageSetUpPr fitToPage="1"/>
   </sheetPr>
   <dimension ref="A1:G67"/>
-  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <sheetFormatPr defaultRowHeight="14.25" x14ac:dyDescent="0.45"/>
   <cols>
-    <col min="1" max="1" width="76.42578125" bestFit="1" customWidth="1"/>
-    <col min="2" max="2" width="6.42578125"/>
-    <col min="3" max="3" width="18.140625" bestFit="1" customWidth="1"/>
-    <col min="4" max="7" width="7.140625" bestFit="1" customWidth="1"/>
+    <col min="1" max="1" width="76.3984375" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="6.3984375"/>
+    <col min="3" max="3" width="18.1328125" bestFit="1" customWidth="1"/>
+    <col min="4" max="7" width="7.1328125" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:7" ht="23.25" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:7" ht="22.15" x14ac:dyDescent="0.45">
       <c r="A1" s="30" t="s">
         <v>0</v>
       </c>
@@ -734,7 +734,7 @@
       <c r="F1" s="2"/>
       <c r="G1" s="2"/>
     </row>
-    <row r="2" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="2" spans="1:7" x14ac:dyDescent="0.45">
       <c r="A2" s="3"/>
       <c r="B2" s="1"/>
       <c r="C2" s="1"/>
@@ -743,7 +743,7 @@
       <c r="F2" s="2"/>
       <c r="G2" s="2"/>
     </row>
-    <row r="3" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="3" spans="1:7" x14ac:dyDescent="0.45">
       <c r="A3" s="3" t="s">
         <v>1</v>
       </c>
@@ -754,7 +754,7 @@
       <c r="F3" s="2"/>
       <c r="G3" s="2"/>
     </row>
-    <row r="4" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="4" spans="1:7" x14ac:dyDescent="0.45">
       <c r="A4" s="3" t="s">
         <v>2</v>
       </c>
@@ -765,7 +765,7 @@
       <c r="F4" s="2"/>
       <c r="G4" s="2"/>
     </row>
-    <row r="5" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="5" spans="1:7" x14ac:dyDescent="0.45">
       <c r="A5" s="3"/>
       <c r="B5" s="3"/>
       <c r="C5" s="1"/>
@@ -774,7 +774,7 @@
       <c r="F5" s="2"/>
       <c r="G5" s="2"/>
     </row>
-    <row r="6" spans="1:7" ht="20.25" x14ac:dyDescent="0.25">
+    <row r="6" spans="1:7" ht="20.25" x14ac:dyDescent="0.45">
       <c r="A6" s="29" t="s">
         <v>3</v>
       </c>
@@ -785,7 +785,7 @@
       <c r="F6" s="2"/>
       <c r="G6" s="2"/>
     </row>
-    <row r="7" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="7" spans="1:7" x14ac:dyDescent="0.45">
       <c r="A7" s="4" t="s">
         <v>4</v>
       </c>
@@ -806,133 +806,133 @@
         <v>9</v>
       </c>
     </row>
-    <row r="8" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="8" spans="1:7" x14ac:dyDescent="0.45">
       <c r="A8" s="7">
-        <v>46303</v>
+        <v>46304</v>
       </c>
       <c r="B8" s="8"/>
       <c r="C8" s="9" t="s">
         <v>10</v>
       </c>
       <c r="D8" s="10">
-        <v>260.22000000000003</v>
+        <v>259.77999999999997</v>
       </c>
       <c r="E8" s="10">
-        <v>236.63</v>
+        <v>237.83</v>
       </c>
       <c r="F8" s="10">
-        <v>246.63</v>
+        <v>247.83</v>
       </c>
       <c r="G8" s="10">
-        <v>234.24</v>
-      </c>
-    </row>
-    <row r="9" spans="1:7" x14ac:dyDescent="0.25">
+        <v>235.44</v>
+      </c>
+    </row>
+    <row r="9" spans="1:7" x14ac:dyDescent="0.45">
       <c r="A9" s="11">
-        <v>46303</v>
+        <v>46304</v>
       </c>
       <c r="B9" s="12"/>
       <c r="C9" s="12" t="s">
         <v>11</v>
       </c>
       <c r="D9" s="13">
-        <v>260.22000000000003</v>
+        <v>259.77999999999997</v>
       </c>
       <c r="E9" s="13">
-        <v>236.63</v>
+        <v>237.83</v>
       </c>
       <c r="F9" s="13">
-        <v>246.63</v>
+        <v>247.83</v>
       </c>
       <c r="G9" s="13">
-        <v>234.24</v>
-      </c>
-    </row>
-    <row r="10" spans="1:7" x14ac:dyDescent="0.25">
+        <v>235.44</v>
+      </c>
+    </row>
+    <row r="10" spans="1:7" x14ac:dyDescent="0.45">
       <c r="A10" s="7">
-        <v>46303</v>
+        <v>46304</v>
       </c>
       <c r="B10" s="8"/>
       <c r="C10" s="9" t="s">
         <v>12</v>
       </c>
       <c r="D10" s="10">
-        <v>256.7</v>
+        <v>255.92</v>
       </c>
       <c r="E10" s="10">
-        <v>237.25</v>
+        <v>238.64</v>
       </c>
       <c r="F10" s="10">
-        <v>247.25</v>
+        <v>248.64</v>
       </c>
       <c r="G10" s="10">
-        <v>235.65</v>
-      </c>
-    </row>
-    <row r="11" spans="1:7" x14ac:dyDescent="0.25">
+        <v>237.04</v>
+      </c>
+    </row>
+    <row r="11" spans="1:7" x14ac:dyDescent="0.45">
       <c r="A11" s="11">
-        <v>46302</v>
+        <v>46303</v>
       </c>
       <c r="B11" s="12"/>
       <c r="C11" s="12" t="s">
         <v>10</v>
       </c>
       <c r="D11" s="13">
-        <v>259.45</v>
+        <v>260.22000000000003</v>
       </c>
       <c r="E11" s="13">
-        <v>234.76</v>
+        <v>236.63</v>
       </c>
       <c r="F11" s="13">
-        <v>244.76</v>
+        <v>246.63</v>
       </c>
       <c r="G11" s="13">
-        <v>232.37</v>
-      </c>
-    </row>
-    <row r="12" spans="1:7" x14ac:dyDescent="0.25">
+        <v>234.24</v>
+      </c>
+    </row>
+    <row r="12" spans="1:7" x14ac:dyDescent="0.45">
       <c r="A12" s="7">
-        <v>46302</v>
+        <v>46303</v>
       </c>
       <c r="B12" s="8"/>
       <c r="C12" s="9" t="s">
         <v>11</v>
       </c>
       <c r="D12" s="10">
-        <v>259.45</v>
+        <v>260.22000000000003</v>
       </c>
       <c r="E12" s="10">
-        <v>234.76</v>
+        <v>236.63</v>
       </c>
       <c r="F12" s="10">
-        <v>244.76</v>
+        <v>246.63</v>
       </c>
       <c r="G12" s="10">
-        <v>232.37</v>
-      </c>
-    </row>
-    <row r="13" spans="1:7" x14ac:dyDescent="0.25">
+        <v>234.24</v>
+      </c>
+    </row>
+    <row r="13" spans="1:7" x14ac:dyDescent="0.45">
       <c r="A13" s="11">
-        <v>46302</v>
+        <v>46303</v>
       </c>
       <c r="B13" s="12"/>
       <c r="C13" s="12" t="s">
         <v>12</v>
       </c>
       <c r="D13" s="13">
-        <v>257.36</v>
+        <v>256.7</v>
       </c>
       <c r="E13" s="13">
-        <v>235.72</v>
+        <v>237.25</v>
       </c>
       <c r="F13" s="13">
-        <v>245.72</v>
+        <v>247.25</v>
       </c>
       <c r="G13" s="13">
-        <v>234.13</v>
-      </c>
-    </row>
-    <row r="14" spans="1:7" x14ac:dyDescent="0.25">
+        <v>235.65</v>
+      </c>
+    </row>
+    <row r="14" spans="1:7" x14ac:dyDescent="0.45">
       <c r="A14" s="14"/>
       <c r="B14" s="14"/>
       <c r="C14" s="15"/>
@@ -941,7 +941,7 @@
       <c r="F14" s="16"/>
       <c r="G14" s="16"/>
     </row>
-    <row r="15" spans="1:7" ht="20.25" x14ac:dyDescent="0.25">
+    <row r="15" spans="1:7" ht="20.25" x14ac:dyDescent="0.45">
       <c r="A15" s="29" t="s">
         <v>13</v>
       </c>
@@ -952,7 +952,7 @@
       <c r="F15" s="17"/>
       <c r="G15" s="17"/>
     </row>
-    <row r="16" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="16" spans="1:7" x14ac:dyDescent="0.45">
       <c r="A16" s="4" t="s">
         <v>4</v>
       </c>
@@ -971,45 +971,45 @@
       </c>
       <c r="G16" s="17"/>
     </row>
-    <row r="17" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="17" spans="1:7" x14ac:dyDescent="0.45">
       <c r="A17" s="7">
-        <v>46303</v>
+        <v>46304</v>
       </c>
       <c r="B17" s="8"/>
       <c r="C17" s="20" t="s">
         <v>14</v>
       </c>
       <c r="D17" s="10">
-        <v>260.07</v>
+        <v>259.24</v>
       </c>
       <c r="E17" s="10">
-        <v>242.36</v>
+        <v>243.72</v>
       </c>
       <c r="F17" s="10">
-        <v>252.36</v>
+        <v>253.72</v>
       </c>
       <c r="G17" s="17"/>
     </row>
-    <row r="18" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="18" spans="1:7" x14ac:dyDescent="0.45">
       <c r="A18" s="11">
-        <v>46302</v>
+        <v>46303</v>
       </c>
       <c r="B18" s="12"/>
       <c r="C18" s="12" t="s">
         <v>14</v>
       </c>
       <c r="D18" s="13">
-        <v>260.83</v>
+        <v>260.07</v>
       </c>
       <c r="E18" s="13">
-        <v>240.93</v>
+        <v>242.36</v>
       </c>
       <c r="F18" s="13">
-        <v>250.93</v>
+        <v>252.36</v>
       </c>
       <c r="G18" s="17"/>
     </row>
-    <row r="19" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="19" spans="1:7" x14ac:dyDescent="0.45">
       <c r="A19" s="14"/>
       <c r="B19" s="14"/>
       <c r="C19" s="15"/>
@@ -1018,7 +1018,7 @@
       <c r="F19" s="16"/>
       <c r="G19" s="17"/>
     </row>
-    <row r="20" spans="1:7" ht="20.25" x14ac:dyDescent="0.25">
+    <row r="20" spans="1:7" ht="20.25" x14ac:dyDescent="0.45">
       <c r="A20" s="29" t="s">
         <v>15</v>
       </c>
@@ -1029,7 +1029,7 @@
       <c r="F20" s="17"/>
       <c r="G20" s="17"/>
     </row>
-    <row r="21" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="21" spans="1:7" x14ac:dyDescent="0.45">
       <c r="A21" s="4" t="s">
         <v>4</v>
       </c>
@@ -1050,217 +1050,217 @@
         <v>9</v>
       </c>
     </row>
-    <row r="22" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="22" spans="1:7" x14ac:dyDescent="0.45">
       <c r="A22" s="7">
-        <v>46303</v>
+        <v>46304</v>
       </c>
       <c r="B22" s="8"/>
       <c r="C22" s="20" t="s">
         <v>16</v>
       </c>
       <c r="D22" s="10">
-        <v>261.35000000000002</v>
+        <v>260.89999999999998</v>
       </c>
       <c r="E22" s="10">
-        <v>236.21</v>
+        <v>237.41</v>
       </c>
       <c r="F22" s="10">
-        <v>245.81</v>
+        <v>247.01</v>
       </c>
       <c r="G22" s="10">
-        <v>232.58</v>
-      </c>
-    </row>
-    <row r="23" spans="1:7" x14ac:dyDescent="0.25">
+        <v>233.78</v>
+      </c>
+    </row>
+    <row r="23" spans="1:7" x14ac:dyDescent="0.45">
       <c r="A23" s="11">
-        <v>46303</v>
+        <v>46304</v>
       </c>
       <c r="B23" s="12"/>
       <c r="C23" s="21" t="s">
         <v>17</v>
       </c>
       <c r="D23" s="13">
-        <v>261.67</v>
+        <v>260.89</v>
       </c>
       <c r="E23" s="13">
-        <v>247.79</v>
+        <v>249.2</v>
       </c>
       <c r="F23" s="13">
-        <v>257.79000000000002</v>
+        <v>259.2</v>
       </c>
       <c r="G23" s="13" t="s">
         <v>18</v>
       </c>
     </row>
-    <row r="24" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="24" spans="1:7" x14ac:dyDescent="0.45">
       <c r="A24" s="7">
-        <v>46303</v>
+        <v>46304</v>
       </c>
       <c r="B24" s="8"/>
       <c r="C24" s="20" t="s">
         <v>19</v>
       </c>
       <c r="D24" s="10">
-        <v>262.01</v>
+        <v>261.22000000000003</v>
       </c>
       <c r="E24" s="10">
-        <v>247.01</v>
+        <v>248.42</v>
       </c>
       <c r="F24" s="10">
-        <v>257.02</v>
+        <v>258.42</v>
       </c>
       <c r="G24" s="10" t="s">
         <v>18</v>
       </c>
     </row>
-    <row r="25" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="25" spans="1:7" x14ac:dyDescent="0.45">
       <c r="A25" s="11">
-        <v>46303</v>
+        <v>46304</v>
       </c>
       <c r="B25" s="12"/>
       <c r="C25" s="21" t="s">
         <v>20</v>
       </c>
       <c r="D25" s="13">
-        <v>258.66000000000003</v>
+        <v>257.88</v>
       </c>
       <c r="E25" s="13">
-        <v>247.27</v>
+        <v>248.68</v>
       </c>
       <c r="F25" s="13">
-        <v>257.27</v>
+        <v>258.68</v>
       </c>
       <c r="G25" s="13">
-        <v>243.11</v>
-      </c>
-    </row>
-    <row r="26" spans="1:7" x14ac:dyDescent="0.25">
+        <v>244.52</v>
+      </c>
+    </row>
+    <row r="26" spans="1:7" x14ac:dyDescent="0.45">
       <c r="A26" s="7">
-        <v>46303</v>
+        <v>46304</v>
       </c>
       <c r="B26" s="8"/>
       <c r="C26" s="20" t="s">
         <v>21</v>
       </c>
       <c r="D26" s="10">
-        <v>260.19</v>
+        <v>259.39999999999998</v>
       </c>
       <c r="E26" s="10">
-        <v>248.82</v>
+        <v>250.25</v>
       </c>
       <c r="F26" s="10">
-        <v>258.82</v>
+        <v>260.25</v>
       </c>
       <c r="G26" s="10" t="s">
         <v>18</v>
       </c>
     </row>
-    <row r="27" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="27" spans="1:7" x14ac:dyDescent="0.45">
       <c r="A27" s="11">
-        <v>46302</v>
+        <v>46303</v>
       </c>
       <c r="B27" s="12"/>
       <c r="C27" s="12" t="s">
         <v>16</v>
       </c>
       <c r="D27" s="13">
-        <v>260.58</v>
+        <v>261.35000000000002</v>
       </c>
       <c r="E27" s="13">
-        <v>234.34</v>
+        <v>236.21</v>
       </c>
       <c r="F27" s="13">
-        <v>243.94</v>
+        <v>245.81</v>
       </c>
       <c r="G27" s="13">
-        <v>230.71</v>
-      </c>
-    </row>
-    <row r="28" spans="1:7" x14ac:dyDescent="0.25">
+        <v>232.58</v>
+      </c>
+    </row>
+    <row r="28" spans="1:7" x14ac:dyDescent="0.45">
       <c r="A28" s="7">
-        <v>46302</v>
+        <v>46303</v>
       </c>
       <c r="B28" s="8"/>
       <c r="C28" s="20" t="s">
         <v>17</v>
       </c>
       <c r="D28" s="10">
-        <v>262.31</v>
+        <v>261.67</v>
       </c>
       <c r="E28" s="22">
-        <v>246.22</v>
+        <v>247.79</v>
       </c>
       <c r="F28" s="22">
-        <v>256.22000000000003</v>
+        <v>257.79000000000002</v>
       </c>
       <c r="G28" s="22" t="s">
         <v>18</v>
       </c>
     </row>
-    <row r="29" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="29" spans="1:7" x14ac:dyDescent="0.45">
       <c r="A29" s="11">
-        <v>46302</v>
+        <v>46303</v>
       </c>
       <c r="B29" s="12"/>
       <c r="C29" s="12" t="s">
         <v>19</v>
       </c>
       <c r="D29" s="13">
-        <v>262.66000000000003</v>
+        <v>262.01</v>
       </c>
       <c r="E29" s="13">
-        <v>245.45</v>
+        <v>247.01</v>
       </c>
       <c r="F29" s="13">
-        <v>255.45</v>
+        <v>257.02</v>
       </c>
       <c r="G29" s="13" t="s">
         <v>18</v>
       </c>
     </row>
-    <row r="30" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="30" spans="1:7" x14ac:dyDescent="0.45">
       <c r="A30" s="7">
-        <v>46302</v>
+        <v>46303</v>
       </c>
       <c r="B30" s="8"/>
       <c r="C30" s="20" t="s">
         <v>20</v>
       </c>
       <c r="D30" s="10">
-        <v>259.32</v>
+        <v>258.66000000000003</v>
       </c>
       <c r="E30" s="22">
-        <v>245.69</v>
+        <v>247.27</v>
       </c>
       <c r="F30" s="22">
-        <v>255.69</v>
+        <v>257.27</v>
       </c>
       <c r="G30" s="22">
-        <v>241.53</v>
-      </c>
-    </row>
-    <row r="31" spans="1:7" x14ac:dyDescent="0.25">
+        <v>243.11</v>
+      </c>
+    </row>
+    <row r="31" spans="1:7" x14ac:dyDescent="0.45">
       <c r="A31" s="11">
-        <v>46302</v>
+        <v>46303</v>
       </c>
       <c r="B31" s="12"/>
       <c r="C31" s="12" t="s">
         <v>21</v>
       </c>
       <c r="D31" s="13">
-        <v>260.87</v>
+        <v>260.19</v>
       </c>
       <c r="E31" s="13">
-        <v>247.23</v>
+        <v>248.82</v>
       </c>
       <c r="F31" s="13">
-        <v>257.23</v>
+        <v>258.82</v>
       </c>
       <c r="G31" s="13" t="s">
         <v>18</v>
       </c>
     </row>
-    <row r="32" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="32" spans="1:7" x14ac:dyDescent="0.45">
       <c r="A32" s="14"/>
       <c r="B32" s="14"/>
       <c r="C32" s="15"/>
@@ -1269,7 +1269,7 @@
       <c r="F32" s="17"/>
       <c r="G32" s="17"/>
     </row>
-    <row r="33" spans="1:7" ht="20.25" x14ac:dyDescent="0.25">
+    <row r="33" spans="1:7" ht="20.25" x14ac:dyDescent="0.45">
       <c r="A33" s="29" t="s">
         <v>22</v>
       </c>
@@ -1280,7 +1280,7 @@
       <c r="F33" s="17"/>
       <c r="G33" s="17"/>
     </row>
-    <row r="34" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="34" spans="1:7" x14ac:dyDescent="0.45">
       <c r="A34" s="23" t="s">
         <v>4</v>
       </c>
@@ -1299,54 +1299,54 @@
       </c>
       <c r="G34" s="17"/>
     </row>
-    <row r="35" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="35" spans="1:7" x14ac:dyDescent="0.45">
       <c r="A35" s="7">
-        <v>46303</v>
+        <v>46304</v>
       </c>
       <c r="B35" s="8"/>
       <c r="C35" s="20" t="s">
         <v>23</v>
       </c>
       <c r="D35" s="10">
-        <v>255.26</v>
+        <v>254.47</v>
       </c>
       <c r="E35" s="10">
-        <v>232.87</v>
+        <v>234.26</v>
       </c>
       <c r="F35" s="10">
-        <v>241.87</v>
+        <v>243.27</v>
       </c>
       <c r="G35" s="17"/>
     </row>
-    <row r="36" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="36" spans="1:7" x14ac:dyDescent="0.45">
       <c r="A36" s="11">
-        <v>46302</v>
+        <v>46303</v>
       </c>
       <c r="B36" s="12"/>
       <c r="C36" s="12" t="s">
         <v>23</v>
       </c>
       <c r="D36" s="13">
-        <v>255.91</v>
+        <v>255.26</v>
       </c>
       <c r="E36" s="13">
-        <v>231.35</v>
+        <v>232.87</v>
       </c>
       <c r="F36" s="13">
-        <v>240.35</v>
+        <v>241.87</v>
       </c>
       <c r="G36" s="17"/>
     </row>
-    <row r="37" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="37" spans="1:7" x14ac:dyDescent="0.45">
       <c r="A37" s="7">
-        <v>46303</v>
+        <v>46304</v>
       </c>
       <c r="B37" s="8"/>
       <c r="C37" s="20" t="s">
         <v>24</v>
       </c>
       <c r="D37" s="10">
-        <v>270.88</v>
+        <v>270.08999999999997</v>
       </c>
       <c r="E37" s="10" t="s">
         <v>18</v>
@@ -1356,16 +1356,16 @@
       </c>
       <c r="G37" s="17"/>
     </row>
-    <row r="38" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="38" spans="1:7" x14ac:dyDescent="0.45">
       <c r="A38" s="11">
-        <v>46302</v>
+        <v>46303</v>
       </c>
       <c r="B38" s="12"/>
       <c r="C38" s="12" t="s">
         <v>24</v>
       </c>
       <c r="D38" s="13">
-        <v>271.52999999999997</v>
+        <v>270.88</v>
       </c>
       <c r="E38" s="13" t="s">
         <v>18</v>
@@ -1375,7 +1375,7 @@
       </c>
       <c r="G38" s="17"/>
     </row>
-    <row r="39" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="39" spans="1:7" x14ac:dyDescent="0.45">
       <c r="A39" s="24"/>
       <c r="B39" s="24"/>
       <c r="C39" s="15"/>
@@ -1384,7 +1384,7 @@
       <c r="F39" s="17"/>
       <c r="G39" s="17"/>
     </row>
-    <row r="40" spans="1:7" ht="20.25" x14ac:dyDescent="0.25">
+    <row r="40" spans="1:7" ht="20.25" x14ac:dyDescent="0.45">
       <c r="A40" s="29" t="s">
         <v>25</v>
       </c>
@@ -1395,7 +1395,7 @@
       <c r="F40" s="17"/>
       <c r="G40" s="17"/>
     </row>
-    <row r="41" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="41" spans="1:7" x14ac:dyDescent="0.45">
       <c r="A41" s="23" t="s">
         <v>4</v>
       </c>
@@ -1414,83 +1414,83 @@
       </c>
       <c r="G41" s="17"/>
     </row>
-    <row r="42" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="42" spans="1:7" x14ac:dyDescent="0.45">
       <c r="A42" s="7">
-        <v>46303</v>
+        <v>46304</v>
       </c>
       <c r="B42" s="8"/>
       <c r="C42" s="20" t="s">
         <v>26</v>
       </c>
       <c r="D42" s="10">
-        <v>265.33999999999997</v>
+        <v>264.58999999999997</v>
       </c>
       <c r="E42" s="10">
-        <v>244.12</v>
+        <v>245.55</v>
       </c>
       <c r="F42" s="10">
-        <v>254.12</v>
+        <v>255.55</v>
       </c>
       <c r="G42" s="17"/>
     </row>
-    <row r="43" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="43" spans="1:7" x14ac:dyDescent="0.45">
       <c r="A43" s="11">
-        <v>46303</v>
+        <v>46304</v>
       </c>
       <c r="B43" s="12"/>
       <c r="C43" s="21" t="s">
         <v>27</v>
       </c>
       <c r="D43" s="13">
-        <v>264.95</v>
+        <v>264.2</v>
       </c>
       <c r="E43" s="13">
-        <v>244.54</v>
+        <v>245.96</v>
       </c>
       <c r="F43" s="13">
-        <v>254.54</v>
+        <v>255.96</v>
       </c>
       <c r="G43" s="17"/>
     </row>
-    <row r="44" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="44" spans="1:7" x14ac:dyDescent="0.45">
       <c r="A44" s="7">
-        <v>46302</v>
+        <v>46303</v>
       </c>
       <c r="B44" s="8"/>
       <c r="C44" s="20" t="s">
         <v>26</v>
       </c>
       <c r="D44" s="10">
-        <v>265.91000000000003</v>
+        <v>265.33999999999997</v>
       </c>
       <c r="E44" s="10">
-        <v>242.51</v>
+        <v>244.12</v>
       </c>
       <c r="F44" s="10">
-        <v>252.51</v>
+        <v>254.12</v>
       </c>
       <c r="G44" s="17"/>
     </row>
-    <row r="45" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="45" spans="1:7" x14ac:dyDescent="0.45">
       <c r="A45" s="11">
-        <v>46302</v>
+        <v>46303</v>
       </c>
       <c r="B45" s="12"/>
       <c r="C45" s="21" t="s">
         <v>27</v>
       </c>
       <c r="D45" s="13">
-        <v>265.52</v>
+        <v>264.95</v>
       </c>
       <c r="E45" s="13">
-        <v>242.92</v>
+        <v>244.54</v>
       </c>
       <c r="F45" s="13">
-        <v>252.92</v>
+        <v>254.54</v>
       </c>
       <c r="G45" s="17"/>
     </row>
-    <row r="46" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="46" spans="1:7" x14ac:dyDescent="0.45">
       <c r="A46" s="14"/>
       <c r="B46" s="24"/>
       <c r="C46" s="15"/>
@@ -1499,7 +1499,7 @@
       <c r="F46" s="16"/>
       <c r="G46" s="17"/>
     </row>
-    <row r="47" spans="1:7" ht="20.25" x14ac:dyDescent="0.25">
+    <row r="47" spans="1:7" ht="20.25" x14ac:dyDescent="0.45">
       <c r="A47" s="25" t="s">
         <v>28</v>
       </c>
@@ -1510,7 +1510,7 @@
       <c r="F47" s="17"/>
       <c r="G47" s="17"/>
     </row>
-    <row r="48" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="48" spans="1:7" x14ac:dyDescent="0.45">
       <c r="A48" s="23" t="s">
         <v>4</v>
       </c>
@@ -1529,83 +1529,83 @@
       </c>
       <c r="G48" s="17"/>
     </row>
-    <row r="49" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="49" spans="1:7" x14ac:dyDescent="0.45">
       <c r="A49" s="7">
-        <v>46303</v>
+        <v>46304</v>
       </c>
       <c r="B49" s="8"/>
       <c r="C49" s="20" t="s">
         <v>29</v>
       </c>
       <c r="D49" s="10">
-        <v>257.33</v>
+        <v>257</v>
       </c>
       <c r="E49" s="10">
-        <v>237.47</v>
+        <v>238.67</v>
       </c>
       <c r="F49" s="10">
-        <v>247.47</v>
+        <v>248.67</v>
       </c>
       <c r="G49" s="28"/>
     </row>
-    <row r="50" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="50" spans="1:7" x14ac:dyDescent="0.45">
       <c r="A50" s="11">
-        <v>46303</v>
+        <v>46304</v>
       </c>
       <c r="B50" s="12"/>
       <c r="C50" s="21" t="s">
         <v>30</v>
       </c>
       <c r="D50" s="13">
-        <v>254.86</v>
+        <v>254.51</v>
       </c>
       <c r="E50" s="13">
-        <v>237.1</v>
+        <v>238.29</v>
       </c>
       <c r="F50" s="13">
-        <v>247.1</v>
+        <v>248.29</v>
       </c>
       <c r="G50" s="28"/>
     </row>
-    <row r="51" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="51" spans="1:7" x14ac:dyDescent="0.45">
       <c r="A51" s="7">
-        <v>46302</v>
+        <v>46303</v>
       </c>
       <c r="B51" s="8"/>
       <c r="C51" s="20" t="s">
         <v>29</v>
       </c>
       <c r="D51" s="10">
-        <v>257.63</v>
+        <v>257.33</v>
       </c>
       <c r="E51" s="10">
-        <v>236.24</v>
+        <v>237.47</v>
       </c>
       <c r="F51" s="10">
-        <v>246.24</v>
+        <v>247.47</v>
       </c>
       <c r="G51" s="17"/>
     </row>
-    <row r="52" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="52" spans="1:7" x14ac:dyDescent="0.45">
       <c r="A52" s="11">
-        <v>46302</v>
+        <v>46303</v>
       </c>
       <c r="B52" s="12"/>
       <c r="C52" s="21" t="s">
         <v>30</v>
       </c>
       <c r="D52" s="13">
-        <v>255.2</v>
+        <v>254.86</v>
       </c>
       <c r="E52" s="13">
-        <v>235.89</v>
+        <v>237.1</v>
       </c>
       <c r="F52" s="13">
-        <v>245.89</v>
+        <v>247.1</v>
       </c>
       <c r="G52" s="17"/>
     </row>
-    <row r="53" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="53" spans="1:7" x14ac:dyDescent="0.45">
       <c r="A53" s="14"/>
       <c r="B53" s="14"/>
       <c r="C53" s="15"/>
@@ -1614,7 +1614,7 @@
       <c r="F53" s="16"/>
       <c r="G53" s="17"/>
     </row>
-    <row r="54" spans="1:7" ht="20.25" x14ac:dyDescent="0.25">
+    <row r="54" spans="1:7" ht="20.25" x14ac:dyDescent="0.45">
       <c r="A54" s="27" t="s">
         <v>31</v>
       </c>
@@ -1625,7 +1625,7 @@
       <c r="F54" s="17"/>
       <c r="G54" s="17"/>
     </row>
-    <row r="55" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="55" spans="1:7" x14ac:dyDescent="0.45">
       <c r="A55" s="23" t="s">
         <v>4</v>
       </c>
@@ -1644,54 +1644,54 @@
       </c>
       <c r="G55" s="17"/>
     </row>
-    <row r="56" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="56" spans="1:7" x14ac:dyDescent="0.45">
       <c r="A56" s="7">
-        <v>46303</v>
+        <v>46304</v>
       </c>
       <c r="B56" s="8"/>
       <c r="C56" s="20" t="s">
         <v>32</v>
       </c>
       <c r="D56" s="10">
-        <v>273.01</v>
+        <v>271.11</v>
       </c>
       <c r="E56" s="10">
-        <v>266.49</v>
+        <v>268.07</v>
       </c>
       <c r="F56" s="10">
-        <v>276.49</v>
+        <v>278.07</v>
       </c>
       <c r="G56" s="17"/>
     </row>
-    <row r="57" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="57" spans="1:7" x14ac:dyDescent="0.45">
       <c r="A57" s="11">
-        <v>46303</v>
+        <v>46304</v>
       </c>
       <c r="B57" s="12"/>
       <c r="C57" s="21" t="s">
         <v>33</v>
       </c>
       <c r="D57" s="13">
-        <v>262.44</v>
+        <v>260.56</v>
       </c>
       <c r="E57" s="13">
-        <v>247.48</v>
+        <v>248.82</v>
       </c>
       <c r="F57" s="13">
-        <v>257.48</v>
+        <v>258.82</v>
       </c>
       <c r="G57" s="17"/>
     </row>
-    <row r="58" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="58" spans="1:7" x14ac:dyDescent="0.45">
       <c r="A58" s="7">
-        <v>46303</v>
+        <v>46304</v>
       </c>
       <c r="B58" s="8"/>
       <c r="C58" s="20" t="s">
         <v>34</v>
       </c>
       <c r="D58" s="10">
-        <v>263.88</v>
+        <v>262.01</v>
       </c>
       <c r="E58" s="10" t="s">
         <v>18</v>
@@ -1701,111 +1701,111 @@
       </c>
       <c r="G58" s="17"/>
     </row>
-    <row r="59" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="59" spans="1:7" x14ac:dyDescent="0.45">
       <c r="A59" s="11">
-        <v>46303</v>
+        <v>46304</v>
       </c>
       <c r="B59" s="12"/>
       <c r="C59" s="21" t="s">
         <v>35</v>
       </c>
       <c r="D59" s="13">
-        <v>258.48</v>
+        <v>258.19</v>
       </c>
       <c r="E59" s="13">
-        <v>241.85</v>
+        <v>243.19</v>
       </c>
       <c r="F59" s="13" t="s">
         <v>18</v>
       </c>
       <c r="G59" s="17"/>
     </row>
-    <row r="60" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="60" spans="1:7" x14ac:dyDescent="0.45">
       <c r="A60" s="7">
-        <v>46303</v>
+        <v>46304</v>
       </c>
       <c r="B60" s="8"/>
       <c r="C60" s="20" t="s">
         <v>36</v>
       </c>
       <c r="D60" s="10">
-        <v>254.31</v>
+        <v>254.02</v>
       </c>
       <c r="E60" s="10">
-        <v>237.8</v>
+        <v>239.14</v>
       </c>
       <c r="F60" s="10">
-        <v>247.8</v>
+        <v>249.14</v>
       </c>
       <c r="G60" s="17"/>
     </row>
-    <row r="61" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="61" spans="1:7" x14ac:dyDescent="0.45">
       <c r="A61" s="11">
-        <v>46303</v>
+        <v>46304</v>
       </c>
       <c r="B61" s="12"/>
       <c r="C61" s="21" t="s">
         <v>37</v>
       </c>
       <c r="D61" s="13">
-        <v>259.13</v>
+        <v>258.29000000000002</v>
       </c>
       <c r="E61" s="13">
-        <v>259.7</v>
+        <v>261.19</v>
       </c>
       <c r="F61" s="13" t="s">
         <v>18</v>
       </c>
       <c r="G61" s="17"/>
     </row>
-    <row r="62" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="62" spans="1:7" x14ac:dyDescent="0.45">
       <c r="A62" s="7">
-        <v>46302</v>
+        <v>46303</v>
       </c>
       <c r="B62" s="8"/>
       <c r="C62" s="20" t="s">
         <v>32</v>
       </c>
       <c r="D62" s="10">
-        <v>273.7</v>
+        <v>273.01</v>
       </c>
       <c r="E62" s="10">
-        <v>264.52</v>
+        <v>266.49</v>
       </c>
       <c r="F62" s="10">
-        <v>274.52</v>
+        <v>276.49</v>
       </c>
       <c r="G62" s="17"/>
     </row>
-    <row r="63" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="63" spans="1:7" x14ac:dyDescent="0.45">
       <c r="A63" s="11">
-        <v>46302</v>
+        <v>46303</v>
       </c>
       <c r="B63" s="12"/>
       <c r="C63" s="21" t="s">
         <v>33</v>
       </c>
       <c r="D63" s="13">
-        <v>263.08</v>
+        <v>262.44</v>
       </c>
       <c r="E63" s="13">
-        <v>246.07</v>
+        <v>247.48</v>
       </c>
       <c r="F63" s="13">
-        <v>256.07</v>
+        <v>257.48</v>
       </c>
       <c r="G63" s="17"/>
     </row>
-    <row r="64" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="64" spans="1:7" x14ac:dyDescent="0.45">
       <c r="A64" s="7">
-        <v>46302</v>
+        <v>46303</v>
       </c>
       <c r="B64" s="8"/>
       <c r="C64" s="20" t="s">
         <v>34</v>
       </c>
       <c r="D64" s="10">
-        <v>264.51</v>
+        <v>263.88</v>
       </c>
       <c r="E64" s="10" t="s">
         <v>18</v>
@@ -1815,55 +1815,55 @@
       </c>
       <c r="G64" s="17"/>
     </row>
-    <row r="65" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="65" spans="1:6" x14ac:dyDescent="0.45">
       <c r="A65" s="11">
-        <v>46302</v>
+        <v>46303</v>
       </c>
       <c r="B65" s="12"/>
       <c r="C65" s="21" t="s">
         <v>35</v>
       </c>
       <c r="D65" s="13">
-        <v>258.70999999999998</v>
+        <v>258.48</v>
       </c>
       <c r="E65" s="13">
-        <v>240.44</v>
+        <v>241.85</v>
       </c>
       <c r="F65" s="13" t="s">
         <v>18</v>
       </c>
     </row>
-    <row r="66" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="66" spans="1:6" x14ac:dyDescent="0.45">
       <c r="A66" s="7">
-        <v>46302</v>
+        <v>46303</v>
       </c>
       <c r="B66" s="8"/>
       <c r="C66" s="20" t="s">
         <v>36</v>
       </c>
       <c r="D66" s="10">
-        <v>254.54</v>
+        <v>254.31</v>
       </c>
       <c r="E66" s="10">
-        <v>236.39</v>
+        <v>237.8</v>
       </c>
       <c r="F66" s="10">
-        <v>246.39</v>
-      </c>
-    </row>
-    <row r="67" spans="1:6" x14ac:dyDescent="0.25">
+        <v>247.8</v>
+      </c>
+    </row>
+    <row r="67" spans="1:6" x14ac:dyDescent="0.45">
       <c r="A67" s="11">
-        <v>46302</v>
+        <v>46303</v>
       </c>
       <c r="B67" s="12"/>
       <c r="C67" s="21" t="s">
         <v>37</v>
       </c>
       <c r="D67" s="13">
-        <v>259.91000000000003</v>
+        <v>259.13</v>
       </c>
       <c r="E67" s="13">
-        <v>257.92</v>
+        <v>259.7</v>
       </c>
       <c r="F67" s="13" t="s">
         <v>18</v>
@@ -1900,17 +1900,6 @@
 </file>
 
 <file path=customXml/item2.xml><?xml version="1.0" encoding="utf-8"?>
-<p:properties xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls">
-  <documentManagement>
-    <lcf76f155ced4ddcb4097134ff3c332f xmlns="87276d81-85f4-4ef2-9e6e-55066304288f">
-      <Terms xmlns="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
-    </lcf76f155ced4ddcb4097134ff3c332f>
-    <TaxCatchAll xmlns="b23b8984-eafa-4e79-985e-54f52f3da58e" xsi:nil="true"/>
-  </documentManagement>
-</p:properties>
-</file>
-
-<file path=customXml/item3.xml><?xml version="1.0" encoding="utf-8"?>
 <ct:contentTypeSchema xmlns:ct="http://schemas.microsoft.com/office/2006/metadata/contentType" xmlns:ma="http://schemas.microsoft.com/office/2006/metadata/properties/metaAttributes" ct:_="" ma:_="" ma:contentTypeName="Document" ma:contentTypeID="0x010100D3632DF5622958439304627C030B0427" ma:contentTypeVersion="18" ma:contentTypeDescription="Create a new document." ma:contentTypeScope="" ma:versionID="8c2ecbce386d6bac497f8eb2d8f0fb7a">
   <xsd:schema xmlns:xsd="http://www.w3.org/2001/XMLSchema" xmlns:xs="http://www.w3.org/2001/XMLSchema" xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:ns2="87276d81-85f4-4ef2-9e6e-55066304288f" xmlns:ns3="39e1dda6-d1d8-4c88-a3b9-f1abc1284bad" xmlns:ns4="b23b8984-eafa-4e79-985e-54f52f3da58e" targetNamespace="http://schemas.microsoft.com/office/2006/metadata/properties" ma:root="true" ma:fieldsID="4cfd0c2f651c1ce156ad4fcb44ea61dd" ns2:_="" ns3:_="" ns4:_="">
     <xsd:import namespace="87276d81-85f4-4ef2-9e6e-55066304288f"/>
@@ -2170,6 +2159,17 @@
 </ct:contentTypeSchema>
 </file>
 
+<file path=customXml/item3.xml><?xml version="1.0" encoding="utf-8"?>
+<p:properties xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls">
+  <documentManagement>
+    <lcf76f155ced4ddcb4097134ff3c332f xmlns="87276d81-85f4-4ef2-9e6e-55066304288f">
+      <Terms xmlns="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
+    </lcf76f155ced4ddcb4097134ff3c332f>
+    <TaxCatchAll xmlns="b23b8984-eafa-4e79-985e-54f52f3da58e" xsi:nil="true"/>
+  </documentManagement>
+</p:properties>
+</file>
+
 <file path=customXml/itemProps1.xml><?xml version="1.0" encoding="utf-8"?>
 <ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{F60519E9-FD90-4339-869C-BC2F85719BB8}">
   <ds:schemaRefs>
@@ -2179,17 +2179,6 @@
 </file>
 
 <file path=customXml/itemProps2.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{57A83D98-2BAE-4D83-823A-D31C464B620C}">
-  <ds:schemaRefs>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/properties"/>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
-    <ds:schemaRef ds:uri="87276d81-85f4-4ef2-9e6e-55066304288f"/>
-    <ds:schemaRef ds:uri="b23b8984-eafa-4e79-985e-54f52f3da58e"/>
-  </ds:schemaRefs>
-</ds:datastoreItem>
-</file>
-
-<file path=customXml/itemProps3.xml><?xml version="1.0" encoding="utf-8"?>
 <ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{B44E1863-2778-41F9-ACBA-48420F931671}">
   <ds:schemaRefs>
     <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/contentType"/>
@@ -2209,6 +2198,17 @@
 </ds:datastoreItem>
 </file>
 
+<file path=customXml/itemProps3.xml><?xml version="1.0" encoding="utf-8"?>
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{57A83D98-2BAE-4D83-823A-D31C464B620C}">
+  <ds:schemaRefs>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/properties"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
+    <ds:schemaRef ds:uri="87276d81-85f4-4ef2-9e6e-55066304288f"/>
+    <ds:schemaRef ds:uri="b23b8984-eafa-4e79-985e-54f52f3da58e"/>
+  </ds:schemaRefs>
+</ds:datastoreItem>
+</file>
+
 <file path=docMetadata/LabelInfo.xml><?xml version="1.0" encoding="utf-8"?>
 <clbl:labelList xmlns:clbl="http://schemas.microsoft.com/office/2020/mipLabelMetadata">
   <clbl:label id="{569bf4a9-87bd-4dbf-a36c-1db5158e5def}" enabled="1" method="Privileged" siteId="{ea80952e-a476-42d4-aaf4-5457852b0f7e}" removed="0"/>

</xml_diff>

<commit_message>
Fri Oct  9 07:30:28 UTC 2026
</commit_message>
<xml_diff>
--- a/bp.com-content-dam-bp-country-sites-en_au-australia-home-products-services-pricing-tgp-excel.xlsx
+++ b/bp.com-content-dam-bp-country-sites-en_au-australia-home-products-services-pricing-tgp-excel.xlsx
@@ -8,14 +8,14 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://bp365.sharepoint.com/sites/WholesalePricing/Shared Documents/B2C/TGP/Daily TGP/Web TGP/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="14_{7AA9A883-8E9D-426C-BA68-AA56CC5C61BF}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="14_{90B6C5B8-2282-405A-89C3-EDF5CC535555}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-8595" yWindow="-16320" windowWidth="29040" windowHeight="15720" xr2:uid="{1B412EEF-F96D-4DF4-A4E9-C7F0F183C2FB}"/>
+    <workbookView xWindow="2205" yWindow="2205" windowWidth="11235" windowHeight="9338" xr2:uid="{1B412EEF-F96D-4DF4-A4E9-C7F0F183C2FB}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
   </sheets>
-  <calcPr calcId="191028" calcOnSave="0"/>
+  <calcPr calcId="191028"/>
   <extLst>
     <ext xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" uri="{140A7094-0E35-4892-8432-C4D2E57EDEB5}">
       <x15:workbookPr chartTrackingRefBase="1"/>
@@ -808,128 +808,128 @@
     </row>
     <row r="8" spans="1:7" x14ac:dyDescent="0.45">
       <c r="A8" s="7">
-        <v>46304</v>
+        <v>46305</v>
       </c>
       <c r="B8" s="8"/>
       <c r="C8" s="9" t="s">
         <v>10</v>
       </c>
       <c r="D8" s="10">
-        <v>259.77999999999997</v>
+        <v>259.31</v>
       </c>
       <c r="E8" s="10">
-        <v>237.83</v>
+        <v>239.15</v>
       </c>
       <c r="F8" s="10">
-        <v>247.83</v>
+        <v>249.15</v>
       </c>
       <c r="G8" s="10">
-        <v>235.44</v>
+        <v>236.77</v>
       </c>
     </row>
     <row r="9" spans="1:7" x14ac:dyDescent="0.45">
       <c r="A9" s="11">
-        <v>46304</v>
+        <v>46305</v>
       </c>
       <c r="B9" s="12"/>
       <c r="C9" s="12" t="s">
         <v>11</v>
       </c>
       <c r="D9" s="13">
-        <v>259.77999999999997</v>
+        <v>259.31</v>
       </c>
       <c r="E9" s="13">
-        <v>237.83</v>
+        <v>239.15</v>
       </c>
       <c r="F9" s="13">
-        <v>247.83</v>
+        <v>249.15</v>
       </c>
       <c r="G9" s="13">
-        <v>235.44</v>
+        <v>236.77</v>
       </c>
     </row>
     <row r="10" spans="1:7" x14ac:dyDescent="0.45">
       <c r="A10" s="7">
-        <v>46304</v>
+        <v>46305</v>
       </c>
       <c r="B10" s="8"/>
       <c r="C10" s="9" t="s">
         <v>12</v>
       </c>
       <c r="D10" s="10">
-        <v>255.92</v>
+        <v>255.41</v>
       </c>
       <c r="E10" s="10">
-        <v>238.64</v>
+        <v>238.27</v>
       </c>
       <c r="F10" s="10">
-        <v>248.64</v>
+        <v>248.27</v>
       </c>
       <c r="G10" s="10">
-        <v>237.04</v>
+        <v>236.68</v>
       </c>
     </row>
     <row r="11" spans="1:7" x14ac:dyDescent="0.45">
       <c r="A11" s="11">
-        <v>46303</v>
+        <v>46304</v>
       </c>
       <c r="B11" s="12"/>
       <c r="C11" s="12" t="s">
         <v>10</v>
       </c>
       <c r="D11" s="13">
-        <v>260.22000000000003</v>
+        <v>259.77999999999997</v>
       </c>
       <c r="E11" s="13">
-        <v>236.63</v>
+        <v>237.83</v>
       </c>
       <c r="F11" s="13">
-        <v>246.63</v>
+        <v>247.83</v>
       </c>
       <c r="G11" s="13">
-        <v>234.24</v>
+        <v>235.44</v>
       </c>
     </row>
     <row r="12" spans="1:7" x14ac:dyDescent="0.45">
       <c r="A12" s="7">
-        <v>46303</v>
+        <v>46304</v>
       </c>
       <c r="B12" s="8"/>
       <c r="C12" s="9" t="s">
         <v>11</v>
       </c>
       <c r="D12" s="10">
-        <v>260.22000000000003</v>
+        <v>259.77999999999997</v>
       </c>
       <c r="E12" s="10">
-        <v>236.63</v>
+        <v>237.83</v>
       </c>
       <c r="F12" s="10">
-        <v>246.63</v>
+        <v>247.83</v>
       </c>
       <c r="G12" s="10">
-        <v>234.24</v>
+        <v>235.44</v>
       </c>
     </row>
     <row r="13" spans="1:7" x14ac:dyDescent="0.45">
       <c r="A13" s="11">
-        <v>46303</v>
+        <v>46304</v>
       </c>
       <c r="B13" s="12"/>
       <c r="C13" s="12" t="s">
         <v>12</v>
       </c>
       <c r="D13" s="13">
-        <v>256.7</v>
+        <v>255.92</v>
       </c>
       <c r="E13" s="13">
-        <v>237.25</v>
+        <v>238.64</v>
       </c>
       <c r="F13" s="13">
-        <v>247.25</v>
+        <v>248.64</v>
       </c>
       <c r="G13" s="13">
-        <v>235.65</v>
+        <v>237.04</v>
       </c>
     </row>
     <row r="14" spans="1:7" x14ac:dyDescent="0.45">
@@ -973,39 +973,39 @@
     </row>
     <row r="17" spans="1:7" x14ac:dyDescent="0.45">
       <c r="A17" s="7">
-        <v>46304</v>
+        <v>46305</v>
       </c>
       <c r="B17" s="8"/>
       <c r="C17" s="20" t="s">
         <v>14</v>
       </c>
       <c r="D17" s="10">
-        <v>259.24</v>
+        <v>258.75</v>
       </c>
       <c r="E17" s="10">
-        <v>243.72</v>
+        <v>243.37</v>
       </c>
       <c r="F17" s="10">
-        <v>253.72</v>
+        <v>253.37</v>
       </c>
       <c r="G17" s="17"/>
     </row>
     <row r="18" spans="1:7" x14ac:dyDescent="0.45">
       <c r="A18" s="11">
-        <v>46303</v>
+        <v>46304</v>
       </c>
       <c r="B18" s="12"/>
       <c r="C18" s="12" t="s">
         <v>14</v>
       </c>
       <c r="D18" s="13">
-        <v>260.07</v>
+        <v>259.24</v>
       </c>
       <c r="E18" s="13">
-        <v>242.36</v>
+        <v>243.72</v>
       </c>
       <c r="F18" s="13">
-        <v>252.36</v>
+        <v>253.72</v>
       </c>
       <c r="G18" s="17"/>
     </row>
@@ -1052,41 +1052,41 @@
     </row>
     <row r="22" spans="1:7" x14ac:dyDescent="0.45">
       <c r="A22" s="7">
-        <v>46304</v>
+        <v>46305</v>
       </c>
       <c r="B22" s="8"/>
       <c r="C22" s="20" t="s">
         <v>16</v>
       </c>
       <c r="D22" s="10">
-        <v>260.89999999999998</v>
+        <v>260.44</v>
       </c>
       <c r="E22" s="10">
-        <v>237.41</v>
+        <v>238.19</v>
       </c>
       <c r="F22" s="10">
-        <v>247.01</v>
+        <v>247.78</v>
       </c>
       <c r="G22" s="10">
-        <v>233.78</v>
+        <v>234.56</v>
       </c>
     </row>
     <row r="23" spans="1:7" x14ac:dyDescent="0.45">
       <c r="A23" s="11">
-        <v>46304</v>
+        <v>46305</v>
       </c>
       <c r="B23" s="12"/>
       <c r="C23" s="21" t="s">
         <v>17</v>
       </c>
       <c r="D23" s="13">
-        <v>260.89</v>
+        <v>260.38</v>
       </c>
       <c r="E23" s="13">
-        <v>249.2</v>
+        <v>248.82</v>
       </c>
       <c r="F23" s="13">
-        <v>259.2</v>
+        <v>258.82</v>
       </c>
       <c r="G23" s="13" t="s">
         <v>18</v>
@@ -1094,20 +1094,20 @@
     </row>
     <row r="24" spans="1:7" x14ac:dyDescent="0.45">
       <c r="A24" s="7">
-        <v>46304</v>
+        <v>46305</v>
       </c>
       <c r="B24" s="8"/>
       <c r="C24" s="20" t="s">
         <v>19</v>
       </c>
       <c r="D24" s="10">
-        <v>261.22000000000003</v>
+        <v>260.72000000000003</v>
       </c>
       <c r="E24" s="10">
-        <v>248.42</v>
+        <v>248.05</v>
       </c>
       <c r="F24" s="10">
-        <v>258.42</v>
+        <v>258.05</v>
       </c>
       <c r="G24" s="10" t="s">
         <v>18</v>
@@ -1115,41 +1115,41 @@
     </row>
     <row r="25" spans="1:7" x14ac:dyDescent="0.45">
       <c r="A25" s="11">
-        <v>46304</v>
+        <v>46305</v>
       </c>
       <c r="B25" s="12"/>
       <c r="C25" s="21" t="s">
         <v>20</v>
       </c>
       <c r="D25" s="13">
-        <v>257.88</v>
+        <v>257.37</v>
       </c>
       <c r="E25" s="13">
-        <v>248.68</v>
+        <v>248.31</v>
       </c>
       <c r="F25" s="13">
-        <v>258.68</v>
+        <v>258.31</v>
       </c>
       <c r="G25" s="13">
-        <v>244.52</v>
+        <v>244.15</v>
       </c>
     </row>
     <row r="26" spans="1:7" x14ac:dyDescent="0.45">
       <c r="A26" s="7">
-        <v>46304</v>
+        <v>46305</v>
       </c>
       <c r="B26" s="8"/>
       <c r="C26" s="20" t="s">
         <v>21</v>
       </c>
       <c r="D26" s="10">
-        <v>259.39999999999998</v>
+        <v>258.89</v>
       </c>
       <c r="E26" s="10">
-        <v>250.25</v>
+        <v>249.87</v>
       </c>
       <c r="F26" s="10">
-        <v>260.25</v>
+        <v>259.87</v>
       </c>
       <c r="G26" s="10" t="s">
         <v>18</v>
@@ -1157,41 +1157,41 @@
     </row>
     <row r="27" spans="1:7" x14ac:dyDescent="0.45">
       <c r="A27" s="11">
-        <v>46303</v>
+        <v>46304</v>
       </c>
       <c r="B27" s="12"/>
       <c r="C27" s="12" t="s">
         <v>16</v>
       </c>
       <c r="D27" s="13">
-        <v>261.35000000000002</v>
+        <v>260.89999999999998</v>
       </c>
       <c r="E27" s="13">
-        <v>236.21</v>
+        <v>237.41</v>
       </c>
       <c r="F27" s="13">
-        <v>245.81</v>
+        <v>247.01</v>
       </c>
       <c r="G27" s="13">
-        <v>232.58</v>
+        <v>233.78</v>
       </c>
     </row>
     <row r="28" spans="1:7" x14ac:dyDescent="0.45">
       <c r="A28" s="7">
-        <v>46303</v>
+        <v>46304</v>
       </c>
       <c r="B28" s="8"/>
       <c r="C28" s="20" t="s">
         <v>17</v>
       </c>
       <c r="D28" s="10">
-        <v>261.67</v>
+        <v>260.89</v>
       </c>
       <c r="E28" s="22">
-        <v>247.79</v>
+        <v>249.2</v>
       </c>
       <c r="F28" s="22">
-        <v>257.79000000000002</v>
+        <v>259.2</v>
       </c>
       <c r="G28" s="22" t="s">
         <v>18</v>
@@ -1199,20 +1199,20 @@
     </row>
     <row r="29" spans="1:7" x14ac:dyDescent="0.45">
       <c r="A29" s="11">
-        <v>46303</v>
+        <v>46304</v>
       </c>
       <c r="B29" s="12"/>
       <c r="C29" s="12" t="s">
         <v>19</v>
       </c>
       <c r="D29" s="13">
-        <v>262.01</v>
+        <v>261.22000000000003</v>
       </c>
       <c r="E29" s="13">
-        <v>247.01</v>
+        <v>248.42</v>
       </c>
       <c r="F29" s="13">
-        <v>257.02</v>
+        <v>258.42</v>
       </c>
       <c r="G29" s="13" t="s">
         <v>18</v>
@@ -1220,41 +1220,41 @@
     </row>
     <row r="30" spans="1:7" x14ac:dyDescent="0.45">
       <c r="A30" s="7">
-        <v>46303</v>
+        <v>46304</v>
       </c>
       <c r="B30" s="8"/>
       <c r="C30" s="20" t="s">
         <v>20</v>
       </c>
       <c r="D30" s="10">
-        <v>258.66000000000003</v>
+        <v>257.88</v>
       </c>
       <c r="E30" s="22">
-        <v>247.27</v>
+        <v>248.68</v>
       </c>
       <c r="F30" s="22">
-        <v>257.27</v>
+        <v>258.68</v>
       </c>
       <c r="G30" s="22">
-        <v>243.11</v>
+        <v>244.52</v>
       </c>
     </row>
     <row r="31" spans="1:7" x14ac:dyDescent="0.45">
       <c r="A31" s="11">
-        <v>46303</v>
+        <v>46304</v>
       </c>
       <c r="B31" s="12"/>
       <c r="C31" s="12" t="s">
         <v>21</v>
       </c>
       <c r="D31" s="13">
-        <v>260.19</v>
+        <v>259.39999999999998</v>
       </c>
       <c r="E31" s="13">
-        <v>248.82</v>
+        <v>250.25</v>
       </c>
       <c r="F31" s="13">
-        <v>258.82</v>
+        <v>260.25</v>
       </c>
       <c r="G31" s="13" t="s">
         <v>18</v>
@@ -1301,52 +1301,52 @@
     </row>
     <row r="35" spans="1:7" x14ac:dyDescent="0.45">
       <c r="A35" s="7">
-        <v>46304</v>
+        <v>46305</v>
       </c>
       <c r="B35" s="8"/>
       <c r="C35" s="20" t="s">
         <v>23</v>
       </c>
       <c r="D35" s="10">
-        <v>254.47</v>
+        <v>253.96</v>
       </c>
       <c r="E35" s="10">
-        <v>234.26</v>
+        <v>234.45</v>
       </c>
       <c r="F35" s="10">
-        <v>243.27</v>
+        <v>243.45</v>
       </c>
       <c r="G35" s="17"/>
     </row>
     <row r="36" spans="1:7" x14ac:dyDescent="0.45">
       <c r="A36" s="11">
-        <v>46303</v>
+        <v>46304</v>
       </c>
       <c r="B36" s="12"/>
       <c r="C36" s="12" t="s">
         <v>23</v>
       </c>
       <c r="D36" s="13">
-        <v>255.26</v>
+        <v>254.47</v>
       </c>
       <c r="E36" s="13">
-        <v>232.87</v>
+        <v>234.26</v>
       </c>
       <c r="F36" s="13">
-        <v>241.87</v>
+        <v>243.27</v>
       </c>
       <c r="G36" s="17"/>
     </row>
     <row r="37" spans="1:7" x14ac:dyDescent="0.45">
       <c r="A37" s="7">
-        <v>46304</v>
+        <v>46305</v>
       </c>
       <c r="B37" s="8"/>
       <c r="C37" s="20" t="s">
         <v>24</v>
       </c>
       <c r="D37" s="10">
-        <v>270.08999999999997</v>
+        <v>269.58</v>
       </c>
       <c r="E37" s="10" t="s">
         <v>18</v>
@@ -1358,14 +1358,14 @@
     </row>
     <row r="38" spans="1:7" x14ac:dyDescent="0.45">
       <c r="A38" s="11">
-        <v>46303</v>
+        <v>46304</v>
       </c>
       <c r="B38" s="12"/>
       <c r="C38" s="12" t="s">
         <v>24</v>
       </c>
       <c r="D38" s="13">
-        <v>270.88</v>
+        <v>270.08999999999997</v>
       </c>
       <c r="E38" s="13" t="s">
         <v>18</v>
@@ -1416,77 +1416,77 @@
     </row>
     <row r="42" spans="1:7" x14ac:dyDescent="0.45">
       <c r="A42" s="7">
-        <v>46304</v>
+        <v>46305</v>
       </c>
       <c r="B42" s="8"/>
       <c r="C42" s="20" t="s">
         <v>26</v>
       </c>
       <c r="D42" s="10">
-        <v>264.58999999999997</v>
+        <v>264.06</v>
       </c>
       <c r="E42" s="10">
-        <v>245.55</v>
+        <v>245.34</v>
       </c>
       <c r="F42" s="10">
-        <v>255.55</v>
+        <v>255.34</v>
       </c>
       <c r="G42" s="17"/>
     </row>
     <row r="43" spans="1:7" x14ac:dyDescent="0.45">
       <c r="A43" s="11">
-        <v>46304</v>
+        <v>46305</v>
       </c>
       <c r="B43" s="12"/>
       <c r="C43" s="21" t="s">
         <v>27</v>
       </c>
       <c r="D43" s="13">
-        <v>264.2</v>
+        <v>263.68</v>
       </c>
       <c r="E43" s="13">
-        <v>245.96</v>
+        <v>245.75</v>
       </c>
       <c r="F43" s="13">
-        <v>255.96</v>
+        <v>255.75</v>
       </c>
       <c r="G43" s="17"/>
     </row>
     <row r="44" spans="1:7" x14ac:dyDescent="0.45">
       <c r="A44" s="7">
-        <v>46303</v>
+        <v>46304</v>
       </c>
       <c r="B44" s="8"/>
       <c r="C44" s="20" t="s">
         <v>26</v>
       </c>
       <c r="D44" s="10">
-        <v>265.33999999999997</v>
+        <v>264.58999999999997</v>
       </c>
       <c r="E44" s="10">
-        <v>244.12</v>
+        <v>245.55</v>
       </c>
       <c r="F44" s="10">
-        <v>254.12</v>
+        <v>255.55</v>
       </c>
       <c r="G44" s="17"/>
     </row>
     <row r="45" spans="1:7" x14ac:dyDescent="0.45">
       <c r="A45" s="11">
-        <v>46303</v>
+        <v>46304</v>
       </c>
       <c r="B45" s="12"/>
       <c r="C45" s="21" t="s">
         <v>27</v>
       </c>
       <c r="D45" s="13">
-        <v>264.95</v>
+        <v>264.2</v>
       </c>
       <c r="E45" s="13">
-        <v>244.54</v>
+        <v>245.96</v>
       </c>
       <c r="F45" s="13">
-        <v>254.54</v>
+        <v>255.96</v>
       </c>
       <c r="G45" s="17"/>
     </row>
@@ -1531,77 +1531,77 @@
     </row>
     <row r="49" spans="1:7" x14ac:dyDescent="0.45">
       <c r="A49" s="7">
-        <v>46304</v>
+        <v>46305</v>
       </c>
       <c r="B49" s="8"/>
       <c r="C49" s="20" t="s">
         <v>29</v>
       </c>
       <c r="D49" s="10">
-        <v>257</v>
+        <v>258.29000000000002</v>
       </c>
       <c r="E49" s="10">
-        <v>238.67</v>
+        <v>240.22</v>
       </c>
       <c r="F49" s="10">
-        <v>248.67</v>
+        <v>250.22</v>
       </c>
       <c r="G49" s="28"/>
     </row>
     <row r="50" spans="1:7" x14ac:dyDescent="0.45">
       <c r="A50" s="11">
-        <v>46304</v>
+        <v>46305</v>
       </c>
       <c r="B50" s="12"/>
       <c r="C50" s="21" t="s">
         <v>30</v>
       </c>
       <c r="D50" s="13">
-        <v>254.51</v>
+        <v>255.79</v>
       </c>
       <c r="E50" s="13">
-        <v>238.29</v>
+        <v>239.84</v>
       </c>
       <c r="F50" s="13">
-        <v>248.29</v>
+        <v>249.84</v>
       </c>
       <c r="G50" s="28"/>
     </row>
     <row r="51" spans="1:7" x14ac:dyDescent="0.45">
       <c r="A51" s="7">
-        <v>46303</v>
+        <v>46304</v>
       </c>
       <c r="B51" s="8"/>
       <c r="C51" s="20" t="s">
         <v>29</v>
       </c>
       <c r="D51" s="10">
-        <v>257.33</v>
+        <v>257</v>
       </c>
       <c r="E51" s="10">
-        <v>237.47</v>
+        <v>238.67</v>
       </c>
       <c r="F51" s="10">
-        <v>247.47</v>
+        <v>248.67</v>
       </c>
       <c r="G51" s="17"/>
     </row>
     <row r="52" spans="1:7" x14ac:dyDescent="0.45">
       <c r="A52" s="11">
-        <v>46303</v>
+        <v>46304</v>
       </c>
       <c r="B52" s="12"/>
       <c r="C52" s="21" t="s">
         <v>30</v>
       </c>
       <c r="D52" s="13">
-        <v>254.86</v>
+        <v>254.51</v>
       </c>
       <c r="E52" s="13">
-        <v>237.1</v>
+        <v>238.29</v>
       </c>
       <c r="F52" s="13">
-        <v>247.1</v>
+        <v>248.29</v>
       </c>
       <c r="G52" s="17"/>
     </row>
@@ -1646,52 +1646,52 @@
     </row>
     <row r="56" spans="1:7" x14ac:dyDescent="0.45">
       <c r="A56" s="7">
-        <v>46304</v>
+        <v>46305</v>
       </c>
       <c r="B56" s="8"/>
       <c r="C56" s="20" t="s">
         <v>32</v>
       </c>
       <c r="D56" s="10">
-        <v>271.11</v>
+        <v>270.06</v>
       </c>
       <c r="E56" s="10">
-        <v>268.07</v>
+        <v>267.62</v>
       </c>
       <c r="F56" s="10">
-        <v>278.07</v>
+        <v>277.62</v>
       </c>
       <c r="G56" s="17"/>
     </row>
     <row r="57" spans="1:7" x14ac:dyDescent="0.45">
       <c r="A57" s="11">
-        <v>46304</v>
+        <v>46305</v>
       </c>
       <c r="B57" s="12"/>
       <c r="C57" s="21" t="s">
         <v>33</v>
       </c>
       <c r="D57" s="13">
-        <v>260.56</v>
+        <v>260.05</v>
       </c>
       <c r="E57" s="13">
-        <v>248.82</v>
+        <v>248.47</v>
       </c>
       <c r="F57" s="13">
-        <v>258.82</v>
+        <v>258.47000000000003</v>
       </c>
       <c r="G57" s="17"/>
     </row>
     <row r="58" spans="1:7" x14ac:dyDescent="0.45">
       <c r="A58" s="7">
-        <v>46304</v>
+        <v>46305</v>
       </c>
       <c r="B58" s="8"/>
       <c r="C58" s="20" t="s">
         <v>34</v>
       </c>
       <c r="D58" s="10">
-        <v>262.01</v>
+        <v>260.95</v>
       </c>
       <c r="E58" s="10" t="s">
         <v>18</v>
@@ -1703,17 +1703,17 @@
     </row>
     <row r="59" spans="1:7" x14ac:dyDescent="0.45">
       <c r="A59" s="11">
-        <v>46304</v>
+        <v>46305</v>
       </c>
       <c r="B59" s="12"/>
       <c r="C59" s="21" t="s">
         <v>35</v>
       </c>
       <c r="D59" s="13">
-        <v>258.19</v>
+        <v>257.70999999999998</v>
       </c>
       <c r="E59" s="13">
-        <v>243.19</v>
+        <v>242.84</v>
       </c>
       <c r="F59" s="13" t="s">
         <v>18</v>
@@ -1722,36 +1722,36 @@
     </row>
     <row r="60" spans="1:7" x14ac:dyDescent="0.45">
       <c r="A60" s="7">
-        <v>46304</v>
+        <v>46305</v>
       </c>
       <c r="B60" s="8"/>
       <c r="C60" s="20" t="s">
         <v>36</v>
       </c>
       <c r="D60" s="10">
-        <v>254.02</v>
+        <v>253.53</v>
       </c>
       <c r="E60" s="10">
-        <v>239.14</v>
+        <v>238.79</v>
       </c>
       <c r="F60" s="10">
-        <v>249.14</v>
+        <v>248.79</v>
       </c>
       <c r="G60" s="17"/>
     </row>
     <row r="61" spans="1:7" x14ac:dyDescent="0.45">
       <c r="A61" s="11">
-        <v>46304</v>
+        <v>46305</v>
       </c>
       <c r="B61" s="12"/>
       <c r="C61" s="21" t="s">
         <v>37</v>
       </c>
       <c r="D61" s="13">
-        <v>258.29000000000002</v>
+        <v>257.81</v>
       </c>
       <c r="E61" s="13">
-        <v>261.19</v>
+        <v>260.77999999999997</v>
       </c>
       <c r="F61" s="13" t="s">
         <v>18</v>
@@ -1760,52 +1760,52 @@
     </row>
     <row r="62" spans="1:7" x14ac:dyDescent="0.45">
       <c r="A62" s="7">
-        <v>46303</v>
+        <v>46304</v>
       </c>
       <c r="B62" s="8"/>
       <c r="C62" s="20" t="s">
         <v>32</v>
       </c>
       <c r="D62" s="10">
-        <v>273.01</v>
+        <v>271.11</v>
       </c>
       <c r="E62" s="10">
-        <v>266.49</v>
+        <v>268.07</v>
       </c>
       <c r="F62" s="10">
-        <v>276.49</v>
+        <v>278.07</v>
       </c>
       <c r="G62" s="17"/>
     </row>
     <row r="63" spans="1:7" x14ac:dyDescent="0.45">
       <c r="A63" s="11">
-        <v>46303</v>
+        <v>46304</v>
       </c>
       <c r="B63" s="12"/>
       <c r="C63" s="21" t="s">
         <v>33</v>
       </c>
       <c r="D63" s="13">
-        <v>262.44</v>
+        <v>260.56</v>
       </c>
       <c r="E63" s="13">
-        <v>247.48</v>
+        <v>248.82</v>
       </c>
       <c r="F63" s="13">
-        <v>257.48</v>
+        <v>258.82</v>
       </c>
       <c r="G63" s="17"/>
     </row>
     <row r="64" spans="1:7" x14ac:dyDescent="0.45">
       <c r="A64" s="7">
-        <v>46303</v>
+        <v>46304</v>
       </c>
       <c r="B64" s="8"/>
       <c r="C64" s="20" t="s">
         <v>34</v>
       </c>
       <c r="D64" s="10">
-        <v>263.88</v>
+        <v>262.01</v>
       </c>
       <c r="E64" s="10" t="s">
         <v>18</v>
@@ -1817,17 +1817,17 @@
     </row>
     <row r="65" spans="1:6" x14ac:dyDescent="0.45">
       <c r="A65" s="11">
-        <v>46303</v>
+        <v>46304</v>
       </c>
       <c r="B65" s="12"/>
       <c r="C65" s="21" t="s">
         <v>35</v>
       </c>
       <c r="D65" s="13">
-        <v>258.48</v>
+        <v>258.19</v>
       </c>
       <c r="E65" s="13">
-        <v>241.85</v>
+        <v>243.19</v>
       </c>
       <c r="F65" s="13" t="s">
         <v>18</v>
@@ -1835,35 +1835,35 @@
     </row>
     <row r="66" spans="1:6" x14ac:dyDescent="0.45">
       <c r="A66" s="7">
-        <v>46303</v>
+        <v>46304</v>
       </c>
       <c r="B66" s="8"/>
       <c r="C66" s="20" t="s">
         <v>36</v>
       </c>
       <c r="D66" s="10">
-        <v>254.31</v>
+        <v>254.02</v>
       </c>
       <c r="E66" s="10">
-        <v>237.8</v>
+        <v>239.14</v>
       </c>
       <c r="F66" s="10">
-        <v>247.8</v>
+        <v>249.14</v>
       </c>
     </row>
     <row r="67" spans="1:6" x14ac:dyDescent="0.45">
       <c r="A67" s="11">
-        <v>46303</v>
+        <v>46304</v>
       </c>
       <c r="B67" s="12"/>
       <c r="C67" s="21" t="s">
         <v>37</v>
       </c>
       <c r="D67" s="13">
-        <v>259.13</v>
+        <v>258.29000000000002</v>
       </c>
       <c r="E67" s="13">
-        <v>259.7</v>
+        <v>261.19</v>
       </c>
       <c r="F67" s="13" t="s">
         <v>18</v>
@@ -1891,12 +1891,14 @@
 </file>
 
 <file path=customXml/item1.xml><?xml version="1.0" encoding="utf-8"?>
-<?mso-contentType ?>
-<FormTemplates xmlns="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms">
-  <Display>DocumentLibraryForm</Display>
-  <Edit>DocumentLibraryForm</Edit>
-  <New>DocumentLibraryForm</New>
-</FormTemplates>
+<p:properties xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls">
+  <documentManagement>
+    <lcf76f155ced4ddcb4097134ff3c332f xmlns="87276d81-85f4-4ef2-9e6e-55066304288f">
+      <Terms xmlns="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
+    </lcf76f155ced4ddcb4097134ff3c332f>
+    <TaxCatchAll xmlns="b23b8984-eafa-4e79-985e-54f52f3da58e" xsi:nil="true"/>
+  </documentManagement>
+</p:properties>
 </file>
 
 <file path=customXml/item2.xml><?xml version="1.0" encoding="utf-8"?>
@@ -2160,20 +2162,21 @@
 </file>
 
 <file path=customXml/item3.xml><?xml version="1.0" encoding="utf-8"?>
-<p:properties xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls">
-  <documentManagement>
-    <lcf76f155ced4ddcb4097134ff3c332f xmlns="87276d81-85f4-4ef2-9e6e-55066304288f">
-      <Terms xmlns="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
-    </lcf76f155ced4ddcb4097134ff3c332f>
-    <TaxCatchAll xmlns="b23b8984-eafa-4e79-985e-54f52f3da58e" xsi:nil="true"/>
-  </documentManagement>
-</p:properties>
+<?mso-contentType ?>
+<FormTemplates xmlns="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms">
+  <Display>DocumentLibraryForm</Display>
+  <Edit>DocumentLibraryForm</Edit>
+  <New>DocumentLibraryForm</New>
+</FormTemplates>
 </file>
 
 <file path=customXml/itemProps1.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{F60519E9-FD90-4339-869C-BC2F85719BB8}">
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{57A83D98-2BAE-4D83-823A-D31C464B620C}">
   <ds:schemaRefs>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/properties"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
+    <ds:schemaRef ds:uri="87276d81-85f4-4ef2-9e6e-55066304288f"/>
+    <ds:schemaRef ds:uri="b23b8984-eafa-4e79-985e-54f52f3da58e"/>
   </ds:schemaRefs>
 </ds:datastoreItem>
 </file>
@@ -2199,12 +2202,9 @@
 </file>
 
 <file path=customXml/itemProps3.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{57A83D98-2BAE-4D83-823A-D31C464B620C}">
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{F60519E9-FD90-4339-869C-BC2F85719BB8}">
   <ds:schemaRefs>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/properties"/>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
-    <ds:schemaRef ds:uri="87276d81-85f4-4ef2-9e6e-55066304288f"/>
-    <ds:schemaRef ds:uri="b23b8984-eafa-4e79-985e-54f52f3da58e"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms"/>
   </ds:schemaRefs>
 </ds:datastoreItem>
 </file>

</xml_diff>

<commit_message>
Mon Oct 12 07:29:23 UTC 2026
</commit_message>
<xml_diff>
--- a/bp.com-content-dam-bp-country-sites-en_au-australia-home-products-services-pricing-tgp-excel.xlsx
+++ b/bp.com-content-dam-bp-country-sites-en_au-australia-home-products-services-pricing-tgp-excel.xlsx
@@ -8,14 +8,14 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://bp365.sharepoint.com/sites/WholesalePricing/Shared Documents/B2C/TGP/Daily TGP/Web TGP/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="14_{90B6C5B8-2282-405A-89C3-EDF5CC535555}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="14_{6F758FC0-36DC-4F4A-B733-FAE0F111399F}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="2205" yWindow="2205" windowWidth="11235" windowHeight="9338" xr2:uid="{1B412EEF-F96D-4DF4-A4E9-C7F0F183C2FB}"/>
+    <workbookView xWindow="-98" yWindow="-98" windowWidth="28996" windowHeight="17475" xr2:uid="{1B412EEF-F96D-4DF4-A4E9-C7F0F183C2FB}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
   </sheets>
-  <calcPr calcId="191028"/>
+  <calcPr calcId="191028" concurrentManualCount="20"/>
   <extLst>
     <ext xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" uri="{140A7094-0E35-4892-8432-C4D2E57EDEB5}">
       <x15:workbookPr chartTrackingRefBase="1"/>
@@ -808,128 +808,128 @@
     </row>
     <row r="8" spans="1:7" x14ac:dyDescent="0.45">
       <c r="A8" s="7">
-        <v>46305</v>
+        <v>46308</v>
       </c>
       <c r="B8" s="8"/>
       <c r="C8" s="9" t="s">
         <v>10</v>
       </c>
       <c r="D8" s="10">
-        <v>259.31</v>
+        <v>259.05</v>
       </c>
       <c r="E8" s="10">
-        <v>239.15</v>
+        <v>237.34</v>
       </c>
       <c r="F8" s="10">
-        <v>249.15</v>
+        <v>247.34</v>
       </c>
       <c r="G8" s="10">
-        <v>236.77</v>
+        <v>234.96</v>
       </c>
     </row>
     <row r="9" spans="1:7" x14ac:dyDescent="0.45">
       <c r="A9" s="11">
-        <v>46305</v>
+        <v>46308</v>
       </c>
       <c r="B9" s="12"/>
       <c r="C9" s="12" t="s">
         <v>11</v>
       </c>
       <c r="D9" s="13">
-        <v>259.31</v>
+        <v>259.05</v>
       </c>
       <c r="E9" s="13">
-        <v>239.15</v>
+        <v>237.34</v>
       </c>
       <c r="F9" s="13">
-        <v>249.15</v>
+        <v>247.34</v>
       </c>
       <c r="G9" s="13">
-        <v>236.77</v>
+        <v>234.96</v>
       </c>
     </row>
     <row r="10" spans="1:7" x14ac:dyDescent="0.45">
       <c r="A10" s="7">
-        <v>46305</v>
+        <v>46308</v>
       </c>
       <c r="B10" s="8"/>
       <c r="C10" s="9" t="s">
         <v>12</v>
       </c>
       <c r="D10" s="10">
-        <v>255.41</v>
+        <v>254.69</v>
       </c>
       <c r="E10" s="10">
-        <v>238.27</v>
+        <v>236.04</v>
       </c>
       <c r="F10" s="10">
-        <v>248.27</v>
+        <v>246.04</v>
       </c>
       <c r="G10" s="10">
-        <v>236.68</v>
+        <v>234.45</v>
       </c>
     </row>
     <row r="11" spans="1:7" x14ac:dyDescent="0.45">
       <c r="A11" s="11">
-        <v>46304</v>
+        <v>46305</v>
       </c>
       <c r="B11" s="12"/>
       <c r="C11" s="12" t="s">
         <v>10</v>
       </c>
       <c r="D11" s="13">
-        <v>259.77999999999997</v>
+        <v>259.31</v>
       </c>
       <c r="E11" s="13">
-        <v>237.83</v>
+        <v>239.15</v>
       </c>
       <c r="F11" s="13">
-        <v>247.83</v>
+        <v>249.15</v>
       </c>
       <c r="G11" s="13">
-        <v>235.44</v>
+        <v>236.77</v>
       </c>
     </row>
     <row r="12" spans="1:7" x14ac:dyDescent="0.45">
       <c r="A12" s="7">
-        <v>46304</v>
+        <v>46305</v>
       </c>
       <c r="B12" s="8"/>
       <c r="C12" s="9" t="s">
         <v>11</v>
       </c>
       <c r="D12" s="10">
-        <v>259.77999999999997</v>
+        <v>259.31</v>
       </c>
       <c r="E12" s="10">
-        <v>237.83</v>
+        <v>239.15</v>
       </c>
       <c r="F12" s="10">
-        <v>247.83</v>
+        <v>249.15</v>
       </c>
       <c r="G12" s="10">
-        <v>235.44</v>
+        <v>236.77</v>
       </c>
     </row>
     <row r="13" spans="1:7" x14ac:dyDescent="0.45">
       <c r="A13" s="11">
-        <v>46304</v>
+        <v>46305</v>
       </c>
       <c r="B13" s="12"/>
       <c r="C13" s="12" t="s">
         <v>12</v>
       </c>
       <c r="D13" s="13">
-        <v>255.92</v>
+        <v>255.41</v>
       </c>
       <c r="E13" s="13">
-        <v>238.64</v>
+        <v>238.27</v>
       </c>
       <c r="F13" s="13">
-        <v>248.64</v>
+        <v>248.27</v>
       </c>
       <c r="G13" s="13">
-        <v>237.04</v>
+        <v>236.68</v>
       </c>
     </row>
     <row r="14" spans="1:7" x14ac:dyDescent="0.45">
@@ -973,39 +973,39 @@
     </row>
     <row r="17" spans="1:7" x14ac:dyDescent="0.45">
       <c r="A17" s="7">
-        <v>46305</v>
+        <v>46308</v>
       </c>
       <c r="B17" s="8"/>
       <c r="C17" s="20" t="s">
         <v>14</v>
       </c>
       <c r="D17" s="10">
-        <v>258.75</v>
+        <v>258.08999999999997</v>
       </c>
       <c r="E17" s="10">
-        <v>243.37</v>
+        <v>241.18</v>
       </c>
       <c r="F17" s="10">
-        <v>253.37</v>
+        <v>251.19</v>
       </c>
       <c r="G17" s="17"/>
     </row>
     <row r="18" spans="1:7" x14ac:dyDescent="0.45">
       <c r="A18" s="11">
-        <v>46304</v>
+        <v>46305</v>
       </c>
       <c r="B18" s="12"/>
       <c r="C18" s="12" t="s">
         <v>14</v>
       </c>
       <c r="D18" s="13">
-        <v>259.24</v>
+        <v>258.75</v>
       </c>
       <c r="E18" s="13">
-        <v>243.72</v>
+        <v>243.37</v>
       </c>
       <c r="F18" s="13">
-        <v>253.72</v>
+        <v>253.37</v>
       </c>
       <c r="G18" s="17"/>
     </row>
@@ -1052,41 +1052,41 @@
     </row>
     <row r="22" spans="1:7" x14ac:dyDescent="0.45">
       <c r="A22" s="7">
-        <v>46305</v>
+        <v>46308</v>
       </c>
       <c r="B22" s="8"/>
       <c r="C22" s="20" t="s">
         <v>16</v>
       </c>
       <c r="D22" s="10">
-        <v>260.44</v>
+        <v>260.18</v>
       </c>
       <c r="E22" s="10">
-        <v>238.19</v>
+        <v>238.02</v>
       </c>
       <c r="F22" s="10">
-        <v>247.78</v>
+        <v>247.62</v>
       </c>
       <c r="G22" s="10">
-        <v>234.56</v>
+        <v>234.39</v>
       </c>
     </row>
     <row r="23" spans="1:7" x14ac:dyDescent="0.45">
       <c r="A23" s="11">
-        <v>46305</v>
+        <v>46308</v>
       </c>
       <c r="B23" s="12"/>
       <c r="C23" s="21" t="s">
         <v>17</v>
       </c>
       <c r="D23" s="13">
-        <v>260.38</v>
+        <v>259.64999999999998</v>
       </c>
       <c r="E23" s="13">
-        <v>248.82</v>
+        <v>246.57</v>
       </c>
       <c r="F23" s="13">
-        <v>258.82</v>
+        <v>256.57</v>
       </c>
       <c r="G23" s="13" t="s">
         <v>18</v>
@@ -1094,20 +1094,20 @@
     </row>
     <row r="24" spans="1:7" x14ac:dyDescent="0.45">
       <c r="A24" s="7">
-        <v>46305</v>
+        <v>46308</v>
       </c>
       <c r="B24" s="8"/>
       <c r="C24" s="20" t="s">
         <v>19</v>
       </c>
       <c r="D24" s="10">
-        <v>260.72000000000003</v>
+        <v>259.99</v>
       </c>
       <c r="E24" s="10">
-        <v>248.05</v>
+        <v>245.8</v>
       </c>
       <c r="F24" s="10">
-        <v>258.05</v>
+        <v>255.8</v>
       </c>
       <c r="G24" s="10" t="s">
         <v>18</v>
@@ -1115,41 +1115,41 @@
     </row>
     <row r="25" spans="1:7" x14ac:dyDescent="0.45">
       <c r="A25" s="11">
-        <v>46305</v>
+        <v>46308</v>
       </c>
       <c r="B25" s="12"/>
       <c r="C25" s="21" t="s">
         <v>20</v>
       </c>
       <c r="D25" s="13">
-        <v>257.37</v>
+        <v>256.66000000000003</v>
       </c>
       <c r="E25" s="13">
-        <v>248.31</v>
+        <v>246.05</v>
       </c>
       <c r="F25" s="13">
-        <v>258.31</v>
+        <v>256.05</v>
       </c>
       <c r="G25" s="13">
-        <v>244.15</v>
+        <v>241.89</v>
       </c>
     </row>
     <row r="26" spans="1:7" x14ac:dyDescent="0.45">
       <c r="A26" s="7">
-        <v>46305</v>
+        <v>46308</v>
       </c>
       <c r="B26" s="8"/>
       <c r="C26" s="20" t="s">
         <v>21</v>
       </c>
       <c r="D26" s="10">
-        <v>258.89</v>
+        <v>258.18</v>
       </c>
       <c r="E26" s="10">
-        <v>249.87</v>
+        <v>247.59</v>
       </c>
       <c r="F26" s="10">
-        <v>259.87</v>
+        <v>257.58999999999997</v>
       </c>
       <c r="G26" s="10" t="s">
         <v>18</v>
@@ -1157,41 +1157,41 @@
     </row>
     <row r="27" spans="1:7" x14ac:dyDescent="0.45">
       <c r="A27" s="11">
-        <v>46304</v>
+        <v>46305</v>
       </c>
       <c r="B27" s="12"/>
       <c r="C27" s="12" t="s">
         <v>16</v>
       </c>
       <c r="D27" s="13">
-        <v>260.89999999999998</v>
+        <v>260.44</v>
       </c>
       <c r="E27" s="13">
-        <v>237.41</v>
+        <v>238.19</v>
       </c>
       <c r="F27" s="13">
-        <v>247.01</v>
+        <v>247.78</v>
       </c>
       <c r="G27" s="13">
-        <v>233.78</v>
+        <v>234.56</v>
       </c>
     </row>
     <row r="28" spans="1:7" x14ac:dyDescent="0.45">
       <c r="A28" s="7">
-        <v>46304</v>
+        <v>46305</v>
       </c>
       <c r="B28" s="8"/>
       <c r="C28" s="20" t="s">
         <v>17</v>
       </c>
       <c r="D28" s="10">
-        <v>260.89</v>
+        <v>260.38</v>
       </c>
       <c r="E28" s="22">
-        <v>249.2</v>
+        <v>248.82</v>
       </c>
       <c r="F28" s="22">
-        <v>259.2</v>
+        <v>258.82</v>
       </c>
       <c r="G28" s="22" t="s">
         <v>18</v>
@@ -1199,20 +1199,20 @@
     </row>
     <row r="29" spans="1:7" x14ac:dyDescent="0.45">
       <c r="A29" s="11">
-        <v>46304</v>
+        <v>46305</v>
       </c>
       <c r="B29" s="12"/>
       <c r="C29" s="12" t="s">
         <v>19</v>
       </c>
       <c r="D29" s="13">
-        <v>261.22000000000003</v>
+        <v>260.72000000000003</v>
       </c>
       <c r="E29" s="13">
-        <v>248.42</v>
+        <v>248.05</v>
       </c>
       <c r="F29" s="13">
-        <v>258.42</v>
+        <v>258.05</v>
       </c>
       <c r="G29" s="13" t="s">
         <v>18</v>
@@ -1220,41 +1220,41 @@
     </row>
     <row r="30" spans="1:7" x14ac:dyDescent="0.45">
       <c r="A30" s="7">
-        <v>46304</v>
+        <v>46305</v>
       </c>
       <c r="B30" s="8"/>
       <c r="C30" s="20" t="s">
         <v>20</v>
       </c>
       <c r="D30" s="10">
-        <v>257.88</v>
+        <v>257.37</v>
       </c>
       <c r="E30" s="22">
-        <v>248.68</v>
+        <v>248.31</v>
       </c>
       <c r="F30" s="22">
-        <v>258.68</v>
+        <v>258.31</v>
       </c>
       <c r="G30" s="22">
-        <v>244.52</v>
+        <v>244.15</v>
       </c>
     </row>
     <row r="31" spans="1:7" x14ac:dyDescent="0.45">
       <c r="A31" s="11">
-        <v>46304</v>
+        <v>46305</v>
       </c>
       <c r="B31" s="12"/>
       <c r="C31" s="12" t="s">
         <v>21</v>
       </c>
       <c r="D31" s="13">
-        <v>259.39999999999998</v>
+        <v>258.89</v>
       </c>
       <c r="E31" s="13">
-        <v>250.25</v>
+        <v>249.87</v>
       </c>
       <c r="F31" s="13">
-        <v>260.25</v>
+        <v>259.87</v>
       </c>
       <c r="G31" s="13" t="s">
         <v>18</v>
@@ -1301,52 +1301,52 @@
     </row>
     <row r="35" spans="1:7" x14ac:dyDescent="0.45">
       <c r="A35" s="7">
-        <v>46305</v>
+        <v>46308</v>
       </c>
       <c r="B35" s="8"/>
       <c r="C35" s="20" t="s">
         <v>23</v>
       </c>
       <c r="D35" s="10">
-        <v>253.96</v>
+        <v>253.24</v>
       </c>
       <c r="E35" s="10">
-        <v>234.45</v>
+        <v>233.87</v>
       </c>
       <c r="F35" s="10">
-        <v>243.45</v>
+        <v>242.87</v>
       </c>
       <c r="G35" s="17"/>
     </row>
     <row r="36" spans="1:7" x14ac:dyDescent="0.45">
       <c r="A36" s="11">
-        <v>46304</v>
+        <v>46305</v>
       </c>
       <c r="B36" s="12"/>
       <c r="C36" s="12" t="s">
         <v>23</v>
       </c>
       <c r="D36" s="13">
-        <v>254.47</v>
+        <v>253.96</v>
       </c>
       <c r="E36" s="13">
-        <v>234.26</v>
+        <v>234.45</v>
       </c>
       <c r="F36" s="13">
-        <v>243.27</v>
+        <v>243.45</v>
       </c>
       <c r="G36" s="17"/>
     </row>
     <row r="37" spans="1:7" x14ac:dyDescent="0.45">
       <c r="A37" s="7">
-        <v>46305</v>
+        <v>46308</v>
       </c>
       <c r="B37" s="8"/>
       <c r="C37" s="20" t="s">
         <v>24</v>
       </c>
       <c r="D37" s="10">
-        <v>269.58</v>
+        <v>268.86</v>
       </c>
       <c r="E37" s="10" t="s">
         <v>18</v>
@@ -1358,14 +1358,14 @@
     </row>
     <row r="38" spans="1:7" x14ac:dyDescent="0.45">
       <c r="A38" s="11">
-        <v>46304</v>
+        <v>46305</v>
       </c>
       <c r="B38" s="12"/>
       <c r="C38" s="12" t="s">
         <v>24</v>
       </c>
       <c r="D38" s="13">
-        <v>270.08999999999997</v>
+        <v>269.58</v>
       </c>
       <c r="E38" s="13" t="s">
         <v>18</v>
@@ -1416,77 +1416,77 @@
     </row>
     <row r="42" spans="1:7" x14ac:dyDescent="0.45">
       <c r="A42" s="7">
-        <v>46305</v>
+        <v>46308</v>
       </c>
       <c r="B42" s="8"/>
       <c r="C42" s="20" t="s">
         <v>26</v>
       </c>
       <c r="D42" s="10">
-        <v>264.06</v>
+        <v>263.3</v>
       </c>
       <c r="E42" s="10">
-        <v>245.34</v>
+        <v>243.64</v>
       </c>
       <c r="F42" s="10">
-        <v>255.34</v>
+        <v>253.64</v>
       </c>
       <c r="G42" s="17"/>
     </row>
     <row r="43" spans="1:7" x14ac:dyDescent="0.45">
       <c r="A43" s="11">
-        <v>46305</v>
+        <v>46308</v>
       </c>
       <c r="B43" s="12"/>
       <c r="C43" s="21" t="s">
         <v>27</v>
       </c>
       <c r="D43" s="13">
-        <v>263.68</v>
+        <v>262.91000000000003</v>
       </c>
       <c r="E43" s="13">
-        <v>245.75</v>
+        <v>244.05</v>
       </c>
       <c r="F43" s="13">
-        <v>255.75</v>
+        <v>254.05</v>
       </c>
       <c r="G43" s="17"/>
     </row>
     <row r="44" spans="1:7" x14ac:dyDescent="0.45">
       <c r="A44" s="7">
-        <v>46304</v>
+        <v>46305</v>
       </c>
       <c r="B44" s="8"/>
       <c r="C44" s="20" t="s">
         <v>26</v>
       </c>
       <c r="D44" s="10">
-        <v>264.58999999999997</v>
+        <v>264.06</v>
       </c>
       <c r="E44" s="10">
-        <v>245.55</v>
+        <v>245.34</v>
       </c>
       <c r="F44" s="10">
-        <v>255.55</v>
+        <v>255.34</v>
       </c>
       <c r="G44" s="17"/>
     </row>
     <row r="45" spans="1:7" x14ac:dyDescent="0.45">
       <c r="A45" s="11">
-        <v>46304</v>
+        <v>46305</v>
       </c>
       <c r="B45" s="12"/>
       <c r="C45" s="21" t="s">
         <v>27</v>
       </c>
       <c r="D45" s="13">
-        <v>264.2</v>
+        <v>263.68</v>
       </c>
       <c r="E45" s="13">
-        <v>245.96</v>
+        <v>245.75</v>
       </c>
       <c r="F45" s="13">
-        <v>255.96</v>
+        <v>255.75</v>
       </c>
       <c r="G45" s="17"/>
     </row>
@@ -1531,77 +1531,77 @@
     </row>
     <row r="49" spans="1:7" x14ac:dyDescent="0.45">
       <c r="A49" s="7">
-        <v>46305</v>
+        <v>46308</v>
       </c>
       <c r="B49" s="8"/>
       <c r="C49" s="20" t="s">
         <v>29</v>
       </c>
       <c r="D49" s="10">
-        <v>258.29000000000002</v>
+        <v>257.98</v>
       </c>
       <c r="E49" s="10">
-        <v>240.22</v>
+        <v>240.01</v>
       </c>
       <c r="F49" s="10">
-        <v>250.22</v>
+        <v>250.01</v>
       </c>
       <c r="G49" s="28"/>
     </row>
     <row r="50" spans="1:7" x14ac:dyDescent="0.45">
       <c r="A50" s="11">
-        <v>46305</v>
+        <v>46308</v>
       </c>
       <c r="B50" s="12"/>
       <c r="C50" s="21" t="s">
         <v>30</v>
       </c>
       <c r="D50" s="13">
-        <v>255.79</v>
+        <v>255.47</v>
       </c>
       <c r="E50" s="13">
-        <v>239.84</v>
+        <v>239.62</v>
       </c>
       <c r="F50" s="13">
-        <v>249.84</v>
+        <v>249.62</v>
       </c>
       <c r="G50" s="28"/>
     </row>
     <row r="51" spans="1:7" x14ac:dyDescent="0.45">
       <c r="A51" s="7">
-        <v>46304</v>
+        <v>46305</v>
       </c>
       <c r="B51" s="8"/>
       <c r="C51" s="20" t="s">
         <v>29</v>
       </c>
       <c r="D51" s="10">
-        <v>257</v>
+        <v>258.29000000000002</v>
       </c>
       <c r="E51" s="10">
-        <v>238.67</v>
+        <v>240.22</v>
       </c>
       <c r="F51" s="10">
-        <v>248.67</v>
+        <v>250.22</v>
       </c>
       <c r="G51" s="17"/>
     </row>
     <row r="52" spans="1:7" x14ac:dyDescent="0.45">
       <c r="A52" s="11">
-        <v>46304</v>
+        <v>46305</v>
       </c>
       <c r="B52" s="12"/>
       <c r="C52" s="21" t="s">
         <v>30</v>
       </c>
       <c r="D52" s="13">
-        <v>254.51</v>
+        <v>255.79</v>
       </c>
       <c r="E52" s="13">
-        <v>238.29</v>
+        <v>239.84</v>
       </c>
       <c r="F52" s="13">
-        <v>248.29</v>
+        <v>249.84</v>
       </c>
       <c r="G52" s="17"/>
     </row>
@@ -1646,52 +1646,52 @@
     </row>
     <row r="56" spans="1:7" x14ac:dyDescent="0.45">
       <c r="A56" s="7">
-        <v>46305</v>
+        <v>46308</v>
       </c>
       <c r="B56" s="8"/>
       <c r="C56" s="20" t="s">
         <v>32</v>
       </c>
       <c r="D56" s="10">
-        <v>270.06</v>
+        <v>269.35000000000002</v>
       </c>
       <c r="E56" s="10">
-        <v>267.62</v>
+        <v>265.16000000000003</v>
       </c>
       <c r="F56" s="10">
-        <v>277.62</v>
+        <v>275.16000000000003</v>
       </c>
       <c r="G56" s="17"/>
     </row>
     <row r="57" spans="1:7" x14ac:dyDescent="0.45">
       <c r="A57" s="11">
-        <v>46305</v>
+        <v>46308</v>
       </c>
       <c r="B57" s="12"/>
       <c r="C57" s="21" t="s">
         <v>33</v>
       </c>
       <c r="D57" s="13">
-        <v>260.05</v>
+        <v>259.32</v>
       </c>
       <c r="E57" s="13">
-        <v>248.47</v>
+        <v>246.32</v>
       </c>
       <c r="F57" s="13">
-        <v>258.47000000000003</v>
+        <v>256.32</v>
       </c>
       <c r="G57" s="17"/>
     </row>
     <row r="58" spans="1:7" x14ac:dyDescent="0.45">
       <c r="A58" s="7">
-        <v>46305</v>
+        <v>46308</v>
       </c>
       <c r="B58" s="8"/>
       <c r="C58" s="20" t="s">
         <v>34</v>
       </c>
       <c r="D58" s="10">
-        <v>260.95</v>
+        <v>260.20999999999998</v>
       </c>
       <c r="E58" s="10" t="s">
         <v>18</v>
@@ -1703,17 +1703,17 @@
     </row>
     <row r="59" spans="1:7" x14ac:dyDescent="0.45">
       <c r="A59" s="11">
-        <v>46305</v>
+        <v>46308</v>
       </c>
       <c r="B59" s="12"/>
       <c r="C59" s="21" t="s">
         <v>35</v>
       </c>
       <c r="D59" s="13">
-        <v>257.70999999999998</v>
+        <v>256.51</v>
       </c>
       <c r="E59" s="13">
-        <v>242.84</v>
+        <v>240.69</v>
       </c>
       <c r="F59" s="13" t="s">
         <v>18</v>
@@ -1722,36 +1722,36 @@
     </row>
     <row r="60" spans="1:7" x14ac:dyDescent="0.45">
       <c r="A60" s="7">
-        <v>46305</v>
+        <v>46308</v>
       </c>
       <c r="B60" s="8"/>
       <c r="C60" s="20" t="s">
         <v>36</v>
       </c>
       <c r="D60" s="10">
-        <v>253.53</v>
+        <v>252.34</v>
       </c>
       <c r="E60" s="10">
-        <v>238.79</v>
+        <v>236.64</v>
       </c>
       <c r="F60" s="10">
-        <v>248.79</v>
+        <v>246.64</v>
       </c>
       <c r="G60" s="17"/>
     </row>
     <row r="61" spans="1:7" x14ac:dyDescent="0.45">
       <c r="A61" s="11">
-        <v>46305</v>
+        <v>46308</v>
       </c>
       <c r="B61" s="12"/>
       <c r="C61" s="21" t="s">
         <v>37</v>
       </c>
       <c r="D61" s="13">
-        <v>257.81</v>
+        <v>257.17</v>
       </c>
       <c r="E61" s="13">
-        <v>260.77999999999997</v>
+        <v>258.42</v>
       </c>
       <c r="F61" s="13" t="s">
         <v>18</v>
@@ -1760,52 +1760,52 @@
     </row>
     <row r="62" spans="1:7" x14ac:dyDescent="0.45">
       <c r="A62" s="7">
-        <v>46304</v>
+        <v>46305</v>
       </c>
       <c r="B62" s="8"/>
       <c r="C62" s="20" t="s">
         <v>32</v>
       </c>
       <c r="D62" s="10">
-        <v>271.11</v>
+        <v>270.06</v>
       </c>
       <c r="E62" s="10">
-        <v>268.07</v>
+        <v>267.62</v>
       </c>
       <c r="F62" s="10">
-        <v>278.07</v>
+        <v>277.62</v>
       </c>
       <c r="G62" s="17"/>
     </row>
     <row r="63" spans="1:7" x14ac:dyDescent="0.45">
       <c r="A63" s="11">
-        <v>46304</v>
+        <v>46305</v>
       </c>
       <c r="B63" s="12"/>
       <c r="C63" s="21" t="s">
         <v>33</v>
       </c>
       <c r="D63" s="13">
-        <v>260.56</v>
+        <v>260.05</v>
       </c>
       <c r="E63" s="13">
-        <v>248.82</v>
+        <v>248.47</v>
       </c>
       <c r="F63" s="13">
-        <v>258.82</v>
+        <v>258.47000000000003</v>
       </c>
       <c r="G63" s="17"/>
     </row>
     <row r="64" spans="1:7" x14ac:dyDescent="0.45">
       <c r="A64" s="7">
-        <v>46304</v>
+        <v>46305</v>
       </c>
       <c r="B64" s="8"/>
       <c r="C64" s="20" t="s">
         <v>34</v>
       </c>
       <c r="D64" s="10">
-        <v>262.01</v>
+        <v>260.95</v>
       </c>
       <c r="E64" s="10" t="s">
         <v>18</v>
@@ -1817,17 +1817,17 @@
     </row>
     <row r="65" spans="1:6" x14ac:dyDescent="0.45">
       <c r="A65" s="11">
-        <v>46304</v>
+        <v>46305</v>
       </c>
       <c r="B65" s="12"/>
       <c r="C65" s="21" t="s">
         <v>35</v>
       </c>
       <c r="D65" s="13">
-        <v>258.19</v>
+        <v>257.70999999999998</v>
       </c>
       <c r="E65" s="13">
-        <v>243.19</v>
+        <v>242.84</v>
       </c>
       <c r="F65" s="13" t="s">
         <v>18</v>
@@ -1835,35 +1835,35 @@
     </row>
     <row r="66" spans="1:6" x14ac:dyDescent="0.45">
       <c r="A66" s="7">
-        <v>46304</v>
+        <v>46305</v>
       </c>
       <c r="B66" s="8"/>
       <c r="C66" s="20" t="s">
         <v>36</v>
       </c>
       <c r="D66" s="10">
-        <v>254.02</v>
+        <v>253.53</v>
       </c>
       <c r="E66" s="10">
-        <v>239.14</v>
+        <v>238.79</v>
       </c>
       <c r="F66" s="10">
-        <v>249.14</v>
+        <v>248.79</v>
       </c>
     </row>
     <row r="67" spans="1:6" x14ac:dyDescent="0.45">
       <c r="A67" s="11">
-        <v>46304</v>
+        <v>46305</v>
       </c>
       <c r="B67" s="12"/>
       <c r="C67" s="21" t="s">
         <v>37</v>
       </c>
       <c r="D67" s="13">
-        <v>258.29000000000002</v>
+        <v>257.81</v>
       </c>
       <c r="E67" s="13">
-        <v>261.19</v>
+        <v>260.77999999999997</v>
       </c>
       <c r="F67" s="13" t="s">
         <v>18</v>
@@ -1902,6 +1902,15 @@
 </file>
 
 <file path=customXml/item2.xml><?xml version="1.0" encoding="utf-8"?>
+<?mso-contentType ?>
+<FormTemplates xmlns="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms">
+  <Display>DocumentLibraryForm</Display>
+  <Edit>DocumentLibraryForm</Edit>
+  <New>DocumentLibraryForm</New>
+</FormTemplates>
+</file>
+
+<file path=customXml/item3.xml><?xml version="1.0" encoding="utf-8"?>
 <ct:contentTypeSchema xmlns:ct="http://schemas.microsoft.com/office/2006/metadata/contentType" xmlns:ma="http://schemas.microsoft.com/office/2006/metadata/properties/metaAttributes" ct:_="" ma:_="" ma:contentTypeName="Document" ma:contentTypeID="0x010100D3632DF5622958439304627C030B0427" ma:contentTypeVersion="18" ma:contentTypeDescription="Create a new document." ma:contentTypeScope="" ma:versionID="8c2ecbce386d6bac497f8eb2d8f0fb7a">
   <xsd:schema xmlns:xsd="http://www.w3.org/2001/XMLSchema" xmlns:xs="http://www.w3.org/2001/XMLSchema" xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:ns2="87276d81-85f4-4ef2-9e6e-55066304288f" xmlns:ns3="39e1dda6-d1d8-4c88-a3b9-f1abc1284bad" xmlns:ns4="b23b8984-eafa-4e79-985e-54f52f3da58e" targetNamespace="http://schemas.microsoft.com/office/2006/metadata/properties" ma:root="true" ma:fieldsID="4cfd0c2f651c1ce156ad4fcb44ea61dd" ns2:_="" ns3:_="" ns4:_="">
     <xsd:import namespace="87276d81-85f4-4ef2-9e6e-55066304288f"/>
@@ -2161,15 +2170,6 @@
 </ct:contentTypeSchema>
 </file>
 
-<file path=customXml/item3.xml><?xml version="1.0" encoding="utf-8"?>
-<?mso-contentType ?>
-<FormTemplates xmlns="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms">
-  <Display>DocumentLibraryForm</Display>
-  <Edit>DocumentLibraryForm</Edit>
-  <New>DocumentLibraryForm</New>
-</FormTemplates>
-</file>
-
 <file path=customXml/itemProps1.xml><?xml version="1.0" encoding="utf-8"?>
 <ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{57A83D98-2BAE-4D83-823A-D31C464B620C}">
   <ds:schemaRefs>
@@ -2182,6 +2182,14 @@
 </file>
 
 <file path=customXml/itemProps2.xml><?xml version="1.0" encoding="utf-8"?>
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{F60519E9-FD90-4339-869C-BC2F85719BB8}">
+  <ds:schemaRefs>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms"/>
+  </ds:schemaRefs>
+</ds:datastoreItem>
+</file>
+
+<file path=customXml/itemProps3.xml><?xml version="1.0" encoding="utf-8"?>
 <ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{B44E1863-2778-41F9-ACBA-48420F931671}">
   <ds:schemaRefs>
     <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/contentType"/>
@@ -2201,14 +2209,6 @@
 </ds:datastoreItem>
 </file>
 
-<file path=customXml/itemProps3.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{F60519E9-FD90-4339-869C-BC2F85719BB8}">
-  <ds:schemaRefs>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms"/>
-  </ds:schemaRefs>
-</ds:datastoreItem>
-</file>
-
 <file path=docMetadata/LabelInfo.xml><?xml version="1.0" encoding="utf-8"?>
 <clbl:labelList xmlns:clbl="http://schemas.microsoft.com/office/2020/mipLabelMetadata">
   <clbl:label id="{569bf4a9-87bd-4dbf-a36c-1db5158e5def}" enabled="1" method="Privileged" siteId="{ea80952e-a476-42d4-aaf4-5457852b0f7e}" removed="0"/>

</xml_diff>

<commit_message>
Tue Oct 13 07:50:22 UTC 2026
</commit_message>
<xml_diff>
--- a/bp.com-content-dam-bp-country-sites-en_au-australia-home-products-services-pricing-tgp-excel.xlsx
+++ b/bp.com-content-dam-bp-country-sites-en_au-australia-home-products-services-pricing-tgp-excel.xlsx
@@ -8,14 +8,14 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://bp365.sharepoint.com/sites/WholesalePricing/Shared Documents/B2C/TGP/Daily TGP/Web TGP/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="14_{6F758FC0-36DC-4F4A-B733-FAE0F111399F}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="14_{CBB2D331-E0D6-490A-A19D-DB494B4EC0C0}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-98" yWindow="-98" windowWidth="28996" windowHeight="17475" xr2:uid="{1B412EEF-F96D-4DF4-A4E9-C7F0F183C2FB}"/>
+    <workbookView xWindow="-28920" yWindow="-60" windowWidth="29040" windowHeight="15720" xr2:uid="{1B412EEF-F96D-4DF4-A4E9-C7F0F183C2FB}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
   </sheets>
-  <calcPr calcId="191028" concurrentManualCount="20"/>
+  <calcPr calcId="191028"/>
   <extLst>
     <ext xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" uri="{140A7094-0E35-4892-8432-C4D2E57EDEB5}">
       <x15:workbookPr chartTrackingRefBase="1"/>
@@ -715,15 +715,15 @@
     <pageSetUpPr fitToPage="1"/>
   </sheetPr>
   <dimension ref="A1:G67"/>
-  <sheetFormatPr defaultRowHeight="14.25" x14ac:dyDescent="0.45"/>
+  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
-    <col min="1" max="1" width="76.3984375" bestFit="1" customWidth="1"/>
-    <col min="2" max="2" width="6.3984375"/>
-    <col min="3" max="3" width="18.1328125" bestFit="1" customWidth="1"/>
-    <col min="4" max="7" width="7.1328125" bestFit="1" customWidth="1"/>
+    <col min="1" max="1" width="76.42578125" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="6.42578125"/>
+    <col min="3" max="3" width="18.140625" bestFit="1" customWidth="1"/>
+    <col min="4" max="7" width="7.140625" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:7" ht="22.15" x14ac:dyDescent="0.45">
+    <row r="1" spans="1:7" ht="23.25" x14ac:dyDescent="0.25">
       <c r="A1" s="30" t="s">
         <v>0</v>
       </c>
@@ -734,7 +734,7 @@
       <c r="F1" s="2"/>
       <c r="G1" s="2"/>
     </row>
-    <row r="2" spans="1:7" x14ac:dyDescent="0.45">
+    <row r="2" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A2" s="3"/>
       <c r="B2" s="1"/>
       <c r="C2" s="1"/>
@@ -743,7 +743,7 @@
       <c r="F2" s="2"/>
       <c r="G2" s="2"/>
     </row>
-    <row r="3" spans="1:7" x14ac:dyDescent="0.45">
+    <row r="3" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A3" s="3" t="s">
         <v>1</v>
       </c>
@@ -754,7 +754,7 @@
       <c r="F3" s="2"/>
       <c r="G3" s="2"/>
     </row>
-    <row r="4" spans="1:7" x14ac:dyDescent="0.45">
+    <row r="4" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A4" s="3" t="s">
         <v>2</v>
       </c>
@@ -765,7 +765,7 @@
       <c r="F4" s="2"/>
       <c r="G4" s="2"/>
     </row>
-    <row r="5" spans="1:7" x14ac:dyDescent="0.45">
+    <row r="5" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A5" s="3"/>
       <c r="B5" s="3"/>
       <c r="C5" s="1"/>
@@ -774,7 +774,7 @@
       <c r="F5" s="2"/>
       <c r="G5" s="2"/>
     </row>
-    <row r="6" spans="1:7" ht="20.25" x14ac:dyDescent="0.45">
+    <row r="6" spans="1:7" ht="20.25" x14ac:dyDescent="0.25">
       <c r="A6" s="29" t="s">
         <v>3</v>
       </c>
@@ -785,7 +785,7 @@
       <c r="F6" s="2"/>
       <c r="G6" s="2"/>
     </row>
-    <row r="7" spans="1:7" x14ac:dyDescent="0.45">
+    <row r="7" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A7" s="4" t="s">
         <v>4</v>
       </c>
@@ -806,133 +806,133 @@
         <v>9</v>
       </c>
     </row>
-    <row r="8" spans="1:7" x14ac:dyDescent="0.45">
+    <row r="8" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A8" s="7">
-        <v>46308</v>
+        <v>46309</v>
       </c>
       <c r="B8" s="8"/>
       <c r="C8" s="9" t="s">
         <v>10</v>
       </c>
       <c r="D8" s="10">
-        <v>259.05</v>
+        <v>258.49</v>
       </c>
       <c r="E8" s="10">
-        <v>237.34</v>
+        <v>236.44</v>
       </c>
       <c r="F8" s="10">
-        <v>247.34</v>
+        <v>246.44</v>
       </c>
       <c r="G8" s="10">
-        <v>234.96</v>
-      </c>
-    </row>
-    <row r="9" spans="1:7" x14ac:dyDescent="0.45">
+        <v>234.05</v>
+      </c>
+    </row>
+    <row r="9" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A9" s="11">
-        <v>46308</v>
+        <v>46309</v>
       </c>
       <c r="B9" s="12"/>
       <c r="C9" s="12" t="s">
         <v>11</v>
       </c>
       <c r="D9" s="13">
-        <v>259.05</v>
+        <v>258.49</v>
       </c>
       <c r="E9" s="13">
-        <v>237.34</v>
+        <v>236.44</v>
       </c>
       <c r="F9" s="13">
-        <v>247.34</v>
+        <v>246.44</v>
       </c>
       <c r="G9" s="13">
-        <v>234.96</v>
-      </c>
-    </row>
-    <row r="10" spans="1:7" x14ac:dyDescent="0.45">
+        <v>234.05</v>
+      </c>
+    </row>
+    <row r="10" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A10" s="7">
-        <v>46308</v>
+        <v>46309</v>
       </c>
       <c r="B10" s="8"/>
       <c r="C10" s="9" t="s">
         <v>12</v>
       </c>
       <c r="D10" s="10">
-        <v>254.69</v>
+        <v>254.19</v>
       </c>
       <c r="E10" s="10">
-        <v>236.04</v>
+        <v>234.71</v>
       </c>
       <c r="F10" s="10">
-        <v>246.04</v>
+        <v>244.71</v>
       </c>
       <c r="G10" s="10">
-        <v>234.45</v>
-      </c>
-    </row>
-    <row r="11" spans="1:7" x14ac:dyDescent="0.45">
+        <v>233.11</v>
+      </c>
+    </row>
+    <row r="11" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A11" s="11">
-        <v>46305</v>
+        <v>46308</v>
       </c>
       <c r="B11" s="12"/>
       <c r="C11" s="12" t="s">
         <v>10</v>
       </c>
       <c r="D11" s="13">
-        <v>259.31</v>
+        <v>259.05</v>
       </c>
       <c r="E11" s="13">
-        <v>239.15</v>
+        <v>237.34</v>
       </c>
       <c r="F11" s="13">
-        <v>249.15</v>
+        <v>247.34</v>
       </c>
       <c r="G11" s="13">
-        <v>236.77</v>
-      </c>
-    </row>
-    <row r="12" spans="1:7" x14ac:dyDescent="0.45">
+        <v>234.96</v>
+      </c>
+    </row>
+    <row r="12" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A12" s="7">
-        <v>46305</v>
+        <v>46308</v>
       </c>
       <c r="B12" s="8"/>
       <c r="C12" s="9" t="s">
         <v>11</v>
       </c>
       <c r="D12" s="10">
-        <v>259.31</v>
+        <v>259.05</v>
       </c>
       <c r="E12" s="10">
-        <v>239.15</v>
+        <v>237.34</v>
       </c>
       <c r="F12" s="10">
-        <v>249.15</v>
+        <v>247.34</v>
       </c>
       <c r="G12" s="10">
-        <v>236.77</v>
-      </c>
-    </row>
-    <row r="13" spans="1:7" x14ac:dyDescent="0.45">
+        <v>234.96</v>
+      </c>
+    </row>
+    <row r="13" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A13" s="11">
-        <v>46305</v>
+        <v>46308</v>
       </c>
       <c r="B13" s="12"/>
       <c r="C13" s="12" t="s">
         <v>12</v>
       </c>
       <c r="D13" s="13">
-        <v>255.41</v>
+        <v>254.69</v>
       </c>
       <c r="E13" s="13">
-        <v>238.27</v>
+        <v>236.04</v>
       </c>
       <c r="F13" s="13">
-        <v>248.27</v>
+        <v>246.04</v>
       </c>
       <c r="G13" s="13">
-        <v>236.68</v>
-      </c>
-    </row>
-    <row r="14" spans="1:7" x14ac:dyDescent="0.45">
+        <v>234.45</v>
+      </c>
+    </row>
+    <row r="14" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A14" s="14"/>
       <c r="B14" s="14"/>
       <c r="C14" s="15"/>
@@ -941,7 +941,7 @@
       <c r="F14" s="16"/>
       <c r="G14" s="16"/>
     </row>
-    <row r="15" spans="1:7" ht="20.25" x14ac:dyDescent="0.45">
+    <row r="15" spans="1:7" ht="20.25" x14ac:dyDescent="0.25">
       <c r="A15" s="29" t="s">
         <v>13</v>
       </c>
@@ -952,7 +952,7 @@
       <c r="F15" s="17"/>
       <c r="G15" s="17"/>
     </row>
-    <row r="16" spans="1:7" x14ac:dyDescent="0.45">
+    <row r="16" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A16" s="4" t="s">
         <v>4</v>
       </c>
@@ -971,45 +971,45 @@
       </c>
       <c r="G16" s="17"/>
     </row>
-    <row r="17" spans="1:7" x14ac:dyDescent="0.45">
+    <row r="17" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A17" s="7">
-        <v>46308</v>
+        <v>46309</v>
       </c>
       <c r="B17" s="8"/>
       <c r="C17" s="20" t="s">
         <v>14</v>
       </c>
       <c r="D17" s="10">
-        <v>258.08999999999997</v>
+        <v>257.64</v>
       </c>
       <c r="E17" s="10">
-        <v>241.18</v>
+        <v>239.88</v>
       </c>
       <c r="F17" s="10">
-        <v>251.19</v>
+        <v>249.88</v>
       </c>
       <c r="G17" s="17"/>
     </row>
-    <row r="18" spans="1:7" x14ac:dyDescent="0.45">
+    <row r="18" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A18" s="11">
-        <v>46305</v>
+        <v>46308</v>
       </c>
       <c r="B18" s="12"/>
       <c r="C18" s="12" t="s">
         <v>14</v>
       </c>
       <c r="D18" s="13">
-        <v>258.75</v>
+        <v>258.08999999999997</v>
       </c>
       <c r="E18" s="13">
-        <v>243.37</v>
+        <v>241.18</v>
       </c>
       <c r="F18" s="13">
-        <v>253.37</v>
+        <v>251.19</v>
       </c>
       <c r="G18" s="17"/>
     </row>
-    <row r="19" spans="1:7" x14ac:dyDescent="0.45">
+    <row r="19" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A19" s="14"/>
       <c r="B19" s="14"/>
       <c r="C19" s="15"/>
@@ -1018,7 +1018,7 @@
       <c r="F19" s="16"/>
       <c r="G19" s="17"/>
     </row>
-    <row r="20" spans="1:7" ht="20.25" x14ac:dyDescent="0.45">
+    <row r="20" spans="1:7" ht="20.25" x14ac:dyDescent="0.25">
       <c r="A20" s="29" t="s">
         <v>15</v>
       </c>
@@ -1029,7 +1029,7 @@
       <c r="F20" s="17"/>
       <c r="G20" s="17"/>
     </row>
-    <row r="21" spans="1:7" x14ac:dyDescent="0.45">
+    <row r="21" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A21" s="4" t="s">
         <v>4</v>
       </c>
@@ -1050,217 +1050,217 @@
         <v>9</v>
       </c>
     </row>
-    <row r="22" spans="1:7" x14ac:dyDescent="0.45">
+    <row r="22" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A22" s="7">
-        <v>46308</v>
+        <v>46309</v>
       </c>
       <c r="B22" s="8"/>
       <c r="C22" s="20" t="s">
         <v>16</v>
       </c>
       <c r="D22" s="10">
-        <v>260.18</v>
+        <v>259.62</v>
       </c>
       <c r="E22" s="10">
-        <v>238.02</v>
+        <v>237.12</v>
       </c>
       <c r="F22" s="10">
-        <v>247.62</v>
+        <v>246.72</v>
       </c>
       <c r="G22" s="10">
-        <v>234.39</v>
-      </c>
-    </row>
-    <row r="23" spans="1:7" x14ac:dyDescent="0.45">
+        <v>233.49</v>
+      </c>
+    </row>
+    <row r="23" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A23" s="11">
-        <v>46308</v>
+        <v>46309</v>
       </c>
       <c r="B23" s="12"/>
       <c r="C23" s="21" t="s">
         <v>17</v>
       </c>
       <c r="D23" s="13">
-        <v>259.64999999999998</v>
+        <v>259.14999999999998</v>
       </c>
       <c r="E23" s="13">
-        <v>246.57</v>
+        <v>245.21</v>
       </c>
       <c r="F23" s="13">
-        <v>256.57</v>
+        <v>255.21</v>
       </c>
       <c r="G23" s="13" t="s">
         <v>18</v>
       </c>
     </row>
-    <row r="24" spans="1:7" x14ac:dyDescent="0.45">
+    <row r="24" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A24" s="7">
-        <v>46308</v>
+        <v>46309</v>
       </c>
       <c r="B24" s="8"/>
       <c r="C24" s="20" t="s">
         <v>19</v>
       </c>
       <c r="D24" s="10">
-        <v>259.99</v>
+        <v>259.5</v>
       </c>
       <c r="E24" s="10">
-        <v>245.8</v>
+        <v>244.45</v>
       </c>
       <c r="F24" s="10">
-        <v>255.8</v>
+        <v>254.45</v>
       </c>
       <c r="G24" s="10" t="s">
         <v>18</v>
       </c>
     </row>
-    <row r="25" spans="1:7" x14ac:dyDescent="0.45">
+    <row r="25" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A25" s="11">
-        <v>46308</v>
+        <v>46309</v>
       </c>
       <c r="B25" s="12"/>
       <c r="C25" s="21" t="s">
         <v>20</v>
       </c>
       <c r="D25" s="13">
-        <v>256.66000000000003</v>
+        <v>256.16000000000003</v>
       </c>
       <c r="E25" s="13">
-        <v>246.05</v>
+        <v>244.69</v>
       </c>
       <c r="F25" s="13">
-        <v>256.05</v>
+        <v>254.69</v>
       </c>
       <c r="G25" s="13">
-        <v>241.89</v>
-      </c>
-    </row>
-    <row r="26" spans="1:7" x14ac:dyDescent="0.45">
+        <v>240.53</v>
+      </c>
+    </row>
+    <row r="26" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A26" s="7">
-        <v>46308</v>
+        <v>46309</v>
       </c>
       <c r="B26" s="8"/>
       <c r="C26" s="20" t="s">
         <v>21</v>
       </c>
       <c r="D26" s="10">
-        <v>258.18</v>
+        <v>257.7</v>
       </c>
       <c r="E26" s="10">
-        <v>247.59</v>
+        <v>246.23</v>
       </c>
       <c r="F26" s="10">
-        <v>257.58999999999997</v>
+        <v>256.23</v>
       </c>
       <c r="G26" s="10" t="s">
         <v>18</v>
       </c>
     </row>
-    <row r="27" spans="1:7" x14ac:dyDescent="0.45">
+    <row r="27" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A27" s="11">
-        <v>46305</v>
+        <v>46308</v>
       </c>
       <c r="B27" s="12"/>
       <c r="C27" s="12" t="s">
         <v>16</v>
       </c>
       <c r="D27" s="13">
-        <v>260.44</v>
+        <v>260.18</v>
       </c>
       <c r="E27" s="13">
-        <v>238.19</v>
+        <v>238.02</v>
       </c>
       <c r="F27" s="13">
-        <v>247.78</v>
+        <v>247.62</v>
       </c>
       <c r="G27" s="13">
-        <v>234.56</v>
-      </c>
-    </row>
-    <row r="28" spans="1:7" x14ac:dyDescent="0.45">
+        <v>234.39</v>
+      </c>
+    </row>
+    <row r="28" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A28" s="7">
-        <v>46305</v>
+        <v>46308</v>
       </c>
       <c r="B28" s="8"/>
       <c r="C28" s="20" t="s">
         <v>17</v>
       </c>
       <c r="D28" s="10">
-        <v>260.38</v>
+        <v>259.64999999999998</v>
       </c>
       <c r="E28" s="22">
-        <v>248.82</v>
+        <v>246.57</v>
       </c>
       <c r="F28" s="22">
-        <v>258.82</v>
+        <v>256.57</v>
       </c>
       <c r="G28" s="22" t="s">
         <v>18</v>
       </c>
     </row>
-    <row r="29" spans="1:7" x14ac:dyDescent="0.45">
+    <row r="29" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A29" s="11">
-        <v>46305</v>
+        <v>46308</v>
       </c>
       <c r="B29" s="12"/>
       <c r="C29" s="12" t="s">
         <v>19</v>
       </c>
       <c r="D29" s="13">
-        <v>260.72000000000003</v>
+        <v>259.99</v>
       </c>
       <c r="E29" s="13">
-        <v>248.05</v>
+        <v>245.8</v>
       </c>
       <c r="F29" s="13">
-        <v>258.05</v>
+        <v>255.8</v>
       </c>
       <c r="G29" s="13" t="s">
         <v>18</v>
       </c>
     </row>
-    <row r="30" spans="1:7" x14ac:dyDescent="0.45">
+    <row r="30" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A30" s="7">
-        <v>46305</v>
+        <v>46308</v>
       </c>
       <c r="B30" s="8"/>
       <c r="C30" s="20" t="s">
         <v>20</v>
       </c>
       <c r="D30" s="10">
-        <v>257.37</v>
+        <v>256.66000000000003</v>
       </c>
       <c r="E30" s="22">
-        <v>248.31</v>
+        <v>246.05</v>
       </c>
       <c r="F30" s="22">
-        <v>258.31</v>
+        <v>256.05</v>
       </c>
       <c r="G30" s="22">
-        <v>244.15</v>
-      </c>
-    </row>
-    <row r="31" spans="1:7" x14ac:dyDescent="0.45">
+        <v>241.89</v>
+      </c>
+    </row>
+    <row r="31" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A31" s="11">
-        <v>46305</v>
+        <v>46308</v>
       </c>
       <c r="B31" s="12"/>
       <c r="C31" s="12" t="s">
         <v>21</v>
       </c>
       <c r="D31" s="13">
-        <v>258.89</v>
+        <v>258.18</v>
       </c>
       <c r="E31" s="13">
-        <v>249.87</v>
+        <v>247.59</v>
       </c>
       <c r="F31" s="13">
-        <v>259.87</v>
+        <v>257.58999999999997</v>
       </c>
       <c r="G31" s="13" t="s">
         <v>18</v>
       </c>
     </row>
-    <row r="32" spans="1:7" x14ac:dyDescent="0.45">
+    <row r="32" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A32" s="14"/>
       <c r="B32" s="14"/>
       <c r="C32" s="15"/>
@@ -1269,7 +1269,7 @@
       <c r="F32" s="17"/>
       <c r="G32" s="17"/>
     </row>
-    <row r="33" spans="1:7" ht="20.25" x14ac:dyDescent="0.45">
+    <row r="33" spans="1:7" ht="20.25" x14ac:dyDescent="0.25">
       <c r="A33" s="29" t="s">
         <v>22</v>
       </c>
@@ -1280,7 +1280,7 @@
       <c r="F33" s="17"/>
       <c r="G33" s="17"/>
     </row>
-    <row r="34" spans="1:7" x14ac:dyDescent="0.45">
+    <row r="34" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A34" s="23" t="s">
         <v>4</v>
       </c>
@@ -1299,54 +1299,54 @@
       </c>
       <c r="G34" s="17"/>
     </row>
-    <row r="35" spans="1:7" x14ac:dyDescent="0.45">
+    <row r="35" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A35" s="7">
-        <v>46308</v>
+        <v>46309</v>
       </c>
       <c r="B35" s="8"/>
       <c r="C35" s="20" t="s">
         <v>23</v>
       </c>
       <c r="D35" s="10">
-        <v>253.24</v>
+        <v>252.75</v>
       </c>
       <c r="E35" s="10">
-        <v>233.87</v>
+        <v>233.09</v>
       </c>
       <c r="F35" s="10">
-        <v>242.87</v>
+        <v>242.09</v>
       </c>
       <c r="G35" s="17"/>
     </row>
-    <row r="36" spans="1:7" x14ac:dyDescent="0.45">
+    <row r="36" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A36" s="11">
-        <v>46305</v>
+        <v>46308</v>
       </c>
       <c r="B36" s="12"/>
       <c r="C36" s="12" t="s">
         <v>23</v>
       </c>
       <c r="D36" s="13">
-        <v>253.96</v>
+        <v>253.24</v>
       </c>
       <c r="E36" s="13">
-        <v>234.45</v>
+        <v>233.87</v>
       </c>
       <c r="F36" s="13">
-        <v>243.45</v>
+        <v>242.87</v>
       </c>
       <c r="G36" s="17"/>
     </row>
-    <row r="37" spans="1:7" x14ac:dyDescent="0.45">
+    <row r="37" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A37" s="7">
-        <v>46308</v>
+        <v>46309</v>
       </c>
       <c r="B37" s="8"/>
       <c r="C37" s="20" t="s">
         <v>24</v>
       </c>
       <c r="D37" s="10">
-        <v>268.86</v>
+        <v>268.37</v>
       </c>
       <c r="E37" s="10" t="s">
         <v>18</v>
@@ -1356,16 +1356,16 @@
       </c>
       <c r="G37" s="17"/>
     </row>
-    <row r="38" spans="1:7" x14ac:dyDescent="0.45">
+    <row r="38" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A38" s="11">
-        <v>46305</v>
+        <v>46308</v>
       </c>
       <c r="B38" s="12"/>
       <c r="C38" s="12" t="s">
         <v>24</v>
       </c>
       <c r="D38" s="13">
-        <v>269.58</v>
+        <v>268.86</v>
       </c>
       <c r="E38" s="13" t="s">
         <v>18</v>
@@ -1375,7 +1375,7 @@
       </c>
       <c r="G38" s="17"/>
     </row>
-    <row r="39" spans="1:7" x14ac:dyDescent="0.45">
+    <row r="39" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A39" s="24"/>
       <c r="B39" s="24"/>
       <c r="C39" s="15"/>
@@ -1384,7 +1384,7 @@
       <c r="F39" s="17"/>
       <c r="G39" s="17"/>
     </row>
-    <row r="40" spans="1:7" ht="20.25" x14ac:dyDescent="0.45">
+    <row r="40" spans="1:7" ht="20.25" x14ac:dyDescent="0.25">
       <c r="A40" s="29" t="s">
         <v>25</v>
       </c>
@@ -1395,7 +1395,7 @@
       <c r="F40" s="17"/>
       <c r="G40" s="17"/>
     </row>
-    <row r="41" spans="1:7" x14ac:dyDescent="0.45">
+    <row r="41" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A41" s="23" t="s">
         <v>4</v>
       </c>
@@ -1414,83 +1414,83 @@
       </c>
       <c r="G41" s="17"/>
     </row>
-    <row r="42" spans="1:7" x14ac:dyDescent="0.45">
+    <row r="42" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A42" s="7">
-        <v>46308</v>
+        <v>46309</v>
       </c>
       <c r="B42" s="8"/>
       <c r="C42" s="20" t="s">
         <v>26</v>
       </c>
       <c r="D42" s="10">
-        <v>263.3</v>
+        <v>262.77</v>
       </c>
       <c r="E42" s="10">
-        <v>243.64</v>
+        <v>242.85</v>
       </c>
       <c r="F42" s="10">
-        <v>253.64</v>
+        <v>252.85</v>
       </c>
       <c r="G42" s="17"/>
     </row>
-    <row r="43" spans="1:7" x14ac:dyDescent="0.45">
+    <row r="43" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A43" s="11">
-        <v>46308</v>
+        <v>46309</v>
       </c>
       <c r="B43" s="12"/>
       <c r="C43" s="21" t="s">
         <v>27</v>
       </c>
       <c r="D43" s="13">
-        <v>262.91000000000003</v>
+        <v>262.38</v>
       </c>
       <c r="E43" s="13">
-        <v>244.05</v>
+        <v>243.26</v>
       </c>
       <c r="F43" s="13">
-        <v>254.05</v>
+        <v>253.26</v>
       </c>
       <c r="G43" s="17"/>
     </row>
-    <row r="44" spans="1:7" x14ac:dyDescent="0.45">
+    <row r="44" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A44" s="7">
-        <v>46305</v>
+        <v>46308</v>
       </c>
       <c r="B44" s="8"/>
       <c r="C44" s="20" t="s">
         <v>26</v>
       </c>
       <c r="D44" s="10">
-        <v>264.06</v>
+        <v>263.3</v>
       </c>
       <c r="E44" s="10">
-        <v>245.34</v>
+        <v>243.64</v>
       </c>
       <c r="F44" s="10">
-        <v>255.34</v>
+        <v>253.64</v>
       </c>
       <c r="G44" s="17"/>
     </row>
-    <row r="45" spans="1:7" x14ac:dyDescent="0.45">
+    <row r="45" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A45" s="11">
-        <v>46305</v>
+        <v>46308</v>
       </c>
       <c r="B45" s="12"/>
       <c r="C45" s="21" t="s">
         <v>27</v>
       </c>
       <c r="D45" s="13">
-        <v>263.68</v>
+        <v>262.91000000000003</v>
       </c>
       <c r="E45" s="13">
-        <v>245.75</v>
+        <v>244.05</v>
       </c>
       <c r="F45" s="13">
-        <v>255.75</v>
+        <v>254.05</v>
       </c>
       <c r="G45" s="17"/>
     </row>
-    <row r="46" spans="1:7" x14ac:dyDescent="0.45">
+    <row r="46" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A46" s="14"/>
       <c r="B46" s="24"/>
       <c r="C46" s="15"/>
@@ -1499,7 +1499,7 @@
       <c r="F46" s="16"/>
       <c r="G46" s="17"/>
     </row>
-    <row r="47" spans="1:7" ht="20.25" x14ac:dyDescent="0.45">
+    <row r="47" spans="1:7" ht="20.25" x14ac:dyDescent="0.25">
       <c r="A47" s="25" t="s">
         <v>28</v>
       </c>
@@ -1510,7 +1510,7 @@
       <c r="F47" s="17"/>
       <c r="G47" s="17"/>
     </row>
-    <row r="48" spans="1:7" x14ac:dyDescent="0.45">
+    <row r="48" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A48" s="23" t="s">
         <v>4</v>
       </c>
@@ -1529,83 +1529,83 @@
       </c>
       <c r="G48" s="17"/>
     </row>
-    <row r="49" spans="1:7" x14ac:dyDescent="0.45">
+    <row r="49" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A49" s="7">
-        <v>46308</v>
+        <v>46309</v>
       </c>
       <c r="B49" s="8"/>
       <c r="C49" s="20" t="s">
         <v>29</v>
       </c>
       <c r="D49" s="10">
-        <v>257.98</v>
+        <v>256.23</v>
       </c>
       <c r="E49" s="10">
-        <v>240.01</v>
+        <v>238.37</v>
       </c>
       <c r="F49" s="10">
-        <v>250.01</v>
+        <v>248.37</v>
       </c>
       <c r="G49" s="28"/>
     </row>
-    <row r="50" spans="1:7" x14ac:dyDescent="0.45">
+    <row r="50" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A50" s="11">
-        <v>46308</v>
+        <v>46309</v>
       </c>
       <c r="B50" s="12"/>
       <c r="C50" s="21" t="s">
         <v>30</v>
       </c>
       <c r="D50" s="13">
-        <v>255.47</v>
+        <v>253.72</v>
       </c>
       <c r="E50" s="13">
-        <v>239.62</v>
+        <v>237.98</v>
       </c>
       <c r="F50" s="13">
-        <v>249.62</v>
+        <v>247.98</v>
       </c>
       <c r="G50" s="28"/>
     </row>
-    <row r="51" spans="1:7" x14ac:dyDescent="0.45">
+    <row r="51" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A51" s="7">
-        <v>46305</v>
+        <v>46308</v>
       </c>
       <c r="B51" s="8"/>
       <c r="C51" s="20" t="s">
         <v>29</v>
       </c>
       <c r="D51" s="10">
-        <v>258.29000000000002</v>
+        <v>257.98</v>
       </c>
       <c r="E51" s="10">
-        <v>240.22</v>
+        <v>240.01</v>
       </c>
       <c r="F51" s="10">
-        <v>250.22</v>
+        <v>250.01</v>
       </c>
       <c r="G51" s="17"/>
     </row>
-    <row r="52" spans="1:7" x14ac:dyDescent="0.45">
+    <row r="52" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A52" s="11">
-        <v>46305</v>
+        <v>46308</v>
       </c>
       <c r="B52" s="12"/>
       <c r="C52" s="21" t="s">
         <v>30</v>
       </c>
       <c r="D52" s="13">
-        <v>255.79</v>
+        <v>255.47</v>
       </c>
       <c r="E52" s="13">
-        <v>239.84</v>
+        <v>239.62</v>
       </c>
       <c r="F52" s="13">
-        <v>249.84</v>
+        <v>249.62</v>
       </c>
       <c r="G52" s="17"/>
     </row>
-    <row r="53" spans="1:7" x14ac:dyDescent="0.45">
+    <row r="53" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A53" s="14"/>
       <c r="B53" s="14"/>
       <c r="C53" s="15"/>
@@ -1614,7 +1614,7 @@
       <c r="F53" s="16"/>
       <c r="G53" s="17"/>
     </row>
-    <row r="54" spans="1:7" ht="20.25" x14ac:dyDescent="0.45">
+    <row r="54" spans="1:7" ht="20.25" x14ac:dyDescent="0.25">
       <c r="A54" s="27" t="s">
         <v>31</v>
       </c>
@@ -1625,7 +1625,7 @@
       <c r="F54" s="17"/>
       <c r="G54" s="17"/>
     </row>
-    <row r="55" spans="1:7" x14ac:dyDescent="0.45">
+    <row r="55" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A55" s="23" t="s">
         <v>4</v>
       </c>
@@ -1644,54 +1644,54 @@
       </c>
       <c r="G55" s="17"/>
     </row>
-    <row r="56" spans="1:7" x14ac:dyDescent="0.45">
+    <row r="56" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A56" s="7">
-        <v>46308</v>
+        <v>46309</v>
       </c>
       <c r="B56" s="8"/>
       <c r="C56" s="20" t="s">
         <v>32</v>
       </c>
       <c r="D56" s="10">
-        <v>269.35000000000002</v>
+        <v>268.86</v>
       </c>
       <c r="E56" s="10">
-        <v>265.16000000000003</v>
+        <v>263.64999999999998</v>
       </c>
       <c r="F56" s="10">
-        <v>275.16000000000003</v>
+        <v>273.64999999999998</v>
       </c>
       <c r="G56" s="17"/>
     </row>
-    <row r="57" spans="1:7" x14ac:dyDescent="0.45">
+    <row r="57" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A57" s="11">
-        <v>46308</v>
+        <v>46309</v>
       </c>
       <c r="B57" s="12"/>
       <c r="C57" s="21" t="s">
         <v>33</v>
       </c>
       <c r="D57" s="13">
-        <v>259.32</v>
+        <v>258.82</v>
       </c>
       <c r="E57" s="13">
-        <v>246.32</v>
+        <v>245.03</v>
       </c>
       <c r="F57" s="13">
-        <v>256.32</v>
+        <v>255.03</v>
       </c>
       <c r="G57" s="17"/>
     </row>
-    <row r="58" spans="1:7" x14ac:dyDescent="0.45">
+    <row r="58" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A58" s="7">
-        <v>46308</v>
+        <v>46309</v>
       </c>
       <c r="B58" s="8"/>
       <c r="C58" s="20" t="s">
         <v>34</v>
       </c>
       <c r="D58" s="10">
-        <v>260.20999999999998</v>
+        <v>259.70999999999998</v>
       </c>
       <c r="E58" s="10" t="s">
         <v>18</v>
@@ -1701,111 +1701,111 @@
       </c>
       <c r="G58" s="17"/>
     </row>
-    <row r="59" spans="1:7" x14ac:dyDescent="0.45">
+    <row r="59" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A59" s="11">
-        <v>46308</v>
+        <v>46309</v>
       </c>
       <c r="B59" s="12"/>
       <c r="C59" s="21" t="s">
         <v>35</v>
       </c>
       <c r="D59" s="13">
-        <v>256.51</v>
+        <v>253.87</v>
       </c>
       <c r="E59" s="13">
-        <v>240.69</v>
+        <v>239.4</v>
       </c>
       <c r="F59" s="13" t="s">
         <v>18</v>
       </c>
       <c r="G59" s="17"/>
     </row>
-    <row r="60" spans="1:7" x14ac:dyDescent="0.45">
+    <row r="60" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A60" s="7">
-        <v>46308</v>
+        <v>46309</v>
       </c>
       <c r="B60" s="8"/>
       <c r="C60" s="20" t="s">
         <v>36</v>
       </c>
       <c r="D60" s="10">
-        <v>252.34</v>
+        <v>249.69</v>
       </c>
       <c r="E60" s="10">
-        <v>236.64</v>
+        <v>235.35</v>
       </c>
       <c r="F60" s="10">
-        <v>246.64</v>
+        <v>245.35</v>
       </c>
       <c r="G60" s="17"/>
     </row>
-    <row r="61" spans="1:7" x14ac:dyDescent="0.45">
+    <row r="61" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A61" s="11">
-        <v>46308</v>
+        <v>46309</v>
       </c>
       <c r="B61" s="12"/>
       <c r="C61" s="21" t="s">
         <v>37</v>
       </c>
       <c r="D61" s="13">
-        <v>257.17</v>
+        <v>256.72000000000003</v>
       </c>
       <c r="E61" s="13">
-        <v>258.42</v>
+        <v>256.99</v>
       </c>
       <c r="F61" s="13" t="s">
         <v>18</v>
       </c>
       <c r="G61" s="17"/>
     </row>
-    <row r="62" spans="1:7" x14ac:dyDescent="0.45">
+    <row r="62" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A62" s="7">
-        <v>46305</v>
+        <v>46308</v>
       </c>
       <c r="B62" s="8"/>
       <c r="C62" s="20" t="s">
         <v>32</v>
       </c>
       <c r="D62" s="10">
-        <v>270.06</v>
+        <v>269.35000000000002</v>
       </c>
       <c r="E62" s="10">
-        <v>267.62</v>
+        <v>265.16000000000003</v>
       </c>
       <c r="F62" s="10">
-        <v>277.62</v>
+        <v>275.16000000000003</v>
       </c>
       <c r="G62" s="17"/>
     </row>
-    <row r="63" spans="1:7" x14ac:dyDescent="0.45">
+    <row r="63" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A63" s="11">
-        <v>46305</v>
+        <v>46308</v>
       </c>
       <c r="B63" s="12"/>
       <c r="C63" s="21" t="s">
         <v>33</v>
       </c>
       <c r="D63" s="13">
-        <v>260.05</v>
+        <v>259.32</v>
       </c>
       <c r="E63" s="13">
-        <v>248.47</v>
+        <v>246.32</v>
       </c>
       <c r="F63" s="13">
-        <v>258.47000000000003</v>
+        <v>256.32</v>
       </c>
       <c r="G63" s="17"/>
     </row>
-    <row r="64" spans="1:7" x14ac:dyDescent="0.45">
+    <row r="64" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A64" s="7">
-        <v>46305</v>
+        <v>46308</v>
       </c>
       <c r="B64" s="8"/>
       <c r="C64" s="20" t="s">
         <v>34</v>
       </c>
       <c r="D64" s="10">
-        <v>260.95</v>
+        <v>260.20999999999998</v>
       </c>
       <c r="E64" s="10" t="s">
         <v>18</v>
@@ -1815,55 +1815,55 @@
       </c>
       <c r="G64" s="17"/>
     </row>
-    <row r="65" spans="1:6" x14ac:dyDescent="0.45">
+    <row r="65" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A65" s="11">
-        <v>46305</v>
+        <v>46308</v>
       </c>
       <c r="B65" s="12"/>
       <c r="C65" s="21" t="s">
         <v>35</v>
       </c>
       <c r="D65" s="13">
-        <v>257.70999999999998</v>
+        <v>256.51</v>
       </c>
       <c r="E65" s="13">
-        <v>242.84</v>
+        <v>240.69</v>
       </c>
       <c r="F65" s="13" t="s">
         <v>18</v>
       </c>
     </row>
-    <row r="66" spans="1:6" x14ac:dyDescent="0.45">
+    <row r="66" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A66" s="7">
-        <v>46305</v>
+        <v>46308</v>
       </c>
       <c r="B66" s="8"/>
       <c r="C66" s="20" t="s">
         <v>36</v>
       </c>
       <c r="D66" s="10">
-        <v>253.53</v>
+        <v>252.34</v>
       </c>
       <c r="E66" s="10">
-        <v>238.79</v>
+        <v>236.64</v>
       </c>
       <c r="F66" s="10">
-        <v>248.79</v>
-      </c>
-    </row>
-    <row r="67" spans="1:6" x14ac:dyDescent="0.45">
+        <v>246.64</v>
+      </c>
+    </row>
+    <row r="67" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A67" s="11">
-        <v>46305</v>
+        <v>46308</v>
       </c>
       <c r="B67" s="12"/>
       <c r="C67" s="21" t="s">
         <v>37</v>
       </c>
       <c r="D67" s="13">
-        <v>257.81</v>
+        <v>257.17</v>
       </c>
       <c r="E67" s="13">
-        <v>260.77999999999997</v>
+        <v>258.42</v>
       </c>
       <c r="F67" s="13" t="s">
         <v>18</v>
@@ -1891,6 +1891,15 @@
 </file>
 
 <file path=customXml/item1.xml><?xml version="1.0" encoding="utf-8"?>
+<?mso-contentType ?>
+<FormTemplates xmlns="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms">
+  <Display>DocumentLibraryForm</Display>
+  <Edit>DocumentLibraryForm</Edit>
+  <New>DocumentLibraryForm</New>
+</FormTemplates>
+</file>
+
+<file path=customXml/item2.xml><?xml version="1.0" encoding="utf-8"?>
 <p:properties xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls">
   <documentManagement>
     <lcf76f155ced4ddcb4097134ff3c332f xmlns="87276d81-85f4-4ef2-9e6e-55066304288f">
@@ -1899,15 +1908,6 @@
     <TaxCatchAll xmlns="b23b8984-eafa-4e79-985e-54f52f3da58e" xsi:nil="true"/>
   </documentManagement>
 </p:properties>
-</file>
-
-<file path=customXml/item2.xml><?xml version="1.0" encoding="utf-8"?>
-<?mso-contentType ?>
-<FormTemplates xmlns="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms">
-  <Display>DocumentLibraryForm</Display>
-  <Edit>DocumentLibraryForm</Edit>
-  <New>DocumentLibraryForm</New>
-</FormTemplates>
 </file>
 
 <file path=customXml/item3.xml><?xml version="1.0" encoding="utf-8"?>
@@ -2171,20 +2171,20 @@
 </file>
 
 <file path=customXml/itemProps1.xml><?xml version="1.0" encoding="utf-8"?>
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{F60519E9-FD90-4339-869C-BC2F85719BB8}">
+  <ds:schemaRefs>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms"/>
+  </ds:schemaRefs>
+</ds:datastoreItem>
+</file>
+
+<file path=customXml/itemProps2.xml><?xml version="1.0" encoding="utf-8"?>
 <ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{57A83D98-2BAE-4D83-823A-D31C464B620C}">
   <ds:schemaRefs>
     <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/properties"/>
     <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
     <ds:schemaRef ds:uri="87276d81-85f4-4ef2-9e6e-55066304288f"/>
     <ds:schemaRef ds:uri="b23b8984-eafa-4e79-985e-54f52f3da58e"/>
-  </ds:schemaRefs>
-</ds:datastoreItem>
-</file>
-
-<file path=customXml/itemProps2.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{F60519E9-FD90-4339-869C-BC2F85719BB8}">
-  <ds:schemaRefs>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms"/>
   </ds:schemaRefs>
 </ds:datastoreItem>
 </file>

</xml_diff>

<commit_message>
Wed Oct 14 06:15:18 UTC 2026
</commit_message>
<xml_diff>
--- a/bp.com-content-dam-bp-country-sites-en_au-australia-home-products-services-pricing-tgp-excel.xlsx
+++ b/bp.com-content-dam-bp-country-sites-en_au-australia-home-products-services-pricing-tgp-excel.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://bp365.sharepoint.com/sites/WholesalePricing/Shared Documents/B2C/TGP/Daily TGP/Web TGP/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="14_{CBB2D331-E0D6-490A-A19D-DB494B4EC0C0}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="14_{93C8CB39-39FD-484F-8341-7F8554D23B25}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-28920" yWindow="-60" windowWidth="29040" windowHeight="15720" xr2:uid="{1B412EEF-F96D-4DF4-A4E9-C7F0F183C2FB}"/>
+    <workbookView xWindow="-110" yWindow="-110" windowWidth="19420" windowHeight="11500" xr2:uid="{1B412EEF-F96D-4DF4-A4E9-C7F0F183C2FB}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
@@ -715,15 +715,15 @@
     <pageSetUpPr fitToPage="1"/>
   </sheetPr>
   <dimension ref="A1:G67"/>
-  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
   <cols>
-    <col min="1" max="1" width="76.42578125" bestFit="1" customWidth="1"/>
-    <col min="2" max="2" width="6.42578125"/>
-    <col min="3" max="3" width="18.140625" bestFit="1" customWidth="1"/>
-    <col min="4" max="7" width="7.140625" bestFit="1" customWidth="1"/>
+    <col min="1" max="1" width="76.453125" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="6.453125"/>
+    <col min="3" max="3" width="18.1796875" bestFit="1" customWidth="1"/>
+    <col min="4" max="7" width="7.1796875" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:7" ht="23.25" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:7" ht="22.5" x14ac:dyDescent="0.35">
       <c r="A1" s="30" t="s">
         <v>0</v>
       </c>
@@ -734,7 +734,7 @@
       <c r="F1" s="2"/>
       <c r="G1" s="2"/>
     </row>
-    <row r="2" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="2" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A2" s="3"/>
       <c r="B2" s="1"/>
       <c r="C2" s="1"/>
@@ -743,7 +743,7 @@
       <c r="F2" s="2"/>
       <c r="G2" s="2"/>
     </row>
-    <row r="3" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="3" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A3" s="3" t="s">
         <v>1</v>
       </c>
@@ -754,7 +754,7 @@
       <c r="F3" s="2"/>
       <c r="G3" s="2"/>
     </row>
-    <row r="4" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="4" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A4" s="3" t="s">
         <v>2</v>
       </c>
@@ -765,7 +765,7 @@
       <c r="F4" s="2"/>
       <c r="G4" s="2"/>
     </row>
-    <row r="5" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="5" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A5" s="3"/>
       <c r="B5" s="3"/>
       <c r="C5" s="1"/>
@@ -774,7 +774,7 @@
       <c r="F5" s="2"/>
       <c r="G5" s="2"/>
     </row>
-    <row r="6" spans="1:7" ht="20.25" x14ac:dyDescent="0.25">
+    <row r="6" spans="1:7" ht="20" x14ac:dyDescent="0.35">
       <c r="A6" s="29" t="s">
         <v>3</v>
       </c>
@@ -785,7 +785,7 @@
       <c r="F6" s="2"/>
       <c r="G6" s="2"/>
     </row>
-    <row r="7" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="7" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A7" s="4" t="s">
         <v>4</v>
       </c>
@@ -806,133 +806,133 @@
         <v>9</v>
       </c>
     </row>
-    <row r="8" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="8" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A8" s="7">
-        <v>46309</v>
+        <v>46310</v>
       </c>
       <c r="B8" s="8"/>
       <c r="C8" s="9" t="s">
         <v>10</v>
       </c>
       <c r="D8" s="10">
-        <v>258.49</v>
+        <v>257.98</v>
       </c>
       <c r="E8" s="10">
-        <v>236.44</v>
+        <v>233.92</v>
       </c>
       <c r="F8" s="10">
-        <v>246.44</v>
+        <v>243.92</v>
       </c>
       <c r="G8" s="10">
-        <v>234.05</v>
-      </c>
-    </row>
-    <row r="9" spans="1:7" x14ac:dyDescent="0.25">
+        <v>231.54</v>
+      </c>
+    </row>
+    <row r="9" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A9" s="11">
-        <v>46309</v>
+        <v>46310</v>
       </c>
       <c r="B9" s="12"/>
       <c r="C9" s="12" t="s">
         <v>11</v>
       </c>
       <c r="D9" s="13">
-        <v>258.49</v>
+        <v>257.98</v>
       </c>
       <c r="E9" s="13">
-        <v>236.44</v>
+        <v>233.92</v>
       </c>
       <c r="F9" s="13">
-        <v>246.44</v>
+        <v>243.92</v>
       </c>
       <c r="G9" s="13">
-        <v>234.05</v>
-      </c>
-    </row>
-    <row r="10" spans="1:7" x14ac:dyDescent="0.25">
+        <v>231.54</v>
+      </c>
+    </row>
+    <row r="10" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A10" s="7">
-        <v>46309</v>
+        <v>46310</v>
       </c>
       <c r="B10" s="8"/>
       <c r="C10" s="9" t="s">
         <v>12</v>
       </c>
       <c r="D10" s="10">
-        <v>254.19</v>
+        <v>255.39</v>
       </c>
       <c r="E10" s="10">
-        <v>234.71</v>
+        <v>232.3</v>
       </c>
       <c r="F10" s="10">
-        <v>244.71</v>
+        <v>242.3</v>
       </c>
       <c r="G10" s="10">
-        <v>233.11</v>
-      </c>
-    </row>
-    <row r="11" spans="1:7" x14ac:dyDescent="0.25">
+        <v>230.71</v>
+      </c>
+    </row>
+    <row r="11" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A11" s="11">
-        <v>46308</v>
+        <v>46309</v>
       </c>
       <c r="B11" s="12"/>
       <c r="C11" s="12" t="s">
         <v>10</v>
       </c>
       <c r="D11" s="13">
-        <v>259.05</v>
+        <v>258.49</v>
       </c>
       <c r="E11" s="13">
-        <v>237.34</v>
+        <v>236.44</v>
       </c>
       <c r="F11" s="13">
-        <v>247.34</v>
+        <v>246.44</v>
       </c>
       <c r="G11" s="13">
-        <v>234.96</v>
-      </c>
-    </row>
-    <row r="12" spans="1:7" x14ac:dyDescent="0.25">
+        <v>234.05</v>
+      </c>
+    </row>
+    <row r="12" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A12" s="7">
-        <v>46308</v>
+        <v>46309</v>
       </c>
       <c r="B12" s="8"/>
       <c r="C12" s="9" t="s">
         <v>11</v>
       </c>
       <c r="D12" s="10">
-        <v>259.05</v>
+        <v>258.49</v>
       </c>
       <c r="E12" s="10">
-        <v>237.34</v>
+        <v>236.44</v>
       </c>
       <c r="F12" s="10">
-        <v>247.34</v>
+        <v>246.44</v>
       </c>
       <c r="G12" s="10">
-        <v>234.96</v>
-      </c>
-    </row>
-    <row r="13" spans="1:7" x14ac:dyDescent="0.25">
+        <v>234.05</v>
+      </c>
+    </row>
+    <row r="13" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A13" s="11">
-        <v>46308</v>
+        <v>46309</v>
       </c>
       <c r="B13" s="12"/>
       <c r="C13" s="12" t="s">
         <v>12</v>
       </c>
       <c r="D13" s="13">
-        <v>254.69</v>
+        <v>254.19</v>
       </c>
       <c r="E13" s="13">
-        <v>236.04</v>
+        <v>234.71</v>
       </c>
       <c r="F13" s="13">
-        <v>246.04</v>
+        <v>244.71</v>
       </c>
       <c r="G13" s="13">
-        <v>234.45</v>
-      </c>
-    </row>
-    <row r="14" spans="1:7" x14ac:dyDescent="0.25">
+        <v>233.11</v>
+      </c>
+    </row>
+    <row r="14" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A14" s="14"/>
       <c r="B14" s="14"/>
       <c r="C14" s="15"/>
@@ -941,7 +941,7 @@
       <c r="F14" s="16"/>
       <c r="G14" s="16"/>
     </row>
-    <row r="15" spans="1:7" ht="20.25" x14ac:dyDescent="0.25">
+    <row r="15" spans="1:7" ht="20" x14ac:dyDescent="0.35">
       <c r="A15" s="29" t="s">
         <v>13</v>
       </c>
@@ -952,7 +952,7 @@
       <c r="F15" s="17"/>
       <c r="G15" s="17"/>
     </row>
-    <row r="16" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="16" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A16" s="4" t="s">
         <v>4</v>
       </c>
@@ -971,45 +971,45 @@
       </c>
       <c r="G16" s="17"/>
     </row>
-    <row r="17" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="17" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A17" s="7">
-        <v>46309</v>
+        <v>46310</v>
       </c>
       <c r="B17" s="8"/>
       <c r="C17" s="20" t="s">
         <v>14</v>
       </c>
       <c r="D17" s="10">
-        <v>257.64</v>
+        <v>258.87</v>
       </c>
       <c r="E17" s="10">
-        <v>239.88</v>
+        <v>237.5</v>
       </c>
       <c r="F17" s="10">
-        <v>249.88</v>
+        <v>247.5</v>
       </c>
       <c r="G17" s="17"/>
     </row>
-    <row r="18" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="18" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A18" s="11">
-        <v>46308</v>
+        <v>46309</v>
       </c>
       <c r="B18" s="12"/>
       <c r="C18" s="12" t="s">
         <v>14</v>
       </c>
       <c r="D18" s="13">
-        <v>258.08999999999997</v>
+        <v>257.64</v>
       </c>
       <c r="E18" s="13">
-        <v>241.18</v>
+        <v>239.88</v>
       </c>
       <c r="F18" s="13">
-        <v>251.19</v>
+        <v>249.88</v>
       </c>
       <c r="G18" s="17"/>
     </row>
-    <row r="19" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="19" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A19" s="14"/>
       <c r="B19" s="14"/>
       <c r="C19" s="15"/>
@@ -1018,7 +1018,7 @@
       <c r="F19" s="16"/>
       <c r="G19" s="17"/>
     </row>
-    <row r="20" spans="1:7" ht="20.25" x14ac:dyDescent="0.25">
+    <row r="20" spans="1:7" ht="20" x14ac:dyDescent="0.35">
       <c r="A20" s="29" t="s">
         <v>15</v>
       </c>
@@ -1029,7 +1029,7 @@
       <c r="F20" s="17"/>
       <c r="G20" s="17"/>
     </row>
-    <row r="21" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="21" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A21" s="4" t="s">
         <v>4</v>
       </c>
@@ -1050,217 +1050,217 @@
         <v>9</v>
       </c>
     </row>
-    <row r="22" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="22" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A22" s="7">
-        <v>46309</v>
+        <v>46310</v>
       </c>
       <c r="B22" s="8"/>
       <c r="C22" s="20" t="s">
         <v>16</v>
       </c>
       <c r="D22" s="10">
-        <v>259.62</v>
+        <v>259.10000000000002</v>
       </c>
       <c r="E22" s="10">
-        <v>237.12</v>
+        <v>234.06</v>
       </c>
       <c r="F22" s="10">
-        <v>246.72</v>
+        <v>243.66</v>
       </c>
       <c r="G22" s="10">
-        <v>233.49</v>
-      </c>
-    </row>
-    <row r="23" spans="1:7" x14ac:dyDescent="0.25">
+        <v>230.43</v>
+      </c>
+    </row>
+    <row r="23" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A23" s="11">
-        <v>46309</v>
+        <v>46310</v>
       </c>
       <c r="B23" s="12"/>
       <c r="C23" s="21" t="s">
         <v>17</v>
       </c>
       <c r="D23" s="13">
-        <v>259.14999999999998</v>
+        <v>260.33999999999997</v>
       </c>
       <c r="E23" s="13">
-        <v>245.21</v>
+        <v>242.79</v>
       </c>
       <c r="F23" s="13">
-        <v>255.21</v>
+        <v>252.79</v>
       </c>
       <c r="G23" s="13" t="s">
         <v>18</v>
       </c>
     </row>
-    <row r="24" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="24" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A24" s="7">
-        <v>46309</v>
+        <v>46310</v>
       </c>
       <c r="B24" s="8"/>
       <c r="C24" s="20" t="s">
         <v>19</v>
       </c>
       <c r="D24" s="10">
-        <v>259.5</v>
+        <v>260.7</v>
       </c>
       <c r="E24" s="10">
-        <v>244.45</v>
+        <v>242.03</v>
       </c>
       <c r="F24" s="10">
-        <v>254.45</v>
+        <v>252.03</v>
       </c>
       <c r="G24" s="10" t="s">
         <v>18</v>
       </c>
     </row>
-    <row r="25" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="25" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A25" s="11">
-        <v>46309</v>
+        <v>46310</v>
       </c>
       <c r="B25" s="12"/>
       <c r="C25" s="21" t="s">
         <v>20</v>
       </c>
       <c r="D25" s="13">
-        <v>256.16000000000003</v>
+        <v>257.36</v>
       </c>
       <c r="E25" s="13">
-        <v>244.69</v>
+        <v>242.26</v>
       </c>
       <c r="F25" s="13">
-        <v>254.69</v>
+        <v>252.26</v>
       </c>
       <c r="G25" s="13">
-        <v>240.53</v>
-      </c>
-    </row>
-    <row r="26" spans="1:7" x14ac:dyDescent="0.25">
+        <v>238.1</v>
+      </c>
+    </row>
+    <row r="26" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A26" s="7">
-        <v>46309</v>
+        <v>46310</v>
       </c>
       <c r="B26" s="8"/>
       <c r="C26" s="20" t="s">
         <v>21</v>
       </c>
       <c r="D26" s="10">
-        <v>257.7</v>
+        <v>258.91000000000003</v>
       </c>
       <c r="E26" s="10">
-        <v>246.23</v>
+        <v>243.78</v>
       </c>
       <c r="F26" s="10">
-        <v>256.23</v>
+        <v>253.78</v>
       </c>
       <c r="G26" s="10" t="s">
         <v>18</v>
       </c>
     </row>
-    <row r="27" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="27" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A27" s="11">
-        <v>46308</v>
+        <v>46309</v>
       </c>
       <c r="B27" s="12"/>
       <c r="C27" s="12" t="s">
         <v>16</v>
       </c>
       <c r="D27" s="13">
-        <v>260.18</v>
+        <v>259.62</v>
       </c>
       <c r="E27" s="13">
-        <v>238.02</v>
+        <v>237.12</v>
       </c>
       <c r="F27" s="13">
-        <v>247.62</v>
+        <v>246.72</v>
       </c>
       <c r="G27" s="13">
-        <v>234.39</v>
-      </c>
-    </row>
-    <row r="28" spans="1:7" x14ac:dyDescent="0.25">
+        <v>233.49</v>
+      </c>
+    </row>
+    <row r="28" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A28" s="7">
-        <v>46308</v>
+        <v>46309</v>
       </c>
       <c r="B28" s="8"/>
       <c r="C28" s="20" t="s">
         <v>17</v>
       </c>
       <c r="D28" s="10">
-        <v>259.64999999999998</v>
+        <v>259.14999999999998</v>
       </c>
       <c r="E28" s="22">
-        <v>246.57</v>
+        <v>245.21</v>
       </c>
       <c r="F28" s="22">
-        <v>256.57</v>
+        <v>255.21</v>
       </c>
       <c r="G28" s="22" t="s">
         <v>18</v>
       </c>
     </row>
-    <row r="29" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="29" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A29" s="11">
-        <v>46308</v>
+        <v>46309</v>
       </c>
       <c r="B29" s="12"/>
       <c r="C29" s="12" t="s">
         <v>19</v>
       </c>
       <c r="D29" s="13">
-        <v>259.99</v>
+        <v>259.5</v>
       </c>
       <c r="E29" s="13">
-        <v>245.8</v>
+        <v>244.45</v>
       </c>
       <c r="F29" s="13">
-        <v>255.8</v>
+        <v>254.45</v>
       </c>
       <c r="G29" s="13" t="s">
         <v>18</v>
       </c>
     </row>
-    <row r="30" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="30" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A30" s="7">
-        <v>46308</v>
+        <v>46309</v>
       </c>
       <c r="B30" s="8"/>
       <c r="C30" s="20" t="s">
         <v>20</v>
       </c>
       <c r="D30" s="10">
-        <v>256.66000000000003</v>
+        <v>256.16000000000003</v>
       </c>
       <c r="E30" s="22">
-        <v>246.05</v>
+        <v>244.69</v>
       </c>
       <c r="F30" s="22">
-        <v>256.05</v>
+        <v>254.69</v>
       </c>
       <c r="G30" s="22">
-        <v>241.89</v>
-      </c>
-    </row>
-    <row r="31" spans="1:7" x14ac:dyDescent="0.25">
+        <v>240.53</v>
+      </c>
+    </row>
+    <row r="31" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A31" s="11">
-        <v>46308</v>
+        <v>46309</v>
       </c>
       <c r="B31" s="12"/>
       <c r="C31" s="12" t="s">
         <v>21</v>
       </c>
       <c r="D31" s="13">
-        <v>258.18</v>
+        <v>257.7</v>
       </c>
       <c r="E31" s="13">
-        <v>247.59</v>
+        <v>246.23</v>
       </c>
       <c r="F31" s="13">
-        <v>257.58999999999997</v>
+        <v>256.23</v>
       </c>
       <c r="G31" s="13" t="s">
         <v>18</v>
       </c>
     </row>
-    <row r="32" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="32" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A32" s="14"/>
       <c r="B32" s="14"/>
       <c r="C32" s="15"/>
@@ -1269,7 +1269,7 @@
       <c r="F32" s="17"/>
       <c r="G32" s="17"/>
     </row>
-    <row r="33" spans="1:7" ht="20.25" x14ac:dyDescent="0.25">
+    <row r="33" spans="1:7" ht="20" x14ac:dyDescent="0.35">
       <c r="A33" s="29" t="s">
         <v>22</v>
       </c>
@@ -1280,7 +1280,7 @@
       <c r="F33" s="17"/>
       <c r="G33" s="17"/>
     </row>
-    <row r="34" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="34" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A34" s="23" t="s">
         <v>4</v>
       </c>
@@ -1299,54 +1299,54 @@
       </c>
       <c r="G34" s="17"/>
     </row>
-    <row r="35" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="35" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A35" s="7">
-        <v>46309</v>
+        <v>46310</v>
       </c>
       <c r="B35" s="8"/>
       <c r="C35" s="20" t="s">
         <v>23</v>
       </c>
       <c r="D35" s="10">
-        <v>252.75</v>
+        <v>253.94</v>
       </c>
       <c r="E35" s="10">
-        <v>233.09</v>
+        <v>231.24</v>
       </c>
       <c r="F35" s="10">
-        <v>242.09</v>
+        <v>240.24</v>
       </c>
       <c r="G35" s="17"/>
     </row>
-    <row r="36" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="36" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A36" s="11">
-        <v>46308</v>
+        <v>46309</v>
       </c>
       <c r="B36" s="12"/>
       <c r="C36" s="12" t="s">
         <v>23</v>
       </c>
       <c r="D36" s="13">
-        <v>253.24</v>
+        <v>252.75</v>
       </c>
       <c r="E36" s="13">
-        <v>233.87</v>
+        <v>233.09</v>
       </c>
       <c r="F36" s="13">
-        <v>242.87</v>
+        <v>242.09</v>
       </c>
       <c r="G36" s="17"/>
     </row>
-    <row r="37" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="37" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A37" s="7">
-        <v>46309</v>
+        <v>46310</v>
       </c>
       <c r="B37" s="8"/>
       <c r="C37" s="20" t="s">
         <v>24</v>
       </c>
       <c r="D37" s="10">
-        <v>268.37</v>
+        <v>269.56</v>
       </c>
       <c r="E37" s="10" t="s">
         <v>18</v>
@@ -1356,16 +1356,16 @@
       </c>
       <c r="G37" s="17"/>
     </row>
-    <row r="38" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="38" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A38" s="11">
-        <v>46308</v>
+        <v>46309</v>
       </c>
       <c r="B38" s="12"/>
       <c r="C38" s="12" t="s">
         <v>24</v>
       </c>
       <c r="D38" s="13">
-        <v>268.86</v>
+        <v>268.37</v>
       </c>
       <c r="E38" s="13" t="s">
         <v>18</v>
@@ -1375,7 +1375,7 @@
       </c>
       <c r="G38" s="17"/>
     </row>
-    <row r="39" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="39" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A39" s="24"/>
       <c r="B39" s="24"/>
       <c r="C39" s="15"/>
@@ -1384,7 +1384,7 @@
       <c r="F39" s="17"/>
       <c r="G39" s="17"/>
     </row>
-    <row r="40" spans="1:7" ht="20.25" x14ac:dyDescent="0.25">
+    <row r="40" spans="1:7" ht="20" x14ac:dyDescent="0.35">
       <c r="A40" s="29" t="s">
         <v>25</v>
       </c>
@@ -1395,7 +1395,7 @@
       <c r="F40" s="17"/>
       <c r="G40" s="17"/>
     </row>
-    <row r="41" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="41" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A41" s="23" t="s">
         <v>4</v>
       </c>
@@ -1414,83 +1414,83 @@
       </c>
       <c r="G41" s="17"/>
     </row>
-    <row r="42" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="42" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A42" s="7">
-        <v>46309</v>
+        <v>46310</v>
       </c>
       <c r="B42" s="8"/>
       <c r="C42" s="20" t="s">
         <v>26</v>
       </c>
       <c r="D42" s="10">
-        <v>262.77</v>
+        <v>263.94</v>
       </c>
       <c r="E42" s="10">
-        <v>242.85</v>
+        <v>241.39</v>
       </c>
       <c r="F42" s="10">
-        <v>252.85</v>
+        <v>251.39</v>
       </c>
       <c r="G42" s="17"/>
     </row>
-    <row r="43" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="43" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A43" s="11">
-        <v>46309</v>
+        <v>46310</v>
       </c>
       <c r="B43" s="12"/>
       <c r="C43" s="21" t="s">
         <v>27</v>
       </c>
       <c r="D43" s="13">
-        <v>262.38</v>
+        <v>263.55</v>
       </c>
       <c r="E43" s="13">
-        <v>243.26</v>
+        <v>241.8</v>
       </c>
       <c r="F43" s="13">
-        <v>253.26</v>
+        <v>251.8</v>
       </c>
       <c r="G43" s="17"/>
     </row>
-    <row r="44" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="44" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A44" s="7">
-        <v>46308</v>
+        <v>46309</v>
       </c>
       <c r="B44" s="8"/>
       <c r="C44" s="20" t="s">
         <v>26</v>
       </c>
       <c r="D44" s="10">
-        <v>263.3</v>
+        <v>262.77</v>
       </c>
       <c r="E44" s="10">
-        <v>243.64</v>
+        <v>242.85</v>
       </c>
       <c r="F44" s="10">
-        <v>253.64</v>
+        <v>252.85</v>
       </c>
       <c r="G44" s="17"/>
     </row>
-    <row r="45" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="45" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A45" s="11">
-        <v>46308</v>
+        <v>46309</v>
       </c>
       <c r="B45" s="12"/>
       <c r="C45" s="21" t="s">
         <v>27</v>
       </c>
       <c r="D45" s="13">
-        <v>262.91000000000003</v>
+        <v>262.38</v>
       </c>
       <c r="E45" s="13">
-        <v>244.05</v>
+        <v>243.26</v>
       </c>
       <c r="F45" s="13">
-        <v>254.05</v>
+        <v>253.26</v>
       </c>
       <c r="G45" s="17"/>
     </row>
-    <row r="46" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="46" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A46" s="14"/>
       <c r="B46" s="24"/>
       <c r="C46" s="15"/>
@@ -1499,7 +1499,7 @@
       <c r="F46" s="16"/>
       <c r="G46" s="17"/>
     </row>
-    <row r="47" spans="1:7" ht="20.25" x14ac:dyDescent="0.25">
+    <row r="47" spans="1:7" ht="20" x14ac:dyDescent="0.35">
       <c r="A47" s="25" t="s">
         <v>28</v>
       </c>
@@ -1510,7 +1510,7 @@
       <c r="F47" s="17"/>
       <c r="G47" s="17"/>
     </row>
-    <row r="48" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="48" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A48" s="23" t="s">
         <v>4</v>
       </c>
@@ -1529,83 +1529,83 @@
       </c>
       <c r="G48" s="17"/>
     </row>
-    <row r="49" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="49" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A49" s="7">
-        <v>46309</v>
+        <v>46310</v>
       </c>
       <c r="B49" s="8"/>
       <c r="C49" s="20" t="s">
         <v>29</v>
       </c>
       <c r="D49" s="10">
-        <v>256.23</v>
+        <v>255.92</v>
       </c>
       <c r="E49" s="10">
-        <v>238.37</v>
+        <v>236.16</v>
       </c>
       <c r="F49" s="10">
-        <v>248.37</v>
+        <v>246.16</v>
       </c>
       <c r="G49" s="28"/>
     </row>
-    <row r="50" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="50" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A50" s="11">
-        <v>46309</v>
+        <v>46310</v>
       </c>
       <c r="B50" s="12"/>
       <c r="C50" s="21" t="s">
         <v>30</v>
       </c>
       <c r="D50" s="13">
-        <v>253.72</v>
+        <v>253.42</v>
       </c>
       <c r="E50" s="13">
-        <v>237.98</v>
+        <v>235.77</v>
       </c>
       <c r="F50" s="13">
-        <v>247.98</v>
+        <v>245.77</v>
       </c>
       <c r="G50" s="28"/>
     </row>
-    <row r="51" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="51" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A51" s="7">
-        <v>46308</v>
+        <v>46309</v>
       </c>
       <c r="B51" s="8"/>
       <c r="C51" s="20" t="s">
         <v>29</v>
       </c>
       <c r="D51" s="10">
-        <v>257.98</v>
+        <v>256.23</v>
       </c>
       <c r="E51" s="10">
-        <v>240.01</v>
+        <v>238.37</v>
       </c>
       <c r="F51" s="10">
-        <v>250.01</v>
+        <v>248.37</v>
       </c>
       <c r="G51" s="17"/>
     </row>
-    <row r="52" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="52" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A52" s="11">
-        <v>46308</v>
+        <v>46309</v>
       </c>
       <c r="B52" s="12"/>
       <c r="C52" s="21" t="s">
         <v>30</v>
       </c>
       <c r="D52" s="13">
-        <v>255.47</v>
+        <v>253.72</v>
       </c>
       <c r="E52" s="13">
-        <v>239.62</v>
+        <v>237.98</v>
       </c>
       <c r="F52" s="13">
-        <v>249.62</v>
+        <v>247.98</v>
       </c>
       <c r="G52" s="17"/>
     </row>
-    <row r="53" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="53" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A53" s="14"/>
       <c r="B53" s="14"/>
       <c r="C53" s="15"/>
@@ -1614,7 +1614,7 @@
       <c r="F53" s="16"/>
       <c r="G53" s="17"/>
     </row>
-    <row r="54" spans="1:7" ht="20.25" x14ac:dyDescent="0.25">
+    <row r="54" spans="1:7" ht="20" x14ac:dyDescent="0.35">
       <c r="A54" s="27" t="s">
         <v>31</v>
       </c>
@@ -1625,7 +1625,7 @@
       <c r="F54" s="17"/>
       <c r="G54" s="17"/>
     </row>
-    <row r="55" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="55" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A55" s="23" t="s">
         <v>4</v>
       </c>
@@ -1644,54 +1644,54 @@
       </c>
       <c r="G55" s="17"/>
     </row>
-    <row r="56" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="56" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A56" s="7">
-        <v>46309</v>
+        <v>46310</v>
       </c>
       <c r="B56" s="8"/>
       <c r="C56" s="20" t="s">
         <v>32</v>
       </c>
       <c r="D56" s="10">
-        <v>268.86</v>
+        <v>270.08</v>
       </c>
       <c r="E56" s="10">
-        <v>263.64999999999998</v>
+        <v>261.08999999999997</v>
       </c>
       <c r="F56" s="10">
-        <v>273.64999999999998</v>
+        <v>271.08999999999997</v>
       </c>
       <c r="G56" s="17"/>
     </row>
-    <row r="57" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="57" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A57" s="11">
-        <v>46309</v>
+        <v>46310</v>
       </c>
       <c r="B57" s="12"/>
       <c r="C57" s="21" t="s">
         <v>33</v>
       </c>
       <c r="D57" s="13">
-        <v>258.82</v>
+        <v>258.04000000000002</v>
       </c>
       <c r="E57" s="13">
-        <v>245.03</v>
+        <v>242.67</v>
       </c>
       <c r="F57" s="13">
-        <v>255.03</v>
+        <v>252.67</v>
       </c>
       <c r="G57" s="17"/>
     </row>
-    <row r="58" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="58" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A58" s="7">
-        <v>46309</v>
+        <v>46310</v>
       </c>
       <c r="B58" s="8"/>
       <c r="C58" s="20" t="s">
         <v>34</v>
       </c>
       <c r="D58" s="10">
-        <v>259.70999999999998</v>
+        <v>258.81</v>
       </c>
       <c r="E58" s="10" t="s">
         <v>18</v>
@@ -1701,111 +1701,111 @@
       </c>
       <c r="G58" s="17"/>
     </row>
-    <row r="59" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="59" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A59" s="11">
-        <v>46309</v>
+        <v>46310</v>
       </c>
       <c r="B59" s="12"/>
       <c r="C59" s="21" t="s">
         <v>35</v>
       </c>
       <c r="D59" s="13">
-        <v>253.87</v>
+        <v>255.11</v>
       </c>
       <c r="E59" s="13">
-        <v>239.4</v>
+        <v>237.04</v>
       </c>
       <c r="F59" s="13" t="s">
         <v>18</v>
       </c>
       <c r="G59" s="17"/>
     </row>
-    <row r="60" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="60" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A60" s="7">
-        <v>46309</v>
+        <v>46310</v>
       </c>
       <c r="B60" s="8"/>
       <c r="C60" s="20" t="s">
         <v>36</v>
       </c>
       <c r="D60" s="10">
-        <v>249.69</v>
+        <v>250.94</v>
       </c>
       <c r="E60" s="10">
-        <v>235.35</v>
+        <v>232.99</v>
       </c>
       <c r="F60" s="10">
-        <v>245.35</v>
+        <v>242.99</v>
       </c>
       <c r="G60" s="17"/>
     </row>
-    <row r="61" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="61" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A61" s="11">
-        <v>46309</v>
+        <v>46310</v>
       </c>
       <c r="B61" s="12"/>
       <c r="C61" s="21" t="s">
         <v>37</v>
       </c>
       <c r="D61" s="13">
-        <v>256.72000000000003</v>
+        <v>257.95999999999998</v>
       </c>
       <c r="E61" s="13">
-        <v>256.99</v>
+        <v>254.49</v>
       </c>
       <c r="F61" s="13" t="s">
         <v>18</v>
       </c>
       <c r="G61" s="17"/>
     </row>
-    <row r="62" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="62" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A62" s="7">
-        <v>46308</v>
+        <v>46309</v>
       </c>
       <c r="B62" s="8"/>
       <c r="C62" s="20" t="s">
         <v>32</v>
       </c>
       <c r="D62" s="10">
-        <v>269.35000000000002</v>
+        <v>268.86</v>
       </c>
       <c r="E62" s="10">
-        <v>265.16000000000003</v>
+        <v>263.64999999999998</v>
       </c>
       <c r="F62" s="10">
-        <v>275.16000000000003</v>
+        <v>273.64999999999998</v>
       </c>
       <c r="G62" s="17"/>
     </row>
-    <row r="63" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="63" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A63" s="11">
-        <v>46308</v>
+        <v>46309</v>
       </c>
       <c r="B63" s="12"/>
       <c r="C63" s="21" t="s">
         <v>33</v>
       </c>
       <c r="D63" s="13">
-        <v>259.32</v>
+        <v>258.82</v>
       </c>
       <c r="E63" s="13">
-        <v>246.32</v>
+        <v>245.03</v>
       </c>
       <c r="F63" s="13">
-        <v>256.32</v>
+        <v>255.03</v>
       </c>
       <c r="G63" s="17"/>
     </row>
-    <row r="64" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="64" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A64" s="7">
-        <v>46308</v>
+        <v>46309</v>
       </c>
       <c r="B64" s="8"/>
       <c r="C64" s="20" t="s">
         <v>34</v>
       </c>
       <c r="D64" s="10">
-        <v>260.20999999999998</v>
+        <v>259.70999999999998</v>
       </c>
       <c r="E64" s="10" t="s">
         <v>18</v>
@@ -1815,55 +1815,55 @@
       </c>
       <c r="G64" s="17"/>
     </row>
-    <row r="65" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="65" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A65" s="11">
-        <v>46308</v>
+        <v>46309</v>
       </c>
       <c r="B65" s="12"/>
       <c r="C65" s="21" t="s">
         <v>35</v>
       </c>
       <c r="D65" s="13">
-        <v>256.51</v>
+        <v>253.87</v>
       </c>
       <c r="E65" s="13">
-        <v>240.69</v>
+        <v>239.4</v>
       </c>
       <c r="F65" s="13" t="s">
         <v>18</v>
       </c>
     </row>
-    <row r="66" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="66" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A66" s="7">
-        <v>46308</v>
+        <v>46309</v>
       </c>
       <c r="B66" s="8"/>
       <c r="C66" s="20" t="s">
         <v>36</v>
       </c>
       <c r="D66" s="10">
-        <v>252.34</v>
+        <v>249.69</v>
       </c>
       <c r="E66" s="10">
-        <v>236.64</v>
+        <v>235.35</v>
       </c>
       <c r="F66" s="10">
-        <v>246.64</v>
-      </c>
-    </row>
-    <row r="67" spans="1:6" x14ac:dyDescent="0.25">
+        <v>245.35</v>
+      </c>
+    </row>
+    <row r="67" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A67" s="11">
-        <v>46308</v>
+        <v>46309</v>
       </c>
       <c r="B67" s="12"/>
       <c r="C67" s="21" t="s">
         <v>37</v>
       </c>
       <c r="D67" s="13">
-        <v>257.17</v>
+        <v>256.72000000000003</v>
       </c>
       <c r="E67" s="13">
-        <v>258.42</v>
+        <v>256.99</v>
       </c>
       <c r="F67" s="13" t="s">
         <v>18</v>

</xml_diff>

<commit_message>
Thu Oct 15 05:57:48 UTC 2026
</commit_message>
<xml_diff>
--- a/bp.com-content-dam-bp-country-sites-en_au-australia-home-products-services-pricing-tgp-excel.xlsx
+++ b/bp.com-content-dam-bp-country-sites-en_au-australia-home-products-services-pricing-tgp-excel.xlsx
@@ -8,14 +8,14 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://bp365.sharepoint.com/sites/WholesalePricing/Shared Documents/B2C/TGP/Daily TGP/Web TGP/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="14_{93C8CB39-39FD-484F-8341-7F8554D23B25}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="14_{FD13E0C4-DF32-43D8-AB1B-C62894DC1629}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-110" yWindow="-110" windowWidth="19420" windowHeight="11500" xr2:uid="{1B412EEF-F96D-4DF4-A4E9-C7F0F183C2FB}"/>
+    <workbookView xWindow="-8595" yWindow="-16320" windowWidth="29040" windowHeight="15720" xr2:uid="{1B412EEF-F96D-4DF4-A4E9-C7F0F183C2FB}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
   </sheets>
-  <calcPr calcId="191028"/>
+  <calcPr calcId="191028" concurrentManualCount="12"/>
   <extLst>
     <ext xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" uri="{140A7094-0E35-4892-8432-C4D2E57EDEB5}">
       <x15:workbookPr chartTrackingRefBase="1"/>
@@ -715,15 +715,15 @@
     <pageSetUpPr fitToPage="1"/>
   </sheetPr>
   <dimension ref="A1:G67"/>
-  <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
+  <sheetFormatPr defaultRowHeight="14.25" x14ac:dyDescent="0.45"/>
   <cols>
-    <col min="1" max="1" width="76.453125" bestFit="1" customWidth="1"/>
-    <col min="2" max="2" width="6.453125"/>
-    <col min="3" max="3" width="18.1796875" bestFit="1" customWidth="1"/>
-    <col min="4" max="7" width="7.1796875" bestFit="1" customWidth="1"/>
+    <col min="1" max="1" width="76.46484375" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="6.46484375"/>
+    <col min="3" max="3" width="18.19921875" bestFit="1" customWidth="1"/>
+    <col min="4" max="7" width="7.19921875" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:7" ht="22.5" x14ac:dyDescent="0.35">
+    <row r="1" spans="1:7" ht="22.15" x14ac:dyDescent="0.45">
       <c r="A1" s="30" t="s">
         <v>0</v>
       </c>
@@ -734,7 +734,7 @@
       <c r="F1" s="2"/>
       <c r="G1" s="2"/>
     </row>
-    <row r="2" spans="1:7" x14ac:dyDescent="0.35">
+    <row r="2" spans="1:7" x14ac:dyDescent="0.45">
       <c r="A2" s="3"/>
       <c r="B2" s="1"/>
       <c r="C2" s="1"/>
@@ -743,7 +743,7 @@
       <c r="F2" s="2"/>
       <c r="G2" s="2"/>
     </row>
-    <row r="3" spans="1:7" x14ac:dyDescent="0.35">
+    <row r="3" spans="1:7" x14ac:dyDescent="0.45">
       <c r="A3" s="3" t="s">
         <v>1</v>
       </c>
@@ -754,7 +754,7 @@
       <c r="F3" s="2"/>
       <c r="G3" s="2"/>
     </row>
-    <row r="4" spans="1:7" x14ac:dyDescent="0.35">
+    <row r="4" spans="1:7" x14ac:dyDescent="0.45">
       <c r="A4" s="3" t="s">
         <v>2</v>
       </c>
@@ -765,7 +765,7 @@
       <c r="F4" s="2"/>
       <c r="G4" s="2"/>
     </row>
-    <row r="5" spans="1:7" x14ac:dyDescent="0.35">
+    <row r="5" spans="1:7" x14ac:dyDescent="0.45">
       <c r="A5" s="3"/>
       <c r="B5" s="3"/>
       <c r="C5" s="1"/>
@@ -774,7 +774,7 @@
       <c r="F5" s="2"/>
       <c r="G5" s="2"/>
     </row>
-    <row r="6" spans="1:7" ht="20" x14ac:dyDescent="0.35">
+    <row r="6" spans="1:7" ht="20.25" x14ac:dyDescent="0.45">
       <c r="A6" s="29" t="s">
         <v>3</v>
       </c>
@@ -785,7 +785,7 @@
       <c r="F6" s="2"/>
       <c r="G6" s="2"/>
     </row>
-    <row r="7" spans="1:7" x14ac:dyDescent="0.35">
+    <row r="7" spans="1:7" x14ac:dyDescent="0.45">
       <c r="A7" s="4" t="s">
         <v>4</v>
       </c>
@@ -806,133 +806,133 @@
         <v>9</v>
       </c>
     </row>
-    <row r="8" spans="1:7" x14ac:dyDescent="0.35">
+    <row r="8" spans="1:7" x14ac:dyDescent="0.45">
       <c r="A8" s="7">
-        <v>46310</v>
+        <v>46311</v>
       </c>
       <c r="B8" s="8"/>
       <c r="C8" s="9" t="s">
         <v>10</v>
       </c>
       <c r="D8" s="10">
-        <v>257.98</v>
+        <v>259.11</v>
       </c>
       <c r="E8" s="10">
-        <v>233.92</v>
+        <v>231.51</v>
       </c>
       <c r="F8" s="10">
-        <v>243.92</v>
+        <v>241.51</v>
       </c>
       <c r="G8" s="10">
-        <v>231.54</v>
-      </c>
-    </row>
-    <row r="9" spans="1:7" x14ac:dyDescent="0.35">
+        <v>229.13</v>
+      </c>
+    </row>
+    <row r="9" spans="1:7" x14ac:dyDescent="0.45">
       <c r="A9" s="11">
-        <v>46310</v>
+        <v>46311</v>
       </c>
       <c r="B9" s="12"/>
       <c r="C9" s="12" t="s">
         <v>11</v>
       </c>
       <c r="D9" s="13">
-        <v>257.98</v>
+        <v>259.11</v>
       </c>
       <c r="E9" s="13">
-        <v>233.92</v>
+        <v>231.51</v>
       </c>
       <c r="F9" s="13">
-        <v>243.92</v>
+        <v>241.51</v>
       </c>
       <c r="G9" s="13">
-        <v>231.54</v>
-      </c>
-    </row>
-    <row r="10" spans="1:7" x14ac:dyDescent="0.35">
+        <v>229.13</v>
+      </c>
+    </row>
+    <row r="10" spans="1:7" x14ac:dyDescent="0.45">
       <c r="A10" s="7">
-        <v>46310</v>
+        <v>46311</v>
       </c>
       <c r="B10" s="8"/>
       <c r="C10" s="9" t="s">
         <v>12</v>
       </c>
       <c r="D10" s="10">
-        <v>255.39</v>
+        <v>256.52</v>
       </c>
       <c r="E10" s="10">
-        <v>232.3</v>
+        <v>229.39</v>
       </c>
       <c r="F10" s="10">
-        <v>242.3</v>
+        <v>239.39</v>
       </c>
       <c r="G10" s="10">
-        <v>230.71</v>
-      </c>
-    </row>
-    <row r="11" spans="1:7" x14ac:dyDescent="0.35">
+        <v>227.79</v>
+      </c>
+    </row>
+    <row r="11" spans="1:7" x14ac:dyDescent="0.45">
       <c r="A11" s="11">
-        <v>46309</v>
+        <v>46310</v>
       </c>
       <c r="B11" s="12"/>
       <c r="C11" s="12" t="s">
         <v>10</v>
       </c>
       <c r="D11" s="13">
-        <v>258.49</v>
+        <v>257.98</v>
       </c>
       <c r="E11" s="13">
-        <v>236.44</v>
+        <v>233.92</v>
       </c>
       <c r="F11" s="13">
-        <v>246.44</v>
+        <v>243.92</v>
       </c>
       <c r="G11" s="13">
-        <v>234.05</v>
-      </c>
-    </row>
-    <row r="12" spans="1:7" x14ac:dyDescent="0.35">
+        <v>231.54</v>
+      </c>
+    </row>
+    <row r="12" spans="1:7" x14ac:dyDescent="0.45">
       <c r="A12" s="7">
-        <v>46309</v>
+        <v>46310</v>
       </c>
       <c r="B12" s="8"/>
       <c r="C12" s="9" t="s">
         <v>11</v>
       </c>
       <c r="D12" s="10">
-        <v>258.49</v>
+        <v>257.98</v>
       </c>
       <c r="E12" s="10">
-        <v>236.44</v>
+        <v>233.92</v>
       </c>
       <c r="F12" s="10">
-        <v>246.44</v>
+        <v>243.92</v>
       </c>
       <c r="G12" s="10">
-        <v>234.05</v>
-      </c>
-    </row>
-    <row r="13" spans="1:7" x14ac:dyDescent="0.35">
+        <v>231.54</v>
+      </c>
+    </row>
+    <row r="13" spans="1:7" x14ac:dyDescent="0.45">
       <c r="A13" s="11">
-        <v>46309</v>
+        <v>46310</v>
       </c>
       <c r="B13" s="12"/>
       <c r="C13" s="12" t="s">
         <v>12</v>
       </c>
       <c r="D13" s="13">
-        <v>254.19</v>
+        <v>255.39</v>
       </c>
       <c r="E13" s="13">
-        <v>234.71</v>
+        <v>232.3</v>
       </c>
       <c r="F13" s="13">
-        <v>244.71</v>
+        <v>242.3</v>
       </c>
       <c r="G13" s="13">
-        <v>233.11</v>
-      </c>
-    </row>
-    <row r="14" spans="1:7" x14ac:dyDescent="0.35">
+        <v>230.71</v>
+      </c>
+    </row>
+    <row r="14" spans="1:7" x14ac:dyDescent="0.45">
       <c r="A14" s="14"/>
       <c r="B14" s="14"/>
       <c r="C14" s="15"/>
@@ -941,7 +941,7 @@
       <c r="F14" s="16"/>
       <c r="G14" s="16"/>
     </row>
-    <row r="15" spans="1:7" ht="20" x14ac:dyDescent="0.35">
+    <row r="15" spans="1:7" ht="20.25" x14ac:dyDescent="0.45">
       <c r="A15" s="29" t="s">
         <v>13</v>
       </c>
@@ -952,7 +952,7 @@
       <c r="F15" s="17"/>
       <c r="G15" s="17"/>
     </row>
-    <row r="16" spans="1:7" x14ac:dyDescent="0.35">
+    <row r="16" spans="1:7" x14ac:dyDescent="0.45">
       <c r="A16" s="4" t="s">
         <v>4</v>
       </c>
@@ -971,45 +971,45 @@
       </c>
       <c r="G16" s="17"/>
     </row>
-    <row r="17" spans="1:7" x14ac:dyDescent="0.35">
+    <row r="17" spans="1:7" x14ac:dyDescent="0.45">
       <c r="A17" s="7">
-        <v>46310</v>
+        <v>46311</v>
       </c>
       <c r="B17" s="8"/>
       <c r="C17" s="20" t="s">
         <v>14</v>
       </c>
       <c r="D17" s="10">
-        <v>258.87</v>
+        <v>260.04000000000002</v>
       </c>
       <c r="E17" s="10">
-        <v>237.5</v>
+        <v>234.62</v>
       </c>
       <c r="F17" s="10">
-        <v>247.5</v>
+        <v>244.62</v>
       </c>
       <c r="G17" s="17"/>
     </row>
-    <row r="18" spans="1:7" x14ac:dyDescent="0.35">
+    <row r="18" spans="1:7" x14ac:dyDescent="0.45">
       <c r="A18" s="11">
-        <v>46309</v>
+        <v>46310</v>
       </c>
       <c r="B18" s="12"/>
       <c r="C18" s="12" t="s">
         <v>14</v>
       </c>
       <c r="D18" s="13">
-        <v>257.64</v>
+        <v>258.87</v>
       </c>
       <c r="E18" s="13">
-        <v>239.88</v>
+        <v>237.5</v>
       </c>
       <c r="F18" s="13">
-        <v>249.88</v>
+        <v>247.5</v>
       </c>
       <c r="G18" s="17"/>
     </row>
-    <row r="19" spans="1:7" x14ac:dyDescent="0.35">
+    <row r="19" spans="1:7" x14ac:dyDescent="0.45">
       <c r="A19" s="14"/>
       <c r="B19" s="14"/>
       <c r="C19" s="15"/>
@@ -1018,7 +1018,7 @@
       <c r="F19" s="16"/>
       <c r="G19" s="17"/>
     </row>
-    <row r="20" spans="1:7" ht="20" x14ac:dyDescent="0.35">
+    <row r="20" spans="1:7" ht="20.25" x14ac:dyDescent="0.45">
       <c r="A20" s="29" t="s">
         <v>15</v>
       </c>
@@ -1029,7 +1029,7 @@
       <c r="F20" s="17"/>
       <c r="G20" s="17"/>
     </row>
-    <row r="21" spans="1:7" x14ac:dyDescent="0.35">
+    <row r="21" spans="1:7" x14ac:dyDescent="0.45">
       <c r="A21" s="4" t="s">
         <v>4</v>
       </c>
@@ -1050,217 +1050,217 @@
         <v>9</v>
       </c>
     </row>
-    <row r="22" spans="1:7" x14ac:dyDescent="0.35">
+    <row r="22" spans="1:7" x14ac:dyDescent="0.45">
       <c r="A22" s="7">
-        <v>46310</v>
+        <v>46311</v>
       </c>
       <c r="B22" s="8"/>
       <c r="C22" s="20" t="s">
         <v>16</v>
       </c>
       <c r="D22" s="10">
-        <v>259.10000000000002</v>
+        <v>260.23</v>
       </c>
       <c r="E22" s="10">
-        <v>234.06</v>
+        <v>231.65</v>
       </c>
       <c r="F22" s="10">
-        <v>243.66</v>
+        <v>241.25</v>
       </c>
       <c r="G22" s="10">
-        <v>230.43</v>
-      </c>
-    </row>
-    <row r="23" spans="1:7" x14ac:dyDescent="0.35">
+        <v>228.02</v>
+      </c>
+    </row>
+    <row r="23" spans="1:7" x14ac:dyDescent="0.45">
       <c r="A23" s="11">
-        <v>46310</v>
+        <v>46311</v>
       </c>
       <c r="B23" s="12"/>
       <c r="C23" s="21" t="s">
         <v>17</v>
       </c>
       <c r="D23" s="13">
-        <v>260.33999999999997</v>
+        <v>261.45999999999998</v>
       </c>
       <c r="E23" s="13">
-        <v>242.79</v>
+        <v>239.85</v>
       </c>
       <c r="F23" s="13">
-        <v>252.79</v>
+        <v>249.85</v>
       </c>
       <c r="G23" s="13" t="s">
         <v>18</v>
       </c>
     </row>
-    <row r="24" spans="1:7" x14ac:dyDescent="0.35">
+    <row r="24" spans="1:7" x14ac:dyDescent="0.45">
       <c r="A24" s="7">
-        <v>46310</v>
+        <v>46311</v>
       </c>
       <c r="B24" s="8"/>
       <c r="C24" s="20" t="s">
         <v>19</v>
       </c>
       <c r="D24" s="10">
-        <v>260.7</v>
+        <v>261.82</v>
       </c>
       <c r="E24" s="10">
-        <v>242.03</v>
+        <v>239.09</v>
       </c>
       <c r="F24" s="10">
-        <v>252.03</v>
+        <v>249.1</v>
       </c>
       <c r="G24" s="10" t="s">
         <v>18</v>
       </c>
     </row>
-    <row r="25" spans="1:7" x14ac:dyDescent="0.35">
+    <row r="25" spans="1:7" x14ac:dyDescent="0.45">
       <c r="A25" s="11">
-        <v>46310</v>
+        <v>46311</v>
       </c>
       <c r="B25" s="12"/>
       <c r="C25" s="21" t="s">
         <v>20</v>
       </c>
       <c r="D25" s="13">
-        <v>257.36</v>
+        <v>258.49</v>
       </c>
       <c r="E25" s="13">
-        <v>242.26</v>
+        <v>239.32</v>
       </c>
       <c r="F25" s="13">
-        <v>252.26</v>
+        <v>249.32</v>
       </c>
       <c r="G25" s="13">
-        <v>238.1</v>
-      </c>
-    </row>
-    <row r="26" spans="1:7" x14ac:dyDescent="0.35">
+        <v>235.16</v>
+      </c>
+    </row>
+    <row r="26" spans="1:7" x14ac:dyDescent="0.45">
       <c r="A26" s="7">
-        <v>46310</v>
+        <v>46311</v>
       </c>
       <c r="B26" s="8"/>
       <c r="C26" s="20" t="s">
         <v>21</v>
       </c>
       <c r="D26" s="10">
-        <v>258.91000000000003</v>
+        <v>260.05</v>
       </c>
       <c r="E26" s="10">
-        <v>243.78</v>
+        <v>240.81</v>
       </c>
       <c r="F26" s="10">
-        <v>253.78</v>
+        <v>250.81</v>
       </c>
       <c r="G26" s="10" t="s">
         <v>18</v>
       </c>
     </row>
-    <row r="27" spans="1:7" x14ac:dyDescent="0.35">
+    <row r="27" spans="1:7" x14ac:dyDescent="0.45">
       <c r="A27" s="11">
-        <v>46309</v>
+        <v>46310</v>
       </c>
       <c r="B27" s="12"/>
       <c r="C27" s="12" t="s">
         <v>16</v>
       </c>
       <c r="D27" s="13">
-        <v>259.62</v>
+        <v>259.10000000000002</v>
       </c>
       <c r="E27" s="13">
-        <v>237.12</v>
+        <v>234.06</v>
       </c>
       <c r="F27" s="13">
-        <v>246.72</v>
+        <v>243.66</v>
       </c>
       <c r="G27" s="13">
-        <v>233.49</v>
-      </c>
-    </row>
-    <row r="28" spans="1:7" x14ac:dyDescent="0.35">
+        <v>230.43</v>
+      </c>
+    </row>
+    <row r="28" spans="1:7" x14ac:dyDescent="0.45">
       <c r="A28" s="7">
-        <v>46309</v>
+        <v>46310</v>
       </c>
       <c r="B28" s="8"/>
       <c r="C28" s="20" t="s">
         <v>17</v>
       </c>
       <c r="D28" s="10">
-        <v>259.14999999999998</v>
+        <v>260.33999999999997</v>
       </c>
       <c r="E28" s="22">
-        <v>245.21</v>
+        <v>242.79</v>
       </c>
       <c r="F28" s="22">
-        <v>255.21</v>
+        <v>252.79</v>
       </c>
       <c r="G28" s="22" t="s">
         <v>18</v>
       </c>
     </row>
-    <row r="29" spans="1:7" x14ac:dyDescent="0.35">
+    <row r="29" spans="1:7" x14ac:dyDescent="0.45">
       <c r="A29" s="11">
-        <v>46309</v>
+        <v>46310</v>
       </c>
       <c r="B29" s="12"/>
       <c r="C29" s="12" t="s">
         <v>19</v>
       </c>
       <c r="D29" s="13">
-        <v>259.5</v>
+        <v>260.7</v>
       </c>
       <c r="E29" s="13">
-        <v>244.45</v>
+        <v>242.03</v>
       </c>
       <c r="F29" s="13">
-        <v>254.45</v>
+        <v>252.03</v>
       </c>
       <c r="G29" s="13" t="s">
         <v>18</v>
       </c>
     </row>
-    <row r="30" spans="1:7" x14ac:dyDescent="0.35">
+    <row r="30" spans="1:7" x14ac:dyDescent="0.45">
       <c r="A30" s="7">
-        <v>46309</v>
+        <v>46310</v>
       </c>
       <c r="B30" s="8"/>
       <c r="C30" s="20" t="s">
         <v>20</v>
       </c>
       <c r="D30" s="10">
-        <v>256.16000000000003</v>
+        <v>257.36</v>
       </c>
       <c r="E30" s="22">
-        <v>244.69</v>
+        <v>242.26</v>
       </c>
       <c r="F30" s="22">
-        <v>254.69</v>
+        <v>252.26</v>
       </c>
       <c r="G30" s="22">
-        <v>240.53</v>
-      </c>
-    </row>
-    <row r="31" spans="1:7" x14ac:dyDescent="0.35">
+        <v>238.1</v>
+      </c>
+    </row>
+    <row r="31" spans="1:7" x14ac:dyDescent="0.45">
       <c r="A31" s="11">
-        <v>46309</v>
+        <v>46310</v>
       </c>
       <c r="B31" s="12"/>
       <c r="C31" s="12" t="s">
         <v>21</v>
       </c>
       <c r="D31" s="13">
-        <v>257.7</v>
+        <v>258.91000000000003</v>
       </c>
       <c r="E31" s="13">
-        <v>246.23</v>
+        <v>243.78</v>
       </c>
       <c r="F31" s="13">
-        <v>256.23</v>
+        <v>253.78</v>
       </c>
       <c r="G31" s="13" t="s">
         <v>18</v>
       </c>
     </row>
-    <row r="32" spans="1:7" x14ac:dyDescent="0.35">
+    <row r="32" spans="1:7" x14ac:dyDescent="0.45">
       <c r="A32" s="14"/>
       <c r="B32" s="14"/>
       <c r="C32" s="15"/>
@@ -1269,7 +1269,7 @@
       <c r="F32" s="17"/>
       <c r="G32" s="17"/>
     </row>
-    <row r="33" spans="1:7" ht="20" x14ac:dyDescent="0.35">
+    <row r="33" spans="1:7" ht="20.25" x14ac:dyDescent="0.45">
       <c r="A33" s="29" t="s">
         <v>22</v>
       </c>
@@ -1280,7 +1280,7 @@
       <c r="F33" s="17"/>
       <c r="G33" s="17"/>
     </row>
-    <row r="34" spans="1:7" x14ac:dyDescent="0.35">
+    <row r="34" spans="1:7" x14ac:dyDescent="0.45">
       <c r="A34" s="23" t="s">
         <v>4</v>
       </c>
@@ -1299,54 +1299,54 @@
       </c>
       <c r="G34" s="17"/>
     </row>
-    <row r="35" spans="1:7" x14ac:dyDescent="0.35">
+    <row r="35" spans="1:7" x14ac:dyDescent="0.45">
       <c r="A35" s="7">
-        <v>46310</v>
+        <v>46311</v>
       </c>
       <c r="B35" s="8"/>
       <c r="C35" s="20" t="s">
         <v>23</v>
       </c>
       <c r="D35" s="10">
-        <v>253.94</v>
+        <v>255.06</v>
       </c>
       <c r="E35" s="10">
-        <v>231.24</v>
+        <v>229.42</v>
       </c>
       <c r="F35" s="10">
-        <v>240.24</v>
+        <v>238.42</v>
       </c>
       <c r="G35" s="17"/>
     </row>
-    <row r="36" spans="1:7" x14ac:dyDescent="0.35">
+    <row r="36" spans="1:7" x14ac:dyDescent="0.45">
       <c r="A36" s="11">
-        <v>46309</v>
+        <v>46310</v>
       </c>
       <c r="B36" s="12"/>
       <c r="C36" s="12" t="s">
         <v>23</v>
       </c>
       <c r="D36" s="13">
-        <v>252.75</v>
+        <v>253.94</v>
       </c>
       <c r="E36" s="13">
-        <v>233.09</v>
+        <v>231.24</v>
       </c>
       <c r="F36" s="13">
-        <v>242.09</v>
+        <v>240.24</v>
       </c>
       <c r="G36" s="17"/>
     </row>
-    <row r="37" spans="1:7" x14ac:dyDescent="0.35">
+    <row r="37" spans="1:7" x14ac:dyDescent="0.45">
       <c r="A37" s="7">
-        <v>46310</v>
+        <v>46311</v>
       </c>
       <c r="B37" s="8"/>
       <c r="C37" s="20" t="s">
         <v>24</v>
       </c>
       <c r="D37" s="10">
-        <v>269.56</v>
+        <v>270.68</v>
       </c>
       <c r="E37" s="10" t="s">
         <v>18</v>
@@ -1356,16 +1356,16 @@
       </c>
       <c r="G37" s="17"/>
     </row>
-    <row r="38" spans="1:7" x14ac:dyDescent="0.35">
+    <row r="38" spans="1:7" x14ac:dyDescent="0.45">
       <c r="A38" s="11">
-        <v>46309</v>
+        <v>46310</v>
       </c>
       <c r="B38" s="12"/>
       <c r="C38" s="12" t="s">
         <v>24</v>
       </c>
       <c r="D38" s="13">
-        <v>268.37</v>
+        <v>269.56</v>
       </c>
       <c r="E38" s="13" t="s">
         <v>18</v>
@@ -1375,7 +1375,7 @@
       </c>
       <c r="G38" s="17"/>
     </row>
-    <row r="39" spans="1:7" x14ac:dyDescent="0.35">
+    <row r="39" spans="1:7" x14ac:dyDescent="0.45">
       <c r="A39" s="24"/>
       <c r="B39" s="24"/>
       <c r="C39" s="15"/>
@@ -1384,7 +1384,7 @@
       <c r="F39" s="17"/>
       <c r="G39" s="17"/>
     </row>
-    <row r="40" spans="1:7" ht="20" x14ac:dyDescent="0.35">
+    <row r="40" spans="1:7" ht="20.25" x14ac:dyDescent="0.45">
       <c r="A40" s="29" t="s">
         <v>25</v>
       </c>
@@ -1395,7 +1395,7 @@
       <c r="F40" s="17"/>
       <c r="G40" s="17"/>
     </row>
-    <row r="41" spans="1:7" x14ac:dyDescent="0.35">
+    <row r="41" spans="1:7" x14ac:dyDescent="0.45">
       <c r="A41" s="23" t="s">
         <v>4</v>
       </c>
@@ -1414,83 +1414,83 @@
       </c>
       <c r="G41" s="17"/>
     </row>
-    <row r="42" spans="1:7" x14ac:dyDescent="0.35">
+    <row r="42" spans="1:7" x14ac:dyDescent="0.45">
       <c r="A42" s="7">
-        <v>46310</v>
+        <v>46311</v>
       </c>
       <c r="B42" s="8"/>
       <c r="C42" s="20" t="s">
         <v>26</v>
       </c>
       <c r="D42" s="10">
-        <v>263.94</v>
+        <v>265.02999999999997</v>
       </c>
       <c r="E42" s="10">
-        <v>241.39</v>
+        <v>239.37</v>
       </c>
       <c r="F42" s="10">
-        <v>251.39</v>
+        <v>249.37</v>
       </c>
       <c r="G42" s="17"/>
     </row>
-    <row r="43" spans="1:7" x14ac:dyDescent="0.35">
+    <row r="43" spans="1:7" x14ac:dyDescent="0.45">
       <c r="A43" s="11">
-        <v>46310</v>
+        <v>46311</v>
       </c>
       <c r="B43" s="12"/>
       <c r="C43" s="21" t="s">
         <v>27</v>
       </c>
       <c r="D43" s="13">
-        <v>263.55</v>
+        <v>264.64</v>
       </c>
       <c r="E43" s="13">
-        <v>241.8</v>
+        <v>239.78</v>
       </c>
       <c r="F43" s="13">
-        <v>251.8</v>
+        <v>249.78</v>
       </c>
       <c r="G43" s="17"/>
     </row>
-    <row r="44" spans="1:7" x14ac:dyDescent="0.35">
+    <row r="44" spans="1:7" x14ac:dyDescent="0.45">
       <c r="A44" s="7">
-        <v>46309</v>
+        <v>46310</v>
       </c>
       <c r="B44" s="8"/>
       <c r="C44" s="20" t="s">
         <v>26</v>
       </c>
       <c r="D44" s="10">
-        <v>262.77</v>
+        <v>263.94</v>
       </c>
       <c r="E44" s="10">
-        <v>242.85</v>
+        <v>241.39</v>
       </c>
       <c r="F44" s="10">
-        <v>252.85</v>
+        <v>251.39</v>
       </c>
       <c r="G44" s="17"/>
     </row>
-    <row r="45" spans="1:7" x14ac:dyDescent="0.35">
+    <row r="45" spans="1:7" x14ac:dyDescent="0.45">
       <c r="A45" s="11">
-        <v>46309</v>
+        <v>46310</v>
       </c>
       <c r="B45" s="12"/>
       <c r="C45" s="21" t="s">
         <v>27</v>
       </c>
       <c r="D45" s="13">
-        <v>262.38</v>
+        <v>263.55</v>
       </c>
       <c r="E45" s="13">
-        <v>243.26</v>
+        <v>241.8</v>
       </c>
       <c r="F45" s="13">
-        <v>253.26</v>
+        <v>251.8</v>
       </c>
       <c r="G45" s="17"/>
     </row>
-    <row r="46" spans="1:7" x14ac:dyDescent="0.35">
+    <row r="46" spans="1:7" x14ac:dyDescent="0.45">
       <c r="A46" s="14"/>
       <c r="B46" s="24"/>
       <c r="C46" s="15"/>
@@ -1499,7 +1499,7 @@
       <c r="F46" s="16"/>
       <c r="G46" s="17"/>
     </row>
-    <row r="47" spans="1:7" ht="20" x14ac:dyDescent="0.35">
+    <row r="47" spans="1:7" ht="20.25" x14ac:dyDescent="0.45">
       <c r="A47" s="25" t="s">
         <v>28</v>
       </c>
@@ -1510,7 +1510,7 @@
       <c r="F47" s="17"/>
       <c r="G47" s="17"/>
     </row>
-    <row r="48" spans="1:7" x14ac:dyDescent="0.35">
+    <row r="48" spans="1:7" x14ac:dyDescent="0.45">
       <c r="A48" s="23" t="s">
         <v>4</v>
       </c>
@@ -1529,83 +1529,83 @@
       </c>
       <c r="G48" s="17"/>
     </row>
-    <row r="49" spans="1:7" x14ac:dyDescent="0.35">
+    <row r="49" spans="1:7" x14ac:dyDescent="0.45">
       <c r="A49" s="7">
-        <v>46310</v>
+        <v>46311</v>
       </c>
       <c r="B49" s="8"/>
       <c r="C49" s="20" t="s">
         <v>29</v>
       </c>
       <c r="D49" s="10">
-        <v>255.92</v>
+        <v>256.41000000000003</v>
       </c>
       <c r="E49" s="10">
-        <v>236.16</v>
+        <v>234.17</v>
       </c>
       <c r="F49" s="10">
-        <v>246.16</v>
+        <v>244.17</v>
       </c>
       <c r="G49" s="28"/>
     </row>
-    <row r="50" spans="1:7" x14ac:dyDescent="0.35">
+    <row r="50" spans="1:7" x14ac:dyDescent="0.45">
       <c r="A50" s="11">
-        <v>46310</v>
+        <v>46311</v>
       </c>
       <c r="B50" s="12"/>
       <c r="C50" s="21" t="s">
         <v>30</v>
       </c>
       <c r="D50" s="13">
-        <v>253.42</v>
+        <v>253.94</v>
       </c>
       <c r="E50" s="13">
-        <v>235.77</v>
+        <v>233.79</v>
       </c>
       <c r="F50" s="13">
-        <v>245.77</v>
+        <v>243.79</v>
       </c>
       <c r="G50" s="28"/>
     </row>
-    <row r="51" spans="1:7" x14ac:dyDescent="0.35">
+    <row r="51" spans="1:7" x14ac:dyDescent="0.45">
       <c r="A51" s="7">
-        <v>46309</v>
+        <v>46310</v>
       </c>
       <c r="B51" s="8"/>
       <c r="C51" s="20" t="s">
         <v>29</v>
       </c>
       <c r="D51" s="10">
-        <v>256.23</v>
+        <v>255.92</v>
       </c>
       <c r="E51" s="10">
-        <v>238.37</v>
+        <v>236.16</v>
       </c>
       <c r="F51" s="10">
-        <v>248.37</v>
+        <v>246.16</v>
       </c>
       <c r="G51" s="17"/>
     </row>
-    <row r="52" spans="1:7" x14ac:dyDescent="0.35">
+    <row r="52" spans="1:7" x14ac:dyDescent="0.45">
       <c r="A52" s="11">
-        <v>46309</v>
+        <v>46310</v>
       </c>
       <c r="B52" s="12"/>
       <c r="C52" s="21" t="s">
         <v>30</v>
       </c>
       <c r="D52" s="13">
-        <v>253.72</v>
+        <v>253.42</v>
       </c>
       <c r="E52" s="13">
-        <v>237.98</v>
+        <v>235.77</v>
       </c>
       <c r="F52" s="13">
-        <v>247.98</v>
+        <v>245.77</v>
       </c>
       <c r="G52" s="17"/>
     </row>
-    <row r="53" spans="1:7" x14ac:dyDescent="0.35">
+    <row r="53" spans="1:7" x14ac:dyDescent="0.45">
       <c r="A53" s="14"/>
       <c r="B53" s="14"/>
       <c r="C53" s="15"/>
@@ -1614,7 +1614,7 @@
       <c r="F53" s="16"/>
       <c r="G53" s="17"/>
     </row>
-    <row r="54" spans="1:7" ht="20" x14ac:dyDescent="0.35">
+    <row r="54" spans="1:7" ht="20.25" x14ac:dyDescent="0.45">
       <c r="A54" s="27" t="s">
         <v>31</v>
       </c>
@@ -1625,7 +1625,7 @@
       <c r="F54" s="17"/>
       <c r="G54" s="17"/>
     </row>
-    <row r="55" spans="1:7" x14ac:dyDescent="0.35">
+    <row r="55" spans="1:7" x14ac:dyDescent="0.45">
       <c r="A55" s="23" t="s">
         <v>4</v>
       </c>
@@ -1644,54 +1644,54 @@
       </c>
       <c r="G55" s="17"/>
     </row>
-    <row r="56" spans="1:7" x14ac:dyDescent="0.35">
+    <row r="56" spans="1:7" x14ac:dyDescent="0.45">
       <c r="A56" s="7">
-        <v>46310</v>
+        <v>46311</v>
       </c>
       <c r="B56" s="8"/>
       <c r="C56" s="20" t="s">
         <v>32</v>
       </c>
       <c r="D56" s="10">
-        <v>270.08</v>
+        <v>271.22000000000003</v>
       </c>
       <c r="E56" s="10">
-        <v>261.08999999999997</v>
+        <v>257.98</v>
       </c>
       <c r="F56" s="10">
-        <v>271.08999999999997</v>
+        <v>267.98</v>
       </c>
       <c r="G56" s="17"/>
     </row>
-    <row r="57" spans="1:7" x14ac:dyDescent="0.35">
+    <row r="57" spans="1:7" x14ac:dyDescent="0.45">
       <c r="A57" s="11">
-        <v>46310</v>
+        <v>46311</v>
       </c>
       <c r="B57" s="12"/>
       <c r="C57" s="21" t="s">
         <v>33</v>
       </c>
       <c r="D57" s="13">
-        <v>258.04000000000002</v>
+        <v>258.06</v>
       </c>
       <c r="E57" s="13">
-        <v>242.67</v>
+        <v>239.81</v>
       </c>
       <c r="F57" s="13">
-        <v>252.67</v>
+        <v>249.81</v>
       </c>
       <c r="G57" s="17"/>
     </row>
-    <row r="58" spans="1:7" x14ac:dyDescent="0.35">
+    <row r="58" spans="1:7" x14ac:dyDescent="0.45">
       <c r="A58" s="7">
-        <v>46310</v>
+        <v>46311</v>
       </c>
       <c r="B58" s="8"/>
       <c r="C58" s="20" t="s">
         <v>34</v>
       </c>
       <c r="D58" s="10">
-        <v>258.81</v>
+        <v>258.83</v>
       </c>
       <c r="E58" s="10" t="s">
         <v>18</v>
@@ -1701,111 +1701,111 @@
       </c>
       <c r="G58" s="17"/>
     </row>
-    <row r="59" spans="1:7" x14ac:dyDescent="0.35">
+    <row r="59" spans="1:7" x14ac:dyDescent="0.45">
       <c r="A59" s="11">
-        <v>46310</v>
+        <v>46311</v>
       </c>
       <c r="B59" s="12"/>
       <c r="C59" s="21" t="s">
         <v>35</v>
       </c>
       <c r="D59" s="13">
-        <v>255.11</v>
+        <v>255.19</v>
       </c>
       <c r="E59" s="13">
-        <v>237.04</v>
+        <v>234.19</v>
       </c>
       <c r="F59" s="13" t="s">
         <v>18</v>
       </c>
       <c r="G59" s="17"/>
     </row>
-    <row r="60" spans="1:7" x14ac:dyDescent="0.35">
+    <row r="60" spans="1:7" x14ac:dyDescent="0.45">
       <c r="A60" s="7">
-        <v>46310</v>
+        <v>46311</v>
       </c>
       <c r="B60" s="8"/>
       <c r="C60" s="20" t="s">
         <v>36</v>
       </c>
       <c r="D60" s="10">
-        <v>250.94</v>
+        <v>251.02</v>
       </c>
       <c r="E60" s="10">
-        <v>232.99</v>
+        <v>230.13</v>
       </c>
       <c r="F60" s="10">
-        <v>242.99</v>
+        <v>240.13</v>
       </c>
       <c r="G60" s="17"/>
     </row>
-    <row r="61" spans="1:7" x14ac:dyDescent="0.35">
+    <row r="61" spans="1:7" x14ac:dyDescent="0.45">
       <c r="A61" s="11">
-        <v>46310</v>
+        <v>46311</v>
       </c>
       <c r="B61" s="12"/>
       <c r="C61" s="21" t="s">
         <v>37</v>
       </c>
       <c r="D61" s="13">
-        <v>257.95999999999998</v>
+        <v>259.14999999999998</v>
       </c>
       <c r="E61" s="13">
-        <v>254.49</v>
+        <v>251.46</v>
       </c>
       <c r="F61" s="13" t="s">
         <v>18</v>
       </c>
       <c r="G61" s="17"/>
     </row>
-    <row r="62" spans="1:7" x14ac:dyDescent="0.35">
+    <row r="62" spans="1:7" x14ac:dyDescent="0.45">
       <c r="A62" s="7">
-        <v>46309</v>
+        <v>46310</v>
       </c>
       <c r="B62" s="8"/>
       <c r="C62" s="20" t="s">
         <v>32</v>
       </c>
       <c r="D62" s="10">
-        <v>268.86</v>
+        <v>270.08</v>
       </c>
       <c r="E62" s="10">
-        <v>263.64999999999998</v>
+        <v>261.08999999999997</v>
       </c>
       <c r="F62" s="10">
-        <v>273.64999999999998</v>
+        <v>271.08999999999997</v>
       </c>
       <c r="G62" s="17"/>
     </row>
-    <row r="63" spans="1:7" x14ac:dyDescent="0.35">
+    <row r="63" spans="1:7" x14ac:dyDescent="0.45">
       <c r="A63" s="11">
-        <v>46309</v>
+        <v>46310</v>
       </c>
       <c r="B63" s="12"/>
       <c r="C63" s="21" t="s">
         <v>33</v>
       </c>
       <c r="D63" s="13">
-        <v>258.82</v>
+        <v>258.04000000000002</v>
       </c>
       <c r="E63" s="13">
-        <v>245.03</v>
+        <v>242.67</v>
       </c>
       <c r="F63" s="13">
-        <v>255.03</v>
+        <v>252.67</v>
       </c>
       <c r="G63" s="17"/>
     </row>
-    <row r="64" spans="1:7" x14ac:dyDescent="0.35">
+    <row r="64" spans="1:7" x14ac:dyDescent="0.45">
       <c r="A64" s="7">
-        <v>46309</v>
+        <v>46310</v>
       </c>
       <c r="B64" s="8"/>
       <c r="C64" s="20" t="s">
         <v>34</v>
       </c>
       <c r="D64" s="10">
-        <v>259.70999999999998</v>
+        <v>258.81</v>
       </c>
       <c r="E64" s="10" t="s">
         <v>18</v>
@@ -1815,55 +1815,55 @@
       </c>
       <c r="G64" s="17"/>
     </row>
-    <row r="65" spans="1:6" x14ac:dyDescent="0.35">
+    <row r="65" spans="1:6" x14ac:dyDescent="0.45">
       <c r="A65" s="11">
-        <v>46309</v>
+        <v>46310</v>
       </c>
       <c r="B65" s="12"/>
       <c r="C65" s="21" t="s">
         <v>35</v>
       </c>
       <c r="D65" s="13">
-        <v>253.87</v>
+        <v>255.11</v>
       </c>
       <c r="E65" s="13">
-        <v>239.4</v>
+        <v>237.04</v>
       </c>
       <c r="F65" s="13" t="s">
         <v>18</v>
       </c>
     </row>
-    <row r="66" spans="1:6" x14ac:dyDescent="0.35">
+    <row r="66" spans="1:6" x14ac:dyDescent="0.45">
       <c r="A66" s="7">
-        <v>46309</v>
+        <v>46310</v>
       </c>
       <c r="B66" s="8"/>
       <c r="C66" s="20" t="s">
         <v>36</v>
       </c>
       <c r="D66" s="10">
-        <v>249.69</v>
+        <v>250.94</v>
       </c>
       <c r="E66" s="10">
-        <v>235.35</v>
+        <v>232.99</v>
       </c>
       <c r="F66" s="10">
-        <v>245.35</v>
-      </c>
-    </row>
-    <row r="67" spans="1:6" x14ac:dyDescent="0.35">
+        <v>242.99</v>
+      </c>
+    </row>
+    <row r="67" spans="1:6" x14ac:dyDescent="0.45">
       <c r="A67" s="11">
-        <v>46309</v>
+        <v>46310</v>
       </c>
       <c r="B67" s="12"/>
       <c r="C67" s="21" t="s">
         <v>37</v>
       </c>
       <c r="D67" s="13">
-        <v>256.72000000000003</v>
+        <v>257.95999999999998</v>
       </c>
       <c r="E67" s="13">
-        <v>256.99</v>
+        <v>254.49</v>
       </c>
       <c r="F67" s="13" t="s">
         <v>18</v>
@@ -1891,26 +1891,6 @@
 </file>
 
 <file path=customXml/item1.xml><?xml version="1.0" encoding="utf-8"?>
-<?mso-contentType ?>
-<FormTemplates xmlns="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms">
-  <Display>DocumentLibraryForm</Display>
-  <Edit>DocumentLibraryForm</Edit>
-  <New>DocumentLibraryForm</New>
-</FormTemplates>
-</file>
-
-<file path=customXml/item2.xml><?xml version="1.0" encoding="utf-8"?>
-<p:properties xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls">
-  <documentManagement>
-    <lcf76f155ced4ddcb4097134ff3c332f xmlns="87276d81-85f4-4ef2-9e6e-55066304288f">
-      <Terms xmlns="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
-    </lcf76f155ced4ddcb4097134ff3c332f>
-    <TaxCatchAll xmlns="b23b8984-eafa-4e79-985e-54f52f3da58e" xsi:nil="true"/>
-  </documentManagement>
-</p:properties>
-</file>
-
-<file path=customXml/item3.xml><?xml version="1.0" encoding="utf-8"?>
 <ct:contentTypeSchema xmlns:ct="http://schemas.microsoft.com/office/2006/metadata/contentType" xmlns:ma="http://schemas.microsoft.com/office/2006/metadata/properties/metaAttributes" ct:_="" ma:_="" ma:contentTypeName="Document" ma:contentTypeID="0x010100D3632DF5622958439304627C030B0427" ma:contentTypeVersion="18" ma:contentTypeDescription="Create a new document." ma:contentTypeScope="" ma:versionID="8c2ecbce386d6bac497f8eb2d8f0fb7a">
   <xsd:schema xmlns:xsd="http://www.w3.org/2001/XMLSchema" xmlns:xs="http://www.w3.org/2001/XMLSchema" xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:ns2="87276d81-85f4-4ef2-9e6e-55066304288f" xmlns:ns3="39e1dda6-d1d8-4c88-a3b9-f1abc1284bad" xmlns:ns4="b23b8984-eafa-4e79-985e-54f52f3da58e" targetNamespace="http://schemas.microsoft.com/office/2006/metadata/properties" ma:root="true" ma:fieldsID="4cfd0c2f651c1ce156ad4fcb44ea61dd" ns2:_="" ns3:_="" ns4:_="">
     <xsd:import namespace="87276d81-85f4-4ef2-9e6e-55066304288f"/>
@@ -2170,26 +2150,27 @@
 </ct:contentTypeSchema>
 </file>
 
-<file path=customXml/itemProps1.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{F60519E9-FD90-4339-869C-BC2F85719BB8}">
-  <ds:schemaRefs>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms"/>
-  </ds:schemaRefs>
-</ds:datastoreItem>
+<file path=customXml/item2.xml><?xml version="1.0" encoding="utf-8"?>
+<?mso-contentType ?>
+<FormTemplates xmlns="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms">
+  <Display>DocumentLibraryForm</Display>
+  <Edit>DocumentLibraryForm</Edit>
+  <New>DocumentLibraryForm</New>
+</FormTemplates>
 </file>
 
-<file path=customXml/itemProps2.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{57A83D98-2BAE-4D83-823A-D31C464B620C}">
-  <ds:schemaRefs>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/properties"/>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
-    <ds:schemaRef ds:uri="87276d81-85f4-4ef2-9e6e-55066304288f"/>
-    <ds:schemaRef ds:uri="b23b8984-eafa-4e79-985e-54f52f3da58e"/>
-  </ds:schemaRefs>
-</ds:datastoreItem>
+<file path=customXml/item3.xml><?xml version="1.0" encoding="utf-8"?>
+<p:properties xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls">
+  <documentManagement>
+    <lcf76f155ced4ddcb4097134ff3c332f xmlns="87276d81-85f4-4ef2-9e6e-55066304288f">
+      <Terms xmlns="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
+    </lcf76f155ced4ddcb4097134ff3c332f>
+    <TaxCatchAll xmlns="b23b8984-eafa-4e79-985e-54f52f3da58e" xsi:nil="true"/>
+  </documentManagement>
+</p:properties>
 </file>
 
-<file path=customXml/itemProps3.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=customXml/itemProps1.xml><?xml version="1.0" encoding="utf-8"?>
 <ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{B44E1863-2778-41F9-ACBA-48420F931671}">
   <ds:schemaRefs>
     <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/contentType"/>
@@ -2209,6 +2190,25 @@
 </ds:datastoreItem>
 </file>
 
+<file path=customXml/itemProps2.xml><?xml version="1.0" encoding="utf-8"?>
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{F60519E9-FD90-4339-869C-BC2F85719BB8}">
+  <ds:schemaRefs>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms"/>
+  </ds:schemaRefs>
+</ds:datastoreItem>
+</file>
+
+<file path=customXml/itemProps3.xml><?xml version="1.0" encoding="utf-8"?>
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{57A83D98-2BAE-4D83-823A-D31C464B620C}">
+  <ds:schemaRefs>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/properties"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
+    <ds:schemaRef ds:uri="87276d81-85f4-4ef2-9e6e-55066304288f"/>
+    <ds:schemaRef ds:uri="b23b8984-eafa-4e79-985e-54f52f3da58e"/>
+  </ds:schemaRefs>
+</ds:datastoreItem>
+</file>
+
 <file path=docMetadata/LabelInfo.xml><?xml version="1.0" encoding="utf-8"?>
 <clbl:labelList xmlns:clbl="http://schemas.microsoft.com/office/2020/mipLabelMetadata">
   <clbl:label id="{569bf4a9-87bd-4dbf-a36c-1db5158e5def}" enabled="1" method="Privileged" siteId="{ea80952e-a476-42d4-aaf4-5457852b0f7e}" removed="0"/>

</xml_diff>

<commit_message>
Fri Oct 16 05:57:04 UTC 2026
</commit_message>
<xml_diff>
--- a/bp.com-content-dam-bp-country-sites-en_au-australia-home-products-services-pricing-tgp-excel.xlsx
+++ b/bp.com-content-dam-bp-country-sites-en_au-australia-home-products-services-pricing-tgp-excel.xlsx
@@ -8,14 +8,14 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://bp365.sharepoint.com/sites/WholesalePricing/Shared Documents/B2C/TGP/Daily TGP/Web TGP/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="14_{FD13E0C4-DF32-43D8-AB1B-C62894DC1629}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="14_{63D386A3-4BDD-4291-8275-DF70A44C5830}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-8595" yWindow="-16320" windowWidth="29040" windowHeight="15720" xr2:uid="{1B412EEF-F96D-4DF4-A4E9-C7F0F183C2FB}"/>
+    <workbookView xWindow="2535" yWindow="-18780" windowWidth="26145" windowHeight="18045" xr2:uid="{1B412EEF-F96D-4DF4-A4E9-C7F0F183C2FB}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
   </sheets>
-  <calcPr calcId="191028" concurrentManualCount="12"/>
+  <calcPr calcId="191028"/>
   <extLst>
     <ext xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" uri="{140A7094-0E35-4892-8432-C4D2E57EDEB5}">
       <x15:workbookPr chartTrackingRefBase="1"/>
@@ -717,10 +717,10 @@
   <dimension ref="A1:G67"/>
   <sheetFormatPr defaultRowHeight="14.25" x14ac:dyDescent="0.45"/>
   <cols>
-    <col min="1" max="1" width="76.46484375" bestFit="1" customWidth="1"/>
-    <col min="2" max="2" width="6.46484375"/>
-    <col min="3" max="3" width="18.19921875" bestFit="1" customWidth="1"/>
-    <col min="4" max="7" width="7.19921875" bestFit="1" customWidth="1"/>
+    <col min="1" max="1" width="76.3984375" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="6.3984375"/>
+    <col min="3" max="3" width="18.1328125" bestFit="1" customWidth="1"/>
+    <col min="4" max="7" width="7.1328125" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:7" ht="22.15" x14ac:dyDescent="0.45">
@@ -808,128 +808,128 @@
     </row>
     <row r="8" spans="1:7" x14ac:dyDescent="0.45">
       <c r="A8" s="7">
-        <v>46311</v>
+        <v>46312</v>
       </c>
       <c r="B8" s="8"/>
       <c r="C8" s="9" t="s">
         <v>10</v>
       </c>
       <c r="D8" s="10">
-        <v>259.11</v>
+        <v>259.14</v>
       </c>
       <c r="E8" s="10">
-        <v>231.51</v>
+        <v>228.77</v>
       </c>
       <c r="F8" s="10">
-        <v>241.51</v>
+        <v>238.77</v>
       </c>
       <c r="G8" s="10">
-        <v>229.13</v>
+        <v>226.39</v>
       </c>
     </row>
     <row r="9" spans="1:7" x14ac:dyDescent="0.45">
       <c r="A9" s="11">
-        <v>46311</v>
+        <v>46312</v>
       </c>
       <c r="B9" s="12"/>
       <c r="C9" s="12" t="s">
         <v>11</v>
       </c>
       <c r="D9" s="13">
-        <v>259.11</v>
+        <v>259.14</v>
       </c>
       <c r="E9" s="13">
-        <v>231.51</v>
+        <v>228.77</v>
       </c>
       <c r="F9" s="13">
-        <v>241.51</v>
+        <v>238.77</v>
       </c>
       <c r="G9" s="13">
-        <v>229.13</v>
+        <v>226.39</v>
       </c>
     </row>
     <row r="10" spans="1:7" x14ac:dyDescent="0.45">
       <c r="A10" s="7">
-        <v>46311</v>
+        <v>46312</v>
       </c>
       <c r="B10" s="8"/>
       <c r="C10" s="9" t="s">
         <v>12</v>
       </c>
       <c r="D10" s="10">
-        <v>256.52</v>
+        <v>255.05</v>
       </c>
       <c r="E10" s="10">
-        <v>229.39</v>
+        <v>226.83</v>
       </c>
       <c r="F10" s="10">
-        <v>239.39</v>
+        <v>236.83</v>
       </c>
       <c r="G10" s="10">
-        <v>227.79</v>
+        <v>225.23</v>
       </c>
     </row>
     <row r="11" spans="1:7" x14ac:dyDescent="0.45">
       <c r="A11" s="11">
-        <v>46310</v>
+        <v>46311</v>
       </c>
       <c r="B11" s="12"/>
       <c r="C11" s="12" t="s">
         <v>10</v>
       </c>
       <c r="D11" s="13">
-        <v>257.98</v>
+        <v>259.11</v>
       </c>
       <c r="E11" s="13">
-        <v>233.92</v>
+        <v>231.51</v>
       </c>
       <c r="F11" s="13">
-        <v>243.92</v>
+        <v>241.51</v>
       </c>
       <c r="G11" s="13">
-        <v>231.54</v>
+        <v>229.13</v>
       </c>
     </row>
     <row r="12" spans="1:7" x14ac:dyDescent="0.45">
       <c r="A12" s="7">
-        <v>46310</v>
+        <v>46311</v>
       </c>
       <c r="B12" s="8"/>
       <c r="C12" s="9" t="s">
         <v>11</v>
       </c>
       <c r="D12" s="10">
-        <v>257.98</v>
+        <v>259.11</v>
       </c>
       <c r="E12" s="10">
-        <v>233.92</v>
+        <v>231.51</v>
       </c>
       <c r="F12" s="10">
-        <v>243.92</v>
+        <v>241.51</v>
       </c>
       <c r="G12" s="10">
-        <v>231.54</v>
+        <v>229.13</v>
       </c>
     </row>
     <row r="13" spans="1:7" x14ac:dyDescent="0.45">
       <c r="A13" s="11">
-        <v>46310</v>
+        <v>46311</v>
       </c>
       <c r="B13" s="12"/>
       <c r="C13" s="12" t="s">
         <v>12</v>
       </c>
       <c r="D13" s="13">
-        <v>255.39</v>
+        <v>256.52</v>
       </c>
       <c r="E13" s="13">
-        <v>232.3</v>
+        <v>229.39</v>
       </c>
       <c r="F13" s="13">
-        <v>242.3</v>
+        <v>239.39</v>
       </c>
       <c r="G13" s="13">
-        <v>230.71</v>
+        <v>227.79</v>
       </c>
     </row>
     <row r="14" spans="1:7" x14ac:dyDescent="0.45">
@@ -973,39 +973,39 @@
     </row>
     <row r="17" spans="1:7" x14ac:dyDescent="0.45">
       <c r="A17" s="7">
-        <v>46311</v>
+        <v>46312</v>
       </c>
       <c r="B17" s="8"/>
       <c r="C17" s="20" t="s">
         <v>14</v>
       </c>
       <c r="D17" s="10">
-        <v>260.04000000000002</v>
+        <v>258.58999999999997</v>
       </c>
       <c r="E17" s="10">
-        <v>234.62</v>
+        <v>230.41</v>
       </c>
       <c r="F17" s="10">
-        <v>244.62</v>
+        <v>240.41</v>
       </c>
       <c r="G17" s="17"/>
     </row>
     <row r="18" spans="1:7" x14ac:dyDescent="0.45">
       <c r="A18" s="11">
-        <v>46310</v>
+        <v>46311</v>
       </c>
       <c r="B18" s="12"/>
       <c r="C18" s="12" t="s">
         <v>14</v>
       </c>
       <c r="D18" s="13">
-        <v>258.87</v>
+        <v>260.04000000000002</v>
       </c>
       <c r="E18" s="13">
-        <v>237.5</v>
+        <v>234.62</v>
       </c>
       <c r="F18" s="13">
-        <v>247.5</v>
+        <v>244.62</v>
       </c>
       <c r="G18" s="17"/>
     </row>
@@ -1052,41 +1052,41 @@
     </row>
     <row r="22" spans="1:7" x14ac:dyDescent="0.45">
       <c r="A22" s="7">
-        <v>46311</v>
+        <v>46312</v>
       </c>
       <c r="B22" s="8"/>
       <c r="C22" s="20" t="s">
         <v>16</v>
       </c>
       <c r="D22" s="10">
-        <v>260.23</v>
+        <v>260.27</v>
       </c>
       <c r="E22" s="10">
-        <v>231.65</v>
+        <v>228.91</v>
       </c>
       <c r="F22" s="10">
-        <v>241.25</v>
+        <v>238.51</v>
       </c>
       <c r="G22" s="10">
-        <v>228.02</v>
+        <v>225.28</v>
       </c>
     </row>
     <row r="23" spans="1:7" x14ac:dyDescent="0.45">
       <c r="A23" s="11">
-        <v>46311</v>
+        <v>46312</v>
       </c>
       <c r="B23" s="12"/>
       <c r="C23" s="21" t="s">
         <v>17</v>
       </c>
       <c r="D23" s="13">
-        <v>261.45999999999998</v>
+        <v>259.99</v>
       </c>
       <c r="E23" s="13">
-        <v>239.85</v>
+        <v>235.62</v>
       </c>
       <c r="F23" s="13">
-        <v>249.85</v>
+        <v>245.62</v>
       </c>
       <c r="G23" s="13" t="s">
         <v>18</v>
@@ -1094,20 +1094,20 @@
     </row>
     <row r="24" spans="1:7" x14ac:dyDescent="0.45">
       <c r="A24" s="7">
-        <v>46311</v>
+        <v>46312</v>
       </c>
       <c r="B24" s="8"/>
       <c r="C24" s="20" t="s">
         <v>19</v>
       </c>
       <c r="D24" s="10">
-        <v>261.82</v>
+        <v>260.35000000000002</v>
       </c>
       <c r="E24" s="10">
-        <v>239.09</v>
+        <v>234.88</v>
       </c>
       <c r="F24" s="10">
-        <v>249.1</v>
+        <v>244.88</v>
       </c>
       <c r="G24" s="10" t="s">
         <v>18</v>
@@ -1115,41 +1115,41 @@
     </row>
     <row r="25" spans="1:7" x14ac:dyDescent="0.45">
       <c r="A25" s="11">
-        <v>46311</v>
+        <v>46312</v>
       </c>
       <c r="B25" s="12"/>
       <c r="C25" s="21" t="s">
         <v>20</v>
       </c>
       <c r="D25" s="13">
-        <v>258.49</v>
+        <v>257.02</v>
       </c>
       <c r="E25" s="13">
-        <v>239.32</v>
+        <v>235.09</v>
       </c>
       <c r="F25" s="13">
-        <v>249.32</v>
+        <v>245.09</v>
       </c>
       <c r="G25" s="13">
-        <v>235.16</v>
+        <v>230.93</v>
       </c>
     </row>
     <row r="26" spans="1:7" x14ac:dyDescent="0.45">
       <c r="A26" s="7">
-        <v>46311</v>
+        <v>46312</v>
       </c>
       <c r="B26" s="8"/>
       <c r="C26" s="20" t="s">
         <v>21</v>
       </c>
       <c r="D26" s="10">
-        <v>260.05</v>
+        <v>258.58</v>
       </c>
       <c r="E26" s="10">
-        <v>240.81</v>
+        <v>236.55</v>
       </c>
       <c r="F26" s="10">
-        <v>250.81</v>
+        <v>246.55</v>
       </c>
       <c r="G26" s="10" t="s">
         <v>18</v>
@@ -1157,41 +1157,41 @@
     </row>
     <row r="27" spans="1:7" x14ac:dyDescent="0.45">
       <c r="A27" s="11">
-        <v>46310</v>
+        <v>46311</v>
       </c>
       <c r="B27" s="12"/>
       <c r="C27" s="12" t="s">
         <v>16</v>
       </c>
       <c r="D27" s="13">
-        <v>259.10000000000002</v>
+        <v>260.23</v>
       </c>
       <c r="E27" s="13">
-        <v>234.06</v>
+        <v>231.65</v>
       </c>
       <c r="F27" s="13">
-        <v>243.66</v>
+        <v>241.25</v>
       </c>
       <c r="G27" s="13">
-        <v>230.43</v>
+        <v>228.02</v>
       </c>
     </row>
     <row r="28" spans="1:7" x14ac:dyDescent="0.45">
       <c r="A28" s="7">
-        <v>46310</v>
+        <v>46311</v>
       </c>
       <c r="B28" s="8"/>
       <c r="C28" s="20" t="s">
         <v>17</v>
       </c>
       <c r="D28" s="10">
-        <v>260.33999999999997</v>
+        <v>261.45999999999998</v>
       </c>
       <c r="E28" s="22">
-        <v>242.79</v>
+        <v>239.85</v>
       </c>
       <c r="F28" s="22">
-        <v>252.79</v>
+        <v>249.85</v>
       </c>
       <c r="G28" s="22" t="s">
         <v>18</v>
@@ -1199,20 +1199,20 @@
     </row>
     <row r="29" spans="1:7" x14ac:dyDescent="0.45">
       <c r="A29" s="11">
-        <v>46310</v>
+        <v>46311</v>
       </c>
       <c r="B29" s="12"/>
       <c r="C29" s="12" t="s">
         <v>19</v>
       </c>
       <c r="D29" s="13">
-        <v>260.7</v>
+        <v>261.82</v>
       </c>
       <c r="E29" s="13">
-        <v>242.03</v>
+        <v>239.09</v>
       </c>
       <c r="F29" s="13">
-        <v>252.03</v>
+        <v>249.1</v>
       </c>
       <c r="G29" s="13" t="s">
         <v>18</v>
@@ -1220,41 +1220,41 @@
     </row>
     <row r="30" spans="1:7" x14ac:dyDescent="0.45">
       <c r="A30" s="7">
-        <v>46310</v>
+        <v>46311</v>
       </c>
       <c r="B30" s="8"/>
       <c r="C30" s="20" t="s">
         <v>20</v>
       </c>
       <c r="D30" s="10">
-        <v>257.36</v>
+        <v>258.49</v>
       </c>
       <c r="E30" s="22">
-        <v>242.26</v>
+        <v>239.32</v>
       </c>
       <c r="F30" s="22">
-        <v>252.26</v>
+        <v>249.32</v>
       </c>
       <c r="G30" s="22">
-        <v>238.1</v>
+        <v>235.16</v>
       </c>
     </row>
     <row r="31" spans="1:7" x14ac:dyDescent="0.45">
       <c r="A31" s="11">
-        <v>46310</v>
+        <v>46311</v>
       </c>
       <c r="B31" s="12"/>
       <c r="C31" s="12" t="s">
         <v>21</v>
       </c>
       <c r="D31" s="13">
-        <v>258.91000000000003</v>
+        <v>260.05</v>
       </c>
       <c r="E31" s="13">
-        <v>243.78</v>
+        <v>240.81</v>
       </c>
       <c r="F31" s="13">
-        <v>253.78</v>
+        <v>250.81</v>
       </c>
       <c r="G31" s="13" t="s">
         <v>18</v>
@@ -1301,52 +1301,52 @@
     </row>
     <row r="35" spans="1:7" x14ac:dyDescent="0.45">
       <c r="A35" s="7">
-        <v>46311</v>
+        <v>46312</v>
       </c>
       <c r="B35" s="8"/>
       <c r="C35" s="20" t="s">
         <v>23</v>
       </c>
       <c r="D35" s="10">
-        <v>255.06</v>
+        <v>253.6</v>
       </c>
       <c r="E35" s="10">
-        <v>229.42</v>
+        <v>226.32</v>
       </c>
       <c r="F35" s="10">
-        <v>238.42</v>
+        <v>235.32</v>
       </c>
       <c r="G35" s="17"/>
     </row>
     <row r="36" spans="1:7" x14ac:dyDescent="0.45">
       <c r="A36" s="11">
-        <v>46310</v>
+        <v>46311</v>
       </c>
       <c r="B36" s="12"/>
       <c r="C36" s="12" t="s">
         <v>23</v>
       </c>
       <c r="D36" s="13">
-        <v>253.94</v>
+        <v>255.06</v>
       </c>
       <c r="E36" s="13">
-        <v>231.24</v>
+        <v>229.42</v>
       </c>
       <c r="F36" s="13">
-        <v>240.24</v>
+        <v>238.42</v>
       </c>
       <c r="G36" s="17"/>
     </row>
     <row r="37" spans="1:7" x14ac:dyDescent="0.45">
       <c r="A37" s="7">
-        <v>46311</v>
+        <v>46312</v>
       </c>
       <c r="B37" s="8"/>
       <c r="C37" s="20" t="s">
         <v>24</v>
       </c>
       <c r="D37" s="10">
-        <v>270.68</v>
+        <v>269.22000000000003</v>
       </c>
       <c r="E37" s="10" t="s">
         <v>18</v>
@@ -1358,14 +1358,14 @@
     </row>
     <row r="38" spans="1:7" x14ac:dyDescent="0.45">
       <c r="A38" s="11">
-        <v>46310</v>
+        <v>46311</v>
       </c>
       <c r="B38" s="12"/>
       <c r="C38" s="12" t="s">
         <v>24</v>
       </c>
       <c r="D38" s="13">
-        <v>269.56</v>
+        <v>270.68</v>
       </c>
       <c r="E38" s="13" t="s">
         <v>18</v>
@@ -1416,77 +1416,77 @@
     </row>
     <row r="42" spans="1:7" x14ac:dyDescent="0.45">
       <c r="A42" s="7">
-        <v>46311</v>
+        <v>46312</v>
       </c>
       <c r="B42" s="8"/>
       <c r="C42" s="20" t="s">
         <v>26</v>
       </c>
       <c r="D42" s="10">
-        <v>265.02999999999997</v>
+        <v>263.54000000000002</v>
       </c>
       <c r="E42" s="10">
-        <v>239.37</v>
+        <v>235.92</v>
       </c>
       <c r="F42" s="10">
-        <v>249.37</v>
+        <v>245.92</v>
       </c>
       <c r="G42" s="17"/>
     </row>
     <row r="43" spans="1:7" x14ac:dyDescent="0.45">
       <c r="A43" s="11">
-        <v>46311</v>
+        <v>46312</v>
       </c>
       <c r="B43" s="12"/>
       <c r="C43" s="21" t="s">
         <v>27</v>
       </c>
       <c r="D43" s="13">
-        <v>264.64</v>
+        <v>263.16000000000003</v>
       </c>
       <c r="E43" s="13">
-        <v>239.78</v>
+        <v>236.33</v>
       </c>
       <c r="F43" s="13">
-        <v>249.78</v>
+        <v>246.33</v>
       </c>
       <c r="G43" s="17"/>
     </row>
     <row r="44" spans="1:7" x14ac:dyDescent="0.45">
       <c r="A44" s="7">
-        <v>46310</v>
+        <v>46311</v>
       </c>
       <c r="B44" s="8"/>
       <c r="C44" s="20" t="s">
         <v>26</v>
       </c>
       <c r="D44" s="10">
-        <v>263.94</v>
+        <v>265.02999999999997</v>
       </c>
       <c r="E44" s="10">
-        <v>241.39</v>
+        <v>239.37</v>
       </c>
       <c r="F44" s="10">
-        <v>251.39</v>
+        <v>249.37</v>
       </c>
       <c r="G44" s="17"/>
     </row>
     <row r="45" spans="1:7" x14ac:dyDescent="0.45">
       <c r="A45" s="11">
-        <v>46310</v>
+        <v>46311</v>
       </c>
       <c r="B45" s="12"/>
       <c r="C45" s="21" t="s">
         <v>27</v>
       </c>
       <c r="D45" s="13">
-        <v>263.55</v>
+        <v>264.64</v>
       </c>
       <c r="E45" s="13">
-        <v>241.8</v>
+        <v>239.78</v>
       </c>
       <c r="F45" s="13">
-        <v>251.8</v>
+        <v>249.78</v>
       </c>
       <c r="G45" s="17"/>
     </row>
@@ -1531,77 +1531,77 @@
     </row>
     <row r="49" spans="1:7" x14ac:dyDescent="0.45">
       <c r="A49" s="7">
-        <v>46311</v>
+        <v>46312</v>
       </c>
       <c r="B49" s="8"/>
       <c r="C49" s="20" t="s">
         <v>29</v>
       </c>
       <c r="D49" s="10">
-        <v>256.41000000000003</v>
+        <v>257.11</v>
       </c>
       <c r="E49" s="10">
-        <v>234.17</v>
+        <v>231.63</v>
       </c>
       <c r="F49" s="10">
-        <v>244.17</v>
+        <v>241.63</v>
       </c>
       <c r="G49" s="28"/>
     </row>
     <row r="50" spans="1:7" x14ac:dyDescent="0.45">
       <c r="A50" s="11">
-        <v>46311</v>
+        <v>46312</v>
       </c>
       <c r="B50" s="12"/>
       <c r="C50" s="21" t="s">
         <v>30</v>
       </c>
       <c r="D50" s="13">
-        <v>253.94</v>
+        <v>254.65</v>
       </c>
       <c r="E50" s="13">
-        <v>233.79</v>
+        <v>231.25</v>
       </c>
       <c r="F50" s="13">
-        <v>243.79</v>
+        <v>241.25</v>
       </c>
       <c r="G50" s="28"/>
     </row>
     <row r="51" spans="1:7" x14ac:dyDescent="0.45">
       <c r="A51" s="7">
-        <v>46310</v>
+        <v>46311</v>
       </c>
       <c r="B51" s="8"/>
       <c r="C51" s="20" t="s">
         <v>29</v>
       </c>
       <c r="D51" s="10">
-        <v>255.92</v>
+        <v>256.41000000000003</v>
       </c>
       <c r="E51" s="10">
-        <v>236.16</v>
+        <v>234.17</v>
       </c>
       <c r="F51" s="10">
-        <v>246.16</v>
+        <v>244.17</v>
       </c>
       <c r="G51" s="17"/>
     </row>
     <row r="52" spans="1:7" x14ac:dyDescent="0.45">
       <c r="A52" s="11">
-        <v>46310</v>
+        <v>46311</v>
       </c>
       <c r="B52" s="12"/>
       <c r="C52" s="21" t="s">
         <v>30</v>
       </c>
       <c r="D52" s="13">
-        <v>253.42</v>
+        <v>253.94</v>
       </c>
       <c r="E52" s="13">
-        <v>235.77</v>
+        <v>233.79</v>
       </c>
       <c r="F52" s="13">
-        <v>245.77</v>
+        <v>243.79</v>
       </c>
       <c r="G52" s="17"/>
     </row>
@@ -1646,52 +1646,52 @@
     </row>
     <row r="56" spans="1:7" x14ac:dyDescent="0.45">
       <c r="A56" s="7">
-        <v>46311</v>
+        <v>46312</v>
       </c>
       <c r="B56" s="8"/>
       <c r="C56" s="20" t="s">
         <v>32</v>
       </c>
       <c r="D56" s="10">
-        <v>271.22000000000003</v>
+        <v>269.75</v>
       </c>
       <c r="E56" s="10">
-        <v>257.98</v>
+        <v>253.71</v>
       </c>
       <c r="F56" s="10">
-        <v>267.98</v>
+        <v>263.70999999999998</v>
       </c>
       <c r="G56" s="17"/>
     </row>
     <row r="57" spans="1:7" x14ac:dyDescent="0.45">
       <c r="A57" s="11">
-        <v>46311</v>
+        <v>46312</v>
       </c>
       <c r="B57" s="12"/>
       <c r="C57" s="21" t="s">
         <v>33</v>
       </c>
       <c r="D57" s="13">
-        <v>258.06</v>
+        <v>257.14</v>
       </c>
       <c r="E57" s="13">
-        <v>239.81</v>
+        <v>235.63</v>
       </c>
       <c r="F57" s="13">
-        <v>249.81</v>
+        <v>245.63</v>
       </c>
       <c r="G57" s="17"/>
     </row>
     <row r="58" spans="1:7" x14ac:dyDescent="0.45">
       <c r="A58" s="7">
-        <v>46311</v>
+        <v>46312</v>
       </c>
       <c r="B58" s="8"/>
       <c r="C58" s="20" t="s">
         <v>34</v>
       </c>
       <c r="D58" s="10">
-        <v>258.83</v>
+        <v>257.89999999999998</v>
       </c>
       <c r="E58" s="10" t="s">
         <v>18</v>
@@ -1703,17 +1703,17 @@
     </row>
     <row r="59" spans="1:7" x14ac:dyDescent="0.45">
       <c r="A59" s="11">
-        <v>46311</v>
+        <v>46312</v>
       </c>
       <c r="B59" s="12"/>
       <c r="C59" s="21" t="s">
         <v>35</v>
       </c>
       <c r="D59" s="13">
-        <v>255.19</v>
+        <v>254.29</v>
       </c>
       <c r="E59" s="13">
-        <v>234.19</v>
+        <v>230.01</v>
       </c>
       <c r="F59" s="13" t="s">
         <v>18</v>
@@ -1722,36 +1722,36 @@
     </row>
     <row r="60" spans="1:7" x14ac:dyDescent="0.45">
       <c r="A60" s="7">
-        <v>46311</v>
+        <v>46312</v>
       </c>
       <c r="B60" s="8"/>
       <c r="C60" s="20" t="s">
         <v>36</v>
       </c>
       <c r="D60" s="10">
-        <v>251.02</v>
+        <v>250.12</v>
       </c>
       <c r="E60" s="10">
-        <v>230.13</v>
+        <v>225.95</v>
       </c>
       <c r="F60" s="10">
-        <v>240.13</v>
+        <v>235.95</v>
       </c>
       <c r="G60" s="17"/>
     </row>
     <row r="61" spans="1:7" x14ac:dyDescent="0.45">
       <c r="A61" s="11">
-        <v>46311</v>
+        <v>46312</v>
       </c>
       <c r="B61" s="12"/>
       <c r="C61" s="21" t="s">
         <v>37</v>
       </c>
       <c r="D61" s="13">
-        <v>259.14999999999998</v>
+        <v>257.7</v>
       </c>
       <c r="E61" s="13">
-        <v>251.46</v>
+        <v>247.2</v>
       </c>
       <c r="F61" s="13" t="s">
         <v>18</v>
@@ -1760,52 +1760,52 @@
     </row>
     <row r="62" spans="1:7" x14ac:dyDescent="0.45">
       <c r="A62" s="7">
-        <v>46310</v>
+        <v>46311</v>
       </c>
       <c r="B62" s="8"/>
       <c r="C62" s="20" t="s">
         <v>32</v>
       </c>
       <c r="D62" s="10">
-        <v>270.08</v>
+        <v>271.22000000000003</v>
       </c>
       <c r="E62" s="10">
-        <v>261.08999999999997</v>
+        <v>257.98</v>
       </c>
       <c r="F62" s="10">
-        <v>271.08999999999997</v>
+        <v>267.98</v>
       </c>
       <c r="G62" s="17"/>
     </row>
     <row r="63" spans="1:7" x14ac:dyDescent="0.45">
       <c r="A63" s="11">
-        <v>46310</v>
+        <v>46311</v>
       </c>
       <c r="B63" s="12"/>
       <c r="C63" s="21" t="s">
         <v>33</v>
       </c>
       <c r="D63" s="13">
-        <v>258.04000000000002</v>
+        <v>258.06</v>
       </c>
       <c r="E63" s="13">
-        <v>242.67</v>
+        <v>239.81</v>
       </c>
       <c r="F63" s="13">
-        <v>252.67</v>
+        <v>249.81</v>
       </c>
       <c r="G63" s="17"/>
     </row>
     <row r="64" spans="1:7" x14ac:dyDescent="0.45">
       <c r="A64" s="7">
-        <v>46310</v>
+        <v>46311</v>
       </c>
       <c r="B64" s="8"/>
       <c r="C64" s="20" t="s">
         <v>34</v>
       </c>
       <c r="D64" s="10">
-        <v>258.81</v>
+        <v>258.83</v>
       </c>
       <c r="E64" s="10" t="s">
         <v>18</v>
@@ -1817,17 +1817,17 @@
     </row>
     <row r="65" spans="1:6" x14ac:dyDescent="0.45">
       <c r="A65" s="11">
-        <v>46310</v>
+        <v>46311</v>
       </c>
       <c r="B65" s="12"/>
       <c r="C65" s="21" t="s">
         <v>35</v>
       </c>
       <c r="D65" s="13">
-        <v>255.11</v>
+        <v>255.19</v>
       </c>
       <c r="E65" s="13">
-        <v>237.04</v>
+        <v>234.19</v>
       </c>
       <c r="F65" s="13" t="s">
         <v>18</v>
@@ -1835,35 +1835,35 @@
     </row>
     <row r="66" spans="1:6" x14ac:dyDescent="0.45">
       <c r="A66" s="7">
-        <v>46310</v>
+        <v>46311</v>
       </c>
       <c r="B66" s="8"/>
       <c r="C66" s="20" t="s">
         <v>36</v>
       </c>
       <c r="D66" s="10">
-        <v>250.94</v>
+        <v>251.02</v>
       </c>
       <c r="E66" s="10">
-        <v>232.99</v>
+        <v>230.13</v>
       </c>
       <c r="F66" s="10">
-        <v>242.99</v>
+        <v>240.13</v>
       </c>
     </row>
     <row r="67" spans="1:6" x14ac:dyDescent="0.45">
       <c r="A67" s="11">
-        <v>46310</v>
+        <v>46311</v>
       </c>
       <c r="B67" s="12"/>
       <c r="C67" s="21" t="s">
         <v>37</v>
       </c>
       <c r="D67" s="13">
-        <v>257.95999999999998</v>
+        <v>259.14999999999998</v>
       </c>
       <c r="E67" s="13">
-        <v>254.49</v>
+        <v>251.46</v>
       </c>
       <c r="F67" s="13" t="s">
         <v>18</v>
@@ -1891,6 +1891,15 @@
 </file>
 
 <file path=customXml/item1.xml><?xml version="1.0" encoding="utf-8"?>
+<?mso-contentType ?>
+<FormTemplates xmlns="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms">
+  <Display>DocumentLibraryForm</Display>
+  <Edit>DocumentLibraryForm</Edit>
+  <New>DocumentLibraryForm</New>
+</FormTemplates>
+</file>
+
+<file path=customXml/item2.xml><?xml version="1.0" encoding="utf-8"?>
 <ct:contentTypeSchema xmlns:ct="http://schemas.microsoft.com/office/2006/metadata/contentType" xmlns:ma="http://schemas.microsoft.com/office/2006/metadata/properties/metaAttributes" ct:_="" ma:_="" ma:contentTypeName="Document" ma:contentTypeID="0x010100D3632DF5622958439304627C030B0427" ma:contentTypeVersion="18" ma:contentTypeDescription="Create a new document." ma:contentTypeScope="" ma:versionID="8c2ecbce386d6bac497f8eb2d8f0fb7a">
   <xsd:schema xmlns:xsd="http://www.w3.org/2001/XMLSchema" xmlns:xs="http://www.w3.org/2001/XMLSchema" xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:ns2="87276d81-85f4-4ef2-9e6e-55066304288f" xmlns:ns3="39e1dda6-d1d8-4c88-a3b9-f1abc1284bad" xmlns:ns4="b23b8984-eafa-4e79-985e-54f52f3da58e" targetNamespace="http://schemas.microsoft.com/office/2006/metadata/properties" ma:root="true" ma:fieldsID="4cfd0c2f651c1ce156ad4fcb44ea61dd" ns2:_="" ns3:_="" ns4:_="">
     <xsd:import namespace="87276d81-85f4-4ef2-9e6e-55066304288f"/>
@@ -2150,15 +2159,6 @@
 </ct:contentTypeSchema>
 </file>
 
-<file path=customXml/item2.xml><?xml version="1.0" encoding="utf-8"?>
-<?mso-contentType ?>
-<FormTemplates xmlns="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms">
-  <Display>DocumentLibraryForm</Display>
-  <Edit>DocumentLibraryForm</Edit>
-  <New>DocumentLibraryForm</New>
-</FormTemplates>
-</file>
-
 <file path=customXml/item3.xml><?xml version="1.0" encoding="utf-8"?>
 <p:properties xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls">
   <documentManagement>
@@ -2171,6 +2171,14 @@
 </file>
 
 <file path=customXml/itemProps1.xml><?xml version="1.0" encoding="utf-8"?>
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{F60519E9-FD90-4339-869C-BC2F85719BB8}">
+  <ds:schemaRefs>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms"/>
+  </ds:schemaRefs>
+</ds:datastoreItem>
+</file>
+
+<file path=customXml/itemProps2.xml><?xml version="1.0" encoding="utf-8"?>
 <ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{B44E1863-2778-41F9-ACBA-48420F931671}">
   <ds:schemaRefs>
     <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/contentType"/>
@@ -2186,14 +2194,6 @@
     <ds:schemaRef ds:uri="http://purl.org/dc/elements/1.1/"/>
     <ds:schemaRef ds:uri="http://purl.org/dc/terms/"/>
     <ds:schemaRef ds:uri="http://schemas.microsoft.com/internal/obd"/>
-  </ds:schemaRefs>
-</ds:datastoreItem>
-</file>
-
-<file path=customXml/itemProps2.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{F60519E9-FD90-4339-869C-BC2F85719BB8}">
-  <ds:schemaRefs>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms"/>
   </ds:schemaRefs>
 </ds:datastoreItem>
 </file>

</xml_diff>

<commit_message>
Mon Oct 19 06:19:45 UTC 2026
</commit_message>
<xml_diff>
--- a/bp.com-content-dam-bp-country-sites-en_au-australia-home-products-services-pricing-tgp-excel.xlsx
+++ b/bp.com-content-dam-bp-country-sites-en_au-australia-home-products-services-pricing-tgp-excel.xlsx
@@ -8,14 +8,14 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://bp365.sharepoint.com/sites/WholesalePricing/Shared Documents/B2C/TGP/Daily TGP/Web TGP/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="14_{63D386A3-4BDD-4291-8275-DF70A44C5830}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="14_{691F818D-7C71-4FD4-B7A8-5797E2161298}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="2535" yWindow="-18780" windowWidth="26145" windowHeight="18045" xr2:uid="{1B412EEF-F96D-4DF4-A4E9-C7F0F183C2FB}"/>
+    <workbookView xWindow="-8310" yWindow="-16395" windowWidth="29040" windowHeight="15720" xr2:uid="{1B412EEF-F96D-4DF4-A4E9-C7F0F183C2FB}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
   </sheets>
-  <calcPr calcId="191028"/>
+  <calcPr calcId="191028" concurrentManualCount="12"/>
   <extLst>
     <ext xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" uri="{140A7094-0E35-4892-8432-C4D2E57EDEB5}">
       <x15:workbookPr chartTrackingRefBase="1"/>
@@ -808,128 +808,128 @@
     </row>
     <row r="8" spans="1:7" x14ac:dyDescent="0.45">
       <c r="A8" s="7">
-        <v>46312</v>
+        <v>46315</v>
       </c>
       <c r="B8" s="8"/>
       <c r="C8" s="9" t="s">
         <v>10</v>
       </c>
       <c r="D8" s="10">
-        <v>259.14</v>
+        <v>258.45</v>
       </c>
       <c r="E8" s="10">
-        <v>228.77</v>
+        <v>226.28</v>
       </c>
       <c r="F8" s="10">
-        <v>238.77</v>
+        <v>236.28</v>
       </c>
       <c r="G8" s="10">
-        <v>226.39</v>
+        <v>223.89</v>
       </c>
     </row>
     <row r="9" spans="1:7" x14ac:dyDescent="0.45">
       <c r="A9" s="11">
-        <v>46312</v>
+        <v>46315</v>
       </c>
       <c r="B9" s="12"/>
       <c r="C9" s="12" t="s">
         <v>11</v>
       </c>
       <c r="D9" s="13">
-        <v>259.14</v>
+        <v>258.45</v>
       </c>
       <c r="E9" s="13">
-        <v>228.77</v>
+        <v>226.28</v>
       </c>
       <c r="F9" s="13">
-        <v>238.77</v>
+        <v>236.28</v>
       </c>
       <c r="G9" s="13">
-        <v>226.39</v>
+        <v>223.89</v>
       </c>
     </row>
     <row r="10" spans="1:7" x14ac:dyDescent="0.45">
       <c r="A10" s="7">
-        <v>46312</v>
+        <v>46315</v>
       </c>
       <c r="B10" s="8"/>
       <c r="C10" s="9" t="s">
         <v>12</v>
       </c>
       <c r="D10" s="10">
-        <v>255.05</v>
+        <v>254.99</v>
       </c>
       <c r="E10" s="10">
-        <v>226.83</v>
+        <v>224.4</v>
       </c>
       <c r="F10" s="10">
-        <v>236.83</v>
+        <v>234.4</v>
       </c>
       <c r="G10" s="10">
-        <v>225.23</v>
+        <v>222.8</v>
       </c>
     </row>
     <row r="11" spans="1:7" x14ac:dyDescent="0.45">
       <c r="A11" s="11">
-        <v>46311</v>
+        <v>46312</v>
       </c>
       <c r="B11" s="12"/>
       <c r="C11" s="12" t="s">
         <v>10</v>
       </c>
       <c r="D11" s="13">
-        <v>259.11</v>
+        <v>259.14</v>
       </c>
       <c r="E11" s="13">
-        <v>231.51</v>
+        <v>228.77</v>
       </c>
       <c r="F11" s="13">
-        <v>241.51</v>
+        <v>238.77</v>
       </c>
       <c r="G11" s="13">
-        <v>229.13</v>
+        <v>226.39</v>
       </c>
     </row>
     <row r="12" spans="1:7" x14ac:dyDescent="0.45">
       <c r="A12" s="7">
-        <v>46311</v>
+        <v>46312</v>
       </c>
       <c r="B12" s="8"/>
       <c r="C12" s="9" t="s">
         <v>11</v>
       </c>
       <c r="D12" s="10">
-        <v>259.11</v>
+        <v>259.14</v>
       </c>
       <c r="E12" s="10">
-        <v>231.51</v>
+        <v>228.77</v>
       </c>
       <c r="F12" s="10">
-        <v>241.51</v>
+        <v>238.77</v>
       </c>
       <c r="G12" s="10">
-        <v>229.13</v>
+        <v>226.39</v>
       </c>
     </row>
     <row r="13" spans="1:7" x14ac:dyDescent="0.45">
       <c r="A13" s="11">
-        <v>46311</v>
+        <v>46312</v>
       </c>
       <c r="B13" s="12"/>
       <c r="C13" s="12" t="s">
         <v>12</v>
       </c>
       <c r="D13" s="13">
-        <v>256.52</v>
+        <v>255.05</v>
       </c>
       <c r="E13" s="13">
-        <v>229.39</v>
+        <v>226.83</v>
       </c>
       <c r="F13" s="13">
-        <v>239.39</v>
+        <v>236.83</v>
       </c>
       <c r="G13" s="13">
-        <v>227.79</v>
+        <v>225.23</v>
       </c>
     </row>
     <row r="14" spans="1:7" x14ac:dyDescent="0.45">
@@ -973,39 +973,39 @@
     </row>
     <row r="17" spans="1:7" x14ac:dyDescent="0.45">
       <c r="A17" s="7">
-        <v>46312</v>
+        <v>46315</v>
       </c>
       <c r="B17" s="8"/>
       <c r="C17" s="20" t="s">
         <v>14</v>
       </c>
       <c r="D17" s="10">
-        <v>258.58999999999997</v>
+        <v>258.48</v>
       </c>
       <c r="E17" s="10">
-        <v>230.41</v>
+        <v>227.38</v>
       </c>
       <c r="F17" s="10">
-        <v>240.41</v>
+        <v>237.38</v>
       </c>
       <c r="G17" s="17"/>
     </row>
     <row r="18" spans="1:7" x14ac:dyDescent="0.45">
       <c r="A18" s="11">
-        <v>46311</v>
+        <v>46312</v>
       </c>
       <c r="B18" s="12"/>
       <c r="C18" s="12" t="s">
         <v>14</v>
       </c>
       <c r="D18" s="13">
-        <v>260.04000000000002</v>
+        <v>258.58999999999997</v>
       </c>
       <c r="E18" s="13">
-        <v>234.62</v>
+        <v>230.41</v>
       </c>
       <c r="F18" s="13">
-        <v>244.62</v>
+        <v>240.41</v>
       </c>
       <c r="G18" s="17"/>
     </row>
@@ -1052,41 +1052,41 @@
     </row>
     <row r="22" spans="1:7" x14ac:dyDescent="0.45">
       <c r="A22" s="7">
-        <v>46312</v>
+        <v>46315</v>
       </c>
       <c r="B22" s="8"/>
       <c r="C22" s="20" t="s">
         <v>16</v>
       </c>
       <c r="D22" s="10">
-        <v>260.27</v>
+        <v>259.57</v>
       </c>
       <c r="E22" s="10">
-        <v>228.91</v>
+        <v>226.42</v>
       </c>
       <c r="F22" s="10">
-        <v>238.51</v>
+        <v>236.02</v>
       </c>
       <c r="G22" s="10">
-        <v>225.28</v>
+        <v>222.79</v>
       </c>
     </row>
     <row r="23" spans="1:7" x14ac:dyDescent="0.45">
       <c r="A23" s="11">
-        <v>46312</v>
+        <v>46315</v>
       </c>
       <c r="B23" s="12"/>
       <c r="C23" s="21" t="s">
         <v>17</v>
       </c>
       <c r="D23" s="13">
-        <v>259.99</v>
+        <v>259.94</v>
       </c>
       <c r="E23" s="13">
-        <v>235.62</v>
+        <v>232.65</v>
       </c>
       <c r="F23" s="13">
-        <v>245.62</v>
+        <v>242.65</v>
       </c>
       <c r="G23" s="13" t="s">
         <v>18</v>
@@ -1094,20 +1094,20 @@
     </row>
     <row r="24" spans="1:7" x14ac:dyDescent="0.45">
       <c r="A24" s="7">
-        <v>46312</v>
+        <v>46315</v>
       </c>
       <c r="B24" s="8"/>
       <c r="C24" s="20" t="s">
         <v>19</v>
       </c>
       <c r="D24" s="10">
-        <v>260.35000000000002</v>
+        <v>260.29000000000002</v>
       </c>
       <c r="E24" s="10">
-        <v>234.88</v>
+        <v>231.92</v>
       </c>
       <c r="F24" s="10">
-        <v>244.88</v>
+        <v>241.92</v>
       </c>
       <c r="G24" s="10" t="s">
         <v>18</v>
@@ -1115,41 +1115,41 @@
     </row>
     <row r="25" spans="1:7" x14ac:dyDescent="0.45">
       <c r="A25" s="11">
-        <v>46312</v>
+        <v>46315</v>
       </c>
       <c r="B25" s="12"/>
       <c r="C25" s="21" t="s">
         <v>20</v>
       </c>
       <c r="D25" s="13">
-        <v>257.02</v>
+        <v>256.95</v>
       </c>
       <c r="E25" s="13">
-        <v>235.09</v>
+        <v>232.13</v>
       </c>
       <c r="F25" s="13">
-        <v>245.09</v>
+        <v>242.13</v>
       </c>
       <c r="G25" s="13">
-        <v>230.93</v>
+        <v>227.97</v>
       </c>
     </row>
     <row r="26" spans="1:7" x14ac:dyDescent="0.45">
       <c r="A26" s="7">
-        <v>46312</v>
+        <v>46315</v>
       </c>
       <c r="B26" s="8"/>
       <c r="C26" s="20" t="s">
         <v>21</v>
       </c>
       <c r="D26" s="10">
-        <v>258.58</v>
+        <v>258.51</v>
       </c>
       <c r="E26" s="10">
-        <v>236.55</v>
+        <v>233.57</v>
       </c>
       <c r="F26" s="10">
-        <v>246.55</v>
+        <v>243.57</v>
       </c>
       <c r="G26" s="10" t="s">
         <v>18</v>
@@ -1157,41 +1157,41 @@
     </row>
     <row r="27" spans="1:7" x14ac:dyDescent="0.45">
       <c r="A27" s="11">
-        <v>46311</v>
+        <v>46312</v>
       </c>
       <c r="B27" s="12"/>
       <c r="C27" s="12" t="s">
         <v>16</v>
       </c>
       <c r="D27" s="13">
-        <v>260.23</v>
+        <v>260.27</v>
       </c>
       <c r="E27" s="13">
-        <v>231.65</v>
+        <v>228.91</v>
       </c>
       <c r="F27" s="13">
-        <v>241.25</v>
+        <v>238.51</v>
       </c>
       <c r="G27" s="13">
-        <v>228.02</v>
+        <v>225.28</v>
       </c>
     </row>
     <row r="28" spans="1:7" x14ac:dyDescent="0.45">
       <c r="A28" s="7">
-        <v>46311</v>
+        <v>46312</v>
       </c>
       <c r="B28" s="8"/>
       <c r="C28" s="20" t="s">
         <v>17</v>
       </c>
       <c r="D28" s="10">
-        <v>261.45999999999998</v>
+        <v>259.99</v>
       </c>
       <c r="E28" s="22">
-        <v>239.85</v>
+        <v>235.62</v>
       </c>
       <c r="F28" s="22">
-        <v>249.85</v>
+        <v>245.62</v>
       </c>
       <c r="G28" s="22" t="s">
         <v>18</v>
@@ -1199,20 +1199,20 @@
     </row>
     <row r="29" spans="1:7" x14ac:dyDescent="0.45">
       <c r="A29" s="11">
-        <v>46311</v>
+        <v>46312</v>
       </c>
       <c r="B29" s="12"/>
       <c r="C29" s="12" t="s">
         <v>19</v>
       </c>
       <c r="D29" s="13">
-        <v>261.82</v>
+        <v>260.35000000000002</v>
       </c>
       <c r="E29" s="13">
-        <v>239.09</v>
+        <v>234.88</v>
       </c>
       <c r="F29" s="13">
-        <v>249.1</v>
+        <v>244.88</v>
       </c>
       <c r="G29" s="13" t="s">
         <v>18</v>
@@ -1220,41 +1220,41 @@
     </row>
     <row r="30" spans="1:7" x14ac:dyDescent="0.45">
       <c r="A30" s="7">
-        <v>46311</v>
+        <v>46312</v>
       </c>
       <c r="B30" s="8"/>
       <c r="C30" s="20" t="s">
         <v>20</v>
       </c>
       <c r="D30" s="10">
-        <v>258.49</v>
+        <v>257.02</v>
       </c>
       <c r="E30" s="22">
-        <v>239.32</v>
+        <v>235.09</v>
       </c>
       <c r="F30" s="22">
-        <v>249.32</v>
+        <v>245.09</v>
       </c>
       <c r="G30" s="22">
-        <v>235.16</v>
+        <v>230.93</v>
       </c>
     </row>
     <row r="31" spans="1:7" x14ac:dyDescent="0.45">
       <c r="A31" s="11">
-        <v>46311</v>
+        <v>46312</v>
       </c>
       <c r="B31" s="12"/>
       <c r="C31" s="12" t="s">
         <v>21</v>
       </c>
       <c r="D31" s="13">
-        <v>260.05</v>
+        <v>258.58</v>
       </c>
       <c r="E31" s="13">
-        <v>240.81</v>
+        <v>236.55</v>
       </c>
       <c r="F31" s="13">
-        <v>250.81</v>
+        <v>246.55</v>
       </c>
       <c r="G31" s="13" t="s">
         <v>18</v>
@@ -1301,52 +1301,52 @@
     </row>
     <row r="35" spans="1:7" x14ac:dyDescent="0.45">
       <c r="A35" s="7">
-        <v>46312</v>
+        <v>46315</v>
       </c>
       <c r="B35" s="8"/>
       <c r="C35" s="20" t="s">
         <v>23</v>
       </c>
       <c r="D35" s="10">
-        <v>253.6</v>
+        <v>253.54</v>
       </c>
       <c r="E35" s="10">
-        <v>226.32</v>
+        <v>223.35</v>
       </c>
       <c r="F35" s="10">
-        <v>235.32</v>
+        <v>232.35</v>
       </c>
       <c r="G35" s="17"/>
     </row>
     <row r="36" spans="1:7" x14ac:dyDescent="0.45">
       <c r="A36" s="11">
-        <v>46311</v>
+        <v>46312</v>
       </c>
       <c r="B36" s="12"/>
       <c r="C36" s="12" t="s">
         <v>23</v>
       </c>
       <c r="D36" s="13">
-        <v>255.06</v>
+        <v>253.6</v>
       </c>
       <c r="E36" s="13">
-        <v>229.42</v>
+        <v>226.32</v>
       </c>
       <c r="F36" s="13">
-        <v>238.42</v>
+        <v>235.32</v>
       </c>
       <c r="G36" s="17"/>
     </row>
     <row r="37" spans="1:7" x14ac:dyDescent="0.45">
       <c r="A37" s="7">
-        <v>46312</v>
+        <v>46315</v>
       </c>
       <c r="B37" s="8"/>
       <c r="C37" s="20" t="s">
         <v>24</v>
       </c>
       <c r="D37" s="10">
-        <v>269.22000000000003</v>
+        <v>269.16000000000003</v>
       </c>
       <c r="E37" s="10" t="s">
         <v>18</v>
@@ -1358,14 +1358,14 @@
     </row>
     <row r="38" spans="1:7" x14ac:dyDescent="0.45">
       <c r="A38" s="11">
-        <v>46311</v>
+        <v>46312</v>
       </c>
       <c r="B38" s="12"/>
       <c r="C38" s="12" t="s">
         <v>24</v>
       </c>
       <c r="D38" s="13">
-        <v>270.68</v>
+        <v>269.22000000000003</v>
       </c>
       <c r="E38" s="13" t="s">
         <v>18</v>
@@ -1416,77 +1416,77 @@
     </row>
     <row r="42" spans="1:7" x14ac:dyDescent="0.45">
       <c r="A42" s="7">
-        <v>46312</v>
+        <v>46315</v>
       </c>
       <c r="B42" s="8"/>
       <c r="C42" s="20" t="s">
         <v>26</v>
       </c>
       <c r="D42" s="10">
-        <v>263.54000000000002</v>
+        <v>263.52</v>
       </c>
       <c r="E42" s="10">
-        <v>235.92</v>
+        <v>233.61</v>
       </c>
       <c r="F42" s="10">
-        <v>245.92</v>
+        <v>243.61</v>
       </c>
       <c r="G42" s="17"/>
     </row>
     <row r="43" spans="1:7" x14ac:dyDescent="0.45">
       <c r="A43" s="11">
-        <v>46312</v>
+        <v>46315</v>
       </c>
       <c r="B43" s="12"/>
       <c r="C43" s="21" t="s">
         <v>27</v>
       </c>
       <c r="D43" s="13">
-        <v>263.16000000000003</v>
+        <v>263.13</v>
       </c>
       <c r="E43" s="13">
-        <v>236.33</v>
+        <v>234.02</v>
       </c>
       <c r="F43" s="13">
-        <v>246.33</v>
+        <v>244.02</v>
       </c>
       <c r="G43" s="17"/>
     </row>
     <row r="44" spans="1:7" x14ac:dyDescent="0.45">
       <c r="A44" s="7">
-        <v>46311</v>
+        <v>46312</v>
       </c>
       <c r="B44" s="8"/>
       <c r="C44" s="20" t="s">
         <v>26</v>
       </c>
       <c r="D44" s="10">
-        <v>265.02999999999997</v>
+        <v>263.54000000000002</v>
       </c>
       <c r="E44" s="10">
-        <v>239.37</v>
+        <v>235.92</v>
       </c>
       <c r="F44" s="10">
-        <v>249.37</v>
+        <v>245.92</v>
       </c>
       <c r="G44" s="17"/>
     </row>
     <row r="45" spans="1:7" x14ac:dyDescent="0.45">
       <c r="A45" s="11">
-        <v>46311</v>
+        <v>46312</v>
       </c>
       <c r="B45" s="12"/>
       <c r="C45" s="21" t="s">
         <v>27</v>
       </c>
       <c r="D45" s="13">
-        <v>264.64</v>
+        <v>263.16000000000003</v>
       </c>
       <c r="E45" s="13">
-        <v>239.78</v>
+        <v>236.33</v>
       </c>
       <c r="F45" s="13">
-        <v>249.78</v>
+        <v>246.33</v>
       </c>
       <c r="G45" s="17"/>
     </row>
@@ -1531,77 +1531,77 @@
     </row>
     <row r="49" spans="1:7" x14ac:dyDescent="0.45">
       <c r="A49" s="7">
-        <v>46312</v>
+        <v>46315</v>
       </c>
       <c r="B49" s="8"/>
       <c r="C49" s="20" t="s">
         <v>29</v>
       </c>
       <c r="D49" s="10">
-        <v>257.11</v>
+        <v>257.32</v>
       </c>
       <c r="E49" s="10">
-        <v>231.63</v>
+        <v>228.32</v>
       </c>
       <c r="F49" s="10">
-        <v>241.63</v>
+        <v>238.32</v>
       </c>
       <c r="G49" s="28"/>
     </row>
     <row r="50" spans="1:7" x14ac:dyDescent="0.45">
       <c r="A50" s="11">
-        <v>46312</v>
+        <v>46315</v>
       </c>
       <c r="B50" s="12"/>
       <c r="C50" s="21" t="s">
         <v>30</v>
       </c>
       <c r="D50" s="13">
-        <v>254.65</v>
+        <v>254.85</v>
       </c>
       <c r="E50" s="13">
-        <v>231.25</v>
+        <v>227.94</v>
       </c>
       <c r="F50" s="13">
-        <v>241.25</v>
+        <v>237.94</v>
       </c>
       <c r="G50" s="28"/>
     </row>
     <row r="51" spans="1:7" x14ac:dyDescent="0.45">
       <c r="A51" s="7">
-        <v>46311</v>
+        <v>46312</v>
       </c>
       <c r="B51" s="8"/>
       <c r="C51" s="20" t="s">
         <v>29</v>
       </c>
       <c r="D51" s="10">
-        <v>256.41000000000003</v>
+        <v>257.11</v>
       </c>
       <c r="E51" s="10">
-        <v>234.17</v>
+        <v>231.63</v>
       </c>
       <c r="F51" s="10">
-        <v>244.17</v>
+        <v>241.63</v>
       </c>
       <c r="G51" s="17"/>
     </row>
     <row r="52" spans="1:7" x14ac:dyDescent="0.45">
       <c r="A52" s="11">
-        <v>46311</v>
+        <v>46312</v>
       </c>
       <c r="B52" s="12"/>
       <c r="C52" s="21" t="s">
         <v>30</v>
       </c>
       <c r="D52" s="13">
-        <v>253.94</v>
+        <v>254.65</v>
       </c>
       <c r="E52" s="13">
-        <v>233.79</v>
+        <v>231.25</v>
       </c>
       <c r="F52" s="13">
-        <v>243.79</v>
+        <v>241.25</v>
       </c>
       <c r="G52" s="17"/>
     </row>
@@ -1646,52 +1646,52 @@
     </row>
     <row r="56" spans="1:7" x14ac:dyDescent="0.45">
       <c r="A56" s="7">
-        <v>46312</v>
+        <v>46315</v>
       </c>
       <c r="B56" s="8"/>
       <c r="C56" s="20" t="s">
         <v>32</v>
       </c>
       <c r="D56" s="10">
-        <v>269.75</v>
+        <v>269.68</v>
       </c>
       <c r="E56" s="10">
-        <v>253.71</v>
+        <v>250.92</v>
       </c>
       <c r="F56" s="10">
-        <v>263.70999999999998</v>
+        <v>260.92</v>
       </c>
       <c r="G56" s="17"/>
     </row>
     <row r="57" spans="1:7" x14ac:dyDescent="0.45">
       <c r="A57" s="11">
-        <v>46312</v>
+        <v>46315</v>
       </c>
       <c r="B57" s="12"/>
       <c r="C57" s="21" t="s">
         <v>33</v>
       </c>
       <c r="D57" s="13">
-        <v>257.14</v>
+        <v>257.08</v>
       </c>
       <c r="E57" s="13">
-        <v>235.63</v>
+        <v>232.62</v>
       </c>
       <c r="F57" s="13">
-        <v>245.63</v>
+        <v>242.62</v>
       </c>
       <c r="G57" s="17"/>
     </row>
     <row r="58" spans="1:7" x14ac:dyDescent="0.45">
       <c r="A58" s="7">
-        <v>46312</v>
+        <v>46315</v>
       </c>
       <c r="B58" s="8"/>
       <c r="C58" s="20" t="s">
         <v>34</v>
       </c>
       <c r="D58" s="10">
-        <v>257.89999999999998</v>
+        <v>257.85000000000002</v>
       </c>
       <c r="E58" s="10" t="s">
         <v>18</v>
@@ -1703,17 +1703,17 @@
     </row>
     <row r="59" spans="1:7" x14ac:dyDescent="0.45">
       <c r="A59" s="11">
-        <v>46312</v>
+        <v>46315</v>
       </c>
       <c r="B59" s="12"/>
       <c r="C59" s="21" t="s">
         <v>35</v>
       </c>
       <c r="D59" s="13">
-        <v>254.29</v>
+        <v>254.18</v>
       </c>
       <c r="E59" s="13">
-        <v>230.01</v>
+        <v>227</v>
       </c>
       <c r="F59" s="13" t="s">
         <v>18</v>
@@ -1722,36 +1722,36 @@
     </row>
     <row r="60" spans="1:7" x14ac:dyDescent="0.45">
       <c r="A60" s="7">
-        <v>46312</v>
+        <v>46315</v>
       </c>
       <c r="B60" s="8"/>
       <c r="C60" s="20" t="s">
         <v>36</v>
       </c>
       <c r="D60" s="10">
-        <v>250.12</v>
+        <v>250</v>
       </c>
       <c r="E60" s="10">
-        <v>225.95</v>
+        <v>222.94</v>
       </c>
       <c r="F60" s="10">
-        <v>235.95</v>
+        <v>232.94</v>
       </c>
       <c r="G60" s="17"/>
     </row>
     <row r="61" spans="1:7" x14ac:dyDescent="0.45">
       <c r="A61" s="11">
-        <v>46312</v>
+        <v>46315</v>
       </c>
       <c r="B61" s="12"/>
       <c r="C61" s="21" t="s">
         <v>37</v>
       </c>
       <c r="D61" s="13">
-        <v>257.7</v>
+        <v>257.58</v>
       </c>
       <c r="E61" s="13">
-        <v>247.2</v>
+        <v>244.33</v>
       </c>
       <c r="F61" s="13" t="s">
         <v>18</v>
@@ -1760,52 +1760,52 @@
     </row>
     <row r="62" spans="1:7" x14ac:dyDescent="0.45">
       <c r="A62" s="7">
-        <v>46311</v>
+        <v>46312</v>
       </c>
       <c r="B62" s="8"/>
       <c r="C62" s="20" t="s">
         <v>32</v>
       </c>
       <c r="D62" s="10">
-        <v>271.22000000000003</v>
+        <v>269.75</v>
       </c>
       <c r="E62" s="10">
-        <v>257.98</v>
+        <v>253.71</v>
       </c>
       <c r="F62" s="10">
-        <v>267.98</v>
+        <v>263.70999999999998</v>
       </c>
       <c r="G62" s="17"/>
     </row>
     <row r="63" spans="1:7" x14ac:dyDescent="0.45">
       <c r="A63" s="11">
-        <v>46311</v>
+        <v>46312</v>
       </c>
       <c r="B63" s="12"/>
       <c r="C63" s="21" t="s">
         <v>33</v>
       </c>
       <c r="D63" s="13">
-        <v>258.06</v>
+        <v>257.14</v>
       </c>
       <c r="E63" s="13">
-        <v>239.81</v>
+        <v>235.63</v>
       </c>
       <c r="F63" s="13">
-        <v>249.81</v>
+        <v>245.63</v>
       </c>
       <c r="G63" s="17"/>
     </row>
     <row r="64" spans="1:7" x14ac:dyDescent="0.45">
       <c r="A64" s="7">
-        <v>46311</v>
+        <v>46312</v>
       </c>
       <c r="B64" s="8"/>
       <c r="C64" s="20" t="s">
         <v>34</v>
       </c>
       <c r="D64" s="10">
-        <v>258.83</v>
+        <v>257.89999999999998</v>
       </c>
       <c r="E64" s="10" t="s">
         <v>18</v>
@@ -1817,17 +1817,17 @@
     </row>
     <row r="65" spans="1:6" x14ac:dyDescent="0.45">
       <c r="A65" s="11">
-        <v>46311</v>
+        <v>46312</v>
       </c>
       <c r="B65" s="12"/>
       <c r="C65" s="21" t="s">
         <v>35</v>
       </c>
       <c r="D65" s="13">
-        <v>255.19</v>
+        <v>254.29</v>
       </c>
       <c r="E65" s="13">
-        <v>234.19</v>
+        <v>230.01</v>
       </c>
       <c r="F65" s="13" t="s">
         <v>18</v>
@@ -1835,35 +1835,35 @@
     </row>
     <row r="66" spans="1:6" x14ac:dyDescent="0.45">
       <c r="A66" s="7">
-        <v>46311</v>
+        <v>46312</v>
       </c>
       <c r="B66" s="8"/>
       <c r="C66" s="20" t="s">
         <v>36</v>
       </c>
       <c r="D66" s="10">
-        <v>251.02</v>
+        <v>250.12</v>
       </c>
       <c r="E66" s="10">
-        <v>230.13</v>
+        <v>225.95</v>
       </c>
       <c r="F66" s="10">
-        <v>240.13</v>
+        <v>235.95</v>
       </c>
     </row>
     <row r="67" spans="1:6" x14ac:dyDescent="0.45">
       <c r="A67" s="11">
-        <v>46311</v>
+        <v>46312</v>
       </c>
       <c r="B67" s="12"/>
       <c r="C67" s="21" t="s">
         <v>37</v>
       </c>
       <c r="D67" s="13">
-        <v>259.14999999999998</v>
+        <v>257.7</v>
       </c>
       <c r="E67" s="13">
-        <v>251.46</v>
+        <v>247.2</v>
       </c>
       <c r="F67" s="13" t="s">
         <v>18</v>
@@ -1891,12 +1891,14 @@
 </file>
 
 <file path=customXml/item1.xml><?xml version="1.0" encoding="utf-8"?>
-<?mso-contentType ?>
-<FormTemplates xmlns="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms">
-  <Display>DocumentLibraryForm</Display>
-  <Edit>DocumentLibraryForm</Edit>
-  <New>DocumentLibraryForm</New>
-</FormTemplates>
+<p:properties xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls">
+  <documentManagement>
+    <lcf76f155ced4ddcb4097134ff3c332f xmlns="87276d81-85f4-4ef2-9e6e-55066304288f">
+      <Terms xmlns="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
+    </lcf76f155ced4ddcb4097134ff3c332f>
+    <TaxCatchAll xmlns="b23b8984-eafa-4e79-985e-54f52f3da58e" xsi:nil="true"/>
+  </documentManagement>
+</p:properties>
 </file>
 
 <file path=customXml/item2.xml><?xml version="1.0" encoding="utf-8"?>
@@ -2160,20 +2162,21 @@
 </file>
 
 <file path=customXml/item3.xml><?xml version="1.0" encoding="utf-8"?>
-<p:properties xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls">
-  <documentManagement>
-    <lcf76f155ced4ddcb4097134ff3c332f xmlns="87276d81-85f4-4ef2-9e6e-55066304288f">
-      <Terms xmlns="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
-    </lcf76f155ced4ddcb4097134ff3c332f>
-    <TaxCatchAll xmlns="b23b8984-eafa-4e79-985e-54f52f3da58e" xsi:nil="true"/>
-  </documentManagement>
-</p:properties>
+<?mso-contentType ?>
+<FormTemplates xmlns="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms">
+  <Display>DocumentLibraryForm</Display>
+  <Edit>DocumentLibraryForm</Edit>
+  <New>DocumentLibraryForm</New>
+</FormTemplates>
 </file>
 
 <file path=customXml/itemProps1.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{F60519E9-FD90-4339-869C-BC2F85719BB8}">
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{57A83D98-2BAE-4D83-823A-D31C464B620C}">
   <ds:schemaRefs>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/properties"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
+    <ds:schemaRef ds:uri="87276d81-85f4-4ef2-9e6e-55066304288f"/>
+    <ds:schemaRef ds:uri="b23b8984-eafa-4e79-985e-54f52f3da58e"/>
   </ds:schemaRefs>
 </ds:datastoreItem>
 </file>
@@ -2199,12 +2202,9 @@
 </file>
 
 <file path=customXml/itemProps3.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{57A83D98-2BAE-4D83-823A-D31C464B620C}">
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{F60519E9-FD90-4339-869C-BC2F85719BB8}">
   <ds:schemaRefs>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/properties"/>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
-    <ds:schemaRef ds:uri="87276d81-85f4-4ef2-9e6e-55066304288f"/>
-    <ds:schemaRef ds:uri="b23b8984-eafa-4e79-985e-54f52f3da58e"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms"/>
   </ds:schemaRefs>
 </ds:datastoreItem>
 </file>

</xml_diff>

<commit_message>
Tue Oct 20 06:08:33 UTC 2026
</commit_message>
<xml_diff>
--- a/bp.com-content-dam-bp-country-sites-en_au-australia-home-products-services-pricing-tgp-excel.xlsx
+++ b/bp.com-content-dam-bp-country-sites-en_au-australia-home-products-services-pricing-tgp-excel.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://bp365.sharepoint.com/sites/WholesalePricing/Shared Documents/B2C/TGP/Daily TGP/Web TGP/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="14_{691F818D-7C71-4FD4-B7A8-5797E2161298}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="14_{C4ACF7A7-558F-4F6C-8016-C29AF31ECD46}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-8310" yWindow="-16395" windowWidth="29040" windowHeight="15720" xr2:uid="{1B412EEF-F96D-4DF4-A4E9-C7F0F183C2FB}"/>
+    <workbookView xWindow="-28920" yWindow="-60" windowWidth="29040" windowHeight="15720" xr2:uid="{1B412EEF-F96D-4DF4-A4E9-C7F0F183C2FB}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
@@ -715,15 +715,15 @@
     <pageSetUpPr fitToPage="1"/>
   </sheetPr>
   <dimension ref="A1:G67"/>
-  <sheetFormatPr defaultRowHeight="14.25" x14ac:dyDescent="0.45"/>
+  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
-    <col min="1" max="1" width="76.3984375" bestFit="1" customWidth="1"/>
-    <col min="2" max="2" width="6.3984375"/>
-    <col min="3" max="3" width="18.1328125" bestFit="1" customWidth="1"/>
-    <col min="4" max="7" width="7.1328125" bestFit="1" customWidth="1"/>
+    <col min="1" max="1" width="76.42578125" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="6.42578125"/>
+    <col min="3" max="3" width="18.140625" bestFit="1" customWidth="1"/>
+    <col min="4" max="7" width="7.140625" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:7" ht="22.15" x14ac:dyDescent="0.45">
+    <row r="1" spans="1:7" ht="23.25" x14ac:dyDescent="0.25">
       <c r="A1" s="30" t="s">
         <v>0</v>
       </c>
@@ -734,7 +734,7 @@
       <c r="F1" s="2"/>
       <c r="G1" s="2"/>
     </row>
-    <row r="2" spans="1:7" x14ac:dyDescent="0.45">
+    <row r="2" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A2" s="3"/>
       <c r="B2" s="1"/>
       <c r="C2" s="1"/>
@@ -743,7 +743,7 @@
       <c r="F2" s="2"/>
       <c r="G2" s="2"/>
     </row>
-    <row r="3" spans="1:7" x14ac:dyDescent="0.45">
+    <row r="3" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A3" s="3" t="s">
         <v>1</v>
       </c>
@@ -754,7 +754,7 @@
       <c r="F3" s="2"/>
       <c r="G3" s="2"/>
     </row>
-    <row r="4" spans="1:7" x14ac:dyDescent="0.45">
+    <row r="4" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A4" s="3" t="s">
         <v>2</v>
       </c>
@@ -765,7 +765,7 @@
       <c r="F4" s="2"/>
       <c r="G4" s="2"/>
     </row>
-    <row r="5" spans="1:7" x14ac:dyDescent="0.45">
+    <row r="5" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A5" s="3"/>
       <c r="B5" s="3"/>
       <c r="C5" s="1"/>
@@ -774,7 +774,7 @@
       <c r="F5" s="2"/>
       <c r="G5" s="2"/>
     </row>
-    <row r="6" spans="1:7" ht="20.25" x14ac:dyDescent="0.45">
+    <row r="6" spans="1:7" ht="20.25" x14ac:dyDescent="0.25">
       <c r="A6" s="29" t="s">
         <v>3</v>
       </c>
@@ -785,7 +785,7 @@
       <c r="F6" s="2"/>
       <c r="G6" s="2"/>
     </row>
-    <row r="7" spans="1:7" x14ac:dyDescent="0.45">
+    <row r="7" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A7" s="4" t="s">
         <v>4</v>
       </c>
@@ -806,133 +806,133 @@
         <v>9</v>
       </c>
     </row>
-    <row r="8" spans="1:7" x14ac:dyDescent="0.45">
+    <row r="8" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A8" s="7">
-        <v>46315</v>
+        <v>46316</v>
       </c>
       <c r="B8" s="8"/>
       <c r="C8" s="9" t="s">
         <v>10</v>
       </c>
       <c r="D8" s="10">
-        <v>258.45</v>
+        <v>258.24</v>
       </c>
       <c r="E8" s="10">
-        <v>226.28</v>
+        <v>223.09</v>
       </c>
       <c r="F8" s="10">
-        <v>236.28</v>
+        <v>233.09</v>
       </c>
       <c r="G8" s="10">
-        <v>223.89</v>
-      </c>
-    </row>
-    <row r="9" spans="1:7" x14ac:dyDescent="0.45">
+        <v>220.71</v>
+      </c>
+    </row>
+    <row r="9" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A9" s="11">
-        <v>46315</v>
+        <v>46316</v>
       </c>
       <c r="B9" s="12"/>
       <c r="C9" s="12" t="s">
         <v>11</v>
       </c>
       <c r="D9" s="13">
-        <v>258.45</v>
+        <v>258.24</v>
       </c>
       <c r="E9" s="13">
-        <v>226.28</v>
+        <v>223.09</v>
       </c>
       <c r="F9" s="13">
-        <v>236.28</v>
+        <v>233.09</v>
       </c>
       <c r="G9" s="13">
-        <v>223.89</v>
-      </c>
-    </row>
-    <row r="10" spans="1:7" x14ac:dyDescent="0.45">
+        <v>220.71</v>
+      </c>
+    </row>
+    <row r="10" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A10" s="7">
-        <v>46315</v>
+        <v>46316</v>
       </c>
       <c r="B10" s="8"/>
       <c r="C10" s="9" t="s">
         <v>12</v>
       </c>
       <c r="D10" s="10">
-        <v>254.99</v>
+        <v>255.43</v>
       </c>
       <c r="E10" s="10">
-        <v>224.4</v>
+        <v>221.84</v>
       </c>
       <c r="F10" s="10">
-        <v>234.4</v>
+        <v>231.84</v>
       </c>
       <c r="G10" s="10">
-        <v>222.8</v>
-      </c>
-    </row>
-    <row r="11" spans="1:7" x14ac:dyDescent="0.45">
+        <v>220.25</v>
+      </c>
+    </row>
+    <row r="11" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A11" s="11">
-        <v>46312</v>
+        <v>46315</v>
       </c>
       <c r="B11" s="12"/>
       <c r="C11" s="12" t="s">
         <v>10</v>
       </c>
       <c r="D11" s="13">
-        <v>259.14</v>
+        <v>258.45</v>
       </c>
       <c r="E11" s="13">
-        <v>228.77</v>
+        <v>226.28</v>
       </c>
       <c r="F11" s="13">
-        <v>238.77</v>
+        <v>236.28</v>
       </c>
       <c r="G11" s="13">
-        <v>226.39</v>
-      </c>
-    </row>
-    <row r="12" spans="1:7" x14ac:dyDescent="0.45">
+        <v>223.89</v>
+      </c>
+    </row>
+    <row r="12" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A12" s="7">
-        <v>46312</v>
+        <v>46315</v>
       </c>
       <c r="B12" s="8"/>
       <c r="C12" s="9" t="s">
         <v>11</v>
       </c>
       <c r="D12" s="10">
-        <v>259.14</v>
+        <v>258.45</v>
       </c>
       <c r="E12" s="10">
-        <v>228.77</v>
+        <v>226.28</v>
       </c>
       <c r="F12" s="10">
-        <v>238.77</v>
+        <v>236.28</v>
       </c>
       <c r="G12" s="10">
-        <v>226.39</v>
-      </c>
-    </row>
-    <row r="13" spans="1:7" x14ac:dyDescent="0.45">
+        <v>223.89</v>
+      </c>
+    </row>
+    <row r="13" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A13" s="11">
-        <v>46312</v>
+        <v>46315</v>
       </c>
       <c r="B13" s="12"/>
       <c r="C13" s="12" t="s">
         <v>12</v>
       </c>
       <c r="D13" s="13">
-        <v>255.05</v>
+        <v>254.99</v>
       </c>
       <c r="E13" s="13">
-        <v>226.83</v>
+        <v>224.4</v>
       </c>
       <c r="F13" s="13">
-        <v>236.83</v>
+        <v>234.4</v>
       </c>
       <c r="G13" s="13">
-        <v>225.23</v>
-      </c>
-    </row>
-    <row r="14" spans="1:7" x14ac:dyDescent="0.45">
+        <v>222.8</v>
+      </c>
+    </row>
+    <row r="14" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A14" s="14"/>
       <c r="B14" s="14"/>
       <c r="C14" s="15"/>
@@ -941,7 +941,7 @@
       <c r="F14" s="16"/>
       <c r="G14" s="16"/>
     </row>
-    <row r="15" spans="1:7" ht="20.25" x14ac:dyDescent="0.45">
+    <row r="15" spans="1:7" ht="20.25" x14ac:dyDescent="0.25">
       <c r="A15" s="29" t="s">
         <v>13</v>
       </c>
@@ -952,7 +952,7 @@
       <c r="F15" s="17"/>
       <c r="G15" s="17"/>
     </row>
-    <row r="16" spans="1:7" x14ac:dyDescent="0.45">
+    <row r="16" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A16" s="4" t="s">
         <v>4</v>
       </c>
@@ -971,45 +971,45 @@
       </c>
       <c r="G16" s="17"/>
     </row>
-    <row r="17" spans="1:7" x14ac:dyDescent="0.45">
+    <row r="17" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A17" s="7">
-        <v>46315</v>
+        <v>46316</v>
       </c>
       <c r="B17" s="8"/>
       <c r="C17" s="20" t="s">
         <v>14</v>
       </c>
       <c r="D17" s="10">
-        <v>258.48</v>
+        <v>258.89</v>
       </c>
       <c r="E17" s="10">
-        <v>227.38</v>
+        <v>224.78</v>
       </c>
       <c r="F17" s="10">
-        <v>237.38</v>
+        <v>234.78</v>
       </c>
       <c r="G17" s="17"/>
     </row>
-    <row r="18" spans="1:7" x14ac:dyDescent="0.45">
+    <row r="18" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A18" s="11">
-        <v>46312</v>
+        <v>46315</v>
       </c>
       <c r="B18" s="12"/>
       <c r="C18" s="12" t="s">
         <v>14</v>
       </c>
       <c r="D18" s="13">
-        <v>258.58999999999997</v>
+        <v>258.48</v>
       </c>
       <c r="E18" s="13">
-        <v>230.41</v>
+        <v>227.38</v>
       </c>
       <c r="F18" s="13">
-        <v>240.41</v>
+        <v>237.38</v>
       </c>
       <c r="G18" s="17"/>
     </row>
-    <row r="19" spans="1:7" x14ac:dyDescent="0.45">
+    <row r="19" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A19" s="14"/>
       <c r="B19" s="14"/>
       <c r="C19" s="15"/>
@@ -1018,7 +1018,7 @@
       <c r="F19" s="16"/>
       <c r="G19" s="17"/>
     </row>
-    <row r="20" spans="1:7" ht="20.25" x14ac:dyDescent="0.45">
+    <row r="20" spans="1:7" ht="20.25" x14ac:dyDescent="0.25">
       <c r="A20" s="29" t="s">
         <v>15</v>
       </c>
@@ -1029,7 +1029,7 @@
       <c r="F20" s="17"/>
       <c r="G20" s="17"/>
     </row>
-    <row r="21" spans="1:7" x14ac:dyDescent="0.45">
+    <row r="21" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A21" s="4" t="s">
         <v>4</v>
       </c>
@@ -1050,217 +1050,217 @@
         <v>9</v>
       </c>
     </row>
-    <row r="22" spans="1:7" x14ac:dyDescent="0.45">
+    <row r="22" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A22" s="7">
-        <v>46315</v>
+        <v>46316</v>
       </c>
       <c r="B22" s="8"/>
       <c r="C22" s="20" t="s">
         <v>16</v>
       </c>
       <c r="D22" s="10">
-        <v>259.57</v>
+        <v>259.37</v>
       </c>
       <c r="E22" s="10">
-        <v>226.42</v>
+        <v>223.23</v>
       </c>
       <c r="F22" s="10">
-        <v>236.02</v>
+        <v>232.83</v>
       </c>
       <c r="G22" s="10">
-        <v>222.79</v>
-      </c>
-    </row>
-    <row r="23" spans="1:7" x14ac:dyDescent="0.45">
+        <v>219.6</v>
+      </c>
+    </row>
+    <row r="23" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A23" s="11">
-        <v>46315</v>
+        <v>46316</v>
       </c>
       <c r="B23" s="12"/>
       <c r="C23" s="21" t="s">
         <v>17</v>
       </c>
       <c r="D23" s="13">
-        <v>259.94</v>
+        <v>260.39</v>
       </c>
       <c r="E23" s="13">
-        <v>232.65</v>
+        <v>230.11</v>
       </c>
       <c r="F23" s="13">
-        <v>242.65</v>
+        <v>240.11</v>
       </c>
       <c r="G23" s="13" t="s">
         <v>18</v>
       </c>
     </row>
-    <row r="24" spans="1:7" x14ac:dyDescent="0.45">
+    <row r="24" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A24" s="7">
-        <v>46315</v>
+        <v>46316</v>
       </c>
       <c r="B24" s="8"/>
       <c r="C24" s="20" t="s">
         <v>19</v>
       </c>
       <c r="D24" s="10">
-        <v>260.29000000000002</v>
+        <v>260.74</v>
       </c>
       <c r="E24" s="10">
-        <v>231.92</v>
+        <v>229.38</v>
       </c>
       <c r="F24" s="10">
-        <v>241.92</v>
+        <v>239.38</v>
       </c>
       <c r="G24" s="10" t="s">
         <v>18</v>
       </c>
     </row>
-    <row r="25" spans="1:7" x14ac:dyDescent="0.45">
+    <row r="25" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A25" s="11">
-        <v>46315</v>
+        <v>46316</v>
       </c>
       <c r="B25" s="12"/>
       <c r="C25" s="21" t="s">
         <v>20</v>
       </c>
       <c r="D25" s="13">
-        <v>256.95</v>
+        <v>257.39999999999998</v>
       </c>
       <c r="E25" s="13">
-        <v>232.13</v>
+        <v>229.59</v>
       </c>
       <c r="F25" s="13">
-        <v>242.13</v>
+        <v>239.59</v>
       </c>
       <c r="G25" s="13">
-        <v>227.97</v>
-      </c>
-    </row>
-    <row r="26" spans="1:7" x14ac:dyDescent="0.45">
+        <v>225.43</v>
+      </c>
+    </row>
+    <row r="26" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A26" s="7">
-        <v>46315</v>
+        <v>46316</v>
       </c>
       <c r="B26" s="8"/>
       <c r="C26" s="20" t="s">
         <v>21</v>
       </c>
       <c r="D26" s="10">
-        <v>258.51</v>
+        <v>258.94</v>
       </c>
       <c r="E26" s="10">
-        <v>233.57</v>
+        <v>231.01</v>
       </c>
       <c r="F26" s="10">
-        <v>243.57</v>
+        <v>241.01</v>
       </c>
       <c r="G26" s="10" t="s">
         <v>18</v>
       </c>
     </row>
-    <row r="27" spans="1:7" x14ac:dyDescent="0.45">
+    <row r="27" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A27" s="11">
-        <v>46312</v>
+        <v>46315</v>
       </c>
       <c r="B27" s="12"/>
       <c r="C27" s="12" t="s">
         <v>16</v>
       </c>
       <c r="D27" s="13">
-        <v>260.27</v>
+        <v>259.57</v>
       </c>
       <c r="E27" s="13">
-        <v>228.91</v>
+        <v>226.42</v>
       </c>
       <c r="F27" s="13">
-        <v>238.51</v>
+        <v>236.02</v>
       </c>
       <c r="G27" s="13">
-        <v>225.28</v>
-      </c>
-    </row>
-    <row r="28" spans="1:7" x14ac:dyDescent="0.45">
+        <v>222.79</v>
+      </c>
+    </row>
+    <row r="28" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A28" s="7">
-        <v>46312</v>
+        <v>46315</v>
       </c>
       <c r="B28" s="8"/>
       <c r="C28" s="20" t="s">
         <v>17</v>
       </c>
       <c r="D28" s="10">
-        <v>259.99</v>
+        <v>259.94</v>
       </c>
       <c r="E28" s="22">
-        <v>235.62</v>
+        <v>232.65</v>
       </c>
       <c r="F28" s="22">
-        <v>245.62</v>
+        <v>242.65</v>
       </c>
       <c r="G28" s="22" t="s">
         <v>18</v>
       </c>
     </row>
-    <row r="29" spans="1:7" x14ac:dyDescent="0.45">
+    <row r="29" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A29" s="11">
-        <v>46312</v>
+        <v>46315</v>
       </c>
       <c r="B29" s="12"/>
       <c r="C29" s="12" t="s">
         <v>19</v>
       </c>
       <c r="D29" s="13">
-        <v>260.35000000000002</v>
+        <v>260.29000000000002</v>
       </c>
       <c r="E29" s="13">
-        <v>234.88</v>
+        <v>231.92</v>
       </c>
       <c r="F29" s="13">
-        <v>244.88</v>
+        <v>241.92</v>
       </c>
       <c r="G29" s="13" t="s">
         <v>18</v>
       </c>
     </row>
-    <row r="30" spans="1:7" x14ac:dyDescent="0.45">
+    <row r="30" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A30" s="7">
-        <v>46312</v>
+        <v>46315</v>
       </c>
       <c r="B30" s="8"/>
       <c r="C30" s="20" t="s">
         <v>20</v>
       </c>
       <c r="D30" s="10">
-        <v>257.02</v>
+        <v>256.95</v>
       </c>
       <c r="E30" s="22">
-        <v>235.09</v>
+        <v>232.13</v>
       </c>
       <c r="F30" s="22">
-        <v>245.09</v>
+        <v>242.13</v>
       </c>
       <c r="G30" s="22">
-        <v>230.93</v>
-      </c>
-    </row>
-    <row r="31" spans="1:7" x14ac:dyDescent="0.45">
+        <v>227.97</v>
+      </c>
+    </row>
+    <row r="31" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A31" s="11">
-        <v>46312</v>
+        <v>46315</v>
       </c>
       <c r="B31" s="12"/>
       <c r="C31" s="12" t="s">
         <v>21</v>
       </c>
       <c r="D31" s="13">
-        <v>258.58</v>
+        <v>258.51</v>
       </c>
       <c r="E31" s="13">
-        <v>236.55</v>
+        <v>233.57</v>
       </c>
       <c r="F31" s="13">
-        <v>246.55</v>
+        <v>243.57</v>
       </c>
       <c r="G31" s="13" t="s">
         <v>18</v>
       </c>
     </row>
-    <row r="32" spans="1:7" x14ac:dyDescent="0.45">
+    <row r="32" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A32" s="14"/>
       <c r="B32" s="14"/>
       <c r="C32" s="15"/>
@@ -1269,7 +1269,7 @@
       <c r="F32" s="17"/>
       <c r="G32" s="17"/>
     </row>
-    <row r="33" spans="1:7" ht="20.25" x14ac:dyDescent="0.45">
+    <row r="33" spans="1:7" ht="20.25" x14ac:dyDescent="0.25">
       <c r="A33" s="29" t="s">
         <v>22</v>
       </c>
@@ -1280,7 +1280,7 @@
       <c r="F33" s="17"/>
       <c r="G33" s="17"/>
     </row>
-    <row r="34" spans="1:7" x14ac:dyDescent="0.45">
+    <row r="34" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A34" s="23" t="s">
         <v>4</v>
       </c>
@@ -1299,54 +1299,54 @@
       </c>
       <c r="G34" s="17"/>
     </row>
-    <row r="35" spans="1:7" x14ac:dyDescent="0.45">
+    <row r="35" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A35" s="7">
-        <v>46315</v>
+        <v>46316</v>
       </c>
       <c r="B35" s="8"/>
       <c r="C35" s="20" t="s">
         <v>23</v>
       </c>
       <c r="D35" s="10">
-        <v>253.54</v>
+        <v>253.98</v>
       </c>
       <c r="E35" s="10">
-        <v>223.35</v>
+        <v>220.8</v>
       </c>
       <c r="F35" s="10">
-        <v>232.35</v>
+        <v>229.8</v>
       </c>
       <c r="G35" s="17"/>
     </row>
-    <row r="36" spans="1:7" x14ac:dyDescent="0.45">
+    <row r="36" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A36" s="11">
-        <v>46312</v>
+        <v>46315</v>
       </c>
       <c r="B36" s="12"/>
       <c r="C36" s="12" t="s">
         <v>23</v>
       </c>
       <c r="D36" s="13">
-        <v>253.6</v>
+        <v>253.54</v>
       </c>
       <c r="E36" s="13">
-        <v>226.32</v>
+        <v>223.35</v>
       </c>
       <c r="F36" s="13">
-        <v>235.32</v>
+        <v>232.35</v>
       </c>
       <c r="G36" s="17"/>
     </row>
-    <row r="37" spans="1:7" x14ac:dyDescent="0.45">
+    <row r="37" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A37" s="7">
-        <v>46315</v>
+        <v>46316</v>
       </c>
       <c r="B37" s="8"/>
       <c r="C37" s="20" t="s">
         <v>24</v>
       </c>
       <c r="D37" s="10">
-        <v>269.16000000000003</v>
+        <v>269.60000000000002</v>
       </c>
       <c r="E37" s="10" t="s">
         <v>18</v>
@@ -1356,16 +1356,16 @@
       </c>
       <c r="G37" s="17"/>
     </row>
-    <row r="38" spans="1:7" x14ac:dyDescent="0.45">
+    <row r="38" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A38" s="11">
-        <v>46312</v>
+        <v>46315</v>
       </c>
       <c r="B38" s="12"/>
       <c r="C38" s="12" t="s">
         <v>24</v>
       </c>
       <c r="D38" s="13">
-        <v>269.22000000000003</v>
+        <v>269.16000000000003</v>
       </c>
       <c r="E38" s="13" t="s">
         <v>18</v>
@@ -1375,7 +1375,7 @@
       </c>
       <c r="G38" s="17"/>
     </row>
-    <row r="39" spans="1:7" x14ac:dyDescent="0.45">
+    <row r="39" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A39" s="24"/>
       <c r="B39" s="24"/>
       <c r="C39" s="15"/>
@@ -1384,7 +1384,7 @@
       <c r="F39" s="17"/>
       <c r="G39" s="17"/>
     </row>
-    <row r="40" spans="1:7" ht="20.25" x14ac:dyDescent="0.45">
+    <row r="40" spans="1:7" ht="20.25" x14ac:dyDescent="0.25">
       <c r="A40" s="29" t="s">
         <v>25</v>
       </c>
@@ -1395,7 +1395,7 @@
       <c r="F40" s="17"/>
       <c r="G40" s="17"/>
     </row>
-    <row r="41" spans="1:7" x14ac:dyDescent="0.45">
+    <row r="41" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A41" s="23" t="s">
         <v>4</v>
       </c>
@@ -1414,83 +1414,83 @@
       </c>
       <c r="G41" s="17"/>
     </row>
-    <row r="42" spans="1:7" x14ac:dyDescent="0.45">
+    <row r="42" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A42" s="7">
-        <v>46315</v>
+        <v>46316</v>
       </c>
       <c r="B42" s="8"/>
       <c r="C42" s="20" t="s">
         <v>26</v>
       </c>
       <c r="D42" s="10">
-        <v>263.52</v>
+        <v>264</v>
       </c>
       <c r="E42" s="10">
-        <v>233.61</v>
+        <v>231.3</v>
       </c>
       <c r="F42" s="10">
-        <v>243.61</v>
+        <v>241.3</v>
       </c>
       <c r="G42" s="17"/>
     </row>
-    <row r="43" spans="1:7" x14ac:dyDescent="0.45">
+    <row r="43" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A43" s="11">
-        <v>46315</v>
+        <v>46316</v>
       </c>
       <c r="B43" s="12"/>
       <c r="C43" s="21" t="s">
         <v>27</v>
       </c>
       <c r="D43" s="13">
-        <v>263.13</v>
+        <v>263.61</v>
       </c>
       <c r="E43" s="13">
-        <v>234.02</v>
+        <v>231.71</v>
       </c>
       <c r="F43" s="13">
-        <v>244.02</v>
+        <v>241.71</v>
       </c>
       <c r="G43" s="17"/>
     </row>
-    <row r="44" spans="1:7" x14ac:dyDescent="0.45">
+    <row r="44" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A44" s="7">
-        <v>46312</v>
+        <v>46315</v>
       </c>
       <c r="B44" s="8"/>
       <c r="C44" s="20" t="s">
         <v>26</v>
       </c>
       <c r="D44" s="10">
-        <v>263.54000000000002</v>
+        <v>263.52</v>
       </c>
       <c r="E44" s="10">
-        <v>235.92</v>
+        <v>233.61</v>
       </c>
       <c r="F44" s="10">
-        <v>245.92</v>
+        <v>243.61</v>
       </c>
       <c r="G44" s="17"/>
     </row>
-    <row r="45" spans="1:7" x14ac:dyDescent="0.45">
+    <row r="45" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A45" s="11">
-        <v>46312</v>
+        <v>46315</v>
       </c>
       <c r="B45" s="12"/>
       <c r="C45" s="21" t="s">
         <v>27</v>
       </c>
       <c r="D45" s="13">
-        <v>263.16000000000003</v>
+        <v>263.13</v>
       </c>
       <c r="E45" s="13">
-        <v>236.33</v>
+        <v>234.02</v>
       </c>
       <c r="F45" s="13">
-        <v>246.33</v>
+        <v>244.02</v>
       </c>
       <c r="G45" s="17"/>
     </row>
-    <row r="46" spans="1:7" x14ac:dyDescent="0.45">
+    <row r="46" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A46" s="14"/>
       <c r="B46" s="24"/>
       <c r="C46" s="15"/>
@@ -1499,7 +1499,7 @@
       <c r="F46" s="16"/>
       <c r="G46" s="17"/>
     </row>
-    <row r="47" spans="1:7" ht="20.25" x14ac:dyDescent="0.45">
+    <row r="47" spans="1:7" ht="20.25" x14ac:dyDescent="0.25">
       <c r="A47" s="25" t="s">
         <v>28</v>
       </c>
@@ -1510,7 +1510,7 @@
       <c r="F47" s="17"/>
       <c r="G47" s="17"/>
     </row>
-    <row r="48" spans="1:7" x14ac:dyDescent="0.45">
+    <row r="48" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A48" s="23" t="s">
         <v>4</v>
       </c>
@@ -1529,83 +1529,83 @@
       </c>
       <c r="G48" s="17"/>
     </row>
-    <row r="49" spans="1:7" x14ac:dyDescent="0.45">
+    <row r="49" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A49" s="7">
-        <v>46315</v>
+        <v>46316</v>
       </c>
       <c r="B49" s="8"/>
       <c r="C49" s="20" t="s">
         <v>29</v>
       </c>
       <c r="D49" s="10">
-        <v>257.32</v>
+        <v>255.72</v>
       </c>
       <c r="E49" s="10">
-        <v>228.32</v>
+        <v>225.15</v>
       </c>
       <c r="F49" s="10">
-        <v>238.32</v>
+        <v>235.15</v>
       </c>
       <c r="G49" s="28"/>
     </row>
-    <row r="50" spans="1:7" x14ac:dyDescent="0.45">
+    <row r="50" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A50" s="11">
-        <v>46315</v>
+        <v>46316</v>
       </c>
       <c r="B50" s="12"/>
       <c r="C50" s="21" t="s">
         <v>30</v>
       </c>
       <c r="D50" s="13">
-        <v>254.85</v>
+        <v>253.24</v>
       </c>
       <c r="E50" s="13">
-        <v>227.94</v>
+        <v>224.75</v>
       </c>
       <c r="F50" s="13">
-        <v>237.94</v>
+        <v>234.75</v>
       </c>
       <c r="G50" s="28"/>
     </row>
-    <row r="51" spans="1:7" x14ac:dyDescent="0.45">
+    <row r="51" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A51" s="7">
-        <v>46312</v>
+        <v>46315</v>
       </c>
       <c r="B51" s="8"/>
       <c r="C51" s="20" t="s">
         <v>29</v>
       </c>
       <c r="D51" s="10">
-        <v>257.11</v>
+        <v>257.32</v>
       </c>
       <c r="E51" s="10">
-        <v>231.63</v>
+        <v>228.32</v>
       </c>
       <c r="F51" s="10">
-        <v>241.63</v>
+        <v>238.32</v>
       </c>
       <c r="G51" s="17"/>
     </row>
-    <row r="52" spans="1:7" x14ac:dyDescent="0.45">
+    <row r="52" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A52" s="11">
-        <v>46312</v>
+        <v>46315</v>
       </c>
       <c r="B52" s="12"/>
       <c r="C52" s="21" t="s">
         <v>30</v>
       </c>
       <c r="D52" s="13">
-        <v>254.65</v>
+        <v>254.85</v>
       </c>
       <c r="E52" s="13">
-        <v>231.25</v>
+        <v>227.94</v>
       </c>
       <c r="F52" s="13">
-        <v>241.25</v>
+        <v>237.94</v>
       </c>
       <c r="G52" s="17"/>
     </row>
-    <row r="53" spans="1:7" x14ac:dyDescent="0.45">
+    <row r="53" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A53" s="14"/>
       <c r="B53" s="14"/>
       <c r="C53" s="15"/>
@@ -1614,7 +1614,7 @@
       <c r="F53" s="16"/>
       <c r="G53" s="17"/>
     </row>
-    <row r="54" spans="1:7" ht="20.25" x14ac:dyDescent="0.45">
+    <row r="54" spans="1:7" ht="20.25" x14ac:dyDescent="0.25">
       <c r="A54" s="27" t="s">
         <v>31</v>
       </c>
@@ -1625,7 +1625,7 @@
       <c r="F54" s="17"/>
       <c r="G54" s="17"/>
     </row>
-    <row r="55" spans="1:7" x14ac:dyDescent="0.45">
+    <row r="55" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A55" s="23" t="s">
         <v>4</v>
       </c>
@@ -1644,54 +1644,54 @@
       </c>
       <c r="G55" s="17"/>
     </row>
-    <row r="56" spans="1:7" x14ac:dyDescent="0.45">
+    <row r="56" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A56" s="7">
-        <v>46315</v>
+        <v>46316</v>
       </c>
       <c r="B56" s="8"/>
       <c r="C56" s="20" t="s">
         <v>32</v>
       </c>
       <c r="D56" s="10">
-        <v>269.68</v>
+        <v>270.11</v>
       </c>
       <c r="E56" s="10">
-        <v>250.92</v>
+        <v>248.54</v>
       </c>
       <c r="F56" s="10">
-        <v>260.92</v>
+        <v>258.54000000000002</v>
       </c>
       <c r="G56" s="17"/>
     </row>
-    <row r="57" spans="1:7" x14ac:dyDescent="0.45">
+    <row r="57" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A57" s="11">
-        <v>46315</v>
+        <v>46316</v>
       </c>
       <c r="B57" s="12"/>
       <c r="C57" s="21" t="s">
         <v>33</v>
       </c>
       <c r="D57" s="13">
-        <v>257.08</v>
+        <v>257.52999999999997</v>
       </c>
       <c r="E57" s="13">
-        <v>232.62</v>
+        <v>230.03</v>
       </c>
       <c r="F57" s="13">
-        <v>242.62</v>
+        <v>240.03</v>
       </c>
       <c r="G57" s="17"/>
     </row>
-    <row r="58" spans="1:7" x14ac:dyDescent="0.45">
+    <row r="58" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A58" s="7">
-        <v>46315</v>
+        <v>46316</v>
       </c>
       <c r="B58" s="8"/>
       <c r="C58" s="20" t="s">
         <v>34</v>
       </c>
       <c r="D58" s="10">
-        <v>257.85000000000002</v>
+        <v>258.31</v>
       </c>
       <c r="E58" s="10" t="s">
         <v>18</v>
@@ -1701,111 +1701,111 @@
       </c>
       <c r="G58" s="17"/>
     </row>
-    <row r="59" spans="1:7" x14ac:dyDescent="0.45">
+    <row r="59" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A59" s="11">
-        <v>46315</v>
+        <v>46316</v>
       </c>
       <c r="B59" s="12"/>
       <c r="C59" s="21" t="s">
         <v>35</v>
       </c>
       <c r="D59" s="13">
-        <v>254.18</v>
+        <v>254.57</v>
       </c>
       <c r="E59" s="13">
-        <v>227</v>
+        <v>224.41</v>
       </c>
       <c r="F59" s="13" t="s">
         <v>18</v>
       </c>
       <c r="G59" s="17"/>
     </row>
-    <row r="60" spans="1:7" x14ac:dyDescent="0.45">
+    <row r="60" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A60" s="7">
-        <v>46315</v>
+        <v>46316</v>
       </c>
       <c r="B60" s="8"/>
       <c r="C60" s="20" t="s">
         <v>36</v>
       </c>
       <c r="D60" s="10">
-        <v>250</v>
+        <v>250.4</v>
       </c>
       <c r="E60" s="10">
-        <v>222.94</v>
+        <v>220.35</v>
       </c>
       <c r="F60" s="10">
-        <v>232.94</v>
+        <v>230.35</v>
       </c>
       <c r="G60" s="17"/>
     </row>
-    <row r="61" spans="1:7" x14ac:dyDescent="0.45">
+    <row r="61" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A61" s="11">
-        <v>46315</v>
+        <v>46316</v>
       </c>
       <c r="B61" s="12"/>
       <c r="C61" s="21" t="s">
         <v>37</v>
       </c>
       <c r="D61" s="13">
-        <v>257.58</v>
+        <v>257.97000000000003</v>
       </c>
       <c r="E61" s="13">
-        <v>244.33</v>
+        <v>241.87</v>
       </c>
       <c r="F61" s="13" t="s">
         <v>18</v>
       </c>
       <c r="G61" s="17"/>
     </row>
-    <row r="62" spans="1:7" x14ac:dyDescent="0.45">
+    <row r="62" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A62" s="7">
-        <v>46312</v>
+        <v>46315</v>
       </c>
       <c r="B62" s="8"/>
       <c r="C62" s="20" t="s">
         <v>32</v>
       </c>
       <c r="D62" s="10">
-        <v>269.75</v>
+        <v>269.68</v>
       </c>
       <c r="E62" s="10">
-        <v>253.71</v>
+        <v>250.92</v>
       </c>
       <c r="F62" s="10">
-        <v>263.70999999999998</v>
+        <v>260.92</v>
       </c>
       <c r="G62" s="17"/>
     </row>
-    <row r="63" spans="1:7" x14ac:dyDescent="0.45">
+    <row r="63" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A63" s="11">
-        <v>46312</v>
+        <v>46315</v>
       </c>
       <c r="B63" s="12"/>
       <c r="C63" s="21" t="s">
         <v>33</v>
       </c>
       <c r="D63" s="13">
-        <v>257.14</v>
+        <v>257.08</v>
       </c>
       <c r="E63" s="13">
-        <v>235.63</v>
+        <v>232.62</v>
       </c>
       <c r="F63" s="13">
-        <v>245.63</v>
+        <v>242.62</v>
       </c>
       <c r="G63" s="17"/>
     </row>
-    <row r="64" spans="1:7" x14ac:dyDescent="0.45">
+    <row r="64" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A64" s="7">
-        <v>46312</v>
+        <v>46315</v>
       </c>
       <c r="B64" s="8"/>
       <c r="C64" s="20" t="s">
         <v>34</v>
       </c>
       <c r="D64" s="10">
-        <v>257.89999999999998</v>
+        <v>257.85000000000002</v>
       </c>
       <c r="E64" s="10" t="s">
         <v>18</v>
@@ -1815,55 +1815,55 @@
       </c>
       <c r="G64" s="17"/>
     </row>
-    <row r="65" spans="1:6" x14ac:dyDescent="0.45">
+    <row r="65" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A65" s="11">
-        <v>46312</v>
+        <v>46315</v>
       </c>
       <c r="B65" s="12"/>
       <c r="C65" s="21" t="s">
         <v>35</v>
       </c>
       <c r="D65" s="13">
-        <v>254.29</v>
+        <v>254.18</v>
       </c>
       <c r="E65" s="13">
-        <v>230.01</v>
+        <v>227</v>
       </c>
       <c r="F65" s="13" t="s">
         <v>18</v>
       </c>
     </row>
-    <row r="66" spans="1:6" x14ac:dyDescent="0.45">
+    <row r="66" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A66" s="7">
-        <v>46312</v>
+        <v>46315</v>
       </c>
       <c r="B66" s="8"/>
       <c r="C66" s="20" t="s">
         <v>36</v>
       </c>
       <c r="D66" s="10">
-        <v>250.12</v>
+        <v>250</v>
       </c>
       <c r="E66" s="10">
-        <v>225.95</v>
+        <v>222.94</v>
       </c>
       <c r="F66" s="10">
-        <v>235.95</v>
-      </c>
-    </row>
-    <row r="67" spans="1:6" x14ac:dyDescent="0.45">
+        <v>232.94</v>
+      </c>
+    </row>
+    <row r="67" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A67" s="11">
-        <v>46312</v>
+        <v>46315</v>
       </c>
       <c r="B67" s="12"/>
       <c r="C67" s="21" t="s">
         <v>37</v>
       </c>
       <c r="D67" s="13">
-        <v>257.7</v>
+        <v>257.58</v>
       </c>
       <c r="E67" s="13">
-        <v>247.2</v>
+        <v>244.33</v>
       </c>
       <c r="F67" s="13" t="s">
         <v>18</v>
@@ -1891,14 +1891,12 @@
 </file>
 
 <file path=customXml/item1.xml><?xml version="1.0" encoding="utf-8"?>
-<p:properties xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls">
-  <documentManagement>
-    <lcf76f155ced4ddcb4097134ff3c332f xmlns="87276d81-85f4-4ef2-9e6e-55066304288f">
-      <Terms xmlns="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
-    </lcf76f155ced4ddcb4097134ff3c332f>
-    <TaxCatchAll xmlns="b23b8984-eafa-4e79-985e-54f52f3da58e" xsi:nil="true"/>
-  </documentManagement>
-</p:properties>
+<?mso-contentType ?>
+<FormTemplates xmlns="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms">
+  <Display>DocumentLibraryForm</Display>
+  <Edit>DocumentLibraryForm</Edit>
+  <New>DocumentLibraryForm</New>
+</FormTemplates>
 </file>
 
 <file path=customXml/item2.xml><?xml version="1.0" encoding="utf-8"?>
@@ -2162,21 +2160,20 @@
 </file>
 
 <file path=customXml/item3.xml><?xml version="1.0" encoding="utf-8"?>
-<?mso-contentType ?>
-<FormTemplates xmlns="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms">
-  <Display>DocumentLibraryForm</Display>
-  <Edit>DocumentLibraryForm</Edit>
-  <New>DocumentLibraryForm</New>
-</FormTemplates>
+<p:properties xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls">
+  <documentManagement>
+    <lcf76f155ced4ddcb4097134ff3c332f xmlns="87276d81-85f4-4ef2-9e6e-55066304288f">
+      <Terms xmlns="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
+    </lcf76f155ced4ddcb4097134ff3c332f>
+    <TaxCatchAll xmlns="b23b8984-eafa-4e79-985e-54f52f3da58e" xsi:nil="true"/>
+  </documentManagement>
+</p:properties>
 </file>
 
 <file path=customXml/itemProps1.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{57A83D98-2BAE-4D83-823A-D31C464B620C}">
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{F60519E9-FD90-4339-869C-BC2F85719BB8}">
   <ds:schemaRefs>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/properties"/>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
-    <ds:schemaRef ds:uri="87276d81-85f4-4ef2-9e6e-55066304288f"/>
-    <ds:schemaRef ds:uri="b23b8984-eafa-4e79-985e-54f52f3da58e"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms"/>
   </ds:schemaRefs>
 </ds:datastoreItem>
 </file>
@@ -2202,9 +2199,12 @@
 </file>
 
 <file path=customXml/itemProps3.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{F60519E9-FD90-4339-869C-BC2F85719BB8}">
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{57A83D98-2BAE-4D83-823A-D31C464B620C}">
   <ds:schemaRefs>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/properties"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
+    <ds:schemaRef ds:uri="87276d81-85f4-4ef2-9e6e-55066304288f"/>
+    <ds:schemaRef ds:uri="b23b8984-eafa-4e79-985e-54f52f3da58e"/>
   </ds:schemaRefs>
 </ds:datastoreItem>
 </file>

</xml_diff>

<commit_message>
Wed Oct 21 06:07:07 UTC 2026
</commit_message>
<xml_diff>
--- a/bp.com-content-dam-bp-country-sites-en_au-australia-home-products-services-pricing-tgp-excel.xlsx
+++ b/bp.com-content-dam-bp-country-sites-en_au-australia-home-products-services-pricing-tgp-excel.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://bp365.sharepoint.com/sites/WholesalePricing/Shared Documents/B2C/TGP/Daily TGP/Web TGP/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="14_{C4ACF7A7-558F-4F6C-8016-C29AF31ECD46}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="14_{635FF1F4-C96D-4C69-B192-FFB0CFF6FE1A}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-28920" yWindow="-60" windowWidth="29040" windowHeight="15720" xr2:uid="{1B412EEF-F96D-4DF4-A4E9-C7F0F183C2FB}"/>
+    <workbookView xWindow="-110" yWindow="-110" windowWidth="19420" windowHeight="11500" xr2:uid="{1B412EEF-F96D-4DF4-A4E9-C7F0F183C2FB}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
@@ -715,15 +715,15 @@
     <pageSetUpPr fitToPage="1"/>
   </sheetPr>
   <dimension ref="A1:G67"/>
-  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
   <cols>
-    <col min="1" max="1" width="76.42578125" bestFit="1" customWidth="1"/>
-    <col min="2" max="2" width="6.42578125"/>
-    <col min="3" max="3" width="18.140625" bestFit="1" customWidth="1"/>
-    <col min="4" max="7" width="7.140625" bestFit="1" customWidth="1"/>
+    <col min="1" max="1" width="76.453125" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="6.453125"/>
+    <col min="3" max="3" width="18.1796875" bestFit="1" customWidth="1"/>
+    <col min="4" max="7" width="7.1796875" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:7" ht="23.25" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:7" ht="22.5" x14ac:dyDescent="0.35">
       <c r="A1" s="30" t="s">
         <v>0</v>
       </c>
@@ -734,7 +734,7 @@
       <c r="F1" s="2"/>
       <c r="G1" s="2"/>
     </row>
-    <row r="2" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="2" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A2" s="3"/>
       <c r="B2" s="1"/>
       <c r="C2" s="1"/>
@@ -743,7 +743,7 @@
       <c r="F2" s="2"/>
       <c r="G2" s="2"/>
     </row>
-    <row r="3" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="3" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A3" s="3" t="s">
         <v>1</v>
       </c>
@@ -754,7 +754,7 @@
       <c r="F3" s="2"/>
       <c r="G3" s="2"/>
     </row>
-    <row r="4" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="4" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A4" s="3" t="s">
         <v>2</v>
       </c>
@@ -765,7 +765,7 @@
       <c r="F4" s="2"/>
       <c r="G4" s="2"/>
     </row>
-    <row r="5" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="5" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A5" s="3"/>
       <c r="B5" s="3"/>
       <c r="C5" s="1"/>
@@ -774,7 +774,7 @@
       <c r="F5" s="2"/>
       <c r="G5" s="2"/>
     </row>
-    <row r="6" spans="1:7" ht="20.25" x14ac:dyDescent="0.25">
+    <row r="6" spans="1:7" ht="20" x14ac:dyDescent="0.35">
       <c r="A6" s="29" t="s">
         <v>3</v>
       </c>
@@ -785,7 +785,7 @@
       <c r="F6" s="2"/>
       <c r="G6" s="2"/>
     </row>
-    <row r="7" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="7" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A7" s="4" t="s">
         <v>4</v>
       </c>
@@ -806,133 +806,133 @@
         <v>9</v>
       </c>
     </row>
-    <row r="8" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="8" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A8" s="7">
-        <v>46316</v>
+        <v>46317</v>
       </c>
       <c r="B8" s="8"/>
       <c r="C8" s="9" t="s">
         <v>10</v>
       </c>
       <c r="D8" s="10">
-        <v>258.24</v>
+        <v>258.68</v>
       </c>
       <c r="E8" s="10">
-        <v>223.09</v>
+        <v>220.69</v>
       </c>
       <c r="F8" s="10">
-        <v>233.09</v>
+        <v>230.69</v>
       </c>
       <c r="G8" s="10">
-        <v>220.71</v>
-      </c>
-    </row>
-    <row r="9" spans="1:7" x14ac:dyDescent="0.25">
+        <v>218.31</v>
+      </c>
+    </row>
+    <row r="9" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A9" s="11">
-        <v>46316</v>
+        <v>46317</v>
       </c>
       <c r="B9" s="12"/>
       <c r="C9" s="12" t="s">
         <v>11</v>
       </c>
       <c r="D9" s="13">
-        <v>258.24</v>
+        <v>258.68</v>
       </c>
       <c r="E9" s="13">
-        <v>223.09</v>
+        <v>220.69</v>
       </c>
       <c r="F9" s="13">
-        <v>233.09</v>
+        <v>230.69</v>
       </c>
       <c r="G9" s="13">
-        <v>220.71</v>
-      </c>
-    </row>
-    <row r="10" spans="1:7" x14ac:dyDescent="0.25">
+        <v>218.31</v>
+      </c>
+    </row>
+    <row r="10" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A10" s="7">
-        <v>46316</v>
+        <v>46317</v>
       </c>
       <c r="B10" s="8"/>
       <c r="C10" s="9" t="s">
         <v>12</v>
       </c>
       <c r="D10" s="10">
-        <v>255.43</v>
+        <v>256.87</v>
       </c>
       <c r="E10" s="10">
-        <v>221.84</v>
+        <v>221</v>
       </c>
       <c r="F10" s="10">
-        <v>231.84</v>
+        <v>231</v>
       </c>
       <c r="G10" s="10">
-        <v>220.25</v>
-      </c>
-    </row>
-    <row r="11" spans="1:7" x14ac:dyDescent="0.25">
+        <v>219.41</v>
+      </c>
+    </row>
+    <row r="11" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A11" s="11">
-        <v>46315</v>
+        <v>46316</v>
       </c>
       <c r="B11" s="12"/>
       <c r="C11" s="12" t="s">
         <v>10</v>
       </c>
       <c r="D11" s="13">
-        <v>258.45</v>
+        <v>258.24</v>
       </c>
       <c r="E11" s="13">
-        <v>226.28</v>
+        <v>223.09</v>
       </c>
       <c r="F11" s="13">
-        <v>236.28</v>
+        <v>233.09</v>
       </c>
       <c r="G11" s="13">
-        <v>223.89</v>
-      </c>
-    </row>
-    <row r="12" spans="1:7" x14ac:dyDescent="0.25">
+        <v>220.71</v>
+      </c>
+    </row>
+    <row r="12" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A12" s="7">
-        <v>46315</v>
+        <v>46316</v>
       </c>
       <c r="B12" s="8"/>
       <c r="C12" s="9" t="s">
         <v>11</v>
       </c>
       <c r="D12" s="10">
-        <v>258.45</v>
+        <v>258.24</v>
       </c>
       <c r="E12" s="10">
-        <v>226.28</v>
+        <v>223.09</v>
       </c>
       <c r="F12" s="10">
-        <v>236.28</v>
+        <v>233.09</v>
       </c>
       <c r="G12" s="10">
-        <v>223.89</v>
-      </c>
-    </row>
-    <row r="13" spans="1:7" x14ac:dyDescent="0.25">
+        <v>220.71</v>
+      </c>
+    </row>
+    <row r="13" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A13" s="11">
-        <v>46315</v>
+        <v>46316</v>
       </c>
       <c r="B13" s="12"/>
       <c r="C13" s="12" t="s">
         <v>12</v>
       </c>
       <c r="D13" s="13">
-        <v>254.99</v>
+        <v>255.43</v>
       </c>
       <c r="E13" s="13">
-        <v>224.4</v>
+        <v>221.84</v>
       </c>
       <c r="F13" s="13">
-        <v>234.4</v>
+        <v>231.84</v>
       </c>
       <c r="G13" s="13">
-        <v>222.8</v>
-      </c>
-    </row>
-    <row r="14" spans="1:7" x14ac:dyDescent="0.25">
+        <v>220.25</v>
+      </c>
+    </row>
+    <row r="14" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A14" s="14"/>
       <c r="B14" s="14"/>
       <c r="C14" s="15"/>
@@ -941,7 +941,7 @@
       <c r="F14" s="16"/>
       <c r="G14" s="16"/>
     </row>
-    <row r="15" spans="1:7" ht="20.25" x14ac:dyDescent="0.25">
+    <row r="15" spans="1:7" ht="20" x14ac:dyDescent="0.35">
       <c r="A15" s="29" t="s">
         <v>13</v>
       </c>
@@ -952,7 +952,7 @@
       <c r="F15" s="17"/>
       <c r="G15" s="17"/>
     </row>
-    <row r="16" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="16" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A16" s="4" t="s">
         <v>4</v>
       </c>
@@ -971,45 +971,45 @@
       </c>
       <c r="G16" s="17"/>
     </row>
-    <row r="17" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="17" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A17" s="7">
-        <v>46316</v>
+        <v>46317</v>
       </c>
       <c r="B17" s="8"/>
       <c r="C17" s="20" t="s">
         <v>14</v>
       </c>
       <c r="D17" s="10">
-        <v>258.89</v>
+        <v>260.29000000000002</v>
       </c>
       <c r="E17" s="10">
-        <v>224.78</v>
+        <v>223.91</v>
       </c>
       <c r="F17" s="10">
-        <v>234.78</v>
+        <v>233.91</v>
       </c>
       <c r="G17" s="17"/>
     </row>
-    <row r="18" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="18" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A18" s="11">
-        <v>46315</v>
+        <v>46316</v>
       </c>
       <c r="B18" s="12"/>
       <c r="C18" s="12" t="s">
         <v>14</v>
       </c>
       <c r="D18" s="13">
-        <v>258.48</v>
+        <v>258.89</v>
       </c>
       <c r="E18" s="13">
-        <v>227.38</v>
+        <v>224.78</v>
       </c>
       <c r="F18" s="13">
-        <v>237.38</v>
+        <v>234.78</v>
       </c>
       <c r="G18" s="17"/>
     </row>
-    <row r="19" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="19" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A19" s="14"/>
       <c r="B19" s="14"/>
       <c r="C19" s="15"/>
@@ -1018,7 +1018,7 @@
       <c r="F19" s="16"/>
       <c r="G19" s="17"/>
     </row>
-    <row r="20" spans="1:7" ht="20.25" x14ac:dyDescent="0.25">
+    <row r="20" spans="1:7" ht="20" x14ac:dyDescent="0.35">
       <c r="A20" s="29" t="s">
         <v>15</v>
       </c>
@@ -1029,7 +1029,7 @@
       <c r="F20" s="17"/>
       <c r="G20" s="17"/>
     </row>
-    <row r="21" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="21" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A21" s="4" t="s">
         <v>4</v>
       </c>
@@ -1050,217 +1050,217 @@
         <v>9</v>
       </c>
     </row>
-    <row r="22" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="22" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A22" s="7">
-        <v>46316</v>
+        <v>46317</v>
       </c>
       <c r="B22" s="8"/>
       <c r="C22" s="20" t="s">
         <v>16</v>
       </c>
       <c r="D22" s="10">
-        <v>259.37</v>
+        <v>259.8</v>
       </c>
       <c r="E22" s="10">
-        <v>223.23</v>
+        <v>220.83</v>
       </c>
       <c r="F22" s="10">
-        <v>232.83</v>
+        <v>230.43</v>
       </c>
       <c r="G22" s="10">
-        <v>219.6</v>
-      </c>
-    </row>
-    <row r="23" spans="1:7" x14ac:dyDescent="0.25">
+        <v>217.2</v>
+      </c>
+    </row>
+    <row r="23" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A23" s="11">
-        <v>46316</v>
+        <v>46317</v>
       </c>
       <c r="B23" s="12"/>
       <c r="C23" s="21" t="s">
         <v>17</v>
       </c>
       <c r="D23" s="13">
-        <v>260.39</v>
+        <v>261.82</v>
       </c>
       <c r="E23" s="13">
-        <v>230.11</v>
+        <v>229.28</v>
       </c>
       <c r="F23" s="13">
-        <v>240.11</v>
+        <v>239.28</v>
       </c>
       <c r="G23" s="13" t="s">
         <v>18</v>
       </c>
     </row>
-    <row r="24" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="24" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A24" s="7">
-        <v>46316</v>
+        <v>46317</v>
       </c>
       <c r="B24" s="8"/>
       <c r="C24" s="20" t="s">
         <v>19</v>
       </c>
       <c r="D24" s="10">
-        <v>260.74</v>
+        <v>262.17</v>
       </c>
       <c r="E24" s="10">
-        <v>229.38</v>
+        <v>228.55</v>
       </c>
       <c r="F24" s="10">
-        <v>239.38</v>
+        <v>238.55</v>
       </c>
       <c r="G24" s="10" t="s">
         <v>18</v>
       </c>
     </row>
-    <row r="25" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="25" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A25" s="11">
-        <v>46316</v>
+        <v>46317</v>
       </c>
       <c r="B25" s="12"/>
       <c r="C25" s="21" t="s">
         <v>20</v>
       </c>
       <c r="D25" s="13">
-        <v>257.39999999999998</v>
+        <v>258.83</v>
       </c>
       <c r="E25" s="13">
-        <v>229.59</v>
+        <v>228.76</v>
       </c>
       <c r="F25" s="13">
-        <v>239.59</v>
+        <v>238.76</v>
       </c>
       <c r="G25" s="13">
-        <v>225.43</v>
-      </c>
-    </row>
-    <row r="26" spans="1:7" x14ac:dyDescent="0.25">
+        <v>224.6</v>
+      </c>
+    </row>
+    <row r="26" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A26" s="7">
-        <v>46316</v>
+        <v>46317</v>
       </c>
       <c r="B26" s="8"/>
       <c r="C26" s="20" t="s">
         <v>21</v>
       </c>
       <c r="D26" s="10">
-        <v>258.94</v>
+        <v>260.37</v>
       </c>
       <c r="E26" s="10">
-        <v>231.01</v>
+        <v>230.18</v>
       </c>
       <c r="F26" s="10">
-        <v>241.01</v>
+        <v>240.18</v>
       </c>
       <c r="G26" s="10" t="s">
         <v>18</v>
       </c>
     </row>
-    <row r="27" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="27" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A27" s="11">
-        <v>46315</v>
+        <v>46316</v>
       </c>
       <c r="B27" s="12"/>
       <c r="C27" s="12" t="s">
         <v>16</v>
       </c>
       <c r="D27" s="13">
-        <v>259.57</v>
+        <v>259.37</v>
       </c>
       <c r="E27" s="13">
-        <v>226.42</v>
+        <v>223.23</v>
       </c>
       <c r="F27" s="13">
-        <v>236.02</v>
+        <v>232.83</v>
       </c>
       <c r="G27" s="13">
-        <v>222.79</v>
-      </c>
-    </row>
-    <row r="28" spans="1:7" x14ac:dyDescent="0.25">
+        <v>219.6</v>
+      </c>
+    </row>
+    <row r="28" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A28" s="7">
-        <v>46315</v>
+        <v>46316</v>
       </c>
       <c r="B28" s="8"/>
       <c r="C28" s="20" t="s">
         <v>17</v>
       </c>
       <c r="D28" s="10">
-        <v>259.94</v>
+        <v>260.39</v>
       </c>
       <c r="E28" s="22">
-        <v>232.65</v>
+        <v>230.11</v>
       </c>
       <c r="F28" s="22">
-        <v>242.65</v>
+        <v>240.11</v>
       </c>
       <c r="G28" s="22" t="s">
         <v>18</v>
       </c>
     </row>
-    <row r="29" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="29" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A29" s="11">
-        <v>46315</v>
+        <v>46316</v>
       </c>
       <c r="B29" s="12"/>
       <c r="C29" s="12" t="s">
         <v>19</v>
       </c>
       <c r="D29" s="13">
-        <v>260.29000000000002</v>
+        <v>260.74</v>
       </c>
       <c r="E29" s="13">
-        <v>231.92</v>
+        <v>229.38</v>
       </c>
       <c r="F29" s="13">
-        <v>241.92</v>
+        <v>239.38</v>
       </c>
       <c r="G29" s="13" t="s">
         <v>18</v>
       </c>
     </row>
-    <row r="30" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="30" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A30" s="7">
-        <v>46315</v>
+        <v>46316</v>
       </c>
       <c r="B30" s="8"/>
       <c r="C30" s="20" t="s">
         <v>20</v>
       </c>
       <c r="D30" s="10">
-        <v>256.95</v>
+        <v>257.39999999999998</v>
       </c>
       <c r="E30" s="22">
-        <v>232.13</v>
+        <v>229.59</v>
       </c>
       <c r="F30" s="22">
-        <v>242.13</v>
+        <v>239.59</v>
       </c>
       <c r="G30" s="22">
-        <v>227.97</v>
-      </c>
-    </row>
-    <row r="31" spans="1:7" x14ac:dyDescent="0.25">
+        <v>225.43</v>
+      </c>
+    </row>
+    <row r="31" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A31" s="11">
-        <v>46315</v>
+        <v>46316</v>
       </c>
       <c r="B31" s="12"/>
       <c r="C31" s="12" t="s">
         <v>21</v>
       </c>
       <c r="D31" s="13">
-        <v>258.51</v>
+        <v>258.94</v>
       </c>
       <c r="E31" s="13">
-        <v>233.57</v>
+        <v>231.01</v>
       </c>
       <c r="F31" s="13">
-        <v>243.57</v>
+        <v>241.01</v>
       </c>
       <c r="G31" s="13" t="s">
         <v>18</v>
       </c>
     </row>
-    <row r="32" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="32" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A32" s="14"/>
       <c r="B32" s="14"/>
       <c r="C32" s="15"/>
@@ -1269,7 +1269,7 @@
       <c r="F32" s="17"/>
       <c r="G32" s="17"/>
     </row>
-    <row r="33" spans="1:7" ht="20.25" x14ac:dyDescent="0.25">
+    <row r="33" spans="1:7" ht="20" x14ac:dyDescent="0.35">
       <c r="A33" s="29" t="s">
         <v>22</v>
       </c>
@@ -1280,7 +1280,7 @@
       <c r="F33" s="17"/>
       <c r="G33" s="17"/>
     </row>
-    <row r="34" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="34" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A34" s="23" t="s">
         <v>4</v>
       </c>
@@ -1299,54 +1299,54 @@
       </c>
       <c r="G34" s="17"/>
     </row>
-    <row r="35" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="35" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A35" s="7">
-        <v>46316</v>
+        <v>46317</v>
       </c>
       <c r="B35" s="8"/>
       <c r="C35" s="20" t="s">
         <v>23</v>
       </c>
       <c r="D35" s="10">
-        <v>253.98</v>
+        <v>255.42</v>
       </c>
       <c r="E35" s="10">
-        <v>220.8</v>
+        <v>219.96</v>
       </c>
       <c r="F35" s="10">
-        <v>229.8</v>
+        <v>228.96</v>
       </c>
       <c r="G35" s="17"/>
     </row>
-    <row r="36" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="36" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A36" s="11">
-        <v>46315</v>
+        <v>46316</v>
       </c>
       <c r="B36" s="12"/>
       <c r="C36" s="12" t="s">
         <v>23</v>
       </c>
       <c r="D36" s="13">
-        <v>253.54</v>
+        <v>253.98</v>
       </c>
       <c r="E36" s="13">
-        <v>223.35</v>
+        <v>220.8</v>
       </c>
       <c r="F36" s="13">
-        <v>232.35</v>
+        <v>229.8</v>
       </c>
       <c r="G36" s="17"/>
     </row>
-    <row r="37" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="37" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A37" s="7">
-        <v>46316</v>
+        <v>46317</v>
       </c>
       <c r="B37" s="8"/>
       <c r="C37" s="20" t="s">
         <v>24</v>
       </c>
       <c r="D37" s="10">
-        <v>269.60000000000002</v>
+        <v>271.04000000000002</v>
       </c>
       <c r="E37" s="10" t="s">
         <v>18</v>
@@ -1356,16 +1356,16 @@
       </c>
       <c r="G37" s="17"/>
     </row>
-    <row r="38" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="38" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A38" s="11">
-        <v>46315</v>
+        <v>46316</v>
       </c>
       <c r="B38" s="12"/>
       <c r="C38" s="12" t="s">
         <v>24</v>
       </c>
       <c r="D38" s="13">
-        <v>269.16000000000003</v>
+        <v>269.60000000000002</v>
       </c>
       <c r="E38" s="13" t="s">
         <v>18</v>
@@ -1375,7 +1375,7 @@
       </c>
       <c r="G38" s="17"/>
     </row>
-    <row r="39" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="39" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A39" s="24"/>
       <c r="B39" s="24"/>
       <c r="C39" s="15"/>
@@ -1384,7 +1384,7 @@
       <c r="F39" s="17"/>
       <c r="G39" s="17"/>
     </row>
-    <row r="40" spans="1:7" ht="20.25" x14ac:dyDescent="0.25">
+    <row r="40" spans="1:7" ht="20" x14ac:dyDescent="0.35">
       <c r="A40" s="29" t="s">
         <v>25</v>
       </c>
@@ -1395,7 +1395,7 @@
       <c r="F40" s="17"/>
       <c r="G40" s="17"/>
     </row>
-    <row r="41" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="41" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A41" s="23" t="s">
         <v>4</v>
       </c>
@@ -1414,83 +1414,83 @@
       </c>
       <c r="G41" s="17"/>
     </row>
-    <row r="42" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="42" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A42" s="7">
-        <v>46316</v>
+        <v>46317</v>
       </c>
       <c r="B42" s="8"/>
       <c r="C42" s="20" t="s">
         <v>26</v>
       </c>
       <c r="D42" s="10">
-        <v>264</v>
+        <v>265.45999999999998</v>
       </c>
       <c r="E42" s="10">
-        <v>231.3</v>
+        <v>230.66</v>
       </c>
       <c r="F42" s="10">
-        <v>241.3</v>
+        <v>240.66</v>
       </c>
       <c r="G42" s="17"/>
     </row>
-    <row r="43" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="43" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A43" s="11">
-        <v>46316</v>
+        <v>46317</v>
       </c>
       <c r="B43" s="12"/>
       <c r="C43" s="21" t="s">
         <v>27</v>
       </c>
       <c r="D43" s="13">
-        <v>263.61</v>
+        <v>265.07</v>
       </c>
       <c r="E43" s="13">
-        <v>231.71</v>
+        <v>231.07</v>
       </c>
       <c r="F43" s="13">
-        <v>241.71</v>
+        <v>241.07</v>
       </c>
       <c r="G43" s="17"/>
     </row>
-    <row r="44" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="44" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A44" s="7">
-        <v>46315</v>
+        <v>46316</v>
       </c>
       <c r="B44" s="8"/>
       <c r="C44" s="20" t="s">
         <v>26</v>
       </c>
       <c r="D44" s="10">
-        <v>263.52</v>
+        <v>264</v>
       </c>
       <c r="E44" s="10">
-        <v>233.61</v>
+        <v>231.3</v>
       </c>
       <c r="F44" s="10">
-        <v>243.61</v>
+        <v>241.3</v>
       </c>
       <c r="G44" s="17"/>
     </row>
-    <row r="45" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="45" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A45" s="11">
-        <v>46315</v>
+        <v>46316</v>
       </c>
       <c r="B45" s="12"/>
       <c r="C45" s="21" t="s">
         <v>27</v>
       </c>
       <c r="D45" s="13">
-        <v>263.13</v>
+        <v>263.61</v>
       </c>
       <c r="E45" s="13">
-        <v>234.02</v>
+        <v>231.71</v>
       </c>
       <c r="F45" s="13">
-        <v>244.02</v>
+        <v>241.71</v>
       </c>
       <c r="G45" s="17"/>
     </row>
-    <row r="46" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="46" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A46" s="14"/>
       <c r="B46" s="24"/>
       <c r="C46" s="15"/>
@@ -1499,7 +1499,7 @@
       <c r="F46" s="16"/>
       <c r="G46" s="17"/>
     </row>
-    <row r="47" spans="1:7" ht="20.25" x14ac:dyDescent="0.25">
+    <row r="47" spans="1:7" ht="20" x14ac:dyDescent="0.35">
       <c r="A47" s="25" t="s">
         <v>28</v>
       </c>
@@ -1510,7 +1510,7 @@
       <c r="F47" s="17"/>
       <c r="G47" s="17"/>
     </row>
-    <row r="48" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="48" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A48" s="23" t="s">
         <v>4</v>
       </c>
@@ -1529,83 +1529,83 @@
       </c>
       <c r="G48" s="17"/>
     </row>
-    <row r="49" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="49" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A49" s="7">
-        <v>46316</v>
+        <v>46317</v>
       </c>
       <c r="B49" s="8"/>
       <c r="C49" s="20" t="s">
         <v>29</v>
       </c>
       <c r="D49" s="10">
-        <v>255.72</v>
+        <v>256.92</v>
       </c>
       <c r="E49" s="10">
-        <v>225.15</v>
+        <v>223.9</v>
       </c>
       <c r="F49" s="10">
-        <v>235.15</v>
+        <v>233.9</v>
       </c>
       <c r="G49" s="28"/>
     </row>
-    <row r="50" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="50" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A50" s="11">
-        <v>46316</v>
+        <v>46317</v>
       </c>
       <c r="B50" s="12"/>
       <c r="C50" s="21" t="s">
         <v>30</v>
       </c>
       <c r="D50" s="13">
-        <v>253.24</v>
+        <v>254.43</v>
       </c>
       <c r="E50" s="13">
-        <v>224.75</v>
+        <v>223.49</v>
       </c>
       <c r="F50" s="13">
-        <v>234.75</v>
+        <v>233.49</v>
       </c>
       <c r="G50" s="28"/>
     </row>
-    <row r="51" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="51" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A51" s="7">
-        <v>46315</v>
+        <v>46316</v>
       </c>
       <c r="B51" s="8"/>
       <c r="C51" s="20" t="s">
         <v>29</v>
       </c>
       <c r="D51" s="10">
-        <v>257.32</v>
+        <v>255.72</v>
       </c>
       <c r="E51" s="10">
-        <v>228.32</v>
+        <v>225.15</v>
       </c>
       <c r="F51" s="10">
-        <v>238.32</v>
+        <v>235.15</v>
       </c>
       <c r="G51" s="17"/>
     </row>
-    <row r="52" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="52" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A52" s="11">
-        <v>46315</v>
+        <v>46316</v>
       </c>
       <c r="B52" s="12"/>
       <c r="C52" s="21" t="s">
         <v>30</v>
       </c>
       <c r="D52" s="13">
-        <v>254.85</v>
+        <v>253.24</v>
       </c>
       <c r="E52" s="13">
-        <v>227.94</v>
+        <v>224.75</v>
       </c>
       <c r="F52" s="13">
-        <v>237.94</v>
+        <v>234.75</v>
       </c>
       <c r="G52" s="17"/>
     </row>
-    <row r="53" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="53" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A53" s="14"/>
       <c r="B53" s="14"/>
       <c r="C53" s="15"/>
@@ -1614,7 +1614,7 @@
       <c r="F53" s="16"/>
       <c r="G53" s="17"/>
     </row>
-    <row r="54" spans="1:7" ht="20.25" x14ac:dyDescent="0.25">
+    <row r="54" spans="1:7" ht="20" x14ac:dyDescent="0.35">
       <c r="A54" s="27" t="s">
         <v>31</v>
       </c>
@@ -1625,7 +1625,7 @@
       <c r="F54" s="17"/>
       <c r="G54" s="17"/>
     </row>
-    <row r="55" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="55" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A55" s="23" t="s">
         <v>4</v>
       </c>
@@ -1644,54 +1644,54 @@
       </c>
       <c r="G55" s="17"/>
     </row>
-    <row r="56" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="56" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A56" s="7">
-        <v>46316</v>
+        <v>46317</v>
       </c>
       <c r="B56" s="8"/>
       <c r="C56" s="20" t="s">
         <v>32</v>
       </c>
       <c r="D56" s="10">
-        <v>270.11</v>
+        <v>271.54000000000002</v>
       </c>
       <c r="E56" s="10">
-        <v>248.54</v>
+        <v>247.85</v>
       </c>
       <c r="F56" s="10">
-        <v>258.54000000000002</v>
+        <v>257.85000000000002</v>
       </c>
       <c r="G56" s="17"/>
     </row>
-    <row r="57" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="57" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A57" s="11">
-        <v>46316</v>
+        <v>46317</v>
       </c>
       <c r="B57" s="12"/>
       <c r="C57" s="21" t="s">
         <v>33</v>
       </c>
       <c r="D57" s="13">
-        <v>257.52999999999997</v>
+        <v>258.42</v>
       </c>
       <c r="E57" s="13">
-        <v>230.03</v>
+        <v>229.16</v>
       </c>
       <c r="F57" s="13">
-        <v>240.03</v>
+        <v>239.16</v>
       </c>
       <c r="G57" s="17"/>
     </row>
-    <row r="58" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="58" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A58" s="7">
-        <v>46316</v>
+        <v>46317</v>
       </c>
       <c r="B58" s="8"/>
       <c r="C58" s="20" t="s">
         <v>34</v>
       </c>
       <c r="D58" s="10">
-        <v>258.31</v>
+        <v>259.2</v>
       </c>
       <c r="E58" s="10" t="s">
         <v>18</v>
@@ -1701,111 +1701,111 @@
       </c>
       <c r="G58" s="17"/>
     </row>
-    <row r="59" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="59" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A59" s="11">
-        <v>46316</v>
+        <v>46317</v>
       </c>
       <c r="B59" s="12"/>
       <c r="C59" s="21" t="s">
         <v>35</v>
       </c>
       <c r="D59" s="13">
-        <v>254.57</v>
+        <v>255.41</v>
       </c>
       <c r="E59" s="13">
-        <v>224.41</v>
+        <v>223.54</v>
       </c>
       <c r="F59" s="13" t="s">
         <v>18</v>
       </c>
       <c r="G59" s="17"/>
     </row>
-    <row r="60" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="60" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A60" s="7">
-        <v>46316</v>
+        <v>46317</v>
       </c>
       <c r="B60" s="8"/>
       <c r="C60" s="20" t="s">
         <v>36</v>
       </c>
       <c r="D60" s="10">
-        <v>250.4</v>
+        <v>251.24</v>
       </c>
       <c r="E60" s="10">
-        <v>220.35</v>
+        <v>219.48</v>
       </c>
       <c r="F60" s="10">
-        <v>230.35</v>
+        <v>229.48</v>
       </c>
       <c r="G60" s="17"/>
     </row>
-    <row r="61" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="61" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A61" s="11">
-        <v>46316</v>
+        <v>46317</v>
       </c>
       <c r="B61" s="12"/>
       <c r="C61" s="21" t="s">
         <v>37</v>
       </c>
       <c r="D61" s="13">
-        <v>257.97000000000003</v>
+        <v>259.37</v>
       </c>
       <c r="E61" s="13">
-        <v>241.87</v>
+        <v>241.11</v>
       </c>
       <c r="F61" s="13" t="s">
         <v>18</v>
       </c>
       <c r="G61" s="17"/>
     </row>
-    <row r="62" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="62" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A62" s="7">
-        <v>46315</v>
+        <v>46316</v>
       </c>
       <c r="B62" s="8"/>
       <c r="C62" s="20" t="s">
         <v>32</v>
       </c>
       <c r="D62" s="10">
-        <v>269.68</v>
+        <v>270.11</v>
       </c>
       <c r="E62" s="10">
-        <v>250.92</v>
+        <v>248.54</v>
       </c>
       <c r="F62" s="10">
-        <v>260.92</v>
+        <v>258.54000000000002</v>
       </c>
       <c r="G62" s="17"/>
     </row>
-    <row r="63" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="63" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A63" s="11">
-        <v>46315</v>
+        <v>46316</v>
       </c>
       <c r="B63" s="12"/>
       <c r="C63" s="21" t="s">
         <v>33</v>
       </c>
       <c r="D63" s="13">
-        <v>257.08</v>
+        <v>257.52999999999997</v>
       </c>
       <c r="E63" s="13">
-        <v>232.62</v>
+        <v>230.03</v>
       </c>
       <c r="F63" s="13">
-        <v>242.62</v>
+        <v>240.03</v>
       </c>
       <c r="G63" s="17"/>
     </row>
-    <row r="64" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="64" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A64" s="7">
-        <v>46315</v>
+        <v>46316</v>
       </c>
       <c r="B64" s="8"/>
       <c r="C64" s="20" t="s">
         <v>34</v>
       </c>
       <c r="D64" s="10">
-        <v>257.85000000000002</v>
+        <v>258.31</v>
       </c>
       <c r="E64" s="10" t="s">
         <v>18</v>
@@ -1815,55 +1815,55 @@
       </c>
       <c r="G64" s="17"/>
     </row>
-    <row r="65" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="65" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A65" s="11">
-        <v>46315</v>
+        <v>46316</v>
       </c>
       <c r="B65" s="12"/>
       <c r="C65" s="21" t="s">
         <v>35</v>
       </c>
       <c r="D65" s="13">
-        <v>254.18</v>
+        <v>254.57</v>
       </c>
       <c r="E65" s="13">
-        <v>227</v>
+        <v>224.41</v>
       </c>
       <c r="F65" s="13" t="s">
         <v>18</v>
       </c>
     </row>
-    <row r="66" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="66" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A66" s="7">
-        <v>46315</v>
+        <v>46316</v>
       </c>
       <c r="B66" s="8"/>
       <c r="C66" s="20" t="s">
         <v>36</v>
       </c>
       <c r="D66" s="10">
-        <v>250</v>
+        <v>250.4</v>
       </c>
       <c r="E66" s="10">
-        <v>222.94</v>
+        <v>220.35</v>
       </c>
       <c r="F66" s="10">
-        <v>232.94</v>
-      </c>
-    </row>
-    <row r="67" spans="1:6" x14ac:dyDescent="0.25">
+        <v>230.35</v>
+      </c>
+    </row>
+    <row r="67" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A67" s="11">
-        <v>46315</v>
+        <v>46316</v>
       </c>
       <c r="B67" s="12"/>
       <c r="C67" s="21" t="s">
         <v>37</v>
       </c>
       <c r="D67" s="13">
-        <v>257.58</v>
+        <v>257.97000000000003</v>
       </c>
       <c r="E67" s="13">
-        <v>244.33</v>
+        <v>241.87</v>
       </c>
       <c r="F67" s="13" t="s">
         <v>18</v>
@@ -1891,6 +1891,17 @@
 </file>
 
 <file path=customXml/item1.xml><?xml version="1.0" encoding="utf-8"?>
+<p:properties xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls">
+  <documentManagement>
+    <lcf76f155ced4ddcb4097134ff3c332f xmlns="87276d81-85f4-4ef2-9e6e-55066304288f">
+      <Terms xmlns="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
+    </lcf76f155ced4ddcb4097134ff3c332f>
+    <TaxCatchAll xmlns="b23b8984-eafa-4e79-985e-54f52f3da58e" xsi:nil="true"/>
+  </documentManagement>
+</p:properties>
+</file>
+
+<file path=customXml/item2.xml><?xml version="1.0" encoding="utf-8"?>
 <?mso-contentType ?>
 <FormTemplates xmlns="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms">
   <Display>DocumentLibraryForm</Display>
@@ -1899,7 +1910,7 @@
 </FormTemplates>
 </file>
 
-<file path=customXml/item2.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=customXml/item3.xml><?xml version="1.0" encoding="utf-8"?>
 <ct:contentTypeSchema xmlns:ct="http://schemas.microsoft.com/office/2006/metadata/contentType" xmlns:ma="http://schemas.microsoft.com/office/2006/metadata/properties/metaAttributes" ct:_="" ma:_="" ma:contentTypeName="Document" ma:contentTypeID="0x010100D3632DF5622958439304627C030B0427" ma:contentTypeVersion="18" ma:contentTypeDescription="Create a new document." ma:contentTypeScope="" ma:versionID="8c2ecbce386d6bac497f8eb2d8f0fb7a">
   <xsd:schema xmlns:xsd="http://www.w3.org/2001/XMLSchema" xmlns:xs="http://www.w3.org/2001/XMLSchema" xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:ns2="87276d81-85f4-4ef2-9e6e-55066304288f" xmlns:ns3="39e1dda6-d1d8-4c88-a3b9-f1abc1284bad" xmlns:ns4="b23b8984-eafa-4e79-985e-54f52f3da58e" targetNamespace="http://schemas.microsoft.com/office/2006/metadata/properties" ma:root="true" ma:fieldsID="4cfd0c2f651c1ce156ad4fcb44ea61dd" ns2:_="" ns3:_="" ns4:_="">
     <xsd:import namespace="87276d81-85f4-4ef2-9e6e-55066304288f"/>
@@ -2159,18 +2170,18 @@
 </ct:contentTypeSchema>
 </file>
 
-<file path=customXml/item3.xml><?xml version="1.0" encoding="utf-8"?>
-<p:properties xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls">
-  <documentManagement>
-    <lcf76f155ced4ddcb4097134ff3c332f xmlns="87276d81-85f4-4ef2-9e6e-55066304288f">
-      <Terms xmlns="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
-    </lcf76f155ced4ddcb4097134ff3c332f>
-    <TaxCatchAll xmlns="b23b8984-eafa-4e79-985e-54f52f3da58e" xsi:nil="true"/>
-  </documentManagement>
-</p:properties>
+<file path=customXml/itemProps1.xml><?xml version="1.0" encoding="utf-8"?>
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{57A83D98-2BAE-4D83-823A-D31C464B620C}">
+  <ds:schemaRefs>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/properties"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
+    <ds:schemaRef ds:uri="87276d81-85f4-4ef2-9e6e-55066304288f"/>
+    <ds:schemaRef ds:uri="b23b8984-eafa-4e79-985e-54f52f3da58e"/>
+  </ds:schemaRefs>
+</ds:datastoreItem>
 </file>
 
-<file path=customXml/itemProps1.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=customXml/itemProps2.xml><?xml version="1.0" encoding="utf-8"?>
 <ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{F60519E9-FD90-4339-869C-BC2F85719BB8}">
   <ds:schemaRefs>
     <ds:schemaRef ds:uri="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms"/>
@@ -2178,7 +2189,7 @@
 </ds:datastoreItem>
 </file>
 
-<file path=customXml/itemProps2.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=customXml/itemProps3.xml><?xml version="1.0" encoding="utf-8"?>
 <ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{B44E1863-2778-41F9-ACBA-48420F931671}">
   <ds:schemaRefs>
     <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/contentType"/>
@@ -2198,17 +2209,6 @@
 </ds:datastoreItem>
 </file>
 
-<file path=customXml/itemProps3.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{57A83D98-2BAE-4D83-823A-D31C464B620C}">
-  <ds:schemaRefs>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/properties"/>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
-    <ds:schemaRef ds:uri="87276d81-85f4-4ef2-9e6e-55066304288f"/>
-    <ds:schemaRef ds:uri="b23b8984-eafa-4e79-985e-54f52f3da58e"/>
-  </ds:schemaRefs>
-</ds:datastoreItem>
-</file>
-
 <file path=docMetadata/LabelInfo.xml><?xml version="1.0" encoding="utf-8"?>
 <clbl:labelList xmlns:clbl="http://schemas.microsoft.com/office/2020/mipLabelMetadata">
   <clbl:label id="{569bf4a9-87bd-4dbf-a36c-1db5158e5def}" enabled="1" method="Privileged" siteId="{ea80952e-a476-42d4-aaf4-5457852b0f7e}" removed="0"/>

</xml_diff>

<commit_message>
Thu Oct 22 06:10:25 UTC 2026
</commit_message>
<xml_diff>
--- a/bp.com-content-dam-bp-country-sites-en_au-australia-home-products-services-pricing-tgp-excel.xlsx
+++ b/bp.com-content-dam-bp-country-sites-en_au-australia-home-products-services-pricing-tgp-excel.xlsx
@@ -8,14 +8,14 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://bp365.sharepoint.com/sites/WholesalePricing/Shared Documents/B2C/TGP/Daily TGP/Web TGP/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="14_{635FF1F4-C96D-4C69-B192-FFB0CFF6FE1A}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="14_{A56F2BA7-A5D4-4540-9A5C-5C5A324CDACF}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-110" yWindow="-110" windowWidth="19420" windowHeight="11500" xr2:uid="{1B412EEF-F96D-4DF4-A4E9-C7F0F183C2FB}"/>
+    <workbookView xWindow="20490" yWindow="-16320" windowWidth="29040" windowHeight="15720" xr2:uid="{1B412EEF-F96D-4DF4-A4E9-C7F0F183C2FB}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
   </sheets>
-  <calcPr calcId="191028" concurrentManualCount="12"/>
+  <calcPr calcId="191028" concurrentManualCount="20"/>
   <extLst>
     <ext xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" uri="{140A7094-0E35-4892-8432-C4D2E57EDEB5}">
       <x15:workbookPr chartTrackingRefBase="1"/>
@@ -715,15 +715,15 @@
     <pageSetUpPr fitToPage="1"/>
   </sheetPr>
   <dimension ref="A1:G67"/>
-  <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
+  <sheetFormatPr defaultRowHeight="14.25" x14ac:dyDescent="0.45"/>
   <cols>
-    <col min="1" max="1" width="76.453125" bestFit="1" customWidth="1"/>
-    <col min="2" max="2" width="6.453125"/>
-    <col min="3" max="3" width="18.1796875" bestFit="1" customWidth="1"/>
-    <col min="4" max="7" width="7.1796875" bestFit="1" customWidth="1"/>
+    <col min="1" max="1" width="76.46484375" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="6.46484375"/>
+    <col min="3" max="3" width="18.19921875" bestFit="1" customWidth="1"/>
+    <col min="4" max="7" width="7.19921875" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:7" ht="22.5" x14ac:dyDescent="0.35">
+    <row r="1" spans="1:7" ht="22.15" x14ac:dyDescent="0.45">
       <c r="A1" s="30" t="s">
         <v>0</v>
       </c>
@@ -734,7 +734,7 @@
       <c r="F1" s="2"/>
       <c r="G1" s="2"/>
     </row>
-    <row r="2" spans="1:7" x14ac:dyDescent="0.35">
+    <row r="2" spans="1:7" x14ac:dyDescent="0.45">
       <c r="A2" s="3"/>
       <c r="B2" s="1"/>
       <c r="C2" s="1"/>
@@ -743,7 +743,7 @@
       <c r="F2" s="2"/>
       <c r="G2" s="2"/>
     </row>
-    <row r="3" spans="1:7" x14ac:dyDescent="0.35">
+    <row r="3" spans="1:7" x14ac:dyDescent="0.45">
       <c r="A3" s="3" t="s">
         <v>1</v>
       </c>
@@ -754,7 +754,7 @@
       <c r="F3" s="2"/>
       <c r="G3" s="2"/>
     </row>
-    <row r="4" spans="1:7" x14ac:dyDescent="0.35">
+    <row r="4" spans="1:7" x14ac:dyDescent="0.45">
       <c r="A4" s="3" t="s">
         <v>2</v>
       </c>
@@ -765,7 +765,7 @@
       <c r="F4" s="2"/>
       <c r="G4" s="2"/>
     </row>
-    <row r="5" spans="1:7" x14ac:dyDescent="0.35">
+    <row r="5" spans="1:7" x14ac:dyDescent="0.45">
       <c r="A5" s="3"/>
       <c r="B5" s="3"/>
       <c r="C5" s="1"/>
@@ -774,7 +774,7 @@
       <c r="F5" s="2"/>
       <c r="G5" s="2"/>
     </row>
-    <row r="6" spans="1:7" ht="20" x14ac:dyDescent="0.35">
+    <row r="6" spans="1:7" ht="20.25" x14ac:dyDescent="0.45">
       <c r="A6" s="29" t="s">
         <v>3</v>
       </c>
@@ -785,7 +785,7 @@
       <c r="F6" s="2"/>
       <c r="G6" s="2"/>
     </row>
-    <row r="7" spans="1:7" x14ac:dyDescent="0.35">
+    <row r="7" spans="1:7" x14ac:dyDescent="0.45">
       <c r="A7" s="4" t="s">
         <v>4</v>
       </c>
@@ -806,133 +806,133 @@
         <v>9</v>
       </c>
     </row>
-    <row r="8" spans="1:7" x14ac:dyDescent="0.35">
+    <row r="8" spans="1:7" x14ac:dyDescent="0.45">
       <c r="A8" s="7">
-        <v>46317</v>
+        <v>46318</v>
       </c>
       <c r="B8" s="8"/>
       <c r="C8" s="9" t="s">
         <v>10</v>
       </c>
       <c r="D8" s="10">
-        <v>258.68</v>
+        <v>260.27999999999997</v>
       </c>
       <c r="E8" s="10">
-        <v>220.69</v>
+        <v>219.56</v>
       </c>
       <c r="F8" s="10">
-        <v>230.69</v>
+        <v>229.56</v>
       </c>
       <c r="G8" s="10">
-        <v>218.31</v>
-      </c>
-    </row>
-    <row r="9" spans="1:7" x14ac:dyDescent="0.35">
+        <v>217.18</v>
+      </c>
+    </row>
+    <row r="9" spans="1:7" x14ac:dyDescent="0.45">
       <c r="A9" s="11">
-        <v>46317</v>
+        <v>46318</v>
       </c>
       <c r="B9" s="12"/>
       <c r="C9" s="12" t="s">
         <v>11</v>
       </c>
       <c r="D9" s="13">
-        <v>258.68</v>
+        <v>260.27999999999997</v>
       </c>
       <c r="E9" s="13">
-        <v>220.69</v>
+        <v>219.56</v>
       </c>
       <c r="F9" s="13">
-        <v>230.69</v>
+        <v>229.56</v>
       </c>
       <c r="G9" s="13">
-        <v>218.31</v>
-      </c>
-    </row>
-    <row r="10" spans="1:7" x14ac:dyDescent="0.35">
+        <v>217.18</v>
+      </c>
+    </row>
+    <row r="10" spans="1:7" x14ac:dyDescent="0.45">
       <c r="A10" s="7">
-        <v>46317</v>
+        <v>46318</v>
       </c>
       <c r="B10" s="8"/>
       <c r="C10" s="9" t="s">
         <v>12</v>
       </c>
       <c r="D10" s="10">
-        <v>256.87</v>
+        <v>257.92</v>
       </c>
       <c r="E10" s="10">
-        <v>221</v>
+        <v>219.87</v>
       </c>
       <c r="F10" s="10">
-        <v>231</v>
+        <v>229.87</v>
       </c>
       <c r="G10" s="10">
-        <v>219.41</v>
-      </c>
-    </row>
-    <row r="11" spans="1:7" x14ac:dyDescent="0.35">
+        <v>218.27</v>
+      </c>
+    </row>
+    <row r="11" spans="1:7" x14ac:dyDescent="0.45">
       <c r="A11" s="11">
-        <v>46316</v>
+        <v>46317</v>
       </c>
       <c r="B11" s="12"/>
       <c r="C11" s="12" t="s">
         <v>10</v>
       </c>
       <c r="D11" s="13">
-        <v>258.24</v>
+        <v>258.68</v>
       </c>
       <c r="E11" s="13">
-        <v>223.09</v>
+        <v>220.69</v>
       </c>
       <c r="F11" s="13">
-        <v>233.09</v>
+        <v>230.69</v>
       </c>
       <c r="G11" s="13">
-        <v>220.71</v>
-      </c>
-    </row>
-    <row r="12" spans="1:7" x14ac:dyDescent="0.35">
+        <v>218.31</v>
+      </c>
+    </row>
+    <row r="12" spans="1:7" x14ac:dyDescent="0.45">
       <c r="A12" s="7">
-        <v>46316</v>
+        <v>46317</v>
       </c>
       <c r="B12" s="8"/>
       <c r="C12" s="9" t="s">
         <v>11</v>
       </c>
       <c r="D12" s="10">
-        <v>258.24</v>
+        <v>258.68</v>
       </c>
       <c r="E12" s="10">
-        <v>223.09</v>
+        <v>220.69</v>
       </c>
       <c r="F12" s="10">
-        <v>233.09</v>
+        <v>230.69</v>
       </c>
       <c r="G12" s="10">
-        <v>220.71</v>
-      </c>
-    </row>
-    <row r="13" spans="1:7" x14ac:dyDescent="0.35">
+        <v>218.31</v>
+      </c>
+    </row>
+    <row r="13" spans="1:7" x14ac:dyDescent="0.45">
       <c r="A13" s="11">
-        <v>46316</v>
+        <v>46317</v>
       </c>
       <c r="B13" s="12"/>
       <c r="C13" s="12" t="s">
         <v>12</v>
       </c>
       <c r="D13" s="13">
-        <v>255.43</v>
+        <v>256.87</v>
       </c>
       <c r="E13" s="13">
-        <v>221.84</v>
+        <v>221</v>
       </c>
       <c r="F13" s="13">
-        <v>231.84</v>
+        <v>231</v>
       </c>
       <c r="G13" s="13">
-        <v>220.25</v>
-      </c>
-    </row>
-    <row r="14" spans="1:7" x14ac:dyDescent="0.35">
+        <v>219.41</v>
+      </c>
+    </row>
+    <row r="14" spans="1:7" x14ac:dyDescent="0.45">
       <c r="A14" s="14"/>
       <c r="B14" s="14"/>
       <c r="C14" s="15"/>
@@ -941,7 +941,7 @@
       <c r="F14" s="16"/>
       <c r="G14" s="16"/>
     </row>
-    <row r="15" spans="1:7" ht="20" x14ac:dyDescent="0.35">
+    <row r="15" spans="1:7" ht="20.25" x14ac:dyDescent="0.45">
       <c r="A15" s="29" t="s">
         <v>13</v>
       </c>
@@ -952,7 +952,7 @@
       <c r="F15" s="17"/>
       <c r="G15" s="17"/>
     </row>
-    <row r="16" spans="1:7" x14ac:dyDescent="0.35">
+    <row r="16" spans="1:7" x14ac:dyDescent="0.45">
       <c r="A16" s="4" t="s">
         <v>4</v>
       </c>
@@ -971,45 +971,45 @@
       </c>
       <c r="G16" s="17"/>
     </row>
-    <row r="17" spans="1:7" x14ac:dyDescent="0.35">
+    <row r="17" spans="1:7" x14ac:dyDescent="0.45">
       <c r="A17" s="7">
-        <v>46317</v>
+        <v>46318</v>
       </c>
       <c r="B17" s="8"/>
       <c r="C17" s="20" t="s">
         <v>14</v>
       </c>
       <c r="D17" s="10">
-        <v>260.29000000000002</v>
+        <v>261.25</v>
       </c>
       <c r="E17" s="10">
-        <v>223.91</v>
+        <v>222.69</v>
       </c>
       <c r="F17" s="10">
-        <v>233.91</v>
+        <v>232.69</v>
       </c>
       <c r="G17" s="17"/>
     </row>
-    <row r="18" spans="1:7" x14ac:dyDescent="0.35">
+    <row r="18" spans="1:7" x14ac:dyDescent="0.45">
       <c r="A18" s="11">
-        <v>46316</v>
+        <v>46317</v>
       </c>
       <c r="B18" s="12"/>
       <c r="C18" s="12" t="s">
         <v>14</v>
       </c>
       <c r="D18" s="13">
-        <v>258.89</v>
+        <v>260.29000000000002</v>
       </c>
       <c r="E18" s="13">
-        <v>224.78</v>
+        <v>223.91</v>
       </c>
       <c r="F18" s="13">
-        <v>234.78</v>
+        <v>233.91</v>
       </c>
       <c r="G18" s="17"/>
     </row>
-    <row r="19" spans="1:7" x14ac:dyDescent="0.35">
+    <row r="19" spans="1:7" x14ac:dyDescent="0.45">
       <c r="A19" s="14"/>
       <c r="B19" s="14"/>
       <c r="C19" s="15"/>
@@ -1018,7 +1018,7 @@
       <c r="F19" s="16"/>
       <c r="G19" s="17"/>
     </row>
-    <row r="20" spans="1:7" ht="20" x14ac:dyDescent="0.35">
+    <row r="20" spans="1:7" ht="20.25" x14ac:dyDescent="0.45">
       <c r="A20" s="29" t="s">
         <v>15</v>
       </c>
@@ -1029,7 +1029,7 @@
       <c r="F20" s="17"/>
       <c r="G20" s="17"/>
     </row>
-    <row r="21" spans="1:7" x14ac:dyDescent="0.35">
+    <row r="21" spans="1:7" x14ac:dyDescent="0.45">
       <c r="A21" s="4" t="s">
         <v>4</v>
       </c>
@@ -1050,217 +1050,217 @@
         <v>9</v>
       </c>
     </row>
-    <row r="22" spans="1:7" x14ac:dyDescent="0.35">
+    <row r="22" spans="1:7" x14ac:dyDescent="0.45">
       <c r="A22" s="7">
-        <v>46317</v>
+        <v>46318</v>
       </c>
       <c r="B22" s="8"/>
       <c r="C22" s="20" t="s">
         <v>16</v>
       </c>
       <c r="D22" s="10">
-        <v>259.8</v>
+        <v>261.39999999999998</v>
       </c>
       <c r="E22" s="10">
-        <v>220.83</v>
+        <v>219.7</v>
       </c>
       <c r="F22" s="10">
-        <v>230.43</v>
+        <v>229.3</v>
       </c>
       <c r="G22" s="10">
-        <v>217.2</v>
-      </c>
-    </row>
-    <row r="23" spans="1:7" x14ac:dyDescent="0.35">
+        <v>216.07</v>
+      </c>
+    </row>
+    <row r="23" spans="1:7" x14ac:dyDescent="0.45">
       <c r="A23" s="11">
-        <v>46317</v>
+        <v>46318</v>
       </c>
       <c r="B23" s="12"/>
       <c r="C23" s="21" t="s">
         <v>17</v>
       </c>
       <c r="D23" s="13">
-        <v>261.82</v>
+        <v>262.89</v>
       </c>
       <c r="E23" s="13">
-        <v>229.28</v>
+        <v>228.17</v>
       </c>
       <c r="F23" s="13">
-        <v>239.28</v>
+        <v>238.17</v>
       </c>
       <c r="G23" s="13" t="s">
         <v>18</v>
       </c>
     </row>
-    <row r="24" spans="1:7" x14ac:dyDescent="0.35">
+    <row r="24" spans="1:7" x14ac:dyDescent="0.45">
       <c r="A24" s="7">
-        <v>46317</v>
+        <v>46318</v>
       </c>
       <c r="B24" s="8"/>
       <c r="C24" s="20" t="s">
         <v>19</v>
       </c>
       <c r="D24" s="10">
-        <v>262.17</v>
+        <v>263.22000000000003</v>
       </c>
       <c r="E24" s="10">
-        <v>228.55</v>
+        <v>227.44</v>
       </c>
       <c r="F24" s="10">
-        <v>238.55</v>
+        <v>237.44</v>
       </c>
       <c r="G24" s="10" t="s">
         <v>18</v>
       </c>
     </row>
-    <row r="25" spans="1:7" x14ac:dyDescent="0.35">
+    <row r="25" spans="1:7" x14ac:dyDescent="0.45">
       <c r="A25" s="11">
-        <v>46317</v>
+        <v>46318</v>
       </c>
       <c r="B25" s="12"/>
       <c r="C25" s="21" t="s">
         <v>20</v>
       </c>
       <c r="D25" s="13">
-        <v>258.83</v>
+        <v>259.88</v>
       </c>
       <c r="E25" s="13">
-        <v>228.76</v>
+        <v>227.66</v>
       </c>
       <c r="F25" s="13">
-        <v>238.76</v>
+        <v>237.66</v>
       </c>
       <c r="G25" s="13">
-        <v>224.6</v>
-      </c>
-    </row>
-    <row r="26" spans="1:7" x14ac:dyDescent="0.35">
+        <v>223.5</v>
+      </c>
+    </row>
+    <row r="26" spans="1:7" x14ac:dyDescent="0.45">
       <c r="A26" s="7">
-        <v>46317</v>
+        <v>46318</v>
       </c>
       <c r="B26" s="8"/>
       <c r="C26" s="20" t="s">
         <v>21</v>
       </c>
       <c r="D26" s="10">
-        <v>260.37</v>
+        <v>261.39999999999998</v>
       </c>
       <c r="E26" s="10">
-        <v>230.18</v>
+        <v>229.07</v>
       </c>
       <c r="F26" s="10">
-        <v>240.18</v>
+        <v>239.07</v>
       </c>
       <c r="G26" s="10" t="s">
         <v>18</v>
       </c>
     </row>
-    <row r="27" spans="1:7" x14ac:dyDescent="0.35">
+    <row r="27" spans="1:7" x14ac:dyDescent="0.45">
       <c r="A27" s="11">
-        <v>46316</v>
+        <v>46317</v>
       </c>
       <c r="B27" s="12"/>
       <c r="C27" s="12" t="s">
         <v>16</v>
       </c>
       <c r="D27" s="13">
-        <v>259.37</v>
+        <v>259.8</v>
       </c>
       <c r="E27" s="13">
-        <v>223.23</v>
+        <v>220.83</v>
       </c>
       <c r="F27" s="13">
-        <v>232.83</v>
+        <v>230.43</v>
       </c>
       <c r="G27" s="13">
-        <v>219.6</v>
-      </c>
-    </row>
-    <row r="28" spans="1:7" x14ac:dyDescent="0.35">
+        <v>217.2</v>
+      </c>
+    </row>
+    <row r="28" spans="1:7" x14ac:dyDescent="0.45">
       <c r="A28" s="7">
-        <v>46316</v>
+        <v>46317</v>
       </c>
       <c r="B28" s="8"/>
       <c r="C28" s="20" t="s">
         <v>17</v>
       </c>
       <c r="D28" s="10">
-        <v>260.39</v>
+        <v>261.82</v>
       </c>
       <c r="E28" s="22">
-        <v>230.11</v>
+        <v>229.28</v>
       </c>
       <c r="F28" s="22">
-        <v>240.11</v>
+        <v>239.28</v>
       </c>
       <c r="G28" s="22" t="s">
         <v>18</v>
       </c>
     </row>
-    <row r="29" spans="1:7" x14ac:dyDescent="0.35">
+    <row r="29" spans="1:7" x14ac:dyDescent="0.45">
       <c r="A29" s="11">
-        <v>46316</v>
+        <v>46317</v>
       </c>
       <c r="B29" s="12"/>
       <c r="C29" s="12" t="s">
         <v>19</v>
       </c>
       <c r="D29" s="13">
-        <v>260.74</v>
+        <v>262.17</v>
       </c>
       <c r="E29" s="13">
-        <v>229.38</v>
+        <v>228.55</v>
       </c>
       <c r="F29" s="13">
-        <v>239.38</v>
+        <v>238.55</v>
       </c>
       <c r="G29" s="13" t="s">
         <v>18</v>
       </c>
     </row>
-    <row r="30" spans="1:7" x14ac:dyDescent="0.35">
+    <row r="30" spans="1:7" x14ac:dyDescent="0.45">
       <c r="A30" s="7">
-        <v>46316</v>
+        <v>46317</v>
       </c>
       <c r="B30" s="8"/>
       <c r="C30" s="20" t="s">
         <v>20</v>
       </c>
       <c r="D30" s="10">
-        <v>257.39999999999998</v>
+        <v>258.83</v>
       </c>
       <c r="E30" s="22">
-        <v>229.59</v>
+        <v>228.76</v>
       </c>
       <c r="F30" s="22">
-        <v>239.59</v>
+        <v>238.76</v>
       </c>
       <c r="G30" s="22">
-        <v>225.43</v>
-      </c>
-    </row>
-    <row r="31" spans="1:7" x14ac:dyDescent="0.35">
+        <v>224.6</v>
+      </c>
+    </row>
+    <row r="31" spans="1:7" x14ac:dyDescent="0.45">
       <c r="A31" s="11">
-        <v>46316</v>
+        <v>46317</v>
       </c>
       <c r="B31" s="12"/>
       <c r="C31" s="12" t="s">
         <v>21</v>
       </c>
       <c r="D31" s="13">
-        <v>258.94</v>
+        <v>260.37</v>
       </c>
       <c r="E31" s="13">
-        <v>231.01</v>
+        <v>230.18</v>
       </c>
       <c r="F31" s="13">
-        <v>241.01</v>
+        <v>240.18</v>
       </c>
       <c r="G31" s="13" t="s">
         <v>18</v>
       </c>
     </row>
-    <row r="32" spans="1:7" x14ac:dyDescent="0.35">
+    <row r="32" spans="1:7" x14ac:dyDescent="0.45">
       <c r="A32" s="14"/>
       <c r="B32" s="14"/>
       <c r="C32" s="15"/>
@@ -1269,7 +1269,7 @@
       <c r="F32" s="17"/>
       <c r="G32" s="17"/>
     </row>
-    <row r="33" spans="1:7" ht="20" x14ac:dyDescent="0.35">
+    <row r="33" spans="1:7" ht="20.25" x14ac:dyDescent="0.45">
       <c r="A33" s="29" t="s">
         <v>22</v>
       </c>
@@ -1280,7 +1280,7 @@
       <c r="F33" s="17"/>
       <c r="G33" s="17"/>
     </row>
-    <row r="34" spans="1:7" x14ac:dyDescent="0.35">
+    <row r="34" spans="1:7" x14ac:dyDescent="0.45">
       <c r="A34" s="23" t="s">
         <v>4</v>
       </c>
@@ -1299,54 +1299,54 @@
       </c>
       <c r="G34" s="17"/>
     </row>
-    <row r="35" spans="1:7" x14ac:dyDescent="0.35">
+    <row r="35" spans="1:7" x14ac:dyDescent="0.45">
       <c r="A35" s="7">
-        <v>46317</v>
+        <v>46318</v>
       </c>
       <c r="B35" s="8"/>
       <c r="C35" s="20" t="s">
         <v>23</v>
       </c>
       <c r="D35" s="10">
-        <v>255.42</v>
+        <v>256.47000000000003</v>
       </c>
       <c r="E35" s="10">
-        <v>219.96</v>
+        <v>218.83</v>
       </c>
       <c r="F35" s="10">
-        <v>228.96</v>
+        <v>227.83</v>
       </c>
       <c r="G35" s="17"/>
     </row>
-    <row r="36" spans="1:7" x14ac:dyDescent="0.35">
+    <row r="36" spans="1:7" x14ac:dyDescent="0.45">
       <c r="A36" s="11">
-        <v>46316</v>
+        <v>46317</v>
       </c>
       <c r="B36" s="12"/>
       <c r="C36" s="12" t="s">
         <v>23</v>
       </c>
       <c r="D36" s="13">
-        <v>253.98</v>
+        <v>255.42</v>
       </c>
       <c r="E36" s="13">
-        <v>220.8</v>
+        <v>219.96</v>
       </c>
       <c r="F36" s="13">
-        <v>229.8</v>
+        <v>228.96</v>
       </c>
       <c r="G36" s="17"/>
     </row>
-    <row r="37" spans="1:7" x14ac:dyDescent="0.35">
+    <row r="37" spans="1:7" x14ac:dyDescent="0.45">
       <c r="A37" s="7">
-        <v>46317</v>
+        <v>46318</v>
       </c>
       <c r="B37" s="8"/>
       <c r="C37" s="20" t="s">
         <v>24</v>
       </c>
       <c r="D37" s="10">
-        <v>271.04000000000002</v>
+        <v>272.08999999999997</v>
       </c>
       <c r="E37" s="10" t="s">
         <v>18</v>
@@ -1356,16 +1356,16 @@
       </c>
       <c r="G37" s="17"/>
     </row>
-    <row r="38" spans="1:7" x14ac:dyDescent="0.35">
+    <row r="38" spans="1:7" x14ac:dyDescent="0.45">
       <c r="A38" s="11">
-        <v>46316</v>
+        <v>46317</v>
       </c>
       <c r="B38" s="12"/>
       <c r="C38" s="12" t="s">
         <v>24</v>
       </c>
       <c r="D38" s="13">
-        <v>269.60000000000002</v>
+        <v>271.04000000000002</v>
       </c>
       <c r="E38" s="13" t="s">
         <v>18</v>
@@ -1375,7 +1375,7 @@
       </c>
       <c r="G38" s="17"/>
     </row>
-    <row r="39" spans="1:7" x14ac:dyDescent="0.35">
+    <row r="39" spans="1:7" x14ac:dyDescent="0.45">
       <c r="A39" s="24"/>
       <c r="B39" s="24"/>
       <c r="C39" s="15"/>
@@ -1384,7 +1384,7 @@
       <c r="F39" s="17"/>
       <c r="G39" s="17"/>
     </row>
-    <row r="40" spans="1:7" ht="20" x14ac:dyDescent="0.35">
+    <row r="40" spans="1:7" ht="20.25" x14ac:dyDescent="0.45">
       <c r="A40" s="29" t="s">
         <v>25</v>
       </c>
@@ -1395,7 +1395,7 @@
       <c r="F40" s="17"/>
       <c r="G40" s="17"/>
     </row>
-    <row r="41" spans="1:7" x14ac:dyDescent="0.35">
+    <row r="41" spans="1:7" x14ac:dyDescent="0.45">
       <c r="A41" s="23" t="s">
         <v>4</v>
       </c>
@@ -1414,83 +1414,83 @@
       </c>
       <c r="G41" s="17"/>
     </row>
-    <row r="42" spans="1:7" x14ac:dyDescent="0.35">
+    <row r="42" spans="1:7" x14ac:dyDescent="0.45">
       <c r="A42" s="7">
-        <v>46317</v>
+        <v>46318</v>
       </c>
       <c r="B42" s="8"/>
       <c r="C42" s="20" t="s">
         <v>26</v>
       </c>
       <c r="D42" s="10">
-        <v>265.45999999999998</v>
+        <v>266.58</v>
       </c>
       <c r="E42" s="10">
-        <v>230.66</v>
+        <v>229.81</v>
       </c>
       <c r="F42" s="10">
-        <v>240.66</v>
+        <v>239.81</v>
       </c>
       <c r="G42" s="17"/>
     </row>
-    <row r="43" spans="1:7" x14ac:dyDescent="0.35">
+    <row r="43" spans="1:7" x14ac:dyDescent="0.45">
       <c r="A43" s="11">
-        <v>46317</v>
+        <v>46318</v>
       </c>
       <c r="B43" s="12"/>
       <c r="C43" s="21" t="s">
         <v>27</v>
       </c>
       <c r="D43" s="13">
-        <v>265.07</v>
+        <v>266.18</v>
       </c>
       <c r="E43" s="13">
-        <v>231.07</v>
+        <v>230.23</v>
       </c>
       <c r="F43" s="13">
-        <v>241.07</v>
+        <v>240.23</v>
       </c>
       <c r="G43" s="17"/>
     </row>
-    <row r="44" spans="1:7" x14ac:dyDescent="0.35">
+    <row r="44" spans="1:7" x14ac:dyDescent="0.45">
       <c r="A44" s="7">
-        <v>46316</v>
+        <v>46317</v>
       </c>
       <c r="B44" s="8"/>
       <c r="C44" s="20" t="s">
         <v>26</v>
       </c>
       <c r="D44" s="10">
-        <v>264</v>
+        <v>265.45999999999998</v>
       </c>
       <c r="E44" s="10">
-        <v>231.3</v>
+        <v>230.66</v>
       </c>
       <c r="F44" s="10">
-        <v>241.3</v>
+        <v>240.66</v>
       </c>
       <c r="G44" s="17"/>
     </row>
-    <row r="45" spans="1:7" x14ac:dyDescent="0.35">
+    <row r="45" spans="1:7" x14ac:dyDescent="0.45">
       <c r="A45" s="11">
-        <v>46316</v>
+        <v>46317</v>
       </c>
       <c r="B45" s="12"/>
       <c r="C45" s="21" t="s">
         <v>27</v>
       </c>
       <c r="D45" s="13">
-        <v>263.61</v>
+        <v>265.07</v>
       </c>
       <c r="E45" s="13">
-        <v>231.71</v>
+        <v>231.07</v>
       </c>
       <c r="F45" s="13">
-        <v>241.71</v>
+        <v>241.07</v>
       </c>
       <c r="G45" s="17"/>
     </row>
-    <row r="46" spans="1:7" x14ac:dyDescent="0.35">
+    <row r="46" spans="1:7" x14ac:dyDescent="0.45">
       <c r="A46" s="14"/>
       <c r="B46" s="24"/>
       <c r="C46" s="15"/>
@@ -1499,7 +1499,7 @@
       <c r="F46" s="16"/>
       <c r="G46" s="17"/>
     </row>
-    <row r="47" spans="1:7" ht="20" x14ac:dyDescent="0.35">
+    <row r="47" spans="1:7" ht="20.25" x14ac:dyDescent="0.45">
       <c r="A47" s="25" t="s">
         <v>28</v>
       </c>
@@ -1510,7 +1510,7 @@
       <c r="F47" s="17"/>
       <c r="G47" s="17"/>
     </row>
-    <row r="48" spans="1:7" x14ac:dyDescent="0.35">
+    <row r="48" spans="1:7" x14ac:dyDescent="0.45">
       <c r="A48" s="23" t="s">
         <v>4</v>
       </c>
@@ -1529,83 +1529,83 @@
       </c>
       <c r="G48" s="17"/>
     </row>
-    <row r="49" spans="1:7" x14ac:dyDescent="0.35">
+    <row r="49" spans="1:7" x14ac:dyDescent="0.45">
       <c r="A49" s="7">
-        <v>46317</v>
+        <v>46318</v>
       </c>
       <c r="B49" s="8"/>
       <c r="C49" s="20" t="s">
         <v>29</v>
       </c>
       <c r="D49" s="10">
-        <v>256.92</v>
+        <v>259.07</v>
       </c>
       <c r="E49" s="10">
-        <v>223.9</v>
+        <v>222.05</v>
       </c>
       <c r="F49" s="10">
-        <v>233.9</v>
+        <v>232.05</v>
       </c>
       <c r="G49" s="28"/>
     </row>
-    <row r="50" spans="1:7" x14ac:dyDescent="0.35">
+    <row r="50" spans="1:7" x14ac:dyDescent="0.45">
       <c r="A50" s="11">
-        <v>46317</v>
+        <v>46318</v>
       </c>
       <c r="B50" s="12"/>
       <c r="C50" s="21" t="s">
         <v>30</v>
       </c>
       <c r="D50" s="13">
-        <v>254.43</v>
+        <v>256.57</v>
       </c>
       <c r="E50" s="13">
-        <v>223.49</v>
+        <v>221.64</v>
       </c>
       <c r="F50" s="13">
-        <v>233.49</v>
+        <v>231.64</v>
       </c>
       <c r="G50" s="28"/>
     </row>
-    <row r="51" spans="1:7" x14ac:dyDescent="0.35">
+    <row r="51" spans="1:7" x14ac:dyDescent="0.45">
       <c r="A51" s="7">
-        <v>46316</v>
+        <v>46317</v>
       </c>
       <c r="B51" s="8"/>
       <c r="C51" s="20" t="s">
         <v>29</v>
       </c>
       <c r="D51" s="10">
-        <v>255.72</v>
+        <v>256.92</v>
       </c>
       <c r="E51" s="10">
-        <v>225.15</v>
+        <v>223.9</v>
       </c>
       <c r="F51" s="10">
-        <v>235.15</v>
+        <v>233.9</v>
       </c>
       <c r="G51" s="17"/>
     </row>
-    <row r="52" spans="1:7" x14ac:dyDescent="0.35">
+    <row r="52" spans="1:7" x14ac:dyDescent="0.45">
       <c r="A52" s="11">
-        <v>46316</v>
+        <v>46317</v>
       </c>
       <c r="B52" s="12"/>
       <c r="C52" s="21" t="s">
         <v>30</v>
       </c>
       <c r="D52" s="13">
-        <v>253.24</v>
+        <v>254.43</v>
       </c>
       <c r="E52" s="13">
-        <v>224.75</v>
+        <v>223.49</v>
       </c>
       <c r="F52" s="13">
-        <v>234.75</v>
+        <v>233.49</v>
       </c>
       <c r="G52" s="17"/>
     </row>
-    <row r="53" spans="1:7" x14ac:dyDescent="0.35">
+    <row r="53" spans="1:7" x14ac:dyDescent="0.45">
       <c r="A53" s="14"/>
       <c r="B53" s="14"/>
       <c r="C53" s="15"/>
@@ -1614,7 +1614,7 @@
       <c r="F53" s="16"/>
       <c r="G53" s="17"/>
     </row>
-    <row r="54" spans="1:7" ht="20" x14ac:dyDescent="0.35">
+    <row r="54" spans="1:7" ht="20.25" x14ac:dyDescent="0.45">
       <c r="A54" s="27" t="s">
         <v>31</v>
       </c>
@@ -1625,7 +1625,7 @@
       <c r="F54" s="17"/>
       <c r="G54" s="17"/>
     </row>
-    <row r="55" spans="1:7" x14ac:dyDescent="0.35">
+    <row r="55" spans="1:7" x14ac:dyDescent="0.45">
       <c r="A55" s="23" t="s">
         <v>4</v>
       </c>
@@ -1644,54 +1644,54 @@
       </c>
       <c r="G55" s="17"/>
     </row>
-    <row r="56" spans="1:7" x14ac:dyDescent="0.35">
+    <row r="56" spans="1:7" x14ac:dyDescent="0.45">
       <c r="A56" s="7">
-        <v>46317</v>
+        <v>46318</v>
       </c>
       <c r="B56" s="8"/>
       <c r="C56" s="20" t="s">
         <v>32</v>
       </c>
       <c r="D56" s="10">
-        <v>271.54000000000002</v>
+        <v>272.56</v>
       </c>
       <c r="E56" s="10">
-        <v>247.85</v>
+        <v>247.07</v>
       </c>
       <c r="F56" s="10">
-        <v>257.85000000000002</v>
+        <v>257.07</v>
       </c>
       <c r="G56" s="17"/>
     </row>
-    <row r="57" spans="1:7" x14ac:dyDescent="0.35">
+    <row r="57" spans="1:7" x14ac:dyDescent="0.45">
       <c r="A57" s="11">
-        <v>46317</v>
+        <v>46318</v>
       </c>
       <c r="B57" s="12"/>
       <c r="C57" s="21" t="s">
         <v>33</v>
       </c>
       <c r="D57" s="13">
-        <v>258.42</v>
+        <v>260.02</v>
       </c>
       <c r="E57" s="13">
-        <v>229.16</v>
+        <v>227.94</v>
       </c>
       <c r="F57" s="13">
-        <v>239.16</v>
+        <v>237.94</v>
       </c>
       <c r="G57" s="17"/>
     </row>
-    <row r="58" spans="1:7" x14ac:dyDescent="0.35">
+    <row r="58" spans="1:7" x14ac:dyDescent="0.45">
       <c r="A58" s="7">
-        <v>46317</v>
+        <v>46318</v>
       </c>
       <c r="B58" s="8"/>
       <c r="C58" s="20" t="s">
         <v>34</v>
       </c>
       <c r="D58" s="10">
-        <v>259.2</v>
+        <v>260.82</v>
       </c>
       <c r="E58" s="10" t="s">
         <v>18</v>
@@ -1701,111 +1701,111 @@
       </c>
       <c r="G58" s="17"/>
     </row>
-    <row r="59" spans="1:7" x14ac:dyDescent="0.35">
+    <row r="59" spans="1:7" x14ac:dyDescent="0.45">
       <c r="A59" s="11">
-        <v>46317</v>
+        <v>46318</v>
       </c>
       <c r="B59" s="12"/>
       <c r="C59" s="21" t="s">
         <v>35</v>
       </c>
       <c r="D59" s="13">
-        <v>255.41</v>
+        <v>256.89999999999998</v>
       </c>
       <c r="E59" s="13">
-        <v>223.54</v>
+        <v>222.32</v>
       </c>
       <c r="F59" s="13" t="s">
         <v>18</v>
       </c>
       <c r="G59" s="17"/>
     </row>
-    <row r="60" spans="1:7" x14ac:dyDescent="0.35">
+    <row r="60" spans="1:7" x14ac:dyDescent="0.45">
       <c r="A60" s="7">
-        <v>46317</v>
+        <v>46318</v>
       </c>
       <c r="B60" s="8"/>
       <c r="C60" s="20" t="s">
         <v>36</v>
       </c>
       <c r="D60" s="10">
-        <v>251.24</v>
+        <v>252.73</v>
       </c>
       <c r="E60" s="10">
-        <v>219.48</v>
+        <v>218.26</v>
       </c>
       <c r="F60" s="10">
-        <v>229.48</v>
+        <v>228.26</v>
       </c>
       <c r="G60" s="17"/>
     </row>
-    <row r="61" spans="1:7" x14ac:dyDescent="0.35">
+    <row r="61" spans="1:7" x14ac:dyDescent="0.45">
       <c r="A61" s="11">
-        <v>46317</v>
+        <v>46318</v>
       </c>
       <c r="B61" s="12"/>
       <c r="C61" s="21" t="s">
         <v>37</v>
       </c>
       <c r="D61" s="13">
-        <v>259.37</v>
+        <v>260.32</v>
       </c>
       <c r="E61" s="13">
-        <v>241.11</v>
+        <v>240.17</v>
       </c>
       <c r="F61" s="13" t="s">
         <v>18</v>
       </c>
       <c r="G61" s="17"/>
     </row>
-    <row r="62" spans="1:7" x14ac:dyDescent="0.35">
+    <row r="62" spans="1:7" x14ac:dyDescent="0.45">
       <c r="A62" s="7">
-        <v>46316</v>
+        <v>46317</v>
       </c>
       <c r="B62" s="8"/>
       <c r="C62" s="20" t="s">
         <v>32</v>
       </c>
       <c r="D62" s="10">
-        <v>270.11</v>
+        <v>271.54000000000002</v>
       </c>
       <c r="E62" s="10">
-        <v>248.54</v>
+        <v>247.85</v>
       </c>
       <c r="F62" s="10">
-        <v>258.54000000000002</v>
+        <v>257.85000000000002</v>
       </c>
       <c r="G62" s="17"/>
     </row>
-    <row r="63" spans="1:7" x14ac:dyDescent="0.35">
+    <row r="63" spans="1:7" x14ac:dyDescent="0.45">
       <c r="A63" s="11">
-        <v>46316</v>
+        <v>46317</v>
       </c>
       <c r="B63" s="12"/>
       <c r="C63" s="21" t="s">
         <v>33</v>
       </c>
       <c r="D63" s="13">
-        <v>257.52999999999997</v>
+        <v>258.42</v>
       </c>
       <c r="E63" s="13">
-        <v>230.03</v>
+        <v>229.16</v>
       </c>
       <c r="F63" s="13">
-        <v>240.03</v>
+        <v>239.16</v>
       </c>
       <c r="G63" s="17"/>
     </row>
-    <row r="64" spans="1:7" x14ac:dyDescent="0.35">
+    <row r="64" spans="1:7" x14ac:dyDescent="0.45">
       <c r="A64" s="7">
-        <v>46316</v>
+        <v>46317</v>
       </c>
       <c r="B64" s="8"/>
       <c r="C64" s="20" t="s">
         <v>34</v>
       </c>
       <c r="D64" s="10">
-        <v>258.31</v>
+        <v>259.2</v>
       </c>
       <c r="E64" s="10" t="s">
         <v>18</v>
@@ -1815,55 +1815,55 @@
       </c>
       <c r="G64" s="17"/>
     </row>
-    <row r="65" spans="1:6" x14ac:dyDescent="0.35">
+    <row r="65" spans="1:6" x14ac:dyDescent="0.45">
       <c r="A65" s="11">
-        <v>46316</v>
+        <v>46317</v>
       </c>
       <c r="B65" s="12"/>
       <c r="C65" s="21" t="s">
         <v>35</v>
       </c>
       <c r="D65" s="13">
-        <v>254.57</v>
+        <v>255.41</v>
       </c>
       <c r="E65" s="13">
-        <v>224.41</v>
+        <v>223.54</v>
       </c>
       <c r="F65" s="13" t="s">
         <v>18</v>
       </c>
     </row>
-    <row r="66" spans="1:6" x14ac:dyDescent="0.35">
+    <row r="66" spans="1:6" x14ac:dyDescent="0.45">
       <c r="A66" s="7">
-        <v>46316</v>
+        <v>46317</v>
       </c>
       <c r="B66" s="8"/>
       <c r="C66" s="20" t="s">
         <v>36</v>
       </c>
       <c r="D66" s="10">
-        <v>250.4</v>
+        <v>251.24</v>
       </c>
       <c r="E66" s="10">
-        <v>220.35</v>
+        <v>219.48</v>
       </c>
       <c r="F66" s="10">
-        <v>230.35</v>
-      </c>
-    </row>
-    <row r="67" spans="1:6" x14ac:dyDescent="0.35">
+        <v>229.48</v>
+      </c>
+    </row>
+    <row r="67" spans="1:6" x14ac:dyDescent="0.45">
       <c r="A67" s="11">
-        <v>46316</v>
+        <v>46317</v>
       </c>
       <c r="B67" s="12"/>
       <c r="C67" s="21" t="s">
         <v>37</v>
       </c>
       <c r="D67" s="13">
-        <v>257.97000000000003</v>
+        <v>259.37</v>
       </c>
       <c r="E67" s="13">
-        <v>241.87</v>
+        <v>241.11</v>
       </c>
       <c r="F67" s="13" t="s">
         <v>18</v>
@@ -1891,6 +1891,15 @@
 </file>
 
 <file path=customXml/item1.xml><?xml version="1.0" encoding="utf-8"?>
+<?mso-contentType ?>
+<FormTemplates xmlns="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms">
+  <Display>DocumentLibraryForm</Display>
+  <Edit>DocumentLibraryForm</Edit>
+  <New>DocumentLibraryForm</New>
+</FormTemplates>
+</file>
+
+<file path=customXml/item2.xml><?xml version="1.0" encoding="utf-8"?>
 <p:properties xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls">
   <documentManagement>
     <lcf76f155ced4ddcb4097134ff3c332f xmlns="87276d81-85f4-4ef2-9e6e-55066304288f">
@@ -1899,15 +1908,6 @@
     <TaxCatchAll xmlns="b23b8984-eafa-4e79-985e-54f52f3da58e" xsi:nil="true"/>
   </documentManagement>
 </p:properties>
-</file>
-
-<file path=customXml/item2.xml><?xml version="1.0" encoding="utf-8"?>
-<?mso-contentType ?>
-<FormTemplates xmlns="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms">
-  <Display>DocumentLibraryForm</Display>
-  <Edit>DocumentLibraryForm</Edit>
-  <New>DocumentLibraryForm</New>
-</FormTemplates>
 </file>
 
 <file path=customXml/item3.xml><?xml version="1.0" encoding="utf-8"?>
@@ -2171,20 +2171,20 @@
 </file>
 
 <file path=customXml/itemProps1.xml><?xml version="1.0" encoding="utf-8"?>
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{F60519E9-FD90-4339-869C-BC2F85719BB8}">
+  <ds:schemaRefs>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms"/>
+  </ds:schemaRefs>
+</ds:datastoreItem>
+</file>
+
+<file path=customXml/itemProps2.xml><?xml version="1.0" encoding="utf-8"?>
 <ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{57A83D98-2BAE-4D83-823A-D31C464B620C}">
   <ds:schemaRefs>
     <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/properties"/>
     <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
     <ds:schemaRef ds:uri="87276d81-85f4-4ef2-9e6e-55066304288f"/>
     <ds:schemaRef ds:uri="b23b8984-eafa-4e79-985e-54f52f3da58e"/>
-  </ds:schemaRefs>
-</ds:datastoreItem>
-</file>
-
-<file path=customXml/itemProps2.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{F60519E9-FD90-4339-869C-BC2F85719BB8}">
-  <ds:schemaRefs>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms"/>
   </ds:schemaRefs>
 </ds:datastoreItem>
 </file>

</xml_diff>

<commit_message>
Fri Oct 23 06:05:55 UTC 2026
</commit_message>
<xml_diff>
--- a/bp.com-content-dam-bp-country-sites-en_au-australia-home-products-services-pricing-tgp-excel.xlsx
+++ b/bp.com-content-dam-bp-country-sites-en_au-australia-home-products-services-pricing-tgp-excel.xlsx
@@ -8,14 +8,14 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://bp365.sharepoint.com/sites/WholesalePricing/Shared Documents/B2C/TGP/Daily TGP/Web TGP/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="14_{A56F2BA7-A5D4-4540-9A5C-5C5A324CDACF}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="14_{76438D39-9C43-4744-BBD8-0A9721CE037B}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="20490" yWindow="-16320" windowWidth="29040" windowHeight="15720" xr2:uid="{1B412EEF-F96D-4DF4-A4E9-C7F0F183C2FB}"/>
+    <workbookView xWindow="20715" yWindow="-16320" windowWidth="29040" windowHeight="15720" xr2:uid="{1B412EEF-F96D-4DF4-A4E9-C7F0F183C2FB}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
   </sheets>
-  <calcPr calcId="191028" concurrentManualCount="20"/>
+  <calcPr calcId="191028" iterateDelta="1E-4"/>
   <extLst>
     <ext xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" uri="{140A7094-0E35-4892-8432-C4D2E57EDEB5}">
       <x15:workbookPr chartTrackingRefBase="1"/>
@@ -808,128 +808,128 @@
     </row>
     <row r="8" spans="1:7" x14ac:dyDescent="0.45">
       <c r="A8" s="7">
-        <v>46318</v>
+        <v>46319</v>
       </c>
       <c r="B8" s="8"/>
       <c r="C8" s="9" t="s">
         <v>10</v>
       </c>
       <c r="D8" s="10">
-        <v>260.27999999999997</v>
+        <v>261.57</v>
       </c>
       <c r="E8" s="10">
-        <v>219.56</v>
+        <v>218.41</v>
       </c>
       <c r="F8" s="10">
-        <v>229.56</v>
+        <v>228.41</v>
       </c>
       <c r="G8" s="10">
-        <v>217.18</v>
+        <v>216.03</v>
       </c>
     </row>
     <row r="9" spans="1:7" x14ac:dyDescent="0.45">
       <c r="A9" s="11">
-        <v>46318</v>
+        <v>46319</v>
       </c>
       <c r="B9" s="12"/>
       <c r="C9" s="12" t="s">
         <v>11</v>
       </c>
       <c r="D9" s="13">
-        <v>260.27999999999997</v>
+        <v>261.57</v>
       </c>
       <c r="E9" s="13">
-        <v>219.56</v>
+        <v>218.41</v>
       </c>
       <c r="F9" s="13">
-        <v>229.56</v>
+        <v>228.41</v>
       </c>
       <c r="G9" s="13">
-        <v>217.18</v>
+        <v>216.03</v>
       </c>
     </row>
     <row r="10" spans="1:7" x14ac:dyDescent="0.45">
       <c r="A10" s="7">
-        <v>46318</v>
+        <v>46319</v>
       </c>
       <c r="B10" s="8"/>
       <c r="C10" s="9" t="s">
         <v>12</v>
       </c>
       <c r="D10" s="10">
-        <v>257.92</v>
+        <v>259.04000000000002</v>
       </c>
       <c r="E10" s="10">
-        <v>219.87</v>
+        <v>219.66</v>
       </c>
       <c r="F10" s="10">
-        <v>229.87</v>
+        <v>229.66</v>
       </c>
       <c r="G10" s="10">
-        <v>218.27</v>
+        <v>218.07</v>
       </c>
     </row>
     <row r="11" spans="1:7" x14ac:dyDescent="0.45">
       <c r="A11" s="11">
-        <v>46317</v>
+        <v>46318</v>
       </c>
       <c r="B11" s="12"/>
       <c r="C11" s="12" t="s">
         <v>10</v>
       </c>
       <c r="D11" s="13">
-        <v>258.68</v>
+        <v>260.27999999999997</v>
       </c>
       <c r="E11" s="13">
-        <v>220.69</v>
+        <v>219.56</v>
       </c>
       <c r="F11" s="13">
-        <v>230.69</v>
+        <v>229.56</v>
       </c>
       <c r="G11" s="13">
-        <v>218.31</v>
+        <v>217.18</v>
       </c>
     </row>
     <row r="12" spans="1:7" x14ac:dyDescent="0.45">
       <c r="A12" s="7">
-        <v>46317</v>
+        <v>46318</v>
       </c>
       <c r="B12" s="8"/>
       <c r="C12" s="9" t="s">
         <v>11</v>
       </c>
       <c r="D12" s="10">
-        <v>258.68</v>
+        <v>260.27999999999997</v>
       </c>
       <c r="E12" s="10">
-        <v>220.69</v>
+        <v>219.56</v>
       </c>
       <c r="F12" s="10">
-        <v>230.69</v>
+        <v>229.56</v>
       </c>
       <c r="G12" s="10">
-        <v>218.31</v>
+        <v>217.18</v>
       </c>
     </row>
     <row r="13" spans="1:7" x14ac:dyDescent="0.45">
       <c r="A13" s="11">
-        <v>46317</v>
+        <v>46318</v>
       </c>
       <c r="B13" s="12"/>
       <c r="C13" s="12" t="s">
         <v>12</v>
       </c>
       <c r="D13" s="13">
-        <v>256.87</v>
+        <v>257.92</v>
       </c>
       <c r="E13" s="13">
-        <v>221</v>
+        <v>219.87</v>
       </c>
       <c r="F13" s="13">
-        <v>231</v>
+        <v>229.87</v>
       </c>
       <c r="G13" s="13">
-        <v>219.41</v>
+        <v>218.27</v>
       </c>
     </row>
     <row r="14" spans="1:7" x14ac:dyDescent="0.45">
@@ -973,39 +973,39 @@
     </row>
     <row r="17" spans="1:7" x14ac:dyDescent="0.45">
       <c r="A17" s="7">
-        <v>46318</v>
+        <v>46319</v>
       </c>
       <c r="B17" s="8"/>
       <c r="C17" s="20" t="s">
         <v>14</v>
       </c>
       <c r="D17" s="10">
-        <v>261.25</v>
+        <v>262.33</v>
       </c>
       <c r="E17" s="10">
-        <v>222.69</v>
+        <v>222.45</v>
       </c>
       <c r="F17" s="10">
-        <v>232.69</v>
+        <v>232.45</v>
       </c>
       <c r="G17" s="17"/>
     </row>
     <row r="18" spans="1:7" x14ac:dyDescent="0.45">
       <c r="A18" s="11">
-        <v>46317</v>
+        <v>46318</v>
       </c>
       <c r="B18" s="12"/>
       <c r="C18" s="12" t="s">
         <v>14</v>
       </c>
       <c r="D18" s="13">
-        <v>260.29000000000002</v>
+        <v>261.25</v>
       </c>
       <c r="E18" s="13">
-        <v>223.91</v>
+        <v>222.69</v>
       </c>
       <c r="F18" s="13">
-        <v>233.91</v>
+        <v>232.69</v>
       </c>
       <c r="G18" s="17"/>
     </row>
@@ -1052,41 +1052,41 @@
     </row>
     <row r="22" spans="1:7" x14ac:dyDescent="0.45">
       <c r="A22" s="7">
-        <v>46318</v>
+        <v>46319</v>
       </c>
       <c r="B22" s="8"/>
       <c r="C22" s="20" t="s">
         <v>16</v>
       </c>
       <c r="D22" s="10">
-        <v>261.39999999999998</v>
+        <v>262.69</v>
       </c>
       <c r="E22" s="10">
-        <v>219.7</v>
+        <v>218.56</v>
       </c>
       <c r="F22" s="10">
-        <v>229.3</v>
+        <v>228.16</v>
       </c>
       <c r="G22" s="10">
-        <v>216.07</v>
+        <v>214.93</v>
       </c>
     </row>
     <row r="23" spans="1:7" x14ac:dyDescent="0.45">
       <c r="A23" s="11">
-        <v>46318</v>
+        <v>46319</v>
       </c>
       <c r="B23" s="12"/>
       <c r="C23" s="21" t="s">
         <v>17</v>
       </c>
       <c r="D23" s="13">
-        <v>262.89</v>
+        <v>264.01</v>
       </c>
       <c r="E23" s="13">
-        <v>228.17</v>
+        <v>227.98</v>
       </c>
       <c r="F23" s="13">
-        <v>238.17</v>
+        <v>237.98</v>
       </c>
       <c r="G23" s="13" t="s">
         <v>18</v>
@@ -1094,20 +1094,20 @@
     </row>
     <row r="24" spans="1:7" x14ac:dyDescent="0.45">
       <c r="A24" s="7">
-        <v>46318</v>
+        <v>46319</v>
       </c>
       <c r="B24" s="8"/>
       <c r="C24" s="20" t="s">
         <v>19</v>
       </c>
       <c r="D24" s="10">
-        <v>263.22000000000003</v>
+        <v>264.33999999999997</v>
       </c>
       <c r="E24" s="10">
-        <v>227.44</v>
+        <v>227.25</v>
       </c>
       <c r="F24" s="10">
-        <v>237.44</v>
+        <v>237.25</v>
       </c>
       <c r="G24" s="10" t="s">
         <v>18</v>
@@ -1115,41 +1115,41 @@
     </row>
     <row r="25" spans="1:7" x14ac:dyDescent="0.45">
       <c r="A25" s="11">
-        <v>46318</v>
+        <v>46319</v>
       </c>
       <c r="B25" s="12"/>
       <c r="C25" s="21" t="s">
         <v>20</v>
       </c>
       <c r="D25" s="13">
-        <v>259.88</v>
+        <v>261.01</v>
       </c>
       <c r="E25" s="13">
-        <v>227.66</v>
+        <v>227.47</v>
       </c>
       <c r="F25" s="13">
-        <v>237.66</v>
+        <v>237.47</v>
       </c>
       <c r="G25" s="13">
-        <v>223.5</v>
+        <v>223.31</v>
       </c>
     </row>
     <row r="26" spans="1:7" x14ac:dyDescent="0.45">
       <c r="A26" s="7">
-        <v>46318</v>
+        <v>46319</v>
       </c>
       <c r="B26" s="8"/>
       <c r="C26" s="20" t="s">
         <v>21</v>
       </c>
       <c r="D26" s="10">
-        <v>261.39999999999998</v>
+        <v>262.5</v>
       </c>
       <c r="E26" s="10">
-        <v>229.07</v>
+        <v>228.88</v>
       </c>
       <c r="F26" s="10">
-        <v>239.07</v>
+        <v>238.88</v>
       </c>
       <c r="G26" s="10" t="s">
         <v>18</v>
@@ -1157,41 +1157,41 @@
     </row>
     <row r="27" spans="1:7" x14ac:dyDescent="0.45">
       <c r="A27" s="11">
-        <v>46317</v>
+        <v>46318</v>
       </c>
       <c r="B27" s="12"/>
       <c r="C27" s="12" t="s">
         <v>16</v>
       </c>
       <c r="D27" s="13">
-        <v>259.8</v>
+        <v>261.39999999999998</v>
       </c>
       <c r="E27" s="13">
-        <v>220.83</v>
+        <v>219.7</v>
       </c>
       <c r="F27" s="13">
-        <v>230.43</v>
+        <v>229.3</v>
       </c>
       <c r="G27" s="13">
-        <v>217.2</v>
+        <v>216.07</v>
       </c>
     </row>
     <row r="28" spans="1:7" x14ac:dyDescent="0.45">
       <c r="A28" s="7">
-        <v>46317</v>
+        <v>46318</v>
       </c>
       <c r="B28" s="8"/>
       <c r="C28" s="20" t="s">
         <v>17</v>
       </c>
       <c r="D28" s="10">
-        <v>261.82</v>
+        <v>262.89</v>
       </c>
       <c r="E28" s="22">
-        <v>229.28</v>
+        <v>228.17</v>
       </c>
       <c r="F28" s="22">
-        <v>239.28</v>
+        <v>238.17</v>
       </c>
       <c r="G28" s="22" t="s">
         <v>18</v>
@@ -1199,20 +1199,20 @@
     </row>
     <row r="29" spans="1:7" x14ac:dyDescent="0.45">
       <c r="A29" s="11">
-        <v>46317</v>
+        <v>46318</v>
       </c>
       <c r="B29" s="12"/>
       <c r="C29" s="12" t="s">
         <v>19</v>
       </c>
       <c r="D29" s="13">
-        <v>262.17</v>
+        <v>263.22000000000003</v>
       </c>
       <c r="E29" s="13">
-        <v>228.55</v>
+        <v>227.44</v>
       </c>
       <c r="F29" s="13">
-        <v>238.55</v>
+        <v>237.44</v>
       </c>
       <c r="G29" s="13" t="s">
         <v>18</v>
@@ -1220,41 +1220,41 @@
     </row>
     <row r="30" spans="1:7" x14ac:dyDescent="0.45">
       <c r="A30" s="7">
-        <v>46317</v>
+        <v>46318</v>
       </c>
       <c r="B30" s="8"/>
       <c r="C30" s="20" t="s">
         <v>20</v>
       </c>
       <c r="D30" s="10">
-        <v>258.83</v>
+        <v>259.88</v>
       </c>
       <c r="E30" s="22">
-        <v>228.76</v>
+        <v>227.66</v>
       </c>
       <c r="F30" s="22">
-        <v>238.76</v>
+        <v>237.66</v>
       </c>
       <c r="G30" s="22">
-        <v>224.6</v>
+        <v>223.5</v>
       </c>
     </row>
     <row r="31" spans="1:7" x14ac:dyDescent="0.45">
       <c r="A31" s="11">
-        <v>46317</v>
+        <v>46318</v>
       </c>
       <c r="B31" s="12"/>
       <c r="C31" s="12" t="s">
         <v>21</v>
       </c>
       <c r="D31" s="13">
-        <v>260.37</v>
+        <v>261.39999999999998</v>
       </c>
       <c r="E31" s="13">
-        <v>230.18</v>
+        <v>229.07</v>
       </c>
       <c r="F31" s="13">
-        <v>240.18</v>
+        <v>239.07</v>
       </c>
       <c r="G31" s="13" t="s">
         <v>18</v>
@@ -1301,52 +1301,52 @@
     </row>
     <row r="35" spans="1:7" x14ac:dyDescent="0.45">
       <c r="A35" s="7">
-        <v>46318</v>
+        <v>46319</v>
       </c>
       <c r="B35" s="8"/>
       <c r="C35" s="20" t="s">
         <v>23</v>
       </c>
       <c r="D35" s="10">
-        <v>256.47000000000003</v>
+        <v>257.58999999999997</v>
       </c>
       <c r="E35" s="10">
-        <v>218.83</v>
+        <v>218.63</v>
       </c>
       <c r="F35" s="10">
-        <v>227.83</v>
+        <v>227.63</v>
       </c>
       <c r="G35" s="17"/>
     </row>
     <row r="36" spans="1:7" x14ac:dyDescent="0.45">
       <c r="A36" s="11">
-        <v>46317</v>
+        <v>46318</v>
       </c>
       <c r="B36" s="12"/>
       <c r="C36" s="12" t="s">
         <v>23</v>
       </c>
       <c r="D36" s="13">
-        <v>255.42</v>
+        <v>256.47000000000003</v>
       </c>
       <c r="E36" s="13">
-        <v>219.96</v>
+        <v>218.83</v>
       </c>
       <c r="F36" s="13">
-        <v>228.96</v>
+        <v>227.83</v>
       </c>
       <c r="G36" s="17"/>
     </row>
     <row r="37" spans="1:7" x14ac:dyDescent="0.45">
       <c r="A37" s="7">
-        <v>46318</v>
+        <v>46319</v>
       </c>
       <c r="B37" s="8"/>
       <c r="C37" s="20" t="s">
         <v>24</v>
       </c>
       <c r="D37" s="10">
-        <v>272.08999999999997</v>
+        <v>273.20999999999998</v>
       </c>
       <c r="E37" s="10" t="s">
         <v>18</v>
@@ -1358,14 +1358,14 @@
     </row>
     <row r="38" spans="1:7" x14ac:dyDescent="0.45">
       <c r="A38" s="11">
-        <v>46317</v>
+        <v>46318</v>
       </c>
       <c r="B38" s="12"/>
       <c r="C38" s="12" t="s">
         <v>24</v>
       </c>
       <c r="D38" s="13">
-        <v>271.04000000000002</v>
+        <v>272.08999999999997</v>
       </c>
       <c r="E38" s="13" t="s">
         <v>18</v>
@@ -1416,77 +1416,77 @@
     </row>
     <row r="42" spans="1:7" x14ac:dyDescent="0.45">
       <c r="A42" s="7">
-        <v>46318</v>
+        <v>46319</v>
       </c>
       <c r="B42" s="8"/>
       <c r="C42" s="20" t="s">
         <v>26</v>
       </c>
       <c r="D42" s="10">
-        <v>266.58</v>
+        <v>267.73</v>
       </c>
       <c r="E42" s="10">
-        <v>229.81</v>
+        <v>229.86</v>
       </c>
       <c r="F42" s="10">
-        <v>239.81</v>
+        <v>239.86</v>
       </c>
       <c r="G42" s="17"/>
     </row>
     <row r="43" spans="1:7" x14ac:dyDescent="0.45">
       <c r="A43" s="11">
-        <v>46318</v>
+        <v>46319</v>
       </c>
       <c r="B43" s="12"/>
       <c r="C43" s="21" t="s">
         <v>27</v>
       </c>
       <c r="D43" s="13">
-        <v>266.18</v>
+        <v>267.33999999999997</v>
       </c>
       <c r="E43" s="13">
-        <v>230.23</v>
+        <v>230.27</v>
       </c>
       <c r="F43" s="13">
-        <v>240.23</v>
+        <v>240.27</v>
       </c>
       <c r="G43" s="17"/>
     </row>
     <row r="44" spans="1:7" x14ac:dyDescent="0.45">
       <c r="A44" s="7">
-        <v>46317</v>
+        <v>46318</v>
       </c>
       <c r="B44" s="8"/>
       <c r="C44" s="20" t="s">
         <v>26</v>
       </c>
       <c r="D44" s="10">
-        <v>265.45999999999998</v>
+        <v>266.58</v>
       </c>
       <c r="E44" s="10">
-        <v>230.66</v>
+        <v>229.81</v>
       </c>
       <c r="F44" s="10">
-        <v>240.66</v>
+        <v>239.81</v>
       </c>
       <c r="G44" s="17"/>
     </row>
     <row r="45" spans="1:7" x14ac:dyDescent="0.45">
       <c r="A45" s="11">
-        <v>46317</v>
+        <v>46318</v>
       </c>
       <c r="B45" s="12"/>
       <c r="C45" s="21" t="s">
         <v>27</v>
       </c>
       <c r="D45" s="13">
-        <v>265.07</v>
+        <v>266.18</v>
       </c>
       <c r="E45" s="13">
-        <v>231.07</v>
+        <v>230.23</v>
       </c>
       <c r="F45" s="13">
-        <v>241.07</v>
+        <v>240.23</v>
       </c>
       <c r="G45" s="17"/>
     </row>
@@ -1531,77 +1531,77 @@
     </row>
     <row r="49" spans="1:7" x14ac:dyDescent="0.45">
       <c r="A49" s="7">
-        <v>46318</v>
+        <v>46319</v>
       </c>
       <c r="B49" s="8"/>
       <c r="C49" s="20" t="s">
         <v>29</v>
       </c>
       <c r="D49" s="10">
-        <v>259.07</v>
+        <v>259.70999999999998</v>
       </c>
       <c r="E49" s="10">
-        <v>222.05</v>
+        <v>221.08</v>
       </c>
       <c r="F49" s="10">
-        <v>232.05</v>
+        <v>231.08</v>
       </c>
       <c r="G49" s="28"/>
     </row>
     <row r="50" spans="1:7" x14ac:dyDescent="0.45">
       <c r="A50" s="11">
-        <v>46318</v>
+        <v>46319</v>
       </c>
       <c r="B50" s="12"/>
       <c r="C50" s="21" t="s">
         <v>30</v>
       </c>
       <c r="D50" s="13">
-        <v>256.57</v>
+        <v>257.22000000000003</v>
       </c>
       <c r="E50" s="13">
-        <v>221.64</v>
+        <v>220.67</v>
       </c>
       <c r="F50" s="13">
-        <v>231.64</v>
+        <v>230.67</v>
       </c>
       <c r="G50" s="28"/>
     </row>
     <row r="51" spans="1:7" x14ac:dyDescent="0.45">
       <c r="A51" s="7">
-        <v>46317</v>
+        <v>46318</v>
       </c>
       <c r="B51" s="8"/>
       <c r="C51" s="20" t="s">
         <v>29</v>
       </c>
       <c r="D51" s="10">
-        <v>256.92</v>
+        <v>259.07</v>
       </c>
       <c r="E51" s="10">
-        <v>223.9</v>
+        <v>222.05</v>
       </c>
       <c r="F51" s="10">
-        <v>233.9</v>
+        <v>232.05</v>
       </c>
       <c r="G51" s="17"/>
     </row>
     <row r="52" spans="1:7" x14ac:dyDescent="0.45">
       <c r="A52" s="11">
-        <v>46317</v>
+        <v>46318</v>
       </c>
       <c r="B52" s="12"/>
       <c r="C52" s="21" t="s">
         <v>30</v>
       </c>
       <c r="D52" s="13">
-        <v>254.43</v>
+        <v>256.57</v>
       </c>
       <c r="E52" s="13">
-        <v>223.49</v>
+        <v>221.64</v>
       </c>
       <c r="F52" s="13">
-        <v>233.49</v>
+        <v>231.64</v>
       </c>
       <c r="G52" s="17"/>
     </row>
@@ -1646,52 +1646,52 @@
     </row>
     <row r="56" spans="1:7" x14ac:dyDescent="0.45">
       <c r="A56" s="7">
-        <v>46318</v>
+        <v>46319</v>
       </c>
       <c r="B56" s="8"/>
       <c r="C56" s="20" t="s">
         <v>32</v>
       </c>
       <c r="D56" s="10">
-        <v>272.56</v>
+        <v>273.66000000000003</v>
       </c>
       <c r="E56" s="10">
-        <v>247.07</v>
+        <v>247.06</v>
       </c>
       <c r="F56" s="10">
-        <v>257.07</v>
+        <v>257.06</v>
       </c>
       <c r="G56" s="17"/>
     </row>
     <row r="57" spans="1:7" x14ac:dyDescent="0.45">
       <c r="A57" s="11">
-        <v>46318</v>
+        <v>46319</v>
       </c>
       <c r="B57" s="12"/>
       <c r="C57" s="21" t="s">
         <v>33</v>
       </c>
       <c r="D57" s="13">
-        <v>260.02</v>
+        <v>261.14</v>
       </c>
       <c r="E57" s="13">
-        <v>227.94</v>
+        <v>227.68</v>
       </c>
       <c r="F57" s="13">
-        <v>237.94</v>
+        <v>237.68</v>
       </c>
       <c r="G57" s="17"/>
     </row>
     <row r="58" spans="1:7" x14ac:dyDescent="0.45">
       <c r="A58" s="7">
-        <v>46318</v>
+        <v>46319</v>
       </c>
       <c r="B58" s="8"/>
       <c r="C58" s="20" t="s">
         <v>34</v>
       </c>
       <c r="D58" s="10">
-        <v>260.82</v>
+        <v>261.95</v>
       </c>
       <c r="E58" s="10" t="s">
         <v>18</v>
@@ -1703,17 +1703,17 @@
     </row>
     <row r="59" spans="1:7" x14ac:dyDescent="0.45">
       <c r="A59" s="11">
-        <v>46318</v>
+        <v>46319</v>
       </c>
       <c r="B59" s="12"/>
       <c r="C59" s="21" t="s">
         <v>35</v>
       </c>
       <c r="D59" s="13">
-        <v>256.89999999999998</v>
+        <v>257.97000000000003</v>
       </c>
       <c r="E59" s="13">
-        <v>222.32</v>
+        <v>222.07</v>
       </c>
       <c r="F59" s="13" t="s">
         <v>18</v>
@@ -1722,36 +1722,36 @@
     </row>
     <row r="60" spans="1:7" x14ac:dyDescent="0.45">
       <c r="A60" s="7">
-        <v>46318</v>
+        <v>46319</v>
       </c>
       <c r="B60" s="8"/>
       <c r="C60" s="20" t="s">
         <v>36</v>
       </c>
       <c r="D60" s="10">
-        <v>252.73</v>
+        <v>253.8</v>
       </c>
       <c r="E60" s="10">
-        <v>218.26</v>
+        <v>218</v>
       </c>
       <c r="F60" s="10">
-        <v>228.26</v>
+        <v>228</v>
       </c>
       <c r="G60" s="17"/>
     </row>
     <row r="61" spans="1:7" x14ac:dyDescent="0.45">
       <c r="A61" s="11">
-        <v>46318</v>
+        <v>46319</v>
       </c>
       <c r="B61" s="12"/>
       <c r="C61" s="21" t="s">
         <v>37</v>
       </c>
       <c r="D61" s="13">
-        <v>260.32</v>
+        <v>261.39</v>
       </c>
       <c r="E61" s="13">
-        <v>240.17</v>
+        <v>240.07</v>
       </c>
       <c r="F61" s="13" t="s">
         <v>18</v>
@@ -1760,52 +1760,52 @@
     </row>
     <row r="62" spans="1:7" x14ac:dyDescent="0.45">
       <c r="A62" s="7">
-        <v>46317</v>
+        <v>46318</v>
       </c>
       <c r="B62" s="8"/>
       <c r="C62" s="20" t="s">
         <v>32</v>
       </c>
       <c r="D62" s="10">
-        <v>271.54000000000002</v>
+        <v>272.56</v>
       </c>
       <c r="E62" s="10">
-        <v>247.85</v>
+        <v>247.07</v>
       </c>
       <c r="F62" s="10">
-        <v>257.85000000000002</v>
+        <v>257.07</v>
       </c>
       <c r="G62" s="17"/>
     </row>
     <row r="63" spans="1:7" x14ac:dyDescent="0.45">
       <c r="A63" s="11">
-        <v>46317</v>
+        <v>46318</v>
       </c>
       <c r="B63" s="12"/>
       <c r="C63" s="21" t="s">
         <v>33</v>
       </c>
       <c r="D63" s="13">
-        <v>258.42</v>
+        <v>260.02</v>
       </c>
       <c r="E63" s="13">
-        <v>229.16</v>
+        <v>227.94</v>
       </c>
       <c r="F63" s="13">
-        <v>239.16</v>
+        <v>237.94</v>
       </c>
       <c r="G63" s="17"/>
     </row>
     <row r="64" spans="1:7" x14ac:dyDescent="0.45">
       <c r="A64" s="7">
-        <v>46317</v>
+        <v>46318</v>
       </c>
       <c r="B64" s="8"/>
       <c r="C64" s="20" t="s">
         <v>34</v>
       </c>
       <c r="D64" s="10">
-        <v>259.2</v>
+        <v>260.82</v>
       </c>
       <c r="E64" s="10" t="s">
         <v>18</v>
@@ -1817,17 +1817,17 @@
     </row>
     <row r="65" spans="1:6" x14ac:dyDescent="0.45">
       <c r="A65" s="11">
-        <v>46317</v>
+        <v>46318</v>
       </c>
       <c r="B65" s="12"/>
       <c r="C65" s="21" t="s">
         <v>35</v>
       </c>
       <c r="D65" s="13">
-        <v>255.41</v>
+        <v>256.89999999999998</v>
       </c>
       <c r="E65" s="13">
-        <v>223.54</v>
+        <v>222.32</v>
       </c>
       <c r="F65" s="13" t="s">
         <v>18</v>
@@ -1835,35 +1835,35 @@
     </row>
     <row r="66" spans="1:6" x14ac:dyDescent="0.45">
       <c r="A66" s="7">
-        <v>46317</v>
+        <v>46318</v>
       </c>
       <c r="B66" s="8"/>
       <c r="C66" s="20" t="s">
         <v>36</v>
       </c>
       <c r="D66" s="10">
-        <v>251.24</v>
+        <v>252.73</v>
       </c>
       <c r="E66" s="10">
-        <v>219.48</v>
+        <v>218.26</v>
       </c>
       <c r="F66" s="10">
-        <v>229.48</v>
+        <v>228.26</v>
       </c>
     </row>
     <row r="67" spans="1:6" x14ac:dyDescent="0.45">
       <c r="A67" s="11">
-        <v>46317</v>
+        <v>46318</v>
       </c>
       <c r="B67" s="12"/>
       <c r="C67" s="21" t="s">
         <v>37</v>
       </c>
       <c r="D67" s="13">
-        <v>259.37</v>
+        <v>260.32</v>
       </c>
       <c r="E67" s="13">
-        <v>241.11</v>
+        <v>240.17</v>
       </c>
       <c r="F67" s="13" t="s">
         <v>18</v>
@@ -1891,26 +1891,6 @@
 </file>
 
 <file path=customXml/item1.xml><?xml version="1.0" encoding="utf-8"?>
-<?mso-contentType ?>
-<FormTemplates xmlns="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms">
-  <Display>DocumentLibraryForm</Display>
-  <Edit>DocumentLibraryForm</Edit>
-  <New>DocumentLibraryForm</New>
-</FormTemplates>
-</file>
-
-<file path=customXml/item2.xml><?xml version="1.0" encoding="utf-8"?>
-<p:properties xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls">
-  <documentManagement>
-    <lcf76f155ced4ddcb4097134ff3c332f xmlns="87276d81-85f4-4ef2-9e6e-55066304288f">
-      <Terms xmlns="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
-    </lcf76f155ced4ddcb4097134ff3c332f>
-    <TaxCatchAll xmlns="b23b8984-eafa-4e79-985e-54f52f3da58e" xsi:nil="true"/>
-  </documentManagement>
-</p:properties>
-</file>
-
-<file path=customXml/item3.xml><?xml version="1.0" encoding="utf-8"?>
 <ct:contentTypeSchema xmlns:ct="http://schemas.microsoft.com/office/2006/metadata/contentType" xmlns:ma="http://schemas.microsoft.com/office/2006/metadata/properties/metaAttributes" ct:_="" ma:_="" ma:contentTypeName="Document" ma:contentTypeID="0x010100D3632DF5622958439304627C030B0427" ma:contentTypeVersion="18" ma:contentTypeDescription="Create a new document." ma:contentTypeScope="" ma:versionID="8c2ecbce386d6bac497f8eb2d8f0fb7a">
   <xsd:schema xmlns:xsd="http://www.w3.org/2001/XMLSchema" xmlns:xs="http://www.w3.org/2001/XMLSchema" xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:ns2="87276d81-85f4-4ef2-9e6e-55066304288f" xmlns:ns3="39e1dda6-d1d8-4c88-a3b9-f1abc1284bad" xmlns:ns4="b23b8984-eafa-4e79-985e-54f52f3da58e" targetNamespace="http://schemas.microsoft.com/office/2006/metadata/properties" ma:root="true" ma:fieldsID="4cfd0c2f651c1ce156ad4fcb44ea61dd" ns2:_="" ns3:_="" ns4:_="">
     <xsd:import namespace="87276d81-85f4-4ef2-9e6e-55066304288f"/>
@@ -2170,26 +2150,27 @@
 </ct:contentTypeSchema>
 </file>
 
-<file path=customXml/itemProps1.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{F60519E9-FD90-4339-869C-BC2F85719BB8}">
-  <ds:schemaRefs>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms"/>
-  </ds:schemaRefs>
-</ds:datastoreItem>
+<file path=customXml/item2.xml><?xml version="1.0" encoding="utf-8"?>
+<p:properties xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls">
+  <documentManagement>
+    <lcf76f155ced4ddcb4097134ff3c332f xmlns="87276d81-85f4-4ef2-9e6e-55066304288f">
+      <Terms xmlns="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
+    </lcf76f155ced4ddcb4097134ff3c332f>
+    <TaxCatchAll xmlns="b23b8984-eafa-4e79-985e-54f52f3da58e" xsi:nil="true"/>
+  </documentManagement>
+</p:properties>
 </file>
 
-<file path=customXml/itemProps2.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{57A83D98-2BAE-4D83-823A-D31C464B620C}">
-  <ds:schemaRefs>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/properties"/>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
-    <ds:schemaRef ds:uri="87276d81-85f4-4ef2-9e6e-55066304288f"/>
-    <ds:schemaRef ds:uri="b23b8984-eafa-4e79-985e-54f52f3da58e"/>
-  </ds:schemaRefs>
-</ds:datastoreItem>
+<file path=customXml/item3.xml><?xml version="1.0" encoding="utf-8"?>
+<?mso-contentType ?>
+<FormTemplates xmlns="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms">
+  <Display>DocumentLibraryForm</Display>
+  <Edit>DocumentLibraryForm</Edit>
+  <New>DocumentLibraryForm</New>
+</FormTemplates>
 </file>
 
-<file path=customXml/itemProps3.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=customXml/itemProps1.xml><?xml version="1.0" encoding="utf-8"?>
 <ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{B44E1863-2778-41F9-ACBA-48420F931671}">
   <ds:schemaRefs>
     <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/contentType"/>
@@ -2209,6 +2190,25 @@
 </ds:datastoreItem>
 </file>
 
+<file path=customXml/itemProps2.xml><?xml version="1.0" encoding="utf-8"?>
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{57A83D98-2BAE-4D83-823A-D31C464B620C}">
+  <ds:schemaRefs>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/properties"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
+    <ds:schemaRef ds:uri="87276d81-85f4-4ef2-9e6e-55066304288f"/>
+    <ds:schemaRef ds:uri="b23b8984-eafa-4e79-985e-54f52f3da58e"/>
+  </ds:schemaRefs>
+</ds:datastoreItem>
+</file>
+
+<file path=customXml/itemProps3.xml><?xml version="1.0" encoding="utf-8"?>
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{F60519E9-FD90-4339-869C-BC2F85719BB8}">
+  <ds:schemaRefs>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms"/>
+  </ds:schemaRefs>
+</ds:datastoreItem>
+</file>
+
 <file path=docMetadata/LabelInfo.xml><?xml version="1.0" encoding="utf-8"?>
 <clbl:labelList xmlns:clbl="http://schemas.microsoft.com/office/2020/mipLabelMetadata">
   <clbl:label id="{569bf4a9-87bd-4dbf-a36c-1db5158e5def}" enabled="1" method="Privileged" siteId="{ea80952e-a476-42d4-aaf4-5457852b0f7e}" removed="0"/>

</xml_diff>

<commit_message>
Mon Oct 26 06:27:24 UTC 2026
</commit_message>
<xml_diff>
--- a/bp.com-content-dam-bp-country-sites-en_au-australia-home-products-services-pricing-tgp-excel.xlsx
+++ b/bp.com-content-dam-bp-country-sites-en_au-australia-home-products-services-pricing-tgp-excel.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://bp365.sharepoint.com/sites/WholesalePricing/Shared Documents/B2C/TGP/Daily TGP/Web TGP/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="14_{76438D39-9C43-4744-BBD8-0A9721CE037B}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="14_{3C6520ED-30A3-48D8-AA5C-460CA0D78066}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="20715" yWindow="-16320" windowWidth="29040" windowHeight="15720" xr2:uid="{1B412EEF-F96D-4DF4-A4E9-C7F0F183C2FB}"/>
+    <workbookView xWindow="20205" yWindow="-16320" windowWidth="29040" windowHeight="15720" xr2:uid="{1B412EEF-F96D-4DF4-A4E9-C7F0F183C2FB}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
@@ -808,128 +808,128 @@
     </row>
     <row r="8" spans="1:7" x14ac:dyDescent="0.45">
       <c r="A8" s="7">
-        <v>46319</v>
+        <v>46322</v>
       </c>
       <c r="B8" s="8"/>
       <c r="C8" s="9" t="s">
         <v>10</v>
       </c>
       <c r="D8" s="10">
-        <v>261.57</v>
+        <v>261.82</v>
       </c>
       <c r="E8" s="10">
-        <v>218.41</v>
+        <v>219.05</v>
       </c>
       <c r="F8" s="10">
-        <v>228.41</v>
+        <v>229.05</v>
       </c>
       <c r="G8" s="10">
-        <v>216.03</v>
+        <v>216.67</v>
       </c>
     </row>
     <row r="9" spans="1:7" x14ac:dyDescent="0.45">
       <c r="A9" s="11">
-        <v>46319</v>
+        <v>46322</v>
       </c>
       <c r="B9" s="12"/>
       <c r="C9" s="12" t="s">
         <v>11</v>
       </c>
       <c r="D9" s="13">
-        <v>261.57</v>
+        <v>261.82</v>
       </c>
       <c r="E9" s="13">
-        <v>218.41</v>
+        <v>219.05</v>
       </c>
       <c r="F9" s="13">
-        <v>228.41</v>
+        <v>229.05</v>
       </c>
       <c r="G9" s="13">
-        <v>216.03</v>
+        <v>216.67</v>
       </c>
     </row>
     <row r="10" spans="1:7" x14ac:dyDescent="0.45">
       <c r="A10" s="7">
-        <v>46319</v>
+        <v>46322</v>
       </c>
       <c r="B10" s="8"/>
       <c r="C10" s="9" t="s">
         <v>12</v>
       </c>
       <c r="D10" s="10">
-        <v>259.04000000000002</v>
+        <v>261.10000000000002</v>
       </c>
       <c r="E10" s="10">
-        <v>219.66</v>
+        <v>221.05</v>
       </c>
       <c r="F10" s="10">
-        <v>229.66</v>
+        <v>231.05</v>
       </c>
       <c r="G10" s="10">
-        <v>218.07</v>
+        <v>219.46</v>
       </c>
     </row>
     <row r="11" spans="1:7" x14ac:dyDescent="0.45">
       <c r="A11" s="11">
-        <v>46318</v>
+        <v>46319</v>
       </c>
       <c r="B11" s="12"/>
       <c r="C11" s="12" t="s">
         <v>10</v>
       </c>
       <c r="D11" s="13">
-        <v>260.27999999999997</v>
+        <v>261.57</v>
       </c>
       <c r="E11" s="13">
-        <v>219.56</v>
+        <v>218.41</v>
       </c>
       <c r="F11" s="13">
-        <v>229.56</v>
+        <v>228.41</v>
       </c>
       <c r="G11" s="13">
-        <v>217.18</v>
+        <v>216.03</v>
       </c>
     </row>
     <row r="12" spans="1:7" x14ac:dyDescent="0.45">
       <c r="A12" s="7">
-        <v>46318</v>
+        <v>46319</v>
       </c>
       <c r="B12" s="8"/>
       <c r="C12" s="9" t="s">
         <v>11</v>
       </c>
       <c r="D12" s="10">
-        <v>260.27999999999997</v>
+        <v>261.57</v>
       </c>
       <c r="E12" s="10">
-        <v>219.56</v>
+        <v>218.41</v>
       </c>
       <c r="F12" s="10">
-        <v>229.56</v>
+        <v>228.41</v>
       </c>
       <c r="G12" s="10">
-        <v>217.18</v>
+        <v>216.03</v>
       </c>
     </row>
     <row r="13" spans="1:7" x14ac:dyDescent="0.45">
       <c r="A13" s="11">
-        <v>46318</v>
+        <v>46319</v>
       </c>
       <c r="B13" s="12"/>
       <c r="C13" s="12" t="s">
         <v>12</v>
       </c>
       <c r="D13" s="13">
-        <v>257.92</v>
+        <v>259.04000000000002</v>
       </c>
       <c r="E13" s="13">
-        <v>219.87</v>
+        <v>219.66</v>
       </c>
       <c r="F13" s="13">
-        <v>229.87</v>
+        <v>229.66</v>
       </c>
       <c r="G13" s="13">
-        <v>218.27</v>
+        <v>218.07</v>
       </c>
     </row>
     <row r="14" spans="1:7" x14ac:dyDescent="0.45">
@@ -973,39 +973,39 @@
     </row>
     <row r="17" spans="1:7" x14ac:dyDescent="0.45">
       <c r="A17" s="7">
-        <v>46319</v>
+        <v>46322</v>
       </c>
       <c r="B17" s="8"/>
       <c r="C17" s="20" t="s">
         <v>14</v>
       </c>
       <c r="D17" s="10">
-        <v>262.33</v>
+        <v>264.39999999999998</v>
       </c>
       <c r="E17" s="10">
-        <v>222.45</v>
+        <v>223.85</v>
       </c>
       <c r="F17" s="10">
-        <v>232.45</v>
+        <v>233.85</v>
       </c>
       <c r="G17" s="17"/>
     </row>
     <row r="18" spans="1:7" x14ac:dyDescent="0.45">
       <c r="A18" s="11">
-        <v>46318</v>
+        <v>46319</v>
       </c>
       <c r="B18" s="12"/>
       <c r="C18" s="12" t="s">
         <v>14</v>
       </c>
       <c r="D18" s="13">
-        <v>261.25</v>
+        <v>262.33</v>
       </c>
       <c r="E18" s="13">
-        <v>222.69</v>
+        <v>222.45</v>
       </c>
       <c r="F18" s="13">
-        <v>232.69</v>
+        <v>232.45</v>
       </c>
       <c r="G18" s="17"/>
     </row>
@@ -1052,41 +1052,41 @@
     </row>
     <row r="22" spans="1:7" x14ac:dyDescent="0.45">
       <c r="A22" s="7">
-        <v>46319</v>
+        <v>46322</v>
       </c>
       <c r="B22" s="8"/>
       <c r="C22" s="20" t="s">
         <v>16</v>
       </c>
       <c r="D22" s="10">
-        <v>262.69</v>
+        <v>262.94</v>
       </c>
       <c r="E22" s="10">
-        <v>218.56</v>
+        <v>218.64</v>
       </c>
       <c r="F22" s="10">
-        <v>228.16</v>
+        <v>228.24</v>
       </c>
       <c r="G22" s="10">
-        <v>214.93</v>
+        <v>215.01</v>
       </c>
     </row>
     <row r="23" spans="1:7" x14ac:dyDescent="0.45">
       <c r="A23" s="11">
-        <v>46319</v>
+        <v>46322</v>
       </c>
       <c r="B23" s="12"/>
       <c r="C23" s="21" t="s">
         <v>17</v>
       </c>
       <c r="D23" s="13">
-        <v>264.01</v>
+        <v>266.07</v>
       </c>
       <c r="E23" s="13">
-        <v>227.98</v>
+        <v>229.37</v>
       </c>
       <c r="F23" s="13">
-        <v>237.98</v>
+        <v>239.37</v>
       </c>
       <c r="G23" s="13" t="s">
         <v>18</v>
@@ -1094,20 +1094,20 @@
     </row>
     <row r="24" spans="1:7" x14ac:dyDescent="0.45">
       <c r="A24" s="7">
-        <v>46319</v>
+        <v>46322</v>
       </c>
       <c r="B24" s="8"/>
       <c r="C24" s="20" t="s">
         <v>19</v>
       </c>
       <c r="D24" s="10">
-        <v>264.33999999999997</v>
+        <v>266.39999999999998</v>
       </c>
       <c r="E24" s="10">
-        <v>227.25</v>
+        <v>228.64</v>
       </c>
       <c r="F24" s="10">
-        <v>237.25</v>
+        <v>238.64</v>
       </c>
       <c r="G24" s="10" t="s">
         <v>18</v>
@@ -1115,41 +1115,41 @@
     </row>
     <row r="25" spans="1:7" x14ac:dyDescent="0.45">
       <c r="A25" s="11">
-        <v>46319</v>
+        <v>46322</v>
       </c>
       <c r="B25" s="12"/>
       <c r="C25" s="21" t="s">
         <v>20</v>
       </c>
       <c r="D25" s="13">
-        <v>261.01</v>
+        <v>263.08</v>
       </c>
       <c r="E25" s="13">
-        <v>227.47</v>
+        <v>228.86</v>
       </c>
       <c r="F25" s="13">
-        <v>237.47</v>
+        <v>238.86</v>
       </c>
       <c r="G25" s="13">
-        <v>223.31</v>
+        <v>224.7</v>
       </c>
     </row>
     <row r="26" spans="1:7" x14ac:dyDescent="0.45">
       <c r="A26" s="7">
-        <v>46319</v>
+        <v>46322</v>
       </c>
       <c r="B26" s="8"/>
       <c r="C26" s="20" t="s">
         <v>21</v>
       </c>
       <c r="D26" s="10">
-        <v>262.5</v>
+        <v>264.57</v>
       </c>
       <c r="E26" s="10">
-        <v>228.88</v>
+        <v>230.28</v>
       </c>
       <c r="F26" s="10">
-        <v>238.88</v>
+        <v>240.28</v>
       </c>
       <c r="G26" s="10" t="s">
         <v>18</v>
@@ -1157,41 +1157,41 @@
     </row>
     <row r="27" spans="1:7" x14ac:dyDescent="0.45">
       <c r="A27" s="11">
-        <v>46318</v>
+        <v>46319</v>
       </c>
       <c r="B27" s="12"/>
       <c r="C27" s="12" t="s">
         <v>16</v>
       </c>
       <c r="D27" s="13">
-        <v>261.39999999999998</v>
+        <v>262.69</v>
       </c>
       <c r="E27" s="13">
-        <v>219.7</v>
+        <v>218.56</v>
       </c>
       <c r="F27" s="13">
-        <v>229.3</v>
+        <v>228.16</v>
       </c>
       <c r="G27" s="13">
-        <v>216.07</v>
+        <v>214.93</v>
       </c>
     </row>
     <row r="28" spans="1:7" x14ac:dyDescent="0.45">
       <c r="A28" s="7">
-        <v>46318</v>
+        <v>46319</v>
       </c>
       <c r="B28" s="8"/>
       <c r="C28" s="20" t="s">
         <v>17</v>
       </c>
       <c r="D28" s="10">
-        <v>262.89</v>
+        <v>264.01</v>
       </c>
       <c r="E28" s="22">
-        <v>228.17</v>
+        <v>227.98</v>
       </c>
       <c r="F28" s="22">
-        <v>238.17</v>
+        <v>237.98</v>
       </c>
       <c r="G28" s="22" t="s">
         <v>18</v>
@@ -1199,20 +1199,20 @@
     </row>
     <row r="29" spans="1:7" x14ac:dyDescent="0.45">
       <c r="A29" s="11">
-        <v>46318</v>
+        <v>46319</v>
       </c>
       <c r="B29" s="12"/>
       <c r="C29" s="12" t="s">
         <v>19</v>
       </c>
       <c r="D29" s="13">
-        <v>263.22000000000003</v>
+        <v>264.33999999999997</v>
       </c>
       <c r="E29" s="13">
-        <v>227.44</v>
+        <v>227.25</v>
       </c>
       <c r="F29" s="13">
-        <v>237.44</v>
+        <v>237.25</v>
       </c>
       <c r="G29" s="13" t="s">
         <v>18</v>
@@ -1220,41 +1220,41 @@
     </row>
     <row r="30" spans="1:7" x14ac:dyDescent="0.45">
       <c r="A30" s="7">
-        <v>46318</v>
+        <v>46319</v>
       </c>
       <c r="B30" s="8"/>
       <c r="C30" s="20" t="s">
         <v>20</v>
       </c>
       <c r="D30" s="10">
-        <v>259.88</v>
+        <v>261.01</v>
       </c>
       <c r="E30" s="22">
-        <v>227.66</v>
+        <v>227.47</v>
       </c>
       <c r="F30" s="22">
-        <v>237.66</v>
+        <v>237.47</v>
       </c>
       <c r="G30" s="22">
-        <v>223.5</v>
+        <v>223.31</v>
       </c>
     </row>
     <row r="31" spans="1:7" x14ac:dyDescent="0.45">
       <c r="A31" s="11">
-        <v>46318</v>
+        <v>46319</v>
       </c>
       <c r="B31" s="12"/>
       <c r="C31" s="12" t="s">
         <v>21</v>
       </c>
       <c r="D31" s="13">
-        <v>261.39999999999998</v>
+        <v>262.5</v>
       </c>
       <c r="E31" s="13">
-        <v>229.07</v>
+        <v>228.88</v>
       </c>
       <c r="F31" s="13">
-        <v>239.07</v>
+        <v>238.88</v>
       </c>
       <c r="G31" s="13" t="s">
         <v>18</v>
@@ -1301,52 +1301,52 @@
     </row>
     <row r="35" spans="1:7" x14ac:dyDescent="0.45">
       <c r="A35" s="7">
-        <v>46319</v>
+        <v>46322</v>
       </c>
       <c r="B35" s="8"/>
       <c r="C35" s="20" t="s">
         <v>23</v>
       </c>
       <c r="D35" s="10">
-        <v>257.58999999999997</v>
+        <v>259.66000000000003</v>
       </c>
       <c r="E35" s="10">
-        <v>218.63</v>
+        <v>220.02</v>
       </c>
       <c r="F35" s="10">
-        <v>227.63</v>
+        <v>229.02</v>
       </c>
       <c r="G35" s="17"/>
     </row>
     <row r="36" spans="1:7" x14ac:dyDescent="0.45">
       <c r="A36" s="11">
-        <v>46318</v>
+        <v>46319</v>
       </c>
       <c r="B36" s="12"/>
       <c r="C36" s="12" t="s">
         <v>23</v>
       </c>
       <c r="D36" s="13">
-        <v>256.47000000000003</v>
+        <v>257.58999999999997</v>
       </c>
       <c r="E36" s="13">
-        <v>218.83</v>
+        <v>218.63</v>
       </c>
       <c r="F36" s="13">
-        <v>227.83</v>
+        <v>227.63</v>
       </c>
       <c r="G36" s="17"/>
     </row>
     <row r="37" spans="1:7" x14ac:dyDescent="0.45">
       <c r="A37" s="7">
-        <v>46319</v>
+        <v>46322</v>
       </c>
       <c r="B37" s="8"/>
       <c r="C37" s="20" t="s">
         <v>24</v>
       </c>
       <c r="D37" s="10">
-        <v>273.20999999999998</v>
+        <v>275.27999999999997</v>
       </c>
       <c r="E37" s="10" t="s">
         <v>18</v>
@@ -1358,14 +1358,14 @@
     </row>
     <row r="38" spans="1:7" x14ac:dyDescent="0.45">
       <c r="A38" s="11">
-        <v>46318</v>
+        <v>46319</v>
       </c>
       <c r="B38" s="12"/>
       <c r="C38" s="12" t="s">
         <v>24</v>
       </c>
       <c r="D38" s="13">
-        <v>272.08999999999997</v>
+        <v>273.20999999999998</v>
       </c>
       <c r="E38" s="13" t="s">
         <v>18</v>
@@ -1416,77 +1416,77 @@
     </row>
     <row r="42" spans="1:7" x14ac:dyDescent="0.45">
       <c r="A42" s="7">
-        <v>46319</v>
+        <v>46322</v>
       </c>
       <c r="B42" s="8"/>
       <c r="C42" s="20" t="s">
         <v>26</v>
       </c>
       <c r="D42" s="10">
-        <v>267.73</v>
+        <v>269.79000000000002</v>
       </c>
       <c r="E42" s="10">
-        <v>229.86</v>
+        <v>231.2</v>
       </c>
       <c r="F42" s="10">
-        <v>239.86</v>
+        <v>241.2</v>
       </c>
       <c r="G42" s="17"/>
     </row>
     <row r="43" spans="1:7" x14ac:dyDescent="0.45">
       <c r="A43" s="11">
-        <v>46319</v>
+        <v>46322</v>
       </c>
       <c r="B43" s="12"/>
       <c r="C43" s="21" t="s">
         <v>27</v>
       </c>
       <c r="D43" s="13">
-        <v>267.33999999999997</v>
+        <v>269.39</v>
       </c>
       <c r="E43" s="13">
-        <v>230.27</v>
+        <v>231.61</v>
       </c>
       <c r="F43" s="13">
-        <v>240.27</v>
+        <v>241.61</v>
       </c>
       <c r="G43" s="17"/>
     </row>
     <row r="44" spans="1:7" x14ac:dyDescent="0.45">
       <c r="A44" s="7">
-        <v>46318</v>
+        <v>46319</v>
       </c>
       <c r="B44" s="8"/>
       <c r="C44" s="20" t="s">
         <v>26</v>
       </c>
       <c r="D44" s="10">
-        <v>266.58</v>
+        <v>267.73</v>
       </c>
       <c r="E44" s="10">
-        <v>229.81</v>
+        <v>229.86</v>
       </c>
       <c r="F44" s="10">
-        <v>239.81</v>
+        <v>239.86</v>
       </c>
       <c r="G44" s="17"/>
     </row>
     <row r="45" spans="1:7" x14ac:dyDescent="0.45">
       <c r="A45" s="11">
-        <v>46318</v>
+        <v>46319</v>
       </c>
       <c r="B45" s="12"/>
       <c r="C45" s="21" t="s">
         <v>27</v>
       </c>
       <c r="D45" s="13">
-        <v>266.18</v>
+        <v>267.33999999999997</v>
       </c>
       <c r="E45" s="13">
-        <v>230.23</v>
+        <v>230.27</v>
       </c>
       <c r="F45" s="13">
-        <v>240.23</v>
+        <v>240.27</v>
       </c>
       <c r="G45" s="17"/>
     </row>
@@ -1531,77 +1531,77 @@
     </row>
     <row r="49" spans="1:7" x14ac:dyDescent="0.45">
       <c r="A49" s="7">
-        <v>46319</v>
+        <v>46322</v>
       </c>
       <c r="B49" s="8"/>
       <c r="C49" s="20" t="s">
         <v>29</v>
       </c>
       <c r="D49" s="10">
-        <v>259.70999999999998</v>
+        <v>260.60000000000002</v>
       </c>
       <c r="E49" s="10">
-        <v>221.08</v>
+        <v>220.83</v>
       </c>
       <c r="F49" s="10">
-        <v>231.08</v>
+        <v>230.83</v>
       </c>
       <c r="G49" s="28"/>
     </row>
     <row r="50" spans="1:7" x14ac:dyDescent="0.45">
       <c r="A50" s="11">
-        <v>46319</v>
+        <v>46322</v>
       </c>
       <c r="B50" s="12"/>
       <c r="C50" s="21" t="s">
         <v>30</v>
       </c>
       <c r="D50" s="13">
-        <v>257.22000000000003</v>
+        <v>258.08</v>
       </c>
       <c r="E50" s="13">
-        <v>220.67</v>
+        <v>220.41</v>
       </c>
       <c r="F50" s="13">
-        <v>230.67</v>
+        <v>230.41</v>
       </c>
       <c r="G50" s="28"/>
     </row>
     <row r="51" spans="1:7" x14ac:dyDescent="0.45">
       <c r="A51" s="7">
-        <v>46318</v>
+        <v>46319</v>
       </c>
       <c r="B51" s="8"/>
       <c r="C51" s="20" t="s">
         <v>29</v>
       </c>
       <c r="D51" s="10">
-        <v>259.07</v>
+        <v>259.70999999999998</v>
       </c>
       <c r="E51" s="10">
-        <v>222.05</v>
+        <v>221.08</v>
       </c>
       <c r="F51" s="10">
-        <v>232.05</v>
+        <v>231.08</v>
       </c>
       <c r="G51" s="17"/>
     </row>
     <row r="52" spans="1:7" x14ac:dyDescent="0.45">
       <c r="A52" s="11">
-        <v>46318</v>
+        <v>46319</v>
       </c>
       <c r="B52" s="12"/>
       <c r="C52" s="21" t="s">
         <v>30</v>
       </c>
       <c r="D52" s="13">
-        <v>256.57</v>
+        <v>257.22000000000003</v>
       </c>
       <c r="E52" s="13">
-        <v>221.64</v>
+        <v>220.67</v>
       </c>
       <c r="F52" s="13">
-        <v>231.64</v>
+        <v>230.67</v>
       </c>
       <c r="G52" s="17"/>
     </row>
@@ -1646,52 +1646,52 @@
     </row>
     <row r="56" spans="1:7" x14ac:dyDescent="0.45">
       <c r="A56" s="7">
-        <v>46319</v>
+        <v>46322</v>
       </c>
       <c r="B56" s="8"/>
       <c r="C56" s="20" t="s">
         <v>32</v>
       </c>
       <c r="D56" s="10">
-        <v>273.66000000000003</v>
+        <v>275.72000000000003</v>
       </c>
       <c r="E56" s="10">
-        <v>247.06</v>
+        <v>248.42</v>
       </c>
       <c r="F56" s="10">
-        <v>257.06</v>
+        <v>258.42</v>
       </c>
       <c r="G56" s="17"/>
     </row>
     <row r="57" spans="1:7" x14ac:dyDescent="0.45">
       <c r="A57" s="11">
-        <v>46319</v>
+        <v>46322</v>
       </c>
       <c r="B57" s="12"/>
       <c r="C57" s="21" t="s">
         <v>33</v>
       </c>
       <c r="D57" s="13">
-        <v>261.14</v>
+        <v>263.20999999999998</v>
       </c>
       <c r="E57" s="13">
-        <v>227.68</v>
+        <v>229.08</v>
       </c>
       <c r="F57" s="13">
-        <v>237.68</v>
+        <v>239.08</v>
       </c>
       <c r="G57" s="17"/>
     </row>
     <row r="58" spans="1:7" x14ac:dyDescent="0.45">
       <c r="A58" s="7">
-        <v>46319</v>
+        <v>46322</v>
       </c>
       <c r="B58" s="8"/>
       <c r="C58" s="20" t="s">
         <v>34</v>
       </c>
       <c r="D58" s="10">
-        <v>261.95</v>
+        <v>264.01</v>
       </c>
       <c r="E58" s="10" t="s">
         <v>18</v>
@@ -1703,17 +1703,17 @@
     </row>
     <row r="59" spans="1:7" x14ac:dyDescent="0.45">
       <c r="A59" s="11">
-        <v>46319</v>
+        <v>46322</v>
       </c>
       <c r="B59" s="12"/>
       <c r="C59" s="21" t="s">
         <v>35</v>
       </c>
       <c r="D59" s="13">
-        <v>257.97000000000003</v>
+        <v>260.02999999999997</v>
       </c>
       <c r="E59" s="13">
-        <v>222.07</v>
+        <v>223.46</v>
       </c>
       <c r="F59" s="13" t="s">
         <v>18</v>
@@ -1722,36 +1722,36 @@
     </row>
     <row r="60" spans="1:7" x14ac:dyDescent="0.45">
       <c r="A60" s="7">
-        <v>46319</v>
+        <v>46322</v>
       </c>
       <c r="B60" s="8"/>
       <c r="C60" s="20" t="s">
         <v>36</v>
       </c>
       <c r="D60" s="10">
-        <v>253.8</v>
+        <v>255.86</v>
       </c>
       <c r="E60" s="10">
-        <v>218</v>
+        <v>219.4</v>
       </c>
       <c r="F60" s="10">
-        <v>228</v>
+        <v>229.4</v>
       </c>
       <c r="G60" s="17"/>
     </row>
     <row r="61" spans="1:7" x14ac:dyDescent="0.45">
       <c r="A61" s="11">
-        <v>46319</v>
+        <v>46322</v>
       </c>
       <c r="B61" s="12"/>
       <c r="C61" s="21" t="s">
         <v>37</v>
       </c>
       <c r="D61" s="13">
-        <v>261.39</v>
+        <v>263.47000000000003</v>
       </c>
       <c r="E61" s="13">
-        <v>240.07</v>
+        <v>241.44</v>
       </c>
       <c r="F61" s="13" t="s">
         <v>18</v>
@@ -1760,52 +1760,52 @@
     </row>
     <row r="62" spans="1:7" x14ac:dyDescent="0.45">
       <c r="A62" s="7">
-        <v>46318</v>
+        <v>46319</v>
       </c>
       <c r="B62" s="8"/>
       <c r="C62" s="20" t="s">
         <v>32</v>
       </c>
       <c r="D62" s="10">
-        <v>272.56</v>
+        <v>273.66000000000003</v>
       </c>
       <c r="E62" s="10">
-        <v>247.07</v>
+        <v>247.06</v>
       </c>
       <c r="F62" s="10">
-        <v>257.07</v>
+        <v>257.06</v>
       </c>
       <c r="G62" s="17"/>
     </row>
     <row r="63" spans="1:7" x14ac:dyDescent="0.45">
       <c r="A63" s="11">
-        <v>46318</v>
+        <v>46319</v>
       </c>
       <c r="B63" s="12"/>
       <c r="C63" s="21" t="s">
         <v>33</v>
       </c>
       <c r="D63" s="13">
-        <v>260.02</v>
+        <v>261.14</v>
       </c>
       <c r="E63" s="13">
-        <v>227.94</v>
+        <v>227.68</v>
       </c>
       <c r="F63" s="13">
-        <v>237.94</v>
+        <v>237.68</v>
       </c>
       <c r="G63" s="17"/>
     </row>
     <row r="64" spans="1:7" x14ac:dyDescent="0.45">
       <c r="A64" s="7">
-        <v>46318</v>
+        <v>46319</v>
       </c>
       <c r="B64" s="8"/>
       <c r="C64" s="20" t="s">
         <v>34</v>
       </c>
       <c r="D64" s="10">
-        <v>260.82</v>
+        <v>261.95</v>
       </c>
       <c r="E64" s="10" t="s">
         <v>18</v>
@@ -1817,17 +1817,17 @@
     </row>
     <row r="65" spans="1:6" x14ac:dyDescent="0.45">
       <c r="A65" s="11">
-        <v>46318</v>
+        <v>46319</v>
       </c>
       <c r="B65" s="12"/>
       <c r="C65" s="21" t="s">
         <v>35</v>
       </c>
       <c r="D65" s="13">
-        <v>256.89999999999998</v>
+        <v>257.97000000000003</v>
       </c>
       <c r="E65" s="13">
-        <v>222.32</v>
+        <v>222.07</v>
       </c>
       <c r="F65" s="13" t="s">
         <v>18</v>
@@ -1835,35 +1835,35 @@
     </row>
     <row r="66" spans="1:6" x14ac:dyDescent="0.45">
       <c r="A66" s="7">
-        <v>46318</v>
+        <v>46319</v>
       </c>
       <c r="B66" s="8"/>
       <c r="C66" s="20" t="s">
         <v>36</v>
       </c>
       <c r="D66" s="10">
-        <v>252.73</v>
+        <v>253.8</v>
       </c>
       <c r="E66" s="10">
-        <v>218.26</v>
+        <v>218</v>
       </c>
       <c r="F66" s="10">
-        <v>228.26</v>
+        <v>228</v>
       </c>
     </row>
     <row r="67" spans="1:6" x14ac:dyDescent="0.45">
       <c r="A67" s="11">
-        <v>46318</v>
+        <v>46319</v>
       </c>
       <c r="B67" s="12"/>
       <c r="C67" s="21" t="s">
         <v>37</v>
       </c>
       <c r="D67" s="13">
-        <v>260.32</v>
+        <v>261.39</v>
       </c>
       <c r="E67" s="13">
-        <v>240.17</v>
+        <v>240.07</v>
       </c>
       <c r="F67" s="13" t="s">
         <v>18</v>
@@ -1891,6 +1891,26 @@
 </file>
 
 <file path=customXml/item1.xml><?xml version="1.0" encoding="utf-8"?>
+<?mso-contentType ?>
+<FormTemplates xmlns="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms">
+  <Display>DocumentLibraryForm</Display>
+  <Edit>DocumentLibraryForm</Edit>
+  <New>DocumentLibraryForm</New>
+</FormTemplates>
+</file>
+
+<file path=customXml/item2.xml><?xml version="1.0" encoding="utf-8"?>
+<p:properties xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls">
+  <documentManagement>
+    <lcf76f155ced4ddcb4097134ff3c332f xmlns="87276d81-85f4-4ef2-9e6e-55066304288f">
+      <Terms xmlns="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
+    </lcf76f155ced4ddcb4097134ff3c332f>
+    <TaxCatchAll xmlns="b23b8984-eafa-4e79-985e-54f52f3da58e" xsi:nil="true"/>
+  </documentManagement>
+</p:properties>
+</file>
+
+<file path=customXml/item3.xml><?xml version="1.0" encoding="utf-8"?>
 <ct:contentTypeSchema xmlns:ct="http://schemas.microsoft.com/office/2006/metadata/contentType" xmlns:ma="http://schemas.microsoft.com/office/2006/metadata/properties/metaAttributes" ct:_="" ma:_="" ma:contentTypeName="Document" ma:contentTypeID="0x010100D3632DF5622958439304627C030B0427" ma:contentTypeVersion="18" ma:contentTypeDescription="Create a new document." ma:contentTypeScope="" ma:versionID="8c2ecbce386d6bac497f8eb2d8f0fb7a">
   <xsd:schema xmlns:xsd="http://www.w3.org/2001/XMLSchema" xmlns:xs="http://www.w3.org/2001/XMLSchema" xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:ns2="87276d81-85f4-4ef2-9e6e-55066304288f" xmlns:ns3="39e1dda6-d1d8-4c88-a3b9-f1abc1284bad" xmlns:ns4="b23b8984-eafa-4e79-985e-54f52f3da58e" targetNamespace="http://schemas.microsoft.com/office/2006/metadata/properties" ma:root="true" ma:fieldsID="4cfd0c2f651c1ce156ad4fcb44ea61dd" ns2:_="" ns3:_="" ns4:_="">
     <xsd:import namespace="87276d81-85f4-4ef2-9e6e-55066304288f"/>
@@ -2150,27 +2170,26 @@
 </ct:contentTypeSchema>
 </file>
 
-<file path=customXml/item2.xml><?xml version="1.0" encoding="utf-8"?>
-<p:properties xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls">
-  <documentManagement>
-    <lcf76f155ced4ddcb4097134ff3c332f xmlns="87276d81-85f4-4ef2-9e6e-55066304288f">
-      <Terms xmlns="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
-    </lcf76f155ced4ddcb4097134ff3c332f>
-    <TaxCatchAll xmlns="b23b8984-eafa-4e79-985e-54f52f3da58e" xsi:nil="true"/>
-  </documentManagement>
-</p:properties>
+<file path=customXml/itemProps1.xml><?xml version="1.0" encoding="utf-8"?>
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{F60519E9-FD90-4339-869C-BC2F85719BB8}">
+  <ds:schemaRefs>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms"/>
+  </ds:schemaRefs>
+</ds:datastoreItem>
 </file>
 
-<file path=customXml/item3.xml><?xml version="1.0" encoding="utf-8"?>
-<?mso-contentType ?>
-<FormTemplates xmlns="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms">
-  <Display>DocumentLibraryForm</Display>
-  <Edit>DocumentLibraryForm</Edit>
-  <New>DocumentLibraryForm</New>
-</FormTemplates>
+<file path=customXml/itemProps2.xml><?xml version="1.0" encoding="utf-8"?>
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{57A83D98-2BAE-4D83-823A-D31C464B620C}">
+  <ds:schemaRefs>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/properties"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
+    <ds:schemaRef ds:uri="87276d81-85f4-4ef2-9e6e-55066304288f"/>
+    <ds:schemaRef ds:uri="b23b8984-eafa-4e79-985e-54f52f3da58e"/>
+  </ds:schemaRefs>
+</ds:datastoreItem>
 </file>
 
-<file path=customXml/itemProps1.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=customXml/itemProps3.xml><?xml version="1.0" encoding="utf-8"?>
 <ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{B44E1863-2778-41F9-ACBA-48420F931671}">
   <ds:schemaRefs>
     <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/contentType"/>
@@ -2190,25 +2209,6 @@
 </ds:datastoreItem>
 </file>
 
-<file path=customXml/itemProps2.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{57A83D98-2BAE-4D83-823A-D31C464B620C}">
-  <ds:schemaRefs>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/properties"/>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
-    <ds:schemaRef ds:uri="87276d81-85f4-4ef2-9e6e-55066304288f"/>
-    <ds:schemaRef ds:uri="b23b8984-eafa-4e79-985e-54f52f3da58e"/>
-  </ds:schemaRefs>
-</ds:datastoreItem>
-</file>
-
-<file path=customXml/itemProps3.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{F60519E9-FD90-4339-869C-BC2F85719BB8}">
-  <ds:schemaRefs>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms"/>
-  </ds:schemaRefs>
-</ds:datastoreItem>
-</file>
-
 <file path=docMetadata/LabelInfo.xml><?xml version="1.0" encoding="utf-8"?>
 <clbl:labelList xmlns:clbl="http://schemas.microsoft.com/office/2020/mipLabelMetadata">
   <clbl:label id="{569bf4a9-87bd-4dbf-a36c-1db5158e5def}" enabled="1" method="Privileged" siteId="{ea80952e-a476-42d4-aaf4-5457852b0f7e}" removed="0"/>

</xml_diff>

<commit_message>
Tue Oct 27 06:25:46 UTC 2026
</commit_message>
<xml_diff>
--- a/bp.com-content-dam-bp-country-sites-en_au-australia-home-products-services-pricing-tgp-excel.xlsx
+++ b/bp.com-content-dam-bp-country-sites-en_au-australia-home-products-services-pricing-tgp-excel.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://bp365.sharepoint.com/sites/WholesalePricing/Shared Documents/B2C/TGP/Daily TGP/Web TGP/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="14_{3C6520ED-30A3-48D8-AA5C-460CA0D78066}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="14_{EF43C469-EB28-4682-8447-7FF2257DA8E5}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="20205" yWindow="-16320" windowWidth="29040" windowHeight="15720" xr2:uid="{1B412EEF-F96D-4DF4-A4E9-C7F0F183C2FB}"/>
+    <workbookView xWindow="-28920" yWindow="-60" windowWidth="29040" windowHeight="15720" xr2:uid="{1B412EEF-F96D-4DF4-A4E9-C7F0F183C2FB}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
@@ -715,15 +715,15 @@
     <pageSetUpPr fitToPage="1"/>
   </sheetPr>
   <dimension ref="A1:G67"/>
-  <sheetFormatPr defaultRowHeight="14.25" x14ac:dyDescent="0.45"/>
+  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
-    <col min="1" max="1" width="76.46484375" bestFit="1" customWidth="1"/>
-    <col min="2" max="2" width="6.46484375"/>
-    <col min="3" max="3" width="18.19921875" bestFit="1" customWidth="1"/>
-    <col min="4" max="7" width="7.19921875" bestFit="1" customWidth="1"/>
+    <col min="1" max="1" width="76.42578125" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="6.42578125"/>
+    <col min="3" max="3" width="18.140625" bestFit="1" customWidth="1"/>
+    <col min="4" max="7" width="7.140625" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:7" ht="22.15" x14ac:dyDescent="0.45">
+    <row r="1" spans="1:7" ht="23.25" x14ac:dyDescent="0.25">
       <c r="A1" s="30" t="s">
         <v>0</v>
       </c>
@@ -734,7 +734,7 @@
       <c r="F1" s="2"/>
       <c r="G1" s="2"/>
     </row>
-    <row r="2" spans="1:7" x14ac:dyDescent="0.45">
+    <row r="2" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A2" s="3"/>
       <c r="B2" s="1"/>
       <c r="C2" s="1"/>
@@ -743,7 +743,7 @@
       <c r="F2" s="2"/>
       <c r="G2" s="2"/>
     </row>
-    <row r="3" spans="1:7" x14ac:dyDescent="0.45">
+    <row r="3" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A3" s="3" t="s">
         <v>1</v>
       </c>
@@ -754,7 +754,7 @@
       <c r="F3" s="2"/>
       <c r="G3" s="2"/>
     </row>
-    <row r="4" spans="1:7" x14ac:dyDescent="0.45">
+    <row r="4" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A4" s="3" t="s">
         <v>2</v>
       </c>
@@ -765,7 +765,7 @@
       <c r="F4" s="2"/>
       <c r="G4" s="2"/>
     </row>
-    <row r="5" spans="1:7" x14ac:dyDescent="0.45">
+    <row r="5" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A5" s="3"/>
       <c r="B5" s="3"/>
       <c r="C5" s="1"/>
@@ -774,7 +774,7 @@
       <c r="F5" s="2"/>
       <c r="G5" s="2"/>
     </row>
-    <row r="6" spans="1:7" ht="20.25" x14ac:dyDescent="0.45">
+    <row r="6" spans="1:7" ht="20.25" x14ac:dyDescent="0.25">
       <c r="A6" s="29" t="s">
         <v>3</v>
       </c>
@@ -785,7 +785,7 @@
       <c r="F6" s="2"/>
       <c r="G6" s="2"/>
     </row>
-    <row r="7" spans="1:7" x14ac:dyDescent="0.45">
+    <row r="7" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A7" s="4" t="s">
         <v>4</v>
       </c>
@@ -806,133 +806,133 @@
         <v>9</v>
       </c>
     </row>
-    <row r="8" spans="1:7" x14ac:dyDescent="0.45">
+    <row r="8" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A8" s="7">
-        <v>46322</v>
+        <v>46323</v>
       </c>
       <c r="B8" s="8"/>
       <c r="C8" s="9" t="s">
         <v>10</v>
       </c>
       <c r="D8" s="10">
-        <v>261.82</v>
+        <v>264.01</v>
       </c>
       <c r="E8" s="10">
-        <v>219.05</v>
+        <v>221.25</v>
       </c>
       <c r="F8" s="10">
-        <v>229.05</v>
+        <v>231.25</v>
       </c>
       <c r="G8" s="10">
-        <v>216.67</v>
-      </c>
-    </row>
-    <row r="9" spans="1:7" x14ac:dyDescent="0.45">
+        <v>218.86</v>
+      </c>
+    </row>
+    <row r="9" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A9" s="11">
-        <v>46322</v>
+        <v>46323</v>
       </c>
       <c r="B9" s="12"/>
       <c r="C9" s="12" t="s">
         <v>11</v>
       </c>
       <c r="D9" s="13">
-        <v>261.82</v>
+        <v>264.01</v>
       </c>
       <c r="E9" s="13">
-        <v>219.05</v>
+        <v>221.25</v>
       </c>
       <c r="F9" s="13">
-        <v>229.05</v>
+        <v>231.25</v>
       </c>
       <c r="G9" s="13">
-        <v>216.67</v>
-      </c>
-    </row>
-    <row r="10" spans="1:7" x14ac:dyDescent="0.45">
+        <v>218.86</v>
+      </c>
+    </row>
+    <row r="10" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A10" s="7">
-        <v>46322</v>
+        <v>46323</v>
       </c>
       <c r="B10" s="8"/>
       <c r="C10" s="9" t="s">
         <v>12</v>
       </c>
       <c r="D10" s="10">
-        <v>261.10000000000002</v>
+        <v>262.29000000000002</v>
       </c>
       <c r="E10" s="10">
-        <v>221.05</v>
+        <v>222.3</v>
       </c>
       <c r="F10" s="10">
-        <v>231.05</v>
+        <v>232.3</v>
       </c>
       <c r="G10" s="10">
-        <v>219.46</v>
-      </c>
-    </row>
-    <row r="11" spans="1:7" x14ac:dyDescent="0.45">
+        <v>220.71</v>
+      </c>
+    </row>
+    <row r="11" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A11" s="11">
-        <v>46319</v>
+        <v>46322</v>
       </c>
       <c r="B11" s="12"/>
       <c r="C11" s="12" t="s">
         <v>10</v>
       </c>
       <c r="D11" s="13">
-        <v>261.57</v>
+        <v>261.82</v>
       </c>
       <c r="E11" s="13">
-        <v>218.41</v>
+        <v>219.05</v>
       </c>
       <c r="F11" s="13">
-        <v>228.41</v>
+        <v>229.05</v>
       </c>
       <c r="G11" s="13">
-        <v>216.03</v>
-      </c>
-    </row>
-    <row r="12" spans="1:7" x14ac:dyDescent="0.45">
+        <v>216.67</v>
+      </c>
+    </row>
+    <row r="12" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A12" s="7">
-        <v>46319</v>
+        <v>46322</v>
       </c>
       <c r="B12" s="8"/>
       <c r="C12" s="9" t="s">
         <v>11</v>
       </c>
       <c r="D12" s="10">
-        <v>261.57</v>
+        <v>261.82</v>
       </c>
       <c r="E12" s="10">
-        <v>218.41</v>
+        <v>219.05</v>
       </c>
       <c r="F12" s="10">
-        <v>228.41</v>
+        <v>229.05</v>
       </c>
       <c r="G12" s="10">
-        <v>216.03</v>
-      </c>
-    </row>
-    <row r="13" spans="1:7" x14ac:dyDescent="0.45">
+        <v>216.67</v>
+      </c>
+    </row>
+    <row r="13" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A13" s="11">
-        <v>46319</v>
+        <v>46322</v>
       </c>
       <c r="B13" s="12"/>
       <c r="C13" s="12" t="s">
         <v>12</v>
       </c>
       <c r="D13" s="13">
-        <v>259.04000000000002</v>
+        <v>261.10000000000002</v>
       </c>
       <c r="E13" s="13">
-        <v>219.66</v>
+        <v>221.05</v>
       </c>
       <c r="F13" s="13">
-        <v>229.66</v>
+        <v>231.05</v>
       </c>
       <c r="G13" s="13">
-        <v>218.07</v>
-      </c>
-    </row>
-    <row r="14" spans="1:7" x14ac:dyDescent="0.45">
+        <v>219.46</v>
+      </c>
+    </row>
+    <row r="14" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A14" s="14"/>
       <c r="B14" s="14"/>
       <c r="C14" s="15"/>
@@ -941,7 +941,7 @@
       <c r="F14" s="16"/>
       <c r="G14" s="16"/>
     </row>
-    <row r="15" spans="1:7" ht="20.25" x14ac:dyDescent="0.45">
+    <row r="15" spans="1:7" ht="20.25" x14ac:dyDescent="0.25">
       <c r="A15" s="29" t="s">
         <v>13</v>
       </c>
@@ -952,7 +952,7 @@
       <c r="F15" s="17"/>
       <c r="G15" s="17"/>
     </row>
-    <row r="16" spans="1:7" x14ac:dyDescent="0.45">
+    <row r="16" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A16" s="4" t="s">
         <v>4</v>
       </c>
@@ -971,45 +971,45 @@
       </c>
       <c r="G16" s="17"/>
     </row>
-    <row r="17" spans="1:7" x14ac:dyDescent="0.45">
+    <row r="17" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A17" s="7">
-        <v>46322</v>
+        <v>46323</v>
       </c>
       <c r="B17" s="8"/>
       <c r="C17" s="20" t="s">
         <v>14</v>
       </c>
       <c r="D17" s="10">
-        <v>264.39999999999998</v>
+        <v>265.62</v>
       </c>
       <c r="E17" s="10">
-        <v>223.85</v>
+        <v>225.12</v>
       </c>
       <c r="F17" s="10">
-        <v>233.85</v>
+        <v>235.12</v>
       </c>
       <c r="G17" s="17"/>
     </row>
-    <row r="18" spans="1:7" x14ac:dyDescent="0.45">
+    <row r="18" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A18" s="11">
-        <v>46319</v>
+        <v>46322</v>
       </c>
       <c r="B18" s="12"/>
       <c r="C18" s="12" t="s">
         <v>14</v>
       </c>
       <c r="D18" s="13">
-        <v>262.33</v>
+        <v>264.39999999999998</v>
       </c>
       <c r="E18" s="13">
-        <v>222.45</v>
+        <v>223.85</v>
       </c>
       <c r="F18" s="13">
-        <v>232.45</v>
+        <v>233.85</v>
       </c>
       <c r="G18" s="17"/>
     </row>
-    <row r="19" spans="1:7" x14ac:dyDescent="0.45">
+    <row r="19" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A19" s="14"/>
       <c r="B19" s="14"/>
       <c r="C19" s="15"/>
@@ -1018,7 +1018,7 @@
       <c r="F19" s="16"/>
       <c r="G19" s="17"/>
     </row>
-    <row r="20" spans="1:7" ht="20.25" x14ac:dyDescent="0.45">
+    <row r="20" spans="1:7" ht="20.25" x14ac:dyDescent="0.25">
       <c r="A20" s="29" t="s">
         <v>15</v>
       </c>
@@ -1029,7 +1029,7 @@
       <c r="F20" s="17"/>
       <c r="G20" s="17"/>
     </row>
-    <row r="21" spans="1:7" x14ac:dyDescent="0.45">
+    <row r="21" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A21" s="4" t="s">
         <v>4</v>
       </c>
@@ -1050,217 +1050,217 @@
         <v>9</v>
       </c>
     </row>
-    <row r="22" spans="1:7" x14ac:dyDescent="0.45">
+    <row r="22" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A22" s="7">
-        <v>46322</v>
+        <v>46323</v>
       </c>
       <c r="B22" s="8"/>
       <c r="C22" s="20" t="s">
         <v>16</v>
       </c>
       <c r="D22" s="10">
-        <v>262.94</v>
+        <v>264.58</v>
       </c>
       <c r="E22" s="10">
-        <v>218.64</v>
+        <v>220.29</v>
       </c>
       <c r="F22" s="10">
-        <v>228.24</v>
+        <v>229.89</v>
       </c>
       <c r="G22" s="10">
-        <v>215.01</v>
-      </c>
-    </row>
-    <row r="23" spans="1:7" x14ac:dyDescent="0.45">
+        <v>216.66</v>
+      </c>
+    </row>
+    <row r="23" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A23" s="11">
-        <v>46322</v>
+        <v>46323</v>
       </c>
       <c r="B23" s="12"/>
       <c r="C23" s="21" t="s">
         <v>17</v>
       </c>
       <c r="D23" s="13">
-        <v>266.07</v>
+        <v>267.26</v>
       </c>
       <c r="E23" s="13">
-        <v>229.37</v>
+        <v>230.61</v>
       </c>
       <c r="F23" s="13">
-        <v>239.37</v>
+        <v>240.61</v>
       </c>
       <c r="G23" s="13" t="s">
         <v>18</v>
       </c>
     </row>
-    <row r="24" spans="1:7" x14ac:dyDescent="0.45">
+    <row r="24" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A24" s="7">
-        <v>46322</v>
+        <v>46323</v>
       </c>
       <c r="B24" s="8"/>
       <c r="C24" s="20" t="s">
         <v>19</v>
       </c>
       <c r="D24" s="10">
-        <v>266.39999999999998</v>
+        <v>267.60000000000002</v>
       </c>
       <c r="E24" s="10">
-        <v>228.64</v>
+        <v>229.88</v>
       </c>
       <c r="F24" s="10">
-        <v>238.64</v>
+        <v>239.88</v>
       </c>
       <c r="G24" s="10" t="s">
         <v>18</v>
       </c>
     </row>
-    <row r="25" spans="1:7" x14ac:dyDescent="0.45">
+    <row r="25" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A25" s="11">
-        <v>46322</v>
+        <v>46323</v>
       </c>
       <c r="B25" s="12"/>
       <c r="C25" s="21" t="s">
         <v>20</v>
       </c>
       <c r="D25" s="13">
-        <v>263.08</v>
+        <v>264.27999999999997</v>
       </c>
       <c r="E25" s="13">
-        <v>228.86</v>
+        <v>230.1</v>
       </c>
       <c r="F25" s="13">
-        <v>238.86</v>
+        <v>240.1</v>
       </c>
       <c r="G25" s="13">
-        <v>224.7</v>
-      </c>
-    </row>
-    <row r="26" spans="1:7" x14ac:dyDescent="0.45">
+        <v>225.94</v>
+      </c>
+    </row>
+    <row r="26" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A26" s="7">
-        <v>46322</v>
+        <v>46323</v>
       </c>
       <c r="B26" s="8"/>
       <c r="C26" s="20" t="s">
         <v>21</v>
       </c>
       <c r="D26" s="10">
-        <v>264.57</v>
+        <v>265.77</v>
       </c>
       <c r="E26" s="10">
-        <v>230.28</v>
+        <v>231.53</v>
       </c>
       <c r="F26" s="10">
-        <v>240.28</v>
+        <v>241.53</v>
       </c>
       <c r="G26" s="10" t="s">
         <v>18</v>
       </c>
     </row>
-    <row r="27" spans="1:7" x14ac:dyDescent="0.45">
+    <row r="27" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A27" s="11">
-        <v>46319</v>
+        <v>46322</v>
       </c>
       <c r="B27" s="12"/>
       <c r="C27" s="12" t="s">
         <v>16</v>
       </c>
       <c r="D27" s="13">
-        <v>262.69</v>
+        <v>262.94</v>
       </c>
       <c r="E27" s="13">
-        <v>218.56</v>
+        <v>218.64</v>
       </c>
       <c r="F27" s="13">
-        <v>228.16</v>
+        <v>228.24</v>
       </c>
       <c r="G27" s="13">
-        <v>214.93</v>
-      </c>
-    </row>
-    <row r="28" spans="1:7" x14ac:dyDescent="0.45">
+        <v>215.01</v>
+      </c>
+    </row>
+    <row r="28" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A28" s="7">
-        <v>46319</v>
+        <v>46322</v>
       </c>
       <c r="B28" s="8"/>
       <c r="C28" s="20" t="s">
         <v>17</v>
       </c>
       <c r="D28" s="10">
-        <v>264.01</v>
+        <v>266.07</v>
       </c>
       <c r="E28" s="22">
-        <v>227.98</v>
+        <v>229.37</v>
       </c>
       <c r="F28" s="22">
-        <v>237.98</v>
+        <v>239.37</v>
       </c>
       <c r="G28" s="22" t="s">
         <v>18</v>
       </c>
     </row>
-    <row r="29" spans="1:7" x14ac:dyDescent="0.45">
+    <row r="29" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A29" s="11">
-        <v>46319</v>
+        <v>46322</v>
       </c>
       <c r="B29" s="12"/>
       <c r="C29" s="12" t="s">
         <v>19</v>
       </c>
       <c r="D29" s="13">
-        <v>264.33999999999997</v>
+        <v>266.39999999999998</v>
       </c>
       <c r="E29" s="13">
-        <v>227.25</v>
+        <v>228.64</v>
       </c>
       <c r="F29" s="13">
-        <v>237.25</v>
+        <v>238.64</v>
       </c>
       <c r="G29" s="13" t="s">
         <v>18</v>
       </c>
     </row>
-    <row r="30" spans="1:7" x14ac:dyDescent="0.45">
+    <row r="30" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A30" s="7">
-        <v>46319</v>
+        <v>46322</v>
       </c>
       <c r="B30" s="8"/>
       <c r="C30" s="20" t="s">
         <v>20</v>
       </c>
       <c r="D30" s="10">
-        <v>261.01</v>
+        <v>263.08</v>
       </c>
       <c r="E30" s="22">
-        <v>227.47</v>
+        <v>228.86</v>
       </c>
       <c r="F30" s="22">
-        <v>237.47</v>
+        <v>238.86</v>
       </c>
       <c r="G30" s="22">
-        <v>223.31</v>
-      </c>
-    </row>
-    <row r="31" spans="1:7" x14ac:dyDescent="0.45">
+        <v>224.7</v>
+      </c>
+    </row>
+    <row r="31" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A31" s="11">
-        <v>46319</v>
+        <v>46322</v>
       </c>
       <c r="B31" s="12"/>
       <c r="C31" s="12" t="s">
         <v>21</v>
       </c>
       <c r="D31" s="13">
-        <v>262.5</v>
+        <v>264.57</v>
       </c>
       <c r="E31" s="13">
-        <v>228.88</v>
+        <v>230.28</v>
       </c>
       <c r="F31" s="13">
-        <v>238.88</v>
+        <v>240.28</v>
       </c>
       <c r="G31" s="13" t="s">
         <v>18</v>
       </c>
     </row>
-    <row r="32" spans="1:7" x14ac:dyDescent="0.45">
+    <row r="32" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A32" s="14"/>
       <c r="B32" s="14"/>
       <c r="C32" s="15"/>
@@ -1269,7 +1269,7 @@
       <c r="F32" s="17"/>
       <c r="G32" s="17"/>
     </row>
-    <row r="33" spans="1:7" ht="20.25" x14ac:dyDescent="0.45">
+    <row r="33" spans="1:7" ht="20.25" x14ac:dyDescent="0.25">
       <c r="A33" s="29" t="s">
         <v>22</v>
       </c>
@@ -1280,7 +1280,7 @@
       <c r="F33" s="17"/>
       <c r="G33" s="17"/>
     </row>
-    <row r="34" spans="1:7" x14ac:dyDescent="0.45">
+    <row r="34" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A34" s="23" t="s">
         <v>4</v>
       </c>
@@ -1299,54 +1299,54 @@
       </c>
       <c r="G34" s="17"/>
     </row>
-    <row r="35" spans="1:7" x14ac:dyDescent="0.45">
+    <row r="35" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A35" s="7">
-        <v>46322</v>
+        <v>46323</v>
       </c>
       <c r="B35" s="8"/>
       <c r="C35" s="20" t="s">
         <v>23</v>
       </c>
       <c r="D35" s="10">
-        <v>259.66000000000003</v>
+        <v>260.85000000000002</v>
       </c>
       <c r="E35" s="10">
-        <v>220.02</v>
+        <v>221.26</v>
       </c>
       <c r="F35" s="10">
-        <v>229.02</v>
+        <v>230.26</v>
       </c>
       <c r="G35" s="17"/>
     </row>
-    <row r="36" spans="1:7" x14ac:dyDescent="0.45">
+    <row r="36" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A36" s="11">
-        <v>46319</v>
+        <v>46322</v>
       </c>
       <c r="B36" s="12"/>
       <c r="C36" s="12" t="s">
         <v>23</v>
       </c>
       <c r="D36" s="13">
-        <v>257.58999999999997</v>
+        <v>259.66000000000003</v>
       </c>
       <c r="E36" s="13">
-        <v>218.63</v>
+        <v>220.02</v>
       </c>
       <c r="F36" s="13">
-        <v>227.63</v>
+        <v>229.02</v>
       </c>
       <c r="G36" s="17"/>
     </row>
-    <row r="37" spans="1:7" x14ac:dyDescent="0.45">
+    <row r="37" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A37" s="7">
-        <v>46322</v>
+        <v>46323</v>
       </c>
       <c r="B37" s="8"/>
       <c r="C37" s="20" t="s">
         <v>24</v>
       </c>
       <c r="D37" s="10">
-        <v>275.27999999999997</v>
+        <v>276.47000000000003</v>
       </c>
       <c r="E37" s="10" t="s">
         <v>18</v>
@@ -1356,16 +1356,16 @@
       </c>
       <c r="G37" s="17"/>
     </row>
-    <row r="38" spans="1:7" x14ac:dyDescent="0.45">
+    <row r="38" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A38" s="11">
-        <v>46319</v>
+        <v>46322</v>
       </c>
       <c r="B38" s="12"/>
       <c r="C38" s="12" t="s">
         <v>24</v>
       </c>
       <c r="D38" s="13">
-        <v>273.20999999999998</v>
+        <v>275.27999999999997</v>
       </c>
       <c r="E38" s="13" t="s">
         <v>18</v>
@@ -1375,7 +1375,7 @@
       </c>
       <c r="G38" s="17"/>
     </row>
-    <row r="39" spans="1:7" x14ac:dyDescent="0.45">
+    <row r="39" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A39" s="24"/>
       <c r="B39" s="24"/>
       <c r="C39" s="15"/>
@@ -1384,7 +1384,7 @@
       <c r="F39" s="17"/>
       <c r="G39" s="17"/>
     </row>
-    <row r="40" spans="1:7" ht="20.25" x14ac:dyDescent="0.45">
+    <row r="40" spans="1:7" ht="20.25" x14ac:dyDescent="0.25">
       <c r="A40" s="29" t="s">
         <v>25</v>
       </c>
@@ -1395,7 +1395,7 @@
       <c r="F40" s="17"/>
       <c r="G40" s="17"/>
     </row>
-    <row r="41" spans="1:7" x14ac:dyDescent="0.45">
+    <row r="41" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A41" s="23" t="s">
         <v>4</v>
       </c>
@@ -1414,83 +1414,83 @@
       </c>
       <c r="G41" s="17"/>
     </row>
-    <row r="42" spans="1:7" x14ac:dyDescent="0.45">
+    <row r="42" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A42" s="7">
-        <v>46322</v>
+        <v>46323</v>
       </c>
       <c r="B42" s="8"/>
       <c r="C42" s="20" t="s">
         <v>26</v>
       </c>
       <c r="D42" s="10">
-        <v>269.79000000000002</v>
+        <v>270.95999999999998</v>
       </c>
       <c r="E42" s="10">
-        <v>231.2</v>
+        <v>232.8</v>
       </c>
       <c r="F42" s="10">
-        <v>241.2</v>
+        <v>242.8</v>
       </c>
       <c r="G42" s="17"/>
     </row>
-    <row r="43" spans="1:7" x14ac:dyDescent="0.45">
+    <row r="43" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A43" s="11">
-        <v>46322</v>
+        <v>46323</v>
       </c>
       <c r="B43" s="12"/>
       <c r="C43" s="21" t="s">
         <v>27</v>
       </c>
       <c r="D43" s="13">
-        <v>269.39</v>
+        <v>270.57</v>
       </c>
       <c r="E43" s="13">
-        <v>231.61</v>
+        <v>233.21</v>
       </c>
       <c r="F43" s="13">
-        <v>241.61</v>
+        <v>243.21</v>
       </c>
       <c r="G43" s="17"/>
     </row>
-    <row r="44" spans="1:7" x14ac:dyDescent="0.45">
+    <row r="44" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A44" s="7">
-        <v>46319</v>
+        <v>46322</v>
       </c>
       <c r="B44" s="8"/>
       <c r="C44" s="20" t="s">
         <v>26</v>
       </c>
       <c r="D44" s="10">
-        <v>267.73</v>
+        <v>269.79000000000002</v>
       </c>
       <c r="E44" s="10">
-        <v>229.86</v>
+        <v>231.2</v>
       </c>
       <c r="F44" s="10">
-        <v>239.86</v>
+        <v>241.2</v>
       </c>
       <c r="G44" s="17"/>
     </row>
-    <row r="45" spans="1:7" x14ac:dyDescent="0.45">
+    <row r="45" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A45" s="11">
-        <v>46319</v>
+        <v>46322</v>
       </c>
       <c r="B45" s="12"/>
       <c r="C45" s="21" t="s">
         <v>27</v>
       </c>
       <c r="D45" s="13">
-        <v>267.33999999999997</v>
+        <v>269.39</v>
       </c>
       <c r="E45" s="13">
-        <v>230.27</v>
+        <v>231.61</v>
       </c>
       <c r="F45" s="13">
-        <v>240.27</v>
+        <v>241.61</v>
       </c>
       <c r="G45" s="17"/>
     </row>
-    <row r="46" spans="1:7" x14ac:dyDescent="0.45">
+    <row r="46" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A46" s="14"/>
       <c r="B46" s="24"/>
       <c r="C46" s="15"/>
@@ -1499,7 +1499,7 @@
       <c r="F46" s="16"/>
       <c r="G46" s="17"/>
     </row>
-    <row r="47" spans="1:7" ht="20.25" x14ac:dyDescent="0.45">
+    <row r="47" spans="1:7" ht="20.25" x14ac:dyDescent="0.25">
       <c r="A47" s="25" t="s">
         <v>28</v>
       </c>
@@ -1510,7 +1510,7 @@
       <c r="F47" s="17"/>
       <c r="G47" s="17"/>
     </row>
-    <row r="48" spans="1:7" x14ac:dyDescent="0.45">
+    <row r="48" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A48" s="23" t="s">
         <v>4</v>
       </c>
@@ -1529,83 +1529,83 @@
       </c>
       <c r="G48" s="17"/>
     </row>
-    <row r="49" spans="1:7" x14ac:dyDescent="0.45">
+    <row r="49" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A49" s="7">
-        <v>46322</v>
+        <v>46323</v>
       </c>
       <c r="B49" s="8"/>
       <c r="C49" s="20" t="s">
         <v>29</v>
       </c>
       <c r="D49" s="10">
-        <v>260.60000000000002</v>
+        <v>261.45</v>
       </c>
       <c r="E49" s="10">
-        <v>220.83</v>
+        <v>221.55</v>
       </c>
       <c r="F49" s="10">
-        <v>230.83</v>
+        <v>231.55</v>
       </c>
       <c r="G49" s="28"/>
     </row>
-    <row r="50" spans="1:7" x14ac:dyDescent="0.45">
+    <row r="50" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A50" s="11">
-        <v>46322</v>
+        <v>46323</v>
       </c>
       <c r="B50" s="12"/>
       <c r="C50" s="21" t="s">
         <v>30</v>
       </c>
       <c r="D50" s="13">
-        <v>258.08</v>
+        <v>258.93</v>
       </c>
       <c r="E50" s="13">
-        <v>220.41</v>
+        <v>221.12</v>
       </c>
       <c r="F50" s="13">
-        <v>230.41</v>
+        <v>231.12</v>
       </c>
       <c r="G50" s="28"/>
     </row>
-    <row r="51" spans="1:7" x14ac:dyDescent="0.45">
+    <row r="51" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A51" s="7">
-        <v>46319</v>
+        <v>46322</v>
       </c>
       <c r="B51" s="8"/>
       <c r="C51" s="20" t="s">
         <v>29</v>
       </c>
       <c r="D51" s="10">
-        <v>259.70999999999998</v>
+        <v>260.60000000000002</v>
       </c>
       <c r="E51" s="10">
-        <v>221.08</v>
+        <v>220.83</v>
       </c>
       <c r="F51" s="10">
-        <v>231.08</v>
+        <v>230.83</v>
       </c>
       <c r="G51" s="17"/>
     </row>
-    <row r="52" spans="1:7" x14ac:dyDescent="0.45">
+    <row r="52" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A52" s="11">
-        <v>46319</v>
+        <v>46322</v>
       </c>
       <c r="B52" s="12"/>
       <c r="C52" s="21" t="s">
         <v>30</v>
       </c>
       <c r="D52" s="13">
-        <v>257.22000000000003</v>
+        <v>258.08</v>
       </c>
       <c r="E52" s="13">
-        <v>220.67</v>
+        <v>220.41</v>
       </c>
       <c r="F52" s="13">
-        <v>230.67</v>
+        <v>230.41</v>
       </c>
       <c r="G52" s="17"/>
     </row>
-    <row r="53" spans="1:7" x14ac:dyDescent="0.45">
+    <row r="53" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A53" s="14"/>
       <c r="B53" s="14"/>
       <c r="C53" s="15"/>
@@ -1614,7 +1614,7 @@
       <c r="F53" s="16"/>
       <c r="G53" s="17"/>
     </row>
-    <row r="54" spans="1:7" ht="20.25" x14ac:dyDescent="0.45">
+    <row r="54" spans="1:7" ht="20.25" x14ac:dyDescent="0.25">
       <c r="A54" s="27" t="s">
         <v>31</v>
       </c>
@@ -1625,7 +1625,7 @@
       <c r="F54" s="17"/>
       <c r="G54" s="17"/>
     </row>
-    <row r="55" spans="1:7" x14ac:dyDescent="0.45">
+    <row r="55" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A55" s="23" t="s">
         <v>4</v>
       </c>
@@ -1644,54 +1644,54 @@
       </c>
       <c r="G55" s="17"/>
     </row>
-    <row r="56" spans="1:7" x14ac:dyDescent="0.45">
+    <row r="56" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A56" s="7">
-        <v>46322</v>
+        <v>46323</v>
       </c>
       <c r="B56" s="8"/>
       <c r="C56" s="20" t="s">
         <v>32</v>
       </c>
       <c r="D56" s="10">
-        <v>275.72000000000003</v>
+        <v>276.92</v>
       </c>
       <c r="E56" s="10">
-        <v>248.42</v>
+        <v>249.57</v>
       </c>
       <c r="F56" s="10">
-        <v>258.42</v>
+        <v>259.57</v>
       </c>
       <c r="G56" s="17"/>
     </row>
-    <row r="57" spans="1:7" x14ac:dyDescent="0.45">
+    <row r="57" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A57" s="11">
-        <v>46322</v>
+        <v>46323</v>
       </c>
       <c r="B57" s="12"/>
       <c r="C57" s="21" t="s">
         <v>33</v>
       </c>
       <c r="D57" s="13">
-        <v>263.20999999999998</v>
+        <v>264.39999999999998</v>
       </c>
       <c r="E57" s="13">
-        <v>229.08</v>
+        <v>230.35</v>
       </c>
       <c r="F57" s="13">
-        <v>239.08</v>
+        <v>240.35</v>
       </c>
       <c r="G57" s="17"/>
     </row>
-    <row r="58" spans="1:7" x14ac:dyDescent="0.45">
+    <row r="58" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A58" s="7">
-        <v>46322</v>
+        <v>46323</v>
       </c>
       <c r="B58" s="8"/>
       <c r="C58" s="20" t="s">
         <v>34</v>
       </c>
       <c r="D58" s="10">
-        <v>264.01</v>
+        <v>265.19</v>
       </c>
       <c r="E58" s="10" t="s">
         <v>18</v>
@@ -1701,111 +1701,111 @@
       </c>
       <c r="G58" s="17"/>
     </row>
-    <row r="59" spans="1:7" x14ac:dyDescent="0.45">
+    <row r="59" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A59" s="11">
-        <v>46322</v>
+        <v>46323</v>
       </c>
       <c r="B59" s="12"/>
       <c r="C59" s="21" t="s">
         <v>35</v>
       </c>
       <c r="D59" s="13">
-        <v>260.02999999999997</v>
+        <v>261.25</v>
       </c>
       <c r="E59" s="13">
-        <v>223.46</v>
+        <v>224.73</v>
       </c>
       <c r="F59" s="13" t="s">
         <v>18</v>
       </c>
       <c r="G59" s="17"/>
     </row>
-    <row r="60" spans="1:7" x14ac:dyDescent="0.45">
+    <row r="60" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A60" s="7">
-        <v>46322</v>
+        <v>46323</v>
       </c>
       <c r="B60" s="8"/>
       <c r="C60" s="20" t="s">
         <v>36</v>
       </c>
       <c r="D60" s="10">
-        <v>255.86</v>
+        <v>257.08999999999997</v>
       </c>
       <c r="E60" s="10">
-        <v>219.4</v>
+        <v>220.67</v>
       </c>
       <c r="F60" s="10">
-        <v>229.4</v>
+        <v>230.67</v>
       </c>
       <c r="G60" s="17"/>
     </row>
-    <row r="61" spans="1:7" x14ac:dyDescent="0.45">
+    <row r="61" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A61" s="11">
-        <v>46322</v>
+        <v>46323</v>
       </c>
       <c r="B61" s="12"/>
       <c r="C61" s="21" t="s">
         <v>37</v>
       </c>
       <c r="D61" s="13">
-        <v>263.47000000000003</v>
+        <v>264.7</v>
       </c>
       <c r="E61" s="13">
-        <v>241.44</v>
+        <v>242.64</v>
       </c>
       <c r="F61" s="13" t="s">
         <v>18</v>
       </c>
       <c r="G61" s="17"/>
     </row>
-    <row r="62" spans="1:7" x14ac:dyDescent="0.45">
+    <row r="62" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A62" s="7">
-        <v>46319</v>
+        <v>46322</v>
       </c>
       <c r="B62" s="8"/>
       <c r="C62" s="20" t="s">
         <v>32</v>
       </c>
       <c r="D62" s="10">
-        <v>273.66000000000003</v>
+        <v>275.72000000000003</v>
       </c>
       <c r="E62" s="10">
-        <v>247.06</v>
+        <v>248.42</v>
       </c>
       <c r="F62" s="10">
-        <v>257.06</v>
+        <v>258.42</v>
       </c>
       <c r="G62" s="17"/>
     </row>
-    <row r="63" spans="1:7" x14ac:dyDescent="0.45">
+    <row r="63" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A63" s="11">
-        <v>46319</v>
+        <v>46322</v>
       </c>
       <c r="B63" s="12"/>
       <c r="C63" s="21" t="s">
         <v>33</v>
       </c>
       <c r="D63" s="13">
-        <v>261.14</v>
+        <v>263.20999999999998</v>
       </c>
       <c r="E63" s="13">
-        <v>227.68</v>
+        <v>229.08</v>
       </c>
       <c r="F63" s="13">
-        <v>237.68</v>
+        <v>239.08</v>
       </c>
       <c r="G63" s="17"/>
     </row>
-    <row r="64" spans="1:7" x14ac:dyDescent="0.45">
+    <row r="64" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A64" s="7">
-        <v>46319</v>
+        <v>46322</v>
       </c>
       <c r="B64" s="8"/>
       <c r="C64" s="20" t="s">
         <v>34</v>
       </c>
       <c r="D64" s="10">
-        <v>261.95</v>
+        <v>264.01</v>
       </c>
       <c r="E64" s="10" t="s">
         <v>18</v>
@@ -1815,55 +1815,55 @@
       </c>
       <c r="G64" s="17"/>
     </row>
-    <row r="65" spans="1:6" x14ac:dyDescent="0.45">
+    <row r="65" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A65" s="11">
-        <v>46319</v>
+        <v>46322</v>
       </c>
       <c r="B65" s="12"/>
       <c r="C65" s="21" t="s">
         <v>35</v>
       </c>
       <c r="D65" s="13">
-        <v>257.97000000000003</v>
+        <v>260.02999999999997</v>
       </c>
       <c r="E65" s="13">
-        <v>222.07</v>
+        <v>223.46</v>
       </c>
       <c r="F65" s="13" t="s">
         <v>18</v>
       </c>
     </row>
-    <row r="66" spans="1:6" x14ac:dyDescent="0.45">
+    <row r="66" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A66" s="7">
-        <v>46319</v>
+        <v>46322</v>
       </c>
       <c r="B66" s="8"/>
       <c r="C66" s="20" t="s">
         <v>36</v>
       </c>
       <c r="D66" s="10">
-        <v>253.8</v>
+        <v>255.86</v>
       </c>
       <c r="E66" s="10">
-        <v>218</v>
+        <v>219.4</v>
       </c>
       <c r="F66" s="10">
-        <v>228</v>
-      </c>
-    </row>
-    <row r="67" spans="1:6" x14ac:dyDescent="0.45">
+        <v>229.4</v>
+      </c>
+    </row>
+    <row r="67" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A67" s="11">
-        <v>46319</v>
+        <v>46322</v>
       </c>
       <c r="B67" s="12"/>
       <c r="C67" s="21" t="s">
         <v>37</v>
       </c>
       <c r="D67" s="13">
-        <v>261.39</v>
+        <v>263.47000000000003</v>
       </c>
       <c r="E67" s="13">
-        <v>240.07</v>
+        <v>241.44</v>
       </c>
       <c r="F67" s="13" t="s">
         <v>18</v>
@@ -1891,15 +1891,6 @@
 </file>
 
 <file path=customXml/item1.xml><?xml version="1.0" encoding="utf-8"?>
-<?mso-contentType ?>
-<FormTemplates xmlns="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms">
-  <Display>DocumentLibraryForm</Display>
-  <Edit>DocumentLibraryForm</Edit>
-  <New>DocumentLibraryForm</New>
-</FormTemplates>
-</file>
-
-<file path=customXml/item2.xml><?xml version="1.0" encoding="utf-8"?>
 <p:properties xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls">
   <documentManagement>
     <lcf76f155ced4ddcb4097134ff3c332f xmlns="87276d81-85f4-4ef2-9e6e-55066304288f">
@@ -1908,6 +1899,15 @@
     <TaxCatchAll xmlns="b23b8984-eafa-4e79-985e-54f52f3da58e" xsi:nil="true"/>
   </documentManagement>
 </p:properties>
+</file>
+
+<file path=customXml/item2.xml><?xml version="1.0" encoding="utf-8"?>
+<?mso-contentType ?>
+<FormTemplates xmlns="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms">
+  <Display>DocumentLibraryForm</Display>
+  <Edit>DocumentLibraryForm</Edit>
+  <New>DocumentLibraryForm</New>
+</FormTemplates>
 </file>
 
 <file path=customXml/item3.xml><?xml version="1.0" encoding="utf-8"?>
@@ -2171,20 +2171,20 @@
 </file>
 
 <file path=customXml/itemProps1.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{F60519E9-FD90-4339-869C-BC2F85719BB8}">
-  <ds:schemaRefs>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms"/>
-  </ds:schemaRefs>
-</ds:datastoreItem>
-</file>
-
-<file path=customXml/itemProps2.xml><?xml version="1.0" encoding="utf-8"?>
 <ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{57A83D98-2BAE-4D83-823A-D31C464B620C}">
   <ds:schemaRefs>
     <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/properties"/>
     <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
     <ds:schemaRef ds:uri="87276d81-85f4-4ef2-9e6e-55066304288f"/>
     <ds:schemaRef ds:uri="b23b8984-eafa-4e79-985e-54f52f3da58e"/>
+  </ds:schemaRefs>
+</ds:datastoreItem>
+</file>
+
+<file path=customXml/itemProps2.xml><?xml version="1.0" encoding="utf-8"?>
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{F60519E9-FD90-4339-869C-BC2F85719BB8}">
+  <ds:schemaRefs>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms"/>
   </ds:schemaRefs>
 </ds:datastoreItem>
 </file>

</xml_diff>

<commit_message>
Wed Oct 28 06:55:35 UTC 2026
</commit_message>
<xml_diff>
--- a/bp.com-content-dam-bp-country-sites-en_au-australia-home-products-services-pricing-tgp-excel.xlsx
+++ b/bp.com-content-dam-bp-country-sites-en_au-australia-home-products-services-pricing-tgp-excel.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://bp365.sharepoint.com/sites/WholesalePricing/Shared Documents/B2C/TGP/Daily TGP/Web TGP/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="14_{EF43C469-EB28-4682-8447-7FF2257DA8E5}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="14_{3B00F6F4-A812-4F69-8117-152783F825CB}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-28920" yWindow="-60" windowWidth="29040" windowHeight="15720" xr2:uid="{1B412EEF-F96D-4DF4-A4E9-C7F0F183C2FB}"/>
   </bookViews>
@@ -808,128 +808,128 @@
     </row>
     <row r="8" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A8" s="7">
-        <v>46323</v>
+        <v>46324</v>
       </c>
       <c r="B8" s="8"/>
       <c r="C8" s="9" t="s">
         <v>10</v>
       </c>
       <c r="D8" s="10">
-        <v>264.01</v>
+        <v>264.29000000000002</v>
       </c>
       <c r="E8" s="10">
-        <v>221.25</v>
+        <v>222.63</v>
       </c>
       <c r="F8" s="10">
-        <v>231.25</v>
+        <v>232.63</v>
       </c>
       <c r="G8" s="10">
-        <v>218.86</v>
+        <v>220.24</v>
       </c>
     </row>
     <row r="9" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A9" s="11">
-        <v>46323</v>
+        <v>46324</v>
       </c>
       <c r="B9" s="12"/>
       <c r="C9" s="12" t="s">
         <v>11</v>
       </c>
       <c r="D9" s="13">
-        <v>264.01</v>
+        <v>264.29000000000002</v>
       </c>
       <c r="E9" s="13">
-        <v>221.25</v>
+        <v>222.63</v>
       </c>
       <c r="F9" s="13">
-        <v>231.25</v>
+        <v>232.63</v>
       </c>
       <c r="G9" s="13">
-        <v>218.86</v>
+        <v>220.24</v>
       </c>
     </row>
     <row r="10" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A10" s="7">
-        <v>46323</v>
+        <v>46324</v>
       </c>
       <c r="B10" s="8"/>
       <c r="C10" s="9" t="s">
         <v>12</v>
       </c>
       <c r="D10" s="10">
-        <v>262.29000000000002</v>
+        <v>262.39999999999998</v>
       </c>
       <c r="E10" s="10">
-        <v>222.3</v>
+        <v>223.52</v>
       </c>
       <c r="F10" s="10">
-        <v>232.3</v>
+        <v>233.52</v>
       </c>
       <c r="G10" s="10">
-        <v>220.71</v>
+        <v>221.93</v>
       </c>
     </row>
     <row r="11" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A11" s="11">
-        <v>46322</v>
+        <v>46323</v>
       </c>
       <c r="B11" s="12"/>
       <c r="C11" s="12" t="s">
         <v>10</v>
       </c>
       <c r="D11" s="13">
-        <v>261.82</v>
+        <v>264.01</v>
       </c>
       <c r="E11" s="13">
-        <v>219.05</v>
+        <v>221.25</v>
       </c>
       <c r="F11" s="13">
-        <v>229.05</v>
+        <v>231.25</v>
       </c>
       <c r="G11" s="13">
-        <v>216.67</v>
+        <v>218.86</v>
       </c>
     </row>
     <row r="12" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A12" s="7">
-        <v>46322</v>
+        <v>46323</v>
       </c>
       <c r="B12" s="8"/>
       <c r="C12" s="9" t="s">
         <v>11</v>
       </c>
       <c r="D12" s="10">
-        <v>261.82</v>
+        <v>264.01</v>
       </c>
       <c r="E12" s="10">
-        <v>219.05</v>
+        <v>221.25</v>
       </c>
       <c r="F12" s="10">
-        <v>229.05</v>
+        <v>231.25</v>
       </c>
       <c r="G12" s="10">
-        <v>216.67</v>
+        <v>218.86</v>
       </c>
     </row>
     <row r="13" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A13" s="11">
-        <v>46322</v>
+        <v>46323</v>
       </c>
       <c r="B13" s="12"/>
       <c r="C13" s="12" t="s">
         <v>12</v>
       </c>
       <c r="D13" s="13">
-        <v>261.10000000000002</v>
+        <v>262.29000000000002</v>
       </c>
       <c r="E13" s="13">
-        <v>221.05</v>
+        <v>222.3</v>
       </c>
       <c r="F13" s="13">
-        <v>231.05</v>
+        <v>232.3</v>
       </c>
       <c r="G13" s="13">
-        <v>219.46</v>
+        <v>220.71</v>
       </c>
     </row>
     <row r="14" spans="1:7" x14ac:dyDescent="0.25">
@@ -973,39 +973,39 @@
     </row>
     <row r="17" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A17" s="7">
-        <v>46323</v>
+        <v>46324</v>
       </c>
       <c r="B17" s="8"/>
       <c r="C17" s="20" t="s">
         <v>14</v>
       </c>
       <c r="D17" s="10">
-        <v>265.62</v>
+        <v>265.72000000000003</v>
       </c>
       <c r="E17" s="10">
-        <v>225.12</v>
+        <v>226.35</v>
       </c>
       <c r="F17" s="10">
-        <v>235.12</v>
+        <v>236.35</v>
       </c>
       <c r="G17" s="17"/>
     </row>
     <row r="18" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A18" s="11">
-        <v>46322</v>
+        <v>46323</v>
       </c>
       <c r="B18" s="12"/>
       <c r="C18" s="12" t="s">
         <v>14</v>
       </c>
       <c r="D18" s="13">
-        <v>264.39999999999998</v>
+        <v>265.62</v>
       </c>
       <c r="E18" s="13">
-        <v>223.85</v>
+        <v>225.12</v>
       </c>
       <c r="F18" s="13">
-        <v>233.85</v>
+        <v>235.12</v>
       </c>
       <c r="G18" s="17"/>
     </row>
@@ -1052,41 +1052,41 @@
     </row>
     <row r="22" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A22" s="7">
-        <v>46323</v>
+        <v>46324</v>
       </c>
       <c r="B22" s="8"/>
       <c r="C22" s="20" t="s">
         <v>16</v>
       </c>
       <c r="D22" s="10">
-        <v>264.58</v>
+        <v>264.86</v>
       </c>
       <c r="E22" s="10">
-        <v>220.29</v>
+        <v>221.67</v>
       </c>
       <c r="F22" s="10">
-        <v>229.89</v>
+        <v>231.27</v>
       </c>
       <c r="G22" s="10">
-        <v>216.66</v>
+        <v>218.04</v>
       </c>
     </row>
     <row r="23" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A23" s="11">
-        <v>46323</v>
+        <v>46324</v>
       </c>
       <c r="B23" s="12"/>
       <c r="C23" s="21" t="s">
         <v>17</v>
       </c>
       <c r="D23" s="13">
-        <v>267.26</v>
+        <v>267.37</v>
       </c>
       <c r="E23" s="13">
-        <v>230.61</v>
+        <v>231.83</v>
       </c>
       <c r="F23" s="13">
-        <v>240.61</v>
+        <v>241.83</v>
       </c>
       <c r="G23" s="13" t="s">
         <v>18</v>
@@ -1094,20 +1094,20 @@
     </row>
     <row r="24" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A24" s="7">
-        <v>46323</v>
+        <v>46324</v>
       </c>
       <c r="B24" s="8"/>
       <c r="C24" s="20" t="s">
         <v>19</v>
       </c>
       <c r="D24" s="10">
-        <v>267.60000000000002</v>
+        <v>267.7</v>
       </c>
       <c r="E24" s="10">
-        <v>229.88</v>
+        <v>231.1</v>
       </c>
       <c r="F24" s="10">
-        <v>239.88</v>
+        <v>241.1</v>
       </c>
       <c r="G24" s="10" t="s">
         <v>18</v>
@@ -1115,41 +1115,41 @@
     </row>
     <row r="25" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A25" s="11">
-        <v>46323</v>
+        <v>46324</v>
       </c>
       <c r="B25" s="12"/>
       <c r="C25" s="21" t="s">
         <v>20</v>
       </c>
       <c r="D25" s="13">
-        <v>264.27999999999997</v>
+        <v>264.38</v>
       </c>
       <c r="E25" s="13">
-        <v>230.1</v>
+        <v>231.33</v>
       </c>
       <c r="F25" s="13">
-        <v>240.1</v>
+        <v>241.33</v>
       </c>
       <c r="G25" s="13">
-        <v>225.94</v>
+        <v>227.17</v>
       </c>
     </row>
     <row r="26" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A26" s="7">
-        <v>46323</v>
+        <v>46324</v>
       </c>
       <c r="B26" s="8"/>
       <c r="C26" s="20" t="s">
         <v>21</v>
       </c>
       <c r="D26" s="10">
-        <v>265.77</v>
+        <v>265.87</v>
       </c>
       <c r="E26" s="10">
-        <v>231.53</v>
+        <v>232.77</v>
       </c>
       <c r="F26" s="10">
-        <v>241.53</v>
+        <v>242.77</v>
       </c>
       <c r="G26" s="10" t="s">
         <v>18</v>
@@ -1157,41 +1157,41 @@
     </row>
     <row r="27" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A27" s="11">
-        <v>46322</v>
+        <v>46323</v>
       </c>
       <c r="B27" s="12"/>
       <c r="C27" s="12" t="s">
         <v>16</v>
       </c>
       <c r="D27" s="13">
-        <v>262.94</v>
+        <v>264.58</v>
       </c>
       <c r="E27" s="13">
-        <v>218.64</v>
+        <v>220.29</v>
       </c>
       <c r="F27" s="13">
-        <v>228.24</v>
+        <v>229.89</v>
       </c>
       <c r="G27" s="13">
-        <v>215.01</v>
+        <v>216.66</v>
       </c>
     </row>
     <row r="28" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A28" s="7">
-        <v>46322</v>
+        <v>46323</v>
       </c>
       <c r="B28" s="8"/>
       <c r="C28" s="20" t="s">
         <v>17</v>
       </c>
       <c r="D28" s="10">
-        <v>266.07</v>
+        <v>267.26</v>
       </c>
       <c r="E28" s="22">
-        <v>229.37</v>
+        <v>230.61</v>
       </c>
       <c r="F28" s="22">
-        <v>239.37</v>
+        <v>240.61</v>
       </c>
       <c r="G28" s="22" t="s">
         <v>18</v>
@@ -1199,20 +1199,20 @@
     </row>
     <row r="29" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A29" s="11">
-        <v>46322</v>
+        <v>46323</v>
       </c>
       <c r="B29" s="12"/>
       <c r="C29" s="12" t="s">
         <v>19</v>
       </c>
       <c r="D29" s="13">
-        <v>266.39999999999998</v>
+        <v>267.60000000000002</v>
       </c>
       <c r="E29" s="13">
-        <v>228.64</v>
+        <v>229.88</v>
       </c>
       <c r="F29" s="13">
-        <v>238.64</v>
+        <v>239.88</v>
       </c>
       <c r="G29" s="13" t="s">
         <v>18</v>
@@ -1220,41 +1220,41 @@
     </row>
     <row r="30" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A30" s="7">
-        <v>46322</v>
+        <v>46323</v>
       </c>
       <c r="B30" s="8"/>
       <c r="C30" s="20" t="s">
         <v>20</v>
       </c>
       <c r="D30" s="10">
-        <v>263.08</v>
+        <v>264.27999999999997</v>
       </c>
       <c r="E30" s="22">
-        <v>228.86</v>
+        <v>230.1</v>
       </c>
       <c r="F30" s="22">
-        <v>238.86</v>
+        <v>240.1</v>
       </c>
       <c r="G30" s="22">
-        <v>224.7</v>
+        <v>225.94</v>
       </c>
     </row>
     <row r="31" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A31" s="11">
-        <v>46322</v>
+        <v>46323</v>
       </c>
       <c r="B31" s="12"/>
       <c r="C31" s="12" t="s">
         <v>21</v>
       </c>
       <c r="D31" s="13">
-        <v>264.57</v>
+        <v>265.77</v>
       </c>
       <c r="E31" s="13">
-        <v>230.28</v>
+        <v>231.53</v>
       </c>
       <c r="F31" s="13">
-        <v>240.28</v>
+        <v>241.53</v>
       </c>
       <c r="G31" s="13" t="s">
         <v>18</v>
@@ -1301,52 +1301,52 @@
     </row>
     <row r="35" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A35" s="7">
-        <v>46323</v>
+        <v>46324</v>
       </c>
       <c r="B35" s="8"/>
       <c r="C35" s="20" t="s">
         <v>23</v>
       </c>
       <c r="D35" s="10">
-        <v>260.85000000000002</v>
+        <v>260.95999999999998</v>
       </c>
       <c r="E35" s="10">
-        <v>221.26</v>
+        <v>222.49</v>
       </c>
       <c r="F35" s="10">
-        <v>230.26</v>
+        <v>231.49</v>
       </c>
       <c r="G35" s="17"/>
     </row>
     <row r="36" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A36" s="11">
-        <v>46322</v>
+        <v>46323</v>
       </c>
       <c r="B36" s="12"/>
       <c r="C36" s="12" t="s">
         <v>23</v>
       </c>
       <c r="D36" s="13">
-        <v>259.66000000000003</v>
+        <v>260.85000000000002</v>
       </c>
       <c r="E36" s="13">
-        <v>220.02</v>
+        <v>221.26</v>
       </c>
       <c r="F36" s="13">
-        <v>229.02</v>
+        <v>230.26</v>
       </c>
       <c r="G36" s="17"/>
     </row>
     <row r="37" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A37" s="7">
-        <v>46323</v>
+        <v>46324</v>
       </c>
       <c r="B37" s="8"/>
       <c r="C37" s="20" t="s">
         <v>24</v>
       </c>
       <c r="D37" s="10">
-        <v>276.47000000000003</v>
+        <v>276.58</v>
       </c>
       <c r="E37" s="10" t="s">
         <v>18</v>
@@ -1358,14 +1358,14 @@
     </row>
     <row r="38" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A38" s="11">
-        <v>46322</v>
+        <v>46323</v>
       </c>
       <c r="B38" s="12"/>
       <c r="C38" s="12" t="s">
         <v>24</v>
       </c>
       <c r="D38" s="13">
-        <v>275.27999999999997</v>
+        <v>276.47000000000003</v>
       </c>
       <c r="E38" s="13" t="s">
         <v>18</v>
@@ -1416,77 +1416,77 @@
     </row>
     <row r="42" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A42" s="7">
-        <v>46323</v>
+        <v>46324</v>
       </c>
       <c r="B42" s="8"/>
       <c r="C42" s="20" t="s">
         <v>26</v>
       </c>
       <c r="D42" s="10">
-        <v>270.95999999999998</v>
+        <v>271.07</v>
       </c>
       <c r="E42" s="10">
-        <v>232.8</v>
+        <v>234.03</v>
       </c>
       <c r="F42" s="10">
-        <v>242.8</v>
+        <v>244.03</v>
       </c>
       <c r="G42" s="17"/>
     </row>
     <row r="43" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A43" s="11">
-        <v>46323</v>
+        <v>46324</v>
       </c>
       <c r="B43" s="12"/>
       <c r="C43" s="21" t="s">
         <v>27</v>
       </c>
       <c r="D43" s="13">
-        <v>270.57</v>
+        <v>270.67</v>
       </c>
       <c r="E43" s="13">
-        <v>233.21</v>
+        <v>234.44</v>
       </c>
       <c r="F43" s="13">
-        <v>243.21</v>
+        <v>244.44</v>
       </c>
       <c r="G43" s="17"/>
     </row>
     <row r="44" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A44" s="7">
-        <v>46322</v>
+        <v>46323</v>
       </c>
       <c r="B44" s="8"/>
       <c r="C44" s="20" t="s">
         <v>26</v>
       </c>
       <c r="D44" s="10">
-        <v>269.79000000000002</v>
+        <v>270.95999999999998</v>
       </c>
       <c r="E44" s="10">
-        <v>231.2</v>
+        <v>232.8</v>
       </c>
       <c r="F44" s="10">
-        <v>241.2</v>
+        <v>242.8</v>
       </c>
       <c r="G44" s="17"/>
     </row>
     <row r="45" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A45" s="11">
-        <v>46322</v>
+        <v>46323</v>
       </c>
       <c r="B45" s="12"/>
       <c r="C45" s="21" t="s">
         <v>27</v>
       </c>
       <c r="D45" s="13">
-        <v>269.39</v>
+        <v>270.57</v>
       </c>
       <c r="E45" s="13">
-        <v>231.61</v>
+        <v>233.21</v>
       </c>
       <c r="F45" s="13">
-        <v>241.61</v>
+        <v>243.21</v>
       </c>
       <c r="G45" s="17"/>
     </row>
@@ -1531,77 +1531,77 @@
     </row>
     <row r="49" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A49" s="7">
-        <v>46323</v>
+        <v>46324</v>
       </c>
       <c r="B49" s="8"/>
       <c r="C49" s="20" t="s">
         <v>29</v>
       </c>
       <c r="D49" s="10">
-        <v>261.45</v>
+        <v>262.76</v>
       </c>
       <c r="E49" s="10">
-        <v>221.55</v>
+        <v>223.28</v>
       </c>
       <c r="F49" s="10">
-        <v>231.55</v>
+        <v>233.28</v>
       </c>
       <c r="G49" s="28"/>
     </row>
     <row r="50" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A50" s="11">
-        <v>46323</v>
+        <v>46324</v>
       </c>
       <c r="B50" s="12"/>
       <c r="C50" s="21" t="s">
         <v>30</v>
       </c>
       <c r="D50" s="13">
-        <v>258.93</v>
+        <v>260.24</v>
       </c>
       <c r="E50" s="13">
-        <v>221.12</v>
+        <v>222.86</v>
       </c>
       <c r="F50" s="13">
-        <v>231.12</v>
+        <v>232.86</v>
       </c>
       <c r="G50" s="28"/>
     </row>
     <row r="51" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A51" s="7">
-        <v>46322</v>
+        <v>46323</v>
       </c>
       <c r="B51" s="8"/>
       <c r="C51" s="20" t="s">
         <v>29</v>
       </c>
       <c r="D51" s="10">
-        <v>260.60000000000002</v>
+        <v>261.45</v>
       </c>
       <c r="E51" s="10">
-        <v>220.83</v>
+        <v>221.55</v>
       </c>
       <c r="F51" s="10">
-        <v>230.83</v>
+        <v>231.55</v>
       </c>
       <c r="G51" s="17"/>
     </row>
     <row r="52" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A52" s="11">
-        <v>46322</v>
+        <v>46323</v>
       </c>
       <c r="B52" s="12"/>
       <c r="C52" s="21" t="s">
         <v>30</v>
       </c>
       <c r="D52" s="13">
-        <v>258.08</v>
+        <v>258.93</v>
       </c>
       <c r="E52" s="13">
-        <v>220.41</v>
+        <v>221.12</v>
       </c>
       <c r="F52" s="13">
-        <v>230.41</v>
+        <v>231.12</v>
       </c>
       <c r="G52" s="17"/>
     </row>
@@ -1646,52 +1646,52 @@
     </row>
     <row r="56" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A56" s="7">
-        <v>46323</v>
+        <v>46324</v>
       </c>
       <c r="B56" s="8"/>
       <c r="C56" s="20" t="s">
         <v>32</v>
       </c>
       <c r="D56" s="10">
-        <v>276.92</v>
+        <v>277.02</v>
       </c>
       <c r="E56" s="10">
-        <v>249.57</v>
+        <v>250.81</v>
       </c>
       <c r="F56" s="10">
-        <v>259.57</v>
+        <v>260.81</v>
       </c>
       <c r="G56" s="17"/>
     </row>
     <row r="57" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A57" s="11">
-        <v>46323</v>
+        <v>46324</v>
       </c>
       <c r="B57" s="12"/>
       <c r="C57" s="21" t="s">
         <v>33</v>
       </c>
       <c r="D57" s="13">
-        <v>264.39999999999998</v>
+        <v>264.5</v>
       </c>
       <c r="E57" s="13">
-        <v>230.35</v>
+        <v>231.56</v>
       </c>
       <c r="F57" s="13">
-        <v>240.35</v>
+        <v>241.56</v>
       </c>
       <c r="G57" s="17"/>
     </row>
     <row r="58" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A58" s="7">
-        <v>46323</v>
+        <v>46324</v>
       </c>
       <c r="B58" s="8"/>
       <c r="C58" s="20" t="s">
         <v>34</v>
       </c>
       <c r="D58" s="10">
-        <v>265.19</v>
+        <v>265.3</v>
       </c>
       <c r="E58" s="10" t="s">
         <v>18</v>
@@ -1703,17 +1703,17 @@
     </row>
     <row r="59" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A59" s="11">
-        <v>46323</v>
+        <v>46324</v>
       </c>
       <c r="B59" s="12"/>
       <c r="C59" s="21" t="s">
         <v>35</v>
       </c>
       <c r="D59" s="13">
-        <v>261.25</v>
+        <v>261.35000000000002</v>
       </c>
       <c r="E59" s="13">
-        <v>224.73</v>
+        <v>225.94</v>
       </c>
       <c r="F59" s="13" t="s">
         <v>18</v>
@@ -1722,36 +1722,36 @@
     </row>
     <row r="60" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A60" s="7">
-        <v>46323</v>
+        <v>46324</v>
       </c>
       <c r="B60" s="8"/>
       <c r="C60" s="20" t="s">
         <v>36</v>
       </c>
       <c r="D60" s="10">
-        <v>257.08999999999997</v>
+        <v>257.19</v>
       </c>
       <c r="E60" s="10">
-        <v>220.67</v>
+        <v>221.88</v>
       </c>
       <c r="F60" s="10">
-        <v>230.67</v>
+        <v>231.88</v>
       </c>
       <c r="G60" s="17"/>
     </row>
     <row r="61" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A61" s="11">
-        <v>46323</v>
+        <v>46324</v>
       </c>
       <c r="B61" s="12"/>
       <c r="C61" s="21" t="s">
         <v>37</v>
       </c>
       <c r="D61" s="13">
-        <v>264.7</v>
+        <v>264.81</v>
       </c>
       <c r="E61" s="13">
-        <v>242.64</v>
+        <v>243.87</v>
       </c>
       <c r="F61" s="13" t="s">
         <v>18</v>
@@ -1760,52 +1760,52 @@
     </row>
     <row r="62" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A62" s="7">
-        <v>46322</v>
+        <v>46323</v>
       </c>
       <c r="B62" s="8"/>
       <c r="C62" s="20" t="s">
         <v>32</v>
       </c>
       <c r="D62" s="10">
-        <v>275.72000000000003</v>
+        <v>276.92</v>
       </c>
       <c r="E62" s="10">
-        <v>248.42</v>
+        <v>249.57</v>
       </c>
       <c r="F62" s="10">
-        <v>258.42</v>
+        <v>259.57</v>
       </c>
       <c r="G62" s="17"/>
     </row>
     <row r="63" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A63" s="11">
-        <v>46322</v>
+        <v>46323</v>
       </c>
       <c r="B63" s="12"/>
       <c r="C63" s="21" t="s">
         <v>33</v>
       </c>
       <c r="D63" s="13">
-        <v>263.20999999999998</v>
+        <v>264.39999999999998</v>
       </c>
       <c r="E63" s="13">
-        <v>229.08</v>
+        <v>230.35</v>
       </c>
       <c r="F63" s="13">
-        <v>239.08</v>
+        <v>240.35</v>
       </c>
       <c r="G63" s="17"/>
     </row>
     <row r="64" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A64" s="7">
-        <v>46322</v>
+        <v>46323</v>
       </c>
       <c r="B64" s="8"/>
       <c r="C64" s="20" t="s">
         <v>34</v>
       </c>
       <c r="D64" s="10">
-        <v>264.01</v>
+        <v>265.19</v>
       </c>
       <c r="E64" s="10" t="s">
         <v>18</v>
@@ -1817,17 +1817,17 @@
     </row>
     <row r="65" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A65" s="11">
-        <v>46322</v>
+        <v>46323</v>
       </c>
       <c r="B65" s="12"/>
       <c r="C65" s="21" t="s">
         <v>35</v>
       </c>
       <c r="D65" s="13">
-        <v>260.02999999999997</v>
+        <v>261.25</v>
       </c>
       <c r="E65" s="13">
-        <v>223.46</v>
+        <v>224.73</v>
       </c>
       <c r="F65" s="13" t="s">
         <v>18</v>
@@ -1835,35 +1835,35 @@
     </row>
     <row r="66" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A66" s="7">
-        <v>46322</v>
+        <v>46323</v>
       </c>
       <c r="B66" s="8"/>
       <c r="C66" s="20" t="s">
         <v>36</v>
       </c>
       <c r="D66" s="10">
-        <v>255.86</v>
+        <v>257.08999999999997</v>
       </c>
       <c r="E66" s="10">
-        <v>219.4</v>
+        <v>220.67</v>
       </c>
       <c r="F66" s="10">
-        <v>229.4</v>
+        <v>230.67</v>
       </c>
     </row>
     <row r="67" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A67" s="11">
-        <v>46322</v>
+        <v>46323</v>
       </c>
       <c r="B67" s="12"/>
       <c r="C67" s="21" t="s">
         <v>37</v>
       </c>
       <c r="D67" s="13">
-        <v>263.47000000000003</v>
+        <v>264.7</v>
       </c>
       <c r="E67" s="13">
-        <v>241.44</v>
+        <v>242.64</v>
       </c>
       <c r="F67" s="13" t="s">
         <v>18</v>
@@ -1891,26 +1891,6 @@
 </file>
 
 <file path=customXml/item1.xml><?xml version="1.0" encoding="utf-8"?>
-<p:properties xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls">
-  <documentManagement>
-    <lcf76f155ced4ddcb4097134ff3c332f xmlns="87276d81-85f4-4ef2-9e6e-55066304288f">
-      <Terms xmlns="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
-    </lcf76f155ced4ddcb4097134ff3c332f>
-    <TaxCatchAll xmlns="b23b8984-eafa-4e79-985e-54f52f3da58e" xsi:nil="true"/>
-  </documentManagement>
-</p:properties>
-</file>
-
-<file path=customXml/item2.xml><?xml version="1.0" encoding="utf-8"?>
-<?mso-contentType ?>
-<FormTemplates xmlns="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms">
-  <Display>DocumentLibraryForm</Display>
-  <Edit>DocumentLibraryForm</Edit>
-  <New>DocumentLibraryForm</New>
-</FormTemplates>
-</file>
-
-<file path=customXml/item3.xml><?xml version="1.0" encoding="utf-8"?>
 <ct:contentTypeSchema xmlns:ct="http://schemas.microsoft.com/office/2006/metadata/contentType" xmlns:ma="http://schemas.microsoft.com/office/2006/metadata/properties/metaAttributes" ct:_="" ma:_="" ma:contentTypeName="Document" ma:contentTypeID="0x010100D3632DF5622958439304627C030B0427" ma:contentTypeVersion="18" ma:contentTypeDescription="Create a new document." ma:contentTypeScope="" ma:versionID="8c2ecbce386d6bac497f8eb2d8f0fb7a">
   <xsd:schema xmlns:xsd="http://www.w3.org/2001/XMLSchema" xmlns:xs="http://www.w3.org/2001/XMLSchema" xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:ns2="87276d81-85f4-4ef2-9e6e-55066304288f" xmlns:ns3="39e1dda6-d1d8-4c88-a3b9-f1abc1284bad" xmlns:ns4="b23b8984-eafa-4e79-985e-54f52f3da58e" targetNamespace="http://schemas.microsoft.com/office/2006/metadata/properties" ma:root="true" ma:fieldsID="4cfd0c2f651c1ce156ad4fcb44ea61dd" ns2:_="" ns3:_="" ns4:_="">
     <xsd:import namespace="87276d81-85f4-4ef2-9e6e-55066304288f"/>
@@ -2170,26 +2150,27 @@
 </ct:contentTypeSchema>
 </file>
 
-<file path=customXml/itemProps1.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{57A83D98-2BAE-4D83-823A-D31C464B620C}">
-  <ds:schemaRefs>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/properties"/>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
-    <ds:schemaRef ds:uri="87276d81-85f4-4ef2-9e6e-55066304288f"/>
-    <ds:schemaRef ds:uri="b23b8984-eafa-4e79-985e-54f52f3da58e"/>
-  </ds:schemaRefs>
-</ds:datastoreItem>
+<file path=customXml/item2.xml><?xml version="1.0" encoding="utf-8"?>
+<p:properties xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls">
+  <documentManagement>
+    <lcf76f155ced4ddcb4097134ff3c332f xmlns="87276d81-85f4-4ef2-9e6e-55066304288f">
+      <Terms xmlns="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
+    </lcf76f155ced4ddcb4097134ff3c332f>
+    <TaxCatchAll xmlns="b23b8984-eafa-4e79-985e-54f52f3da58e" xsi:nil="true"/>
+  </documentManagement>
+</p:properties>
 </file>
 
-<file path=customXml/itemProps2.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{F60519E9-FD90-4339-869C-BC2F85719BB8}">
-  <ds:schemaRefs>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms"/>
-  </ds:schemaRefs>
-</ds:datastoreItem>
+<file path=customXml/item3.xml><?xml version="1.0" encoding="utf-8"?>
+<?mso-contentType ?>
+<FormTemplates xmlns="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms">
+  <Display>DocumentLibraryForm</Display>
+  <Edit>DocumentLibraryForm</Edit>
+  <New>DocumentLibraryForm</New>
+</FormTemplates>
 </file>
 
-<file path=customXml/itemProps3.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=customXml/itemProps1.xml><?xml version="1.0" encoding="utf-8"?>
 <ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{B44E1863-2778-41F9-ACBA-48420F931671}">
   <ds:schemaRefs>
     <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/contentType"/>
@@ -2209,6 +2190,25 @@
 </ds:datastoreItem>
 </file>
 
+<file path=customXml/itemProps2.xml><?xml version="1.0" encoding="utf-8"?>
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{57A83D98-2BAE-4D83-823A-D31C464B620C}">
+  <ds:schemaRefs>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/properties"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
+    <ds:schemaRef ds:uri="87276d81-85f4-4ef2-9e6e-55066304288f"/>
+    <ds:schemaRef ds:uri="b23b8984-eafa-4e79-985e-54f52f3da58e"/>
+  </ds:schemaRefs>
+</ds:datastoreItem>
+</file>
+
+<file path=customXml/itemProps3.xml><?xml version="1.0" encoding="utf-8"?>
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{F60519E9-FD90-4339-869C-BC2F85719BB8}">
+  <ds:schemaRefs>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms"/>
+  </ds:schemaRefs>
+</ds:datastoreItem>
+</file>
+
 <file path=docMetadata/LabelInfo.xml><?xml version="1.0" encoding="utf-8"?>
 <clbl:labelList xmlns:clbl="http://schemas.microsoft.com/office/2020/mipLabelMetadata">
   <clbl:label id="{569bf4a9-87bd-4dbf-a36c-1db5158e5def}" enabled="1" method="Privileged" siteId="{ea80952e-a476-42d4-aaf4-5457852b0f7e}" removed="0"/>

</xml_diff>

<commit_message>
Thu Oct 29 07:15:19 UTC 2026
</commit_message>
<xml_diff>
--- a/bp.com-content-dam-bp-country-sites-en_au-australia-home-products-services-pricing-tgp-excel.xlsx
+++ b/bp.com-content-dam-bp-country-sites-en_au-australia-home-products-services-pricing-tgp-excel.xlsx
@@ -8,14 +8,14 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://bp365.sharepoint.com/sites/WholesalePricing/Shared Documents/B2C/TGP/Daily TGP/Web TGP/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="14_{3B00F6F4-A812-4F69-8117-152783F825CB}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="14_{070D2867-47D3-47C8-9C5B-3EECDA49C555}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-28920" yWindow="-60" windowWidth="29040" windowHeight="15720" xr2:uid="{1B412EEF-F96D-4DF4-A4E9-C7F0F183C2FB}"/>
+    <workbookView xWindow="-8595" yWindow="-16320" windowWidth="29040" windowHeight="15720" xr2:uid="{1B412EEF-F96D-4DF4-A4E9-C7F0F183C2FB}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
   </sheets>
-  <calcPr calcId="191028" iterateDelta="1E-4"/>
+  <calcPr calcId="191028"/>
   <extLst>
     <ext xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" uri="{140A7094-0E35-4892-8432-C4D2E57EDEB5}">
       <x15:workbookPr chartTrackingRefBase="1"/>
@@ -715,15 +715,15 @@
     <pageSetUpPr fitToPage="1"/>
   </sheetPr>
   <dimension ref="A1:G67"/>
-  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <sheetFormatPr defaultRowHeight="14.25" x14ac:dyDescent="0.45"/>
   <cols>
-    <col min="1" max="1" width="76.42578125" bestFit="1" customWidth="1"/>
-    <col min="2" max="2" width="6.42578125"/>
-    <col min="3" max="3" width="18.140625" bestFit="1" customWidth="1"/>
-    <col min="4" max="7" width="7.140625" bestFit="1" customWidth="1"/>
+    <col min="1" max="1" width="76.3984375" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="6.3984375"/>
+    <col min="3" max="3" width="18.1328125" bestFit="1" customWidth="1"/>
+    <col min="4" max="7" width="7.1328125" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:7" ht="23.25" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:7" ht="22.15" x14ac:dyDescent="0.45">
       <c r="A1" s="30" t="s">
         <v>0</v>
       </c>
@@ -734,7 +734,7 @@
       <c r="F1" s="2"/>
       <c r="G1" s="2"/>
     </row>
-    <row r="2" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="2" spans="1:7" x14ac:dyDescent="0.45">
       <c r="A2" s="3"/>
       <c r="B2" s="1"/>
       <c r="C2" s="1"/>
@@ -743,7 +743,7 @@
       <c r="F2" s="2"/>
       <c r="G2" s="2"/>
     </row>
-    <row r="3" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="3" spans="1:7" x14ac:dyDescent="0.45">
       <c r="A3" s="3" t="s">
         <v>1</v>
       </c>
@@ -754,7 +754,7 @@
       <c r="F3" s="2"/>
       <c r="G3" s="2"/>
     </row>
-    <row r="4" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="4" spans="1:7" x14ac:dyDescent="0.45">
       <c r="A4" s="3" t="s">
         <v>2</v>
       </c>
@@ -765,7 +765,7 @@
       <c r="F4" s="2"/>
       <c r="G4" s="2"/>
     </row>
-    <row r="5" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="5" spans="1:7" x14ac:dyDescent="0.45">
       <c r="A5" s="3"/>
       <c r="B5" s="3"/>
       <c r="C5" s="1"/>
@@ -774,7 +774,7 @@
       <c r="F5" s="2"/>
       <c r="G5" s="2"/>
     </row>
-    <row r="6" spans="1:7" ht="20.25" x14ac:dyDescent="0.25">
+    <row r="6" spans="1:7" ht="20.25" x14ac:dyDescent="0.45">
       <c r="A6" s="29" t="s">
         <v>3</v>
       </c>
@@ -785,7 +785,7 @@
       <c r="F6" s="2"/>
       <c r="G6" s="2"/>
     </row>
-    <row r="7" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="7" spans="1:7" x14ac:dyDescent="0.45">
       <c r="A7" s="4" t="s">
         <v>4</v>
       </c>
@@ -806,133 +806,133 @@
         <v>9</v>
       </c>
     </row>
-    <row r="8" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="8" spans="1:7" x14ac:dyDescent="0.45">
       <c r="A8" s="7">
-        <v>46324</v>
+        <v>46325</v>
       </c>
       <c r="B8" s="8"/>
       <c r="C8" s="9" t="s">
         <v>10</v>
       </c>
       <c r="D8" s="10">
-        <v>264.29000000000002</v>
+        <v>263.52</v>
       </c>
       <c r="E8" s="10">
-        <v>222.63</v>
+        <v>223.6</v>
       </c>
       <c r="F8" s="10">
-        <v>232.63</v>
+        <v>233.6</v>
       </c>
       <c r="G8" s="10">
-        <v>220.24</v>
-      </c>
-    </row>
-    <row r="9" spans="1:7" x14ac:dyDescent="0.25">
+        <v>221.22</v>
+      </c>
+    </row>
+    <row r="9" spans="1:7" x14ac:dyDescent="0.45">
       <c r="A9" s="11">
-        <v>46324</v>
+        <v>46325</v>
       </c>
       <c r="B9" s="12"/>
       <c r="C9" s="12" t="s">
         <v>11</v>
       </c>
       <c r="D9" s="13">
-        <v>264.29000000000002</v>
+        <v>263.52</v>
       </c>
       <c r="E9" s="13">
-        <v>222.63</v>
+        <v>223.6</v>
       </c>
       <c r="F9" s="13">
-        <v>232.63</v>
+        <v>233.6</v>
       </c>
       <c r="G9" s="13">
-        <v>220.24</v>
-      </c>
-    </row>
-    <row r="10" spans="1:7" x14ac:dyDescent="0.25">
+        <v>221.22</v>
+      </c>
+    </row>
+    <row r="10" spans="1:7" x14ac:dyDescent="0.45">
       <c r="A10" s="7">
-        <v>46324</v>
+        <v>46325</v>
       </c>
       <c r="B10" s="8"/>
       <c r="C10" s="9" t="s">
         <v>12</v>
       </c>
       <c r="D10" s="10">
-        <v>262.39999999999998</v>
+        <v>260.48</v>
       </c>
       <c r="E10" s="10">
-        <v>223.52</v>
+        <v>224.47</v>
       </c>
       <c r="F10" s="10">
-        <v>233.52</v>
+        <v>234.47</v>
       </c>
       <c r="G10" s="10">
-        <v>221.93</v>
-      </c>
-    </row>
-    <row r="11" spans="1:7" x14ac:dyDescent="0.25">
+        <v>222.87</v>
+      </c>
+    </row>
+    <row r="11" spans="1:7" x14ac:dyDescent="0.45">
       <c r="A11" s="11">
-        <v>46323</v>
+        <v>46324</v>
       </c>
       <c r="B11" s="12"/>
       <c r="C11" s="12" t="s">
         <v>10</v>
       </c>
       <c r="D11" s="13">
-        <v>264.01</v>
+        <v>264.29000000000002</v>
       </c>
       <c r="E11" s="13">
-        <v>221.25</v>
+        <v>222.63</v>
       </c>
       <c r="F11" s="13">
-        <v>231.25</v>
+        <v>232.63</v>
       </c>
       <c r="G11" s="13">
-        <v>218.86</v>
-      </c>
-    </row>
-    <row r="12" spans="1:7" x14ac:dyDescent="0.25">
+        <v>220.24</v>
+      </c>
+    </row>
+    <row r="12" spans="1:7" x14ac:dyDescent="0.45">
       <c r="A12" s="7">
-        <v>46323</v>
+        <v>46324</v>
       </c>
       <c r="B12" s="8"/>
       <c r="C12" s="9" t="s">
         <v>11</v>
       </c>
       <c r="D12" s="10">
-        <v>264.01</v>
+        <v>264.29000000000002</v>
       </c>
       <c r="E12" s="10">
-        <v>221.25</v>
+        <v>222.63</v>
       </c>
       <c r="F12" s="10">
-        <v>231.25</v>
+        <v>232.63</v>
       </c>
       <c r="G12" s="10">
-        <v>218.86</v>
-      </c>
-    </row>
-    <row r="13" spans="1:7" x14ac:dyDescent="0.25">
+        <v>220.24</v>
+      </c>
+    </row>
+    <row r="13" spans="1:7" x14ac:dyDescent="0.45">
       <c r="A13" s="11">
-        <v>46323</v>
+        <v>46324</v>
       </c>
       <c r="B13" s="12"/>
       <c r="C13" s="12" t="s">
         <v>12</v>
       </c>
       <c r="D13" s="13">
-        <v>262.29000000000002</v>
+        <v>262.39999999999998</v>
       </c>
       <c r="E13" s="13">
-        <v>222.3</v>
+        <v>223.52</v>
       </c>
       <c r="F13" s="13">
-        <v>232.3</v>
+        <v>233.52</v>
       </c>
       <c r="G13" s="13">
-        <v>220.71</v>
-      </c>
-    </row>
-    <row r="14" spans="1:7" x14ac:dyDescent="0.25">
+        <v>221.93</v>
+      </c>
+    </row>
+    <row r="14" spans="1:7" x14ac:dyDescent="0.45">
       <c r="A14" s="14"/>
       <c r="B14" s="14"/>
       <c r="C14" s="15"/>
@@ -941,7 +941,7 @@
       <c r="F14" s="16"/>
       <c r="G14" s="16"/>
     </row>
-    <row r="15" spans="1:7" ht="20.25" x14ac:dyDescent="0.25">
+    <row r="15" spans="1:7" ht="20.25" x14ac:dyDescent="0.45">
       <c r="A15" s="29" t="s">
         <v>13</v>
       </c>
@@ -952,7 +952,7 @@
       <c r="F15" s="17"/>
       <c r="G15" s="17"/>
     </row>
-    <row r="16" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="16" spans="1:7" x14ac:dyDescent="0.45">
       <c r="A16" s="4" t="s">
         <v>4</v>
       </c>
@@ -971,45 +971,45 @@
       </c>
       <c r="G16" s="17"/>
     </row>
-    <row r="17" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="17" spans="1:7" x14ac:dyDescent="0.45">
       <c r="A17" s="7">
-        <v>46324</v>
+        <v>46325</v>
       </c>
       <c r="B17" s="8"/>
       <c r="C17" s="20" t="s">
         <v>14</v>
       </c>
       <c r="D17" s="10">
-        <v>265.72000000000003</v>
+        <v>263.83</v>
       </c>
       <c r="E17" s="10">
-        <v>226.35</v>
+        <v>227.31</v>
       </c>
       <c r="F17" s="10">
-        <v>236.35</v>
+        <v>237.31</v>
       </c>
       <c r="G17" s="17"/>
     </row>
-    <row r="18" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="18" spans="1:7" x14ac:dyDescent="0.45">
       <c r="A18" s="11">
-        <v>46323</v>
+        <v>46324</v>
       </c>
       <c r="B18" s="12"/>
       <c r="C18" s="12" t="s">
         <v>14</v>
       </c>
       <c r="D18" s="13">
-        <v>265.62</v>
+        <v>265.72000000000003</v>
       </c>
       <c r="E18" s="13">
-        <v>225.12</v>
+        <v>226.35</v>
       </c>
       <c r="F18" s="13">
-        <v>235.12</v>
+        <v>236.35</v>
       </c>
       <c r="G18" s="17"/>
     </row>
-    <row r="19" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="19" spans="1:7" x14ac:dyDescent="0.45">
       <c r="A19" s="14"/>
       <c r="B19" s="14"/>
       <c r="C19" s="15"/>
@@ -1018,7 +1018,7 @@
       <c r="F19" s="16"/>
       <c r="G19" s="17"/>
     </row>
-    <row r="20" spans="1:7" ht="20.25" x14ac:dyDescent="0.25">
+    <row r="20" spans="1:7" ht="20.25" x14ac:dyDescent="0.45">
       <c r="A20" s="29" t="s">
         <v>15</v>
       </c>
@@ -1029,7 +1029,7 @@
       <c r="F20" s="17"/>
       <c r="G20" s="17"/>
     </row>
-    <row r="21" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="21" spans="1:7" x14ac:dyDescent="0.45">
       <c r="A21" s="4" t="s">
         <v>4</v>
       </c>
@@ -1050,217 +1050,217 @@
         <v>9</v>
       </c>
     </row>
-    <row r="22" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="22" spans="1:7" x14ac:dyDescent="0.45">
       <c r="A22" s="7">
-        <v>46324</v>
+        <v>46325</v>
       </c>
       <c r="B22" s="8"/>
       <c r="C22" s="20" t="s">
         <v>16</v>
       </c>
       <c r="D22" s="10">
-        <v>264.86</v>
+        <v>264.08999999999997</v>
       </c>
       <c r="E22" s="10">
-        <v>221.67</v>
+        <v>222.64</v>
       </c>
       <c r="F22" s="10">
-        <v>231.27</v>
+        <v>232.24</v>
       </c>
       <c r="G22" s="10">
-        <v>218.04</v>
-      </c>
-    </row>
-    <row r="23" spans="1:7" x14ac:dyDescent="0.25">
+        <v>219.01</v>
+      </c>
+    </row>
+    <row r="23" spans="1:7" x14ac:dyDescent="0.45">
       <c r="A23" s="11">
-        <v>46324</v>
+        <v>46325</v>
       </c>
       <c r="B23" s="12"/>
       <c r="C23" s="21" t="s">
         <v>17</v>
       </c>
       <c r="D23" s="13">
-        <v>267.37</v>
+        <v>265.45</v>
       </c>
       <c r="E23" s="13">
-        <v>231.83</v>
+        <v>232.77</v>
       </c>
       <c r="F23" s="13">
-        <v>241.83</v>
+        <v>242.77</v>
       </c>
       <c r="G23" s="13" t="s">
         <v>18</v>
       </c>
     </row>
-    <row r="24" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="24" spans="1:7" x14ac:dyDescent="0.45">
       <c r="A24" s="7">
-        <v>46324</v>
+        <v>46325</v>
       </c>
       <c r="B24" s="8"/>
       <c r="C24" s="20" t="s">
         <v>19</v>
       </c>
       <c r="D24" s="10">
-        <v>267.7</v>
+        <v>265.77999999999997</v>
       </c>
       <c r="E24" s="10">
-        <v>231.1</v>
+        <v>232.04</v>
       </c>
       <c r="F24" s="10">
-        <v>241.1</v>
+        <v>242.04</v>
       </c>
       <c r="G24" s="10" t="s">
         <v>18</v>
       </c>
     </row>
-    <row r="25" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="25" spans="1:7" x14ac:dyDescent="0.45">
       <c r="A25" s="11">
-        <v>46324</v>
+        <v>46325</v>
       </c>
       <c r="B25" s="12"/>
       <c r="C25" s="21" t="s">
         <v>20</v>
       </c>
       <c r="D25" s="13">
-        <v>264.38</v>
+        <v>262.47000000000003</v>
       </c>
       <c r="E25" s="13">
-        <v>231.33</v>
+        <v>232.26</v>
       </c>
       <c r="F25" s="13">
-        <v>241.33</v>
+        <v>242.26</v>
       </c>
       <c r="G25" s="13">
-        <v>227.17</v>
-      </c>
-    </row>
-    <row r="26" spans="1:7" x14ac:dyDescent="0.25">
+        <v>228.1</v>
+      </c>
+    </row>
+    <row r="26" spans="1:7" x14ac:dyDescent="0.45">
       <c r="A26" s="7">
-        <v>46324</v>
+        <v>46325</v>
       </c>
       <c r="B26" s="8"/>
       <c r="C26" s="20" t="s">
         <v>21</v>
       </c>
       <c r="D26" s="10">
-        <v>265.87</v>
+        <v>263.95999999999998</v>
       </c>
       <c r="E26" s="10">
-        <v>232.77</v>
+        <v>233.71</v>
       </c>
       <c r="F26" s="10">
-        <v>242.77</v>
+        <v>243.71</v>
       </c>
       <c r="G26" s="10" t="s">
         <v>18</v>
       </c>
     </row>
-    <row r="27" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="27" spans="1:7" x14ac:dyDescent="0.45">
       <c r="A27" s="11">
-        <v>46323</v>
+        <v>46324</v>
       </c>
       <c r="B27" s="12"/>
       <c r="C27" s="12" t="s">
         <v>16</v>
       </c>
       <c r="D27" s="13">
-        <v>264.58</v>
+        <v>264.86</v>
       </c>
       <c r="E27" s="13">
-        <v>220.29</v>
+        <v>221.67</v>
       </c>
       <c r="F27" s="13">
-        <v>229.89</v>
+        <v>231.27</v>
       </c>
       <c r="G27" s="13">
-        <v>216.66</v>
-      </c>
-    </row>
-    <row r="28" spans="1:7" x14ac:dyDescent="0.25">
+        <v>218.04</v>
+      </c>
+    </row>
+    <row r="28" spans="1:7" x14ac:dyDescent="0.45">
       <c r="A28" s="7">
-        <v>46323</v>
+        <v>46324</v>
       </c>
       <c r="B28" s="8"/>
       <c r="C28" s="20" t="s">
         <v>17</v>
       </c>
       <c r="D28" s="10">
-        <v>267.26</v>
+        <v>267.37</v>
       </c>
       <c r="E28" s="22">
-        <v>230.61</v>
+        <v>231.83</v>
       </c>
       <c r="F28" s="22">
-        <v>240.61</v>
+        <v>241.83</v>
       </c>
       <c r="G28" s="22" t="s">
         <v>18</v>
       </c>
     </row>
-    <row r="29" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="29" spans="1:7" x14ac:dyDescent="0.45">
       <c r="A29" s="11">
-        <v>46323</v>
+        <v>46324</v>
       </c>
       <c r="B29" s="12"/>
       <c r="C29" s="12" t="s">
         <v>19</v>
       </c>
       <c r="D29" s="13">
-        <v>267.60000000000002</v>
+        <v>267.7</v>
       </c>
       <c r="E29" s="13">
-        <v>229.88</v>
+        <v>231.1</v>
       </c>
       <c r="F29" s="13">
-        <v>239.88</v>
+        <v>241.1</v>
       </c>
       <c r="G29" s="13" t="s">
         <v>18</v>
       </c>
     </row>
-    <row r="30" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="30" spans="1:7" x14ac:dyDescent="0.45">
       <c r="A30" s="7">
-        <v>46323</v>
+        <v>46324</v>
       </c>
       <c r="B30" s="8"/>
       <c r="C30" s="20" t="s">
         <v>20</v>
       </c>
       <c r="D30" s="10">
-        <v>264.27999999999997</v>
+        <v>264.38</v>
       </c>
       <c r="E30" s="22">
-        <v>230.1</v>
+        <v>231.33</v>
       </c>
       <c r="F30" s="22">
-        <v>240.1</v>
+        <v>241.33</v>
       </c>
       <c r="G30" s="22">
-        <v>225.94</v>
-      </c>
-    </row>
-    <row r="31" spans="1:7" x14ac:dyDescent="0.25">
+        <v>227.17</v>
+      </c>
+    </row>
+    <row r="31" spans="1:7" x14ac:dyDescent="0.45">
       <c r="A31" s="11">
-        <v>46323</v>
+        <v>46324</v>
       </c>
       <c r="B31" s="12"/>
       <c r="C31" s="12" t="s">
         <v>21</v>
       </c>
       <c r="D31" s="13">
-        <v>265.77</v>
+        <v>265.87</v>
       </c>
       <c r="E31" s="13">
-        <v>231.53</v>
+        <v>232.77</v>
       </c>
       <c r="F31" s="13">
-        <v>241.53</v>
+        <v>242.77</v>
       </c>
       <c r="G31" s="13" t="s">
         <v>18</v>
       </c>
     </row>
-    <row r="32" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="32" spans="1:7" x14ac:dyDescent="0.45">
       <c r="A32" s="14"/>
       <c r="B32" s="14"/>
       <c r="C32" s="15"/>
@@ -1269,7 +1269,7 @@
       <c r="F32" s="17"/>
       <c r="G32" s="17"/>
     </row>
-    <row r="33" spans="1:7" ht="20.25" x14ac:dyDescent="0.25">
+    <row r="33" spans="1:7" ht="20.25" x14ac:dyDescent="0.45">
       <c r="A33" s="29" t="s">
         <v>22</v>
       </c>
@@ -1280,7 +1280,7 @@
       <c r="F33" s="17"/>
       <c r="G33" s="17"/>
     </row>
-    <row r="34" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="34" spans="1:7" x14ac:dyDescent="0.45">
       <c r="A34" s="23" t="s">
         <v>4</v>
       </c>
@@ -1299,54 +1299,54 @@
       </c>
       <c r="G34" s="17"/>
     </row>
-    <row r="35" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="35" spans="1:7" x14ac:dyDescent="0.45">
       <c r="A35" s="7">
-        <v>46324</v>
+        <v>46325</v>
       </c>
       <c r="B35" s="8"/>
       <c r="C35" s="20" t="s">
         <v>23</v>
       </c>
       <c r="D35" s="10">
-        <v>260.95999999999998</v>
+        <v>259.04000000000002</v>
       </c>
       <c r="E35" s="10">
-        <v>222.49</v>
+        <v>223.43</v>
       </c>
       <c r="F35" s="10">
-        <v>231.49</v>
+        <v>232.43</v>
       </c>
       <c r="G35" s="17"/>
     </row>
-    <row r="36" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="36" spans="1:7" x14ac:dyDescent="0.45">
       <c r="A36" s="11">
-        <v>46323</v>
+        <v>46324</v>
       </c>
       <c r="B36" s="12"/>
       <c r="C36" s="12" t="s">
         <v>23</v>
       </c>
       <c r="D36" s="13">
-        <v>260.85000000000002</v>
+        <v>260.95999999999998</v>
       </c>
       <c r="E36" s="13">
-        <v>221.26</v>
+        <v>222.49</v>
       </c>
       <c r="F36" s="13">
-        <v>230.26</v>
+        <v>231.49</v>
       </c>
       <c r="G36" s="17"/>
     </row>
-    <row r="37" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="37" spans="1:7" x14ac:dyDescent="0.45">
       <c r="A37" s="7">
-        <v>46324</v>
+        <v>46325</v>
       </c>
       <c r="B37" s="8"/>
       <c r="C37" s="20" t="s">
         <v>24</v>
       </c>
       <c r="D37" s="10">
-        <v>276.58</v>
+        <v>274.66000000000003</v>
       </c>
       <c r="E37" s="10" t="s">
         <v>18</v>
@@ -1356,16 +1356,16 @@
       </c>
       <c r="G37" s="17"/>
     </row>
-    <row r="38" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="38" spans="1:7" x14ac:dyDescent="0.45">
       <c r="A38" s="11">
-        <v>46323</v>
+        <v>46324</v>
       </c>
       <c r="B38" s="12"/>
       <c r="C38" s="12" t="s">
         <v>24</v>
       </c>
       <c r="D38" s="13">
-        <v>276.47000000000003</v>
+        <v>276.58</v>
       </c>
       <c r="E38" s="13" t="s">
         <v>18</v>
@@ -1375,7 +1375,7 @@
       </c>
       <c r="G38" s="17"/>
     </row>
-    <row r="39" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="39" spans="1:7" x14ac:dyDescent="0.45">
       <c r="A39" s="24"/>
       <c r="B39" s="24"/>
       <c r="C39" s="15"/>
@@ -1384,7 +1384,7 @@
       <c r="F39" s="17"/>
       <c r="G39" s="17"/>
     </row>
-    <row r="40" spans="1:7" ht="20.25" x14ac:dyDescent="0.25">
+    <row r="40" spans="1:7" ht="20.25" x14ac:dyDescent="0.45">
       <c r="A40" s="29" t="s">
         <v>25</v>
       </c>
@@ -1395,7 +1395,7 @@
       <c r="F40" s="17"/>
       <c r="G40" s="17"/>
     </row>
-    <row r="41" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="41" spans="1:7" x14ac:dyDescent="0.45">
       <c r="A41" s="23" t="s">
         <v>4</v>
       </c>
@@ -1414,83 +1414,83 @@
       </c>
       <c r="G41" s="17"/>
     </row>
-    <row r="42" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="42" spans="1:7" x14ac:dyDescent="0.45">
       <c r="A42" s="7">
-        <v>46324</v>
+        <v>46325</v>
       </c>
       <c r="B42" s="8"/>
       <c r="C42" s="20" t="s">
         <v>26</v>
       </c>
       <c r="D42" s="10">
-        <v>271.07</v>
+        <v>269.13</v>
       </c>
       <c r="E42" s="10">
-        <v>234.03</v>
+        <v>234.96</v>
       </c>
       <c r="F42" s="10">
-        <v>244.03</v>
+        <v>244.96</v>
       </c>
       <c r="G42" s="17"/>
     </row>
-    <row r="43" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="43" spans="1:7" x14ac:dyDescent="0.45">
       <c r="A43" s="11">
-        <v>46324</v>
+        <v>46325</v>
       </c>
       <c r="B43" s="12"/>
       <c r="C43" s="21" t="s">
         <v>27</v>
       </c>
       <c r="D43" s="13">
-        <v>270.67</v>
+        <v>268.74</v>
       </c>
       <c r="E43" s="13">
-        <v>234.44</v>
+        <v>235.38</v>
       </c>
       <c r="F43" s="13">
-        <v>244.44</v>
+        <v>245.38</v>
       </c>
       <c r="G43" s="17"/>
     </row>
-    <row r="44" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="44" spans="1:7" x14ac:dyDescent="0.45">
       <c r="A44" s="7">
-        <v>46323</v>
+        <v>46324</v>
       </c>
       <c r="B44" s="8"/>
       <c r="C44" s="20" t="s">
         <v>26</v>
       </c>
       <c r="D44" s="10">
-        <v>270.95999999999998</v>
+        <v>271.07</v>
       </c>
       <c r="E44" s="10">
-        <v>232.8</v>
+        <v>234.03</v>
       </c>
       <c r="F44" s="10">
-        <v>242.8</v>
+        <v>244.03</v>
       </c>
       <c r="G44" s="17"/>
     </row>
-    <row r="45" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="45" spans="1:7" x14ac:dyDescent="0.45">
       <c r="A45" s="11">
-        <v>46323</v>
+        <v>46324</v>
       </c>
       <c r="B45" s="12"/>
       <c r="C45" s="21" t="s">
         <v>27</v>
       </c>
       <c r="D45" s="13">
-        <v>270.57</v>
+        <v>270.67</v>
       </c>
       <c r="E45" s="13">
-        <v>233.21</v>
+        <v>234.44</v>
       </c>
       <c r="F45" s="13">
-        <v>243.21</v>
+        <v>244.44</v>
       </c>
       <c r="G45" s="17"/>
     </row>
-    <row r="46" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="46" spans="1:7" x14ac:dyDescent="0.45">
       <c r="A46" s="14"/>
       <c r="B46" s="24"/>
       <c r="C46" s="15"/>
@@ -1499,7 +1499,7 @@
       <c r="F46" s="16"/>
       <c r="G46" s="17"/>
     </row>
-    <row r="47" spans="1:7" ht="20.25" x14ac:dyDescent="0.25">
+    <row r="47" spans="1:7" ht="20.25" x14ac:dyDescent="0.45">
       <c r="A47" s="25" t="s">
         <v>28</v>
       </c>
@@ -1510,7 +1510,7 @@
       <c r="F47" s="17"/>
       <c r="G47" s="17"/>
     </row>
-    <row r="48" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="48" spans="1:7" x14ac:dyDescent="0.45">
       <c r="A48" s="23" t="s">
         <v>4</v>
       </c>
@@ -1529,83 +1529,83 @@
       </c>
       <c r="G48" s="17"/>
     </row>
-    <row r="49" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="49" spans="1:7" x14ac:dyDescent="0.45">
       <c r="A49" s="7">
-        <v>46324</v>
+        <v>46325</v>
       </c>
       <c r="B49" s="8"/>
       <c r="C49" s="20" t="s">
         <v>29</v>
       </c>
       <c r="D49" s="10">
-        <v>262.76</v>
+        <v>263.20999999999998</v>
       </c>
       <c r="E49" s="10">
-        <v>223.28</v>
+        <v>223.93</v>
       </c>
       <c r="F49" s="10">
-        <v>233.28</v>
+        <v>233.93</v>
       </c>
       <c r="G49" s="28"/>
     </row>
-    <row r="50" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="50" spans="1:7" x14ac:dyDescent="0.45">
       <c r="A50" s="11">
-        <v>46324</v>
+        <v>46325</v>
       </c>
       <c r="B50" s="12"/>
       <c r="C50" s="21" t="s">
         <v>30</v>
       </c>
       <c r="D50" s="13">
-        <v>260.24</v>
+        <v>260.7</v>
       </c>
       <c r="E50" s="13">
-        <v>222.86</v>
+        <v>223.5</v>
       </c>
       <c r="F50" s="13">
-        <v>232.86</v>
+        <v>233.5</v>
       </c>
       <c r="G50" s="28"/>
     </row>
-    <row r="51" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="51" spans="1:7" x14ac:dyDescent="0.45">
       <c r="A51" s="7">
-        <v>46323</v>
+        <v>46324</v>
       </c>
       <c r="B51" s="8"/>
       <c r="C51" s="20" t="s">
         <v>29</v>
       </c>
       <c r="D51" s="10">
-        <v>261.45</v>
+        <v>262.76</v>
       </c>
       <c r="E51" s="10">
-        <v>221.55</v>
+        <v>223.28</v>
       </c>
       <c r="F51" s="10">
-        <v>231.55</v>
+        <v>233.28</v>
       </c>
       <c r="G51" s="17"/>
     </row>
-    <row r="52" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="52" spans="1:7" x14ac:dyDescent="0.45">
       <c r="A52" s="11">
-        <v>46323</v>
+        <v>46324</v>
       </c>
       <c r="B52" s="12"/>
       <c r="C52" s="21" t="s">
         <v>30</v>
       </c>
       <c r="D52" s="13">
-        <v>258.93</v>
+        <v>260.24</v>
       </c>
       <c r="E52" s="13">
-        <v>221.12</v>
+        <v>222.86</v>
       </c>
       <c r="F52" s="13">
-        <v>231.12</v>
+        <v>232.86</v>
       </c>
       <c r="G52" s="17"/>
     </row>
-    <row r="53" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="53" spans="1:7" x14ac:dyDescent="0.45">
       <c r="A53" s="14"/>
       <c r="B53" s="14"/>
       <c r="C53" s="15"/>
@@ -1614,7 +1614,7 @@
       <c r="F53" s="16"/>
       <c r="G53" s="17"/>
     </row>
-    <row r="54" spans="1:7" ht="20.25" x14ac:dyDescent="0.25">
+    <row r="54" spans="1:7" ht="20.25" x14ac:dyDescent="0.45">
       <c r="A54" s="27" t="s">
         <v>31</v>
       </c>
@@ -1625,7 +1625,7 @@
       <c r="F54" s="17"/>
       <c r="G54" s="17"/>
     </row>
-    <row r="55" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="55" spans="1:7" x14ac:dyDescent="0.45">
       <c r="A55" s="23" t="s">
         <v>4</v>
       </c>
@@ -1644,54 +1644,54 @@
       </c>
       <c r="G55" s="17"/>
     </row>
-    <row r="56" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="56" spans="1:7" x14ac:dyDescent="0.45">
       <c r="A56" s="7">
-        <v>46324</v>
+        <v>46325</v>
       </c>
       <c r="B56" s="8"/>
       <c r="C56" s="20" t="s">
         <v>32</v>
       </c>
       <c r="D56" s="10">
-        <v>277.02</v>
+        <v>275.10000000000002</v>
       </c>
       <c r="E56" s="10">
-        <v>250.81</v>
+        <v>251.67</v>
       </c>
       <c r="F56" s="10">
-        <v>260.81</v>
+        <v>261.67</v>
       </c>
       <c r="G56" s="17"/>
     </row>
-    <row r="57" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="57" spans="1:7" x14ac:dyDescent="0.45">
       <c r="A57" s="11">
-        <v>46324</v>
+        <v>46325</v>
       </c>
       <c r="B57" s="12"/>
       <c r="C57" s="21" t="s">
         <v>33</v>
       </c>
       <c r="D57" s="13">
-        <v>264.5</v>
+        <v>263.13</v>
       </c>
       <c r="E57" s="13">
-        <v>231.56</v>
+        <v>232.52</v>
       </c>
       <c r="F57" s="13">
-        <v>241.56</v>
+        <v>242.52</v>
       </c>
       <c r="G57" s="17"/>
     </row>
-    <row r="58" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="58" spans="1:7" x14ac:dyDescent="0.45">
       <c r="A58" s="7">
-        <v>46324</v>
+        <v>46325</v>
       </c>
       <c r="B58" s="8"/>
       <c r="C58" s="20" t="s">
         <v>34</v>
       </c>
       <c r="D58" s="10">
-        <v>265.3</v>
+        <v>263.93</v>
       </c>
       <c r="E58" s="10" t="s">
         <v>18</v>
@@ -1701,111 +1701,111 @@
       </c>
       <c r="G58" s="17"/>
     </row>
-    <row r="59" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="59" spans="1:7" x14ac:dyDescent="0.45">
       <c r="A59" s="11">
-        <v>46324</v>
+        <v>46325</v>
       </c>
       <c r="B59" s="12"/>
       <c r="C59" s="21" t="s">
         <v>35</v>
       </c>
       <c r="D59" s="13">
-        <v>261.35000000000002</v>
+        <v>260.02</v>
       </c>
       <c r="E59" s="13">
-        <v>225.94</v>
+        <v>226.9</v>
       </c>
       <c r="F59" s="13" t="s">
         <v>18</v>
       </c>
       <c r="G59" s="17"/>
     </row>
-    <row r="60" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="60" spans="1:7" x14ac:dyDescent="0.45">
       <c r="A60" s="7">
-        <v>46324</v>
+        <v>46325</v>
       </c>
       <c r="B60" s="8"/>
       <c r="C60" s="20" t="s">
         <v>36</v>
       </c>
       <c r="D60" s="10">
-        <v>257.19</v>
+        <v>255.85</v>
       </c>
       <c r="E60" s="10">
-        <v>221.88</v>
+        <v>222.84</v>
       </c>
       <c r="F60" s="10">
-        <v>231.88</v>
+        <v>232.84</v>
       </c>
       <c r="G60" s="17"/>
     </row>
-    <row r="61" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="61" spans="1:7" x14ac:dyDescent="0.45">
       <c r="A61" s="11">
-        <v>46324</v>
+        <v>46325</v>
       </c>
       <c r="B61" s="12"/>
       <c r="C61" s="21" t="s">
         <v>37</v>
       </c>
       <c r="D61" s="13">
-        <v>264.81</v>
+        <v>262.92</v>
       </c>
       <c r="E61" s="13">
-        <v>243.87</v>
+        <v>244.77</v>
       </c>
       <c r="F61" s="13" t="s">
         <v>18</v>
       </c>
       <c r="G61" s="17"/>
     </row>
-    <row r="62" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="62" spans="1:7" x14ac:dyDescent="0.45">
       <c r="A62" s="7">
-        <v>46323</v>
+        <v>46324</v>
       </c>
       <c r="B62" s="8"/>
       <c r="C62" s="20" t="s">
         <v>32</v>
       </c>
       <c r="D62" s="10">
-        <v>276.92</v>
+        <v>277.02</v>
       </c>
       <c r="E62" s="10">
-        <v>249.57</v>
+        <v>250.81</v>
       </c>
       <c r="F62" s="10">
-        <v>259.57</v>
+        <v>260.81</v>
       </c>
       <c r="G62" s="17"/>
     </row>
-    <row r="63" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="63" spans="1:7" x14ac:dyDescent="0.45">
       <c r="A63" s="11">
-        <v>46323</v>
+        <v>46324</v>
       </c>
       <c r="B63" s="12"/>
       <c r="C63" s="21" t="s">
         <v>33</v>
       </c>
       <c r="D63" s="13">
-        <v>264.39999999999998</v>
+        <v>264.5</v>
       </c>
       <c r="E63" s="13">
-        <v>230.35</v>
+        <v>231.56</v>
       </c>
       <c r="F63" s="13">
-        <v>240.35</v>
+        <v>241.56</v>
       </c>
       <c r="G63" s="17"/>
     </row>
-    <row r="64" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="64" spans="1:7" x14ac:dyDescent="0.45">
       <c r="A64" s="7">
-        <v>46323</v>
+        <v>46324</v>
       </c>
       <c r="B64" s="8"/>
       <c r="C64" s="20" t="s">
         <v>34</v>
       </c>
       <c r="D64" s="10">
-        <v>265.19</v>
+        <v>265.3</v>
       </c>
       <c r="E64" s="10" t="s">
         <v>18</v>
@@ -1815,55 +1815,55 @@
       </c>
       <c r="G64" s="17"/>
     </row>
-    <row r="65" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="65" spans="1:6" x14ac:dyDescent="0.45">
       <c r="A65" s="11">
-        <v>46323</v>
+        <v>46324</v>
       </c>
       <c r="B65" s="12"/>
       <c r="C65" s="21" t="s">
         <v>35</v>
       </c>
       <c r="D65" s="13">
-        <v>261.25</v>
+        <v>261.35000000000002</v>
       </c>
       <c r="E65" s="13">
-        <v>224.73</v>
+        <v>225.94</v>
       </c>
       <c r="F65" s="13" t="s">
         <v>18</v>
       </c>
     </row>
-    <row r="66" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="66" spans="1:6" x14ac:dyDescent="0.45">
       <c r="A66" s="7">
-        <v>46323</v>
+        <v>46324</v>
       </c>
       <c r="B66" s="8"/>
       <c r="C66" s="20" t="s">
         <v>36</v>
       </c>
       <c r="D66" s="10">
-        <v>257.08999999999997</v>
+        <v>257.19</v>
       </c>
       <c r="E66" s="10">
-        <v>220.67</v>
+        <v>221.88</v>
       </c>
       <c r="F66" s="10">
-        <v>230.67</v>
-      </c>
-    </row>
-    <row r="67" spans="1:6" x14ac:dyDescent="0.25">
+        <v>231.88</v>
+      </c>
+    </row>
+    <row r="67" spans="1:6" x14ac:dyDescent="0.45">
       <c r="A67" s="11">
-        <v>46323</v>
+        <v>46324</v>
       </c>
       <c r="B67" s="12"/>
       <c r="C67" s="21" t="s">
         <v>37</v>
       </c>
       <c r="D67" s="13">
-        <v>264.7</v>
+        <v>264.81</v>
       </c>
       <c r="E67" s="13">
-        <v>242.64</v>
+        <v>243.87</v>
       </c>
       <c r="F67" s="13" t="s">
         <v>18</v>
@@ -1891,6 +1891,17 @@
 </file>
 
 <file path=customXml/item1.xml><?xml version="1.0" encoding="utf-8"?>
+<p:properties xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls">
+  <documentManagement>
+    <lcf76f155ced4ddcb4097134ff3c332f xmlns="87276d81-85f4-4ef2-9e6e-55066304288f">
+      <Terms xmlns="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
+    </lcf76f155ced4ddcb4097134ff3c332f>
+    <TaxCatchAll xmlns="b23b8984-eafa-4e79-985e-54f52f3da58e" xsi:nil="true"/>
+  </documentManagement>
+</p:properties>
+</file>
+
+<file path=customXml/item2.xml><?xml version="1.0" encoding="utf-8"?>
 <ct:contentTypeSchema xmlns:ct="http://schemas.microsoft.com/office/2006/metadata/contentType" xmlns:ma="http://schemas.microsoft.com/office/2006/metadata/properties/metaAttributes" ct:_="" ma:_="" ma:contentTypeName="Document" ma:contentTypeID="0x010100D3632DF5622958439304627C030B0427" ma:contentTypeVersion="18" ma:contentTypeDescription="Create a new document." ma:contentTypeScope="" ma:versionID="8c2ecbce386d6bac497f8eb2d8f0fb7a">
   <xsd:schema xmlns:xsd="http://www.w3.org/2001/XMLSchema" xmlns:xs="http://www.w3.org/2001/XMLSchema" xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:ns2="87276d81-85f4-4ef2-9e6e-55066304288f" xmlns:ns3="39e1dda6-d1d8-4c88-a3b9-f1abc1284bad" xmlns:ns4="b23b8984-eafa-4e79-985e-54f52f3da58e" targetNamespace="http://schemas.microsoft.com/office/2006/metadata/properties" ma:root="true" ma:fieldsID="4cfd0c2f651c1ce156ad4fcb44ea61dd" ns2:_="" ns3:_="" ns4:_="">
     <xsd:import namespace="87276d81-85f4-4ef2-9e6e-55066304288f"/>
@@ -2150,17 +2161,6 @@
 </ct:contentTypeSchema>
 </file>
 
-<file path=customXml/item2.xml><?xml version="1.0" encoding="utf-8"?>
-<p:properties xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls">
-  <documentManagement>
-    <lcf76f155ced4ddcb4097134ff3c332f xmlns="87276d81-85f4-4ef2-9e6e-55066304288f">
-      <Terms xmlns="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
-    </lcf76f155ced4ddcb4097134ff3c332f>
-    <TaxCatchAll xmlns="b23b8984-eafa-4e79-985e-54f52f3da58e" xsi:nil="true"/>
-  </documentManagement>
-</p:properties>
-</file>
-
 <file path=customXml/item3.xml><?xml version="1.0" encoding="utf-8"?>
 <?mso-contentType ?>
 <FormTemplates xmlns="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms">
@@ -2171,6 +2171,17 @@
 </file>
 
 <file path=customXml/itemProps1.xml><?xml version="1.0" encoding="utf-8"?>
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{57A83D98-2BAE-4D83-823A-D31C464B620C}">
+  <ds:schemaRefs>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/properties"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
+    <ds:schemaRef ds:uri="87276d81-85f4-4ef2-9e6e-55066304288f"/>
+    <ds:schemaRef ds:uri="b23b8984-eafa-4e79-985e-54f52f3da58e"/>
+  </ds:schemaRefs>
+</ds:datastoreItem>
+</file>
+
+<file path=customXml/itemProps2.xml><?xml version="1.0" encoding="utf-8"?>
 <ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{B44E1863-2778-41F9-ACBA-48420F931671}">
   <ds:schemaRefs>
     <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/contentType"/>
@@ -2190,17 +2201,6 @@
 </ds:datastoreItem>
 </file>
 
-<file path=customXml/itemProps2.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{57A83D98-2BAE-4D83-823A-D31C464B620C}">
-  <ds:schemaRefs>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/properties"/>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
-    <ds:schemaRef ds:uri="87276d81-85f4-4ef2-9e6e-55066304288f"/>
-    <ds:schemaRef ds:uri="b23b8984-eafa-4e79-985e-54f52f3da58e"/>
-  </ds:schemaRefs>
-</ds:datastoreItem>
-</file>
-
 <file path=customXml/itemProps3.xml><?xml version="1.0" encoding="utf-8"?>
 <ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{F60519E9-FD90-4339-869C-BC2F85719BB8}">
   <ds:schemaRefs>

</xml_diff>

<commit_message>
Fri Oct 30 07:18:07 UTC 2026
</commit_message>
<xml_diff>
--- a/bp.com-content-dam-bp-country-sites-en_au-australia-home-products-services-pricing-tgp-excel.xlsx
+++ b/bp.com-content-dam-bp-country-sites-en_au-australia-home-products-services-pricing-tgp-excel.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="30326"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="30430"/>
   <workbookPr codeName="ThisWorkbook" defaultThemeVersion="166925"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://bp365.sharepoint.com/sites/WholesalePricing/Shared Documents/B2C/TGP/Daily TGP/Web TGP/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="14_{070D2867-47D3-47C8-9C5B-3EECDA49C555}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="14_{ABB54110-BA5D-41B1-94F0-C0982332FB93}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-8595" yWindow="-16320" windowWidth="29040" windowHeight="15720" xr2:uid="{1B412EEF-F96D-4DF4-A4E9-C7F0F183C2FB}"/>
+    <workbookView xWindow="-110" yWindow="-110" windowWidth="19420" windowHeight="11500" xr2:uid="{1B412EEF-F96D-4DF4-A4E9-C7F0F183C2FB}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
@@ -715,15 +715,15 @@
     <pageSetUpPr fitToPage="1"/>
   </sheetPr>
   <dimension ref="A1:G67"/>
-  <sheetFormatPr defaultRowHeight="14.25" x14ac:dyDescent="0.45"/>
+  <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
   <cols>
-    <col min="1" max="1" width="76.3984375" bestFit="1" customWidth="1"/>
-    <col min="2" max="2" width="6.3984375"/>
-    <col min="3" max="3" width="18.1328125" bestFit="1" customWidth="1"/>
-    <col min="4" max="7" width="7.1328125" bestFit="1" customWidth="1"/>
+    <col min="1" max="1" width="76.453125" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="6.453125"/>
+    <col min="3" max="3" width="18.08984375" bestFit="1" customWidth="1"/>
+    <col min="4" max="7" width="7.08984375" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:7" ht="22.15" x14ac:dyDescent="0.45">
+    <row r="1" spans="1:7" ht="22.5" x14ac:dyDescent="0.35">
       <c r="A1" s="30" t="s">
         <v>0</v>
       </c>
@@ -734,7 +734,7 @@
       <c r="F1" s="2"/>
       <c r="G1" s="2"/>
     </row>
-    <row r="2" spans="1:7" x14ac:dyDescent="0.45">
+    <row r="2" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A2" s="3"/>
       <c r="B2" s="1"/>
       <c r="C2" s="1"/>
@@ -743,7 +743,7 @@
       <c r="F2" s="2"/>
       <c r="G2" s="2"/>
     </row>
-    <row r="3" spans="1:7" x14ac:dyDescent="0.45">
+    <row r="3" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A3" s="3" t="s">
         <v>1</v>
       </c>
@@ -754,7 +754,7 @@
       <c r="F3" s="2"/>
       <c r="G3" s="2"/>
     </row>
-    <row r="4" spans="1:7" x14ac:dyDescent="0.45">
+    <row r="4" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A4" s="3" t="s">
         <v>2</v>
       </c>
@@ -765,7 +765,7 @@
       <c r="F4" s="2"/>
       <c r="G4" s="2"/>
     </row>
-    <row r="5" spans="1:7" x14ac:dyDescent="0.45">
+    <row r="5" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A5" s="3"/>
       <c r="B5" s="3"/>
       <c r="C5" s="1"/>
@@ -774,7 +774,7 @@
       <c r="F5" s="2"/>
       <c r="G5" s="2"/>
     </row>
-    <row r="6" spans="1:7" ht="20.25" x14ac:dyDescent="0.45">
+    <row r="6" spans="1:7" ht="20" x14ac:dyDescent="0.35">
       <c r="A6" s="29" t="s">
         <v>3</v>
       </c>
@@ -785,7 +785,7 @@
       <c r="F6" s="2"/>
       <c r="G6" s="2"/>
     </row>
-    <row r="7" spans="1:7" x14ac:dyDescent="0.45">
+    <row r="7" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A7" s="4" t="s">
         <v>4</v>
       </c>
@@ -806,133 +806,133 @@
         <v>9</v>
       </c>
     </row>
-    <row r="8" spans="1:7" x14ac:dyDescent="0.45">
+    <row r="8" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A8" s="7">
-        <v>46325</v>
+        <v>46326</v>
       </c>
       <c r="B8" s="8"/>
       <c r="C8" s="9" t="s">
         <v>10</v>
       </c>
       <c r="D8" s="10">
-        <v>263.52</v>
+        <v>261.8</v>
       </c>
       <c r="E8" s="10">
-        <v>223.6</v>
+        <v>224.04</v>
       </c>
       <c r="F8" s="10">
-        <v>233.6</v>
+        <v>234.04</v>
       </c>
       <c r="G8" s="10">
-        <v>221.22</v>
-      </c>
-    </row>
-    <row r="9" spans="1:7" x14ac:dyDescent="0.45">
+        <v>221.66</v>
+      </c>
+    </row>
+    <row r="9" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A9" s="11">
-        <v>46325</v>
+        <v>46326</v>
       </c>
       <c r="B9" s="12"/>
       <c r="C9" s="12" t="s">
         <v>11</v>
       </c>
       <c r="D9" s="13">
-        <v>263.52</v>
+        <v>261.8</v>
       </c>
       <c r="E9" s="13">
-        <v>223.6</v>
+        <v>224.04</v>
       </c>
       <c r="F9" s="13">
-        <v>233.6</v>
+        <v>234.04</v>
       </c>
       <c r="G9" s="13">
-        <v>221.22</v>
-      </c>
-    </row>
-    <row r="10" spans="1:7" x14ac:dyDescent="0.45">
+        <v>221.66</v>
+      </c>
+    </row>
+    <row r="10" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A10" s="7">
-        <v>46325</v>
+        <v>46326</v>
       </c>
       <c r="B10" s="8"/>
       <c r="C10" s="9" t="s">
         <v>12</v>
       </c>
       <c r="D10" s="10">
-        <v>260.48</v>
+        <v>258.3</v>
       </c>
       <c r="E10" s="10">
-        <v>224.47</v>
+        <v>224.43</v>
       </c>
       <c r="F10" s="10">
-        <v>234.47</v>
+        <v>234.43</v>
       </c>
       <c r="G10" s="10">
-        <v>222.87</v>
-      </c>
-    </row>
-    <row r="11" spans="1:7" x14ac:dyDescent="0.45">
+        <v>222.83</v>
+      </c>
+    </row>
+    <row r="11" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A11" s="11">
-        <v>46324</v>
+        <v>46325</v>
       </c>
       <c r="B11" s="12"/>
       <c r="C11" s="12" t="s">
         <v>10</v>
       </c>
       <c r="D11" s="13">
-        <v>264.29000000000002</v>
+        <v>263.52</v>
       </c>
       <c r="E11" s="13">
-        <v>222.63</v>
+        <v>223.6</v>
       </c>
       <c r="F11" s="13">
-        <v>232.63</v>
+        <v>233.6</v>
       </c>
       <c r="G11" s="13">
-        <v>220.24</v>
-      </c>
-    </row>
-    <row r="12" spans="1:7" x14ac:dyDescent="0.45">
+        <v>221.22</v>
+      </c>
+    </row>
+    <row r="12" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A12" s="7">
-        <v>46324</v>
+        <v>46325</v>
       </c>
       <c r="B12" s="8"/>
       <c r="C12" s="9" t="s">
         <v>11</v>
       </c>
       <c r="D12" s="10">
-        <v>264.29000000000002</v>
+        <v>263.52</v>
       </c>
       <c r="E12" s="10">
-        <v>222.63</v>
+        <v>223.6</v>
       </c>
       <c r="F12" s="10">
-        <v>232.63</v>
+        <v>233.6</v>
       </c>
       <c r="G12" s="10">
-        <v>220.24</v>
-      </c>
-    </row>
-    <row r="13" spans="1:7" x14ac:dyDescent="0.45">
+        <v>221.22</v>
+      </c>
+    </row>
+    <row r="13" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A13" s="11">
-        <v>46324</v>
+        <v>46325</v>
       </c>
       <c r="B13" s="12"/>
       <c r="C13" s="12" t="s">
         <v>12</v>
       </c>
       <c r="D13" s="13">
-        <v>262.39999999999998</v>
+        <v>260.48</v>
       </c>
       <c r="E13" s="13">
-        <v>223.52</v>
+        <v>224.47</v>
       </c>
       <c r="F13" s="13">
-        <v>233.52</v>
+        <v>234.47</v>
       </c>
       <c r="G13" s="13">
-        <v>221.93</v>
-      </c>
-    </row>
-    <row r="14" spans="1:7" x14ac:dyDescent="0.45">
+        <v>222.87</v>
+      </c>
+    </row>
+    <row r="14" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A14" s="14"/>
       <c r="B14" s="14"/>
       <c r="C14" s="15"/>
@@ -941,7 +941,7 @@
       <c r="F14" s="16"/>
       <c r="G14" s="16"/>
     </row>
-    <row r="15" spans="1:7" ht="20.25" x14ac:dyDescent="0.45">
+    <row r="15" spans="1:7" ht="20" x14ac:dyDescent="0.35">
       <c r="A15" s="29" t="s">
         <v>13</v>
       </c>
@@ -952,7 +952,7 @@
       <c r="F15" s="17"/>
       <c r="G15" s="17"/>
     </row>
-    <row r="16" spans="1:7" x14ac:dyDescent="0.45">
+    <row r="16" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A16" s="4" t="s">
         <v>4</v>
       </c>
@@ -971,45 +971,45 @@
       </c>
       <c r="G16" s="17"/>
     </row>
-    <row r="17" spans="1:7" x14ac:dyDescent="0.45">
+    <row r="17" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A17" s="7">
-        <v>46325</v>
+        <v>46326</v>
       </c>
       <c r="B17" s="8"/>
       <c r="C17" s="20" t="s">
         <v>14</v>
       </c>
       <c r="D17" s="10">
-        <v>263.83</v>
+        <v>261.69</v>
       </c>
       <c r="E17" s="10">
-        <v>227.31</v>
+        <v>227.32</v>
       </c>
       <c r="F17" s="10">
-        <v>237.31</v>
+        <v>237.32</v>
       </c>
       <c r="G17" s="17"/>
     </row>
-    <row r="18" spans="1:7" x14ac:dyDescent="0.45">
+    <row r="18" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A18" s="11">
-        <v>46324</v>
+        <v>46325</v>
       </c>
       <c r="B18" s="12"/>
       <c r="C18" s="12" t="s">
         <v>14</v>
       </c>
       <c r="D18" s="13">
-        <v>265.72000000000003</v>
+        <v>263.83</v>
       </c>
       <c r="E18" s="13">
-        <v>226.35</v>
+        <v>227.31</v>
       </c>
       <c r="F18" s="13">
-        <v>236.35</v>
+        <v>237.31</v>
       </c>
       <c r="G18" s="17"/>
     </row>
-    <row r="19" spans="1:7" x14ac:dyDescent="0.45">
+    <row r="19" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A19" s="14"/>
       <c r="B19" s="14"/>
       <c r="C19" s="15"/>
@@ -1018,7 +1018,7 @@
       <c r="F19" s="16"/>
       <c r="G19" s="17"/>
     </row>
-    <row r="20" spans="1:7" ht="20.25" x14ac:dyDescent="0.45">
+    <row r="20" spans="1:7" ht="20" x14ac:dyDescent="0.35">
       <c r="A20" s="29" t="s">
         <v>15</v>
       </c>
@@ -1029,7 +1029,7 @@
       <c r="F20" s="17"/>
       <c r="G20" s="17"/>
     </row>
-    <row r="21" spans="1:7" x14ac:dyDescent="0.45">
+    <row r="21" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A21" s="4" t="s">
         <v>4</v>
       </c>
@@ -1050,217 +1050,217 @@
         <v>9</v>
       </c>
     </row>
-    <row r="22" spans="1:7" x14ac:dyDescent="0.45">
+    <row r="22" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A22" s="7">
-        <v>46325</v>
+        <v>46326</v>
       </c>
       <c r="B22" s="8"/>
       <c r="C22" s="20" t="s">
         <v>16</v>
       </c>
       <c r="D22" s="10">
-        <v>264.08999999999997</v>
+        <v>262.37</v>
       </c>
       <c r="E22" s="10">
-        <v>222.64</v>
+        <v>223.08</v>
       </c>
       <c r="F22" s="10">
-        <v>232.24</v>
+        <v>232.68</v>
       </c>
       <c r="G22" s="10">
-        <v>219.01</v>
-      </c>
-    </row>
-    <row r="23" spans="1:7" x14ac:dyDescent="0.45">
+        <v>219.45</v>
+      </c>
+    </row>
+    <row r="23" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A23" s="11">
-        <v>46325</v>
+        <v>46326</v>
       </c>
       <c r="B23" s="12"/>
       <c r="C23" s="21" t="s">
         <v>17</v>
       </c>
       <c r="D23" s="13">
-        <v>265.45</v>
+        <v>263.26</v>
       </c>
       <c r="E23" s="13">
-        <v>232.77</v>
+        <v>232.71</v>
       </c>
       <c r="F23" s="13">
-        <v>242.77</v>
+        <v>242.72</v>
       </c>
       <c r="G23" s="13" t="s">
         <v>18</v>
       </c>
     </row>
-    <row r="24" spans="1:7" x14ac:dyDescent="0.45">
+    <row r="24" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A24" s="7">
-        <v>46325</v>
+        <v>46326</v>
       </c>
       <c r="B24" s="8"/>
       <c r="C24" s="20" t="s">
         <v>19</v>
       </c>
       <c r="D24" s="10">
-        <v>265.77999999999997</v>
+        <v>263.60000000000002</v>
       </c>
       <c r="E24" s="10">
-        <v>232.04</v>
+        <v>231.98</v>
       </c>
       <c r="F24" s="10">
-        <v>242.04</v>
+        <v>241.98</v>
       </c>
       <c r="G24" s="10" t="s">
         <v>18</v>
       </c>
     </row>
-    <row r="25" spans="1:7" x14ac:dyDescent="0.45">
+    <row r="25" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A25" s="11">
-        <v>46325</v>
+        <v>46326</v>
       </c>
       <c r="B25" s="12"/>
       <c r="C25" s="21" t="s">
         <v>20</v>
       </c>
       <c r="D25" s="13">
-        <v>262.47000000000003</v>
+        <v>260.29000000000002</v>
       </c>
       <c r="E25" s="13">
-        <v>232.26</v>
+        <v>232.2</v>
       </c>
       <c r="F25" s="13">
-        <v>242.26</v>
+        <v>242.2</v>
       </c>
       <c r="G25" s="13">
-        <v>228.1</v>
-      </c>
-    </row>
-    <row r="26" spans="1:7" x14ac:dyDescent="0.45">
+        <v>228.04</v>
+      </c>
+    </row>
+    <row r="26" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A26" s="7">
-        <v>46325</v>
+        <v>46326</v>
       </c>
       <c r="B26" s="8"/>
       <c r="C26" s="20" t="s">
         <v>21</v>
       </c>
       <c r="D26" s="10">
-        <v>263.95999999999998</v>
+        <v>261.79000000000002</v>
       </c>
       <c r="E26" s="10">
-        <v>233.71</v>
+        <v>233.65</v>
       </c>
       <c r="F26" s="10">
-        <v>243.71</v>
+        <v>243.65</v>
       </c>
       <c r="G26" s="10" t="s">
         <v>18</v>
       </c>
     </row>
-    <row r="27" spans="1:7" x14ac:dyDescent="0.45">
+    <row r="27" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A27" s="11">
-        <v>46324</v>
+        <v>46325</v>
       </c>
       <c r="B27" s="12"/>
       <c r="C27" s="12" t="s">
         <v>16</v>
       </c>
       <c r="D27" s="13">
-        <v>264.86</v>
+        <v>264.08999999999997</v>
       </c>
       <c r="E27" s="13">
-        <v>221.67</v>
+        <v>222.64</v>
       </c>
       <c r="F27" s="13">
-        <v>231.27</v>
+        <v>232.24</v>
       </c>
       <c r="G27" s="13">
-        <v>218.04</v>
-      </c>
-    </row>
-    <row r="28" spans="1:7" x14ac:dyDescent="0.45">
+        <v>219.01</v>
+      </c>
+    </row>
+    <row r="28" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A28" s="7">
-        <v>46324</v>
+        <v>46325</v>
       </c>
       <c r="B28" s="8"/>
       <c r="C28" s="20" t="s">
         <v>17</v>
       </c>
       <c r="D28" s="10">
-        <v>267.37</v>
+        <v>265.45</v>
       </c>
       <c r="E28" s="22">
-        <v>231.83</v>
+        <v>232.77</v>
       </c>
       <c r="F28" s="22">
-        <v>241.83</v>
+        <v>242.77</v>
       </c>
       <c r="G28" s="22" t="s">
         <v>18</v>
       </c>
     </row>
-    <row r="29" spans="1:7" x14ac:dyDescent="0.45">
+    <row r="29" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A29" s="11">
-        <v>46324</v>
+        <v>46325</v>
       </c>
       <c r="B29" s="12"/>
       <c r="C29" s="12" t="s">
         <v>19</v>
       </c>
       <c r="D29" s="13">
-        <v>267.7</v>
+        <v>265.77999999999997</v>
       </c>
       <c r="E29" s="13">
-        <v>231.1</v>
+        <v>232.04</v>
       </c>
       <c r="F29" s="13">
-        <v>241.1</v>
+        <v>242.04</v>
       </c>
       <c r="G29" s="13" t="s">
         <v>18</v>
       </c>
     </row>
-    <row r="30" spans="1:7" x14ac:dyDescent="0.45">
+    <row r="30" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A30" s="7">
-        <v>46324</v>
+        <v>46325</v>
       </c>
       <c r="B30" s="8"/>
       <c r="C30" s="20" t="s">
         <v>20</v>
       </c>
       <c r="D30" s="10">
-        <v>264.38</v>
+        <v>262.47000000000003</v>
       </c>
       <c r="E30" s="22">
-        <v>231.33</v>
+        <v>232.26</v>
       </c>
       <c r="F30" s="22">
-        <v>241.33</v>
+        <v>242.26</v>
       </c>
       <c r="G30" s="22">
-        <v>227.17</v>
-      </c>
-    </row>
-    <row r="31" spans="1:7" x14ac:dyDescent="0.45">
+        <v>228.1</v>
+      </c>
+    </row>
+    <row r="31" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A31" s="11">
-        <v>46324</v>
+        <v>46325</v>
       </c>
       <c r="B31" s="12"/>
       <c r="C31" s="12" t="s">
         <v>21</v>
       </c>
       <c r="D31" s="13">
-        <v>265.87</v>
+        <v>263.95999999999998</v>
       </c>
       <c r="E31" s="13">
-        <v>232.77</v>
+        <v>233.71</v>
       </c>
       <c r="F31" s="13">
-        <v>242.77</v>
+        <v>243.71</v>
       </c>
       <c r="G31" s="13" t="s">
         <v>18</v>
       </c>
     </row>
-    <row r="32" spans="1:7" x14ac:dyDescent="0.45">
+    <row r="32" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A32" s="14"/>
       <c r="B32" s="14"/>
       <c r="C32" s="15"/>
@@ -1269,7 +1269,7 @@
       <c r="F32" s="17"/>
       <c r="G32" s="17"/>
     </row>
-    <row r="33" spans="1:7" ht="20.25" x14ac:dyDescent="0.45">
+    <row r="33" spans="1:7" ht="20" x14ac:dyDescent="0.35">
       <c r="A33" s="29" t="s">
         <v>22</v>
       </c>
@@ -1280,7 +1280,7 @@
       <c r="F33" s="17"/>
       <c r="G33" s="17"/>
     </row>
-    <row r="34" spans="1:7" x14ac:dyDescent="0.45">
+    <row r="34" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A34" s="23" t="s">
         <v>4</v>
       </c>
@@ -1299,54 +1299,54 @@
       </c>
       <c r="G34" s="17"/>
     </row>
-    <row r="35" spans="1:7" x14ac:dyDescent="0.45">
+    <row r="35" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A35" s="7">
-        <v>46325</v>
+        <v>46326</v>
       </c>
       <c r="B35" s="8"/>
       <c r="C35" s="20" t="s">
         <v>23</v>
       </c>
       <c r="D35" s="10">
-        <v>259.04000000000002</v>
+        <v>256.86</v>
       </c>
       <c r="E35" s="10">
-        <v>223.43</v>
+        <v>223.39</v>
       </c>
       <c r="F35" s="10">
-        <v>232.43</v>
+        <v>232.39</v>
       </c>
       <c r="G35" s="17"/>
     </row>
-    <row r="36" spans="1:7" x14ac:dyDescent="0.45">
+    <row r="36" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A36" s="11">
-        <v>46324</v>
+        <v>46325</v>
       </c>
       <c r="B36" s="12"/>
       <c r="C36" s="12" t="s">
         <v>23</v>
       </c>
       <c r="D36" s="13">
-        <v>260.95999999999998</v>
+        <v>259.04000000000002</v>
       </c>
       <c r="E36" s="13">
-        <v>222.49</v>
+        <v>223.43</v>
       </c>
       <c r="F36" s="13">
-        <v>231.49</v>
+        <v>232.43</v>
       </c>
       <c r="G36" s="17"/>
     </row>
-    <row r="37" spans="1:7" x14ac:dyDescent="0.45">
+    <row r="37" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A37" s="7">
-        <v>46325</v>
+        <v>46326</v>
       </c>
       <c r="B37" s="8"/>
       <c r="C37" s="20" t="s">
         <v>24</v>
       </c>
       <c r="D37" s="10">
-        <v>274.66000000000003</v>
+        <v>272.48</v>
       </c>
       <c r="E37" s="10" t="s">
         <v>18</v>
@@ -1356,16 +1356,16 @@
       </c>
       <c r="G37" s="17"/>
     </row>
-    <row r="38" spans="1:7" x14ac:dyDescent="0.45">
+    <row r="38" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A38" s="11">
-        <v>46324</v>
+        <v>46325</v>
       </c>
       <c r="B38" s="12"/>
       <c r="C38" s="12" t="s">
         <v>24</v>
       </c>
       <c r="D38" s="13">
-        <v>276.58</v>
+        <v>274.66000000000003</v>
       </c>
       <c r="E38" s="13" t="s">
         <v>18</v>
@@ -1375,7 +1375,7 @@
       </c>
       <c r="G38" s="17"/>
     </row>
-    <row r="39" spans="1:7" x14ac:dyDescent="0.45">
+    <row r="39" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A39" s="24"/>
       <c r="B39" s="24"/>
       <c r="C39" s="15"/>
@@ -1384,7 +1384,7 @@
       <c r="F39" s="17"/>
       <c r="G39" s="17"/>
     </row>
-    <row r="40" spans="1:7" ht="20.25" x14ac:dyDescent="0.45">
+    <row r="40" spans="1:7" ht="20" x14ac:dyDescent="0.35">
       <c r="A40" s="29" t="s">
         <v>25</v>
       </c>
@@ -1395,7 +1395,7 @@
       <c r="F40" s="17"/>
       <c r="G40" s="17"/>
     </row>
-    <row r="41" spans="1:7" x14ac:dyDescent="0.45">
+    <row r="41" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A41" s="23" t="s">
         <v>4</v>
       </c>
@@ -1414,83 +1414,83 @@
       </c>
       <c r="G41" s="17"/>
     </row>
-    <row r="42" spans="1:7" x14ac:dyDescent="0.45">
+    <row r="42" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A42" s="7">
-        <v>46325</v>
+        <v>46326</v>
       </c>
       <c r="B42" s="8"/>
       <c r="C42" s="20" t="s">
         <v>26</v>
       </c>
       <c r="D42" s="10">
-        <v>269.13</v>
+        <v>266.91000000000003</v>
       </c>
       <c r="E42" s="10">
-        <v>234.96</v>
+        <v>234.9</v>
       </c>
       <c r="F42" s="10">
-        <v>244.96</v>
+        <v>244.9</v>
       </c>
       <c r="G42" s="17"/>
     </row>
-    <row r="43" spans="1:7" x14ac:dyDescent="0.45">
+    <row r="43" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A43" s="11">
-        <v>46325</v>
+        <v>46326</v>
       </c>
       <c r="B43" s="12"/>
       <c r="C43" s="21" t="s">
         <v>27</v>
       </c>
       <c r="D43" s="13">
-        <v>268.74</v>
+        <v>266.52</v>
       </c>
       <c r="E43" s="13">
-        <v>235.38</v>
+        <v>235.31</v>
       </c>
       <c r="F43" s="13">
-        <v>245.38</v>
+        <v>245.31</v>
       </c>
       <c r="G43" s="17"/>
     </row>
-    <row r="44" spans="1:7" x14ac:dyDescent="0.45">
+    <row r="44" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A44" s="7">
-        <v>46324</v>
+        <v>46325</v>
       </c>
       <c r="B44" s="8"/>
       <c r="C44" s="20" t="s">
         <v>26</v>
       </c>
       <c r="D44" s="10">
-        <v>271.07</v>
+        <v>269.13</v>
       </c>
       <c r="E44" s="10">
-        <v>234.03</v>
+        <v>234.96</v>
       </c>
       <c r="F44" s="10">
-        <v>244.03</v>
+        <v>244.96</v>
       </c>
       <c r="G44" s="17"/>
     </row>
-    <row r="45" spans="1:7" x14ac:dyDescent="0.45">
+    <row r="45" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A45" s="11">
-        <v>46324</v>
+        <v>46325</v>
       </c>
       <c r="B45" s="12"/>
       <c r="C45" s="21" t="s">
         <v>27</v>
       </c>
       <c r="D45" s="13">
-        <v>270.67</v>
+        <v>268.74</v>
       </c>
       <c r="E45" s="13">
-        <v>234.44</v>
+        <v>235.38</v>
       </c>
       <c r="F45" s="13">
-        <v>244.44</v>
+        <v>245.38</v>
       </c>
       <c r="G45" s="17"/>
     </row>
-    <row r="46" spans="1:7" x14ac:dyDescent="0.45">
+    <row r="46" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A46" s="14"/>
       <c r="B46" s="24"/>
       <c r="C46" s="15"/>
@@ -1499,7 +1499,7 @@
       <c r="F46" s="16"/>
       <c r="G46" s="17"/>
     </row>
-    <row r="47" spans="1:7" ht="20.25" x14ac:dyDescent="0.45">
+    <row r="47" spans="1:7" ht="20" x14ac:dyDescent="0.35">
       <c r="A47" s="25" t="s">
         <v>28</v>
       </c>
@@ -1510,7 +1510,7 @@
       <c r="F47" s="17"/>
       <c r="G47" s="17"/>
     </row>
-    <row r="48" spans="1:7" x14ac:dyDescent="0.45">
+    <row r="48" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A48" s="23" t="s">
         <v>4</v>
       </c>
@@ -1529,83 +1529,83 @@
       </c>
       <c r="G48" s="17"/>
     </row>
-    <row r="49" spans="1:7" x14ac:dyDescent="0.45">
+    <row r="49" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A49" s="7">
-        <v>46325</v>
+        <v>46326</v>
       </c>
       <c r="B49" s="8"/>
       <c r="C49" s="20" t="s">
         <v>29</v>
       </c>
       <c r="D49" s="10">
-        <v>263.20999999999998</v>
+        <v>261.82</v>
       </c>
       <c r="E49" s="10">
-        <v>223.93</v>
+        <v>223.52</v>
       </c>
       <c r="F49" s="10">
-        <v>233.93</v>
+        <v>233.52</v>
       </c>
       <c r="G49" s="28"/>
     </row>
-    <row r="50" spans="1:7" x14ac:dyDescent="0.45">
+    <row r="50" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A50" s="11">
-        <v>46325</v>
+        <v>46326</v>
       </c>
       <c r="B50" s="12"/>
       <c r="C50" s="21" t="s">
         <v>30</v>
       </c>
       <c r="D50" s="13">
-        <v>260.7</v>
+        <v>259.32</v>
       </c>
       <c r="E50" s="13">
-        <v>223.5</v>
+        <v>223.11</v>
       </c>
       <c r="F50" s="13">
-        <v>233.5</v>
+        <v>233.11</v>
       </c>
       <c r="G50" s="28"/>
     </row>
-    <row r="51" spans="1:7" x14ac:dyDescent="0.45">
+    <row r="51" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A51" s="7">
-        <v>46324</v>
+        <v>46325</v>
       </c>
       <c r="B51" s="8"/>
       <c r="C51" s="20" t="s">
         <v>29</v>
       </c>
       <c r="D51" s="10">
-        <v>262.76</v>
+        <v>263.20999999999998</v>
       </c>
       <c r="E51" s="10">
-        <v>223.28</v>
+        <v>223.93</v>
       </c>
       <c r="F51" s="10">
-        <v>233.28</v>
+        <v>233.93</v>
       </c>
       <c r="G51" s="17"/>
     </row>
-    <row r="52" spans="1:7" x14ac:dyDescent="0.45">
+    <row r="52" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A52" s="11">
-        <v>46324</v>
+        <v>46325</v>
       </c>
       <c r="B52" s="12"/>
       <c r="C52" s="21" t="s">
         <v>30</v>
       </c>
       <c r="D52" s="13">
-        <v>260.24</v>
+        <v>260.7</v>
       </c>
       <c r="E52" s="13">
-        <v>222.86</v>
+        <v>223.5</v>
       </c>
       <c r="F52" s="13">
-        <v>232.86</v>
+        <v>233.5</v>
       </c>
       <c r="G52" s="17"/>
     </row>
-    <row r="53" spans="1:7" x14ac:dyDescent="0.45">
+    <row r="53" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A53" s="14"/>
       <c r="B53" s="14"/>
       <c r="C53" s="15"/>
@@ -1614,7 +1614,7 @@
       <c r="F53" s="16"/>
       <c r="G53" s="17"/>
     </row>
-    <row r="54" spans="1:7" ht="20.25" x14ac:dyDescent="0.45">
+    <row r="54" spans="1:7" ht="20" x14ac:dyDescent="0.35">
       <c r="A54" s="27" t="s">
         <v>31</v>
       </c>
@@ -1625,7 +1625,7 @@
       <c r="F54" s="17"/>
       <c r="G54" s="17"/>
     </row>
-    <row r="55" spans="1:7" x14ac:dyDescent="0.45">
+    <row r="55" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A55" s="23" t="s">
         <v>4</v>
       </c>
@@ -1644,54 +1644,54 @@
       </c>
       <c r="G55" s="17"/>
     </row>
-    <row r="56" spans="1:7" x14ac:dyDescent="0.45">
+    <row r="56" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A56" s="7">
-        <v>46325</v>
+        <v>46326</v>
       </c>
       <c r="B56" s="8"/>
       <c r="C56" s="20" t="s">
         <v>32</v>
       </c>
       <c r="D56" s="10">
-        <v>275.10000000000002</v>
+        <v>272.92</v>
       </c>
       <c r="E56" s="10">
-        <v>251.67</v>
+        <v>251.44</v>
       </c>
       <c r="F56" s="10">
-        <v>261.67</v>
+        <v>261.44</v>
       </c>
       <c r="G56" s="17"/>
     </row>
-    <row r="57" spans="1:7" x14ac:dyDescent="0.45">
+    <row r="57" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A57" s="11">
-        <v>46325</v>
+        <v>46326</v>
       </c>
       <c r="B57" s="12"/>
       <c r="C57" s="21" t="s">
         <v>33</v>
       </c>
       <c r="D57" s="13">
-        <v>263.13</v>
+        <v>260.94</v>
       </c>
       <c r="E57" s="13">
-        <v>232.52</v>
+        <v>232.53</v>
       </c>
       <c r="F57" s="13">
-        <v>242.52</v>
+        <v>242.53</v>
       </c>
       <c r="G57" s="17"/>
     </row>
-    <row r="58" spans="1:7" x14ac:dyDescent="0.45">
+    <row r="58" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A58" s="7">
-        <v>46325</v>
+        <v>46326</v>
       </c>
       <c r="B58" s="8"/>
       <c r="C58" s="20" t="s">
         <v>34</v>
       </c>
       <c r="D58" s="10">
-        <v>263.93</v>
+        <v>261.74</v>
       </c>
       <c r="E58" s="10" t="s">
         <v>18</v>
@@ -1701,111 +1701,111 @@
       </c>
       <c r="G58" s="17"/>
     </row>
-    <row r="59" spans="1:7" x14ac:dyDescent="0.45">
+    <row r="59" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A59" s="11">
-        <v>46325</v>
+        <v>46326</v>
       </c>
       <c r="B59" s="12"/>
       <c r="C59" s="21" t="s">
         <v>35</v>
       </c>
       <c r="D59" s="13">
-        <v>260.02</v>
+        <v>257.89999999999998</v>
       </c>
       <c r="E59" s="13">
-        <v>226.9</v>
+        <v>226.91</v>
       </c>
       <c r="F59" s="13" t="s">
         <v>18</v>
       </c>
       <c r="G59" s="17"/>
     </row>
-    <row r="60" spans="1:7" x14ac:dyDescent="0.45">
+    <row r="60" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A60" s="7">
-        <v>46325</v>
+        <v>46326</v>
       </c>
       <c r="B60" s="8"/>
       <c r="C60" s="20" t="s">
         <v>36</v>
       </c>
       <c r="D60" s="10">
-        <v>255.85</v>
+        <v>253.73</v>
       </c>
       <c r="E60" s="10">
-        <v>222.84</v>
+        <v>222.85</v>
       </c>
       <c r="F60" s="10">
-        <v>232.84</v>
+        <v>232.85</v>
       </c>
       <c r="G60" s="17"/>
     </row>
-    <row r="61" spans="1:7" x14ac:dyDescent="0.45">
+    <row r="61" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A61" s="11">
-        <v>46325</v>
+        <v>46326</v>
       </c>
       <c r="B61" s="12"/>
       <c r="C61" s="21" t="s">
         <v>37</v>
       </c>
       <c r="D61" s="13">
-        <v>262.92</v>
+        <v>260.8</v>
       </c>
       <c r="E61" s="13">
-        <v>244.77</v>
+        <v>244.62</v>
       </c>
       <c r="F61" s="13" t="s">
         <v>18</v>
       </c>
       <c r="G61" s="17"/>
     </row>
-    <row r="62" spans="1:7" x14ac:dyDescent="0.45">
+    <row r="62" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A62" s="7">
-        <v>46324</v>
+        <v>46325</v>
       </c>
       <c r="B62" s="8"/>
       <c r="C62" s="20" t="s">
         <v>32</v>
       </c>
       <c r="D62" s="10">
-        <v>277.02</v>
+        <v>275.10000000000002</v>
       </c>
       <c r="E62" s="10">
-        <v>250.81</v>
+        <v>251.67</v>
       </c>
       <c r="F62" s="10">
-        <v>260.81</v>
+        <v>261.67</v>
       </c>
       <c r="G62" s="17"/>
     </row>
-    <row r="63" spans="1:7" x14ac:dyDescent="0.45">
+    <row r="63" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A63" s="11">
-        <v>46324</v>
+        <v>46325</v>
       </c>
       <c r="B63" s="12"/>
       <c r="C63" s="21" t="s">
         <v>33</v>
       </c>
       <c r="D63" s="13">
-        <v>264.5</v>
+        <v>263.13</v>
       </c>
       <c r="E63" s="13">
-        <v>231.56</v>
+        <v>232.52</v>
       </c>
       <c r="F63" s="13">
-        <v>241.56</v>
+        <v>242.52</v>
       </c>
       <c r="G63" s="17"/>
     </row>
-    <row r="64" spans="1:7" x14ac:dyDescent="0.45">
+    <row r="64" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A64" s="7">
-        <v>46324</v>
+        <v>46325</v>
       </c>
       <c r="B64" s="8"/>
       <c r="C64" s="20" t="s">
         <v>34</v>
       </c>
       <c r="D64" s="10">
-        <v>265.3</v>
+        <v>263.93</v>
       </c>
       <c r="E64" s="10" t="s">
         <v>18</v>
@@ -1815,55 +1815,55 @@
       </c>
       <c r="G64" s="17"/>
     </row>
-    <row r="65" spans="1:6" x14ac:dyDescent="0.45">
+    <row r="65" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A65" s="11">
-        <v>46324</v>
+        <v>46325</v>
       </c>
       <c r="B65" s="12"/>
       <c r="C65" s="21" t="s">
         <v>35</v>
       </c>
       <c r="D65" s="13">
-        <v>261.35000000000002</v>
+        <v>260.02</v>
       </c>
       <c r="E65" s="13">
-        <v>225.94</v>
+        <v>226.9</v>
       </c>
       <c r="F65" s="13" t="s">
         <v>18</v>
       </c>
     </row>
-    <row r="66" spans="1:6" x14ac:dyDescent="0.45">
+    <row r="66" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A66" s="7">
-        <v>46324</v>
+        <v>46325</v>
       </c>
       <c r="B66" s="8"/>
       <c r="C66" s="20" t="s">
         <v>36</v>
       </c>
       <c r="D66" s="10">
-        <v>257.19</v>
+        <v>255.85</v>
       </c>
       <c r="E66" s="10">
-        <v>221.88</v>
+        <v>222.84</v>
       </c>
       <c r="F66" s="10">
-        <v>231.88</v>
-      </c>
-    </row>
-    <row r="67" spans="1:6" x14ac:dyDescent="0.45">
+        <v>232.84</v>
+      </c>
+    </row>
+    <row r="67" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A67" s="11">
-        <v>46324</v>
+        <v>46325</v>
       </c>
       <c r="B67" s="12"/>
       <c r="C67" s="21" t="s">
         <v>37</v>
       </c>
       <c r="D67" s="13">
-        <v>264.81</v>
+        <v>262.92</v>
       </c>
       <c r="E67" s="13">
-        <v>243.87</v>
+        <v>244.77</v>
       </c>
       <c r="F67" s="13" t="s">
         <v>18</v>
@@ -1891,17 +1891,6 @@
 </file>
 
 <file path=customXml/item1.xml><?xml version="1.0" encoding="utf-8"?>
-<p:properties xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls">
-  <documentManagement>
-    <lcf76f155ced4ddcb4097134ff3c332f xmlns="87276d81-85f4-4ef2-9e6e-55066304288f">
-      <Terms xmlns="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
-    </lcf76f155ced4ddcb4097134ff3c332f>
-    <TaxCatchAll xmlns="b23b8984-eafa-4e79-985e-54f52f3da58e" xsi:nil="true"/>
-  </documentManagement>
-</p:properties>
-</file>
-
-<file path=customXml/item2.xml><?xml version="1.0" encoding="utf-8"?>
 <ct:contentTypeSchema xmlns:ct="http://schemas.microsoft.com/office/2006/metadata/contentType" xmlns:ma="http://schemas.microsoft.com/office/2006/metadata/properties/metaAttributes" ct:_="" ma:_="" ma:contentTypeName="Document" ma:contentTypeID="0x010100D3632DF5622958439304627C030B0427" ma:contentTypeVersion="18" ma:contentTypeDescription="Create a new document." ma:contentTypeScope="" ma:versionID="8c2ecbce386d6bac497f8eb2d8f0fb7a">
   <xsd:schema xmlns:xsd="http://www.w3.org/2001/XMLSchema" xmlns:xs="http://www.w3.org/2001/XMLSchema" xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:ns2="87276d81-85f4-4ef2-9e6e-55066304288f" xmlns:ns3="39e1dda6-d1d8-4c88-a3b9-f1abc1284bad" xmlns:ns4="b23b8984-eafa-4e79-985e-54f52f3da58e" targetNamespace="http://schemas.microsoft.com/office/2006/metadata/properties" ma:root="true" ma:fieldsID="4cfd0c2f651c1ce156ad4fcb44ea61dd" ns2:_="" ns3:_="" ns4:_="">
     <xsd:import namespace="87276d81-85f4-4ef2-9e6e-55066304288f"/>
@@ -2161,6 +2150,17 @@
 </ct:contentTypeSchema>
 </file>
 
+<file path=customXml/item2.xml><?xml version="1.0" encoding="utf-8"?>
+<p:properties xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls">
+  <documentManagement>
+    <lcf76f155ced4ddcb4097134ff3c332f xmlns="87276d81-85f4-4ef2-9e6e-55066304288f">
+      <Terms xmlns="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
+    </lcf76f155ced4ddcb4097134ff3c332f>
+    <TaxCatchAll xmlns="b23b8984-eafa-4e79-985e-54f52f3da58e" xsi:nil="true"/>
+  </documentManagement>
+</p:properties>
+</file>
+
 <file path=customXml/item3.xml><?xml version="1.0" encoding="utf-8"?>
 <?mso-contentType ?>
 <FormTemplates xmlns="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms">
@@ -2171,17 +2171,6 @@
 </file>
 
 <file path=customXml/itemProps1.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{57A83D98-2BAE-4D83-823A-D31C464B620C}">
-  <ds:schemaRefs>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/properties"/>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
-    <ds:schemaRef ds:uri="87276d81-85f4-4ef2-9e6e-55066304288f"/>
-    <ds:schemaRef ds:uri="b23b8984-eafa-4e79-985e-54f52f3da58e"/>
-  </ds:schemaRefs>
-</ds:datastoreItem>
-</file>
-
-<file path=customXml/itemProps2.xml><?xml version="1.0" encoding="utf-8"?>
 <ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{B44E1863-2778-41F9-ACBA-48420F931671}">
   <ds:schemaRefs>
     <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/contentType"/>
@@ -2201,6 +2190,17 @@
 </ds:datastoreItem>
 </file>
 
+<file path=customXml/itemProps2.xml><?xml version="1.0" encoding="utf-8"?>
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{57A83D98-2BAE-4D83-823A-D31C464B620C}">
+  <ds:schemaRefs>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/properties"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
+    <ds:schemaRef ds:uri="87276d81-85f4-4ef2-9e6e-55066304288f"/>
+    <ds:schemaRef ds:uri="b23b8984-eafa-4e79-985e-54f52f3da58e"/>
+  </ds:schemaRefs>
+</ds:datastoreItem>
+</file>
+
 <file path=customXml/itemProps3.xml><?xml version="1.0" encoding="utf-8"?>
 <ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{F60519E9-FD90-4339-869C-BC2F85719BB8}">
   <ds:schemaRefs>

</xml_diff>